<commit_message>
fix(parts): site items were double-counted (probe+site), pack prices were multiplied by piece count
</commit_message>
<xml_diff>
--- a/docs/sub-mission_parts.xlsx
+++ b/docs/sub-mission_parts.xlsx
@@ -1683,7 +1683,7 @@
         </is>
       </c>
       <c r="D28" s="7" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E28" s="6" t="inlineStr">
         <is>
@@ -1694,7 +1694,7 @@
         <v>3</v>
       </c>
       <c r="G28" s="8" t="n">
-        <v>18</v>
+        <v>3</v>
       </c>
       <c r="H28" s="7" t="inlineStr">
         <is>
@@ -1950,7 +1950,7 @@
       <c r="E33" s="14" t="n"/>
       <c r="F33" s="15" t="n"/>
       <c r="G33" s="15" t="n">
-        <v>64</v>
+        <v>49</v>
       </c>
       <c r="H33" s="14" t="n"/>
       <c r="I33" s="14" t="n"/>
@@ -2430,7 +2430,7 @@
         </is>
       </c>
       <c r="D44" s="7" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E44" s="6" t="inlineStr">
         <is>
@@ -2441,7 +2441,7 @@
         <v>20</v>
       </c>
       <c r="G44" s="8" t="n">
-        <v>80</v>
+        <v>20</v>
       </c>
       <c r="H44" s="7" t="inlineStr">
         <is>
@@ -2477,7 +2477,7 @@
       <c r="E45" s="14" t="n"/>
       <c r="F45" s="15" t="n"/>
       <c r="G45" s="15" t="n">
-        <v>465.45</v>
+        <v>405.45</v>
       </c>
       <c r="H45" s="14" t="n"/>
       <c r="I45" s="14" t="n"/>
@@ -2565,7 +2565,7 @@
         </is>
       </c>
       <c r="D49" s="7" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="E49" s="6" t="inlineStr">
         <is>
@@ -2576,7 +2576,7 @@
         <v>6</v>
       </c>
       <c r="G49" s="8" t="n">
-        <v>72</v>
+        <v>6</v>
       </c>
       <c r="H49" s="7" t="inlineStr">
         <is>
@@ -2668,7 +2668,7 @@
       <c r="E51" s="14" t="n"/>
       <c r="F51" s="15" t="n"/>
       <c r="G51" s="15" t="n">
-        <v>72</v>
+        <v>6</v>
       </c>
       <c r="H51" s="14" t="n"/>
       <c r="I51" s="14" t="n"/>
@@ -3794,7 +3794,7 @@
         </is>
       </c>
       <c r="D79" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E79" s="6" t="inlineStr">
         <is>
@@ -3805,7 +3805,7 @@
         <v>25</v>
       </c>
       <c r="G79" s="8" t="n">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="H79" s="7" t="inlineStr">
         <is>
@@ -3850,7 +3850,7 @@
         </is>
       </c>
       <c r="D80" s="18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E80" s="17" t="inlineStr">
         <is>
@@ -3861,7 +3861,7 @@
         <v>18</v>
       </c>
       <c r="G80" s="19" t="n">
-        <v>36</v>
+        <v>18</v>
       </c>
       <c r="H80" s="18" t="inlineStr">
         <is>
@@ -3906,7 +3906,7 @@
         </is>
       </c>
       <c r="D81" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E81" s="6" t="inlineStr">
         <is>
@@ -3917,7 +3917,7 @@
         <v>8</v>
       </c>
       <c r="G81" s="8" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="H81" s="7" t="inlineStr">
         <is>
@@ -3962,7 +3962,7 @@
         </is>
       </c>
       <c r="D82" s="18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E82" s="17" t="inlineStr">
         <is>
@@ -3973,7 +3973,7 @@
         <v>9</v>
       </c>
       <c r="G82" s="19" t="n">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="H82" s="18" t="inlineStr">
         <is>
@@ -4014,7 +4014,7 @@
         </is>
       </c>
       <c r="D83" s="18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E83" s="17" t="inlineStr">
         <is>
@@ -4025,7 +4025,7 @@
         <v>6</v>
       </c>
       <c r="G83" s="19" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H83" s="18" t="inlineStr">
         <is>
@@ -4066,7 +4066,7 @@
         </is>
       </c>
       <c r="D84" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E84" s="6" t="inlineStr">
         <is>
@@ -4077,7 +4077,7 @@
         <v>3</v>
       </c>
       <c r="G84" s="8" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="H84" s="7" t="inlineStr">
         <is>
@@ -4118,7 +4118,7 @@
         </is>
       </c>
       <c r="D85" s="7" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E85" s="6" t="inlineStr">
         <is>
@@ -4129,7 +4129,7 @@
         <v>1</v>
       </c>
       <c r="G85" s="8" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H85" s="7" t="inlineStr">
         <is>
@@ -4174,7 +4174,7 @@
         </is>
       </c>
       <c r="D86" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E86" s="6" t="inlineStr">
         <is>
@@ -4185,7 +4185,7 @@
         <v>5</v>
       </c>
       <c r="G86" s="8" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="H86" s="7" t="inlineStr">
         <is>
@@ -4230,7 +4230,7 @@
         </is>
       </c>
       <c r="D87" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E87" s="6" t="inlineStr">
         <is>
@@ -4241,7 +4241,7 @@
         <v>9</v>
       </c>
       <c r="G87" s="8" t="n">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="H87" s="7" t="inlineStr">
         <is>
@@ -4286,7 +4286,7 @@
         </is>
       </c>
       <c r="D88" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E88" s="6" t="inlineStr">
         <is>
@@ -4297,7 +4297,7 @@
         <v>10</v>
       </c>
       <c r="G88" s="8" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="H88" s="7" t="inlineStr">
         <is>
@@ -4338,7 +4338,7 @@
         </is>
       </c>
       <c r="D89" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E89" s="6" t="inlineStr">
         <is>
@@ -4349,7 +4349,7 @@
         <v>4</v>
       </c>
       <c r="G89" s="8" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="H89" s="7" t="inlineStr">
         <is>
@@ -4394,7 +4394,7 @@
         </is>
       </c>
       <c r="D90" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E90" s="6" t="inlineStr">
         <is>
@@ -4405,7 +4405,7 @@
         <v>4</v>
       </c>
       <c r="G90" s="8" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="H90" s="7" t="inlineStr">
         <is>
@@ -4450,7 +4450,7 @@
         </is>
       </c>
       <c r="D91" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E91" s="6" t="inlineStr">
         <is>
@@ -4461,7 +4461,7 @@
         <v>3</v>
       </c>
       <c r="G91" s="8" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="H91" s="7" t="inlineStr">
         <is>
@@ -4501,7 +4501,7 @@
       <c r="E92" s="14" t="n"/>
       <c r="F92" s="15" t="n"/>
       <c r="G92" s="15" t="n">
-        <v>231</v>
+        <v>105</v>
       </c>
       <c r="H92" s="14" t="n"/>
       <c r="I92" s="14" t="n"/>
@@ -5466,7 +5466,7 @@
       <c r="E119" s="14" t="n"/>
       <c r="F119" s="14" t="n"/>
       <c r="G119" s="25" t="n">
-        <v>1089.31</v>
+        <v>834.3100000000001</v>
       </c>
     </row>
     <row r="120">
@@ -5481,7 +5481,7 @@
       <c r="E120" s="14" t="n"/>
       <c r="F120" s="14" t="n"/>
       <c r="G120" s="27" t="n">
-        <v>508</v>
+        <v>496</v>
       </c>
     </row>
     <row r="121">
@@ -5496,7 +5496,7 @@
       <c r="E121" s="14" t="n"/>
       <c r="F121" s="14" t="n"/>
       <c r="G121" s="29" t="n">
-        <v>1597.31</v>
+        <v>1330.31</v>
       </c>
     </row>
     <row r="122">
@@ -5526,7 +5526,7 @@
       <c r="E123" s="14" t="n"/>
       <c r="F123" s="14" t="n"/>
       <c r="G123" s="33" t="n">
-        <v>1527.31</v>
+        <v>1260.31</v>
       </c>
     </row>
   </sheetData>
@@ -5650,7 +5650,7 @@
         </is>
       </c>
       <c r="B6" s="36" t="n">
-        <v>64</v>
+        <v>49</v>
       </c>
       <c r="C6" s="36" t="n">
         <v>0</v>
@@ -5666,7 +5666,7 @@
         </is>
       </c>
       <c r="B7" s="36" t="n">
-        <v>111.45</v>
+        <v>51.45</v>
       </c>
       <c r="C7" s="36" t="n">
         <v>354</v>
@@ -5682,7 +5682,7 @@
         </is>
       </c>
       <c r="B8" s="36" t="n">
-        <v>72</v>
+        <v>6</v>
       </c>
       <c r="C8" s="36" t="n">
         <v>0</v>
@@ -5730,10 +5730,10 @@
         </is>
       </c>
       <c r="B11" s="36" t="n">
-        <v>207</v>
+        <v>93</v>
       </c>
       <c r="C11" s="36" t="n">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="D11" s="14" t="n">
         <v>13</v>
@@ -5794,10 +5794,10 @@
         </is>
       </c>
       <c r="B15" s="38" t="n">
-        <v>1089.31</v>
+        <v>834.3100000000001</v>
       </c>
       <c r="C15" s="38" t="n">
-        <v>508</v>
+        <v>496</v>
       </c>
       <c r="D15" s="39" t="n"/>
     </row>

</xml_diff>

<commit_message>
fix(gateway): single-channel Wio-E5 gateway replaces RAK2287 mini-PCIe (which needs a Pi HAT); concentrator demoted to optional upgrade
</commit_message>
<xml_diff>
--- a/docs/sub-mission_parts.xlsx
+++ b/docs/sub-mission_parts.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Parts list'!$A$4:$L$123</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Parts list'!$A$4:$L$124</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Parts list'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -628,7 +628,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L123"/>
+  <dimension ref="A1:L124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4524,12 +4524,12 @@
       </c>
       <c r="B95" s="5" t="inlineStr">
         <is>
-          <t>Gateway concentrator</t>
+          <t>Gateway radio (single-channel)</t>
         </is>
       </c>
       <c r="C95" s="6" t="inlineStr">
         <is>
-          <t>RAK2287 SX1302 868MHz mini-PCIe + Pi HAT</t>
+          <t>Wio-E5 mini SX1262 868MHz + USB-UART bridge; plugs into RPi USB, no soldering</t>
         </is>
       </c>
       <c r="D95" s="7" t="n">
@@ -4541,14 +4541,14 @@
         </is>
       </c>
       <c r="F95" s="8" t="n">
-        <v>120</v>
+        <v>18</v>
       </c>
       <c r="G95" s="8" t="n">
-        <v>120</v>
+        <v>18</v>
       </c>
       <c r="H95" s="7" t="inlineStr">
         <is>
-          <t>REQUIRED*</t>
+          <t>REQUIRED</t>
         </is>
       </c>
       <c r="I95" s="7" t="inlineStr">
@@ -4563,12 +4563,12 @@
       </c>
       <c r="K95" s="5" t="inlineStr">
         <is>
-          <t>quote</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="L95" s="6" t="inlineStr">
         <is>
-          <t>*only if own LoRa gateway; NB-IoT variant drops it</t>
+          <t>single-channel Wio-E5 gateway: same radio as the probe, no concentrator needed | Concentrator NOT needed: our nodes share one channel/SF. Add 0-15 min TX jitter per node.</t>
         </is>
       </c>
     </row>
@@ -4624,7 +4624,7 @@
       </c>
       <c r="L96" s="17" t="inlineStr">
         <is>
-          <t>YOU ALREADY HAVE THIS - reuse, zero soldering</t>
+          <t>YOU ALREADY HAVE THIS - reuse, zero soldering | YOU ALREADY HAVE THIS - reuse, zero soldering; runs the gateway service</t>
         </is>
       </c>
     </row>
@@ -4680,7 +4680,7 @@
       </c>
       <c r="L97" s="6" t="inlineStr">
         <is>
-          <t>range-critical part | THE range-critical part</t>
+          <t>range-critical part | range-critical: gateway antenna gain + mast height set the link</t>
         </is>
       </c>
     </row>
@@ -4793,310 +4793,314 @@
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="13" t="inlineStr">
+      <c r="A100" s="20" t="inlineStr">
+        <is>
+          <t>I06</t>
+        </is>
+      </c>
+      <c r="B100" s="20" t="inlineStr">
+        <is>
+          <t>Concentrator upgrade (optional)</t>
+        </is>
+      </c>
+      <c r="C100" s="21" t="inlineStr">
+        <is>
+          <t>RAK2287 SX1302 mini-PCIe MODULE + RAK2287 Pi HAT (module alone is unusable - RPi has no mini-PCIe)</t>
+        </is>
+      </c>
+      <c r="D100" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="E100" s="21" t="inlineStr">
+        <is>
+          <t>rakwireless reseller</t>
+        </is>
+      </c>
+      <c r="F100" s="23" t="n">
+        <v>145</v>
+      </c>
+      <c r="G100" s="23" t="n">
+        <v>145</v>
+      </c>
+      <c r="H100" s="22" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="I100" s="22" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="J100" s="20" t="inlineStr">
+        <is>
+          <t>socketed reusable</t>
+        </is>
+      </c>
+      <c r="K100" s="20" t="inlineStr">
+        <is>
+          <t>quote</t>
+        </is>
+      </c>
+      <c r="L100" s="21" t="inlineStr">
+        <is>
+          <t>RAK2287 concentrator + Pi HAT, only for multi-SF/public TTN; module alone will not fit a Pi | Only for multi-SF / multi-channel / public TTN. Single-channel Wio-E5 gateway is enough for our 20 nodes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="13" t="inlineStr">
         <is>
           <t>subtotal - Gateway (base station)</t>
         </is>
       </c>
-      <c r="B100" s="14" t="n"/>
-      <c r="C100" s="14" t="n"/>
-      <c r="D100" s="14" t="n"/>
-      <c r="E100" s="14" t="n"/>
-      <c r="F100" s="15" t="n"/>
-      <c r="G100" s="15" t="n">
-        <v>300</v>
-      </c>
-      <c r="H100" s="14" t="n"/>
-      <c r="I100" s="14" t="n"/>
-      <c r="J100" s="14" t="n"/>
-      <c r="K100" s="14" t="n"/>
-      <c r="L100" s="14" t="n"/>
-    </row>
-    <row r="102" ht="20" customHeight="1">
-      <c r="A102" s="4" t="inlineStr">
+      <c r="B101" s="14" t="n"/>
+      <c r="C101" s="14" t="n"/>
+      <c r="D101" s="14" t="n"/>
+      <c r="E101" s="14" t="n"/>
+      <c r="F101" s="15" t="n"/>
+      <c r="G101" s="15" t="n">
+        <v>343</v>
+      </c>
+      <c r="H101" s="14" t="n"/>
+      <c r="I101" s="14" t="n"/>
+      <c r="J101" s="14" t="n"/>
+      <c r="K101" s="14" t="n"/>
+      <c r="L101" s="14" t="n"/>
+    </row>
+    <row r="103" ht="20" customHeight="1">
+      <c r="A103" s="4" t="inlineStr">
         <is>
           <t>10. Consumables</t>
-        </is>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" s="16" t="inlineStr">
-        <is>
-          <t>J01</t>
-        </is>
-      </c>
-      <c r="B103" s="16" t="inlineStr">
-        <is>
-          <t>Filament ASA</t>
-        </is>
-      </c>
-      <c r="C103" s="17" t="inlineStr">
-        <is>
-          <t>Prusament ASA 850g</t>
-        </is>
-      </c>
-      <c r="D103" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="E103" s="17" t="inlineStr">
-        <is>
-          <t>prusa3d.com</t>
-        </is>
-      </c>
-      <c r="F103" s="19" t="n">
-        <v>32</v>
-      </c>
-      <c r="G103" s="19" t="n">
-        <v>32</v>
-      </c>
-      <c r="H103" s="18" t="inlineStr">
-        <is>
-          <t>REQUIRED</t>
-        </is>
-      </c>
-      <c r="I103" s="18" t="inlineStr">
-        <is>
-          <t>CHECK</t>
-        </is>
-      </c>
-      <c r="J103" s="16" t="inlineStr">
-        <is>
-          <t>consumable</t>
-        </is>
-      </c>
-      <c r="K103" s="16" t="inlineStr">
-        <is>
-          <t>verified</t>
-        </is>
-      </c>
-      <c r="L103" s="17" t="inlineStr">
-        <is>
-          <t>you may only have PETG/PLA - ASA needed for UV/water</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="16" t="inlineStr">
         <is>
+          <t>J01</t>
+        </is>
+      </c>
+      <c r="B104" s="16" t="inlineStr">
+        <is>
+          <t>Filament ASA</t>
+        </is>
+      </c>
+      <c r="C104" s="17" t="inlineStr">
+        <is>
+          <t>Prusament ASA 850g</t>
+        </is>
+      </c>
+      <c r="D104" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E104" s="17" t="inlineStr">
+        <is>
+          <t>prusa3d.com</t>
+        </is>
+      </c>
+      <c r="F104" s="19" t="n">
+        <v>32</v>
+      </c>
+      <c r="G104" s="19" t="n">
+        <v>32</v>
+      </c>
+      <c r="H104" s="18" t="inlineStr">
+        <is>
+          <t>REQUIRED</t>
+        </is>
+      </c>
+      <c r="I104" s="18" t="inlineStr">
+        <is>
+          <t>CHECK</t>
+        </is>
+      </c>
+      <c r="J104" s="16" t="inlineStr">
+        <is>
+          <t>consumable</t>
+        </is>
+      </c>
+      <c r="K104" s="16" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="L104" s="17" t="inlineStr">
+        <is>
+          <t>you may only have PETG/PLA - ASA needed for UV/water</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="16" t="inlineStr">
+        <is>
           <t>J02</t>
         </is>
       </c>
-      <c r="B104" s="16" t="inlineStr">
+      <c r="B105" s="16" t="inlineStr">
         <is>
           <t>Filament PC Blend</t>
         </is>
       </c>
-      <c r="C104" s="17" t="inlineStr">
+      <c r="C105" s="17" t="inlineStr">
         <is>
           <t>Prusament PC Blend 970g (for wall/structural)</t>
         </is>
       </c>
-      <c r="D104" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="E104" s="17" t="inlineStr">
+      <c r="D105" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E105" s="17" t="inlineStr">
         <is>
           <t>prusa3d.com</t>
         </is>
       </c>
-      <c r="F104" s="19" t="n">
+      <c r="F105" s="19" t="n">
         <v>40</v>
       </c>
-      <c r="G104" s="19" t="n">
+      <c r="G105" s="19" t="n">
         <v>40</v>
       </c>
-      <c r="H104" s="18" t="inlineStr">
-        <is>
-          <t>REQUIRED</t>
-        </is>
-      </c>
-      <c r="I104" s="18" t="inlineStr">
+      <c r="H105" s="18" t="inlineStr">
+        <is>
+          <t>REQUIRED</t>
+        </is>
+      </c>
+      <c r="I105" s="18" t="inlineStr">
         <is>
           <t>CHECK</t>
         </is>
       </c>
-      <c r="J104" s="16" t="inlineStr">
+      <c r="J105" s="16" t="inlineStr">
         <is>
           <t>consumable</t>
         </is>
       </c>
-      <c r="K104" s="16" t="inlineStr">
-        <is>
-          <t>verified</t>
-        </is>
-      </c>
-      <c r="L104" s="17" t="inlineStr"/>
-    </row>
-    <row r="105">
-      <c r="A105" s="5" t="inlineStr">
-        <is>
-          <t>J03</t>
-        </is>
-      </c>
-      <c r="B105" s="5" t="inlineStr">
-        <is>
-          <t>Epoxy barrier</t>
-        </is>
-      </c>
-      <c r="C105" s="6" t="inlineStr">
-        <is>
-          <t>West System 105 + 206</t>
-        </is>
-      </c>
-      <c r="D105" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E105" s="6" t="inlineStr">
-        <is>
-          <t>techfun.sk</t>
-        </is>
-      </c>
-      <c r="F105" s="8" t="n">
-        <v>18</v>
-      </c>
-      <c r="G105" s="8" t="n">
-        <v>18</v>
-      </c>
-      <c r="H105" s="7" t="inlineStr">
-        <is>
-          <t>REQUIRED</t>
-        </is>
-      </c>
-      <c r="I105" s="7" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="J105" s="5" t="inlineStr">
-        <is>
-          <t>consumable</t>
-        </is>
-      </c>
-      <c r="K105" s="5" t="inlineStr">
-        <is>
-          <t>verified</t>
-        </is>
-      </c>
-      <c r="L105" s="6" t="inlineStr"/>
+      <c r="K105" s="16" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="L105" s="17" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" s="5" t="inlineStr">
         <is>
+          <t>J03</t>
+        </is>
+      </c>
+      <c r="B106" s="5" t="inlineStr">
+        <is>
+          <t>Epoxy barrier</t>
+        </is>
+      </c>
+      <c r="C106" s="6" t="inlineStr">
+        <is>
+          <t>West System 105 + 206</t>
+        </is>
+      </c>
+      <c r="D106" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E106" s="6" t="inlineStr">
+        <is>
+          <t>techfun.sk</t>
+        </is>
+      </c>
+      <c r="F106" s="8" t="n">
+        <v>18</v>
+      </c>
+      <c r="G106" s="8" t="n">
+        <v>18</v>
+      </c>
+      <c r="H106" s="7" t="inlineStr">
+        <is>
+          <t>REQUIRED</t>
+        </is>
+      </c>
+      <c r="I106" s="7" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="J106" s="5" t="inlineStr">
+        <is>
+          <t>consumable</t>
+        </is>
+      </c>
+      <c r="K106" s="5" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="L106" s="6" t="inlineStr"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="5" t="inlineStr">
+        <is>
           <t>J04</t>
         </is>
       </c>
-      <c r="B106" s="5" t="inlineStr">
+      <c r="B107" s="5" t="inlineStr">
         <is>
           <t>Conformal coat</t>
         </is>
       </c>
-      <c r="C106" s="6" t="inlineStr">
+      <c r="C107" s="6" t="inlineStr">
         <is>
           <t>Electrolube acrylic 200ml</t>
         </is>
       </c>
-      <c r="D106" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E106" s="6" t="inlineStr">
+      <c r="D107" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E107" s="6" t="inlineStr">
         <is>
           <t>tme.eu</t>
         </is>
       </c>
-      <c r="F106" s="8" t="n">
+      <c r="F107" s="8" t="n">
         <v>14</v>
       </c>
-      <c r="G106" s="8" t="n">
+      <c r="G107" s="8" t="n">
         <v>14</v>
       </c>
-      <c r="H106" s="7" t="inlineStr">
-        <is>
-          <t>REQUIRED</t>
-        </is>
-      </c>
-      <c r="I106" s="7" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="J106" s="5" t="inlineStr">
+      <c r="H107" s="7" t="inlineStr">
+        <is>
+          <t>REQUIRED</t>
+        </is>
+      </c>
+      <c r="I107" s="7" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="J107" s="5" t="inlineStr">
         <is>
           <t>consumable</t>
         </is>
       </c>
-      <c r="K106" s="5" t="inlineStr">
-        <is>
-          <t>verified</t>
-        </is>
-      </c>
-      <c r="L106" s="6" t="inlineStr"/>
-    </row>
-    <row r="107">
-      <c r="A107" s="16" t="inlineStr">
-        <is>
-          <t>J05</t>
-        </is>
-      </c>
-      <c r="B107" s="16" t="inlineStr">
-        <is>
-          <t>Silicone grease</t>
-        </is>
-      </c>
-      <c r="C107" s="17" t="inlineStr">
-        <is>
-          <t>Molykote 111 100g</t>
-        </is>
-      </c>
-      <c r="D107" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="E107" s="17" t="inlineStr">
-        <is>
-          <t>tme.eu</t>
-        </is>
-      </c>
-      <c r="F107" s="19" t="n">
-        <v>9</v>
-      </c>
-      <c r="G107" s="19" t="n">
-        <v>9</v>
-      </c>
-      <c r="H107" s="18" t="inlineStr">
-        <is>
-          <t>REQUIRED</t>
-        </is>
-      </c>
-      <c r="I107" s="18" t="inlineStr">
-        <is>
-          <t>CHECK</t>
-        </is>
-      </c>
-      <c r="J107" s="16" t="inlineStr">
-        <is>
-          <t>consumable</t>
-        </is>
-      </c>
-      <c r="K107" s="16" t="inlineStr">
-        <is>
-          <t>verified</t>
-        </is>
-      </c>
-      <c r="L107" s="17" t="inlineStr"/>
+      <c r="K107" s="5" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="L107" s="6" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" s="16" t="inlineStr">
         <is>
-          <t>J06</t>
+          <t>J05</t>
         </is>
       </c>
       <c r="B108" s="16" t="inlineStr">
         <is>
-          <t>Threadlocker</t>
+          <t>Silicone grease</t>
         </is>
       </c>
       <c r="C108" s="17" t="inlineStr">
         <is>
-          <t>Loctite 243 + 406</t>
+          <t>Molykote 111 100g</t>
         </is>
       </c>
       <c r="D108" s="18" t="n">
@@ -5108,10 +5112,10 @@
         </is>
       </c>
       <c r="F108" s="19" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="G108" s="19" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="H108" s="18" t="inlineStr">
         <is>
@@ -5138,17 +5142,17 @@
     <row r="109">
       <c r="A109" s="16" t="inlineStr">
         <is>
-          <t>J07</t>
+          <t>J06</t>
         </is>
       </c>
       <c r="B109" s="16" t="inlineStr">
         <is>
-          <t>Heat-set inserts</t>
+          <t>Threadlocker</t>
         </is>
       </c>
       <c r="C109" s="17" t="inlineStr">
         <is>
-          <t>M3/M4 brass assortment</t>
+          <t>Loctite 243 + 406</t>
         </is>
       </c>
       <c r="D109" s="18" t="n">
@@ -5160,10 +5164,10 @@
         </is>
       </c>
       <c r="F109" s="19" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="G109" s="19" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="H109" s="18" t="inlineStr">
         <is>
@@ -5190,152 +5194,148 @@
     <row r="110">
       <c r="A110" s="16" t="inlineStr">
         <is>
+          <t>J07</t>
+        </is>
+      </c>
+      <c r="B110" s="16" t="inlineStr">
+        <is>
+          <t>Heat-set inserts</t>
+        </is>
+      </c>
+      <c r="C110" s="17" t="inlineStr">
+        <is>
+          <t>M3/M4 brass assortment</t>
+        </is>
+      </c>
+      <c r="D110" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E110" s="17" t="inlineStr">
+        <is>
+          <t>tme.eu</t>
+        </is>
+      </c>
+      <c r="F110" s="19" t="n">
+        <v>6</v>
+      </c>
+      <c r="G110" s="19" t="n">
+        <v>6</v>
+      </c>
+      <c r="H110" s="18" t="inlineStr">
+        <is>
+          <t>REQUIRED</t>
+        </is>
+      </c>
+      <c r="I110" s="18" t="inlineStr">
+        <is>
+          <t>CHECK</t>
+        </is>
+      </c>
+      <c r="J110" s="16" t="inlineStr">
+        <is>
+          <t>consumable</t>
+        </is>
+      </c>
+      <c r="K110" s="16" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="L110" s="17" t="inlineStr"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="16" t="inlineStr">
+        <is>
           <t>J08</t>
         </is>
       </c>
-      <c r="B110" s="16" t="inlineStr">
+      <c r="B111" s="16" t="inlineStr">
         <is>
           <t>O-ring kit</t>
         </is>
       </c>
-      <c r="C110" s="17" t="inlineStr">
+      <c r="C111" s="17" t="inlineStr">
         <is>
           <t>NBR metric assortment</t>
         </is>
       </c>
-      <c r="D110" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="E110" s="17" t="inlineStr">
+      <c r="D111" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E111" s="17" t="inlineStr">
         <is>
           <t>tme.eu</t>
         </is>
       </c>
-      <c r="F110" s="19" t="n">
+      <c r="F111" s="19" t="n">
         <v>12</v>
       </c>
-      <c r="G110" s="19" t="n">
+      <c r="G111" s="19" t="n">
         <v>12</v>
       </c>
-      <c r="H110" s="18" t="inlineStr">
-        <is>
-          <t>REQUIRED</t>
-        </is>
-      </c>
-      <c r="I110" s="18" t="inlineStr">
+      <c r="H111" s="18" t="inlineStr">
+        <is>
+          <t>REQUIRED</t>
+        </is>
+      </c>
+      <c r="I111" s="18" t="inlineStr">
         <is>
           <t>CHECK</t>
         </is>
       </c>
-      <c r="J110" s="16" t="inlineStr">
+      <c r="J111" s="16" t="inlineStr">
         <is>
           <t>consumable</t>
         </is>
       </c>
-      <c r="K110" s="16" t="inlineStr">
-        <is>
-          <t>verified</t>
-        </is>
-      </c>
-      <c r="L110" s="17" t="inlineStr"/>
-    </row>
-    <row r="111">
-      <c r="A111" s="13" t="inlineStr">
+      <c r="K111" s="16" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="L111" s="17" t="inlineStr"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="13" t="inlineStr">
         <is>
           <t>subtotal - Consumables</t>
         </is>
       </c>
-      <c r="B111" s="14" t="n"/>
-      <c r="C111" s="14" t="n"/>
-      <c r="D111" s="14" t="n"/>
-      <c r="E111" s="14" t="n"/>
-      <c r="F111" s="15" t="n"/>
-      <c r="G111" s="15" t="n">
+      <c r="B112" s="14" t="n"/>
+      <c r="C112" s="14" t="n"/>
+      <c r="D112" s="14" t="n"/>
+      <c r="E112" s="14" t="n"/>
+      <c r="F112" s="15" t="n"/>
+      <c r="G112" s="15" t="n">
         <v>142</v>
       </c>
-      <c r="H111" s="14" t="n"/>
-      <c r="I111" s="14" t="n"/>
-      <c r="J111" s="14" t="n"/>
-      <c r="K111" s="14" t="n"/>
-      <c r="L111" s="14" t="n"/>
-    </row>
-    <row r="113" ht="20" customHeight="1">
-      <c r="A113" s="4" t="inlineStr">
+      <c r="H112" s="14" t="n"/>
+      <c r="I112" s="14" t="n"/>
+      <c r="J112" s="14" t="n"/>
+      <c r="K112" s="14" t="n"/>
+      <c r="L112" s="14" t="n"/>
+    </row>
+    <row r="114" ht="20" customHeight="1">
+      <c r="A114" s="4" t="inlineStr">
         <is>
           <t>11. Tooling (one-off)</t>
-        </is>
-      </c>
-    </row>
-    <row r="114">
-      <c r="A114" s="16" t="inlineStr">
-        <is>
-          <t>K01</t>
-        </is>
-      </c>
-      <c r="B114" s="16" t="inlineStr">
-        <is>
-          <t>Vacuum chamber</t>
-        </is>
-      </c>
-      <c r="C114" s="17" t="inlineStr">
-        <is>
-          <t>Bel-Art F42025 + gauge + pump</t>
-        </is>
-      </c>
-      <c r="D114" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="E114" s="17" t="inlineStr">
-        <is>
-          <t>tme.eu</t>
-        </is>
-      </c>
-      <c r="F114" s="19" t="n">
-        <v>85</v>
-      </c>
-      <c r="G114" s="19" t="n">
-        <v>85</v>
-      </c>
-      <c r="H114" s="18" t="inlineStr">
-        <is>
-          <t>RECOMMENDED</t>
-        </is>
-      </c>
-      <c r="I114" s="18" t="inlineStr">
-        <is>
-          <t>CHECK</t>
-        </is>
-      </c>
-      <c r="J114" s="16" t="inlineStr">
-        <is>
-          <t>reusable tool</t>
-        </is>
-      </c>
-      <c r="K114" s="16" t="inlineStr">
-        <is>
-          <t>verified</t>
-        </is>
-      </c>
-      <c r="L114" s="17" t="inlineStr">
-        <is>
-          <t>acceptance test rig; borrow if possible | acceptance test rig (one-off)</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="16" t="inlineStr">
         <is>
-          <t>K02</t>
+          <t>K01</t>
         </is>
       </c>
       <c r="B115" s="16" t="inlineStr">
         <is>
-          <t>Torque driver</t>
+          <t>Vacuum chamber</t>
         </is>
       </c>
       <c r="C115" s="17" t="inlineStr">
         <is>
-          <t>Wiha 28506 1.2Nm</t>
+          <t>Bel-Art F42025 + gauge + pump</t>
         </is>
       </c>
       <c r="D115" s="18" t="n">
@@ -5347,10 +5347,10 @@
         </is>
       </c>
       <c r="F115" s="19" t="n">
-        <v>40</v>
+        <v>85</v>
       </c>
       <c r="G115" s="19" t="n">
-        <v>40</v>
+        <v>85</v>
       </c>
       <c r="H115" s="18" t="inlineStr">
         <is>
@@ -5374,105 +5374,146 @@
       </c>
       <c r="L115" s="17" t="inlineStr">
         <is>
-          <t>one-off</t>
+          <t>acceptance test rig; borrow if possible | acceptance test rig (one-off)</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="16" t="inlineStr">
         <is>
+          <t>K02</t>
+        </is>
+      </c>
+      <c r="B116" s="16" t="inlineStr">
+        <is>
+          <t>Torque driver</t>
+        </is>
+      </c>
+      <c r="C116" s="17" t="inlineStr">
+        <is>
+          <t>Wiha 28506 1.2Nm</t>
+        </is>
+      </c>
+      <c r="D116" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E116" s="17" t="inlineStr">
+        <is>
+          <t>tme.eu</t>
+        </is>
+      </c>
+      <c r="F116" s="19" t="n">
+        <v>40</v>
+      </c>
+      <c r="G116" s="19" t="n">
+        <v>40</v>
+      </c>
+      <c r="H116" s="18" t="inlineStr">
+        <is>
+          <t>RECOMMENDED</t>
+        </is>
+      </c>
+      <c r="I116" s="18" t="inlineStr">
+        <is>
+          <t>CHECK</t>
+        </is>
+      </c>
+      <c r="J116" s="16" t="inlineStr">
+        <is>
+          <t>reusable tool</t>
+        </is>
+      </c>
+      <c r="K116" s="16" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="L116" s="17" t="inlineStr">
+        <is>
+          <t>one-off</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="16" t="inlineStr">
+        <is>
           <t>K03</t>
         </is>
       </c>
-      <c r="B116" s="16" t="inlineStr">
+      <c r="B117" s="16" t="inlineStr">
         <is>
           <t>Spring balance</t>
         </is>
       </c>
-      <c r="C116" s="17" t="inlineStr">
+      <c r="C117" s="17" t="inlineStr">
         <is>
           <t>0-5N for coupling slip jig</t>
         </is>
       </c>
-      <c r="D116" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="E116" s="17" t="inlineStr">
+      <c r="D117" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E117" s="17" t="inlineStr">
         <is>
           <t>local</t>
         </is>
       </c>
-      <c r="F116" s="19" t="n">
+      <c r="F117" s="19" t="n">
         <v>5</v>
       </c>
-      <c r="G116" s="19" t="n">
+      <c r="G117" s="19" t="n">
         <v>5</v>
       </c>
-      <c r="H116" s="18" t="inlineStr">
+      <c r="H117" s="18" t="inlineStr">
         <is>
           <t>RECOMMENDED</t>
         </is>
       </c>
-      <c r="I116" s="18" t="inlineStr">
+      <c r="I117" s="18" t="inlineStr">
         <is>
           <t>CHECK</t>
         </is>
       </c>
-      <c r="J116" s="16" t="inlineStr">
+      <c r="J117" s="16" t="inlineStr">
         <is>
           <t>reusable tool</t>
         </is>
       </c>
-      <c r="K116" s="16" t="inlineStr">
-        <is>
-          <t>verified</t>
-        </is>
-      </c>
-      <c r="L116" s="17" t="inlineStr">
+      <c r="K117" s="16" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="L117" s="17" t="inlineStr">
         <is>
           <t>needed for cogging/slip measurement | one-off</t>
         </is>
       </c>
     </row>
-    <row r="117">
-      <c r="A117" s="13" t="inlineStr">
+    <row r="118">
+      <c r="A118" s="13" t="inlineStr">
         <is>
           <t>subtotal - Tooling (one-off)</t>
         </is>
       </c>
-      <c r="B117" s="14" t="n"/>
-      <c r="C117" s="14" t="n"/>
-      <c r="D117" s="14" t="n"/>
-      <c r="E117" s="14" t="n"/>
-      <c r="F117" s="15" t="n"/>
-      <c r="G117" s="15" t="n">
+      <c r="B118" s="14" t="n"/>
+      <c r="C118" s="14" t="n"/>
+      <c r="D118" s="14" t="n"/>
+      <c r="E118" s="14" t="n"/>
+      <c r="F118" s="15" t="n"/>
+      <c r="G118" s="15" t="n">
         <v>130</v>
       </c>
-      <c r="H117" s="14" t="n"/>
-      <c r="I117" s="14" t="n"/>
-      <c r="J117" s="14" t="n"/>
-      <c r="K117" s="14" t="n"/>
-      <c r="L117" s="14" t="n"/>
-    </row>
-    <row r="119">
-      <c r="A119" s="24" t="inlineStr">
+      <c r="H118" s="14" t="n"/>
+      <c r="I118" s="14" t="n"/>
+      <c r="J118" s="14" t="n"/>
+      <c r="K118" s="14" t="n"/>
+      <c r="L118" s="14" t="n"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="24" t="inlineStr">
         <is>
           <t>REQUIRED (everything needed to build and deploy)</t>
-        </is>
-      </c>
-      <c r="B119" s="14" t="n"/>
-      <c r="C119" s="14" t="n"/>
-      <c r="D119" s="14" t="n"/>
-      <c r="E119" s="14" t="n"/>
-      <c r="F119" s="14" t="n"/>
-      <c r="G119" s="25" t="n">
-        <v>834.3100000000001</v>
-      </c>
-    </row>
-    <row r="120">
-      <c r="A120" s="26" t="inlineStr">
-        <is>
-          <t>recommended add-ons (DO, level probe, anti-theft, tools)</t>
         </is>
       </c>
       <c r="B120" s="14" t="n"/>
@@ -5480,14 +5521,14 @@
       <c r="D120" s="14" t="n"/>
       <c r="E120" s="14" t="n"/>
       <c r="F120" s="14" t="n"/>
-      <c r="G120" s="27" t="n">
-        <v>496</v>
+      <c r="G120" s="25" t="n">
+        <v>732.3100000000001</v>
       </c>
     </row>
     <row r="121">
-      <c r="A121" s="28" t="inlineStr">
-        <is>
-          <t>TOTAL if you buy everything</t>
+      <c r="A121" s="26" t="inlineStr">
+        <is>
+          <t>recommended add-ons (DO, level probe, anti-theft, tools)</t>
         </is>
       </c>
       <c r="B121" s="14" t="n"/>
@@ -5495,14 +5536,14 @@
       <c r="D121" s="14" t="n"/>
       <c r="E121" s="14" t="n"/>
       <c r="F121" s="14" t="n"/>
-      <c r="G121" s="29" t="n">
-        <v>1330.31</v>
+      <c r="G121" s="27" t="n">
+        <v>641</v>
       </c>
     </row>
     <row r="122">
-      <c r="A122" s="30" t="inlineStr">
-        <is>
-          <t>saved by reusing what you already own</t>
+      <c r="A122" s="28" t="inlineStr">
+        <is>
+          <t>TOTAL if you buy everything</t>
         </is>
       </c>
       <c r="B122" s="14" t="n"/>
@@ -5510,14 +5551,14 @@
       <c r="D122" s="14" t="n"/>
       <c r="E122" s="14" t="n"/>
       <c r="F122" s="14" t="n"/>
-      <c r="G122" s="31" t="n">
-        <v>-70</v>
+      <c r="G122" s="29" t="n">
+        <v>1373.31</v>
       </c>
     </row>
     <row r="123">
-      <c r="A123" s="32" t="inlineStr">
-        <is>
-          <t>net if you reuse your Raspberry Pi etc.</t>
+      <c r="A123" s="30" t="inlineStr">
+        <is>
+          <t>saved by reusing what you already own</t>
         </is>
       </c>
       <c r="B123" s="14" t="n"/>
@@ -5525,41 +5566,56 @@
       <c r="D123" s="14" t="n"/>
       <c r="E123" s="14" t="n"/>
       <c r="F123" s="14" t="n"/>
-      <c r="G123" s="33" t="n">
-        <v>1260.31</v>
+      <c r="G123" s="31" t="n">
+        <v>-70</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="32" t="inlineStr">
+        <is>
+          <t>net if you reuse your Raspberry Pi etc.</t>
+        </is>
+      </c>
+      <c r="B124" s="14" t="n"/>
+      <c r="C124" s="14" t="n"/>
+      <c r="D124" s="14" t="n"/>
+      <c r="E124" s="14" t="n"/>
+      <c r="F124" s="14" t="n"/>
+      <c r="G124" s="33" t="n">
+        <v>1303.31</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:L123"/>
+  <autoFilter ref="A4:L124"/>
   <mergeCells count="29">
     <mergeCell ref="A78:L78"/>
     <mergeCell ref="A16:L16"/>
     <mergeCell ref="A51:E51"/>
     <mergeCell ref="A120:F120"/>
     <mergeCell ref="A45:E45"/>
-    <mergeCell ref="A113:L113"/>
     <mergeCell ref="A2:L2"/>
     <mergeCell ref="A47:L47"/>
     <mergeCell ref="A5:L5"/>
     <mergeCell ref="A23:L23"/>
+    <mergeCell ref="A118:E118"/>
     <mergeCell ref="A122:F122"/>
     <mergeCell ref="A53:L53"/>
     <mergeCell ref="A56:E56"/>
     <mergeCell ref="A35:L35"/>
     <mergeCell ref="A21:E21"/>
     <mergeCell ref="A121:F121"/>
+    <mergeCell ref="A101:E101"/>
     <mergeCell ref="A76:E76"/>
     <mergeCell ref="A33:E33"/>
     <mergeCell ref="A58:L58"/>
-    <mergeCell ref="A102:L102"/>
     <mergeCell ref="A14:E14"/>
-    <mergeCell ref="A100:E100"/>
+    <mergeCell ref="A114:L114"/>
     <mergeCell ref="A123:F123"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A94:L94"/>
-    <mergeCell ref="A119:F119"/>
-    <mergeCell ref="A117:E117"/>
-    <mergeCell ref="A111:E111"/>
+    <mergeCell ref="A103:L103"/>
+    <mergeCell ref="A112:E112"/>
+    <mergeCell ref="A124:F124"/>
     <mergeCell ref="A92:E92"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5746,13 +5802,13 @@
         </is>
       </c>
       <c r="B12" s="36" t="n">
-        <v>300</v>
+        <v>198</v>
       </c>
       <c r="C12" s="36" t="n">
-        <v>0</v>
+        <v>145</v>
       </c>
       <c r="D12" s="14" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="13">
@@ -5794,10 +5850,10 @@
         </is>
       </c>
       <c r="B15" s="38" t="n">
-        <v>834.3100000000001</v>
+        <v>732.3100000000001</v>
       </c>
       <c r="C15" s="38" t="n">
-        <v>496</v>
+        <v>641</v>
       </c>
       <c r="D15" s="39" t="n"/>
     </row>

</xml_diff>

<commit_message>
docs: clarify Wio-E5 mini = STM32WLE5JC board (same SKU as gateway radio), buy 3
</commit_message>
<xml_diff>
--- a/docs/sub-mission_parts.xlsx
+++ b/docs/sub-mission_parts.xlsx
@@ -2943,7 +2943,7 @@
       </c>
       <c r="C61" s="6" t="inlineStr">
         <is>
-          <t>Wio-E5 SX1262 868MHz mini board</t>
+          <t>Wio-E5 mini = STM32WLE5JC (MCU+LoRa) + USB-C + CH340; 868 MHz, SMA antenna</t>
         </is>
       </c>
       <c r="D61" s="7" t="n">
@@ -2980,7 +2980,11 @@
           <t>verified</t>
         </is>
       </c>
-      <c r="L61" s="6" t="inlineStr"/>
+      <c r="L61" s="6" t="inlineStr">
+        <is>
+          <t>same board as gateway I01; in the probe USB-C unused (two USB devices cannot link) - connect over UART TX/RX/3V3/GND</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="5" t="inlineStr">
@@ -4529,7 +4533,7 @@
       </c>
       <c r="C95" s="6" t="inlineStr">
         <is>
-          <t>Wio-E5 mini SX1262 868MHz + USB-UART bridge; plugs into RPi USB, no soldering</t>
+          <t>Wio-E5 mini = STM32WLE5JC + USB-C + CH340; plugs straight into RPi USB</t>
         </is>
       </c>
       <c r="D95" s="7" t="n">
@@ -4568,7 +4572,7 @@
       </c>
       <c r="L95" s="6" t="inlineStr">
         <is>
-          <t>single-channel Wio-E5 gateway: same radio as the probe, no concentrator needed | Concentrator NOT needed: our nodes share one channel/SF. Add 0-15 min TX jitter per node.</t>
+          <t>single-channel Wio-E5 gateway: same radio as the probe, no concentrator needed | identical SKU to probe radio G03 - one firmware image both sides; buy 3 (1 probe, 1 gateway, 1 spare/range-test)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
simplify: Wio-E5 mini as the single brain (MCU+LoRa) in probe and gateway; ESP32-S3 dropped
</commit_message>
<xml_diff>
--- a/docs/sub-mission_parts.xlsx
+++ b/docs/sub-mission_parts.xlsx
@@ -2875,58 +2875,58 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="16" t="inlineStr">
+      <c r="A60" s="9" t="inlineStr">
         <is>
           <t>G02</t>
         </is>
       </c>
-      <c r="B60" s="16" t="inlineStr">
-        <is>
-          <t>MCU</t>
-        </is>
-      </c>
-      <c r="C60" s="17" t="inlineStr">
-        <is>
-          <t>LaskaKit ESP32-S3-DEVKit (~12uA sleep)</t>
-        </is>
-      </c>
-      <c r="D60" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="E60" s="17" t="inlineStr">
+      <c r="B60" s="9" t="inlineStr">
+        <is>
+          <t>MCU (NOT USED in simple build)</t>
+        </is>
+      </c>
+      <c r="C60" s="10" t="inlineStr">
+        <is>
+          <t>LaskaKit ESP32-S3-DEVKit</t>
+        </is>
+      </c>
+      <c r="D60" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E60" s="10" t="inlineStr">
         <is>
           <t>laskakit.cz</t>
         </is>
       </c>
-      <c r="F60" s="19" t="n">
-        <v>12</v>
-      </c>
-      <c r="G60" s="19" t="n">
-        <v>12</v>
-      </c>
-      <c r="H60" s="18" t="inlineStr">
-        <is>
-          <t>REQUIRED</t>
-        </is>
-      </c>
-      <c r="I60" s="18" t="inlineStr">
+      <c r="F60" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G60" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H60" s="11" t="inlineStr">
+        <is>
+          <t>DROP</t>
+        </is>
+      </c>
+      <c r="I60" s="11" t="inlineStr">
         <is>
           <t>CHECK</t>
         </is>
       </c>
-      <c r="J60" s="16" t="inlineStr">
+      <c r="J60" s="9" t="inlineStr">
         <is>
           <t>socketed reusable</t>
         </is>
       </c>
-      <c r="K60" s="16" t="inlineStr">
-        <is>
-          <t>verified</t>
-        </is>
-      </c>
-      <c r="L60" s="17" t="inlineStr">
-        <is>
-          <t>you have classic ESP32 devkits; S3 is different</t>
+      <c r="K60" s="9" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="L60" s="10" t="inlineStr">
+        <is>
+          <t>not used: Wio-E5 mini is the single brain (MCU + radio) | DROPPED: Wio-E5 mini is the single brain (MCU+LoRa). Bring back only if we need more GPIO/dual-core.</t>
         </is>
       </c>
     </row>
@@ -2938,12 +2938,12 @@
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>Radio</t>
+          <t>MCU + radio (single board)</t>
         </is>
       </c>
       <c r="C61" s="6" t="inlineStr">
         <is>
-          <t>Wio-E5 mini = STM32WLE5JC (MCU+LoRa) + USB-C + CH340; 868 MHz, SMA antenna</t>
+          <t>Seeed Wio-E5 mini: STM32WLE5JC Cortex-M4 + SX126x LoRa 868 MHz, USB-C, ADC/I2C/UART/GPIO</t>
         </is>
       </c>
       <c r="D61" s="7" t="n">
@@ -2982,7 +2982,7 @@
       </c>
       <c r="L61" s="6" t="inlineStr">
         <is>
-          <t>same board as gateway I01; in the probe USB-C unused (two USB devices cannot link) - connect over UART TX/RX/3V3/GND</t>
+          <t>does EVERYTHING in the probe: sensors + LoRa + duty cycle. u.FL/SMA antenna connector - check which, both work</t>
         </is>
       </c>
     </row>
@@ -3092,7 +3092,11 @@
           <t>verified</t>
         </is>
       </c>
-      <c r="L63" s="6" t="inlineStr"/>
+      <c r="L63" s="6" t="inlineStr">
+        <is>
+          <t>u.FL -&gt; SMA pigtail; skip if your board ships with SMA already</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="5" t="inlineStr">
@@ -3766,7 +3770,7 @@
       <c r="E76" s="14" t="n"/>
       <c r="F76" s="15" t="n"/>
       <c r="G76" s="15" t="n">
-        <v>118.9</v>
+        <v>106.9</v>
       </c>
       <c r="H76" s="14" t="n"/>
       <c r="I76" s="14" t="n"/>
@@ -4572,7 +4576,7 @@
       </c>
       <c r="L95" s="6" t="inlineStr">
         <is>
-          <t>single-channel Wio-E5 gateway: same radio as the probe, no concentrator needed | identical SKU to probe radio G03 - one firmware image both sides; buy 3 (1 probe, 1 gateway, 1 spare/range-test)</t>
+          <t>single-channel Wio-E5 gateway: same radio as the probe, no concentrator needed | same board as G03; USB-C straight into the Pi; runs the packet listener</t>
         </is>
       </c>
     </row>
@@ -5526,7 +5530,7 @@
       <c r="E120" s="14" t="n"/>
       <c r="F120" s="14" t="n"/>
       <c r="G120" s="25" t="n">
-        <v>732.3100000000001</v>
+        <v>720.3100000000001</v>
       </c>
     </row>
     <row r="121">
@@ -5556,7 +5560,7 @@
       <c r="E122" s="14" t="n"/>
       <c r="F122" s="14" t="n"/>
       <c r="G122" s="29" t="n">
-        <v>1373.31</v>
+        <v>1361.31</v>
       </c>
     </row>
     <row r="123">
@@ -5586,7 +5590,7 @@
       <c r="E124" s="14" t="n"/>
       <c r="F124" s="14" t="n"/>
       <c r="G124" s="33" t="n">
-        <v>1303.31</v>
+        <v>1291.31</v>
       </c>
     </row>
   </sheetData>
@@ -5774,7 +5778,7 @@
         </is>
       </c>
       <c r="B10" s="36" t="n">
-        <v>118.9</v>
+        <v>106.9</v>
       </c>
       <c r="C10" s="36" t="n">
         <v>0</v>
@@ -5854,7 +5858,7 @@
         </is>
       </c>
       <c r="B15" s="38" t="n">
-        <v>732.3100000000001</v>
+        <v>720.3100000000001</v>
       </c>
       <c r="C15" s="38" t="n">
         <v>641</v>

</xml_diff>

<commit_message>
docs: build procedure with gates + order sheet by shop with spares; cad: collar clamp replaces block-through-wall, visible cable run
</commit_message>
<xml_diff>
--- a/docs/sub-mission_parts.xlsx
+++ b/docs/sub-mission_parts.xlsx
@@ -8,7 +8,8 @@
   </bookViews>
   <sheets>
     <sheet name="Parts list" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Order (by shop)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Parts list'!$A$4:$L$124</definedName>
@@ -23,7 +24,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0.00 &quot;EUR&quot;"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="17">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -88,6 +89,19 @@
       <color rgb="00404040"/>
       <sz val="9"/>
     </font>
+    <font>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="007F6000"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="007F6000"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="11">
     <fill>
@@ -142,7 +156,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -164,11 +178,55 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -263,6 +321,40 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1178,10 +1270,10 @@
           <t>subtotal - Rotor &amp; drivetrain (wet side)</t>
         </is>
       </c>
-      <c r="B14" s="14" t="n"/>
-      <c r="C14" s="14" t="n"/>
-      <c r="D14" s="14" t="n"/>
-      <c r="E14" s="14" t="n"/>
+      <c r="B14" s="42" t="n"/>
+      <c r="C14" s="42" t="n"/>
+      <c r="D14" s="42" t="n"/>
+      <c r="E14" s="43" t="n"/>
       <c r="F14" s="15" t="n"/>
       <c r="G14" s="15" t="n">
         <v>8.16</v>
@@ -1425,10 +1517,10 @@
           <t>subtotal - Magnetic coupling</t>
         </is>
       </c>
-      <c r="B21" s="14" t="n"/>
-      <c r="C21" s="14" t="n"/>
-      <c r="D21" s="14" t="n"/>
-      <c r="E21" s="14" t="n"/>
+      <c r="B21" s="42" t="n"/>
+      <c r="C21" s="42" t="n"/>
+      <c r="D21" s="42" t="n"/>
+      <c r="E21" s="43" t="n"/>
       <c r="F21" s="15" t="n"/>
       <c r="G21" s="15" t="n">
         <v>18.8</v>
@@ -1944,10 +2036,10 @@
           <t>subtotal - Generator pod &amp; sealing</t>
         </is>
       </c>
-      <c r="B33" s="14" t="n"/>
-      <c r="C33" s="14" t="n"/>
-      <c r="D33" s="14" t="n"/>
-      <c r="E33" s="14" t="n"/>
+      <c r="B33" s="42" t="n"/>
+      <c r="C33" s="42" t="n"/>
+      <c r="D33" s="42" t="n"/>
+      <c r="E33" s="43" t="n"/>
       <c r="F33" s="15" t="n"/>
       <c r="G33" s="15" t="n">
         <v>49</v>
@@ -2471,10 +2563,10 @@
           <t>subtotal - Sensors</t>
         </is>
       </c>
-      <c r="B45" s="14" t="n"/>
-      <c r="C45" s="14" t="n"/>
-      <c r="D45" s="14" t="n"/>
-      <c r="E45" s="14" t="n"/>
+      <c r="B45" s="42" t="n"/>
+      <c r="C45" s="42" t="n"/>
+      <c r="D45" s="42" t="n"/>
+      <c r="E45" s="43" t="n"/>
       <c r="F45" s="15" t="n"/>
       <c r="G45" s="15" t="n">
         <v>405.45</v>
@@ -2662,10 +2754,10 @@
           <t>subtotal - Sensor cage &amp; mounting</t>
         </is>
       </c>
-      <c r="B51" s="14" t="n"/>
-      <c r="C51" s="14" t="n"/>
-      <c r="D51" s="14" t="n"/>
-      <c r="E51" s="14" t="n"/>
+      <c r="B51" s="42" t="n"/>
+      <c r="C51" s="42" t="n"/>
+      <c r="D51" s="42" t="n"/>
+      <c r="E51" s="43" t="n"/>
       <c r="F51" s="15" t="n"/>
       <c r="G51" s="15" t="n">
         <v>6</v>
@@ -2797,10 +2889,10 @@
           <t>subtotal - Wet-dry interface (cable)</t>
         </is>
       </c>
-      <c r="B56" s="14" t="n"/>
-      <c r="C56" s="14" t="n"/>
-      <c r="D56" s="14" t="n"/>
-      <c r="E56" s="14" t="n"/>
+      <c r="B56" s="42" t="n"/>
+      <c r="C56" s="42" t="n"/>
+      <c r="D56" s="42" t="n"/>
+      <c r="E56" s="43" t="n"/>
       <c r="F56" s="15" t="n"/>
       <c r="G56" s="15" t="n">
         <v>47</v>
@@ -3764,10 +3856,10 @@
           <t>subtotal - Electronics (dry box)</t>
         </is>
       </c>
-      <c r="B76" s="14" t="n"/>
-      <c r="C76" s="14" t="n"/>
-      <c r="D76" s="14" t="n"/>
-      <c r="E76" s="14" t="n"/>
+      <c r="B76" s="42" t="n"/>
+      <c r="C76" s="42" t="n"/>
+      <c r="D76" s="42" t="n"/>
+      <c r="E76" s="43" t="n"/>
       <c r="F76" s="15" t="n"/>
       <c r="G76" s="15" t="n">
         <v>106.9</v>
@@ -4503,10 +4595,10 @@
           <t>subtotal - Structure &amp; site</t>
         </is>
       </c>
-      <c r="B92" s="14" t="n"/>
-      <c r="C92" s="14" t="n"/>
-      <c r="D92" s="14" t="n"/>
-      <c r="E92" s="14" t="n"/>
+      <c r="B92" s="42" t="n"/>
+      <c r="C92" s="42" t="n"/>
+      <c r="D92" s="42" t="n"/>
+      <c r="E92" s="43" t="n"/>
       <c r="F92" s="15" t="n"/>
       <c r="G92" s="15" t="n">
         <v>105</v>
@@ -4862,10 +4954,10 @@
           <t>subtotal - Gateway (base station)</t>
         </is>
       </c>
-      <c r="B101" s="14" t="n"/>
-      <c r="C101" s="14" t="n"/>
-      <c r="D101" s="14" t="n"/>
-      <c r="E101" s="14" t="n"/>
+      <c r="B101" s="42" t="n"/>
+      <c r="C101" s="42" t="n"/>
+      <c r="D101" s="42" t="n"/>
+      <c r="E101" s="43" t="n"/>
       <c r="F101" s="15" t="n"/>
       <c r="G101" s="15" t="n">
         <v>343</v>
@@ -5309,10 +5401,10 @@
           <t>subtotal - Consumables</t>
         </is>
       </c>
-      <c r="B112" s="14" t="n"/>
-      <c r="C112" s="14" t="n"/>
-      <c r="D112" s="14" t="n"/>
-      <c r="E112" s="14" t="n"/>
+      <c r="B112" s="42" t="n"/>
+      <c r="C112" s="42" t="n"/>
+      <c r="D112" s="42" t="n"/>
+      <c r="E112" s="43" t="n"/>
       <c r="F112" s="15" t="n"/>
       <c r="G112" s="15" t="n">
         <v>142</v>
@@ -5504,10 +5596,10 @@
           <t>subtotal - Tooling (one-off)</t>
         </is>
       </c>
-      <c r="B118" s="14" t="n"/>
-      <c r="C118" s="14" t="n"/>
-      <c r="D118" s="14" t="n"/>
-      <c r="E118" s="14" t="n"/>
+      <c r="B118" s="42" t="n"/>
+      <c r="C118" s="42" t="n"/>
+      <c r="D118" s="42" t="n"/>
+      <c r="E118" s="43" t="n"/>
       <c r="F118" s="15" t="n"/>
       <c r="G118" s="15" t="n">
         <v>130</v>
@@ -5524,11 +5616,11 @@
           <t>REQUIRED (everything needed to build and deploy)</t>
         </is>
       </c>
-      <c r="B120" s="14" t="n"/>
-      <c r="C120" s="14" t="n"/>
-      <c r="D120" s="14" t="n"/>
-      <c r="E120" s="14" t="n"/>
-      <c r="F120" s="14" t="n"/>
+      <c r="B120" s="42" t="n"/>
+      <c r="C120" s="42" t="n"/>
+      <c r="D120" s="42" t="n"/>
+      <c r="E120" s="42" t="n"/>
+      <c r="F120" s="43" t="n"/>
       <c r="G120" s="25" t="n">
         <v>720.3100000000001</v>
       </c>
@@ -5539,11 +5631,11 @@
           <t>recommended add-ons (DO, level probe, anti-theft, tools)</t>
         </is>
       </c>
-      <c r="B121" s="14" t="n"/>
-      <c r="C121" s="14" t="n"/>
-      <c r="D121" s="14" t="n"/>
-      <c r="E121" s="14" t="n"/>
-      <c r="F121" s="14" t="n"/>
+      <c r="B121" s="42" t="n"/>
+      <c r="C121" s="42" t="n"/>
+      <c r="D121" s="42" t="n"/>
+      <c r="E121" s="42" t="n"/>
+      <c r="F121" s="43" t="n"/>
       <c r="G121" s="27" t="n">
         <v>641</v>
       </c>
@@ -5554,11 +5646,11 @@
           <t>TOTAL if you buy everything</t>
         </is>
       </c>
-      <c r="B122" s="14" t="n"/>
-      <c r="C122" s="14" t="n"/>
-      <c r="D122" s="14" t="n"/>
-      <c r="E122" s="14" t="n"/>
-      <c r="F122" s="14" t="n"/>
+      <c r="B122" s="42" t="n"/>
+      <c r="C122" s="42" t="n"/>
+      <c r="D122" s="42" t="n"/>
+      <c r="E122" s="42" t="n"/>
+      <c r="F122" s="43" t="n"/>
       <c r="G122" s="29" t="n">
         <v>1361.31</v>
       </c>
@@ -5569,11 +5661,11 @@
           <t>saved by reusing what you already own</t>
         </is>
       </c>
-      <c r="B123" s="14" t="n"/>
-      <c r="C123" s="14" t="n"/>
-      <c r="D123" s="14" t="n"/>
-      <c r="E123" s="14" t="n"/>
-      <c r="F123" s="14" t="n"/>
+      <c r="B123" s="42" t="n"/>
+      <c r="C123" s="42" t="n"/>
+      <c r="D123" s="42" t="n"/>
+      <c r="E123" s="42" t="n"/>
+      <c r="F123" s="43" t="n"/>
       <c r="G123" s="31" t="n">
         <v>-70</v>
       </c>
@@ -5584,11 +5676,11 @@
           <t>net if you reuse your Raspberry Pi etc.</t>
         </is>
       </c>
-      <c r="B124" s="14" t="n"/>
-      <c r="C124" s="14" t="n"/>
-      <c r="D124" s="14" t="n"/>
-      <c r="E124" s="14" t="n"/>
-      <c r="F124" s="14" t="n"/>
+      <c r="B124" s="42" t="n"/>
+      <c r="C124" s="42" t="n"/>
+      <c r="D124" s="42" t="n"/>
+      <c r="E124" s="42" t="n"/>
+      <c r="F124" s="43" t="n"/>
       <c r="G124" s="33" t="n">
         <v>1291.31</v>
       </c>
@@ -5598,8 +5690,8 @@
   <mergeCells count="29">
     <mergeCell ref="A78:L78"/>
     <mergeCell ref="A16:L16"/>
+    <mergeCell ref="A120:F120"/>
     <mergeCell ref="A51:E51"/>
-    <mergeCell ref="A120:F120"/>
     <mergeCell ref="A45:E45"/>
     <mergeCell ref="A2:L2"/>
     <mergeCell ref="A47:L47"/>
@@ -5637,6 +5729,2780 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
+  <dimension ref="A1:G143"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="62" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="34" t="inlineStr">
+        <is>
+          <t>ORDER SHEET - grouped by shop, quantities already include spares</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="44" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B3" s="44" t="inlineStr">
+        <is>
+          <t>Part</t>
+        </is>
+      </c>
+      <c r="C3" s="44" t="inlineStr">
+        <is>
+          <t>Qty needed</t>
+        </is>
+      </c>
+      <c r="D3" s="44" t="inlineStr">
+        <is>
+          <t>BUY THIS</t>
+        </is>
+      </c>
+      <c r="E3" s="44" t="inlineStr">
+        <is>
+          <t>Unit EUR</t>
+        </is>
+      </c>
+      <c r="F3" s="44" t="inlineStr">
+        <is>
+          <t>Line EUR</t>
+        </is>
+      </c>
+      <c r="G3" s="44" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="45" t="inlineStr">
+        <is>
+          <t>TME</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="59" t="inlineStr">
+        <is>
+          <t>A04</t>
+        </is>
+      </c>
+      <c r="B5" s="47" t="inlineStr">
+        <is>
+          <t>Wet bearing</t>
+        </is>
+      </c>
+      <c r="C5" s="59" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5" s="60" t="n">
+        <v>4</v>
+      </c>
+      <c r="E5" s="61" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="F5" s="61" t="n">
+        <v>4.72</v>
+      </c>
+      <c r="G5" s="47" t="inlineStr">
+        <is>
+          <t>83 pcs in stock; JFM-0507-05 flanged 1.48 USD alt</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="59" t="inlineStr">
+        <is>
+          <t>A06</t>
+        </is>
+      </c>
+      <c r="B6" s="47" t="inlineStr">
+        <is>
+          <t>Set screw</t>
+        </is>
+      </c>
+      <c r="C6" s="59" t="n">
+        <v>2</v>
+      </c>
+      <c r="D6" s="60" t="n">
+        <v>4</v>
+      </c>
+      <c r="E6" s="61" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" s="61" t="n">
+        <v>4</v>
+      </c>
+      <c r="G6" s="47" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="59" t="inlineStr">
+        <is>
+          <t>C03</t>
+        </is>
+      </c>
+      <c r="B7" s="47" t="inlineStr">
+        <is>
+          <t>Pod O-ring</t>
+        </is>
+      </c>
+      <c r="C7" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" s="60" t="n">
+        <v>3</v>
+      </c>
+      <c r="E7" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="F7" s="61" t="n">
+        <v>9</v>
+      </c>
+      <c r="G7" s="47" t="inlineStr">
+        <is>
+          <t>grease Molykote 111</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="59" t="inlineStr">
+        <is>
+          <t>C05</t>
+        </is>
+      </c>
+      <c r="B8" s="47" t="inlineStr">
+        <is>
+          <t>Pod clamp screws</t>
+        </is>
+      </c>
+      <c r="C8" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="60" t="n">
+        <v>3</v>
+      </c>
+      <c r="E8" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="F8" s="61" t="n">
+        <v>9</v>
+      </c>
+      <c r="G8" s="47" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="59" t="inlineStr">
+        <is>
+          <t>C07</t>
+        </is>
+      </c>
+      <c r="B9" s="47" t="inlineStr">
+        <is>
+          <t>Cable gland wet side</t>
+        </is>
+      </c>
+      <c r="C9" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="60" t="n">
+        <v>2</v>
+      </c>
+      <c r="E9" s="61" t="n">
+        <v>12</v>
+      </c>
+      <c r="F9" s="61" t="n">
+        <v>24</v>
+      </c>
+      <c r="G9" s="47" t="inlineStr">
+        <is>
+          <t>NOT YET IN MODEL - add boss</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="59" t="inlineStr">
+        <is>
+          <t>C09</t>
+        </is>
+      </c>
+      <c r="B10" s="47" t="inlineStr">
+        <is>
+          <t>Generator mount</t>
+        </is>
+      </c>
+      <c r="C10" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" s="60" t="n">
+        <v>3</v>
+      </c>
+      <c r="E10" s="61" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="G10" s="47" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="59" t="inlineStr">
+        <is>
+          <t>D06</t>
+        </is>
+      </c>
+      <c r="B11" s="47" t="inlineStr">
+        <is>
+          <t>EC/TDS</t>
+        </is>
+      </c>
+      <c r="C11" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" s="60" t="n">
+        <v>2</v>
+      </c>
+      <c r="E11" s="61" t="n">
+        <v>14</v>
+      </c>
+      <c r="F11" s="61" t="n">
+        <v>28</v>
+      </c>
+      <c r="G11" s="47" t="inlineStr">
+        <is>
+          <t>+-10% FS is the weakest sensor; use as trend indicator, site-calibrate</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="59" t="inlineStr">
+        <is>
+          <t>D08</t>
+        </is>
+      </c>
+      <c r="B12" s="47" t="inlineStr">
+        <is>
+          <t>Sensor cable</t>
+        </is>
+      </c>
+      <c r="C12" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" s="60" t="n">
+        <v>2</v>
+      </c>
+      <c r="E12" s="61" t="n">
+        <v>20</v>
+      </c>
+      <c r="F12" s="61" t="n">
+        <v>40</v>
+      </c>
+      <c r="G12" s="47" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="59" t="inlineStr">
+        <is>
+          <t>E02</t>
+        </is>
+      </c>
+      <c r="B13" s="47" t="inlineStr">
+        <is>
+          <t>Cage fasteners</t>
+        </is>
+      </c>
+      <c r="C13" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" s="60" t="n">
+        <v>2</v>
+      </c>
+      <c r="E13" s="61" t="n">
+        <v>6</v>
+      </c>
+      <c r="F13" s="61" t="n">
+        <v>12</v>
+      </c>
+      <c r="G13" s="47" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="59" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="B14" s="47" t="inlineStr">
+        <is>
+          <t>Cable</t>
+        </is>
+      </c>
+      <c r="C14" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="61" t="n">
+        <v>35</v>
+      </c>
+      <c r="F14" s="61" t="n">
+        <v>35</v>
+      </c>
+      <c r="G14" s="47" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="59" t="inlineStr">
+        <is>
+          <t>F02</t>
+        </is>
+      </c>
+      <c r="B15" s="47" t="inlineStr">
+        <is>
+          <t>Bulkhead connector</t>
+        </is>
+      </c>
+      <c r="C15" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" s="60" t="n">
+        <v>2</v>
+      </c>
+      <c r="E15" s="61" t="n">
+        <v>12</v>
+      </c>
+      <c r="F15" s="61" t="n">
+        <v>24</v>
+      </c>
+      <c r="G15" s="47" t="inlineStr">
+        <is>
+          <t>cost cut from 85 EUR wet-mate</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="59" t="inlineStr">
+        <is>
+          <t>G01</t>
+        </is>
+      </c>
+      <c r="B16" s="47" t="inlineStr">
+        <is>
+          <t>Enclosure</t>
+        </is>
+      </c>
+      <c r="C16" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" s="60" t="n">
+        <v>2</v>
+      </c>
+      <c r="E16" s="61" t="n">
+        <v>22</v>
+      </c>
+      <c r="F16" s="61" t="n">
+        <v>44</v>
+      </c>
+      <c r="G16" s="47" t="inlineStr">
+        <is>
+          <t>in model as site_box</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="59" t="inlineStr">
+        <is>
+          <t>G05</t>
+        </is>
+      </c>
+      <c r="B17" s="47" t="inlineStr">
+        <is>
+          <t>Antenna pigtail</t>
+        </is>
+      </c>
+      <c r="C17" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" s="60" t="n">
+        <v>3</v>
+      </c>
+      <c r="E17" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="F17" s="61" t="n">
+        <v>9</v>
+      </c>
+      <c r="G17" s="47" t="inlineStr">
+        <is>
+          <t>u.FL -&gt; SMA pigtail; skip if your board ships with SMA already</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="59" t="inlineStr">
+        <is>
+          <t>G06</t>
+        </is>
+      </c>
+      <c r="B18" s="47" t="inlineStr">
+        <is>
+          <t>Boost harvester</t>
+        </is>
+      </c>
+      <c r="C18" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" s="60" t="n">
+        <v>2</v>
+      </c>
+      <c r="E18" s="61" t="n">
+        <v>5</v>
+      </c>
+      <c r="F18" s="61" t="n">
+        <v>10</v>
+      </c>
+      <c r="G18" s="47" t="inlineStr">
+        <is>
+          <t>needed when EMF below bus</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="59" t="inlineStr">
+        <is>
+          <t>G07</t>
+        </is>
+      </c>
+      <c r="B19" s="47" t="inlineStr">
+        <is>
+          <t>Buck</t>
+        </is>
+      </c>
+      <c r="C19" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" s="60" t="n">
+        <v>3</v>
+      </c>
+      <c r="E19" s="61" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F19" s="61" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="G19" s="47" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="59" t="inlineStr">
+        <is>
+          <t>G08</t>
+        </is>
+      </c>
+      <c r="B20" s="47" t="inlineStr">
+        <is>
+          <t>Rectifier</t>
+        </is>
+      </c>
+      <c r="C20" s="59" t="n">
+        <v>6</v>
+      </c>
+      <c r="D20" s="60" t="n">
+        <v>8</v>
+      </c>
+      <c r="E20" s="61" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="F20" s="61" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="G20" s="47" t="inlineStr">
+        <is>
+          <t>452k in stock</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="59" t="inlineStr">
+        <is>
+          <t>G09</t>
+        </is>
+      </c>
+      <c r="B21" s="47" t="inlineStr">
+        <is>
+          <t>Clamp</t>
+        </is>
+      </c>
+      <c r="C21" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" s="60" t="n">
+        <v>3</v>
+      </c>
+      <c r="E21" s="61" t="n">
+        <v>4</v>
+      </c>
+      <c r="F21" s="61" t="n">
+        <v>12</v>
+      </c>
+      <c r="G21" s="47" t="inlineStr">
+        <is>
+          <t>overvoltage protection</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="59" t="inlineStr">
+        <is>
+          <t>G10</t>
+        </is>
+      </c>
+      <c r="B22" s="47" t="inlineStr">
+        <is>
+          <t>Supercap</t>
+        </is>
+      </c>
+      <c r="C22" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" s="60" t="n">
+        <v>2</v>
+      </c>
+      <c r="E22" s="61" t="n">
+        <v>11</v>
+      </c>
+      <c r="F22" s="61" t="n">
+        <v>22</v>
+      </c>
+      <c r="G22" s="47" t="inlineStr">
+        <is>
+          <t>NO coin-cell EDLC (50ohm ESR kills TX)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="59" t="inlineStr">
+        <is>
+          <t>G11</t>
+        </is>
+      </c>
+      <c r="B23" s="47" t="inlineStr">
+        <is>
+          <t>Voltage supervisor</t>
+        </is>
+      </c>
+      <c r="C23" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" s="60" t="n">
+        <v>3</v>
+      </c>
+      <c r="E23" s="61" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F23" s="61" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="G23" s="47" t="inlineStr">
+        <is>
+          <t>gates buck at 4.8V</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="59" t="inlineStr">
+        <is>
+          <t>G12</t>
+        </is>
+      </c>
+      <c r="B24" s="47" t="inlineStr">
+        <is>
+          <t>Load switch</t>
+        </is>
+      </c>
+      <c r="C24" s="59" t="n">
+        <v>2</v>
+      </c>
+      <c r="D24" s="60" t="n">
+        <v>4</v>
+      </c>
+      <c r="E24" s="61" t="n">
+        <v>1</v>
+      </c>
+      <c r="F24" s="61" t="n">
+        <v>4</v>
+      </c>
+      <c r="G24" s="47" t="inlineStr">
+        <is>
+          <t>removes ground-loop need</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="59" t="inlineStr">
+        <is>
+          <t>G16</t>
+        </is>
+      </c>
+      <c r="B25" s="47" t="inlineStr">
+        <is>
+          <t>Protection</t>
+        </is>
+      </c>
+      <c r="C25" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" s="60" t="n">
+        <v>2</v>
+      </c>
+      <c r="E25" s="61" t="n">
+        <v>6</v>
+      </c>
+      <c r="F25" s="61" t="n">
+        <v>12</v>
+      </c>
+      <c r="G25" s="47" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="59" t="inlineStr">
+        <is>
+          <t>G17</t>
+        </is>
+      </c>
+      <c r="B26" s="47" t="inlineStr">
+        <is>
+          <t>Cable glands</t>
+        </is>
+      </c>
+      <c r="C26" s="59" t="n">
+        <v>3</v>
+      </c>
+      <c r="D26" s="60" t="n">
+        <v>5</v>
+      </c>
+      <c r="E26" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="F26" s="61" t="n">
+        <v>15</v>
+      </c>
+      <c r="G26" s="47" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="59" t="inlineStr">
+        <is>
+          <t>H06</t>
+        </is>
+      </c>
+      <c r="B27" s="47" t="inlineStr">
+        <is>
+          <t>Hinge collar</t>
+        </is>
+      </c>
+      <c r="C27" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D27" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="E27" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="F27" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="G27" s="47" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="59" t="inlineStr">
+        <is>
+          <t>H07</t>
+        </is>
+      </c>
+      <c r="B28" s="47" t="inlineStr">
+        <is>
+          <t>Shear pin</t>
+        </is>
+      </c>
+      <c r="C28" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D28" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="E28" s="61" t="n">
+        <v>1</v>
+      </c>
+      <c r="F28" s="61" t="n">
+        <v>1</v>
+      </c>
+      <c r="G28" s="47" t="inlineStr">
+        <is>
+          <t>releases pod on &gt;150N debris hit</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="59" t="inlineStr">
+        <is>
+          <t>H09</t>
+        </is>
+      </c>
+      <c r="B29" s="47" t="inlineStr">
+        <is>
+          <t>Guy line</t>
+        </is>
+      </c>
+      <c r="C29" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D29" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" s="61" t="n">
+        <v>9</v>
+      </c>
+      <c r="F29" s="61" t="n">
+        <v>9</v>
+      </c>
+      <c r="G29" s="47" t="inlineStr">
+        <is>
+          <t>45deg up/downstream</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="59" t="inlineStr">
+        <is>
+          <t>H11</t>
+        </is>
+      </c>
+      <c r="B30" s="47" t="inlineStr">
+        <is>
+          <t>Safety cable</t>
+        </is>
+      </c>
+      <c r="C30" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D30" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="E30" s="61" t="n">
+        <v>4</v>
+      </c>
+      <c r="F30" s="61" t="n">
+        <v>4</v>
+      </c>
+      <c r="G30" s="47" t="inlineStr">
+        <is>
+          <t>theft/flood retention</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="59" t="inlineStr">
+        <is>
+          <t>I04</t>
+        </is>
+      </c>
+      <c r="B31" s="47" t="inlineStr">
+        <is>
+          <t>Enclosure</t>
+        </is>
+      </c>
+      <c r="C31" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D31" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="E31" s="61" t="n">
+        <v>35</v>
+      </c>
+      <c r="F31" s="61" t="n">
+        <v>35</v>
+      </c>
+      <c r="G31" s="47" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="59" t="inlineStr">
+        <is>
+          <t>J04</t>
+        </is>
+      </c>
+      <c r="B32" s="47" t="inlineStr">
+        <is>
+          <t>Conformal coat</t>
+        </is>
+      </c>
+      <c r="C32" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D32" s="60" t="n">
+        <v>2</v>
+      </c>
+      <c r="E32" s="61" t="n">
+        <v>14</v>
+      </c>
+      <c r="F32" s="61" t="n">
+        <v>28</v>
+      </c>
+      <c r="G32" s="47" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="59" t="inlineStr">
+        <is>
+          <t>J05</t>
+        </is>
+      </c>
+      <c r="B33" s="47" t="inlineStr">
+        <is>
+          <t>Silicone grease</t>
+        </is>
+      </c>
+      <c r="C33" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D33" s="60" t="n">
+        <v>2</v>
+      </c>
+      <c r="E33" s="61" t="n">
+        <v>9</v>
+      </c>
+      <c r="F33" s="61" t="n">
+        <v>18</v>
+      </c>
+      <c r="G33" s="47" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="59" t="inlineStr">
+        <is>
+          <t>J06</t>
+        </is>
+      </c>
+      <c r="B34" s="47" t="inlineStr">
+        <is>
+          <t>Threadlocker</t>
+        </is>
+      </c>
+      <c r="C34" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D34" s="60" t="n">
+        <v>2</v>
+      </c>
+      <c r="E34" s="61" t="n">
+        <v>11</v>
+      </c>
+      <c r="F34" s="61" t="n">
+        <v>22</v>
+      </c>
+      <c r="G34" s="47" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="59" t="inlineStr">
+        <is>
+          <t>J07</t>
+        </is>
+      </c>
+      <c r="B35" s="47" t="inlineStr">
+        <is>
+          <t>Heat-set inserts</t>
+        </is>
+      </c>
+      <c r="C35" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D35" s="60" t="n">
+        <v>2</v>
+      </c>
+      <c r="E35" s="61" t="n">
+        <v>6</v>
+      </c>
+      <c r="F35" s="61" t="n">
+        <v>12</v>
+      </c>
+      <c r="G35" s="47" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="59" t="inlineStr">
+        <is>
+          <t>J08</t>
+        </is>
+      </c>
+      <c r="B36" s="47" t="inlineStr">
+        <is>
+          <t>O-ring kit</t>
+        </is>
+      </c>
+      <c r="C36" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D36" s="60" t="n">
+        <v>2</v>
+      </c>
+      <c r="E36" s="61" t="n">
+        <v>12</v>
+      </c>
+      <c r="F36" s="61" t="n">
+        <v>24</v>
+      </c>
+      <c r="G36" s="47" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="50" t="inlineStr">
+        <is>
+          <t>subtotal TME</t>
+        </is>
+      </c>
+      <c r="B37" s="51" t="n"/>
+      <c r="C37" s="51" t="n"/>
+      <c r="D37" s="51" t="n"/>
+      <c r="E37" s="51" t="n"/>
+      <c r="F37" s="15" t="n">
+        <v>489.92</v>
+      </c>
+      <c r="G37" s="51" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="45" t="inlineStr">
+        <is>
+          <t>techfun.sk</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="59" t="inlineStr">
+        <is>
+          <t>B04</t>
+        </is>
+      </c>
+      <c r="B40" s="47" t="inlineStr">
+        <is>
+          <t>Potting compound</t>
+        </is>
+      </c>
+      <c r="C40" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D40" s="60" t="n">
+        <v>2</v>
+      </c>
+      <c r="E40" s="61" t="n">
+        <v>14</v>
+      </c>
+      <c r="F40" s="61" t="n">
+        <v>28</v>
+      </c>
+      <c r="G40" s="47" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="59" t="inlineStr">
+        <is>
+          <t>D04</t>
+        </is>
+      </c>
+      <c r="B41" s="47" t="inlineStr">
+        <is>
+          <t>Temperature</t>
+        </is>
+      </c>
+      <c r="C41" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D41" s="60" t="n">
+        <v>2</v>
+      </c>
+      <c r="E41" s="61" t="n">
+        <v>5</v>
+      </c>
+      <c r="F41" s="61" t="n">
+        <v>10</v>
+      </c>
+      <c r="G41" s="47" t="inlineStr">
+        <is>
+          <t>in model as sensor_ntc</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="59" t="inlineStr">
+        <is>
+          <t>D07</t>
+        </is>
+      </c>
+      <c r="B42" s="47" t="inlineStr">
+        <is>
+          <t>Turbidity</t>
+        </is>
+      </c>
+      <c r="C42" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D42" s="60" t="n">
+        <v>2</v>
+      </c>
+      <c r="E42" s="61" t="n">
+        <v>12.45</v>
+      </c>
+      <c r="F42" s="61" t="n">
+        <v>24.9</v>
+      </c>
+      <c r="G42" s="47" t="inlineStr">
+        <is>
+          <t>6 in stock; in model as sensor_turb</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="59" t="inlineStr">
+        <is>
+          <t>G03</t>
+        </is>
+      </c>
+      <c r="B43" s="47" t="inlineStr">
+        <is>
+          <t>MCU + radio (single board)</t>
+        </is>
+      </c>
+      <c r="C43" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D43" s="60" t="n">
+        <v>2</v>
+      </c>
+      <c r="E43" s="61" t="n">
+        <v>15</v>
+      </c>
+      <c r="F43" s="61" t="n">
+        <v>30</v>
+      </c>
+      <c r="G43" s="47" t="inlineStr">
+        <is>
+          <t>does EVERYTHING in the probe: sensors + LoRa + duty cycle. u.FL/SMA an</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="59" t="inlineStr">
+        <is>
+          <t>J03</t>
+        </is>
+      </c>
+      <c r="B44" s="47" t="inlineStr">
+        <is>
+          <t>Epoxy barrier</t>
+        </is>
+      </c>
+      <c r="C44" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D44" s="60" t="n">
+        <v>2</v>
+      </c>
+      <c r="E44" s="61" t="n">
+        <v>18</v>
+      </c>
+      <c r="F44" s="61" t="n">
+        <v>36</v>
+      </c>
+      <c r="G44" s="47" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="50" t="inlineStr">
+        <is>
+          <t>subtotal techfun.sk</t>
+        </is>
+      </c>
+      <c r="B45" s="51" t="n"/>
+      <c r="C45" s="51" t="n"/>
+      <c r="D45" s="51" t="n"/>
+      <c r="E45" s="51" t="n"/>
+      <c r="F45" s="15" t="n">
+        <v>128.9</v>
+      </c>
+      <c r="G45" s="51" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="45" t="inlineStr">
+        <is>
+          <t>local / other</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="59" t="inlineStr">
+        <is>
+          <t>A01</t>
+        </is>
+      </c>
+      <c r="B48" s="47" t="inlineStr">
+        <is>
+          <t>Blade</t>
+        </is>
+      </c>
+      <c r="C48" s="59" t="n">
+        <v>3</v>
+      </c>
+      <c r="D48" s="60" t="n">
+        <v>5</v>
+      </c>
+      <c r="E48" s="61" t="n">
+        <v>0</v>
+      </c>
+      <c r="F48" s="61" t="n">
+        <v>0</v>
+      </c>
+      <c r="G48" s="47" t="inlineStr">
+        <is>
+          <t>ASA or ASA-CF; 6 perimeters; epoxy coat; spare blade = fuse for branch</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="59" t="inlineStr">
+        <is>
+          <t>A02</t>
+        </is>
+      </c>
+      <c r="B49" s="47" t="inlineStr">
+        <is>
+          <t>Hub</t>
+        </is>
+      </c>
+      <c r="C49" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D49" s="60" t="n">
+        <v>3</v>
+      </c>
+      <c r="E49" s="61" t="n">
+        <v>0</v>
+      </c>
+      <c r="F49" s="61" t="n">
+        <v>0</v>
+      </c>
+      <c r="G49" s="47" t="inlineStr">
+        <is>
+          <t>brass inserts M4 from TME</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="59" t="inlineStr">
+        <is>
+          <t>A07</t>
+        </is>
+      </c>
+      <c r="B50" s="47" t="inlineStr">
+        <is>
+          <t>Weed guard ring</t>
+        </is>
+      </c>
+      <c r="C50" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D50" s="60" t="n">
+        <v>3</v>
+      </c>
+      <c r="E50" s="61" t="n">
+        <v>0</v>
+      </c>
+      <c r="F50" s="61" t="n">
+        <v>0</v>
+      </c>
+      <c r="G50" s="47" t="inlineStr">
+        <is>
+          <t>in model as weed_guard</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="59" t="inlineStr">
+        <is>
+          <t>B02</t>
+        </is>
+      </c>
+      <c r="B51" s="47" t="inlineStr">
+        <is>
+          <t>Magnet cup</t>
+        </is>
+      </c>
+      <c r="C51" s="59" t="n">
+        <v>2</v>
+      </c>
+      <c r="D51" s="60" t="n">
+        <v>4</v>
+      </c>
+      <c r="E51" s="61" t="n">
+        <v>0</v>
+      </c>
+      <c r="F51" s="61" t="n">
+        <v>0</v>
+      </c>
+      <c r="G51" s="47" t="inlineStr">
+        <is>
+          <t>in model as magcup</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="59" t="inlineStr">
+        <is>
+          <t>C01</t>
+        </is>
+      </c>
+      <c r="B52" s="47" t="inlineStr">
+        <is>
+          <t>Pod barrel</t>
+        </is>
+      </c>
+      <c r="C52" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D52" s="60" t="n">
+        <v>3</v>
+      </c>
+      <c r="E52" s="61" t="n">
+        <v>0</v>
+      </c>
+      <c r="F52" s="61" t="n">
+        <v>0</v>
+      </c>
+      <c r="G52" s="47" t="inlineStr">
+        <is>
+          <t>in model as pod</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="59" t="inlineStr">
+        <is>
+          <t>C02</t>
+        </is>
+      </c>
+      <c r="B53" s="47" t="inlineStr">
+        <is>
+          <t>Tail cone</t>
+        </is>
+      </c>
+      <c r="C53" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D53" s="60" t="n">
+        <v>3</v>
+      </c>
+      <c r="E53" s="61" t="n">
+        <v>0</v>
+      </c>
+      <c r="F53" s="61" t="n">
+        <v>0</v>
+      </c>
+      <c r="G53" s="47" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="59" t="inlineStr">
+        <is>
+          <t>C04</t>
+        </is>
+      </c>
+      <c r="B54" s="47" t="inlineStr">
+        <is>
+          <t>O-ring groove</t>
+        </is>
+      </c>
+      <c r="C54" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D54" s="60" t="n">
+        <v>3</v>
+      </c>
+      <c r="E54" s="61" t="n">
+        <v>0</v>
+      </c>
+      <c r="F54" s="61" t="n">
+        <v>0</v>
+      </c>
+      <c r="G54" s="47" t="inlineStr">
+        <is>
+          <t>NOT YET IN MODEL - add to pod</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="59" t="inlineStr">
+        <is>
+          <t>C06</t>
+        </is>
+      </c>
+      <c r="B55" s="47" t="inlineStr">
+        <is>
+          <t>Desiccant</t>
+        </is>
+      </c>
+      <c r="C55" s="59" t="n">
+        <v>2</v>
+      </c>
+      <c r="D55" s="60" t="n">
+        <v>4</v>
+      </c>
+      <c r="E55" s="61" t="n">
+        <v>2</v>
+      </c>
+      <c r="F55" s="61" t="n">
+        <v>8</v>
+      </c>
+      <c r="G55" s="47" t="inlineStr">
+        <is>
+          <t>replace at service</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="59" t="inlineStr">
+        <is>
+          <t>E01</t>
+        </is>
+      </c>
+      <c r="B56" s="47" t="inlineStr">
+        <is>
+          <t>Sensor cage</t>
+        </is>
+      </c>
+      <c r="C56" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D56" s="60" t="n">
+        <v>3</v>
+      </c>
+      <c r="E56" s="61" t="n">
+        <v>0</v>
+      </c>
+      <c r="F56" s="61" t="n">
+        <v>0</v>
+      </c>
+      <c r="G56" s="47" t="inlineStr">
+        <is>
+          <t>in model as cage</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="59" t="inlineStr">
+        <is>
+          <t>E03</t>
+        </is>
+      </c>
+      <c r="B57" s="47" t="inlineStr">
+        <is>
+          <t>Sensor holders</t>
+        </is>
+      </c>
+      <c r="C57" s="59" t="n">
+        <v>5</v>
+      </c>
+      <c r="D57" s="60" t="n">
+        <v>7</v>
+      </c>
+      <c r="E57" s="61" t="n">
+        <v>0</v>
+      </c>
+      <c r="F57" s="61" t="n">
+        <v>0</v>
+      </c>
+      <c r="G57" s="47" t="inlineStr">
+        <is>
+          <t>in model as sensor bodies</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="59" t="inlineStr">
+        <is>
+          <t>H02</t>
+        </is>
+      </c>
+      <c r="B58" s="47" t="inlineStr">
+        <is>
+          <t>Pole</t>
+        </is>
+      </c>
+      <c r="C58" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D58" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="E58" s="61" t="n">
+        <v>18</v>
+      </c>
+      <c r="F58" s="61" t="n">
+        <v>18</v>
+      </c>
+      <c r="G58" s="47" t="inlineStr">
+        <is>
+          <t>removable mast pinned into receiver</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="59" t="inlineStr">
+        <is>
+          <t>H03</t>
+        </is>
+      </c>
+      <c r="B59" s="47" t="inlineStr">
+        <is>
+          <t>Receiver sleeve</t>
+        </is>
+      </c>
+      <c r="C59" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D59" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="E59" s="61" t="n">
+        <v>8</v>
+      </c>
+      <c r="F59" s="61" t="n">
+        <v>8</v>
+      </c>
+      <c r="G59" s="47" t="inlineStr">
+        <is>
+          <t>pinned mast interface</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="59" t="inlineStr">
+        <is>
+          <t>I02</t>
+        </is>
+      </c>
+      <c r="B60" s="47" t="inlineStr">
+        <is>
+          <t>Compute</t>
+        </is>
+      </c>
+      <c r="C60" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D60" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="E60" s="61" t="n">
+        <v>70</v>
+      </c>
+      <c r="F60" s="61" t="n">
+        <v>70</v>
+      </c>
+      <c r="G60" s="47" t="inlineStr">
+        <is>
+          <t>YOU ALREADY HAVE THIS - reuse, zero soldering; runs the gateway servic</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="50" t="inlineStr">
+        <is>
+          <t>subtotal local / other</t>
+        </is>
+      </c>
+      <c r="B61" s="51" t="n"/>
+      <c r="C61" s="51" t="n"/>
+      <c r="D61" s="51" t="n"/>
+      <c r="E61" s="51" t="n"/>
+      <c r="F61" s="15" t="n">
+        <v>104</v>
+      </c>
+      <c r="G61" s="51" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="45" t="inlineStr">
+        <is>
+          <t>Hornbach / stavebniny</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="59" t="inlineStr">
+        <is>
+          <t>H01</t>
+        </is>
+      </c>
+      <c r="B64" s="47" t="inlineStr">
+        <is>
+          <t>Ground screw anchor</t>
+        </is>
+      </c>
+      <c r="C64" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D64" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="E64" s="61" t="n">
+        <v>25</v>
+      </c>
+      <c r="F64" s="61" t="n">
+        <v>25</v>
+      </c>
+      <c r="G64" s="47" t="inlineStr">
+        <is>
+          <t>1-2kN lateral - covers flood case</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="59" t="inlineStr">
+        <is>
+          <t>H04</t>
+        </is>
+      </c>
+      <c r="B65" s="47" t="inlineStr">
+        <is>
+          <t>Arm tube</t>
+        </is>
+      </c>
+      <c r="C65" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D65" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="E65" s="61" t="n">
+        <v>9</v>
+      </c>
+      <c r="F65" s="61" t="n">
+        <v>9</v>
+      </c>
+      <c r="G65" s="47" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="59" t="inlineStr">
+        <is>
+          <t>H05</t>
+        </is>
+      </c>
+      <c r="B66" s="47" t="inlineStr">
+        <is>
+          <t>Drop tube</t>
+        </is>
+      </c>
+      <c r="C66" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D66" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="E66" s="61" t="n">
+        <v>6</v>
+      </c>
+      <c r="F66" s="61" t="n">
+        <v>6</v>
+      </c>
+      <c r="G66" s="47" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="59" t="inlineStr">
+        <is>
+          <t>H10</t>
+        </is>
+      </c>
+      <c r="B67" s="47" t="inlineStr">
+        <is>
+          <t>Guy anchor</t>
+        </is>
+      </c>
+      <c r="C67" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D67" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="E67" s="61" t="n">
+        <v>10</v>
+      </c>
+      <c r="F67" s="61" t="n">
+        <v>10</v>
+      </c>
+      <c r="G67" s="47" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="59" t="inlineStr">
+        <is>
+          <t>I05</t>
+        </is>
+      </c>
+      <c r="B68" s="47" t="inlineStr">
+        <is>
+          <t>Mast</t>
+        </is>
+      </c>
+      <c r="C68" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D68" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="E68" s="61" t="n">
+        <v>30</v>
+      </c>
+      <c r="F68" s="61" t="n">
+        <v>30</v>
+      </c>
+      <c r="G68" s="47" t="inlineStr">
+        <is>
+          <t>height sets range</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="50" t="inlineStr">
+        <is>
+          <t>subtotal Hornbach / stavebniny</t>
+        </is>
+      </c>
+      <c r="B69" s="51" t="n"/>
+      <c r="C69" s="51" t="n"/>
+      <c r="D69" s="51" t="n"/>
+      <c r="E69" s="51" t="n"/>
+      <c r="F69" s="15" t="n">
+        <v>80</v>
+      </c>
+      <c r="G69" s="51" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="45" t="inlineStr">
+        <is>
+          <t>Prusa3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="59" t="inlineStr">
+        <is>
+          <t>J01</t>
+        </is>
+      </c>
+      <c r="B72" s="47" t="inlineStr">
+        <is>
+          <t>Filament ASA</t>
+        </is>
+      </c>
+      <c r="C72" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D72" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="E72" s="61" t="n">
+        <v>32</v>
+      </c>
+      <c r="F72" s="61" t="n">
+        <v>32</v>
+      </c>
+      <c r="G72" s="47" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="59" t="inlineStr">
+        <is>
+          <t>J02</t>
+        </is>
+      </c>
+      <c r="B73" s="47" t="inlineStr">
+        <is>
+          <t>Filament PC Blend</t>
+        </is>
+      </c>
+      <c r="C73" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D73" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="E73" s="61" t="n">
+        <v>40</v>
+      </c>
+      <c r="F73" s="61" t="n">
+        <v>40</v>
+      </c>
+      <c r="G73" s="47" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="50" t="inlineStr">
+        <is>
+          <t>subtotal Prusa3D</t>
+        </is>
+      </c>
+      <c r="B74" s="51" t="n"/>
+      <c r="C74" s="51" t="n"/>
+      <c r="D74" s="51" t="n"/>
+      <c r="E74" s="51" t="n"/>
+      <c r="F74" s="15" t="n">
+        <v>72</v>
+      </c>
+      <c r="G74" s="51" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="45" t="inlineStr">
+        <is>
+          <t>x-teamrc.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="59" t="inlineStr">
+        <is>
+          <t>C08</t>
+        </is>
+      </c>
+      <c r="B77" s="47" t="inlineStr">
+        <is>
+          <t>Generator</t>
+        </is>
+      </c>
+      <c r="C77" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D77" s="60" t="n">
+        <v>2</v>
+      </c>
+      <c r="E77" s="61" t="n">
+        <v>26</v>
+      </c>
+      <c r="F77" s="61" t="n">
+        <v>52</v>
+      </c>
+      <c r="G77" s="47" t="inlineStr">
+        <is>
+          <t>XTG3506 preferred: encoder = free RPM/flow</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="50" t="inlineStr">
+        <is>
+          <t>subtotal x-teamrc.com</t>
+        </is>
+      </c>
+      <c r="B78" s="51" t="n"/>
+      <c r="C78" s="51" t="n"/>
+      <c r="D78" s="51" t="n"/>
+      <c r="E78" s="51" t="n"/>
+      <c r="F78" s="15" t="n">
+        <v>52</v>
+      </c>
+      <c r="G78" s="51" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="45" t="inlineStr">
+        <is>
+          <t>i4wifi.cz</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="59" t="inlineStr">
+        <is>
+          <t>I03</t>
+        </is>
+      </c>
+      <c r="B81" s="47" t="inlineStr">
+        <is>
+          <t>Antenna</t>
+        </is>
+      </c>
+      <c r="C81" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D81" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="E81" s="61" t="n">
+        <v>45</v>
+      </c>
+      <c r="F81" s="61" t="n">
+        <v>45</v>
+      </c>
+      <c r="G81" s="47" t="inlineStr">
+        <is>
+          <t>range-critical: gateway antenna gain + mast height set the link</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="50" t="inlineStr">
+        <is>
+          <t>subtotal i4wifi.cz</t>
+        </is>
+      </c>
+      <c r="B82" s="51" t="n"/>
+      <c r="C82" s="51" t="n"/>
+      <c r="D82" s="51" t="n"/>
+      <c r="E82" s="51" t="n"/>
+      <c r="F82" s="15" t="n">
+        <v>45</v>
+      </c>
+      <c r="G82" s="51" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="45" t="inlineStr">
+        <is>
+          <t>RAK reseller</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="59" t="inlineStr">
+        <is>
+          <t>I01</t>
+        </is>
+      </c>
+      <c r="B85" s="47" t="inlineStr">
+        <is>
+          <t>Gateway radio (single-channel)</t>
+        </is>
+      </c>
+      <c r="C85" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D85" s="60" t="n">
+        <v>2</v>
+      </c>
+      <c r="E85" s="61" t="n">
+        <v>18</v>
+      </c>
+      <c r="F85" s="61" t="n">
+        <v>36</v>
+      </c>
+      <c r="G85" s="47" t="inlineStr">
+        <is>
+          <t>same board as G03; USB-C straight into the Pi; runs the packet listene</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="50" t="inlineStr">
+        <is>
+          <t>subtotal RAK reseller</t>
+        </is>
+      </c>
+      <c r="B86" s="51" t="n"/>
+      <c r="C86" s="51" t="n"/>
+      <c r="D86" s="51" t="n"/>
+      <c r="E86" s="51" t="n"/>
+      <c r="F86" s="15" t="n">
+        <v>36</v>
+      </c>
+      <c r="G86" s="51" t="n"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="45" t="inlineStr">
+        <is>
+          <t>laskakit.cz</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="59" t="inlineStr">
+        <is>
+          <t>G13</t>
+        </is>
+      </c>
+      <c r="B89" s="47" t="inlineStr">
+        <is>
+          <t>Barometer</t>
+        </is>
+      </c>
+      <c r="C89" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D89" s="60" t="n">
+        <v>2</v>
+      </c>
+      <c r="E89" s="61" t="n">
+        <v>6</v>
+      </c>
+      <c r="F89" s="61" t="n">
+        <v>12</v>
+      </c>
+      <c r="G89" s="47" t="inlineStr">
+        <is>
+          <t>pressure reference for MS5837</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="59" t="inlineStr">
+        <is>
+          <t>G15</t>
+        </is>
+      </c>
+      <c r="B90" s="47" t="inlineStr">
+        <is>
+          <t>Connectors</t>
+        </is>
+      </c>
+      <c r="C90" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D90" s="60" t="n">
+        <v>2</v>
+      </c>
+      <c r="E90" s="61" t="n">
+        <v>10</v>
+      </c>
+      <c r="F90" s="61" t="n">
+        <v>20</v>
+      </c>
+      <c r="G90" s="47" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="50" t="inlineStr">
+        <is>
+          <t>subtotal laskakit.cz</t>
+        </is>
+      </c>
+      <c r="B91" s="51" t="n"/>
+      <c r="C91" s="51" t="n"/>
+      <c r="D91" s="51" t="n"/>
+      <c r="E91" s="51" t="n"/>
+      <c r="F91" s="15" t="n">
+        <v>32</v>
+      </c>
+      <c r="G91" s="51" t="n"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="45" t="inlineStr">
+        <is>
+          <t>neven.cz</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="59" t="inlineStr">
+        <is>
+          <t>G04</t>
+        </is>
+      </c>
+      <c r="B94" s="47" t="inlineStr">
+        <is>
+          <t>Antenna probe</t>
+        </is>
+      </c>
+      <c r="C94" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D94" s="60" t="n">
+        <v>2</v>
+      </c>
+      <c r="E94" s="61" t="n">
+        <v>6</v>
+      </c>
+      <c r="F94" s="61" t="n">
+        <v>12</v>
+      </c>
+      <c r="G94" s="47" t="inlineStr">
+        <is>
+          <t>149 CZK</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="50" t="inlineStr">
+        <is>
+          <t>subtotal neven.cz</t>
+        </is>
+      </c>
+      <c r="B95" s="51" t="n"/>
+      <c r="C95" s="51" t="n"/>
+      <c r="D95" s="51" t="n"/>
+      <c r="E95" s="51" t="n"/>
+      <c r="F95" s="15" t="n">
+        <v>12</v>
+      </c>
+      <c r="G95" s="51" t="n"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="45" t="inlineStr">
+        <is>
+          <t>nerezmaterial.cz</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="59" t="inlineStr">
+        <is>
+          <t>A03</t>
+        </is>
+      </c>
+      <c r="B98" s="47" t="inlineStr">
+        <is>
+          <t>Wet shaft</t>
+        </is>
+      </c>
+      <c r="C98" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D98" s="60" t="n">
+        <v>3</v>
+      </c>
+      <c r="E98" s="61" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="F98" s="61" t="n">
+        <v>7.800000000000001</v>
+      </c>
+      <c r="G98" s="47" t="inlineStr">
+        <is>
+          <t>3m bar 63.1 CZK makes ~26 shafts</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="59" t="inlineStr">
+        <is>
+          <t>A05</t>
+        </is>
+      </c>
+      <c r="B99" s="47" t="inlineStr">
+        <is>
+          <t>Bearing carrier tube</t>
+        </is>
+      </c>
+      <c r="C99" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D99" s="60" t="n">
+        <v>3</v>
+      </c>
+      <c r="E99" s="61" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="F99" s="61" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="G99" s="47" t="inlineStr">
+        <is>
+          <t>cut from Ø12 bar stock</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="59" t="inlineStr">
+        <is>
+          <t>B03</t>
+        </is>
+      </c>
+      <c r="B100" s="47" t="inlineStr">
+        <is>
+          <t>Separation wall</t>
+        </is>
+      </c>
+      <c r="C100" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D100" s="60" t="n">
+        <v>3</v>
+      </c>
+      <c r="E100" s="61" t="n">
+        <v>0</v>
+      </c>
+      <c r="F100" s="61" t="n">
+        <v>0</v>
+      </c>
+      <c r="G100" s="47" t="inlineStr">
+        <is>
+          <t>MUST be solid 5mm; no penetration</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="50" t="inlineStr">
+        <is>
+          <t>subtotal nerezmaterial.cz</t>
+        </is>
+      </c>
+      <c r="B101" s="51" t="n"/>
+      <c r="C101" s="51" t="n"/>
+      <c r="D101" s="51" t="n"/>
+      <c r="E101" s="51" t="n"/>
+      <c r="F101" s="15" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="G101" s="51" t="n"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="45" t="inlineStr">
+        <is>
+          <t>JLCPCB</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="59" t="inlineStr">
+        <is>
+          <t>G14</t>
+        </is>
+      </c>
+      <c r="B104" s="47" t="inlineStr">
+        <is>
+          <t>PCB</t>
+        </is>
+      </c>
+      <c r="C104" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D104" s="60" t="n">
+        <v>3</v>
+      </c>
+      <c r="E104" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="F104" s="61" t="n">
+        <v>9</v>
+      </c>
+      <c r="G104" s="47" t="inlineStr">
+        <is>
+          <t>panel of 10 amortises</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="50" t="inlineStr">
+        <is>
+          <t>subtotal JLCPCB</t>
+        </is>
+      </c>
+      <c r="B105" s="51" t="n"/>
+      <c r="C105" s="51" t="n"/>
+      <c r="D105" s="51" t="n"/>
+      <c r="E105" s="51" t="n"/>
+      <c r="F105" s="15" t="n">
+        <v>9</v>
+      </c>
+      <c r="G105" s="51" t="n"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="45" t="inlineStr">
+        <is>
+          <t>magsy.sk</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="59" t="inlineStr">
+        <is>
+          <t>B01</t>
+        </is>
+      </c>
+      <c r="B108" s="47" t="inlineStr">
+        <is>
+          <t>Magnet</t>
+        </is>
+      </c>
+      <c r="C108" s="59" t="n">
+        <v>16</v>
+      </c>
+      <c r="D108" s="60" t="n">
+        <v>18</v>
+      </c>
+      <c r="E108" s="61" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F108" s="61" t="n">
+        <v>5.399999999999999</v>
+      </c>
+      <c r="G108" s="47" t="inlineStr">
+        <is>
+          <t>~0.30 EUR at 51+ pcs canned; bare N52 must not touch water</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="50" t="inlineStr">
+        <is>
+          <t>subtotal magsy.sk</t>
+        </is>
+      </c>
+      <c r="B109" s="51" t="n"/>
+      <c r="C109" s="51" t="n"/>
+      <c r="D109" s="51" t="n"/>
+      <c r="E109" s="51" t="n"/>
+      <c r="F109" s="15" t="n">
+        <v>5.399999999999999</v>
+      </c>
+      <c r="G109" s="51" t="n"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="54" t="inlineStr">
+        <is>
+          <t>OPTIONAL / RECOMMENDED add-ons - order only if budget allows</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="45" t="inlineStr">
+        <is>
+          <t>TME</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="59" t="inlineStr">
+        <is>
+          <t>D05</t>
+        </is>
+      </c>
+      <c r="B113" s="47" t="inlineStr">
+        <is>
+          <t>Level / stage probe</t>
+        </is>
+      </c>
+      <c r="C113" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D113" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="E113" s="61" t="n">
+        <v>110</v>
+      </c>
+      <c r="F113" s="61" t="n">
+        <v>110</v>
+      </c>
+      <c r="G113" s="47" t="inlineStr">
+        <is>
+          <t>MS5837-30BA REJECTED: gel element must be dried daily, 24h max submers</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="59" t="inlineStr">
+        <is>
+          <t>H12</t>
+        </is>
+      </c>
+      <c r="B114" s="47" t="inlineStr">
+        <is>
+          <t>Security fastener</t>
+        </is>
+      </c>
+      <c r="C114" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D114" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="E114" s="61" t="n">
+        <v>4</v>
+      </c>
+      <c r="F114" s="61" t="n">
+        <v>4</v>
+      </c>
+      <c r="G114" s="47" t="inlineStr">
+        <is>
+          <t>anti-theft</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="59" t="inlineStr">
+        <is>
+          <t>K01</t>
+        </is>
+      </c>
+      <c r="B115" s="47" t="inlineStr">
+        <is>
+          <t>Vacuum chamber</t>
+        </is>
+      </c>
+      <c r="C115" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D115" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="E115" s="61" t="n">
+        <v>85</v>
+      </c>
+      <c r="F115" s="61" t="n">
+        <v>85</v>
+      </c>
+      <c r="G115" s="47" t="inlineStr">
+        <is>
+          <t>acceptance test rig (one-off)</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="59" t="inlineStr">
+        <is>
+          <t>K02</t>
+        </is>
+      </c>
+      <c r="B116" s="47" t="inlineStr">
+        <is>
+          <t>Torque driver</t>
+        </is>
+      </c>
+      <c r="C116" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D116" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="E116" s="61" t="n">
+        <v>40</v>
+      </c>
+      <c r="F116" s="61" t="n">
+        <v>40</v>
+      </c>
+      <c r="G116" s="47" t="inlineStr">
+        <is>
+          <t>one-off</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="50" t="inlineStr">
+        <is>
+          <t>subtotal TME</t>
+        </is>
+      </c>
+      <c r="B117" s="51" t="n"/>
+      <c r="C117" s="51" t="n"/>
+      <c r="D117" s="51" t="n"/>
+      <c r="E117" s="51" t="n"/>
+      <c r="F117" s="15" t="n">
+        <v>239</v>
+      </c>
+      <c r="G117" s="51" t="n"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="45" t="inlineStr">
+        <is>
+          <t>global-ic.sk</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="59" t="inlineStr">
+        <is>
+          <t>D09</t>
+        </is>
+      </c>
+      <c r="B120" s="47" t="inlineStr">
+        <is>
+          <t>Dissolved oxygen kit</t>
+        </is>
+      </c>
+      <c r="C120" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D120" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="E120" s="61" t="n">
+        <v>175</v>
+      </c>
+      <c r="F120" s="61" t="n">
+        <v>175</v>
+      </c>
+      <c r="G120" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HIGHEST-VALUE channel (Budca = hypoxia); membrane 1-2 months in muddy </t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="50" t="inlineStr">
+        <is>
+          <t>subtotal global-ic.sk</t>
+        </is>
+      </c>
+      <c r="B121" s="51" t="n"/>
+      <c r="C121" s="51" t="n"/>
+      <c r="D121" s="51" t="n"/>
+      <c r="E121" s="51" t="n"/>
+      <c r="F121" s="15" t="n">
+        <v>175</v>
+      </c>
+      <c r="G121" s="51" t="n"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="45" t="inlineStr">
+        <is>
+          <t>RAK reseller</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="59" t="inlineStr">
+        <is>
+          <t>I06</t>
+        </is>
+      </c>
+      <c r="B124" s="47" t="inlineStr">
+        <is>
+          <t>Concentrator upgrade (optional)</t>
+        </is>
+      </c>
+      <c r="C124" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D124" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="E124" s="61" t="n">
+        <v>145</v>
+      </c>
+      <c r="F124" s="61" t="n">
+        <v>145</v>
+      </c>
+      <c r="G124" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Only for multi-SF / multi-channel / public TTN. Single-channel Wio-E5 </t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="50" t="inlineStr">
+        <is>
+          <t>subtotal RAK reseller</t>
+        </is>
+      </c>
+      <c r="B125" s="51" t="n"/>
+      <c r="C125" s="51" t="n"/>
+      <c r="D125" s="51" t="n"/>
+      <c r="E125" s="51" t="n"/>
+      <c r="F125" s="15" t="n">
+        <v>145</v>
+      </c>
+      <c r="G125" s="51" t="n"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="45" t="inlineStr">
+        <is>
+          <t>techfun.sk</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="59" t="inlineStr">
+        <is>
+          <t>D01</t>
+        </is>
+      </c>
+      <c r="B128" s="47" t="inlineStr">
+        <is>
+          <t>pH electrode</t>
+        </is>
+      </c>
+      <c r="C128" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D128" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="E128" s="61" t="n">
+        <v>39</v>
+      </c>
+      <c r="F128" s="61" t="n">
+        <v>39</v>
+      </c>
+      <c r="G128" s="47" t="inlineStr">
+        <is>
+          <t>OPTIONAL per site; 14-30 day service; +-0.1 pH after 2-pt cal</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="59" t="inlineStr">
+        <is>
+          <t>D02</t>
+        </is>
+      </c>
+      <c r="B129" s="47" t="inlineStr">
+        <is>
+          <t>pH spare electrode</t>
+        </is>
+      </c>
+      <c r="C129" s="59" t="n">
+        <v>2</v>
+      </c>
+      <c r="D129" s="60" t="n">
+        <v>3</v>
+      </c>
+      <c r="E129" s="61" t="n">
+        <v>9</v>
+      </c>
+      <c r="F129" s="61" t="n">
+        <v>27</v>
+      </c>
+      <c r="G129" s="47" t="inlineStr">
+        <is>
+          <t>consumable</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="59" t="inlineStr">
+        <is>
+          <t>D03</t>
+        </is>
+      </c>
+      <c r="B130" s="47" t="inlineStr">
+        <is>
+          <t>pH buffer</t>
+        </is>
+      </c>
+      <c r="C130" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D130" s="60" t="n">
+        <v>2</v>
+      </c>
+      <c r="E130" s="61" t="n">
+        <v>12</v>
+      </c>
+      <c r="F130" s="61" t="n">
+        <v>24</v>
+      </c>
+      <c r="G130" s="47" t="inlineStr">
+        <is>
+          <t>consumable</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="50" t="inlineStr">
+        <is>
+          <t>subtotal techfun.sk</t>
+        </is>
+      </c>
+      <c r="B131" s="51" t="n"/>
+      <c r="C131" s="51" t="n"/>
+      <c r="D131" s="51" t="n"/>
+      <c r="E131" s="51" t="n"/>
+      <c r="F131" s="15" t="n">
+        <v>90</v>
+      </c>
+      <c r="G131" s="51" t="n"/>
+    </row>
+    <row r="133">
+      <c r="A133" s="45" t="inlineStr">
+        <is>
+          <t>local / other</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="59" t="inlineStr">
+        <is>
+          <t>H13</t>
+        </is>
+      </c>
+      <c r="B134" s="47" t="inlineStr">
+        <is>
+          <t>Site label</t>
+        </is>
+      </c>
+      <c r="C134" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D134" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="E134" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="F134" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="G134" s="47" t="inlineStr">
+        <is>
+          <t>anti-theft by making it unsellable</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="59" t="inlineStr">
+        <is>
+          <t>K03</t>
+        </is>
+      </c>
+      <c r="B135" s="47" t="inlineStr">
+        <is>
+          <t>Spring balance</t>
+        </is>
+      </c>
+      <c r="C135" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D135" s="60" t="n">
+        <v>2</v>
+      </c>
+      <c r="E135" s="61" t="n">
+        <v>5</v>
+      </c>
+      <c r="F135" s="61" t="n">
+        <v>10</v>
+      </c>
+      <c r="G135" s="47" t="inlineStr">
+        <is>
+          <t>one-off</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="50" t="inlineStr">
+        <is>
+          <t>subtotal local / other</t>
+        </is>
+      </c>
+      <c r="B136" s="51" t="n"/>
+      <c r="C136" s="51" t="n"/>
+      <c r="D136" s="51" t="n"/>
+      <c r="E136" s="51" t="n"/>
+      <c r="F136" s="15" t="n">
+        <v>13</v>
+      </c>
+      <c r="G136" s="51" t="n"/>
+    </row>
+    <row r="138">
+      <c r="A138" s="45" t="inlineStr">
+        <is>
+          <t>Hornbach / stavebniny</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="59" t="inlineStr">
+        <is>
+          <t>H08</t>
+        </is>
+      </c>
+      <c r="B139" s="47" t="inlineStr">
+        <is>
+          <t>Yaw strut</t>
+        </is>
+      </c>
+      <c r="C139" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D139" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="E139" s="61" t="n">
+        <v>5</v>
+      </c>
+      <c r="F139" s="61" t="n">
+        <v>5</v>
+      </c>
+      <c r="G139" s="47" t="inlineStr">
+        <is>
+          <t>anti-flutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="50" t="inlineStr">
+        <is>
+          <t>subtotal Hornbach / stavebniny</t>
+        </is>
+      </c>
+      <c r="B140" s="51" t="n"/>
+      <c r="C140" s="51" t="n"/>
+      <c r="D140" s="51" t="n"/>
+      <c r="E140" s="51" t="n"/>
+      <c r="F140" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="G140" s="51" t="n"/>
+    </row>
+    <row r="142">
+      <c r="A142" s="55" t="inlineStr">
+        <is>
+          <t>optional add-ons subtotal: 667.00 EUR (DO, depth probe, pH, tools, concentrator)</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="52" t="inlineStr">
+        <is>
+          <t>GRAND TOTAL to order (required, with spares)</t>
+        </is>
+      </c>
+      <c r="F143" s="53" t="n">
+        <v>1077.62</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="42">
+    <mergeCell ref="A97:G97"/>
+    <mergeCell ref="A82:E82"/>
+    <mergeCell ref="A4:G4"/>
+    <mergeCell ref="A45:E45"/>
+    <mergeCell ref="A61:E61"/>
+    <mergeCell ref="A112:G112"/>
+    <mergeCell ref="A63:G63"/>
+    <mergeCell ref="A93:G93"/>
+    <mergeCell ref="A111:G111"/>
+    <mergeCell ref="A69:E69"/>
+    <mergeCell ref="A78:E78"/>
+    <mergeCell ref="A127:G127"/>
+    <mergeCell ref="A39:G39"/>
+    <mergeCell ref="A37:E37"/>
+    <mergeCell ref="A142:G142"/>
+    <mergeCell ref="A74:E74"/>
+    <mergeCell ref="A138:G138"/>
+    <mergeCell ref="A107:G107"/>
+    <mergeCell ref="A103:G103"/>
+    <mergeCell ref="A136:E136"/>
+    <mergeCell ref="A105:E105"/>
+    <mergeCell ref="A123:G123"/>
+    <mergeCell ref="A143:E143"/>
+    <mergeCell ref="A119:G119"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A88:G88"/>
+    <mergeCell ref="A95:E95"/>
+    <mergeCell ref="A101:E101"/>
+    <mergeCell ref="A86:E86"/>
+    <mergeCell ref="A133:G133"/>
+    <mergeCell ref="A84:G84"/>
+    <mergeCell ref="A91:E91"/>
+    <mergeCell ref="A109:E109"/>
+    <mergeCell ref="A131:E131"/>
+    <mergeCell ref="A140:E140"/>
+    <mergeCell ref="A80:G80"/>
+    <mergeCell ref="A125:E125"/>
+    <mergeCell ref="A121:E121"/>
+    <mergeCell ref="A117:E117"/>
+    <mergeCell ref="A76:G76"/>
+    <mergeCell ref="A71:G71"/>
+    <mergeCell ref="A47:G47"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:D29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>

<commit_message>
repo: tidy - generated meshes and caches out of git, legacy SCAD/renders/FreeCAD tools to archive/, docs reorganised, firmware/ merged, README rewritten. cad: coupling wall is its own part, blade rebuilt as a real propeller (chord was along the shaft)
</commit_message>
<xml_diff>
--- a/docs/sub-mission_parts.xlsx
+++ b/docs/sub-mission_parts.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Parts list" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Order (by shop)" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Summary" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parts list" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Order (by shop)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Parts list'!$A$4:$L$124</definedName>
@@ -226,7 +226,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -343,6 +343,9 @@
     <xf numFmtId="164" fontId="14" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="15" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -5793,7 +5796,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="59" t="inlineStr">
+      <c r="A5" s="62" t="inlineStr">
         <is>
           <t>A04</t>
         </is>
@@ -5803,16 +5806,16 @@
           <t>Wet bearing</t>
         </is>
       </c>
-      <c r="C5" s="59" t="n">
+      <c r="C5" s="62" t="n">
         <v>2</v>
       </c>
-      <c r="D5" s="60" t="n">
+      <c r="D5" s="63" t="n">
         <v>4</v>
       </c>
-      <c r="E5" s="61" t="n">
+      <c r="E5" s="64" t="n">
         <v>1.18</v>
       </c>
-      <c r="F5" s="61" t="n">
+      <c r="F5" s="64" t="n">
         <v>4.72</v>
       </c>
       <c r="G5" s="47" t="inlineStr">
@@ -5822,7 +5825,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="59" t="inlineStr">
+      <c r="A6" s="62" t="inlineStr">
         <is>
           <t>A06</t>
         </is>
@@ -5832,22 +5835,22 @@
           <t>Set screw</t>
         </is>
       </c>
-      <c r="C6" s="59" t="n">
+      <c r="C6" s="62" t="n">
         <v>2</v>
       </c>
-      <c r="D6" s="60" t="n">
+      <c r="D6" s="63" t="n">
         <v>4</v>
       </c>
-      <c r="E6" s="61" t="n">
-        <v>1</v>
-      </c>
-      <c r="F6" s="61" t="n">
+      <c r="E6" s="64" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" s="64" t="n">
         <v>4</v>
       </c>
       <c r="G6" s="47" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="59" t="inlineStr">
+      <c r="A7" s="62" t="inlineStr">
         <is>
           <t>C03</t>
         </is>
@@ -5857,16 +5860,16 @@
           <t>Pod O-ring</t>
         </is>
       </c>
-      <c r="C7" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D7" s="60" t="n">
+      <c r="C7" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" s="63" t="n">
         <v>3</v>
       </c>
-      <c r="E7" s="61" t="n">
+      <c r="E7" s="64" t="n">
         <v>3</v>
       </c>
-      <c r="F7" s="61" t="n">
+      <c r="F7" s="64" t="n">
         <v>9</v>
       </c>
       <c r="G7" s="47" t="inlineStr">
@@ -5876,7 +5879,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="59" t="inlineStr">
+      <c r="A8" s="62" t="inlineStr">
         <is>
           <t>C05</t>
         </is>
@@ -5886,22 +5889,22 @@
           <t>Pod clamp screws</t>
         </is>
       </c>
-      <c r="C8" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D8" s="60" t="n">
+      <c r="C8" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="63" t="n">
         <v>3</v>
       </c>
-      <c r="E8" s="61" t="n">
+      <c r="E8" s="64" t="n">
         <v>3</v>
       </c>
-      <c r="F8" s="61" t="n">
+      <c r="F8" s="64" t="n">
         <v>9</v>
       </c>
       <c r="G8" s="47" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="59" t="inlineStr">
+      <c r="A9" s="62" t="inlineStr">
         <is>
           <t>C07</t>
         </is>
@@ -5911,16 +5914,16 @@
           <t>Cable gland wet side</t>
         </is>
       </c>
-      <c r="C9" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D9" s="60" t="n">
+      <c r="C9" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="63" t="n">
         <v>2</v>
       </c>
-      <c r="E9" s="61" t="n">
+      <c r="E9" s="64" t="n">
         <v>12</v>
       </c>
-      <c r="F9" s="61" t="n">
+      <c r="F9" s="64" t="n">
         <v>24</v>
       </c>
       <c r="G9" s="47" t="inlineStr">
@@ -5930,7 +5933,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="59" t="inlineStr">
+      <c r="A10" s="62" t="inlineStr">
         <is>
           <t>C09</t>
         </is>
@@ -5940,22 +5943,22 @@
           <t>Generator mount</t>
         </is>
       </c>
-      <c r="C10" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D10" s="60" t="n">
+      <c r="C10" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" s="63" t="n">
         <v>3</v>
       </c>
-      <c r="E10" s="61" t="n">
-        <v>1</v>
-      </c>
-      <c r="F10" s="61" t="n">
+      <c r="E10" s="64" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" s="64" t="n">
         <v>3</v>
       </c>
       <c r="G10" s="47" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="59" t="inlineStr">
+      <c r="A11" s="62" t="inlineStr">
         <is>
           <t>D06</t>
         </is>
@@ -5965,16 +5968,16 @@
           <t>EC/TDS</t>
         </is>
       </c>
-      <c r="C11" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D11" s="60" t="n">
+      <c r="C11" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" s="63" t="n">
         <v>2</v>
       </c>
-      <c r="E11" s="61" t="n">
+      <c r="E11" s="64" t="n">
         <v>14</v>
       </c>
-      <c r="F11" s="61" t="n">
+      <c r="F11" s="64" t="n">
         <v>28</v>
       </c>
       <c r="G11" s="47" t="inlineStr">
@@ -5984,7 +5987,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="59" t="inlineStr">
+      <c r="A12" s="62" t="inlineStr">
         <is>
           <t>D08</t>
         </is>
@@ -5994,22 +5997,22 @@
           <t>Sensor cable</t>
         </is>
       </c>
-      <c r="C12" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D12" s="60" t="n">
+      <c r="C12" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" s="63" t="n">
         <v>2</v>
       </c>
-      <c r="E12" s="61" t="n">
+      <c r="E12" s="64" t="n">
         <v>20</v>
       </c>
-      <c r="F12" s="61" t="n">
+      <c r="F12" s="64" t="n">
         <v>40</v>
       </c>
       <c r="G12" s="47" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="59" t="inlineStr">
+      <c r="A13" s="62" t="inlineStr">
         <is>
           <t>E02</t>
         </is>
@@ -6019,22 +6022,22 @@
           <t>Cage fasteners</t>
         </is>
       </c>
-      <c r="C13" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D13" s="60" t="n">
+      <c r="C13" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" s="63" t="n">
         <v>2</v>
       </c>
-      <c r="E13" s="61" t="n">
+      <c r="E13" s="64" t="n">
         <v>6</v>
       </c>
-      <c r="F13" s="61" t="n">
+      <c r="F13" s="64" t="n">
         <v>12</v>
       </c>
       <c r="G13" s="47" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="59" t="inlineStr">
+      <c r="A14" s="62" t="inlineStr">
         <is>
           <t>F01</t>
         </is>
@@ -6044,22 +6047,22 @@
           <t>Cable</t>
         </is>
       </c>
-      <c r="C14" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D14" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="E14" s="61" t="n">
+      <c r="C14" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="64" t="n">
         <v>35</v>
       </c>
-      <c r="F14" s="61" t="n">
+      <c r="F14" s="64" t="n">
         <v>35</v>
       </c>
       <c r="G14" s="47" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="59" t="inlineStr">
+      <c r="A15" s="62" t="inlineStr">
         <is>
           <t>F02</t>
         </is>
@@ -6069,16 +6072,16 @@
           <t>Bulkhead connector</t>
         </is>
       </c>
-      <c r="C15" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D15" s="60" t="n">
+      <c r="C15" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" s="63" t="n">
         <v>2</v>
       </c>
-      <c r="E15" s="61" t="n">
+      <c r="E15" s="64" t="n">
         <v>12</v>
       </c>
-      <c r="F15" s="61" t="n">
+      <c r="F15" s="64" t="n">
         <v>24</v>
       </c>
       <c r="G15" s="47" t="inlineStr">
@@ -6088,7 +6091,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="59" t="inlineStr">
+      <c r="A16" s="62" t="inlineStr">
         <is>
           <t>G01</t>
         </is>
@@ -6098,16 +6101,16 @@
           <t>Enclosure</t>
         </is>
       </c>
-      <c r="C16" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D16" s="60" t="n">
+      <c r="C16" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" s="63" t="n">
         <v>2</v>
       </c>
-      <c r="E16" s="61" t="n">
+      <c r="E16" s="64" t="n">
         <v>22</v>
       </c>
-      <c r="F16" s="61" t="n">
+      <c r="F16" s="64" t="n">
         <v>44</v>
       </c>
       <c r="G16" s="47" t="inlineStr">
@@ -6117,7 +6120,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="59" t="inlineStr">
+      <c r="A17" s="62" t="inlineStr">
         <is>
           <t>G05</t>
         </is>
@@ -6127,16 +6130,16 @@
           <t>Antenna pigtail</t>
         </is>
       </c>
-      <c r="C17" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D17" s="60" t="n">
+      <c r="C17" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" s="63" t="n">
         <v>3</v>
       </c>
-      <c r="E17" s="61" t="n">
+      <c r="E17" s="64" t="n">
         <v>3</v>
       </c>
-      <c r="F17" s="61" t="n">
+      <c r="F17" s="64" t="n">
         <v>9</v>
       </c>
       <c r="G17" s="47" t="inlineStr">
@@ -6146,7 +6149,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="59" t="inlineStr">
+      <c r="A18" s="62" t="inlineStr">
         <is>
           <t>G06</t>
         </is>
@@ -6156,16 +6159,16 @@
           <t>Boost harvester</t>
         </is>
       </c>
-      <c r="C18" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D18" s="60" t="n">
+      <c r="C18" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" s="63" t="n">
         <v>2</v>
       </c>
-      <c r="E18" s="61" t="n">
+      <c r="E18" s="64" t="n">
         <v>5</v>
       </c>
-      <c r="F18" s="61" t="n">
+      <c r="F18" s="64" t="n">
         <v>10</v>
       </c>
       <c r="G18" s="47" t="inlineStr">
@@ -6175,7 +6178,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="59" t="inlineStr">
+      <c r="A19" s="62" t="inlineStr">
         <is>
           <t>G07</t>
         </is>
@@ -6185,22 +6188,22 @@
           <t>Buck</t>
         </is>
       </c>
-      <c r="C19" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D19" s="60" t="n">
+      <c r="C19" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" s="63" t="n">
         <v>3</v>
       </c>
-      <c r="E19" s="61" t="n">
+      <c r="E19" s="64" t="n">
         <v>2.5</v>
       </c>
-      <c r="F19" s="61" t="n">
+      <c r="F19" s="64" t="n">
         <v>7.5</v>
       </c>
       <c r="G19" s="47" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="59" t="inlineStr">
+      <c r="A20" s="62" t="inlineStr">
         <is>
           <t>G08</t>
         </is>
@@ -6210,16 +6213,16 @@
           <t>Rectifier</t>
         </is>
       </c>
-      <c r="C20" s="59" t="n">
+      <c r="C20" s="62" t="n">
         <v>6</v>
       </c>
-      <c r="D20" s="60" t="n">
+      <c r="D20" s="63" t="n">
         <v>8</v>
       </c>
-      <c r="E20" s="61" t="n">
+      <c r="E20" s="64" t="n">
         <v>0.15</v>
       </c>
-      <c r="F20" s="61" t="n">
+      <c r="F20" s="64" t="n">
         <v>1.2</v>
       </c>
       <c r="G20" s="47" t="inlineStr">
@@ -6229,7 +6232,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="59" t="inlineStr">
+      <c r="A21" s="62" t="inlineStr">
         <is>
           <t>G09</t>
         </is>
@@ -6239,16 +6242,16 @@
           <t>Clamp</t>
         </is>
       </c>
-      <c r="C21" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D21" s="60" t="n">
+      <c r="C21" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" s="63" t="n">
         <v>3</v>
       </c>
-      <c r="E21" s="61" t="n">
+      <c r="E21" s="64" t="n">
         <v>4</v>
       </c>
-      <c r="F21" s="61" t="n">
+      <c r="F21" s="64" t="n">
         <v>12</v>
       </c>
       <c r="G21" s="47" t="inlineStr">
@@ -6258,7 +6261,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="59" t="inlineStr">
+      <c r="A22" s="62" t="inlineStr">
         <is>
           <t>G10</t>
         </is>
@@ -6268,16 +6271,16 @@
           <t>Supercap</t>
         </is>
       </c>
-      <c r="C22" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D22" s="60" t="n">
+      <c r="C22" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" s="63" t="n">
         <v>2</v>
       </c>
-      <c r="E22" s="61" t="n">
+      <c r="E22" s="64" t="n">
         <v>11</v>
       </c>
-      <c r="F22" s="61" t="n">
+      <c r="F22" s="64" t="n">
         <v>22</v>
       </c>
       <c r="G22" s="47" t="inlineStr">
@@ -6287,7 +6290,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="59" t="inlineStr">
+      <c r="A23" s="62" t="inlineStr">
         <is>
           <t>G11</t>
         </is>
@@ -6297,16 +6300,16 @@
           <t>Voltage supervisor</t>
         </is>
       </c>
-      <c r="C23" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D23" s="60" t="n">
+      <c r="C23" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" s="63" t="n">
         <v>3</v>
       </c>
-      <c r="E23" s="61" t="n">
+      <c r="E23" s="64" t="n">
         <v>1.5</v>
       </c>
-      <c r="F23" s="61" t="n">
+      <c r="F23" s="64" t="n">
         <v>4.5</v>
       </c>
       <c r="G23" s="47" t="inlineStr">
@@ -6316,7 +6319,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="59" t="inlineStr">
+      <c r="A24" s="62" t="inlineStr">
         <is>
           <t>G12</t>
         </is>
@@ -6326,16 +6329,16 @@
           <t>Load switch</t>
         </is>
       </c>
-      <c r="C24" s="59" t="n">
+      <c r="C24" s="62" t="n">
         <v>2</v>
       </c>
-      <c r="D24" s="60" t="n">
+      <c r="D24" s="63" t="n">
         <v>4</v>
       </c>
-      <c r="E24" s="61" t="n">
-        <v>1</v>
-      </c>
-      <c r="F24" s="61" t="n">
+      <c r="E24" s="64" t="n">
+        <v>1</v>
+      </c>
+      <c r="F24" s="64" t="n">
         <v>4</v>
       </c>
       <c r="G24" s="47" t="inlineStr">
@@ -6345,7 +6348,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="59" t="inlineStr">
+      <c r="A25" s="62" t="inlineStr">
         <is>
           <t>G16</t>
         </is>
@@ -6355,22 +6358,22 @@
           <t>Protection</t>
         </is>
       </c>
-      <c r="C25" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D25" s="60" t="n">
+      <c r="C25" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" s="63" t="n">
         <v>2</v>
       </c>
-      <c r="E25" s="61" t="n">
+      <c r="E25" s="64" t="n">
         <v>6</v>
       </c>
-      <c r="F25" s="61" t="n">
+      <c r="F25" s="64" t="n">
         <v>12</v>
       </c>
       <c r="G25" s="47" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="59" t="inlineStr">
+      <c r="A26" s="62" t="inlineStr">
         <is>
           <t>G17</t>
         </is>
@@ -6380,22 +6383,22 @@
           <t>Cable glands</t>
         </is>
       </c>
-      <c r="C26" s="59" t="n">
+      <c r="C26" s="62" t="n">
         <v>3</v>
       </c>
-      <c r="D26" s="60" t="n">
+      <c r="D26" s="63" t="n">
         <v>5</v>
       </c>
-      <c r="E26" s="61" t="n">
+      <c r="E26" s="64" t="n">
         <v>3</v>
       </c>
-      <c r="F26" s="61" t="n">
+      <c r="F26" s="64" t="n">
         <v>15</v>
       </c>
       <c r="G26" s="47" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="59" t="inlineStr">
+      <c r="A27" s="62" t="inlineStr">
         <is>
           <t>H06</t>
         </is>
@@ -6405,22 +6408,22 @@
           <t>Hinge collar</t>
         </is>
       </c>
-      <c r="C27" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D27" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="E27" s="61" t="n">
+      <c r="C27" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D27" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="E27" s="64" t="n">
         <v>3</v>
       </c>
-      <c r="F27" s="61" t="n">
+      <c r="F27" s="64" t="n">
         <v>3</v>
       </c>
       <c r="G27" s="47" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="59" t="inlineStr">
+      <c r="A28" s="62" t="inlineStr">
         <is>
           <t>H07</t>
         </is>
@@ -6430,16 +6433,16 @@
           <t>Shear pin</t>
         </is>
       </c>
-      <c r="C28" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D28" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="E28" s="61" t="n">
-        <v>1</v>
-      </c>
-      <c r="F28" s="61" t="n">
+      <c r="C28" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D28" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="E28" s="64" t="n">
+        <v>1</v>
+      </c>
+      <c r="F28" s="64" t="n">
         <v>1</v>
       </c>
       <c r="G28" s="47" t="inlineStr">
@@ -6449,7 +6452,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="59" t="inlineStr">
+      <c r="A29" s="62" t="inlineStr">
         <is>
           <t>H09</t>
         </is>
@@ -6459,16 +6462,16 @@
           <t>Guy line</t>
         </is>
       </c>
-      <c r="C29" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D29" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="E29" s="61" t="n">
+      <c r="C29" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D29" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" s="64" t="n">
         <v>9</v>
       </c>
-      <c r="F29" s="61" t="n">
+      <c r="F29" s="64" t="n">
         <v>9</v>
       </c>
       <c r="G29" s="47" t="inlineStr">
@@ -6478,7 +6481,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="59" t="inlineStr">
+      <c r="A30" s="62" t="inlineStr">
         <is>
           <t>H11</t>
         </is>
@@ -6488,16 +6491,16 @@
           <t>Safety cable</t>
         </is>
       </c>
-      <c r="C30" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D30" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="E30" s="61" t="n">
+      <c r="C30" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D30" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="E30" s="64" t="n">
         <v>4</v>
       </c>
-      <c r="F30" s="61" t="n">
+      <c r="F30" s="64" t="n">
         <v>4</v>
       </c>
       <c r="G30" s="47" t="inlineStr">
@@ -6507,7 +6510,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="59" t="inlineStr">
+      <c r="A31" s="62" t="inlineStr">
         <is>
           <t>I04</t>
         </is>
@@ -6517,22 +6520,22 @@
           <t>Enclosure</t>
         </is>
       </c>
-      <c r="C31" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D31" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="E31" s="61" t="n">
+      <c r="C31" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D31" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="E31" s="64" t="n">
         <v>35</v>
       </c>
-      <c r="F31" s="61" t="n">
+      <c r="F31" s="64" t="n">
         <v>35</v>
       </c>
       <c r="G31" s="47" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" s="59" t="inlineStr">
+      <c r="A32" s="62" t="inlineStr">
         <is>
           <t>J04</t>
         </is>
@@ -6542,22 +6545,22 @@
           <t>Conformal coat</t>
         </is>
       </c>
-      <c r="C32" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D32" s="60" t="n">
+      <c r="C32" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D32" s="63" t="n">
         <v>2</v>
       </c>
-      <c r="E32" s="61" t="n">
+      <c r="E32" s="64" t="n">
         <v>14</v>
       </c>
-      <c r="F32" s="61" t="n">
+      <c r="F32" s="64" t="n">
         <v>28</v>
       </c>
       <c r="G32" s="47" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" s="59" t="inlineStr">
+      <c r="A33" s="62" t="inlineStr">
         <is>
           <t>J05</t>
         </is>
@@ -6567,22 +6570,22 @@
           <t>Silicone grease</t>
         </is>
       </c>
-      <c r="C33" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D33" s="60" t="n">
+      <c r="C33" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D33" s="63" t="n">
         <v>2</v>
       </c>
-      <c r="E33" s="61" t="n">
+      <c r="E33" s="64" t="n">
         <v>9</v>
       </c>
-      <c r="F33" s="61" t="n">
+      <c r="F33" s="64" t="n">
         <v>18</v>
       </c>
       <c r="G33" s="47" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" s="59" t="inlineStr">
+      <c r="A34" s="62" t="inlineStr">
         <is>
           <t>J06</t>
         </is>
@@ -6592,22 +6595,22 @@
           <t>Threadlocker</t>
         </is>
       </c>
-      <c r="C34" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D34" s="60" t="n">
+      <c r="C34" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D34" s="63" t="n">
         <v>2</v>
       </c>
-      <c r="E34" s="61" t="n">
+      <c r="E34" s="64" t="n">
         <v>11</v>
       </c>
-      <c r="F34" s="61" t="n">
+      <c r="F34" s="64" t="n">
         <v>22</v>
       </c>
       <c r="G34" s="47" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="59" t="inlineStr">
+      <c r="A35" s="62" t="inlineStr">
         <is>
           <t>J07</t>
         </is>
@@ -6617,22 +6620,22 @@
           <t>Heat-set inserts</t>
         </is>
       </c>
-      <c r="C35" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D35" s="60" t="n">
+      <c r="C35" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D35" s="63" t="n">
         <v>2</v>
       </c>
-      <c r="E35" s="61" t="n">
+      <c r="E35" s="64" t="n">
         <v>6</v>
       </c>
-      <c r="F35" s="61" t="n">
+      <c r="F35" s="64" t="n">
         <v>12</v>
       </c>
       <c r="G35" s="47" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" s="59" t="inlineStr">
+      <c r="A36" s="62" t="inlineStr">
         <is>
           <t>J08</t>
         </is>
@@ -6642,16 +6645,16 @@
           <t>O-ring kit</t>
         </is>
       </c>
-      <c r="C36" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D36" s="60" t="n">
+      <c r="C36" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D36" s="63" t="n">
         <v>2</v>
       </c>
-      <c r="E36" s="61" t="n">
+      <c r="E36" s="64" t="n">
         <v>12</v>
       </c>
-      <c r="F36" s="61" t="n">
+      <c r="F36" s="64" t="n">
         <v>24</v>
       </c>
       <c r="G36" s="47" t="inlineStr"/>
@@ -6679,7 +6682,7 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="59" t="inlineStr">
+      <c r="A40" s="62" t="inlineStr">
         <is>
           <t>B04</t>
         </is>
@@ -6689,22 +6692,22 @@
           <t>Potting compound</t>
         </is>
       </c>
-      <c r="C40" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D40" s="60" t="n">
+      <c r="C40" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D40" s="63" t="n">
         <v>2</v>
       </c>
-      <c r="E40" s="61" t="n">
+      <c r="E40" s="64" t="n">
         <v>14</v>
       </c>
-      <c r="F40" s="61" t="n">
+      <c r="F40" s="64" t="n">
         <v>28</v>
       </c>
       <c r="G40" s="47" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" s="59" t="inlineStr">
+      <c r="A41" s="62" t="inlineStr">
         <is>
           <t>D04</t>
         </is>
@@ -6714,16 +6717,16 @@
           <t>Temperature</t>
         </is>
       </c>
-      <c r="C41" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D41" s="60" t="n">
+      <c r="C41" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D41" s="63" t="n">
         <v>2</v>
       </c>
-      <c r="E41" s="61" t="n">
+      <c r="E41" s="64" t="n">
         <v>5</v>
       </c>
-      <c r="F41" s="61" t="n">
+      <c r="F41" s="64" t="n">
         <v>10</v>
       </c>
       <c r="G41" s="47" t="inlineStr">
@@ -6733,7 +6736,7 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="59" t="inlineStr">
+      <c r="A42" s="62" t="inlineStr">
         <is>
           <t>D07</t>
         </is>
@@ -6743,16 +6746,16 @@
           <t>Turbidity</t>
         </is>
       </c>
-      <c r="C42" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D42" s="60" t="n">
+      <c r="C42" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D42" s="63" t="n">
         <v>2</v>
       </c>
-      <c r="E42" s="61" t="n">
+      <c r="E42" s="64" t="n">
         <v>12.45</v>
       </c>
-      <c r="F42" s="61" t="n">
+      <c r="F42" s="64" t="n">
         <v>24.9</v>
       </c>
       <c r="G42" s="47" t="inlineStr">
@@ -6762,7 +6765,7 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="59" t="inlineStr">
+      <c r="A43" s="62" t="inlineStr">
         <is>
           <t>G03</t>
         </is>
@@ -6772,16 +6775,16 @@
           <t>MCU + radio (single board)</t>
         </is>
       </c>
-      <c r="C43" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D43" s="60" t="n">
+      <c r="C43" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D43" s="63" t="n">
         <v>2</v>
       </c>
-      <c r="E43" s="61" t="n">
+      <c r="E43" s="64" t="n">
         <v>15</v>
       </c>
-      <c r="F43" s="61" t="n">
+      <c r="F43" s="64" t="n">
         <v>30</v>
       </c>
       <c r="G43" s="47" t="inlineStr">
@@ -6791,7 +6794,7 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="59" t="inlineStr">
+      <c r="A44" s="62" t="inlineStr">
         <is>
           <t>J03</t>
         </is>
@@ -6801,16 +6804,16 @@
           <t>Epoxy barrier</t>
         </is>
       </c>
-      <c r="C44" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D44" s="60" t="n">
+      <c r="C44" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D44" s="63" t="n">
         <v>2</v>
       </c>
-      <c r="E44" s="61" t="n">
+      <c r="E44" s="64" t="n">
         <v>18</v>
       </c>
-      <c r="F44" s="61" t="n">
+      <c r="F44" s="64" t="n">
         <v>36</v>
       </c>
       <c r="G44" s="47" t="inlineStr"/>
@@ -6838,7 +6841,7 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="59" t="inlineStr">
+      <c r="A48" s="62" t="inlineStr">
         <is>
           <t>A01</t>
         </is>
@@ -6848,16 +6851,16 @@
           <t>Blade</t>
         </is>
       </c>
-      <c r="C48" s="59" t="n">
+      <c r="C48" s="62" t="n">
         <v>3</v>
       </c>
-      <c r="D48" s="60" t="n">
+      <c r="D48" s="63" t="n">
         <v>5</v>
       </c>
-      <c r="E48" s="61" t="n">
+      <c r="E48" s="64" t="n">
         <v>0</v>
       </c>
-      <c r="F48" s="61" t="n">
+      <c r="F48" s="64" t="n">
         <v>0</v>
       </c>
       <c r="G48" s="47" t="inlineStr">
@@ -6867,7 +6870,7 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="59" t="inlineStr">
+      <c r="A49" s="62" t="inlineStr">
         <is>
           <t>A02</t>
         </is>
@@ -6877,16 +6880,16 @@
           <t>Hub</t>
         </is>
       </c>
-      <c r="C49" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D49" s="60" t="n">
+      <c r="C49" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D49" s="63" t="n">
         <v>3</v>
       </c>
-      <c r="E49" s="61" t="n">
+      <c r="E49" s="64" t="n">
         <v>0</v>
       </c>
-      <c r="F49" s="61" t="n">
+      <c r="F49" s="64" t="n">
         <v>0</v>
       </c>
       <c r="G49" s="47" t="inlineStr">
@@ -6896,7 +6899,7 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="59" t="inlineStr">
+      <c r="A50" s="62" t="inlineStr">
         <is>
           <t>A07</t>
         </is>
@@ -6906,16 +6909,16 @@
           <t>Weed guard ring</t>
         </is>
       </c>
-      <c r="C50" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D50" s="60" t="n">
+      <c r="C50" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D50" s="63" t="n">
         <v>3</v>
       </c>
-      <c r="E50" s="61" t="n">
+      <c r="E50" s="64" t="n">
         <v>0</v>
       </c>
-      <c r="F50" s="61" t="n">
+      <c r="F50" s="64" t="n">
         <v>0</v>
       </c>
       <c r="G50" s="47" t="inlineStr">
@@ -6925,7 +6928,7 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="59" t="inlineStr">
+      <c r="A51" s="62" t="inlineStr">
         <is>
           <t>B02</t>
         </is>
@@ -6935,16 +6938,16 @@
           <t>Magnet cup</t>
         </is>
       </c>
-      <c r="C51" s="59" t="n">
+      <c r="C51" s="62" t="n">
         <v>2</v>
       </c>
-      <c r="D51" s="60" t="n">
+      <c r="D51" s="63" t="n">
         <v>4</v>
       </c>
-      <c r="E51" s="61" t="n">
+      <c r="E51" s="64" t="n">
         <v>0</v>
       </c>
-      <c r="F51" s="61" t="n">
+      <c r="F51" s="64" t="n">
         <v>0</v>
       </c>
       <c r="G51" s="47" t="inlineStr">
@@ -6954,7 +6957,7 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="59" t="inlineStr">
+      <c r="A52" s="62" t="inlineStr">
         <is>
           <t>C01</t>
         </is>
@@ -6964,16 +6967,16 @@
           <t>Pod barrel</t>
         </is>
       </c>
-      <c r="C52" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D52" s="60" t="n">
+      <c r="C52" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D52" s="63" t="n">
         <v>3</v>
       </c>
-      <c r="E52" s="61" t="n">
+      <c r="E52" s="64" t="n">
         <v>0</v>
       </c>
-      <c r="F52" s="61" t="n">
+      <c r="F52" s="64" t="n">
         <v>0</v>
       </c>
       <c r="G52" s="47" t="inlineStr">
@@ -6983,7 +6986,7 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="59" t="inlineStr">
+      <c r="A53" s="62" t="inlineStr">
         <is>
           <t>C02</t>
         </is>
@@ -6993,22 +6996,22 @@
           <t>Tail cone</t>
         </is>
       </c>
-      <c r="C53" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D53" s="60" t="n">
+      <c r="C53" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D53" s="63" t="n">
         <v>3</v>
       </c>
-      <c r="E53" s="61" t="n">
+      <c r="E53" s="64" t="n">
         <v>0</v>
       </c>
-      <c r="F53" s="61" t="n">
+      <c r="F53" s="64" t="n">
         <v>0</v>
       </c>
       <c r="G53" s="47" t="inlineStr"/>
     </row>
     <row r="54">
-      <c r="A54" s="59" t="inlineStr">
+      <c r="A54" s="62" t="inlineStr">
         <is>
           <t>C04</t>
         </is>
@@ -7018,16 +7021,16 @@
           <t>O-ring groove</t>
         </is>
       </c>
-      <c r="C54" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D54" s="60" t="n">
+      <c r="C54" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D54" s="63" t="n">
         <v>3</v>
       </c>
-      <c r="E54" s="61" t="n">
+      <c r="E54" s="64" t="n">
         <v>0</v>
       </c>
-      <c r="F54" s="61" t="n">
+      <c r="F54" s="64" t="n">
         <v>0</v>
       </c>
       <c r="G54" s="47" t="inlineStr">
@@ -7037,7 +7040,7 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="59" t="inlineStr">
+      <c r="A55" s="62" t="inlineStr">
         <is>
           <t>C06</t>
         </is>
@@ -7047,16 +7050,16 @@
           <t>Desiccant</t>
         </is>
       </c>
-      <c r="C55" s="59" t="n">
+      <c r="C55" s="62" t="n">
         <v>2</v>
       </c>
-      <c r="D55" s="60" t="n">
+      <c r="D55" s="63" t="n">
         <v>4</v>
       </c>
-      <c r="E55" s="61" t="n">
+      <c r="E55" s="64" t="n">
         <v>2</v>
       </c>
-      <c r="F55" s="61" t="n">
+      <c r="F55" s="64" t="n">
         <v>8</v>
       </c>
       <c r="G55" s="47" t="inlineStr">
@@ -7066,7 +7069,7 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="59" t="inlineStr">
+      <c r="A56" s="62" t="inlineStr">
         <is>
           <t>E01</t>
         </is>
@@ -7076,16 +7079,16 @@
           <t>Sensor cage</t>
         </is>
       </c>
-      <c r="C56" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D56" s="60" t="n">
+      <c r="C56" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D56" s="63" t="n">
         <v>3</v>
       </c>
-      <c r="E56" s="61" t="n">
+      <c r="E56" s="64" t="n">
         <v>0</v>
       </c>
-      <c r="F56" s="61" t="n">
+      <c r="F56" s="64" t="n">
         <v>0</v>
       </c>
       <c r="G56" s="47" t="inlineStr">
@@ -7095,7 +7098,7 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="59" t="inlineStr">
+      <c r="A57" s="62" t="inlineStr">
         <is>
           <t>E03</t>
         </is>
@@ -7105,16 +7108,16 @@
           <t>Sensor holders</t>
         </is>
       </c>
-      <c r="C57" s="59" t="n">
+      <c r="C57" s="62" t="n">
         <v>5</v>
       </c>
-      <c r="D57" s="60" t="n">
+      <c r="D57" s="63" t="n">
         <v>7</v>
       </c>
-      <c r="E57" s="61" t="n">
+      <c r="E57" s="64" t="n">
         <v>0</v>
       </c>
-      <c r="F57" s="61" t="n">
+      <c r="F57" s="64" t="n">
         <v>0</v>
       </c>
       <c r="G57" s="47" t="inlineStr">
@@ -7124,7 +7127,7 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="59" t="inlineStr">
+      <c r="A58" s="62" t="inlineStr">
         <is>
           <t>H02</t>
         </is>
@@ -7134,16 +7137,16 @@
           <t>Pole</t>
         </is>
       </c>
-      <c r="C58" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D58" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="E58" s="61" t="n">
+      <c r="C58" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D58" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="E58" s="64" t="n">
         <v>18</v>
       </c>
-      <c r="F58" s="61" t="n">
+      <c r="F58" s="64" t="n">
         <v>18</v>
       </c>
       <c r="G58" s="47" t="inlineStr">
@@ -7153,7 +7156,7 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="59" t="inlineStr">
+      <c r="A59" s="62" t="inlineStr">
         <is>
           <t>H03</t>
         </is>
@@ -7163,16 +7166,16 @@
           <t>Receiver sleeve</t>
         </is>
       </c>
-      <c r="C59" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D59" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="E59" s="61" t="n">
+      <c r="C59" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D59" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="E59" s="64" t="n">
         <v>8</v>
       </c>
-      <c r="F59" s="61" t="n">
+      <c r="F59" s="64" t="n">
         <v>8</v>
       </c>
       <c r="G59" s="47" t="inlineStr">
@@ -7182,7 +7185,7 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="59" t="inlineStr">
+      <c r="A60" s="62" t="inlineStr">
         <is>
           <t>I02</t>
         </is>
@@ -7192,16 +7195,16 @@
           <t>Compute</t>
         </is>
       </c>
-      <c r="C60" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D60" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="E60" s="61" t="n">
+      <c r="C60" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D60" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="E60" s="64" t="n">
         <v>70</v>
       </c>
-      <c r="F60" s="61" t="n">
+      <c r="F60" s="64" t="n">
         <v>70</v>
       </c>
       <c r="G60" s="47" t="inlineStr">
@@ -7233,7 +7236,7 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="59" t="inlineStr">
+      <c r="A64" s="62" t="inlineStr">
         <is>
           <t>H01</t>
         </is>
@@ -7243,16 +7246,16 @@
           <t>Ground screw anchor</t>
         </is>
       </c>
-      <c r="C64" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D64" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="E64" s="61" t="n">
+      <c r="C64" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D64" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="E64" s="64" t="n">
         <v>25</v>
       </c>
-      <c r="F64" s="61" t="n">
+      <c r="F64" s="64" t="n">
         <v>25</v>
       </c>
       <c r="G64" s="47" t="inlineStr">
@@ -7262,7 +7265,7 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="59" t="inlineStr">
+      <c r="A65" s="62" t="inlineStr">
         <is>
           <t>H04</t>
         </is>
@@ -7272,22 +7275,22 @@
           <t>Arm tube</t>
         </is>
       </c>
-      <c r="C65" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D65" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="E65" s="61" t="n">
+      <c r="C65" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D65" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="E65" s="64" t="n">
         <v>9</v>
       </c>
-      <c r="F65" s="61" t="n">
+      <c r="F65" s="64" t="n">
         <v>9</v>
       </c>
       <c r="G65" s="47" t="inlineStr"/>
     </row>
     <row r="66">
-      <c r="A66" s="59" t="inlineStr">
+      <c r="A66" s="62" t="inlineStr">
         <is>
           <t>H05</t>
         </is>
@@ -7297,22 +7300,22 @@
           <t>Drop tube</t>
         </is>
       </c>
-      <c r="C66" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D66" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="E66" s="61" t="n">
+      <c r="C66" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D66" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="E66" s="64" t="n">
         <v>6</v>
       </c>
-      <c r="F66" s="61" t="n">
+      <c r="F66" s="64" t="n">
         <v>6</v>
       </c>
       <c r="G66" s="47" t="inlineStr"/>
     </row>
     <row r="67">
-      <c r="A67" s="59" t="inlineStr">
+      <c r="A67" s="62" t="inlineStr">
         <is>
           <t>H10</t>
         </is>
@@ -7322,22 +7325,22 @@
           <t>Guy anchor</t>
         </is>
       </c>
-      <c r="C67" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D67" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="E67" s="61" t="n">
+      <c r="C67" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D67" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="E67" s="64" t="n">
         <v>10</v>
       </c>
-      <c r="F67" s="61" t="n">
+      <c r="F67" s="64" t="n">
         <v>10</v>
       </c>
       <c r="G67" s="47" t="inlineStr"/>
     </row>
     <row r="68">
-      <c r="A68" s="59" t="inlineStr">
+      <c r="A68" s="62" t="inlineStr">
         <is>
           <t>I05</t>
         </is>
@@ -7347,16 +7350,16 @@
           <t>Mast</t>
         </is>
       </c>
-      <c r="C68" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D68" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="E68" s="61" t="n">
+      <c r="C68" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D68" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="E68" s="64" t="n">
         <v>30</v>
       </c>
-      <c r="F68" s="61" t="n">
+      <c r="F68" s="64" t="n">
         <v>30</v>
       </c>
       <c r="G68" s="47" t="inlineStr">
@@ -7388,7 +7391,7 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="59" t="inlineStr">
+      <c r="A72" s="62" t="inlineStr">
         <is>
           <t>J01</t>
         </is>
@@ -7398,22 +7401,22 @@
           <t>Filament ASA</t>
         </is>
       </c>
-      <c r="C72" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D72" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="E72" s="61" t="n">
+      <c r="C72" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D72" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="E72" s="64" t="n">
         <v>32</v>
       </c>
-      <c r="F72" s="61" t="n">
+      <c r="F72" s="64" t="n">
         <v>32</v>
       </c>
       <c r="G72" s="47" t="inlineStr"/>
     </row>
     <row r="73">
-      <c r="A73" s="59" t="inlineStr">
+      <c r="A73" s="62" t="inlineStr">
         <is>
           <t>J02</t>
         </is>
@@ -7423,16 +7426,16 @@
           <t>Filament PC Blend</t>
         </is>
       </c>
-      <c r="C73" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D73" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="E73" s="61" t="n">
+      <c r="C73" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D73" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="E73" s="64" t="n">
         <v>40</v>
       </c>
-      <c r="F73" s="61" t="n">
+      <c r="F73" s="64" t="n">
         <v>40</v>
       </c>
       <c r="G73" s="47" t="inlineStr"/>
@@ -7460,7 +7463,7 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="59" t="inlineStr">
+      <c r="A77" s="62" t="inlineStr">
         <is>
           <t>C08</t>
         </is>
@@ -7470,16 +7473,16 @@
           <t>Generator</t>
         </is>
       </c>
-      <c r="C77" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D77" s="60" t="n">
+      <c r="C77" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D77" s="63" t="n">
         <v>2</v>
       </c>
-      <c r="E77" s="61" t="n">
+      <c r="E77" s="64" t="n">
         <v>26</v>
       </c>
-      <c r="F77" s="61" t="n">
+      <c r="F77" s="64" t="n">
         <v>52</v>
       </c>
       <c r="G77" s="47" t="inlineStr">
@@ -7511,7 +7514,7 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="59" t="inlineStr">
+      <c r="A81" s="62" t="inlineStr">
         <is>
           <t>I03</t>
         </is>
@@ -7521,16 +7524,16 @@
           <t>Antenna</t>
         </is>
       </c>
-      <c r="C81" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D81" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="E81" s="61" t="n">
+      <c r="C81" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D81" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="E81" s="64" t="n">
         <v>45</v>
       </c>
-      <c r="F81" s="61" t="n">
+      <c r="F81" s="64" t="n">
         <v>45</v>
       </c>
       <c r="G81" s="47" t="inlineStr">
@@ -7562,7 +7565,7 @@
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="59" t="inlineStr">
+      <c r="A85" s="62" t="inlineStr">
         <is>
           <t>I01</t>
         </is>
@@ -7572,16 +7575,16 @@
           <t>Gateway radio (single-channel)</t>
         </is>
       </c>
-      <c r="C85" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D85" s="60" t="n">
+      <c r="C85" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D85" s="63" t="n">
         <v>2</v>
       </c>
-      <c r="E85" s="61" t="n">
+      <c r="E85" s="64" t="n">
         <v>18</v>
       </c>
-      <c r="F85" s="61" t="n">
+      <c r="F85" s="64" t="n">
         <v>36</v>
       </c>
       <c r="G85" s="47" t="inlineStr">
@@ -7613,7 +7616,7 @@
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="59" t="inlineStr">
+      <c r="A89" s="62" t="inlineStr">
         <is>
           <t>G13</t>
         </is>
@@ -7623,16 +7626,16 @@
           <t>Barometer</t>
         </is>
       </c>
-      <c r="C89" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D89" s="60" t="n">
+      <c r="C89" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D89" s="63" t="n">
         <v>2</v>
       </c>
-      <c r="E89" s="61" t="n">
+      <c r="E89" s="64" t="n">
         <v>6</v>
       </c>
-      <c r="F89" s="61" t="n">
+      <c r="F89" s="64" t="n">
         <v>12</v>
       </c>
       <c r="G89" s="47" t="inlineStr">
@@ -7642,7 +7645,7 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="59" t="inlineStr">
+      <c r="A90" s="62" t="inlineStr">
         <is>
           <t>G15</t>
         </is>
@@ -7652,16 +7655,16 @@
           <t>Connectors</t>
         </is>
       </c>
-      <c r="C90" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D90" s="60" t="n">
+      <c r="C90" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D90" s="63" t="n">
         <v>2</v>
       </c>
-      <c r="E90" s="61" t="n">
+      <c r="E90" s="64" t="n">
         <v>10</v>
       </c>
-      <c r="F90" s="61" t="n">
+      <c r="F90" s="64" t="n">
         <v>20</v>
       </c>
       <c r="G90" s="47" t="inlineStr"/>
@@ -7689,7 +7692,7 @@
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="59" t="inlineStr">
+      <c r="A94" s="62" t="inlineStr">
         <is>
           <t>G04</t>
         </is>
@@ -7699,16 +7702,16 @@
           <t>Antenna probe</t>
         </is>
       </c>
-      <c r="C94" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D94" s="60" t="n">
+      <c r="C94" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D94" s="63" t="n">
         <v>2</v>
       </c>
-      <c r="E94" s="61" t="n">
+      <c r="E94" s="64" t="n">
         <v>6</v>
       </c>
-      <c r="F94" s="61" t="n">
+      <c r="F94" s="64" t="n">
         <v>12</v>
       </c>
       <c r="G94" s="47" t="inlineStr">
@@ -7740,7 +7743,7 @@
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="59" t="inlineStr">
+      <c r="A98" s="62" t="inlineStr">
         <is>
           <t>A03</t>
         </is>
@@ -7750,16 +7753,16 @@
           <t>Wet shaft</t>
         </is>
       </c>
-      <c r="C98" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D98" s="60" t="n">
+      <c r="C98" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D98" s="63" t="n">
         <v>3</v>
       </c>
-      <c r="E98" s="61" t="n">
+      <c r="E98" s="64" t="n">
         <v>2.6</v>
       </c>
-      <c r="F98" s="61" t="n">
+      <c r="F98" s="64" t="n">
         <v>7.800000000000001</v>
       </c>
       <c r="G98" s="47" t="inlineStr">
@@ -7769,7 +7772,7 @@
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="59" t="inlineStr">
+      <c r="A99" s="62" t="inlineStr">
         <is>
           <t>A05</t>
         </is>
@@ -7779,16 +7782,16 @@
           <t>Bearing carrier tube</t>
         </is>
       </c>
-      <c r="C99" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D99" s="60" t="n">
+      <c r="C99" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D99" s="63" t="n">
         <v>3</v>
       </c>
-      <c r="E99" s="61" t="n">
+      <c r="E99" s="64" t="n">
         <v>1.2</v>
       </c>
-      <c r="F99" s="61" t="n">
+      <c r="F99" s="64" t="n">
         <v>3.6</v>
       </c>
       <c r="G99" s="47" t="inlineStr">
@@ -7798,7 +7801,7 @@
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="59" t="inlineStr">
+      <c r="A100" s="62" t="inlineStr">
         <is>
           <t>B03</t>
         </is>
@@ -7808,16 +7811,16 @@
           <t>Separation wall</t>
         </is>
       </c>
-      <c r="C100" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D100" s="60" t="n">
+      <c r="C100" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D100" s="63" t="n">
         <v>3</v>
       </c>
-      <c r="E100" s="61" t="n">
+      <c r="E100" s="64" t="n">
         <v>0</v>
       </c>
-      <c r="F100" s="61" t="n">
+      <c r="F100" s="64" t="n">
         <v>0</v>
       </c>
       <c r="G100" s="47" t="inlineStr">
@@ -7849,7 +7852,7 @@
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="59" t="inlineStr">
+      <c r="A104" s="62" t="inlineStr">
         <is>
           <t>G14</t>
         </is>
@@ -7859,16 +7862,16 @@
           <t>PCB</t>
         </is>
       </c>
-      <c r="C104" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D104" s="60" t="n">
+      <c r="C104" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D104" s="63" t="n">
         <v>3</v>
       </c>
-      <c r="E104" s="61" t="n">
+      <c r="E104" s="64" t="n">
         <v>3</v>
       </c>
-      <c r="F104" s="61" t="n">
+      <c r="F104" s="64" t="n">
         <v>9</v>
       </c>
       <c r="G104" s="47" t="inlineStr">
@@ -7900,7 +7903,7 @@
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="59" t="inlineStr">
+      <c r="A108" s="62" t="inlineStr">
         <is>
           <t>B01</t>
         </is>
@@ -7910,16 +7913,16 @@
           <t>Magnet</t>
         </is>
       </c>
-      <c r="C108" s="59" t="n">
+      <c r="C108" s="62" t="n">
         <v>16</v>
       </c>
-      <c r="D108" s="60" t="n">
+      <c r="D108" s="63" t="n">
         <v>18</v>
       </c>
-      <c r="E108" s="61" t="n">
+      <c r="E108" s="64" t="n">
         <v>0.3</v>
       </c>
-      <c r="F108" s="61" t="n">
+      <c r="F108" s="64" t="n">
         <v>5.399999999999999</v>
       </c>
       <c r="G108" s="47" t="inlineStr">
@@ -7958,7 +7961,7 @@
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="59" t="inlineStr">
+      <c r="A113" s="62" t="inlineStr">
         <is>
           <t>D05</t>
         </is>
@@ -7968,16 +7971,16 @@
           <t>Level / stage probe</t>
         </is>
       </c>
-      <c r="C113" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D113" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="E113" s="61" t="n">
+      <c r="C113" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D113" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="E113" s="64" t="n">
         <v>110</v>
       </c>
-      <c r="F113" s="61" t="n">
+      <c r="F113" s="64" t="n">
         <v>110</v>
       </c>
       <c r="G113" s="47" t="inlineStr">
@@ -7987,7 +7990,7 @@
       </c>
     </row>
     <row r="114">
-      <c r="A114" s="59" t="inlineStr">
+      <c r="A114" s="62" t="inlineStr">
         <is>
           <t>H12</t>
         </is>
@@ -7997,16 +8000,16 @@
           <t>Security fastener</t>
         </is>
       </c>
-      <c r="C114" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D114" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="E114" s="61" t="n">
+      <c r="C114" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D114" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="E114" s="64" t="n">
         <v>4</v>
       </c>
-      <c r="F114" s="61" t="n">
+      <c r="F114" s="64" t="n">
         <v>4</v>
       </c>
       <c r="G114" s="47" t="inlineStr">
@@ -8016,7 +8019,7 @@
       </c>
     </row>
     <row r="115">
-      <c r="A115" s="59" t="inlineStr">
+      <c r="A115" s="62" t="inlineStr">
         <is>
           <t>K01</t>
         </is>
@@ -8026,16 +8029,16 @@
           <t>Vacuum chamber</t>
         </is>
       </c>
-      <c r="C115" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D115" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="E115" s="61" t="n">
+      <c r="C115" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D115" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="E115" s="64" t="n">
         <v>85</v>
       </c>
-      <c r="F115" s="61" t="n">
+      <c r="F115" s="64" t="n">
         <v>85</v>
       </c>
       <c r="G115" s="47" t="inlineStr">
@@ -8045,7 +8048,7 @@
       </c>
     </row>
     <row r="116">
-      <c r="A116" s="59" t="inlineStr">
+      <c r="A116" s="62" t="inlineStr">
         <is>
           <t>K02</t>
         </is>
@@ -8055,16 +8058,16 @@
           <t>Torque driver</t>
         </is>
       </c>
-      <c r="C116" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D116" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="E116" s="61" t="n">
+      <c r="C116" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D116" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="E116" s="64" t="n">
         <v>40</v>
       </c>
-      <c r="F116" s="61" t="n">
+      <c r="F116" s="64" t="n">
         <v>40</v>
       </c>
       <c r="G116" s="47" t="inlineStr">
@@ -8096,7 +8099,7 @@
       </c>
     </row>
     <row r="120">
-      <c r="A120" s="59" t="inlineStr">
+      <c r="A120" s="62" t="inlineStr">
         <is>
           <t>D09</t>
         </is>
@@ -8106,16 +8109,16 @@
           <t>Dissolved oxygen kit</t>
         </is>
       </c>
-      <c r="C120" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D120" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="E120" s="61" t="n">
+      <c r="C120" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D120" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="E120" s="64" t="n">
         <v>175</v>
       </c>
-      <c r="F120" s="61" t="n">
+      <c r="F120" s="64" t="n">
         <v>175</v>
       </c>
       <c r="G120" s="47" t="inlineStr">
@@ -8147,7 +8150,7 @@
       </c>
     </row>
     <row r="124">
-      <c r="A124" s="59" t="inlineStr">
+      <c r="A124" s="62" t="inlineStr">
         <is>
           <t>I06</t>
         </is>
@@ -8157,16 +8160,16 @@
           <t>Concentrator upgrade (optional)</t>
         </is>
       </c>
-      <c r="C124" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D124" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="E124" s="61" t="n">
+      <c r="C124" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D124" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="E124" s="64" t="n">
         <v>145</v>
       </c>
-      <c r="F124" s="61" t="n">
+      <c r="F124" s="64" t="n">
         <v>145</v>
       </c>
       <c r="G124" s="47" t="inlineStr">
@@ -8198,7 +8201,7 @@
       </c>
     </row>
     <row r="128">
-      <c r="A128" s="59" t="inlineStr">
+      <c r="A128" s="62" t="inlineStr">
         <is>
           <t>D01</t>
         </is>
@@ -8208,16 +8211,16 @@
           <t>pH electrode</t>
         </is>
       </c>
-      <c r="C128" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D128" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="E128" s="61" t="n">
+      <c r="C128" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D128" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="E128" s="64" t="n">
         <v>39</v>
       </c>
-      <c r="F128" s="61" t="n">
+      <c r="F128" s="64" t="n">
         <v>39</v>
       </c>
       <c r="G128" s="47" t="inlineStr">
@@ -8227,7 +8230,7 @@
       </c>
     </row>
     <row r="129">
-      <c r="A129" s="59" t="inlineStr">
+      <c r="A129" s="62" t="inlineStr">
         <is>
           <t>D02</t>
         </is>
@@ -8237,16 +8240,16 @@
           <t>pH spare electrode</t>
         </is>
       </c>
-      <c r="C129" s="59" t="n">
+      <c r="C129" s="62" t="n">
         <v>2</v>
       </c>
-      <c r="D129" s="60" t="n">
+      <c r="D129" s="63" t="n">
         <v>3</v>
       </c>
-      <c r="E129" s="61" t="n">
+      <c r="E129" s="64" t="n">
         <v>9</v>
       </c>
-      <c r="F129" s="61" t="n">
+      <c r="F129" s="64" t="n">
         <v>27</v>
       </c>
       <c r="G129" s="47" t="inlineStr">
@@ -8256,7 +8259,7 @@
       </c>
     </row>
     <row r="130">
-      <c r="A130" s="59" t="inlineStr">
+      <c r="A130" s="62" t="inlineStr">
         <is>
           <t>D03</t>
         </is>
@@ -8266,16 +8269,16 @@
           <t>pH buffer</t>
         </is>
       </c>
-      <c r="C130" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D130" s="60" t="n">
+      <c r="C130" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D130" s="63" t="n">
         <v>2</v>
       </c>
-      <c r="E130" s="61" t="n">
+      <c r="E130" s="64" t="n">
         <v>12</v>
       </c>
-      <c r="F130" s="61" t="n">
+      <c r="F130" s="64" t="n">
         <v>24</v>
       </c>
       <c r="G130" s="47" t="inlineStr">
@@ -8307,7 +8310,7 @@
       </c>
     </row>
     <row r="134">
-      <c r="A134" s="59" t="inlineStr">
+      <c r="A134" s="62" t="inlineStr">
         <is>
           <t>H13</t>
         </is>
@@ -8317,16 +8320,16 @@
           <t>Site label</t>
         </is>
       </c>
-      <c r="C134" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D134" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="E134" s="61" t="n">
+      <c r="C134" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D134" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="E134" s="64" t="n">
         <v>3</v>
       </c>
-      <c r="F134" s="61" t="n">
+      <c r="F134" s="64" t="n">
         <v>3</v>
       </c>
       <c r="G134" s="47" t="inlineStr">
@@ -8336,7 +8339,7 @@
       </c>
     </row>
     <row r="135">
-      <c r="A135" s="59" t="inlineStr">
+      <c r="A135" s="62" t="inlineStr">
         <is>
           <t>K03</t>
         </is>
@@ -8346,16 +8349,16 @@
           <t>Spring balance</t>
         </is>
       </c>
-      <c r="C135" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D135" s="60" t="n">
+      <c r="C135" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D135" s="63" t="n">
         <v>2</v>
       </c>
-      <c r="E135" s="61" t="n">
+      <c r="E135" s="64" t="n">
         <v>5</v>
       </c>
-      <c r="F135" s="61" t="n">
+      <c r="F135" s="64" t="n">
         <v>10</v>
       </c>
       <c r="G135" s="47" t="inlineStr">
@@ -8387,7 +8390,7 @@
       </c>
     </row>
     <row r="139">
-      <c r="A139" s="59" t="inlineStr">
+      <c r="A139" s="62" t="inlineStr">
         <is>
           <t>H08</t>
         </is>
@@ -8397,16 +8400,16 @@
           <t>Yaw strut</t>
         </is>
       </c>
-      <c r="C139" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D139" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="E139" s="61" t="n">
+      <c r="C139" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D139" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="E139" s="64" t="n">
         <v>5</v>
       </c>
-      <c r="F139" s="61" t="n">
+      <c r="F139" s="64" t="n">
         <v>5</v>
       </c>
       <c r="G139" s="47" t="inlineStr">

</xml_diff>

<commit_message>
order: cut to a 30-minute water test in three shops
The goal changed: one dry-day dunk, 30 minutes, then a look. That deletes most
of the engineering that only pays off over a season.

- probe runs from a USB power bank in the dry box, so the whole energy chain
  goes (supercap, boost, buck, rectifier, clamp, supervisor, load switches, PCB)
- no generator: the pod carries a dummy mass, the cage carries the sensors
- no level probe (110) and no TDS for a single 30-minute dip
- sources collapsed to three online shops: TME, techfun.sk, magsy.sk. The gateway
  board and both antennas move to techfun (same Seeed board, no fourth postage).
  Local desiccant and the spring balance are town purchases, no postage.
- 4 mm stainless shaft -> an M5 A4 bolt shank, or the local metal shop
- phase 1 = 31 lines, 228.61 EUR goods, ~244 landed, well inside the 450 cap
</commit_message>
<xml_diff>
--- a/docs/sub-mission_parts.xlsx
+++ b/docs/sub-mission_parts.xlsx
@@ -269,7 +269,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="72">
+  <cellXfs count="69">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -404,15 +404,6 @@
       <alignment horizontal="right" vertical="top"/>
     </xf>
     <xf numFmtId="4" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="4" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -807,7 +798,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F125"/>
+  <dimension ref="A1:F113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -835,7 +826,7 @@
     <row r="3" ht="26" customHeight="1">
       <c r="A3" s="44" t="inlineStr">
         <is>
-          <t>44 lines      goods 408.11 EUR      shipping est. 25.00 EUR      LANDED 433.11 EUR</t>
+          <t>31 lines      goods 228.61 EUR      shipping est. 25.00 EUR      LANDED 253.61 EUR</t>
         </is>
       </c>
     </row>
@@ -846,7 +837,7 @@
         </is>
       </c>
       <c r="F5" s="46" t="n">
-        <v>156.26</v>
+        <v>115.36</v>
       </c>
     </row>
     <row r="6">
@@ -933,46 +924,46 @@
         <v>22</v>
       </c>
     </row>
-    <row r="9" ht="29" customHeight="1">
+    <row r="9" ht="15.5" customHeight="1">
       <c r="A9" s="49" t="inlineStr">
         <is>
-          <t>D06</t>
+          <t>C07</t>
         </is>
       </c>
       <c r="B9" s="49" t="inlineStr">
         <is>
-          <t>EC/TDS</t>
+          <t>Cable gland wet side</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>DFRobot SEN0244 Gravity analog TDS module + probe  -  +-10% FS is the weakest sensor; use as trend indicator, site-calibrate</t>
+          <t>Lapp Skintop MS-M 12x1.5 + Scotchcast 2131  -  NOT YET IN MODEL - add boss</t>
         </is>
       </c>
       <c r="D9" s="50" t="n">
         <v>1</v>
       </c>
       <c r="E9" s="51" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F9" s="51" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="10" ht="15.5" customHeight="1">
       <c r="A10" s="52" t="inlineStr">
         <is>
-          <t>C07</t>
+          <t>F02</t>
         </is>
       </c>
       <c r="B10" s="52" t="inlineStr">
         <is>
-          <t>Cable gland wet side</t>
+          <t>Bulkhead connector</t>
         </is>
       </c>
       <c r="C10" s="53" t="inlineStr">
         <is>
-          <t>Lapp Skintop MS-M 12x1.5 + Scotchcast 2131  -  NOT YET IN MODEL - add boss</t>
+          <t>potted gland entry (NOT SubConn)  -  cost cut from 85 EUR wet-mate</t>
         </is>
       </c>
       <c r="D10" s="54" t="n">
@@ -988,95 +979,95 @@
     <row r="11" ht="15.5" customHeight="1">
       <c r="A11" s="49" t="inlineStr">
         <is>
-          <t>F02</t>
+          <t>G17</t>
         </is>
       </c>
       <c r="B11" s="49" t="inlineStr">
         <is>
-          <t>Bulkhead connector</t>
+          <t>Cable glands</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>potted gland entry (NOT SubConn)  -  cost cut from 85 EUR wet-mate</t>
+          <t>M12 IP68 potted x3</t>
         </is>
       </c>
       <c r="D11" s="50" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E11" s="51" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="F11" s="51" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="12" ht="15.5" customHeight="1">
       <c r="A12" s="52" t="inlineStr">
         <is>
-          <t>G10</t>
+          <t>E02</t>
         </is>
       </c>
       <c r="B12" s="52" t="inlineStr">
         <is>
-          <t>Supercap</t>
+          <t>Cage fasteners</t>
         </is>
       </c>
       <c r="C12" s="53" t="inlineStr">
         <is>
-          <t>Eaton XLR-4R0507 LIC 500F 4.0V  -  NO coin-cell EDLC (50ohm ESR kills TX)</t>
+          <t>M3x10 A4 + nylok</t>
         </is>
       </c>
       <c r="D12" s="54" t="n">
         <v>1</v>
       </c>
       <c r="E12" s="55" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="F12" s="55" t="n">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="13" ht="15.5" customHeight="1">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="13" ht="29" customHeight="1">
       <c r="A13" s="49" t="inlineStr">
         <is>
-          <t>G17</t>
+          <t>G16</t>
         </is>
       </c>
       <c r="B13" s="49" t="inlineStr">
         <is>
-          <t>Cable glands</t>
+          <t>Protection</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>M12 IP68 potted x3</t>
+          <t>Fuse 0.5A + TVS + ESD array  -  NEMAM - poistka 0.5A + TVS SMBJ5.0A + ESD array (SOT-23-6)</t>
         </is>
       </c>
       <c r="D13" s="50" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E13" s="51" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F13" s="51" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="14" ht="15.5" customHeight="1">
       <c r="A14" s="52" t="inlineStr">
         <is>
-          <t>E02</t>
+          <t>J07</t>
         </is>
       </c>
       <c r="B14" s="52" t="inlineStr">
         <is>
-          <t>Cage fasteners</t>
+          <t>Heat-set inserts</t>
         </is>
       </c>
       <c r="C14" s="53" t="inlineStr">
         <is>
-          <t>M3x10 A4 + nylok</t>
+          <t>M3/M4 brass assortment</t>
         </is>
       </c>
       <c r="D14" s="54" t="n">
@@ -1092,2175 +1083,1947 @@
     <row r="15" ht="29" customHeight="1">
       <c r="A15" s="49" t="inlineStr">
         <is>
-          <t>G16</t>
+          <t>G05</t>
         </is>
       </c>
       <c r="B15" s="49" t="inlineStr">
         <is>
-          <t>Protection</t>
+          <t>Antenna pigtail</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>Fuse 0.5A + TVS + ESD array  -  NEMAM - poistka 0.5A + TVS SMBJ5.0A + ESD array (SOT-23-6)</t>
+          <t>u.FL to SMA bulkhead 15cm  -  u.FL -&gt; SMA pigtail; skip if your board ships with SMA already</t>
         </is>
       </c>
       <c r="D15" s="50" t="n">
         <v>1</v>
       </c>
       <c r="E15" s="51" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F15" s="51" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="16" ht="15.5" customHeight="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16" ht="29" customHeight="1">
       <c r="A16" s="52" t="inlineStr">
         <is>
-          <t>J07</t>
+          <t>A04</t>
         </is>
       </c>
       <c r="B16" s="52" t="inlineStr">
         <is>
-          <t>Heat-set inserts</t>
+          <t>Wet bearing</t>
         </is>
       </c>
       <c r="C16" s="53" t="inlineStr">
         <is>
-          <t>M3/M4 brass assortment</t>
+          <t>igus iglidur J plain bearing JSM-0507-05 5x7x5mm  -  83 pcs in stock; JFM-0507-05 flanged 1.48 USD alt</t>
         </is>
       </c>
       <c r="D16" s="54" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E16" s="55" t="n">
-        <v>6</v>
+        <v>1.18</v>
       </c>
       <c r="F16" s="55" t="n">
-        <v>6</v>
+        <v>2.36</v>
       </c>
     </row>
     <row r="17" ht="15.5" customHeight="1">
       <c r="A17" s="49" t="inlineStr">
         <is>
-          <t>G06</t>
+          <t>A06</t>
         </is>
       </c>
       <c r="B17" s="49" t="inlineStr">
         <is>
-          <t>Boost harvester</t>
+          <t>Set screw</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>LTC3105EFE MPPT boost  -  needed when EMF below bus</t>
+          <t>M4x8 316SS cup point ISO 4029</t>
         </is>
       </c>
       <c r="D17" s="50" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E17" s="51" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F17" s="51" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="18" ht="15.5" customHeight="1">
-      <c r="A18" s="52" t="inlineStr">
-        <is>
-          <t>G09</t>
-        </is>
-      </c>
-      <c r="B18" s="52" t="inlineStr">
-        <is>
-          <t>Clamp</t>
-        </is>
-      </c>
-      <c r="C18" s="53" t="inlineStr">
-        <is>
-          <t>TL431LIAQ + MJD127T4G + PWR263S 3.3R dump  -  overvoltage protection</t>
-        </is>
-      </c>
-      <c r="D18" s="54" t="n">
-        <v>1</v>
-      </c>
-      <c r="E18" s="55" t="n">
-        <v>4</v>
-      </c>
-      <c r="F18" s="55" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="19" ht="29" customHeight="1">
-      <c r="A19" s="49" t="inlineStr">
-        <is>
-          <t>G05</t>
-        </is>
-      </c>
-      <c r="B19" s="49" t="inlineStr">
-        <is>
-          <t>Antenna pigtail</t>
-        </is>
-      </c>
-      <c r="C19" s="6" t="inlineStr">
-        <is>
-          <t>u.FL to SMA bulkhead 15cm  -  u.FL -&gt; SMA pigtail; skip if your board ships with SMA already</t>
-        </is>
-      </c>
-      <c r="D19" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="E19" s="51" t="n">
-        <v>3</v>
-      </c>
-      <c r="F19" s="51" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="20" ht="15.5" customHeight="1">
-      <c r="A20" s="52" t="inlineStr">
-        <is>
-          <t>G07</t>
-        </is>
-      </c>
-      <c r="B20" s="52" t="inlineStr">
-        <is>
-          <t>Buck</t>
-        </is>
-      </c>
-      <c r="C20" s="53" t="inlineStr">
-        <is>
-          <t>TPS62A02DRC step-down</t>
-        </is>
-      </c>
-      <c r="D20" s="54" t="n">
-        <v>1</v>
-      </c>
-      <c r="E20" s="55" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="F20" s="55" t="n">
-        <v>2.5</v>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="45" t="inlineStr">
+        <is>
+          <t>TECHFUN.SK</t>
+        </is>
+      </c>
+      <c r="F19" s="46" t="n">
+        <v>94.45</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="47" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B20" s="47" t="inlineStr">
+        <is>
+          <t>Part</t>
+        </is>
+      </c>
+      <c r="C20" s="47" t="inlineStr">
+        <is>
+          <t>Specification / note</t>
+        </is>
+      </c>
+      <c r="D20" s="48" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="E20" s="48" t="inlineStr">
+        <is>
+          <t>Unit EUR</t>
+        </is>
+      </c>
+      <c r="F20" s="48" t="inlineStr">
+        <is>
+          <t>Total EUR</t>
+        </is>
       </c>
     </row>
     <row r="21" ht="29" customHeight="1">
       <c r="A21" s="49" t="inlineStr">
         <is>
-          <t>A04</t>
+          <t>I01</t>
         </is>
       </c>
       <c r="B21" s="49" t="inlineStr">
         <is>
-          <t>Wet bearing</t>
+          <t>Gateway radio (single-channel)</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>igus iglidur J plain bearing JSM-0507-05 5x7x5mm  -  83 pcs in stock; JFM-0507-05 flanged 1.48 USD alt</t>
+          <t>Wio-E5 mini = STM32WLE5JC + USB-C + CH340; plugs straight into RPi USB  -  druha Wio-E5 do USB na Raspberry Pi - bez nej nema kto prijimat</t>
         </is>
       </c>
       <c r="D21" s="50" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E21" s="51" t="n">
-        <v>1.18</v>
+        <v>18</v>
       </c>
       <c r="F21" s="51" t="n">
-        <v>2.36</v>
+        <v>18</v>
       </c>
     </row>
     <row r="22" ht="15.5" customHeight="1">
       <c r="A22" s="52" t="inlineStr">
         <is>
-          <t>A06</t>
+          <t>J03</t>
         </is>
       </c>
       <c r="B22" s="52" t="inlineStr">
         <is>
-          <t>Set screw</t>
+          <t>Epoxy barrier</t>
         </is>
       </c>
       <c r="C22" s="53" t="inlineStr">
         <is>
-          <t>M4x8 316SS cup point ISO 4029</t>
+          <t>West System 105 + 206</t>
         </is>
       </c>
       <c r="D22" s="54" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E22" s="55" t="n">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="F22" s="55" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="23" ht="15.5" customHeight="1">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="23" ht="42.5" customHeight="1">
       <c r="A23" s="49" t="inlineStr">
         <is>
-          <t>G12</t>
+          <t>G03</t>
         </is>
       </c>
       <c r="B23" s="49" t="inlineStr">
         <is>
-          <t>Load switch</t>
+          <t>MCU + radio (single board)</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>TPS22860 x2 for pH/EC sequencing  -  removes ground-loop need</t>
+          <t>Seeed Wio-E5 mini: STM32WLE5JC Cortex-M4 + SX126x LoRa 868 MHz, USB-C, ADC/I2C/UART/GPIO  -  does EVERYTHING in the probe: sensors + LoRa + duty cycle. u.FL/SMA antenna connector - check which, both work</t>
         </is>
       </c>
       <c r="D23" s="50" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E23" s="51" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="F23" s="51" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
     </row>
     <row r="24" ht="15.5" customHeight="1">
       <c r="A24" s="52" t="inlineStr">
         <is>
-          <t>G11</t>
+          <t>B04</t>
         </is>
       </c>
       <c r="B24" s="52" t="inlineStr">
         <is>
-          <t>Voltage supervisor</t>
+          <t>Potting compound</t>
         </is>
       </c>
       <c r="C24" s="53" t="inlineStr">
         <is>
-          <t>TLV840 nanopower  -  gates buck at 4.8V</t>
+          <t>3M Scotch-Weld DP270 black 25ml</t>
         </is>
       </c>
       <c r="D24" s="54" t="n">
         <v>1</v>
       </c>
       <c r="E24" s="55" t="n">
-        <v>1.5</v>
+        <v>14</v>
       </c>
       <c r="F24" s="55" t="n">
-        <v>1.5</v>
+        <v>14</v>
       </c>
     </row>
     <row r="25" ht="15.5" customHeight="1">
       <c r="A25" s="49" t="inlineStr">
         <is>
+          <t>D07</t>
+        </is>
+      </c>
+      <c r="B25" s="49" t="inlineStr">
+        <is>
+          <t>Turbidity</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>DFRobot SEN0189 (0-4.5V analog)  -  6 in stock; in model as sensor_turb</t>
+        </is>
+      </c>
+      <c r="D25" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" s="51" t="n">
+        <v>12.45</v>
+      </c>
+      <c r="F25" s="51" t="n">
+        <v>12.45</v>
+      </c>
+    </row>
+    <row r="26" ht="29" customHeight="1">
+      <c r="A26" s="52" t="inlineStr">
+        <is>
+          <t>G04</t>
+        </is>
+      </c>
+      <c r="B26" s="52" t="inlineStr">
+        <is>
+          <t>Antenna probe</t>
+        </is>
+      </c>
+      <c r="C26" s="53" t="inlineStr">
+        <is>
+          <t>868MHz 5dBi SMA-M omni 195mm  -  2 ks: jeden na sondu (SMA na doske), jeden na gateway</t>
+        </is>
+      </c>
+      <c r="D26" s="54" t="n">
+        <v>2</v>
+      </c>
+      <c r="E26" s="55" t="n">
+        <v>6</v>
+      </c>
+      <c r="F26" s="55" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="27" ht="15.5" customHeight="1">
+      <c r="A27" s="49" t="inlineStr">
+        <is>
+          <t>D04</t>
+        </is>
+      </c>
+      <c r="B27" s="49" t="inlineStr">
+        <is>
+          <t>Temperature</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>DS18B20 waterproof 1m cable  -  in model as sensor_ntc</t>
+        </is>
+      </c>
+      <c r="D27" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E27" s="51" t="n">
+        <v>5</v>
+      </c>
+      <c r="F27" s="51" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="29" ht="20" customHeight="1">
+      <c r="A29" s="45" t="inlineStr">
+        <is>
+          <t>LOCAL / SHOP</t>
+        </is>
+      </c>
+      <c r="F29" s="46" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="47" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B30" s="47" t="inlineStr">
+        <is>
+          <t>Part</t>
+        </is>
+      </c>
+      <c r="C30" s="47" t="inlineStr">
+        <is>
+          <t>Specification / note</t>
+        </is>
+      </c>
+      <c r="D30" s="48" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="E30" s="48" t="inlineStr">
+        <is>
+          <t>Unit EUR</t>
+        </is>
+      </c>
+      <c r="F30" s="48" t="inlineStr">
+        <is>
+          <t>Total EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="15.5" customHeight="1">
+      <c r="A31" s="49" t="inlineStr">
+        <is>
+          <t>K03</t>
+        </is>
+      </c>
+      <c r="B31" s="49" t="inlineStr">
+        <is>
+          <t>Spring balance</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="inlineStr">
+        <is>
+          <t>0-5N for coupling slip jig  -  one-off</t>
+        </is>
+      </c>
+      <c r="D31" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E31" s="51" t="n">
+        <v>5</v>
+      </c>
+      <c r="F31" s="51" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="32" ht="15.5" customHeight="1">
+      <c r="A32" s="52" t="inlineStr">
+        <is>
+          <t>C06</t>
+        </is>
+      </c>
+      <c r="B32" s="52" t="inlineStr">
+        <is>
+          <t>Desiccant</t>
+        </is>
+      </c>
+      <c r="C32" s="53" t="inlineStr">
+        <is>
+          <t>5g silica gel with indicator  -  replace at service</t>
+        </is>
+      </c>
+      <c r="D32" s="54" t="n">
+        <v>2</v>
+      </c>
+      <c r="E32" s="55" t="n">
+        <v>2</v>
+      </c>
+      <c r="F32" s="55" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="33" ht="29" customHeight="1">
+      <c r="A33" s="49" t="inlineStr">
+        <is>
+          <t>C04</t>
+        </is>
+      </c>
+      <c r="B33" s="49" t="inlineStr">
+        <is>
+          <t>O-ring groove</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="inlineStr">
+        <is>
+          <t>2.2mm wide x 1.8mm deep machined/printed into pod rim  -  NOT YET IN MODEL - add to pod</t>
+        </is>
+      </c>
+      <c r="D33" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E33" s="51" t="n">
+        <v>0</v>
+      </c>
+      <c r="F33" s="51" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" ht="20" customHeight="1">
+      <c r="A35" s="45" t="inlineStr">
+        <is>
+          <t>MAGSY.SK</t>
+        </is>
+      </c>
+      <c r="F35" s="46" t="n">
+        <v>8.800000000000001</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="47" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B36" s="47" t="inlineStr">
+        <is>
+          <t>Part</t>
+        </is>
+      </c>
+      <c r="C36" s="47" t="inlineStr">
+        <is>
+          <t>Specification / note</t>
+        </is>
+      </c>
+      <c r="D36" s="48" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="E36" s="48" t="inlineStr">
+        <is>
+          <t>Unit EUR</t>
+        </is>
+      </c>
+      <c r="F36" s="48" t="inlineStr">
+        <is>
+          <t>Total EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="42.5" customHeight="1">
+      <c r="A37" s="49" t="inlineStr">
+        <is>
+          <t>B01</t>
+        </is>
+      </c>
+      <c r="B37" s="49" t="inlineStr">
+        <is>
+          <t>Magnet</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="inlineStr">
+        <is>
+          <t>N52 D10x5 axially magnetised, canned 316L or epoxy potted  -  8 per cup, pitch r28 on D70 cup; price for D10 canned to re-verify; bare N52 must not touch water</t>
+        </is>
+      </c>
+      <c r="D37" s="50" t="n">
+        <v>16</v>
+      </c>
+      <c r="E37" s="51" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="F37" s="51" t="n">
+        <v>8.800000000000001</v>
+      </c>
+    </row>
+    <row r="39" ht="20" customHeight="1">
+      <c r="A39" s="45" t="inlineStr">
+        <is>
+          <t>PRINTED IN-HOUSE</t>
+        </is>
+      </c>
+      <c r="F39" s="46" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="47" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B40" s="47" t="inlineStr">
+        <is>
+          <t>Part</t>
+        </is>
+      </c>
+      <c r="C40" s="47" t="inlineStr">
+        <is>
+          <t>Specification / note</t>
+        </is>
+      </c>
+      <c r="D40" s="48" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="E40" s="48" t="inlineStr">
+        <is>
+          <t>Unit EUR</t>
+        </is>
+      </c>
+      <c r="F40" s="48" t="inlineStr">
+        <is>
+          <t>Total EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="15.5" customHeight="1">
+      <c r="A41" s="49" t="inlineStr">
+        <is>
+          <t>C09</t>
+        </is>
+      </c>
+      <c r="B41" s="49" t="inlineStr">
+        <is>
+          <t>Generator mount</t>
+        </is>
+      </c>
+      <c r="C41" s="6" t="inlineStr">
+        <is>
+          <t>printed cradle + 4x M3x8 A4</t>
+        </is>
+      </c>
+      <c r="D41" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E41" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="F41" s="51" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" ht="29" customHeight="1">
+      <c r="A42" s="52" t="inlineStr">
+        <is>
+          <t>A01</t>
+        </is>
+      </c>
+      <c r="B42" s="52" t="inlineStr">
+        <is>
+          <t>Blade</t>
+        </is>
+      </c>
+      <c r="C42" s="53" t="inlineStr">
+        <is>
+          <t>triple-blade rotor blade NACA4412 D220mm root pitch 28deg tip 2deg  -  ASA or ASA-CF; 6 perimeters; epoxy coat; spare blade = fuse for branch strike</t>
+        </is>
+      </c>
+      <c r="D42" s="54" t="n">
+        <v>3</v>
+      </c>
+      <c r="E42" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="F42" s="55" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" ht="29" customHeight="1">
+      <c r="A43" s="49" t="inlineStr">
+        <is>
+          <t>A02</t>
+        </is>
+      </c>
+      <c r="B43" s="49" t="inlineStr">
+        <is>
+          <t>Hub</t>
+        </is>
+      </c>
+      <c r="C43" s="6" t="inlineStr">
+        <is>
+          <t>Ø64x46mm with 2x M4 heat-set inserts and Ø5 H7 shaft bore  -  brass inserts M4 from TME</t>
+        </is>
+      </c>
+      <c r="D43" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E43" s="51" t="n">
+        <v>0</v>
+      </c>
+      <c r="F43" s="51" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" ht="29" customHeight="1">
+      <c r="A44" s="52" t="inlineStr">
+        <is>
+          <t>B02</t>
+        </is>
+      </c>
+      <c r="B44" s="52" t="inlineStr">
+        <is>
+          <t>Magnet cup</t>
+        </is>
+      </c>
+      <c r="C44" s="53" t="inlineStr">
+        <is>
+          <t>D70 rim, 8 pockets D10.2x5.2, printed ASA  -  pockets 10.2 dia (magnet 10 + 0.2 glue), 0.2 mm epoxy recess</t>
+        </is>
+      </c>
+      <c r="D44" s="54" t="n">
+        <v>2</v>
+      </c>
+      <c r="E44" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="F44" s="55" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" ht="15.5" customHeight="1">
+      <c r="A45" s="49" t="inlineStr">
+        <is>
+          <t>C01</t>
+        </is>
+      </c>
+      <c r="B45" s="49" t="inlineStr">
+        <is>
+          <t>Pod barrel</t>
+        </is>
+      </c>
+      <c r="C45" s="6" t="inlineStr">
+        <is>
+          <t>Ø110x120mm printed ASA wall 2.4mm + epoxy barrier  -  in model as pod</t>
+        </is>
+      </c>
+      <c r="D45" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E45" s="51" t="n">
+        <v>0</v>
+      </c>
+      <c r="F45" s="51" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" ht="15.5" customHeight="1">
+      <c r="A46" s="52" t="inlineStr">
+        <is>
+          <t>C02</t>
+        </is>
+      </c>
+      <c r="B46" s="52" t="inlineStr">
+        <is>
+          <t>Tail cone</t>
+        </is>
+      </c>
+      <c r="C46" s="53" t="inlineStr">
+        <is>
+          <t>printed integral</t>
+        </is>
+      </c>
+      <c r="D46" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="E46" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="F46" s="55" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" ht="15.5" customHeight="1">
+      <c r="A47" s="49" t="inlineStr">
+        <is>
+          <t>E01</t>
+        </is>
+      </c>
+      <c r="B47" s="49" t="inlineStr">
+        <is>
+          <t>Sensor cage</t>
+        </is>
+      </c>
+      <c r="C47" s="6" t="inlineStr">
+        <is>
+          <t>Ø130x150 printed ASA 12 slots  -  in model as cage</t>
+        </is>
+      </c>
+      <c r="D47" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E47" s="51" t="n">
+        <v>0</v>
+      </c>
+      <c r="F47" s="51" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" ht="29" customHeight="1">
+      <c r="A48" s="52" t="inlineStr">
+        <is>
+          <t>E03</t>
+        </is>
+      </c>
+      <c r="B48" s="52" t="inlineStr">
+        <is>
+          <t>Sensor holders</t>
+        </is>
+      </c>
+      <c r="C48" s="53" t="inlineStr">
+        <is>
+          <t>printed clips for pH/TDS/turbidity/NTC/MS5837  -  in model as sensor bodies</t>
+        </is>
+      </c>
+      <c r="D48" s="54" t="n">
+        <v>5</v>
+      </c>
+      <c r="E48" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="F48" s="55" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" ht="20" customHeight="1">
+      <c r="A50" s="45" t="inlineStr">
+        <is>
+          <t>NEREZMATERIAL.CZ</t>
+        </is>
+      </c>
+      <c r="F50" s="46" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="47" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B51" s="47" t="inlineStr">
+        <is>
+          <t>Part</t>
+        </is>
+      </c>
+      <c r="C51" s="47" t="inlineStr">
+        <is>
+          <t>Specification / note</t>
+        </is>
+      </c>
+      <c r="D51" s="48" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="E51" s="48" t="inlineStr">
+        <is>
+          <t>Unit EUR</t>
+        </is>
+      </c>
+      <c r="F51" s="48" t="inlineStr">
+        <is>
+          <t>Total EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="29" customHeight="1">
+      <c r="A52" s="49" t="inlineStr">
+        <is>
+          <t>B03</t>
+        </is>
+      </c>
+      <c r="B52" s="49" t="inlineStr">
+        <is>
+          <t>Separation wall</t>
+        </is>
+      </c>
+      <c r="C52" s="6" t="inlineStr">
+        <is>
+          <t>D106 x 4 mm - RECOMMENDED integral with the pod bulkhead (no separate part)  -  4 mm per CAD, not 5; integral removes O-ring C03 and screws C05</t>
+        </is>
+      </c>
+      <c r="D52" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E52" s="51" t="n">
+        <v>0</v>
+      </c>
+      <c r="F52" s="51" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" ht="18" customHeight="1">
+      <c r="A54" s="56" t="inlineStr">
+        <is>
+          <t>GOODS</t>
+        </is>
+      </c>
+      <c r="F54" s="57" t="n">
+        <v>228.61</v>
+      </c>
+    </row>
+    <row r="55" ht="18" customHeight="1">
+      <c r="A55" s="56" t="inlineStr">
+        <is>
+          <t>shipping, estimated</t>
+        </is>
+      </c>
+      <c r="F55" s="57" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="56" ht="22" customHeight="1">
+      <c r="A56" s="58" t="inlineStr">
+        <is>
+          <t>LANDED TOTAL</t>
+        </is>
+      </c>
+      <c r="F56" s="59" t="n">
+        <v>253.61</v>
+      </c>
+    </row>
+    <row r="59" ht="22" customHeight="1">
+      <c r="A59" s="60" t="inlineStr">
+        <is>
+          <t>NOT IN THIS ORDER</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="61" t="inlineStr">
+        <is>
+          <t>PHASE 2 - BUY LATER</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="29" customHeight="1">
+      <c r="A61" s="62" t="inlineStr">
+        <is>
+          <t>A03</t>
+        </is>
+      </c>
+      <c r="B61" s="62" t="inlineStr">
+        <is>
+          <t>Wet shaft</t>
+        </is>
+      </c>
+      <c r="C61" s="63" t="inlineStr">
+        <is>
+          <t>lokalny zeleziar / Hornbach M5 A4 srob - 4. obchod sa nerata, nema postu; 3m bar 63.1 CZK makes ~26 shafts</t>
+        </is>
+      </c>
+      <c r="E61" s="64" t="inlineStr">
+        <is>
+          <t>2.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="15.5" customHeight="1">
+      <c r="A62" s="62" t="inlineStr">
+        <is>
+          <t>C03</t>
+        </is>
+      </c>
+      <c r="B62" s="62" t="inlineStr">
+        <is>
+          <t>Pod O-ring</t>
+        </is>
+      </c>
+      <c r="C62" s="63" t="inlineStr">
+        <is>
+          <t>grease Molykote 111</t>
+        </is>
+      </c>
+      <c r="E62" s="64" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="15.5" customHeight="1">
+      <c r="A63" s="62" t="inlineStr">
+        <is>
+          <t>C05</t>
+        </is>
+      </c>
+      <c r="B63" s="62" t="inlineStr">
+        <is>
+          <t>Pod clamp screws</t>
+        </is>
+      </c>
+      <c r="C63" s="63" t="inlineStr"/>
+      <c r="E63" s="64" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="29" customHeight="1">
+      <c r="A64" s="62" t="inlineStr">
+        <is>
+          <t>C08</t>
+        </is>
+      </c>
+      <c r="B64" s="62" t="inlineStr">
+        <is>
+          <t>Generator</t>
+        </is>
+      </c>
+      <c r="C64" s="63" t="inlineStr">
+        <is>
+          <t>TEST BEZ GENERATORA: klietka + senzory stacia, generator je dalsi nakup; XTG3506 preferred: encoder = free RPM/flow</t>
+        </is>
+      </c>
+      <c r="E64" s="64" t="inlineStr">
+        <is>
+          <t>26.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="15.5" customHeight="1">
+      <c r="A65" s="62" t="inlineStr">
+        <is>
+          <t>D01</t>
+        </is>
+      </c>
+      <c r="B65" s="62" t="inlineStr">
+        <is>
+          <t>pH electrode</t>
+        </is>
+      </c>
+      <c r="C65" s="63" t="inlineStr">
+        <is>
+          <t>OPTIONAL per site; 14-30 day service; +-0.1 pH after 2-pt cal</t>
+        </is>
+      </c>
+      <c r="E65" s="64" t="inlineStr">
+        <is>
+          <t>39.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="15.5" customHeight="1">
+      <c r="A66" s="62" t="inlineStr">
+        <is>
+          <t>D02</t>
+        </is>
+      </c>
+      <c r="B66" s="62" t="inlineStr">
+        <is>
+          <t>pH spare electrode</t>
+        </is>
+      </c>
+      <c r="C66" s="63" t="inlineStr">
+        <is>
+          <t>consumable</t>
+        </is>
+      </c>
+      <c r="E66" s="64" t="inlineStr">
+        <is>
+          <t>9.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="15.5" customHeight="1">
+      <c r="A67" s="62" t="inlineStr">
+        <is>
+          <t>D03</t>
+        </is>
+      </c>
+      <c r="B67" s="62" t="inlineStr">
+        <is>
+          <t>pH buffer</t>
+        </is>
+      </c>
+      <c r="C67" s="63" t="inlineStr">
+        <is>
+          <t>consumable</t>
+        </is>
+      </c>
+      <c r="E67" s="64" t="inlineStr">
+        <is>
+          <t>12.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="29" customHeight="1">
+      <c r="A68" s="62" t="inlineStr">
+        <is>
+          <t>D09</t>
+        </is>
+      </c>
+      <c r="B68" s="62" t="inlineStr">
+        <is>
+          <t>Dissolved oxygen kit</t>
+        </is>
+      </c>
+      <c r="C68" s="63" t="inlineStr">
+        <is>
+          <t>HIGHEST-VALUE channel (Budca = hypoxia); membrane 1-2 months in muddy water; 0.5M NaOH filling solution NOT shipped by air - source locally</t>
+        </is>
+      </c>
+      <c r="E68" s="64" t="inlineStr">
+        <is>
+          <t>175.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="15.5" customHeight="1">
+      <c r="A69" s="62" t="inlineStr">
+        <is>
+          <t>D05</t>
+        </is>
+      </c>
+      <c r="B69" s="62" t="inlineStr">
+        <is>
+          <t>Level / stage probe</t>
+        </is>
+      </c>
+      <c r="C69" s="63" t="inlineStr">
+        <is>
+          <t>MS5837-30BA REJECTED: gel element must be dried daily, 24h max submersion</t>
+        </is>
+      </c>
+      <c r="E69" s="64" t="inlineStr">
+        <is>
+          <t>110.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="15.5" customHeight="1">
+      <c r="A70" s="62" t="inlineStr">
+        <is>
+          <t>D06</t>
+        </is>
+      </c>
+      <c r="B70" s="62" t="inlineStr">
+        <is>
+          <t>EC/TDS</t>
+        </is>
+      </c>
+      <c r="C70" s="63" t="inlineStr">
+        <is>
+          <t>+-10% FS is the weakest sensor; use as trend indicator, site-calibrate</t>
+        </is>
+      </c>
+      <c r="E70" s="64" t="inlineStr">
+        <is>
+          <t>14.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="15.5" customHeight="1">
+      <c r="A71" s="62" t="inlineStr">
+        <is>
+          <t>D08</t>
+        </is>
+      </c>
+      <c r="B71" s="62" t="inlineStr">
+        <is>
+          <t>Sensor cable</t>
+        </is>
+      </c>
+      <c r="C71" s="63" t="inlineStr"/>
+      <c r="E71" s="64" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="15.5" customHeight="1">
+      <c r="A72" s="62" t="inlineStr">
+        <is>
+          <t>G06</t>
+        </is>
+      </c>
+      <c r="B72" s="62" t="inlineStr">
+        <is>
+          <t>Boost harvester</t>
+        </is>
+      </c>
+      <c r="C72" s="63" t="inlineStr">
+        <is>
+          <t>needed when EMF below bus</t>
+        </is>
+      </c>
+      <c r="E72" s="64" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="15.5" customHeight="1">
+      <c r="A73" s="62" t="inlineStr">
+        <is>
+          <t>G07</t>
+        </is>
+      </c>
+      <c r="B73" s="62" t="inlineStr">
+        <is>
+          <t>Buck</t>
+        </is>
+      </c>
+      <c r="C73" s="63" t="inlineStr"/>
+      <c r="E73" s="64" t="inlineStr">
+        <is>
+          <t>2.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="15.5" customHeight="1">
+      <c r="A74" s="62" t="inlineStr">
+        <is>
           <t>G08</t>
         </is>
       </c>
-      <c r="B25" s="49" t="inlineStr">
+      <c r="B74" s="62" t="inlineStr">
         <is>
           <t>Rectifier</t>
         </is>
       </c>
-      <c r="C25" s="6" t="inlineStr">
-        <is>
-          <t>Nexperia PMEG2010AEB 20V 1A SOD-523  -  452k in stock</t>
-        </is>
-      </c>
-      <c r="D25" s="50" t="n">
-        <v>6</v>
-      </c>
-      <c r="E25" s="51" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="F25" s="51" t="n">
-        <v>0.9</v>
-      </c>
-    </row>
-    <row r="26" ht="15.5" customHeight="1">
-      <c r="A26" s="56" t="inlineStr">
+      <c r="C74" s="63" t="inlineStr">
+        <is>
+          <t>452k in stock</t>
+        </is>
+      </c>
+      <c r="E74" s="64" t="inlineStr">
+        <is>
+          <t>0.15</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="15.5" customHeight="1">
+      <c r="A75" s="62" t="inlineStr">
+        <is>
+          <t>G09</t>
+        </is>
+      </c>
+      <c r="B75" s="62" t="inlineStr">
+        <is>
+          <t>Clamp</t>
+        </is>
+      </c>
+      <c r="C75" s="63" t="inlineStr">
+        <is>
+          <t>overvoltage protection</t>
+        </is>
+      </c>
+      <c r="E75" s="64" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="15.5" customHeight="1">
+      <c r="A76" s="62" t="inlineStr">
+        <is>
+          <t>G10</t>
+        </is>
+      </c>
+      <c r="B76" s="62" t="inlineStr">
+        <is>
+          <t>Supercap</t>
+        </is>
+      </c>
+      <c r="C76" s="63" t="inlineStr">
+        <is>
+          <t>NO coin-cell EDLC (50ohm ESR kills TX)</t>
+        </is>
+      </c>
+      <c r="E76" s="64" t="inlineStr">
+        <is>
+          <t>11.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="15.5" customHeight="1">
+      <c r="A77" s="62" t="inlineStr">
+        <is>
+          <t>G11</t>
+        </is>
+      </c>
+      <c r="B77" s="62" t="inlineStr">
+        <is>
+          <t>Voltage supervisor</t>
+        </is>
+      </c>
+      <c r="C77" s="63" t="inlineStr">
+        <is>
+          <t>gates buck at 4.8V</t>
+        </is>
+      </c>
+      <c r="E77" s="64" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="15.5" customHeight="1">
+      <c r="A78" s="62" t="inlineStr">
+        <is>
+          <t>G12</t>
+        </is>
+      </c>
+      <c r="B78" s="62" t="inlineStr">
+        <is>
+          <t>Load switch</t>
+        </is>
+      </c>
+      <c r="C78" s="63" t="inlineStr">
+        <is>
+          <t>removes ground-loop need</t>
+        </is>
+      </c>
+      <c r="E78" s="64" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="15.5" customHeight="1">
+      <c r="A79" s="62" t="inlineStr">
+        <is>
+          <t>G13</t>
+        </is>
+      </c>
+      <c r="B79" s="62" t="inlineStr">
+        <is>
+          <t>Barometer</t>
+        </is>
+      </c>
+      <c r="C79" s="63" t="inlineStr">
+        <is>
+          <t>pressure reference for MS5837</t>
+        </is>
+      </c>
+      <c r="E79" s="64" t="inlineStr">
+        <is>
+          <t>6.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="15.5" customHeight="1">
+      <c r="A80" s="62" t="inlineStr">
+        <is>
+          <t>G14</t>
+        </is>
+      </c>
+      <c r="B80" s="62" t="inlineStr">
+        <is>
+          <t>PCB</t>
+        </is>
+      </c>
+      <c r="C80" s="63" t="inlineStr">
+        <is>
+          <t>panel of 10 amortises</t>
+        </is>
+      </c>
+      <c r="E80" s="64" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="15.5" customHeight="1">
+      <c r="A81" s="62" t="inlineStr">
+        <is>
+          <t>G15</t>
+        </is>
+      </c>
+      <c r="B81" s="62" t="inlineStr">
+        <is>
+          <t>Connectors</t>
+        </is>
+      </c>
+      <c r="C81" s="63" t="inlineStr"/>
+      <c r="E81" s="64" t="inlineStr">
+        <is>
+          <t>10.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="15.5" customHeight="1">
+      <c r="A82" s="62" t="inlineStr">
+        <is>
+          <t>H01</t>
+        </is>
+      </c>
+      <c r="B82" s="62" t="inlineStr">
+        <is>
+          <t>Ground screw anchor</t>
+        </is>
+      </c>
+      <c r="C82" s="63" t="inlineStr">
+        <is>
+          <t>1-2kN lateral - covers flood case</t>
+        </is>
+      </c>
+      <c r="E82" s="64" t="inlineStr">
+        <is>
+          <t>25.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="15.5" customHeight="1">
+      <c r="A83" s="62" t="inlineStr">
+        <is>
+          <t>H02</t>
+        </is>
+      </c>
+      <c r="B83" s="62" t="inlineStr">
+        <is>
+          <t>Pole</t>
+        </is>
+      </c>
+      <c r="C83" s="63" t="inlineStr">
+        <is>
+          <t>removable mast pinned into receiver</t>
+        </is>
+      </c>
+      <c r="E83" s="64" t="inlineStr">
+        <is>
+          <t>18.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="15.5" customHeight="1">
+      <c r="A84" s="62" t="inlineStr">
+        <is>
+          <t>H03</t>
+        </is>
+      </c>
+      <c r="B84" s="62" t="inlineStr">
+        <is>
+          <t>Receiver sleeve</t>
+        </is>
+      </c>
+      <c r="C84" s="63" t="inlineStr">
+        <is>
+          <t>pinned mast interface</t>
+        </is>
+      </c>
+      <c r="E84" s="64" t="inlineStr">
+        <is>
+          <t>8.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="15.5" customHeight="1">
+      <c r="A85" s="62" t="inlineStr">
+        <is>
+          <t>H04</t>
+        </is>
+      </c>
+      <c r="B85" s="62" t="inlineStr">
+        <is>
+          <t>Arm tube</t>
+        </is>
+      </c>
+      <c r="C85" s="63" t="inlineStr"/>
+      <c r="E85" s="64" t="inlineStr">
+        <is>
+          <t>9.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="15.5" customHeight="1">
+      <c r="A86" s="62" t="inlineStr">
+        <is>
+          <t>H05</t>
+        </is>
+      </c>
+      <c r="B86" s="62" t="inlineStr">
+        <is>
+          <t>Drop tube</t>
+        </is>
+      </c>
+      <c r="C86" s="63" t="inlineStr"/>
+      <c r="E86" s="64" t="inlineStr">
+        <is>
+          <t>6.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="15.5" customHeight="1">
+      <c r="A87" s="62" t="inlineStr">
+        <is>
+          <t>H06</t>
+        </is>
+      </c>
+      <c r="B87" s="62" t="inlineStr">
+        <is>
+          <t>Hinge collar</t>
+        </is>
+      </c>
+      <c r="C87" s="63" t="inlineStr"/>
+      <c r="E87" s="64" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="15.5" customHeight="1">
+      <c r="A88" s="62" t="inlineStr">
+        <is>
+          <t>H07</t>
+        </is>
+      </c>
+      <c r="B88" s="62" t="inlineStr">
+        <is>
+          <t>Shear pin</t>
+        </is>
+      </c>
+      <c r="C88" s="63" t="inlineStr">
+        <is>
+          <t>releases pod on &gt;150N debris hit</t>
+        </is>
+      </c>
+      <c r="E88" s="64" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="15.5" customHeight="1">
+      <c r="A89" s="62" t="inlineStr">
+        <is>
+          <t>H08</t>
+        </is>
+      </c>
+      <c r="B89" s="62" t="inlineStr">
+        <is>
+          <t>Yaw strut</t>
+        </is>
+      </c>
+      <c r="C89" s="63" t="inlineStr">
+        <is>
+          <t>anti-flutter</t>
+        </is>
+      </c>
+      <c r="E89" s="64" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="15.5" customHeight="1">
+      <c r="A90" s="62" t="inlineStr">
+        <is>
+          <t>H09</t>
+        </is>
+      </c>
+      <c r="B90" s="62" t="inlineStr">
+        <is>
+          <t>Guy line</t>
+        </is>
+      </c>
+      <c r="C90" s="63" t="inlineStr">
+        <is>
+          <t>45deg up/downstream</t>
+        </is>
+      </c>
+      <c r="E90" s="64" t="inlineStr">
+        <is>
+          <t>9.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="15.5" customHeight="1">
+      <c r="A91" s="62" t="inlineStr">
+        <is>
+          <t>H10</t>
+        </is>
+      </c>
+      <c r="B91" s="62" t="inlineStr">
+        <is>
+          <t>Guy anchor</t>
+        </is>
+      </c>
+      <c r="C91" s="63" t="inlineStr"/>
+      <c r="E91" s="64" t="inlineStr">
+        <is>
+          <t>10.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="15.5" customHeight="1">
+      <c r="A92" s="62" t="inlineStr">
+        <is>
+          <t>H11</t>
+        </is>
+      </c>
+      <c r="B92" s="62" t="inlineStr">
+        <is>
+          <t>Safety cable</t>
+        </is>
+      </c>
+      <c r="C92" s="63" t="inlineStr">
+        <is>
+          <t>theft/flood retention</t>
+        </is>
+      </c>
+      <c r="E92" s="64" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="15.5" customHeight="1">
+      <c r="A93" s="62" t="inlineStr">
+        <is>
+          <t>H12</t>
+        </is>
+      </c>
+      <c r="B93" s="62" t="inlineStr">
+        <is>
+          <t>Security fastener</t>
+        </is>
+      </c>
+      <c r="C93" s="63" t="inlineStr">
+        <is>
+          <t>anti-theft</t>
+        </is>
+      </c>
+      <c r="E93" s="64" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" ht="15.5" customHeight="1">
+      <c r="A94" s="62" t="inlineStr">
+        <is>
+          <t>H13</t>
+        </is>
+      </c>
+      <c r="B94" s="62" t="inlineStr">
+        <is>
+          <t>Site label</t>
+        </is>
+      </c>
+      <c r="C94" s="63" t="inlineStr">
+        <is>
+          <t>anti-theft by making it unsellable</t>
+        </is>
+      </c>
+      <c r="E94" s="64" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" ht="15.5" customHeight="1">
+      <c r="A95" s="62" t="inlineStr">
+        <is>
+          <t>I02</t>
+        </is>
+      </c>
+      <c r="B95" s="62" t="inlineStr">
+        <is>
+          <t>Compute</t>
+        </is>
+      </c>
+      <c r="C95" s="63" t="inlineStr">
+        <is>
+          <t>YOU ALREADY HAVE THIS - reuse, zero soldering; runs the gateway service</t>
+        </is>
+      </c>
+      <c r="E95" s="64" t="inlineStr">
+        <is>
+          <t>70.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="96" ht="15.5" customHeight="1">
+      <c r="A96" s="62" t="inlineStr">
+        <is>
+          <t>I03</t>
+        </is>
+      </c>
+      <c r="B96" s="62" t="inlineStr">
+        <is>
+          <t>Antenna</t>
+        </is>
+      </c>
+      <c r="C96" s="63" t="inlineStr">
+        <is>
+          <t>range-critical: gateway antenna gain + mast height set the link</t>
+        </is>
+      </c>
+      <c r="E96" s="64" t="inlineStr">
+        <is>
+          <t>45.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" ht="15.5" customHeight="1">
+      <c r="A97" s="62" t="inlineStr">
+        <is>
+          <t>I04</t>
+        </is>
+      </c>
+      <c r="B97" s="62" t="inlineStr">
+        <is>
+          <t>Enclosure</t>
+        </is>
+      </c>
+      <c r="C97" s="63" t="inlineStr"/>
+      <c r="E97" s="64" t="inlineStr">
+        <is>
+          <t>35.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="98" ht="15.5" customHeight="1">
+      <c r="A98" s="62" t="inlineStr">
+        <is>
+          <t>I05</t>
+        </is>
+      </c>
+      <c r="B98" s="62" t="inlineStr">
+        <is>
+          <t>Mast</t>
+        </is>
+      </c>
+      <c r="C98" s="63" t="inlineStr">
+        <is>
+          <t>height sets range</t>
+        </is>
+      </c>
+      <c r="E98" s="64" t="inlineStr">
+        <is>
+          <t>30.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="99" ht="15.5" customHeight="1">
+      <c r="A99" s="62" t="inlineStr">
+        <is>
+          <t>I06</t>
+        </is>
+      </c>
+      <c r="B99" s="62" t="inlineStr">
+        <is>
+          <t>Concentrator upgrade (optional)</t>
+        </is>
+      </c>
+      <c r="C99" s="63" t="inlineStr">
+        <is>
+          <t>Only for multi-SF / multi-channel / public TTN. Single-channel Wio-E5 gateway is enough for our 20 nodes.</t>
+        </is>
+      </c>
+      <c r="E99" s="64" t="inlineStr">
+        <is>
+          <t>145.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="100" ht="15.5" customHeight="1">
+      <c r="A100" s="62" t="inlineStr">
+        <is>
+          <t>J01</t>
+        </is>
+      </c>
+      <c r="B100" s="62" t="inlineStr">
+        <is>
+          <t>Filament ASA</t>
+        </is>
+      </c>
+      <c r="C100" s="63" t="inlineStr">
+        <is>
+          <t>ABS z domaceho spoolu, nie ASA; UV je len na brehu</t>
+        </is>
+      </c>
+      <c r="E100" s="64" t="inlineStr">
+        <is>
+          <t>32.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" ht="15.5" customHeight="1">
+      <c r="A101" s="62" t="inlineStr">
+        <is>
+          <t>J02</t>
+        </is>
+      </c>
+      <c r="B101" s="62" t="inlineStr">
+        <is>
+          <t>Filament PC Blend</t>
+        </is>
+      </c>
+      <c r="C101" s="63" t="inlineStr"/>
+      <c r="E101" s="64" t="inlineStr">
+        <is>
+          <t>40.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" ht="15.5" customHeight="1">
+      <c r="A102" s="62" t="inlineStr">
+        <is>
+          <t>J04</t>
+        </is>
+      </c>
+      <c r="B102" s="62" t="inlineStr">
+        <is>
+          <t>Conformal coat</t>
+        </is>
+      </c>
+      <c r="C102" s="63" t="inlineStr"/>
+      <c r="E102" s="64" t="inlineStr">
+        <is>
+          <t>14.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="103" ht="15.5" customHeight="1">
+      <c r="A103" s="62" t="inlineStr">
         <is>
           <t>J05</t>
         </is>
       </c>
-      <c r="B26" s="56" t="inlineStr">
+      <c r="B103" s="62" t="inlineStr">
         <is>
           <t>Silicone grease</t>
         </is>
       </c>
-      <c r="C26" s="17" t="inlineStr">
-        <is>
-          <t>MAM  |  Molykote 111 100g  -  MAM - doma</t>
-        </is>
-      </c>
-      <c r="D26" s="57" t="n">
-        <v>1</v>
-      </c>
-      <c r="E26" s="58" t="n">
-        <v>9</v>
-      </c>
-      <c r="F26" s="58" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" ht="20" customHeight="1">
-      <c r="A28" s="45" t="inlineStr">
-        <is>
-          <t>SENSORSONE (QUOTE)</t>
-        </is>
-      </c>
-      <c r="F28" s="46" t="n">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="47" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B29" s="47" t="inlineStr">
-        <is>
-          <t>Part</t>
-        </is>
-      </c>
-      <c r="C29" s="47" t="inlineStr">
-        <is>
-          <t>Specification / note</t>
-        </is>
-      </c>
-      <c r="D29" s="48" t="inlineStr">
-        <is>
-          <t>Qty</t>
-        </is>
-      </c>
-      <c r="E29" s="48" t="inlineStr">
-        <is>
-          <t>Unit EUR</t>
-        </is>
-      </c>
-      <c r="F29" s="48" t="inlineStr">
-        <is>
-          <t>Total EUR</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="42.5" customHeight="1">
-      <c r="A30" s="49" t="inlineStr">
-        <is>
-          <t>D05</t>
-        </is>
-      </c>
-      <c r="B30" s="49" t="inlineStr">
-        <is>
-          <t>Level / stage probe</t>
-        </is>
-      </c>
-      <c r="C30" s="6" t="inlineStr">
-        <is>
-          <t>Submersible IP68 316L, 0-1 mH2O, 0.5-4.5V out, 5m cable, permanent immersion rated  -  MS5837-30BA REJECTED: gel element must be dried daily, 24h max submersion</t>
-        </is>
-      </c>
-      <c r="D30" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="E30" s="51" t="n">
-        <v>110</v>
-      </c>
-      <c r="F30" s="51" t="n">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="32" ht="20" customHeight="1">
-      <c r="A32" s="45" t="inlineStr">
-        <is>
-          <t>TECHFUN.SK</t>
-        </is>
-      </c>
-      <c r="F32" s="46" t="n">
-        <v>64.45</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="47" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B33" s="47" t="inlineStr">
-        <is>
-          <t>Part</t>
-        </is>
-      </c>
-      <c r="C33" s="47" t="inlineStr">
-        <is>
-          <t>Specification / note</t>
-        </is>
-      </c>
-      <c r="D33" s="48" t="inlineStr">
-        <is>
-          <t>Qty</t>
-        </is>
-      </c>
-      <c r="E33" s="48" t="inlineStr">
-        <is>
-          <t>Unit EUR</t>
-        </is>
-      </c>
-      <c r="F33" s="48" t="inlineStr">
-        <is>
-          <t>Total EUR</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="15.5" customHeight="1">
-      <c r="A34" s="49" t="inlineStr">
-        <is>
-          <t>J03</t>
-        </is>
-      </c>
-      <c r="B34" s="49" t="inlineStr">
-        <is>
-          <t>Epoxy barrier</t>
-        </is>
-      </c>
-      <c r="C34" s="6" t="inlineStr">
-        <is>
-          <t>West System 105 + 206</t>
-        </is>
-      </c>
-      <c r="D34" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="E34" s="51" t="n">
-        <v>18</v>
-      </c>
-      <c r="F34" s="51" t="n">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="35" ht="42.5" customHeight="1">
-      <c r="A35" s="52" t="inlineStr">
-        <is>
-          <t>G03</t>
-        </is>
-      </c>
-      <c r="B35" s="52" t="inlineStr">
-        <is>
-          <t>MCU + radio (single board)</t>
-        </is>
-      </c>
-      <c r="C35" s="53" t="inlineStr">
-        <is>
-          <t>Seeed Wio-E5 mini: STM32WLE5JC Cortex-M4 + SX126x LoRa 868 MHz, USB-C, ADC/I2C/UART/GPIO  -  does EVERYTHING in the probe: sensors + LoRa + duty cycle. u.FL/SMA antenna connector - check which, both work</t>
-        </is>
-      </c>
-      <c r="D35" s="54" t="n">
-        <v>1</v>
-      </c>
-      <c r="E35" s="55" t="n">
-        <v>15</v>
-      </c>
-      <c r="F35" s="55" t="n">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="36" ht="15.5" customHeight="1">
-      <c r="A36" s="49" t="inlineStr">
-        <is>
-          <t>B04</t>
-        </is>
-      </c>
-      <c r="B36" s="49" t="inlineStr">
-        <is>
-          <t>Potting compound</t>
-        </is>
-      </c>
-      <c r="C36" s="6" t="inlineStr">
-        <is>
-          <t>3M Scotch-Weld DP270 black 25ml</t>
-        </is>
-      </c>
-      <c r="D36" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="E36" s="51" t="n">
-        <v>14</v>
-      </c>
-      <c r="F36" s="51" t="n">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="37" ht="15.5" customHeight="1">
-      <c r="A37" s="52" t="inlineStr">
-        <is>
-          <t>D07</t>
-        </is>
-      </c>
-      <c r="B37" s="52" t="inlineStr">
-        <is>
-          <t>Turbidity</t>
-        </is>
-      </c>
-      <c r="C37" s="53" t="inlineStr">
-        <is>
-          <t>DFRobot SEN0189 (0-4.5V analog)  -  6 in stock; in model as sensor_turb</t>
-        </is>
-      </c>
-      <c r="D37" s="54" t="n">
-        <v>1</v>
-      </c>
-      <c r="E37" s="55" t="n">
-        <v>12.45</v>
-      </c>
-      <c r="F37" s="55" t="n">
-        <v>12.45</v>
-      </c>
-    </row>
-    <row r="38" ht="15.5" customHeight="1">
-      <c r="A38" s="49" t="inlineStr">
-        <is>
-          <t>D04</t>
-        </is>
-      </c>
-      <c r="B38" s="49" t="inlineStr">
-        <is>
-          <t>Temperature</t>
-        </is>
-      </c>
-      <c r="C38" s="6" t="inlineStr">
-        <is>
-          <t>DS18B20 waterproof 1m cable  -  in model as sensor_ntc</t>
-        </is>
-      </c>
-      <c r="D38" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="E38" s="51" t="n">
-        <v>5</v>
-      </c>
-      <c r="F38" s="51" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="40" ht="20" customHeight="1">
-      <c r="A40" s="45" t="inlineStr">
-        <is>
-          <t>LOCAL / SHOP</t>
-        </is>
-      </c>
-      <c r="F40" s="46" t="n">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="47" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B41" s="47" t="inlineStr">
-        <is>
-          <t>Part</t>
-        </is>
-      </c>
-      <c r="C41" s="47" t="inlineStr">
-        <is>
-          <t>Specification / note</t>
-        </is>
-      </c>
-      <c r="D41" s="48" t="inlineStr">
-        <is>
-          <t>Qty</t>
-        </is>
-      </c>
-      <c r="E41" s="48" t="inlineStr">
-        <is>
-          <t>Unit EUR</t>
-        </is>
-      </c>
-      <c r="F41" s="48" t="inlineStr">
-        <is>
-          <t>Total EUR</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="29" customHeight="1">
-      <c r="A42" s="49" t="inlineStr">
-        <is>
-          <t>I01</t>
-        </is>
-      </c>
-      <c r="B42" s="49" t="inlineStr">
-        <is>
-          <t>Gateway radio (single-channel)</t>
-        </is>
-      </c>
-      <c r="C42" s="6" t="inlineStr">
-        <is>
-          <t>Wio-E5 mini = STM32WLE5JC + USB-C + CH340; plugs straight into RPi USB  -  druha Wio-E5 do USB na Raspberry Pi - bez nej nema kto prijimat</t>
-        </is>
-      </c>
-      <c r="D42" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="E42" s="51" t="n">
-        <v>18</v>
-      </c>
-      <c r="F42" s="51" t="n">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="43" ht="15.5" customHeight="1">
-      <c r="A43" s="52" t="inlineStr">
-        <is>
-          <t>K03</t>
-        </is>
-      </c>
-      <c r="B43" s="52" t="inlineStr">
-        <is>
-          <t>Spring balance</t>
-        </is>
-      </c>
-      <c r="C43" s="53" t="inlineStr">
-        <is>
-          <t>0-5N for coupling slip jig  -  one-off</t>
-        </is>
-      </c>
-      <c r="D43" s="54" t="n">
-        <v>1</v>
-      </c>
-      <c r="E43" s="55" t="n">
-        <v>5</v>
-      </c>
-      <c r="F43" s="55" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="44" ht="15.5" customHeight="1">
-      <c r="A44" s="49" t="inlineStr">
-        <is>
-          <t>C06</t>
-        </is>
-      </c>
-      <c r="B44" s="49" t="inlineStr">
-        <is>
-          <t>Desiccant</t>
-        </is>
-      </c>
-      <c r="C44" s="6" t="inlineStr">
-        <is>
-          <t>5g silica gel with indicator  -  replace at service</t>
-        </is>
-      </c>
-      <c r="D44" s="50" t="n">
-        <v>2</v>
-      </c>
-      <c r="E44" s="51" t="n">
-        <v>2</v>
-      </c>
-      <c r="F44" s="51" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="45" ht="29" customHeight="1">
-      <c r="A45" s="52" t="inlineStr">
-        <is>
-          <t>C04</t>
-        </is>
-      </c>
-      <c r="B45" s="52" t="inlineStr">
-        <is>
-          <t>O-ring groove</t>
-        </is>
-      </c>
-      <c r="C45" s="53" t="inlineStr">
-        <is>
-          <t>2.2mm wide x 1.8mm deep machined/printed into pod rim  -  NOT YET IN MODEL - add to pod</t>
-        </is>
-      </c>
-      <c r="D45" s="54" t="n">
-        <v>1</v>
-      </c>
-      <c r="E45" s="55" t="n">
-        <v>0</v>
-      </c>
-      <c r="F45" s="55" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47" ht="20" customHeight="1">
-      <c r="A47" s="45" t="inlineStr">
-        <is>
-          <t>X-TEAMRC.COM</t>
-        </is>
-      </c>
-      <c r="F47" s="46" t="n">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="47" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B48" s="47" t="inlineStr">
-        <is>
-          <t>Part</t>
-        </is>
-      </c>
-      <c r="C48" s="47" t="inlineStr">
-        <is>
-          <t>Specification / note</t>
-        </is>
-      </c>
-      <c r="D48" s="48" t="inlineStr">
-        <is>
-          <t>Qty</t>
-        </is>
-      </c>
-      <c r="E48" s="48" t="inlineStr">
-        <is>
-          <t>Unit EUR</t>
-        </is>
-      </c>
-      <c r="F48" s="48" t="inlineStr">
-        <is>
-          <t>Total EUR</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" ht="29" customHeight="1">
-      <c r="A49" s="49" t="inlineStr">
-        <is>
-          <t>C08</t>
-        </is>
-      </c>
-      <c r="B49" s="49" t="inlineStr">
-        <is>
-          <t>Generator</t>
-        </is>
-      </c>
-      <c r="C49" s="6" t="inlineStr">
-        <is>
-          <t>T-Motor GB2208 KV128 or X-TEAM XTG3506 (24N22P 6ohm w/ AS5048A encoder)  -  XTG3506 preferred: encoder = free RPM/flow</t>
-        </is>
-      </c>
-      <c r="D49" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="E49" s="51" t="n">
-        <v>26</v>
-      </c>
-      <c r="F49" s="51" t="n">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="51" ht="20" customHeight="1">
-      <c r="A51" s="45" t="inlineStr">
-        <is>
-          <t>NEVEN.CZ</t>
-        </is>
-      </c>
-      <c r="F51" s="46" t="n">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="47" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B52" s="47" t="inlineStr">
-        <is>
-          <t>Part</t>
-        </is>
-      </c>
-      <c r="C52" s="47" t="inlineStr">
-        <is>
-          <t>Specification / note</t>
-        </is>
-      </c>
-      <c r="D52" s="48" t="inlineStr">
-        <is>
-          <t>Qty</t>
-        </is>
-      </c>
-      <c r="E52" s="48" t="inlineStr">
-        <is>
-          <t>Unit EUR</t>
-        </is>
-      </c>
-      <c r="F52" s="48" t="inlineStr">
-        <is>
-          <t>Total EUR</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" ht="29" customHeight="1">
-      <c r="A53" s="49" t="inlineStr">
-        <is>
-          <t>G04</t>
-        </is>
-      </c>
-      <c r="B53" s="49" t="inlineStr">
-        <is>
-          <t>Antenna probe</t>
-        </is>
-      </c>
-      <c r="C53" s="6" t="inlineStr">
-        <is>
-          <t>868MHz 5dBi SMA-M omni 195mm  -  2 ks: jeden na sondu (SMA na doske), jeden na gateway</t>
-        </is>
-      </c>
-      <c r="D53" s="50" t="n">
-        <v>2</v>
-      </c>
-      <c r="E53" s="51" t="n">
-        <v>6</v>
-      </c>
-      <c r="F53" s="51" t="n">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="55" ht="20" customHeight="1">
-      <c r="A55" s="45" t="inlineStr">
-        <is>
-          <t>MAGSY.SK</t>
-        </is>
-      </c>
-      <c r="F55" s="46" t="n">
-        <v>8.800000000000001</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="47" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B56" s="47" t="inlineStr">
-        <is>
-          <t>Part</t>
-        </is>
-      </c>
-      <c r="C56" s="47" t="inlineStr">
-        <is>
-          <t>Specification / note</t>
-        </is>
-      </c>
-      <c r="D56" s="48" t="inlineStr">
-        <is>
-          <t>Qty</t>
-        </is>
-      </c>
-      <c r="E56" s="48" t="inlineStr">
-        <is>
-          <t>Unit EUR</t>
-        </is>
-      </c>
-      <c r="F56" s="48" t="inlineStr">
-        <is>
-          <t>Total EUR</t>
-        </is>
-      </c>
-    </row>
-    <row r="57" ht="42.5" customHeight="1">
-      <c r="A57" s="49" t="inlineStr">
-        <is>
-          <t>B01</t>
-        </is>
-      </c>
-      <c r="B57" s="49" t="inlineStr">
-        <is>
-          <t>Magnet</t>
-        </is>
-      </c>
-      <c r="C57" s="6" t="inlineStr">
-        <is>
-          <t>N52 D10x5 axially magnetised, canned 316L or epoxy potted  -  8 per cup, pitch r28 on D70 cup; price for D10 canned to re-verify; bare N52 must not touch water</t>
-        </is>
-      </c>
-      <c r="D57" s="50" t="n">
-        <v>16</v>
-      </c>
-      <c r="E57" s="51" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="F57" s="51" t="n">
-        <v>8.800000000000001</v>
-      </c>
-    </row>
-    <row r="59" ht="20" customHeight="1">
-      <c r="A59" s="45" t="inlineStr">
-        <is>
-          <t>NEREZMATERIAL.CZ</t>
-        </is>
-      </c>
-      <c r="F59" s="46" t="n">
-        <v>2.6</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="47" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B60" s="47" t="inlineStr">
-        <is>
-          <t>Part</t>
-        </is>
-      </c>
-      <c r="C60" s="47" t="inlineStr">
-        <is>
-          <t>Specification / note</t>
-        </is>
-      </c>
-      <c r="D60" s="48" t="inlineStr">
-        <is>
-          <t>Qty</t>
-        </is>
-      </c>
-      <c r="E60" s="48" t="inlineStr">
-        <is>
-          <t>Unit EUR</t>
-        </is>
-      </c>
-      <c r="F60" s="48" t="inlineStr">
-        <is>
-          <t>Total EUR</t>
-        </is>
-      </c>
-    </row>
-    <row r="61" ht="29" customHeight="1">
-      <c r="A61" s="49" t="inlineStr">
-        <is>
-          <t>A03</t>
-        </is>
-      </c>
-      <c r="B61" s="49" t="inlineStr">
-        <is>
-          <t>Wet shaft</t>
-        </is>
-      </c>
-      <c r="C61" s="6" t="inlineStr">
-        <is>
-          <t>316L Ø5 h6 x 115mm ground; 2 flats each end  -  3m bar 63.1 CZK makes ~26 shafts</t>
-        </is>
-      </c>
-      <c r="D61" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="E61" s="51" t="n">
-        <v>2.6</v>
-      </c>
-      <c r="F61" s="51" t="n">
-        <v>2.6</v>
-      </c>
-    </row>
-    <row r="62" ht="29" customHeight="1">
-      <c r="A62" s="52" t="inlineStr">
-        <is>
-          <t>B03</t>
-        </is>
-      </c>
-      <c r="B62" s="52" t="inlineStr">
-        <is>
-          <t>Separation wall</t>
-        </is>
-      </c>
-      <c r="C62" s="53" t="inlineStr">
-        <is>
-          <t>D106 x 4 mm - RECOMMENDED integral with the pod bulkhead (no separate part)  -  4 mm per CAD, not 5; integral removes O-ring C03 and screws C05</t>
-        </is>
-      </c>
-      <c r="D62" s="54" t="n">
-        <v>1</v>
-      </c>
-      <c r="E62" s="55" t="n">
-        <v>0</v>
-      </c>
-      <c r="F62" s="55" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="64" ht="20" customHeight="1">
-      <c r="A64" s="45" t="inlineStr">
-        <is>
-          <t>PRINTED IN-HOUSE</t>
-        </is>
-      </c>
-      <c r="F64" s="46" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="47" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B65" s="47" t="inlineStr">
-        <is>
-          <t>Part</t>
-        </is>
-      </c>
-      <c r="C65" s="47" t="inlineStr">
-        <is>
-          <t>Specification / note</t>
-        </is>
-      </c>
-      <c r="D65" s="48" t="inlineStr">
-        <is>
-          <t>Qty</t>
-        </is>
-      </c>
-      <c r="E65" s="48" t="inlineStr">
-        <is>
-          <t>Unit EUR</t>
-        </is>
-      </c>
-      <c r="F65" s="48" t="inlineStr">
-        <is>
-          <t>Total EUR</t>
-        </is>
-      </c>
-    </row>
-    <row r="66" ht="15.5" customHeight="1">
-      <c r="A66" s="49" t="inlineStr">
-        <is>
-          <t>C09</t>
-        </is>
-      </c>
-      <c r="B66" s="49" t="inlineStr">
-        <is>
-          <t>Generator mount</t>
-        </is>
-      </c>
-      <c r="C66" s="6" t="inlineStr">
-        <is>
-          <t>printed cradle + 4x M3x8 A4</t>
-        </is>
-      </c>
-      <c r="D66" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="E66" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="F66" s="51" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="67" ht="29" customHeight="1">
-      <c r="A67" s="52" t="inlineStr">
-        <is>
-          <t>A01</t>
-        </is>
-      </c>
-      <c r="B67" s="52" t="inlineStr">
-        <is>
-          <t>Blade</t>
-        </is>
-      </c>
-      <c r="C67" s="53" t="inlineStr">
-        <is>
-          <t>triple-blade rotor blade NACA4412 D220mm root pitch 28deg tip 2deg  -  ASA or ASA-CF; 6 perimeters; epoxy coat; spare blade = fuse for branch strike</t>
-        </is>
-      </c>
-      <c r="D67" s="54" t="n">
-        <v>3</v>
-      </c>
-      <c r="E67" s="55" t="n">
-        <v>0</v>
-      </c>
-      <c r="F67" s="55" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="68" ht="29" customHeight="1">
-      <c r="A68" s="49" t="inlineStr">
-        <is>
-          <t>A02</t>
-        </is>
-      </c>
-      <c r="B68" s="49" t="inlineStr">
-        <is>
-          <t>Hub</t>
-        </is>
-      </c>
-      <c r="C68" s="6" t="inlineStr">
-        <is>
-          <t>Ø64x46mm with 2x M4 heat-set inserts and Ø5 H7 shaft bore  -  brass inserts M4 from TME</t>
-        </is>
-      </c>
-      <c r="D68" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="E68" s="51" t="n">
-        <v>0</v>
-      </c>
-      <c r="F68" s="51" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="69" ht="29" customHeight="1">
-      <c r="A69" s="52" t="inlineStr">
-        <is>
-          <t>B02</t>
-        </is>
-      </c>
-      <c r="B69" s="52" t="inlineStr">
-        <is>
-          <t>Magnet cup</t>
-        </is>
-      </c>
-      <c r="C69" s="53" t="inlineStr">
-        <is>
-          <t>D70 rim, 8 pockets D10.2x5.2, printed ASA  -  pockets 10.2 dia (magnet 10 + 0.2 glue), 0.2 mm epoxy recess</t>
-        </is>
-      </c>
-      <c r="D69" s="54" t="n">
-        <v>2</v>
-      </c>
-      <c r="E69" s="55" t="n">
-        <v>0</v>
-      </c>
-      <c r="F69" s="55" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="70" ht="15.5" customHeight="1">
-      <c r="A70" s="49" t="inlineStr">
-        <is>
-          <t>C01</t>
-        </is>
-      </c>
-      <c r="B70" s="49" t="inlineStr">
-        <is>
-          <t>Pod barrel</t>
-        </is>
-      </c>
-      <c r="C70" s="6" t="inlineStr">
-        <is>
-          <t>Ø110x120mm printed ASA wall 2.4mm + epoxy barrier  -  in model as pod</t>
-        </is>
-      </c>
-      <c r="D70" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="E70" s="51" t="n">
-        <v>0</v>
-      </c>
-      <c r="F70" s="51" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="71" ht="15.5" customHeight="1">
-      <c r="A71" s="52" t="inlineStr">
-        <is>
-          <t>C02</t>
-        </is>
-      </c>
-      <c r="B71" s="52" t="inlineStr">
-        <is>
-          <t>Tail cone</t>
-        </is>
-      </c>
-      <c r="C71" s="53" t="inlineStr">
-        <is>
-          <t>printed integral</t>
-        </is>
-      </c>
-      <c r="D71" s="54" t="n">
-        <v>1</v>
-      </c>
-      <c r="E71" s="55" t="n">
-        <v>0</v>
-      </c>
-      <c r="F71" s="55" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="72" ht="15.5" customHeight="1">
-      <c r="A72" s="49" t="inlineStr">
-        <is>
-          <t>E01</t>
-        </is>
-      </c>
-      <c r="B72" s="49" t="inlineStr">
-        <is>
-          <t>Sensor cage</t>
-        </is>
-      </c>
-      <c r="C72" s="6" t="inlineStr">
-        <is>
-          <t>Ø130x150 printed ASA 12 slots  -  in model as cage</t>
-        </is>
-      </c>
-      <c r="D72" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="E72" s="51" t="n">
-        <v>0</v>
-      </c>
-      <c r="F72" s="51" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="73" ht="29" customHeight="1">
-      <c r="A73" s="52" t="inlineStr">
-        <is>
-          <t>E03</t>
-        </is>
-      </c>
-      <c r="B73" s="52" t="inlineStr">
-        <is>
-          <t>Sensor holders</t>
-        </is>
-      </c>
-      <c r="C73" s="53" t="inlineStr">
-        <is>
-          <t>printed clips for pH/TDS/turbidity/NTC/MS5837  -  in model as sensor bodies</t>
-        </is>
-      </c>
-      <c r="D73" s="54" t="n">
-        <v>5</v>
-      </c>
-      <c r="E73" s="55" t="n">
-        <v>0</v>
-      </c>
-      <c r="F73" s="55" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="75" ht="20" customHeight="1">
-      <c r="A75" s="45" t="inlineStr">
-        <is>
-          <t>PRUSA3D</t>
-        </is>
-      </c>
-      <c r="F75" s="46" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="47" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B76" s="47" t="inlineStr">
-        <is>
-          <t>Part</t>
-        </is>
-      </c>
-      <c r="C76" s="47" t="inlineStr">
-        <is>
-          <t>Specification / note</t>
-        </is>
-      </c>
-      <c r="D76" s="48" t="inlineStr">
-        <is>
-          <t>Qty</t>
-        </is>
-      </c>
-      <c r="E76" s="48" t="inlineStr">
-        <is>
-          <t>Unit EUR</t>
-        </is>
-      </c>
-      <c r="F76" s="48" t="inlineStr">
-        <is>
-          <t>Total EUR</t>
-        </is>
-      </c>
-    </row>
-    <row r="77" ht="29" customHeight="1">
-      <c r="A77" s="56" t="inlineStr">
-        <is>
-          <t>J01</t>
-        </is>
-      </c>
-      <c r="B77" s="56" t="inlineStr">
-        <is>
-          <t>Filament ASA</t>
-        </is>
-      </c>
-      <c r="C77" s="17" t="inlineStr">
-        <is>
-          <t>MAM  |  Prusament ASA 850g  -  ABS z domaceho spoolu, nie ASA; UV je len na brehu</t>
-        </is>
-      </c>
-      <c r="D77" s="57" t="n">
-        <v>1</v>
-      </c>
-      <c r="E77" s="58" t="n">
-        <v>32</v>
-      </c>
-      <c r="F77" s="58" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="79" ht="18" customHeight="1">
-      <c r="A79" s="59" t="inlineStr">
-        <is>
-          <t>GOODS</t>
-        </is>
-      </c>
-      <c r="F79" s="60" t="n">
-        <v>408.11</v>
-      </c>
-    </row>
-    <row r="80" ht="18" customHeight="1">
-      <c r="A80" s="59" t="inlineStr">
-        <is>
-          <t>shipping, estimated</t>
-        </is>
-      </c>
-      <c r="F80" s="60" t="n">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="81" ht="22" customHeight="1">
-      <c r="A81" s="61" t="inlineStr">
-        <is>
-          <t>LANDED TOTAL</t>
-        </is>
-      </c>
-      <c r="F81" s="62" t="n">
-        <v>433.11</v>
-      </c>
-    </row>
-    <row r="84" ht="22" customHeight="1">
-      <c r="A84" s="63" t="inlineStr">
-        <is>
-          <t>NOT IN THIS ORDER</t>
-        </is>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" s="64" t="inlineStr">
-        <is>
-          <t>PHASE 2 - BUY LATER</t>
-        </is>
-      </c>
-    </row>
-    <row r="86" ht="15.5" customHeight="1">
-      <c r="A86" s="65" t="inlineStr">
-        <is>
-          <t>C03</t>
-        </is>
-      </c>
-      <c r="B86" s="65" t="inlineStr">
-        <is>
-          <t>Pod O-ring</t>
-        </is>
-      </c>
-      <c r="C86" s="66" t="inlineStr">
-        <is>
-          <t>grease Molykote 111</t>
-        </is>
-      </c>
-      <c r="E86" s="67" t="inlineStr">
-        <is>
-          <t>3.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="87" ht="15.5" customHeight="1">
-      <c r="A87" s="65" t="inlineStr">
-        <is>
-          <t>C05</t>
-        </is>
-      </c>
-      <c r="B87" s="65" t="inlineStr">
-        <is>
-          <t>Pod clamp screws</t>
-        </is>
-      </c>
-      <c r="C87" s="66" t="inlineStr"/>
-      <c r="E87" s="67" t="inlineStr">
-        <is>
-          <t>3.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="88" ht="15.5" customHeight="1">
-      <c r="A88" s="65" t="inlineStr">
-        <is>
-          <t>D01</t>
-        </is>
-      </c>
-      <c r="B88" s="65" t="inlineStr">
-        <is>
-          <t>pH electrode</t>
-        </is>
-      </c>
-      <c r="C88" s="66" t="inlineStr">
-        <is>
-          <t>OPTIONAL per site; 14-30 day service; +-0.1 pH after 2-pt cal</t>
-        </is>
-      </c>
-      <c r="E88" s="67" t="inlineStr">
-        <is>
-          <t>39.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="89" ht="15.5" customHeight="1">
-      <c r="A89" s="65" t="inlineStr">
-        <is>
-          <t>D02</t>
-        </is>
-      </c>
-      <c r="B89" s="65" t="inlineStr">
-        <is>
-          <t>pH spare electrode</t>
-        </is>
-      </c>
-      <c r="C89" s="66" t="inlineStr">
-        <is>
-          <t>consumable</t>
-        </is>
-      </c>
-      <c r="E89" s="67" t="inlineStr">
+      <c r="C103" s="63" t="inlineStr">
+        <is>
+          <t>MAM - doma</t>
+        </is>
+      </c>
+      <c r="E103" s="64" t="inlineStr">
         <is>
           <t>9.0</t>
         </is>
       </c>
     </row>
-    <row r="90" ht="15.5" customHeight="1">
-      <c r="A90" s="65" t="inlineStr">
-        <is>
-          <t>D03</t>
-        </is>
-      </c>
-      <c r="B90" s="65" t="inlineStr">
-        <is>
-          <t>pH buffer</t>
-        </is>
-      </c>
-      <c r="C90" s="66" t="inlineStr">
-        <is>
-          <t>consumable</t>
-        </is>
-      </c>
-      <c r="E90" s="67" t="inlineStr">
+    <row r="104" ht="15.5" customHeight="1">
+      <c r="A104" s="62" t="inlineStr">
+        <is>
+          <t>J06</t>
+        </is>
+      </c>
+      <c r="B104" s="62" t="inlineStr">
+        <is>
+          <t>Threadlocker</t>
+        </is>
+      </c>
+      <c r="C104" s="63" t="inlineStr"/>
+      <c r="E104" s="64" t="inlineStr">
+        <is>
+          <t>11.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" ht="15.5" customHeight="1">
+      <c r="A105" s="62" t="inlineStr">
+        <is>
+          <t>J08</t>
+        </is>
+      </c>
+      <c r="B105" s="62" t="inlineStr">
+        <is>
+          <t>O-ring kit</t>
+        </is>
+      </c>
+      <c r="C105" s="63" t="inlineStr"/>
+      <c r="E105" s="64" t="inlineStr">
         <is>
           <t>12.0</t>
         </is>
       </c>
     </row>
-    <row r="91" ht="29" customHeight="1">
-      <c r="A91" s="65" t="inlineStr">
-        <is>
-          <t>D09</t>
-        </is>
-      </c>
-      <c r="B91" s="65" t="inlineStr">
-        <is>
-          <t>Dissolved oxygen kit</t>
-        </is>
-      </c>
-      <c r="C91" s="66" t="inlineStr">
-        <is>
-          <t>HIGHEST-VALUE channel (Budca = hypoxia); membrane 1-2 months in muddy water; 0.5M NaOH filling solution NOT shipped by air - source locally</t>
-        </is>
-      </c>
-      <c r="E91" s="67" t="inlineStr">
-        <is>
-          <t>175.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="92" ht="15.5" customHeight="1">
-      <c r="A92" s="65" t="inlineStr">
-        <is>
-          <t>D08</t>
-        </is>
-      </c>
-      <c r="B92" s="65" t="inlineStr">
-        <is>
-          <t>Sensor cable</t>
-        </is>
-      </c>
-      <c r="C92" s="66" t="inlineStr"/>
-      <c r="E92" s="67" t="inlineStr">
-        <is>
-          <t>20.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="93" ht="15.5" customHeight="1">
-      <c r="A93" s="65" t="inlineStr">
-        <is>
-          <t>G13</t>
-        </is>
-      </c>
-      <c r="B93" s="65" t="inlineStr">
-        <is>
-          <t>Barometer</t>
-        </is>
-      </c>
-      <c r="C93" s="66" t="inlineStr">
-        <is>
-          <t>pressure reference for MS5837</t>
-        </is>
-      </c>
-      <c r="E93" s="67" t="inlineStr">
-        <is>
-          <t>6.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="94" ht="15.5" customHeight="1">
-      <c r="A94" s="65" t="inlineStr">
-        <is>
-          <t>G14</t>
-        </is>
-      </c>
-      <c r="B94" s="65" t="inlineStr">
-        <is>
-          <t>PCB</t>
-        </is>
-      </c>
-      <c r="C94" s="66" t="inlineStr">
-        <is>
-          <t>panel of 10 amortises</t>
-        </is>
-      </c>
-      <c r="E94" s="67" t="inlineStr">
-        <is>
-          <t>3.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="95" ht="15.5" customHeight="1">
-      <c r="A95" s="65" t="inlineStr">
-        <is>
-          <t>G15</t>
-        </is>
-      </c>
-      <c r="B95" s="65" t="inlineStr">
-        <is>
-          <t>Connectors</t>
-        </is>
-      </c>
-      <c r="C95" s="66" t="inlineStr"/>
-      <c r="E95" s="67" t="inlineStr">
-        <is>
-          <t>10.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="96" ht="15.5" customHeight="1">
-      <c r="A96" s="65" t="inlineStr">
-        <is>
-          <t>H01</t>
-        </is>
-      </c>
-      <c r="B96" s="65" t="inlineStr">
-        <is>
-          <t>Ground screw anchor</t>
-        </is>
-      </c>
-      <c r="C96" s="66" t="inlineStr">
-        <is>
-          <t>1-2kN lateral - covers flood case</t>
-        </is>
-      </c>
-      <c r="E96" s="67" t="inlineStr">
-        <is>
-          <t>25.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="97" ht="15.5" customHeight="1">
-      <c r="A97" s="65" t="inlineStr">
-        <is>
-          <t>H02</t>
-        </is>
-      </c>
-      <c r="B97" s="65" t="inlineStr">
-        <is>
-          <t>Pole</t>
-        </is>
-      </c>
-      <c r="C97" s="66" t="inlineStr">
-        <is>
-          <t>removable mast pinned into receiver</t>
-        </is>
-      </c>
-      <c r="E97" s="67" t="inlineStr">
-        <is>
-          <t>18.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="98" ht="15.5" customHeight="1">
-      <c r="A98" s="65" t="inlineStr">
-        <is>
-          <t>H03</t>
-        </is>
-      </c>
-      <c r="B98" s="65" t="inlineStr">
-        <is>
-          <t>Receiver sleeve</t>
-        </is>
-      </c>
-      <c r="C98" s="66" t="inlineStr">
-        <is>
-          <t>pinned mast interface</t>
-        </is>
-      </c>
-      <c r="E98" s="67" t="inlineStr">
-        <is>
-          <t>8.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="99" ht="15.5" customHeight="1">
-      <c r="A99" s="65" t="inlineStr">
-        <is>
-          <t>H04</t>
-        </is>
-      </c>
-      <c r="B99" s="65" t="inlineStr">
-        <is>
-          <t>Arm tube</t>
-        </is>
-      </c>
-      <c r="C99" s="66" t="inlineStr"/>
-      <c r="E99" s="67" t="inlineStr">
-        <is>
-          <t>9.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="100" ht="15.5" customHeight="1">
-      <c r="A100" s="65" t="inlineStr">
-        <is>
-          <t>H05</t>
-        </is>
-      </c>
-      <c r="B100" s="65" t="inlineStr">
-        <is>
-          <t>Drop tube</t>
-        </is>
-      </c>
-      <c r="C100" s="66" t="inlineStr"/>
-      <c r="E100" s="67" t="inlineStr">
-        <is>
-          <t>6.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="101" ht="15.5" customHeight="1">
-      <c r="A101" s="65" t="inlineStr">
-        <is>
-          <t>H06</t>
-        </is>
-      </c>
-      <c r="B101" s="65" t="inlineStr">
-        <is>
-          <t>Hinge collar</t>
-        </is>
-      </c>
-      <c r="C101" s="66" t="inlineStr"/>
-      <c r="E101" s="67" t="inlineStr">
-        <is>
-          <t>3.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="102" ht="15.5" customHeight="1">
-      <c r="A102" s="65" t="inlineStr">
-        <is>
-          <t>H07</t>
-        </is>
-      </c>
-      <c r="B102" s="65" t="inlineStr">
-        <is>
-          <t>Shear pin</t>
-        </is>
-      </c>
-      <c r="C102" s="66" t="inlineStr">
-        <is>
-          <t>releases pod on &gt;150N debris hit</t>
-        </is>
-      </c>
-      <c r="E102" s="67" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="103" ht="15.5" customHeight="1">
-      <c r="A103" s="65" t="inlineStr">
-        <is>
-          <t>H08</t>
-        </is>
-      </c>
-      <c r="B103" s="65" t="inlineStr">
-        <is>
-          <t>Yaw strut</t>
-        </is>
-      </c>
-      <c r="C103" s="66" t="inlineStr">
-        <is>
-          <t>anti-flutter</t>
-        </is>
-      </c>
-      <c r="E103" s="67" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="104" ht="15.5" customHeight="1">
-      <c r="A104" s="65" t="inlineStr">
-        <is>
-          <t>H09</t>
-        </is>
-      </c>
-      <c r="B104" s="65" t="inlineStr">
-        <is>
-          <t>Guy line</t>
-        </is>
-      </c>
-      <c r="C104" s="66" t="inlineStr">
-        <is>
-          <t>45deg up/downstream</t>
-        </is>
-      </c>
-      <c r="E104" s="67" t="inlineStr">
-        <is>
-          <t>9.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="105" ht="15.5" customHeight="1">
-      <c r="A105" s="65" t="inlineStr">
-        <is>
-          <t>H10</t>
-        </is>
-      </c>
-      <c r="B105" s="65" t="inlineStr">
-        <is>
-          <t>Guy anchor</t>
-        </is>
-      </c>
-      <c r="C105" s="66" t="inlineStr"/>
-      <c r="E105" s="67" t="inlineStr">
-        <is>
-          <t>10.0</t>
-        </is>
-      </c>
-    </row>
     <row r="106" ht="15.5" customHeight="1">
-      <c r="A106" s="65" t="inlineStr">
-        <is>
-          <t>H11</t>
-        </is>
-      </c>
-      <c r="B106" s="65" t="inlineStr">
-        <is>
-          <t>Safety cable</t>
-        </is>
-      </c>
-      <c r="C106" s="66" t="inlineStr">
-        <is>
-          <t>theft/flood retention</t>
-        </is>
-      </c>
-      <c r="E106" s="67" t="inlineStr">
-        <is>
-          <t>4.0</t>
+      <c r="A106" s="62" t="inlineStr">
+        <is>
+          <t>K01</t>
+        </is>
+      </c>
+      <c r="B106" s="62" t="inlineStr">
+        <is>
+          <t>Vacuum chamber</t>
+        </is>
+      </c>
+      <c r="C106" s="63" t="inlineStr">
+        <is>
+          <t>acceptance test rig (one-off)</t>
+        </is>
+      </c>
+      <c r="E106" s="64" t="inlineStr">
+        <is>
+          <t>85.0</t>
         </is>
       </c>
     </row>
     <row r="107" ht="15.5" customHeight="1">
-      <c r="A107" s="65" t="inlineStr">
-        <is>
-          <t>H12</t>
-        </is>
-      </c>
-      <c r="B107" s="65" t="inlineStr">
-        <is>
-          <t>Security fastener</t>
-        </is>
-      </c>
-      <c r="C107" s="66" t="inlineStr">
-        <is>
-          <t>anti-theft</t>
-        </is>
-      </c>
-      <c r="E107" s="67" t="inlineStr">
-        <is>
-          <t>4.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="108" ht="15.5" customHeight="1">
-      <c r="A108" s="65" t="inlineStr">
-        <is>
-          <t>H13</t>
-        </is>
-      </c>
-      <c r="B108" s="65" t="inlineStr">
-        <is>
-          <t>Site label</t>
-        </is>
-      </c>
-      <c r="C108" s="66" t="inlineStr">
-        <is>
-          <t>anti-theft by making it unsellable</t>
-        </is>
-      </c>
-      <c r="E108" s="67" t="inlineStr">
-        <is>
-          <t>3.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="109" ht="15.5" customHeight="1">
+      <c r="A107" s="62" t="inlineStr">
+        <is>
+          <t>K02</t>
+        </is>
+      </c>
+      <c r="B107" s="62" t="inlineStr">
+        <is>
+          <t>Torque driver</t>
+        </is>
+      </c>
+      <c r="C107" s="63" t="inlineStr">
+        <is>
+          <t>one-off</t>
+        </is>
+      </c>
+      <c r="E107" s="64" t="inlineStr">
+        <is>
+          <t>40.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
       <c r="A109" s="65" t="inlineStr">
         <is>
-          <t>I02</t>
-        </is>
-      </c>
-      <c r="B109" s="65" t="inlineStr">
-        <is>
-          <t>Compute</t>
-        </is>
-      </c>
-      <c r="C109" s="66" t="inlineStr">
-        <is>
-          <t>YOU ALREADY HAVE THIS - reuse, zero soldering; runs the gateway service</t>
-        </is>
-      </c>
-      <c r="E109" s="67" t="inlineStr">
-        <is>
-          <t>70.0</t>
+          <t>CUT - DEAD LINE, DO NOT BUY</t>
         </is>
       </c>
     </row>
     <row r="110" ht="15.5" customHeight="1">
-      <c r="A110" s="65" t="inlineStr">
-        <is>
-          <t>I03</t>
-        </is>
-      </c>
-      <c r="B110" s="65" t="inlineStr">
-        <is>
-          <t>Antenna</t>
-        </is>
-      </c>
-      <c r="C110" s="66" t="inlineStr">
-        <is>
-          <t>range-critical: gateway antenna gain + mast height set the link</t>
-        </is>
-      </c>
-      <c r="E110" s="67" t="inlineStr">
-        <is>
-          <t>45.0</t>
+      <c r="A110" s="62" t="inlineStr">
+        <is>
+          <t>A05</t>
+        </is>
+      </c>
+      <c r="B110" s="62" t="inlineStr">
+        <is>
+          <t>Bearing carrier tube</t>
+        </is>
+      </c>
+      <c r="C110" s="63" t="inlineStr">
+        <is>
+          <t>CUT: superseded - the bearing carrier is the printed spider (wet_carrier)</t>
+        </is>
+      </c>
+      <c r="E110" s="66" t="inlineStr">
+        <is>
+          <t>1.2</t>
         </is>
       </c>
     </row>
     <row r="111" ht="15.5" customHeight="1">
-      <c r="A111" s="65" t="inlineStr">
-        <is>
-          <t>I04</t>
-        </is>
-      </c>
-      <c r="B111" s="65" t="inlineStr">
-        <is>
-          <t>Enclosure</t>
-        </is>
-      </c>
-      <c r="C111" s="66" t="inlineStr"/>
-      <c r="E111" s="67" t="inlineStr">
-        <is>
-          <t>35.0</t>
+      <c r="A111" s="62" t="inlineStr">
+        <is>
+          <t>A07</t>
+        </is>
+      </c>
+      <c r="B111" s="62" t="inlineStr">
+        <is>
+          <t>Weed guard ring</t>
+        </is>
+      </c>
+      <c r="C111" s="63" t="inlineStr">
+        <is>
+          <t>CUT: killed by design - replaced by the nose cone D64-&gt;D12; a ring on struts upstream is an algae scythe</t>
+        </is>
+      </c>
+      <c r="E111" s="66" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="112" ht="15.5" customHeight="1">
-      <c r="A112" s="65" t="inlineStr">
-        <is>
-          <t>I05</t>
-        </is>
-      </c>
-      <c r="B112" s="65" t="inlineStr">
-        <is>
-          <t>Mast</t>
-        </is>
-      </c>
-      <c r="C112" s="66" t="inlineStr">
-        <is>
-          <t>height sets range</t>
-        </is>
-      </c>
-      <c r="E112" s="67" t="inlineStr">
-        <is>
-          <t>30.0</t>
+      <c r="A112" s="62" t="inlineStr">
+        <is>
+          <t>A08</t>
+        </is>
+      </c>
+      <c r="B112" s="62" t="inlineStr">
+        <is>
+          <t>Blade safety retainer</t>
+        </is>
+      </c>
+      <c r="C112" s="63" t="inlineStr">
+        <is>
+          <t>CUT: killed by design - a tether on a 110 mm blade is a flail, and the hole is a stress riser at the root</t>
+        </is>
+      </c>
+      <c r="E112" s="66" t="inlineStr">
+        <is>
+          <t>2.0</t>
         </is>
       </c>
     </row>
     <row r="113" ht="15.5" customHeight="1">
-      <c r="A113" s="65" t="inlineStr">
-        <is>
-          <t>J02</t>
-        </is>
-      </c>
-      <c r="B113" s="65" t="inlineStr">
-        <is>
-          <t>Filament PC Blend</t>
-        </is>
-      </c>
-      <c r="C113" s="66" t="inlineStr"/>
-      <c r="E113" s="67" t="inlineStr">
-        <is>
-          <t>40.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="114" ht="15.5" customHeight="1">
-      <c r="A114" s="65" t="inlineStr">
-        <is>
-          <t>J04</t>
-        </is>
-      </c>
-      <c r="B114" s="65" t="inlineStr">
-        <is>
-          <t>Conformal coat</t>
-        </is>
-      </c>
-      <c r="C114" s="66" t="inlineStr"/>
-      <c r="E114" s="67" t="inlineStr">
-        <is>
-          <t>14.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="115" ht="15.5" customHeight="1">
-      <c r="A115" s="65" t="inlineStr">
-        <is>
-          <t>J06</t>
-        </is>
-      </c>
-      <c r="B115" s="65" t="inlineStr">
-        <is>
-          <t>Threadlocker</t>
-        </is>
-      </c>
-      <c r="C115" s="66" t="inlineStr"/>
-      <c r="E115" s="67" t="inlineStr">
-        <is>
-          <t>11.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="116" ht="15.5" customHeight="1">
-      <c r="A116" s="65" t="inlineStr">
-        <is>
-          <t>J08</t>
-        </is>
-      </c>
-      <c r="B116" s="65" t="inlineStr">
-        <is>
-          <t>O-ring kit</t>
-        </is>
-      </c>
-      <c r="C116" s="66" t="inlineStr"/>
-      <c r="E116" s="67" t="inlineStr">
-        <is>
-          <t>12.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="117" ht="15.5" customHeight="1">
-      <c r="A117" s="65" t="inlineStr">
-        <is>
-          <t>K01</t>
-        </is>
-      </c>
-      <c r="B117" s="65" t="inlineStr">
-        <is>
-          <t>Vacuum chamber</t>
-        </is>
-      </c>
-      <c r="C117" s="66" t="inlineStr">
-        <is>
-          <t>acceptance test rig (one-off)</t>
-        </is>
-      </c>
-      <c r="E117" s="67" t="inlineStr">
-        <is>
-          <t>85.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="118" ht="15.5" customHeight="1">
-      <c r="A118" s="65" t="inlineStr">
-        <is>
-          <t>K02</t>
-        </is>
-      </c>
-      <c r="B118" s="65" t="inlineStr">
-        <is>
-          <t>Torque driver</t>
-        </is>
-      </c>
-      <c r="C118" s="66" t="inlineStr">
-        <is>
-          <t>one-off</t>
-        </is>
-      </c>
-      <c r="E118" s="67" t="inlineStr">
-        <is>
-          <t>40.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="120">
-      <c r="A120" s="68" t="inlineStr">
-        <is>
-          <t>CUT - DEAD LINE, DO NOT BUY</t>
-        </is>
-      </c>
-    </row>
-    <row r="121" ht="15.5" customHeight="1">
-      <c r="A121" s="65" t="inlineStr">
-        <is>
-          <t>A05</t>
-        </is>
-      </c>
-      <c r="B121" s="65" t="inlineStr">
-        <is>
-          <t>Bearing carrier tube</t>
-        </is>
-      </c>
-      <c r="C121" s="66" t="inlineStr">
-        <is>
-          <t>CUT: superseded - the bearing carrier is the printed spider (wet_carrier)</t>
-        </is>
-      </c>
-      <c r="E121" s="69" t="inlineStr">
-        <is>
-          <t>1.2</t>
-        </is>
-      </c>
-    </row>
-    <row r="122" ht="15.5" customHeight="1">
-      <c r="A122" s="65" t="inlineStr">
-        <is>
-          <t>A07</t>
-        </is>
-      </c>
-      <c r="B122" s="65" t="inlineStr">
-        <is>
-          <t>Weed guard ring</t>
-        </is>
-      </c>
-      <c r="C122" s="66" t="inlineStr">
-        <is>
-          <t>CUT: killed by design - replaced by the nose cone D64-&gt;D12; a ring on struts upstream is an algae scythe</t>
-        </is>
-      </c>
-      <c r="E122" s="69" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="123" ht="15.5" customHeight="1">
-      <c r="A123" s="65" t="inlineStr">
-        <is>
-          <t>A08</t>
-        </is>
-      </c>
-      <c r="B123" s="65" t="inlineStr">
-        <is>
-          <t>Blade safety retainer</t>
-        </is>
-      </c>
-      <c r="C123" s="66" t="inlineStr">
-        <is>
-          <t>CUT: killed by design - a tether on a 110 mm blade is a flail, and the hole is a stress riser at the root</t>
-        </is>
-      </c>
-      <c r="E123" s="69" t="inlineStr">
-        <is>
-          <t>2.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="124" ht="15.5" customHeight="1">
-      <c r="A124" s="65" t="inlineStr">
+      <c r="A113" s="62" t="inlineStr">
         <is>
           <t>G02</t>
         </is>
       </c>
-      <c r="B124" s="65" t="inlineStr">
+      <c r="B113" s="62" t="inlineStr">
         <is>
           <t>MCU (NOT USED in simple build)</t>
         </is>
       </c>
-      <c r="C124" s="66" t="inlineStr">
+      <c r="C113" s="63" t="inlineStr">
         <is>
           <t>DROPPED: Wio-E5 mini is the single brain (MCU+LoRa). Bring back only if we need more GPIO/dual-core.</t>
         </is>
       </c>
-      <c r="E124" s="69" t="inlineStr">
+      <c r="E113" s="66" t="inlineStr">
         <is>
           <t>0.0</t>
         </is>
       </c>
     </row>
-    <row r="125" ht="15.5" customHeight="1">
-      <c r="A125" s="65" t="inlineStr">
-        <is>
-          <t>I06</t>
-        </is>
-      </c>
-      <c r="B125" s="65" t="inlineStr">
-        <is>
-          <t>Concentrator upgrade (optional)</t>
-        </is>
-      </c>
-      <c r="C125" s="66" t="inlineStr">
-        <is>
-          <t>Only for multi-SF / multi-channel / public TTN. Single-channel Wio-E5 gateway is enough for our 20 nodes.</t>
-        </is>
-      </c>
-      <c r="E125" s="69" t="inlineStr">
-        <is>
-          <t>145.0</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="17">
+  <mergeCells count="13">
     <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A39:E39"/>
+    <mergeCell ref="A29:E29"/>
+    <mergeCell ref="A35:E35"/>
+    <mergeCell ref="A50:E50"/>
     <mergeCell ref="A55:E55"/>
-    <mergeCell ref="A59:E59"/>
-    <mergeCell ref="A81:E81"/>
-    <mergeCell ref="A84:F84"/>
-    <mergeCell ref="A64:E64"/>
+    <mergeCell ref="A54:E54"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A28:E28"/>
-    <mergeCell ref="A51:E51"/>
-    <mergeCell ref="A47:E47"/>
+    <mergeCell ref="A19:E19"/>
     <mergeCell ref="A5:E5"/>
-    <mergeCell ref="A75:E75"/>
-    <mergeCell ref="A32:E32"/>
     <mergeCell ref="A3:F3"/>
-    <mergeCell ref="A80:E80"/>
-    <mergeCell ref="A40:E40"/>
-    <mergeCell ref="A79:E79"/>
+    <mergeCell ref="A56:E56"/>
+    <mergeCell ref="A59:F59"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
@@ -3538,7 +3301,7 @@
       </c>
       <c r="L8" s="6" t="inlineStr">
         <is>
-          <t>3m bar 63.1 CZK makes ~26 shafts</t>
+          <t>lokalny zeleziar / Hornbach M5 A4 srob - 4. obchod sa nerata, nema postu; 3m bar 63.1 CZK makes ~26 shafts</t>
         </is>
       </c>
     </row>
@@ -3824,10 +3587,10 @@
           <t>subtotal - Rotor &amp; drivetrain (wet side)</t>
         </is>
       </c>
-      <c r="B14" s="70" t="n"/>
-      <c r="C14" s="70" t="n"/>
-      <c r="D14" s="70" t="n"/>
-      <c r="E14" s="71" t="n"/>
+      <c r="B14" s="67" t="n"/>
+      <c r="C14" s="67" t="n"/>
+      <c r="D14" s="67" t="n"/>
+      <c r="E14" s="68" t="n"/>
       <c r="F14" s="15" t="n"/>
       <c r="G14" s="15" t="n">
         <v>8.16</v>
@@ -4071,10 +3834,10 @@
           <t>subtotal - Magnetic coupling</t>
         </is>
       </c>
-      <c r="B21" s="70" t="n"/>
-      <c r="C21" s="70" t="n"/>
-      <c r="D21" s="70" t="n"/>
-      <c r="E21" s="71" t="n"/>
+      <c r="B21" s="67" t="n"/>
+      <c r="C21" s="67" t="n"/>
+      <c r="D21" s="67" t="n"/>
+      <c r="E21" s="68" t="n"/>
       <c r="F21" s="15" t="n"/>
       <c r="G21" s="15" t="n">
         <v>22.8</v>
@@ -4385,7 +4148,7 @@
       </c>
       <c r="E29" s="6" t="inlineStr">
         <is>
-          <t>local</t>
+          <t>local shop</t>
         </is>
       </c>
       <c r="F29" s="8" t="n">
@@ -4528,7 +4291,7 @@
       </c>
       <c r="L31" s="17" t="inlineStr">
         <is>
-          <t>check your motor box first - v0 used a robot motor | XTG3506 preferred: encoder = free RPM/flow</t>
+          <t>check your motor box first - v0 used a robot motor | TEST BEZ GENERATORA: klietka + senzory stacia, generator je dalsi nakup; XTG3506 preferred: encoder = free RPM/flow</t>
         </is>
       </c>
     </row>
@@ -4553,7 +4316,7 @@
       </c>
       <c r="E32" s="6" t="inlineStr">
         <is>
-          <t>printed + tme</t>
+          <t>printed in-house</t>
         </is>
       </c>
       <c r="F32" s="8" t="n">
@@ -4590,10 +4353,10 @@
           <t>subtotal - Generator pod &amp; sealing</t>
         </is>
       </c>
-      <c r="B33" s="70" t="n"/>
-      <c r="C33" s="70" t="n"/>
-      <c r="D33" s="70" t="n"/>
-      <c r="E33" s="71" t="n"/>
+      <c r="B33" s="67" t="n"/>
+      <c r="C33" s="67" t="n"/>
+      <c r="D33" s="67" t="n"/>
+      <c r="E33" s="68" t="n"/>
       <c r="F33" s="15" t="n"/>
       <c r="G33" s="15" t="n">
         <v>49</v>
@@ -5117,10 +4880,10 @@
           <t>subtotal - Sensors</t>
         </is>
       </c>
-      <c r="B45" s="70" t="n"/>
-      <c r="C45" s="70" t="n"/>
-      <c r="D45" s="70" t="n"/>
-      <c r="E45" s="71" t="n"/>
+      <c r="B45" s="67" t="n"/>
+      <c r="C45" s="67" t="n"/>
+      <c r="D45" s="67" t="n"/>
+      <c r="E45" s="68" t="n"/>
       <c r="F45" s="15" t="n"/>
       <c r="G45" s="15" t="n">
         <v>405.45</v>
@@ -5308,10 +5071,10 @@
           <t>subtotal - Sensor cage &amp; mounting</t>
         </is>
       </c>
-      <c r="B51" s="70" t="n"/>
-      <c r="C51" s="70" t="n"/>
-      <c r="D51" s="70" t="n"/>
-      <c r="E51" s="71" t="n"/>
+      <c r="B51" s="67" t="n"/>
+      <c r="C51" s="67" t="n"/>
+      <c r="D51" s="67" t="n"/>
+      <c r="E51" s="68" t="n"/>
       <c r="F51" s="15" t="n"/>
       <c r="G51" s="15" t="n">
         <v>6</v>
@@ -5443,10 +5206,10 @@
           <t>subtotal - Wet-dry interface (cable)</t>
         </is>
       </c>
-      <c r="B56" s="70" t="n"/>
-      <c r="C56" s="70" t="n"/>
-      <c r="D56" s="70" t="n"/>
-      <c r="E56" s="71" t="n"/>
+      <c r="B56" s="67" t="n"/>
+      <c r="C56" s="67" t="n"/>
+      <c r="D56" s="67" t="n"/>
+      <c r="E56" s="68" t="n"/>
       <c r="F56" s="15" t="n"/>
       <c r="G56" s="15" t="n">
         <v>47</v>
@@ -5653,7 +5416,7 @@
       </c>
       <c r="E62" s="6" t="inlineStr">
         <is>
-          <t>neven.cz</t>
+          <t>techfun.sk</t>
         </is>
       </c>
       <c r="F62" s="8" t="n">
@@ -6414,10 +6177,10 @@
           <t>subtotal - Electronics (dry box)</t>
         </is>
       </c>
-      <c r="B76" s="70" t="n"/>
-      <c r="C76" s="70" t="n"/>
-      <c r="D76" s="70" t="n"/>
-      <c r="E76" s="71" t="n"/>
+      <c r="B76" s="67" t="n"/>
+      <c r="C76" s="67" t="n"/>
+      <c r="D76" s="67" t="n"/>
+      <c r="E76" s="68" t="n"/>
       <c r="F76" s="15" t="n"/>
       <c r="G76" s="15" t="n">
         <v>112.9</v>
@@ -7153,10 +6916,10 @@
           <t>subtotal - Structure &amp; site</t>
         </is>
       </c>
-      <c r="B92" s="70" t="n"/>
-      <c r="C92" s="70" t="n"/>
-      <c r="D92" s="70" t="n"/>
-      <c r="E92" s="71" t="n"/>
+      <c r="B92" s="67" t="n"/>
+      <c r="C92" s="67" t="n"/>
+      <c r="D92" s="67" t="n"/>
+      <c r="E92" s="68" t="n"/>
       <c r="F92" s="15" t="n"/>
       <c r="G92" s="15" t="n">
         <v>105</v>
@@ -7195,7 +6958,7 @@
       </c>
       <c r="E95" s="6" t="inlineStr">
         <is>
-          <t>rakwireless reseller</t>
+          <t>techfun.sk</t>
         </is>
       </c>
       <c r="F95" s="8" t="n">
@@ -7512,10 +7275,10 @@
           <t>subtotal - Gateway (base station)</t>
         </is>
       </c>
-      <c r="B101" s="70" t="n"/>
-      <c r="C101" s="70" t="n"/>
-      <c r="D101" s="70" t="n"/>
-      <c r="E101" s="71" t="n"/>
+      <c r="B101" s="67" t="n"/>
+      <c r="C101" s="67" t="n"/>
+      <c r="D101" s="67" t="n"/>
+      <c r="E101" s="68" t="n"/>
       <c r="F101" s="15" t="n"/>
       <c r="G101" s="15" t="n">
         <v>343</v>
@@ -7963,10 +7726,10 @@
           <t>subtotal - Consumables</t>
         </is>
       </c>
-      <c r="B112" s="70" t="n"/>
-      <c r="C112" s="70" t="n"/>
-      <c r="D112" s="70" t="n"/>
-      <c r="E112" s="71" t="n"/>
+      <c r="B112" s="67" t="n"/>
+      <c r="C112" s="67" t="n"/>
+      <c r="D112" s="67" t="n"/>
+      <c r="E112" s="68" t="n"/>
       <c r="F112" s="15" t="n"/>
       <c r="G112" s="15" t="n">
         <v>142</v>
@@ -8117,7 +7880,7 @@
       </c>
       <c r="E117" s="17" t="inlineStr">
         <is>
-          <t>local</t>
+          <t>local shop</t>
         </is>
       </c>
       <c r="F117" s="19" t="n">
@@ -8158,10 +7921,10 @@
           <t>subtotal - Tooling (one-off)</t>
         </is>
       </c>
-      <c r="B118" s="70" t="n"/>
-      <c r="C118" s="70" t="n"/>
-      <c r="D118" s="70" t="n"/>
-      <c r="E118" s="71" t="n"/>
+      <c r="B118" s="67" t="n"/>
+      <c r="C118" s="67" t="n"/>
+      <c r="D118" s="67" t="n"/>
+      <c r="E118" s="68" t="n"/>
       <c r="F118" s="15" t="n"/>
       <c r="G118" s="15" t="n">
         <v>130</v>
@@ -8178,11 +7941,11 @@
           <t>REQUIRED (everything needed to build and deploy)</t>
         </is>
       </c>
-      <c r="B120" s="70" t="n"/>
-      <c r="C120" s="70" t="n"/>
-      <c r="D120" s="70" t="n"/>
-      <c r="E120" s="70" t="n"/>
-      <c r="F120" s="71" t="n"/>
+      <c r="B120" s="67" t="n"/>
+      <c r="C120" s="67" t="n"/>
+      <c r="D120" s="67" t="n"/>
+      <c r="E120" s="67" t="n"/>
+      <c r="F120" s="68" t="n"/>
       <c r="G120" s="25" t="n">
         <v>730.3100000000001</v>
       </c>
@@ -8193,11 +7956,11 @@
           <t>recommended add-ons (DO, level probe, anti-theft, tools)</t>
         </is>
       </c>
-      <c r="B121" s="70" t="n"/>
-      <c r="C121" s="70" t="n"/>
-      <c r="D121" s="70" t="n"/>
-      <c r="E121" s="70" t="n"/>
-      <c r="F121" s="71" t="n"/>
+      <c r="B121" s="67" t="n"/>
+      <c r="C121" s="67" t="n"/>
+      <c r="D121" s="67" t="n"/>
+      <c r="E121" s="67" t="n"/>
+      <c r="F121" s="68" t="n"/>
       <c r="G121" s="27" t="n">
         <v>641</v>
       </c>
@@ -8208,11 +7971,11 @@
           <t>TOTAL if you buy everything</t>
         </is>
       </c>
-      <c r="B122" s="70" t="n"/>
-      <c r="C122" s="70" t="n"/>
-      <c r="D122" s="70" t="n"/>
-      <c r="E122" s="70" t="n"/>
-      <c r="F122" s="71" t="n"/>
+      <c r="B122" s="67" t="n"/>
+      <c r="C122" s="67" t="n"/>
+      <c r="D122" s="67" t="n"/>
+      <c r="E122" s="67" t="n"/>
+      <c r="F122" s="68" t="n"/>
       <c r="G122" s="29" t="n">
         <v>1371.31</v>
       </c>
@@ -8223,11 +7986,11 @@
           <t>saved by reusing what you already own</t>
         </is>
       </c>
-      <c r="B123" s="70" t="n"/>
-      <c r="C123" s="70" t="n"/>
-      <c r="D123" s="70" t="n"/>
-      <c r="E123" s="70" t="n"/>
-      <c r="F123" s="71" t="n"/>
+      <c r="B123" s="67" t="n"/>
+      <c r="C123" s="67" t="n"/>
+      <c r="D123" s="67" t="n"/>
+      <c r="E123" s="67" t="n"/>
+      <c r="F123" s="68" t="n"/>
       <c r="G123" s="31" t="n">
         <v>-70</v>
       </c>
@@ -8238,11 +8001,11 @@
           <t>net if you reuse your Raspberry Pi etc.</t>
         </is>
       </c>
-      <c r="B124" s="70" t="n"/>
-      <c r="C124" s="70" t="n"/>
-      <c r="D124" s="70" t="n"/>
-      <c r="E124" s="70" t="n"/>
-      <c r="F124" s="71" t="n"/>
+      <c r="B124" s="67" t="n"/>
+      <c r="C124" s="67" t="n"/>
+      <c r="D124" s="67" t="n"/>
+      <c r="E124" s="67" t="n"/>
+      <c r="F124" s="68" t="n"/>
       <c r="G124" s="33" t="n">
         <v>1301.31</v>
       </c>

</xml_diff>

<commit_message>
order: put the back joint back in
The pod still has an opening at the back where the cage adapter bolts on. An
integral bulkhead only seals the front, so the O-ring and its clamp screws are
part of the dunk test, not a later phase.

phase 1: 33 lines, 234.61 EUR goods
</commit_message>
<xml_diff>
--- a/docs/sub-mission_parts.xlsx
+++ b/docs/sub-mission_parts.xlsx
@@ -826,7 +826,7 @@
     <row r="3" ht="26" customHeight="1">
       <c r="A3" s="44" t="inlineStr">
         <is>
-          <t>31 lines      goods 228.61 EUR      shipping est. 25.00 EUR      LANDED 253.61 EUR</t>
+          <t>33 lines      goods 234.61 EUR      shipping est. 25.00 EUR      LANDED 259.61 EUR</t>
         </is>
       </c>
     </row>
@@ -837,7 +837,7 @@
         </is>
       </c>
       <c r="F5" s="46" t="n">
-        <v>115.36</v>
+        <v>121.36</v>
       </c>
     </row>
     <row r="6">
@@ -1080,20 +1080,20 @@
         <v>6</v>
       </c>
     </row>
-    <row r="15" ht="29" customHeight="1">
+    <row r="15" ht="15.5" customHeight="1">
       <c r="A15" s="49" t="inlineStr">
         <is>
-          <t>G05</t>
+          <t>C03</t>
         </is>
       </c>
       <c r="B15" s="49" t="inlineStr">
         <is>
-          <t>Antenna pigtail</t>
+          <t>Pod O-ring</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>u.FL to SMA bulkhead 15cm  -  u.FL -&gt; SMA pigtail; skip if your board ships with SMA already</t>
+          <t>NBR 70 Ø100x2.5  -  zadny spoj podu - bez neho sa pri ponoreni natecie</t>
         </is>
       </c>
       <c r="D15" s="50" t="n">
@@ -1109,605 +1109,605 @@
     <row r="16" ht="29" customHeight="1">
       <c r="A16" s="52" t="inlineStr">
         <is>
+          <t>C05</t>
+        </is>
+      </c>
+      <c r="B16" s="52" t="inlineStr">
+        <is>
+          <t>Pod clamp screws</t>
+        </is>
+      </c>
+      <c r="C16" s="53" t="inlineStr">
+        <is>
+          <t>M4x30 A4 + washers  -  drzi zadny spoj; integralny bulkhead riesi len prednu stranu</t>
+        </is>
+      </c>
+      <c r="D16" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" s="55" t="n">
+        <v>3</v>
+      </c>
+      <c r="F16" s="55" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17" ht="29" customHeight="1">
+      <c r="A17" s="49" t="inlineStr">
+        <is>
+          <t>G05</t>
+        </is>
+      </c>
+      <c r="B17" s="49" t="inlineStr">
+        <is>
+          <t>Antenna pigtail</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>u.FL to SMA bulkhead 15cm  -  u.FL -&gt; SMA pigtail; skip if your board ships with SMA already</t>
+        </is>
+      </c>
+      <c r="D17" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="F17" s="51" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="18" ht="29" customHeight="1">
+      <c r="A18" s="52" t="inlineStr">
+        <is>
           <t>A04</t>
         </is>
       </c>
-      <c r="B16" s="52" t="inlineStr">
+      <c r="B18" s="52" t="inlineStr">
         <is>
           <t>Wet bearing</t>
         </is>
       </c>
-      <c r="C16" s="53" t="inlineStr">
+      <c r="C18" s="53" t="inlineStr">
         <is>
           <t>igus iglidur J plain bearing JSM-0507-05 5x7x5mm  -  83 pcs in stock; JFM-0507-05 flanged 1.48 USD alt</t>
         </is>
       </c>
-      <c r="D16" s="54" t="n">
+      <c r="D18" s="54" t="n">
         <v>2</v>
       </c>
-      <c r="E16" s="55" t="n">
+      <c r="E18" s="55" t="n">
         <v>1.18</v>
       </c>
-      <c r="F16" s="55" t="n">
+      <c r="F18" s="55" t="n">
         <v>2.36</v>
       </c>
     </row>
-    <row r="17" ht="15.5" customHeight="1">
-      <c r="A17" s="49" t="inlineStr">
+    <row r="19" ht="15.5" customHeight="1">
+      <c r="A19" s="49" t="inlineStr">
         <is>
           <t>A06</t>
         </is>
       </c>
-      <c r="B17" s="49" t="inlineStr">
+      <c r="B19" s="49" t="inlineStr">
         <is>
           <t>Set screw</t>
         </is>
       </c>
-      <c r="C17" s="6" t="inlineStr">
+      <c r="C19" s="6" t="inlineStr">
         <is>
           <t>M4x8 316SS cup point ISO 4029</t>
         </is>
       </c>
-      <c r="D17" s="50" t="n">
+      <c r="D19" s="50" t="n">
         <v>2</v>
       </c>
-      <c r="E17" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="F17" s="51" t="n">
+      <c r="E19" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="F19" s="51" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="45" t="inlineStr">
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="45" t="inlineStr">
         <is>
           <t>TECHFUN.SK</t>
         </is>
       </c>
-      <c r="F19" s="46" t="n">
+      <c r="F21" s="46" t="n">
         <v>94.45</v>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="47" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="47" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B20" s="47" t="inlineStr">
+      <c r="B22" s="47" t="inlineStr">
         <is>
           <t>Part</t>
         </is>
       </c>
-      <c r="C20" s="47" t="inlineStr">
+      <c r="C22" s="47" t="inlineStr">
         <is>
           <t>Specification / note</t>
         </is>
       </c>
-      <c r="D20" s="48" t="inlineStr">
+      <c r="D22" s="48" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="E20" s="48" t="inlineStr">
+      <c r="E22" s="48" t="inlineStr">
         <is>
           <t>Unit EUR</t>
         </is>
       </c>
-      <c r="F20" s="48" t="inlineStr">
+      <c r="F22" s="48" t="inlineStr">
         <is>
           <t>Total EUR</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="29" customHeight="1">
-      <c r="A21" s="49" t="inlineStr">
+    <row r="23" ht="29" customHeight="1">
+      <c r="A23" s="49" t="inlineStr">
         <is>
           <t>I01</t>
         </is>
       </c>
-      <c r="B21" s="49" t="inlineStr">
+      <c r="B23" s="49" t="inlineStr">
         <is>
           <t>Gateway radio (single-channel)</t>
         </is>
       </c>
-      <c r="C21" s="6" t="inlineStr">
+      <c r="C23" s="6" t="inlineStr">
         <is>
           <t>Wio-E5 mini = STM32WLE5JC + USB-C + CH340; plugs straight into RPi USB  -  druha Wio-E5 do USB na Raspberry Pi - bez nej nema kto prijimat</t>
         </is>
       </c>
-      <c r="D21" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="E21" s="51" t="n">
+      <c r="D23" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" s="51" t="n">
         <v>18</v>
       </c>
-      <c r="F21" s="51" t="n">
+      <c r="F23" s="51" t="n">
         <v>18</v>
-      </c>
-    </row>
-    <row r="22" ht="15.5" customHeight="1">
-      <c r="A22" s="52" t="inlineStr">
-        <is>
-          <t>J03</t>
-        </is>
-      </c>
-      <c r="B22" s="52" t="inlineStr">
-        <is>
-          <t>Epoxy barrier</t>
-        </is>
-      </c>
-      <c r="C22" s="53" t="inlineStr">
-        <is>
-          <t>West System 105 + 206</t>
-        </is>
-      </c>
-      <c r="D22" s="54" t="n">
-        <v>1</v>
-      </c>
-      <c r="E22" s="55" t="n">
-        <v>18</v>
-      </c>
-      <c r="F22" s="55" t="n">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="23" ht="42.5" customHeight="1">
-      <c r="A23" s="49" t="inlineStr">
-        <is>
-          <t>G03</t>
-        </is>
-      </c>
-      <c r="B23" s="49" t="inlineStr">
-        <is>
-          <t>MCU + radio (single board)</t>
-        </is>
-      </c>
-      <c r="C23" s="6" t="inlineStr">
-        <is>
-          <t>Seeed Wio-E5 mini: STM32WLE5JC Cortex-M4 + SX126x LoRa 868 MHz, USB-C, ADC/I2C/UART/GPIO  -  does EVERYTHING in the probe: sensors + LoRa + duty cycle. u.FL/SMA antenna connector - check which, both work</t>
-        </is>
-      </c>
-      <c r="D23" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="E23" s="51" t="n">
-        <v>15</v>
-      </c>
-      <c r="F23" s="51" t="n">
-        <v>15</v>
       </c>
     </row>
     <row r="24" ht="15.5" customHeight="1">
       <c r="A24" s="52" t="inlineStr">
         <is>
+          <t>J03</t>
+        </is>
+      </c>
+      <c r="B24" s="52" t="inlineStr">
+        <is>
+          <t>Epoxy barrier</t>
+        </is>
+      </c>
+      <c r="C24" s="53" t="inlineStr">
+        <is>
+          <t>West System 105 + 206</t>
+        </is>
+      </c>
+      <c r="D24" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" s="55" t="n">
+        <v>18</v>
+      </c>
+      <c r="F24" s="55" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="25" ht="42.5" customHeight="1">
+      <c r="A25" s="49" t="inlineStr">
+        <is>
+          <t>G03</t>
+        </is>
+      </c>
+      <c r="B25" s="49" t="inlineStr">
+        <is>
+          <t>MCU + radio (single board)</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>Seeed Wio-E5 mini: STM32WLE5JC Cortex-M4 + SX126x LoRa 868 MHz, USB-C, ADC/I2C/UART/GPIO  -  does EVERYTHING in the probe: sensors + LoRa + duty cycle. u.FL/SMA antenna connector - check which, both work</t>
+        </is>
+      </c>
+      <c r="D25" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" s="51" t="n">
+        <v>15</v>
+      </c>
+      <c r="F25" s="51" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="26" ht="15.5" customHeight="1">
+      <c r="A26" s="52" t="inlineStr">
+        <is>
           <t>B04</t>
         </is>
       </c>
-      <c r="B24" s="52" t="inlineStr">
+      <c r="B26" s="52" t="inlineStr">
         <is>
           <t>Potting compound</t>
         </is>
       </c>
-      <c r="C24" s="53" t="inlineStr">
+      <c r="C26" s="53" t="inlineStr">
         <is>
           <t>3M Scotch-Weld DP270 black 25ml</t>
         </is>
       </c>
-      <c r="D24" s="54" t="n">
-        <v>1</v>
-      </c>
-      <c r="E24" s="55" t="n">
+      <c r="D26" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" s="55" t="n">
         <v>14</v>
       </c>
-      <c r="F24" s="55" t="n">
+      <c r="F26" s="55" t="n">
         <v>14</v>
-      </c>
-    </row>
-    <row r="25" ht="15.5" customHeight="1">
-      <c r="A25" s="49" t="inlineStr">
-        <is>
-          <t>D07</t>
-        </is>
-      </c>
-      <c r="B25" s="49" t="inlineStr">
-        <is>
-          <t>Turbidity</t>
-        </is>
-      </c>
-      <c r="C25" s="6" t="inlineStr">
-        <is>
-          <t>DFRobot SEN0189 (0-4.5V analog)  -  6 in stock; in model as sensor_turb</t>
-        </is>
-      </c>
-      <c r="D25" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="E25" s="51" t="n">
-        <v>12.45</v>
-      </c>
-      <c r="F25" s="51" t="n">
-        <v>12.45</v>
-      </c>
-    </row>
-    <row r="26" ht="29" customHeight="1">
-      <c r="A26" s="52" t="inlineStr">
-        <is>
-          <t>G04</t>
-        </is>
-      </c>
-      <c r="B26" s="52" t="inlineStr">
-        <is>
-          <t>Antenna probe</t>
-        </is>
-      </c>
-      <c r="C26" s="53" t="inlineStr">
-        <is>
-          <t>868MHz 5dBi SMA-M omni 195mm  -  2 ks: jeden na sondu (SMA na doske), jeden na gateway</t>
-        </is>
-      </c>
-      <c r="D26" s="54" t="n">
-        <v>2</v>
-      </c>
-      <c r="E26" s="55" t="n">
-        <v>6</v>
-      </c>
-      <c r="F26" s="55" t="n">
-        <v>12</v>
       </c>
     </row>
     <row r="27" ht="15.5" customHeight="1">
       <c r="A27" s="49" t="inlineStr">
         <is>
+          <t>D07</t>
+        </is>
+      </c>
+      <c r="B27" s="49" t="inlineStr">
+        <is>
+          <t>Turbidity</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>DFRobot SEN0189 (0-4.5V analog)  -  6 in stock; in model as sensor_turb</t>
+        </is>
+      </c>
+      <c r="D27" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E27" s="51" t="n">
+        <v>12.45</v>
+      </c>
+      <c r="F27" s="51" t="n">
+        <v>12.45</v>
+      </c>
+    </row>
+    <row r="28" ht="29" customHeight="1">
+      <c r="A28" s="52" t="inlineStr">
+        <is>
+          <t>G04</t>
+        </is>
+      </c>
+      <c r="B28" s="52" t="inlineStr">
+        <is>
+          <t>Antenna probe</t>
+        </is>
+      </c>
+      <c r="C28" s="53" t="inlineStr">
+        <is>
+          <t>868MHz 5dBi SMA-M omni 195mm  -  2 ks: jeden na sondu (SMA na doske), jeden na gateway</t>
+        </is>
+      </c>
+      <c r="D28" s="54" t="n">
+        <v>2</v>
+      </c>
+      <c r="E28" s="55" t="n">
+        <v>6</v>
+      </c>
+      <c r="F28" s="55" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="29" ht="15.5" customHeight="1">
+      <c r="A29" s="49" t="inlineStr">
+        <is>
           <t>D04</t>
         </is>
       </c>
-      <c r="B27" s="49" t="inlineStr">
+      <c r="B29" s="49" t="inlineStr">
         <is>
           <t>Temperature</t>
         </is>
       </c>
-      <c r="C27" s="6" t="inlineStr">
+      <c r="C29" s="6" t="inlineStr">
         <is>
           <t>DS18B20 waterproof 1m cable  -  in model as sensor_ntc</t>
         </is>
       </c>
-      <c r="D27" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="E27" s="51" t="n">
+      <c r="D29" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" s="51" t="n">
         <v>5</v>
       </c>
-      <c r="F27" s="51" t="n">
+      <c r="F29" s="51" t="n">
         <v>5</v>
       </c>
     </row>
-    <row r="29" ht="20" customHeight="1">
-      <c r="A29" s="45" t="inlineStr">
+    <row r="31" ht="20" customHeight="1">
+      <c r="A31" s="45" t="inlineStr">
         <is>
           <t>LOCAL / SHOP</t>
         </is>
       </c>
-      <c r="F29" s="46" t="n">
+      <c r="F31" s="46" t="n">
         <v>9</v>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="47" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="47" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B30" s="47" t="inlineStr">
+      <c r="B32" s="47" t="inlineStr">
         <is>
           <t>Part</t>
         </is>
       </c>
-      <c r="C30" s="47" t="inlineStr">
+      <c r="C32" s="47" t="inlineStr">
         <is>
           <t>Specification / note</t>
         </is>
       </c>
-      <c r="D30" s="48" t="inlineStr">
+      <c r="D32" s="48" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="E30" s="48" t="inlineStr">
+      <c r="E32" s="48" t="inlineStr">
         <is>
           <t>Unit EUR</t>
         </is>
       </c>
-      <c r="F30" s="48" t="inlineStr">
+      <c r="F32" s="48" t="inlineStr">
         <is>
           <t>Total EUR</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="15.5" customHeight="1">
-      <c r="A31" s="49" t="inlineStr">
+    <row r="33" ht="15.5" customHeight="1">
+      <c r="A33" s="49" t="inlineStr">
         <is>
           <t>K03</t>
         </is>
       </c>
-      <c r="B31" s="49" t="inlineStr">
+      <c r="B33" s="49" t="inlineStr">
         <is>
           <t>Spring balance</t>
         </is>
       </c>
-      <c r="C31" s="6" t="inlineStr">
+      <c r="C33" s="6" t="inlineStr">
         <is>
           <t>0-5N for coupling slip jig  -  one-off</t>
         </is>
       </c>
-      <c r="D31" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="E31" s="51" t="n">
+      <c r="D33" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E33" s="51" t="n">
         <v>5</v>
       </c>
-      <c r="F31" s="51" t="n">
+      <c r="F33" s="51" t="n">
         <v>5</v>
       </c>
     </row>
-    <row r="32" ht="15.5" customHeight="1">
-      <c r="A32" s="52" t="inlineStr">
+    <row r="34" ht="15.5" customHeight="1">
+      <c r="A34" s="52" t="inlineStr">
         <is>
           <t>C06</t>
         </is>
       </c>
-      <c r="B32" s="52" t="inlineStr">
+      <c r="B34" s="52" t="inlineStr">
         <is>
           <t>Desiccant</t>
         </is>
       </c>
-      <c r="C32" s="53" t="inlineStr">
+      <c r="C34" s="53" t="inlineStr">
         <is>
           <t>5g silica gel with indicator  -  replace at service</t>
         </is>
       </c>
-      <c r="D32" s="54" t="n">
+      <c r="D34" s="54" t="n">
         <v>2</v>
       </c>
-      <c r="E32" s="55" t="n">
+      <c r="E34" s="55" t="n">
         <v>2</v>
       </c>
-      <c r="F32" s="55" t="n">
+      <c r="F34" s="55" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="33" ht="29" customHeight="1">
-      <c r="A33" s="49" t="inlineStr">
+    <row r="35" ht="29" customHeight="1">
+      <c r="A35" s="49" t="inlineStr">
         <is>
           <t>C04</t>
         </is>
       </c>
-      <c r="B33" s="49" t="inlineStr">
+      <c r="B35" s="49" t="inlineStr">
         <is>
           <t>O-ring groove</t>
         </is>
       </c>
-      <c r="C33" s="6" t="inlineStr">
+      <c r="C35" s="6" t="inlineStr">
         <is>
           <t>2.2mm wide x 1.8mm deep machined/printed into pod rim  -  NOT YET IN MODEL - add to pod</t>
         </is>
       </c>
-      <c r="D33" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="E33" s="51" t="n">
+      <c r="D35" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E35" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="F33" s="51" t="n">
+      <c r="F35" s="51" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="35" ht="20" customHeight="1">
-      <c r="A35" s="45" t="inlineStr">
+    <row r="37" ht="20" customHeight="1">
+      <c r="A37" s="45" t="inlineStr">
         <is>
           <t>MAGSY.SK</t>
         </is>
       </c>
-      <c r="F35" s="46" t="n">
+      <c r="F37" s="46" t="n">
         <v>8.800000000000001</v>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="47" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="47" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B36" s="47" t="inlineStr">
+      <c r="B38" s="47" t="inlineStr">
         <is>
           <t>Part</t>
         </is>
       </c>
-      <c r="C36" s="47" t="inlineStr">
+      <c r="C38" s="47" t="inlineStr">
         <is>
           <t>Specification / note</t>
         </is>
       </c>
-      <c r="D36" s="48" t="inlineStr">
+      <c r="D38" s="48" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="E36" s="48" t="inlineStr">
+      <c r="E38" s="48" t="inlineStr">
         <is>
           <t>Unit EUR</t>
         </is>
       </c>
-      <c r="F36" s="48" t="inlineStr">
+      <c r="F38" s="48" t="inlineStr">
         <is>
           <t>Total EUR</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="42.5" customHeight="1">
-      <c r="A37" s="49" t="inlineStr">
+    <row r="39" ht="42.5" customHeight="1">
+      <c r="A39" s="49" t="inlineStr">
         <is>
           <t>B01</t>
         </is>
       </c>
-      <c r="B37" s="49" t="inlineStr">
+      <c r="B39" s="49" t="inlineStr">
         <is>
           <t>Magnet</t>
         </is>
       </c>
-      <c r="C37" s="6" t="inlineStr">
+      <c r="C39" s="6" t="inlineStr">
         <is>
           <t>N52 D10x5 axially magnetised, canned 316L or epoxy potted  -  8 per cup, pitch r28 on D70 cup; price for D10 canned to re-verify; bare N52 must not touch water</t>
         </is>
       </c>
-      <c r="D37" s="50" t="n">
+      <c r="D39" s="50" t="n">
         <v>16</v>
       </c>
-      <c r="E37" s="51" t="n">
+      <c r="E39" s="51" t="n">
         <v>0.55</v>
       </c>
-      <c r="F37" s="51" t="n">
+      <c r="F39" s="51" t="n">
         <v>8.800000000000001</v>
       </c>
     </row>
-    <row r="39" ht="20" customHeight="1">
-      <c r="A39" s="45" t="inlineStr">
+    <row r="41" ht="20" customHeight="1">
+      <c r="A41" s="45" t="inlineStr">
         <is>
           <t>PRINTED IN-HOUSE</t>
         </is>
       </c>
-      <c r="F39" s="46" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="47" t="inlineStr">
+      <c r="F41" s="46" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="47" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B40" s="47" t="inlineStr">
+      <c r="B42" s="47" t="inlineStr">
         <is>
           <t>Part</t>
         </is>
       </c>
-      <c r="C40" s="47" t="inlineStr">
+      <c r="C42" s="47" t="inlineStr">
         <is>
           <t>Specification / note</t>
         </is>
       </c>
-      <c r="D40" s="48" t="inlineStr">
+      <c r="D42" s="48" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="E40" s="48" t="inlineStr">
+      <c r="E42" s="48" t="inlineStr">
         <is>
           <t>Unit EUR</t>
         </is>
       </c>
-      <c r="F40" s="48" t="inlineStr">
+      <c r="F42" s="48" t="inlineStr">
         <is>
           <t>Total EUR</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="15.5" customHeight="1">
-      <c r="A41" s="49" t="inlineStr">
+    <row r="43" ht="15.5" customHeight="1">
+      <c r="A43" s="49" t="inlineStr">
         <is>
           <t>C09</t>
         </is>
       </c>
-      <c r="B41" s="49" t="inlineStr">
+      <c r="B43" s="49" t="inlineStr">
         <is>
           <t>Generator mount</t>
         </is>
       </c>
-      <c r="C41" s="6" t="inlineStr">
+      <c r="C43" s="6" t="inlineStr">
         <is>
           <t>printed cradle + 4x M3x8 A4</t>
         </is>
       </c>
-      <c r="D41" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="E41" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="F41" s="51" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="42" ht="29" customHeight="1">
-      <c r="A42" s="52" t="inlineStr">
-        <is>
-          <t>A01</t>
-        </is>
-      </c>
-      <c r="B42" s="52" t="inlineStr">
-        <is>
-          <t>Blade</t>
-        </is>
-      </c>
-      <c r="C42" s="53" t="inlineStr">
-        <is>
-          <t>triple-blade rotor blade NACA4412 D220mm root pitch 28deg tip 2deg  -  ASA or ASA-CF; 6 perimeters; epoxy coat; spare blade = fuse for branch strike</t>
-        </is>
-      </c>
-      <c r="D42" s="54" t="n">
-        <v>3</v>
-      </c>
-      <c r="E42" s="55" t="n">
-        <v>0</v>
-      </c>
-      <c r="F42" s="55" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43" ht="29" customHeight="1">
-      <c r="A43" s="49" t="inlineStr">
-        <is>
-          <t>A02</t>
-        </is>
-      </c>
-      <c r="B43" s="49" t="inlineStr">
-        <is>
-          <t>Hub</t>
-        </is>
-      </c>
-      <c r="C43" s="6" t="inlineStr">
-        <is>
-          <t>Ø64x46mm with 2x M4 heat-set inserts and Ø5 H7 shaft bore  -  brass inserts M4 from TME</t>
-        </is>
-      </c>
       <c r="D43" s="50" t="n">
         <v>1</v>
       </c>
       <c r="E43" s="51" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F43" s="51" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="44" ht="29" customHeight="1">
       <c r="A44" s="52" t="inlineStr">
         <is>
-          <t>B02</t>
+          <t>A01</t>
         </is>
       </c>
       <c r="B44" s="52" t="inlineStr">
         <is>
-          <t>Magnet cup</t>
+          <t>Blade</t>
         </is>
       </c>
       <c r="C44" s="53" t="inlineStr">
         <is>
-          <t>D70 rim, 8 pockets D10.2x5.2, printed ASA  -  pockets 10.2 dia (magnet 10 + 0.2 glue), 0.2 mm epoxy recess</t>
+          <t>triple-blade rotor blade NACA4412 D220mm root pitch 28deg tip 2deg  -  ASA or ASA-CF; 6 perimeters; epoxy coat; spare blade = fuse for branch strike</t>
         </is>
       </c>
       <c r="D44" s="54" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E44" s="55" t="n">
         <v>0</v>
@@ -1716,20 +1716,20 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" ht="15.5" customHeight="1">
+    <row r="45" ht="29" customHeight="1">
       <c r="A45" s="49" t="inlineStr">
         <is>
-          <t>C01</t>
+          <t>A02</t>
         </is>
       </c>
       <c r="B45" s="49" t="inlineStr">
         <is>
-          <t>Pod barrel</t>
+          <t>Hub</t>
         </is>
       </c>
       <c r="C45" s="6" t="inlineStr">
         <is>
-          <t>Ø110x120mm printed ASA wall 2.4mm + epoxy barrier  -  in model as pod</t>
+          <t>Ø64x46mm with 2x M4 heat-set inserts and Ø5 H7 shaft bore  -  brass inserts M4 from TME</t>
         </is>
       </c>
       <c r="D45" s="50" t="n">
@@ -1742,24 +1742,24 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" ht="15.5" customHeight="1">
+    <row r="46" ht="29" customHeight="1">
       <c r="A46" s="52" t="inlineStr">
         <is>
-          <t>C02</t>
+          <t>B02</t>
         </is>
       </c>
       <c r="B46" s="52" t="inlineStr">
         <is>
-          <t>Tail cone</t>
+          <t>Magnet cup</t>
         </is>
       </c>
       <c r="C46" s="53" t="inlineStr">
         <is>
-          <t>printed integral</t>
+          <t>D70 rim, 8 pockets D10.2x5.2, printed ASA  -  pockets 10.2 dia (magnet 10 + 0.2 glue), 0.2 mm epoxy recess</t>
         </is>
       </c>
       <c r="D46" s="54" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E46" s="55" t="n">
         <v>0</v>
@@ -1771,17 +1771,17 @@
     <row r="47" ht="15.5" customHeight="1">
       <c r="A47" s="49" t="inlineStr">
         <is>
-          <t>E01</t>
+          <t>C01</t>
         </is>
       </c>
       <c r="B47" s="49" t="inlineStr">
         <is>
-          <t>Sensor cage</t>
+          <t>Pod barrel</t>
         </is>
       </c>
       <c r="C47" s="6" t="inlineStr">
         <is>
-          <t>Ø130x150 printed ASA 12 slots  -  in model as cage</t>
+          <t>Ø110x120mm printed ASA wall 2.4mm + epoxy barrier  -  in model as pod</t>
         </is>
       </c>
       <c r="D47" s="50" t="n">
@@ -1794,24 +1794,24 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" ht="29" customHeight="1">
+    <row r="48" ht="15.5" customHeight="1">
       <c r="A48" s="52" t="inlineStr">
         <is>
-          <t>E03</t>
+          <t>C02</t>
         </is>
       </c>
       <c r="B48" s="52" t="inlineStr">
         <is>
-          <t>Sensor holders</t>
+          <t>Tail cone</t>
         </is>
       </c>
       <c r="C48" s="53" t="inlineStr">
         <is>
-          <t>printed clips for pH/TDS/turbidity/NTC/MS5837  -  in model as sensor bodies</t>
+          <t>printed integral</t>
         </is>
       </c>
       <c r="D48" s="54" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E48" s="55" t="n">
         <v>0</v>
@@ -1820,177 +1820,189 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" ht="20" customHeight="1">
-      <c r="A50" s="45" t="inlineStr">
+    <row r="49" ht="15.5" customHeight="1">
+      <c r="A49" s="49" t="inlineStr">
+        <is>
+          <t>E01</t>
+        </is>
+      </c>
+      <c r="B49" s="49" t="inlineStr">
+        <is>
+          <t>Sensor cage</t>
+        </is>
+      </c>
+      <c r="C49" s="6" t="inlineStr">
+        <is>
+          <t>Ø130x150 printed ASA 12 slots  -  in model as cage</t>
+        </is>
+      </c>
+      <c r="D49" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E49" s="51" t="n">
+        <v>0</v>
+      </c>
+      <c r="F49" s="51" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" ht="29" customHeight="1">
+      <c r="A50" s="52" t="inlineStr">
+        <is>
+          <t>E03</t>
+        </is>
+      </c>
+      <c r="B50" s="52" t="inlineStr">
+        <is>
+          <t>Sensor holders</t>
+        </is>
+      </c>
+      <c r="C50" s="53" t="inlineStr">
+        <is>
+          <t>printed clips for pH/TDS/turbidity/NTC/MS5837  -  in model as sensor bodies</t>
+        </is>
+      </c>
+      <c r="D50" s="54" t="n">
+        <v>5</v>
+      </c>
+      <c r="E50" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="F50" s="55" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" ht="20" customHeight="1">
+      <c r="A52" s="45" t="inlineStr">
         <is>
           <t>NEREZMATERIAL.CZ</t>
         </is>
       </c>
-      <c r="F50" s="46" t="n">
+      <c r="F52" s="46" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="47" t="inlineStr">
+    <row r="53">
+      <c r="A53" s="47" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B51" s="47" t="inlineStr">
+      <c r="B53" s="47" t="inlineStr">
         <is>
           <t>Part</t>
         </is>
       </c>
-      <c r="C51" s="47" t="inlineStr">
+      <c r="C53" s="47" t="inlineStr">
         <is>
           <t>Specification / note</t>
         </is>
       </c>
-      <c r="D51" s="48" t="inlineStr">
+      <c r="D53" s="48" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="E51" s="48" t="inlineStr">
+      <c r="E53" s="48" t="inlineStr">
         <is>
           <t>Unit EUR</t>
         </is>
       </c>
-      <c r="F51" s="48" t="inlineStr">
+      <c r="F53" s="48" t="inlineStr">
         <is>
           <t>Total EUR</t>
         </is>
       </c>
     </row>
-    <row r="52" ht="29" customHeight="1">
-      <c r="A52" s="49" t="inlineStr">
+    <row r="54" ht="29" customHeight="1">
+      <c r="A54" s="49" t="inlineStr">
         <is>
           <t>B03</t>
         </is>
       </c>
-      <c r="B52" s="49" t="inlineStr">
+      <c r="B54" s="49" t="inlineStr">
         <is>
           <t>Separation wall</t>
         </is>
       </c>
-      <c r="C52" s="6" t="inlineStr">
+      <c r="C54" s="6" t="inlineStr">
         <is>
           <t>D106 x 4 mm - RECOMMENDED integral with the pod bulkhead (no separate part)  -  4 mm per CAD, not 5; integral removes O-ring C03 and screws C05</t>
         </is>
       </c>
-      <c r="D52" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="E52" s="51" t="n">
+      <c r="D54" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E54" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="F52" s="51" t="n">
+      <c r="F54" s="51" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="54" ht="18" customHeight="1">
-      <c r="A54" s="56" t="inlineStr">
+    <row r="56" ht="18" customHeight="1">
+      <c r="A56" s="56" t="inlineStr">
         <is>
           <t>GOODS</t>
         </is>
       </c>
-      <c r="F54" s="57" t="n">
-        <v>228.61</v>
-      </c>
-    </row>
-    <row r="55" ht="18" customHeight="1">
-      <c r="A55" s="56" t="inlineStr">
+      <c r="F56" s="57" t="n">
+        <v>234.61</v>
+      </c>
+    </row>
+    <row r="57" ht="18" customHeight="1">
+      <c r="A57" s="56" t="inlineStr">
         <is>
           <t>shipping, estimated</t>
         </is>
       </c>
-      <c r="F55" s="57" t="n">
+      <c r="F57" s="57" t="n">
         <v>25</v>
       </c>
     </row>
-    <row r="56" ht="22" customHeight="1">
-      <c r="A56" s="58" t="inlineStr">
+    <row r="58" ht="22" customHeight="1">
+      <c r="A58" s="58" t="inlineStr">
         <is>
           <t>LANDED TOTAL</t>
         </is>
       </c>
-      <c r="F56" s="59" t="n">
-        <v>253.61</v>
-      </c>
-    </row>
-    <row r="59" ht="22" customHeight="1">
-      <c r="A59" s="60" t="inlineStr">
+      <c r="F58" s="59" t="n">
+        <v>259.61</v>
+      </c>
+    </row>
+    <row r="61" ht="22" customHeight="1">
+      <c r="A61" s="60" t="inlineStr">
         <is>
           <t>NOT IN THIS ORDER</t>
         </is>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" s="61" t="inlineStr">
+    <row r="62">
+      <c r="A62" s="61" t="inlineStr">
         <is>
           <t>PHASE 2 - BUY LATER</t>
         </is>
       </c>
     </row>
-    <row r="61" ht="29" customHeight="1">
-      <c r="A61" s="62" t="inlineStr">
+    <row r="63" ht="29" customHeight="1">
+      <c r="A63" s="62" t="inlineStr">
         <is>
           <t>A03</t>
         </is>
       </c>
-      <c r="B61" s="62" t="inlineStr">
+      <c r="B63" s="62" t="inlineStr">
         <is>
           <t>Wet shaft</t>
         </is>
       </c>
-      <c r="C61" s="63" t="inlineStr">
+      <c r="C63" s="63" t="inlineStr">
         <is>
           <t>lokalny zeleziar / Hornbach M5 A4 srob - 4. obchod sa nerata, nema postu; 3m bar 63.1 CZK makes ~26 shafts</t>
         </is>
       </c>
-      <c r="E61" s="64" t="inlineStr">
+      <c r="E63" s="64" t="inlineStr">
         <is>
           <t>2.6</t>
-        </is>
-      </c>
-    </row>
-    <row r="62" ht="15.5" customHeight="1">
-      <c r="A62" s="62" t="inlineStr">
-        <is>
-          <t>C03</t>
-        </is>
-      </c>
-      <c r="B62" s="62" t="inlineStr">
-        <is>
-          <t>Pod O-ring</t>
-        </is>
-      </c>
-      <c r="C62" s="63" t="inlineStr">
-        <is>
-          <t>grease Molykote 111</t>
-        </is>
-      </c>
-      <c r="E62" s="64" t="inlineStr">
-        <is>
-          <t>3.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="63" ht="15.5" customHeight="1">
-      <c r="A63" s="62" t="inlineStr">
-        <is>
-          <t>C05</t>
-        </is>
-      </c>
-      <c r="B63" s="62" t="inlineStr">
-        <is>
-          <t>Pod clamp screws</t>
-        </is>
-      </c>
-      <c r="C63" s="63" t="inlineStr"/>
-      <c r="E63" s="64" t="inlineStr">
-        <is>
-          <t>3.0</t>
         </is>
       </c>
     </row>
@@ -3011,19 +3023,19 @@
     </row>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="A21:E21"/>
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A39:E39"/>
-    <mergeCell ref="A29:E29"/>
-    <mergeCell ref="A35:E35"/>
-    <mergeCell ref="A50:E50"/>
-    <mergeCell ref="A55:E55"/>
-    <mergeCell ref="A54:E54"/>
+    <mergeCell ref="A57:E57"/>
+    <mergeCell ref="A52:E52"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A19:E19"/>
+    <mergeCell ref="A41:E41"/>
+    <mergeCell ref="A61:F61"/>
     <mergeCell ref="A5:E5"/>
+    <mergeCell ref="A37:E37"/>
+    <mergeCell ref="A31:E31"/>
     <mergeCell ref="A3:F3"/>
+    <mergeCell ref="A58:E58"/>
     <mergeCell ref="A56:E56"/>
-    <mergeCell ref="A59:F59"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
@@ -4015,7 +4027,7 @@
       </c>
       <c r="L26" s="6" t="inlineStr">
         <is>
-          <t>grease Molykote 111</t>
+          <t>zadny spoj podu - bez neho sa pri ponoreni natecie</t>
         </is>
       </c>
     </row>
@@ -4125,7 +4137,11 @@
           <t>verified</t>
         </is>
       </c>
-      <c r="L28" s="6" t="inlineStr"/>
+      <c r="L28" s="6" t="inlineStr">
+        <is>
+          <t>drzi zadny spoj; integralny bulkhead riesi len prednu stranu</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">

</xml_diff>

<commit_message>
sourcing: the Wio-E5 is not in any CZ/SK shop, and the antenna ships with the board
- techfun returns zero products for wio-e5; laskakit carries RAK4630/4631, not
  Seeed. Verified by their own search pages, not assumed.
- G03 and I01 therefore point at Seeed direct (24 EUR) or OpenELAB EU; both
  marked quote, not verified.
- G04 and G05 drop out of the order: every Wio-E5 mini ships with an EU868
  antenna, and the board already has an SMA, so no pigtail unless the antenna
  is routed through a bulkhead.
- phase 1: 31 lines, 234.61 EUR goods
</commit_message>
<xml_diff>
--- a/docs/sub-mission_parts.xlsx
+++ b/docs/sub-mission_parts.xlsx
@@ -826,7 +826,7 @@
     <row r="3" ht="26" customHeight="1">
       <c r="A3" s="44" t="inlineStr">
         <is>
-          <t>33 lines      goods 234.61 EUR      shipping est. 25.00 EUR      LANDED 259.61 EUR</t>
+          <t>31 lines      goods 234.61 EUR      shipping est. 25.00 EUR      LANDED 259.61 EUR</t>
         </is>
       </c>
     </row>
@@ -837,7 +837,7 @@
         </is>
       </c>
       <c r="F5" s="46" t="n">
-        <v>121.36</v>
+        <v>118.36</v>
       </c>
     </row>
     <row r="6">
@@ -1135,579 +1135,579 @@
     <row r="17" ht="29" customHeight="1">
       <c r="A17" s="49" t="inlineStr">
         <is>
-          <t>G05</t>
+          <t>A04</t>
         </is>
       </c>
       <c r="B17" s="49" t="inlineStr">
         <is>
-          <t>Antenna pigtail</t>
+          <t>Wet bearing</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>u.FL to SMA bulkhead 15cm  -  u.FL -&gt; SMA pigtail; skip if your board ships with SMA already</t>
+          <t>igus iglidur J plain bearing JSM-0507-05 5x7x5mm  -  83 pcs in stock; JFM-0507-05 flanged 1.48 USD alt</t>
         </is>
       </c>
       <c r="D17" s="50" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E17" s="51" t="n">
-        <v>3</v>
+        <v>1.18</v>
       </c>
       <c r="F17" s="51" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="18" ht="29" customHeight="1">
+        <v>2.36</v>
+      </c>
+    </row>
+    <row r="18" ht="15.5" customHeight="1">
       <c r="A18" s="52" t="inlineStr">
         <is>
-          <t>A04</t>
+          <t>A06</t>
         </is>
       </c>
       <c r="B18" s="52" t="inlineStr">
         <is>
-          <t>Wet bearing</t>
+          <t>Set screw</t>
         </is>
       </c>
       <c r="C18" s="53" t="inlineStr">
         <is>
-          <t>igus iglidur J plain bearing JSM-0507-05 5x7x5mm  -  83 pcs in stock; JFM-0507-05 flanged 1.48 USD alt</t>
+          <t>M4x8 316SS cup point ISO 4029</t>
         </is>
       </c>
       <c r="D18" s="54" t="n">
         <v>2</v>
       </c>
       <c r="E18" s="55" t="n">
-        <v>1.18</v>
+        <v>1</v>
       </c>
       <c r="F18" s="55" t="n">
-        <v>2.36</v>
-      </c>
-    </row>
-    <row r="19" ht="15.5" customHeight="1">
-      <c r="A19" s="49" t="inlineStr">
-        <is>
-          <t>A06</t>
-        </is>
-      </c>
-      <c r="B19" s="49" t="inlineStr">
-        <is>
-          <t>Set screw</t>
-        </is>
-      </c>
-      <c r="C19" s="6" t="inlineStr">
-        <is>
-          <t>M4x8 316SS cup point ISO 4029</t>
-        </is>
-      </c>
-      <c r="D19" s="50" t="n">
         <v>2</v>
       </c>
-      <c r="E19" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="F19" s="51" t="n">
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="45" t="inlineStr">
+        <is>
+          <t>LOCAL / SHOP</t>
+        </is>
+      </c>
+      <c r="F20" s="46" t="n">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="47" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B21" s="47" t="inlineStr">
+        <is>
+          <t>Part</t>
+        </is>
+      </c>
+      <c r="C21" s="47" t="inlineStr">
+        <is>
+          <t>Specification / note</t>
+        </is>
+      </c>
+      <c r="D21" s="48" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="E21" s="48" t="inlineStr">
+        <is>
+          <t>Unit EUR</t>
+        </is>
+      </c>
+      <c r="F21" s="48" t="inlineStr">
+        <is>
+          <t>Total EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="42.5" customHeight="1">
+      <c r="A22" s="49" t="inlineStr">
+        <is>
+          <t>G03</t>
+        </is>
+      </c>
+      <c r="B22" s="49" t="inlineStr">
+        <is>
+          <t>MCU + radio (single board)</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>Seeed Wio-E5 mini: STM32WLE5JC Cortex-M4 + SX126x LoRa 868 MHz, USB-C, ADC/I2C/UART/GPIO  -  NIE je v techfun ani laskakit (overene 26.10.2026); Seeed $24.99, OpenELAB EU ~22.85; kazda doska obsahuje EU868 antenu</t>
+        </is>
+      </c>
+      <c r="D22" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" s="51" t="n">
+        <v>24</v>
+      </c>
+      <c r="F22" s="51" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="23" ht="42.5" customHeight="1">
+      <c r="A23" s="52" t="inlineStr">
+        <is>
+          <t>I01</t>
+        </is>
+      </c>
+      <c r="B23" s="52" t="inlineStr">
+        <is>
+          <t>Gateway radio (single-channel)</t>
+        </is>
+      </c>
+      <c r="C23" s="53" t="inlineStr">
+        <is>
+          <t>Wio-E5 mini = STM32WLE5JC + USB-C + CH340; plugs straight into RPi USB  -  NIE je v techfun ani laskakit (overene 26.10.2026); Seeed $24.99, OpenELAB EU ~22.85; kazda doska obsahuje EU868 antenu</t>
+        </is>
+      </c>
+      <c r="D23" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" s="55" t="n">
+        <v>24</v>
+      </c>
+      <c r="F23" s="55" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="24" ht="15.5" customHeight="1">
+      <c r="A24" s="49" t="inlineStr">
+        <is>
+          <t>K03</t>
+        </is>
+      </c>
+      <c r="B24" s="49" t="inlineStr">
+        <is>
+          <t>Spring balance</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>0-5N for coupling slip jig  -  one-off</t>
+        </is>
+      </c>
+      <c r="D24" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" s="51" t="n">
+        <v>5</v>
+      </c>
+      <c r="F24" s="51" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="25" ht="15.5" customHeight="1">
+      <c r="A25" s="52" t="inlineStr">
+        <is>
+          <t>C06</t>
+        </is>
+      </c>
+      <c r="B25" s="52" t="inlineStr">
+        <is>
+          <t>Desiccant</t>
+        </is>
+      </c>
+      <c r="C25" s="53" t="inlineStr">
+        <is>
+          <t>5g silica gel with indicator  -  replace at service</t>
+        </is>
+      </c>
+      <c r="D25" s="54" t="n">
         <v>2</v>
       </c>
-    </row>
-    <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="45" t="inlineStr">
+      <c r="E25" s="55" t="n">
+        <v>2</v>
+      </c>
+      <c r="F25" s="55" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="26" ht="29" customHeight="1">
+      <c r="A26" s="49" t="inlineStr">
+        <is>
+          <t>C04</t>
+        </is>
+      </c>
+      <c r="B26" s="49" t="inlineStr">
+        <is>
+          <t>O-ring groove</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>2.2mm wide x 1.8mm deep machined/printed into pod rim  -  NOT YET IN MODEL - add to pod</t>
+        </is>
+      </c>
+      <c r="D26" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" s="51" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" s="51" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" ht="20" customHeight="1">
+      <c r="A28" s="45" t="inlineStr">
         <is>
           <t>TECHFUN.SK</t>
         </is>
       </c>
-      <c r="F21" s="46" t="n">
-        <v>94.45</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="47" t="inlineStr">
+      <c r="F28" s="46" t="n">
+        <v>49.45</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="47" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B22" s="47" t="inlineStr">
+      <c r="B29" s="47" t="inlineStr">
         <is>
           <t>Part</t>
         </is>
       </c>
-      <c r="C22" s="47" t="inlineStr">
+      <c r="C29" s="47" t="inlineStr">
         <is>
           <t>Specification / note</t>
         </is>
       </c>
-      <c r="D22" s="48" t="inlineStr">
+      <c r="D29" s="48" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="E22" s="48" t="inlineStr">
+      <c r="E29" s="48" t="inlineStr">
         <is>
           <t>Unit EUR</t>
         </is>
       </c>
-      <c r="F22" s="48" t="inlineStr">
+      <c r="F29" s="48" t="inlineStr">
         <is>
           <t>Total EUR</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="29" customHeight="1">
-      <c r="A23" s="49" t="inlineStr">
-        <is>
-          <t>I01</t>
-        </is>
-      </c>
-      <c r="B23" s="49" t="inlineStr">
-        <is>
-          <t>Gateway radio (single-channel)</t>
-        </is>
-      </c>
-      <c r="C23" s="6" t="inlineStr">
-        <is>
-          <t>Wio-E5 mini = STM32WLE5JC + USB-C + CH340; plugs straight into RPi USB  -  druha Wio-E5 do USB na Raspberry Pi - bez nej nema kto prijimat</t>
-        </is>
-      </c>
-      <c r="D23" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="E23" s="51" t="n">
+    <row r="30" ht="15.5" customHeight="1">
+      <c r="A30" s="49" t="inlineStr">
+        <is>
+          <t>J03</t>
+        </is>
+      </c>
+      <c r="B30" s="49" t="inlineStr">
+        <is>
+          <t>Epoxy barrier</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>West System 105 + 206</t>
+        </is>
+      </c>
+      <c r="D30" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E30" s="51" t="n">
         <v>18</v>
       </c>
-      <c r="F23" s="51" t="n">
+      <c r="F30" s="51" t="n">
         <v>18</v>
       </c>
     </row>
-    <row r="24" ht="15.5" customHeight="1">
-      <c r="A24" s="52" t="inlineStr">
-        <is>
-          <t>J03</t>
-        </is>
-      </c>
-      <c r="B24" s="52" t="inlineStr">
-        <is>
-          <t>Epoxy barrier</t>
-        </is>
-      </c>
-      <c r="C24" s="53" t="inlineStr">
-        <is>
-          <t>West System 105 + 206</t>
-        </is>
-      </c>
-      <c r="D24" s="54" t="n">
-        <v>1</v>
-      </c>
-      <c r="E24" s="55" t="n">
-        <v>18</v>
-      </c>
-      <c r="F24" s="55" t="n">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="25" ht="42.5" customHeight="1">
-      <c r="A25" s="49" t="inlineStr">
-        <is>
-          <t>G03</t>
-        </is>
-      </c>
-      <c r="B25" s="49" t="inlineStr">
-        <is>
-          <t>MCU + radio (single board)</t>
-        </is>
-      </c>
-      <c r="C25" s="6" t="inlineStr">
-        <is>
-          <t>Seeed Wio-E5 mini: STM32WLE5JC Cortex-M4 + SX126x LoRa 868 MHz, USB-C, ADC/I2C/UART/GPIO  -  does EVERYTHING in the probe: sensors + LoRa + duty cycle. u.FL/SMA antenna connector - check which, both work</t>
-        </is>
-      </c>
-      <c r="D25" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="E25" s="51" t="n">
-        <v>15</v>
-      </c>
-      <c r="F25" s="51" t="n">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="26" ht="15.5" customHeight="1">
-      <c r="A26" s="52" t="inlineStr">
+    <row r="31" ht="15.5" customHeight="1">
+      <c r="A31" s="52" t="inlineStr">
         <is>
           <t>B04</t>
         </is>
       </c>
-      <c r="B26" s="52" t="inlineStr">
+      <c r="B31" s="52" t="inlineStr">
         <is>
           <t>Potting compound</t>
         </is>
       </c>
-      <c r="C26" s="53" t="inlineStr">
+      <c r="C31" s="53" t="inlineStr">
         <is>
           <t>3M Scotch-Weld DP270 black 25ml</t>
         </is>
       </c>
-      <c r="D26" s="54" t="n">
-        <v>1</v>
-      </c>
-      <c r="E26" s="55" t="n">
+      <c r="D31" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="E31" s="55" t="n">
         <v>14</v>
       </c>
-      <c r="F26" s="55" t="n">
+      <c r="F31" s="55" t="n">
         <v>14</v>
       </c>
     </row>
-    <row r="27" ht="15.5" customHeight="1">
-      <c r="A27" s="49" t="inlineStr">
+    <row r="32" ht="15.5" customHeight="1">
+      <c r="A32" s="49" t="inlineStr">
         <is>
           <t>D07</t>
         </is>
       </c>
-      <c r="B27" s="49" t="inlineStr">
+      <c r="B32" s="49" t="inlineStr">
         <is>
           <t>Turbidity</t>
         </is>
       </c>
-      <c r="C27" s="6" t="inlineStr">
+      <c r="C32" s="6" t="inlineStr">
         <is>
           <t>DFRobot SEN0189 (0-4.5V analog)  -  6 in stock; in model as sensor_turb</t>
         </is>
       </c>
-      <c r="D27" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="E27" s="51" t="n">
+      <c r="D32" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E32" s="51" t="n">
         <v>12.45</v>
       </c>
-      <c r="F27" s="51" t="n">
+      <c r="F32" s="51" t="n">
         <v>12.45</v>
       </c>
     </row>
-    <row r="28" ht="29" customHeight="1">
-      <c r="A28" s="52" t="inlineStr">
-        <is>
-          <t>G04</t>
-        </is>
-      </c>
-      <c r="B28" s="52" t="inlineStr">
-        <is>
-          <t>Antenna probe</t>
-        </is>
-      </c>
-      <c r="C28" s="53" t="inlineStr">
-        <is>
-          <t>868MHz 5dBi SMA-M omni 195mm  -  2 ks: jeden na sondu (SMA na doske), jeden na gateway</t>
-        </is>
-      </c>
-      <c r="D28" s="54" t="n">
-        <v>2</v>
-      </c>
-      <c r="E28" s="55" t="n">
-        <v>6</v>
-      </c>
-      <c r="F28" s="55" t="n">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="29" ht="15.5" customHeight="1">
-      <c r="A29" s="49" t="inlineStr">
+    <row r="33" ht="15.5" customHeight="1">
+      <c r="A33" s="52" t="inlineStr">
         <is>
           <t>D04</t>
         </is>
       </c>
-      <c r="B29" s="49" t="inlineStr">
+      <c r="B33" s="52" t="inlineStr">
         <is>
           <t>Temperature</t>
         </is>
       </c>
-      <c r="C29" s="6" t="inlineStr">
+      <c r="C33" s="53" t="inlineStr">
         <is>
           <t>DS18B20 waterproof 1m cable  -  in model as sensor_ntc</t>
         </is>
       </c>
-      <c r="D29" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="E29" s="51" t="n">
+      <c r="D33" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="E33" s="55" t="n">
         <v>5</v>
       </c>
-      <c r="F29" s="51" t="n">
+      <c r="F33" s="55" t="n">
         <v>5</v>
       </c>
     </row>
-    <row r="31" ht="20" customHeight="1">
-      <c r="A31" s="45" t="inlineStr">
-        <is>
-          <t>LOCAL / SHOP</t>
-        </is>
-      </c>
-      <c r="F31" s="46" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="47" t="inlineStr">
+    <row r="35" ht="20" customHeight="1">
+      <c r="A35" s="45" t="inlineStr">
+        <is>
+          <t>MAGSY.SK</t>
+        </is>
+      </c>
+      <c r="F35" s="46" t="n">
+        <v>8.800000000000001</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="47" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B32" s="47" t="inlineStr">
+      <c r="B36" s="47" t="inlineStr">
         <is>
           <t>Part</t>
         </is>
       </c>
-      <c r="C32" s="47" t="inlineStr">
+      <c r="C36" s="47" t="inlineStr">
         <is>
           <t>Specification / note</t>
         </is>
       </c>
-      <c r="D32" s="48" t="inlineStr">
+      <c r="D36" s="48" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="E32" s="48" t="inlineStr">
+      <c r="E36" s="48" t="inlineStr">
         <is>
           <t>Unit EUR</t>
         </is>
       </c>
-      <c r="F32" s="48" t="inlineStr">
+      <c r="F36" s="48" t="inlineStr">
         <is>
           <t>Total EUR</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="15.5" customHeight="1">
-      <c r="A33" s="49" t="inlineStr">
-        <is>
-          <t>K03</t>
-        </is>
-      </c>
-      <c r="B33" s="49" t="inlineStr">
-        <is>
-          <t>Spring balance</t>
-        </is>
-      </c>
-      <c r="C33" s="6" t="inlineStr">
-        <is>
-          <t>0-5N for coupling slip jig  -  one-off</t>
-        </is>
-      </c>
-      <c r="D33" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="E33" s="51" t="n">
-        <v>5</v>
-      </c>
-      <c r="F33" s="51" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="34" ht="15.5" customHeight="1">
-      <c r="A34" s="52" t="inlineStr">
-        <is>
-          <t>C06</t>
-        </is>
-      </c>
-      <c r="B34" s="52" t="inlineStr">
-        <is>
-          <t>Desiccant</t>
-        </is>
-      </c>
-      <c r="C34" s="53" t="inlineStr">
-        <is>
-          <t>5g silica gel with indicator  -  replace at service</t>
-        </is>
-      </c>
-      <c r="D34" s="54" t="n">
-        <v>2</v>
-      </c>
-      <c r="E34" s="55" t="n">
-        <v>2</v>
-      </c>
-      <c r="F34" s="55" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="35" ht="29" customHeight="1">
-      <c r="A35" s="49" t="inlineStr">
-        <is>
-          <t>C04</t>
-        </is>
-      </c>
-      <c r="B35" s="49" t="inlineStr">
-        <is>
-          <t>O-ring groove</t>
-        </is>
-      </c>
-      <c r="C35" s="6" t="inlineStr">
-        <is>
-          <t>2.2mm wide x 1.8mm deep machined/printed into pod rim  -  NOT YET IN MODEL - add to pod</t>
-        </is>
-      </c>
-      <c r="D35" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="E35" s="51" t="n">
+    <row r="37" ht="42.5" customHeight="1">
+      <c r="A37" s="49" t="inlineStr">
+        <is>
+          <t>B01</t>
+        </is>
+      </c>
+      <c r="B37" s="49" t="inlineStr">
+        <is>
+          <t>Magnet</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="inlineStr">
+        <is>
+          <t>N52 D10x5 axially magnetised, canned 316L or epoxy potted  -  8 per cup, pitch r28 on D70 cup; price for D10 canned to re-verify; bare N52 must not touch water</t>
+        </is>
+      </c>
+      <c r="D37" s="50" t="n">
+        <v>16</v>
+      </c>
+      <c r="E37" s="51" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="F37" s="51" t="n">
+        <v>8.800000000000001</v>
+      </c>
+    </row>
+    <row r="39" ht="20" customHeight="1">
+      <c r="A39" s="45" t="inlineStr">
+        <is>
+          <t>PRINTED IN-HOUSE</t>
+        </is>
+      </c>
+      <c r="F39" s="46" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="47" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B40" s="47" t="inlineStr">
+        <is>
+          <t>Part</t>
+        </is>
+      </c>
+      <c r="C40" s="47" t="inlineStr">
+        <is>
+          <t>Specification / note</t>
+        </is>
+      </c>
+      <c r="D40" s="48" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="E40" s="48" t="inlineStr">
+        <is>
+          <t>Unit EUR</t>
+        </is>
+      </c>
+      <c r="F40" s="48" t="inlineStr">
+        <is>
+          <t>Total EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="15.5" customHeight="1">
+      <c r="A41" s="49" t="inlineStr">
+        <is>
+          <t>C09</t>
+        </is>
+      </c>
+      <c r="B41" s="49" t="inlineStr">
+        <is>
+          <t>Generator mount</t>
+        </is>
+      </c>
+      <c r="C41" s="6" t="inlineStr">
+        <is>
+          <t>printed cradle + 4x M3x8 A4</t>
+        </is>
+      </c>
+      <c r="D41" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E41" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="F41" s="51" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" ht="29" customHeight="1">
+      <c r="A42" s="52" t="inlineStr">
+        <is>
+          <t>A01</t>
+        </is>
+      </c>
+      <c r="B42" s="52" t="inlineStr">
+        <is>
+          <t>Blade</t>
+        </is>
+      </c>
+      <c r="C42" s="53" t="inlineStr">
+        <is>
+          <t>triple-blade rotor blade NACA4412 D220mm root pitch 28deg tip 2deg  -  ASA or ASA-CF; 6 perimeters; epoxy coat; spare blade = fuse for branch strike</t>
+        </is>
+      </c>
+      <c r="D42" s="54" t="n">
+        <v>3</v>
+      </c>
+      <c r="E42" s="55" t="n">
         <v>0</v>
       </c>
-      <c r="F35" s="51" t="n">
+      <c r="F42" s="55" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="37" ht="20" customHeight="1">
-      <c r="A37" s="45" t="inlineStr">
-        <is>
-          <t>MAGSY.SK</t>
-        </is>
-      </c>
-      <c r="F37" s="46" t="n">
-        <v>8.800000000000001</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="47" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B38" s="47" t="inlineStr">
-        <is>
-          <t>Part</t>
-        </is>
-      </c>
-      <c r="C38" s="47" t="inlineStr">
-        <is>
-          <t>Specification / note</t>
-        </is>
-      </c>
-      <c r="D38" s="48" t="inlineStr">
-        <is>
-          <t>Qty</t>
-        </is>
-      </c>
-      <c r="E38" s="48" t="inlineStr">
-        <is>
-          <t>Unit EUR</t>
-        </is>
-      </c>
-      <c r="F38" s="48" t="inlineStr">
-        <is>
-          <t>Total EUR</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="42.5" customHeight="1">
-      <c r="A39" s="49" t="inlineStr">
-        <is>
-          <t>B01</t>
-        </is>
-      </c>
-      <c r="B39" s="49" t="inlineStr">
-        <is>
-          <t>Magnet</t>
-        </is>
-      </c>
-      <c r="C39" s="6" t="inlineStr">
-        <is>
-          <t>N52 D10x5 axially magnetised, canned 316L or epoxy potted  -  8 per cup, pitch r28 on D70 cup; price for D10 canned to re-verify; bare N52 must not touch water</t>
-        </is>
-      </c>
-      <c r="D39" s="50" t="n">
-        <v>16</v>
-      </c>
-      <c r="E39" s="51" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="F39" s="51" t="n">
-        <v>8.800000000000001</v>
-      </c>
-    </row>
-    <row r="41" ht="20" customHeight="1">
-      <c r="A41" s="45" t="inlineStr">
-        <is>
-          <t>PRINTED IN-HOUSE</t>
-        </is>
-      </c>
-      <c r="F41" s="46" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="47" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B42" s="47" t="inlineStr">
-        <is>
-          <t>Part</t>
-        </is>
-      </c>
-      <c r="C42" s="47" t="inlineStr">
-        <is>
-          <t>Specification / note</t>
-        </is>
-      </c>
-      <c r="D42" s="48" t="inlineStr">
-        <is>
-          <t>Qty</t>
-        </is>
-      </c>
-      <c r="E42" s="48" t="inlineStr">
-        <is>
-          <t>Unit EUR</t>
-        </is>
-      </c>
-      <c r="F42" s="48" t="inlineStr">
-        <is>
-          <t>Total EUR</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="15.5" customHeight="1">
+    <row r="43" ht="29" customHeight="1">
       <c r="A43" s="49" t="inlineStr">
         <is>
-          <t>C09</t>
+          <t>A02</t>
         </is>
       </c>
       <c r="B43" s="49" t="inlineStr">
         <is>
-          <t>Generator mount</t>
+          <t>Hub</t>
         </is>
       </c>
       <c r="C43" s="6" t="inlineStr">
         <is>
-          <t>printed cradle + 4x M3x8 A4</t>
+          <t>Ø64x46mm with 2x M4 heat-set inserts and Ø5 H7 shaft bore  -  brass inserts M4 from TME</t>
         </is>
       </c>
       <c r="D43" s="50" t="n">
         <v>1</v>
       </c>
       <c r="E43" s="51" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F43" s="51" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44" ht="29" customHeight="1">
       <c r="A44" s="52" t="inlineStr">
         <is>
-          <t>A01</t>
+          <t>B02</t>
         </is>
       </c>
       <c r="B44" s="52" t="inlineStr">
         <is>
-          <t>Blade</t>
+          <t>Magnet cup</t>
         </is>
       </c>
       <c r="C44" s="53" t="inlineStr">
         <is>
-          <t>triple-blade rotor blade NACA4412 D220mm root pitch 28deg tip 2deg  -  ASA or ASA-CF; 6 perimeters; epoxy coat; spare blade = fuse for branch strike</t>
+          <t>D70 rim, 8 pockets D10.2x5.2, printed ASA  -  pockets 10.2 dia (magnet 10 + 0.2 glue), 0.2 mm epoxy recess</t>
         </is>
       </c>
       <c r="D44" s="54" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E44" s="55" t="n">
         <v>0</v>
@@ -1716,20 +1716,20 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" ht="29" customHeight="1">
+    <row r="45" ht="15.5" customHeight="1">
       <c r="A45" s="49" t="inlineStr">
         <is>
-          <t>A02</t>
+          <t>C01</t>
         </is>
       </c>
       <c r="B45" s="49" t="inlineStr">
         <is>
-          <t>Hub</t>
+          <t>Pod barrel</t>
         </is>
       </c>
       <c r="C45" s="6" t="inlineStr">
         <is>
-          <t>Ø64x46mm with 2x M4 heat-set inserts and Ø5 H7 shaft bore  -  brass inserts M4 from TME</t>
+          <t>Ø110x120mm printed ASA wall 2.4mm + epoxy barrier  -  in model as pod</t>
         </is>
       </c>
       <c r="D45" s="50" t="n">
@@ -1742,24 +1742,24 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" ht="29" customHeight="1">
+    <row r="46" ht="15.5" customHeight="1">
       <c r="A46" s="52" t="inlineStr">
         <is>
-          <t>B02</t>
+          <t>C02</t>
         </is>
       </c>
       <c r="B46" s="52" t="inlineStr">
         <is>
-          <t>Magnet cup</t>
+          <t>Tail cone</t>
         </is>
       </c>
       <c r="C46" s="53" t="inlineStr">
         <is>
-          <t>D70 rim, 8 pockets D10.2x5.2, printed ASA  -  pockets 10.2 dia (magnet 10 + 0.2 glue), 0.2 mm epoxy recess</t>
+          <t>printed integral</t>
         </is>
       </c>
       <c r="D46" s="54" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E46" s="55" t="n">
         <v>0</v>
@@ -1771,17 +1771,17 @@
     <row r="47" ht="15.5" customHeight="1">
       <c r="A47" s="49" t="inlineStr">
         <is>
-          <t>C01</t>
+          <t>E01</t>
         </is>
       </c>
       <c r="B47" s="49" t="inlineStr">
         <is>
-          <t>Pod barrel</t>
+          <t>Sensor cage</t>
         </is>
       </c>
       <c r="C47" s="6" t="inlineStr">
         <is>
-          <t>Ø110x120mm printed ASA wall 2.4mm + epoxy barrier  -  in model as pod</t>
+          <t>Ø130x150 printed ASA 12 slots  -  in model as cage</t>
         </is>
       </c>
       <c r="D47" s="50" t="n">
@@ -1794,24 +1794,24 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" ht="15.5" customHeight="1">
+    <row r="48" ht="29" customHeight="1">
       <c r="A48" s="52" t="inlineStr">
         <is>
-          <t>C02</t>
+          <t>E03</t>
         </is>
       </c>
       <c r="B48" s="52" t="inlineStr">
         <is>
-          <t>Tail cone</t>
+          <t>Sensor holders</t>
         </is>
       </c>
       <c r="C48" s="53" t="inlineStr">
         <is>
-          <t>printed integral</t>
+          <t>printed clips for pH/TDS/turbidity/NTC/MS5837  -  in model as sensor bodies</t>
         </is>
       </c>
       <c r="D48" s="54" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E48" s="55" t="n">
         <v>0</v>
@@ -1820,361 +1820,353 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" ht="15.5" customHeight="1">
-      <c r="A49" s="49" t="inlineStr">
-        <is>
-          <t>E01</t>
-        </is>
-      </c>
-      <c r="B49" s="49" t="inlineStr">
-        <is>
-          <t>Sensor cage</t>
-        </is>
-      </c>
-      <c r="C49" s="6" t="inlineStr">
-        <is>
-          <t>Ø130x150 printed ASA 12 slots  -  in model as cage</t>
-        </is>
-      </c>
-      <c r="D49" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="E49" s="51" t="n">
+    <row r="50" ht="20" customHeight="1">
+      <c r="A50" s="45" t="inlineStr">
+        <is>
+          <t>NEREZMATERIAL.CZ</t>
+        </is>
+      </c>
+      <c r="F50" s="46" t="n">
         <v>0</v>
       </c>
-      <c r="F49" s="51" t="n">
+    </row>
+    <row r="51">
+      <c r="A51" s="47" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B51" s="47" t="inlineStr">
+        <is>
+          <t>Part</t>
+        </is>
+      </c>
+      <c r="C51" s="47" t="inlineStr">
+        <is>
+          <t>Specification / note</t>
+        </is>
+      </c>
+      <c r="D51" s="48" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="E51" s="48" t="inlineStr">
+        <is>
+          <t>Unit EUR</t>
+        </is>
+      </c>
+      <c r="F51" s="48" t="inlineStr">
+        <is>
+          <t>Total EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="29" customHeight="1">
+      <c r="A52" s="49" t="inlineStr">
+        <is>
+          <t>B03</t>
+        </is>
+      </c>
+      <c r="B52" s="49" t="inlineStr">
+        <is>
+          <t>Separation wall</t>
+        </is>
+      </c>
+      <c r="C52" s="6" t="inlineStr">
+        <is>
+          <t>D106 x 4 mm - RECOMMENDED integral with the pod bulkhead (no separate part)  -  4 mm per CAD, not 5; integral removes O-ring C03 and screws C05</t>
+        </is>
+      </c>
+      <c r="D52" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E52" s="51" t="n">
         <v>0</v>
       </c>
-    </row>
-    <row r="50" ht="29" customHeight="1">
-      <c r="A50" s="52" t="inlineStr">
-        <is>
-          <t>E03</t>
-        </is>
-      </c>
-      <c r="B50" s="52" t="inlineStr">
-        <is>
-          <t>Sensor holders</t>
-        </is>
-      </c>
-      <c r="C50" s="53" t="inlineStr">
-        <is>
-          <t>printed clips for pH/TDS/turbidity/NTC/MS5837  -  in model as sensor bodies</t>
-        </is>
-      </c>
-      <c r="D50" s="54" t="n">
-        <v>5</v>
-      </c>
-      <c r="E50" s="55" t="n">
+      <c r="F52" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="F50" s="55" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52" ht="20" customHeight="1">
-      <c r="A52" s="45" t="inlineStr">
-        <is>
-          <t>NEREZMATERIAL.CZ</t>
-        </is>
-      </c>
-      <c r="F52" s="46" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="47" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B53" s="47" t="inlineStr">
-        <is>
-          <t>Part</t>
-        </is>
-      </c>
-      <c r="C53" s="47" t="inlineStr">
-        <is>
-          <t>Specification / note</t>
-        </is>
-      </c>
-      <c r="D53" s="48" t="inlineStr">
-        <is>
-          <t>Qty</t>
-        </is>
-      </c>
-      <c r="E53" s="48" t="inlineStr">
-        <is>
-          <t>Unit EUR</t>
-        </is>
-      </c>
-      <c r="F53" s="48" t="inlineStr">
-        <is>
-          <t>Total EUR</t>
-        </is>
-      </c>
-    </row>
-    <row r="54" ht="29" customHeight="1">
-      <c r="A54" s="49" t="inlineStr">
-        <is>
-          <t>B03</t>
-        </is>
-      </c>
-      <c r="B54" s="49" t="inlineStr">
-        <is>
-          <t>Separation wall</t>
-        </is>
-      </c>
-      <c r="C54" s="6" t="inlineStr">
-        <is>
-          <t>D106 x 4 mm - RECOMMENDED integral with the pod bulkhead (no separate part)  -  4 mm per CAD, not 5; integral removes O-ring C03 and screws C05</t>
-        </is>
-      </c>
-      <c r="D54" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="E54" s="51" t="n">
-        <v>0</v>
-      </c>
-      <c r="F54" s="51" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="56" ht="18" customHeight="1">
-      <c r="A56" s="56" t="inlineStr">
+    </row>
+    <row r="54" ht="18" customHeight="1">
+      <c r="A54" s="56" t="inlineStr">
         <is>
           <t>GOODS</t>
         </is>
       </c>
-      <c r="F56" s="57" t="n">
+      <c r="F54" s="57" t="n">
         <v>234.61</v>
       </c>
     </row>
-    <row r="57" ht="18" customHeight="1">
-      <c r="A57" s="56" t="inlineStr">
+    <row r="55" ht="18" customHeight="1">
+      <c r="A55" s="56" t="inlineStr">
         <is>
           <t>shipping, estimated</t>
         </is>
       </c>
-      <c r="F57" s="57" t="n">
+      <c r="F55" s="57" t="n">
         <v>25</v>
       </c>
     </row>
-    <row r="58" ht="22" customHeight="1">
-      <c r="A58" s="58" t="inlineStr">
+    <row r="56" ht="22" customHeight="1">
+      <c r="A56" s="58" t="inlineStr">
         <is>
           <t>LANDED TOTAL</t>
         </is>
       </c>
-      <c r="F58" s="59" t="n">
+      <c r="F56" s="59" t="n">
         <v>259.61</v>
       </c>
     </row>
-    <row r="61" ht="22" customHeight="1">
-      <c r="A61" s="60" t="inlineStr">
+    <row r="59" ht="22" customHeight="1">
+      <c r="A59" s="60" t="inlineStr">
         <is>
           <t>NOT IN THIS ORDER</t>
         </is>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" s="61" t="inlineStr">
+    <row r="60">
+      <c r="A60" s="61" t="inlineStr">
         <is>
           <t>PHASE 2 - BUY LATER</t>
         </is>
       </c>
     </row>
-    <row r="63" ht="29" customHeight="1">
+    <row r="61" ht="29" customHeight="1">
+      <c r="A61" s="62" t="inlineStr">
+        <is>
+          <t>A03</t>
+        </is>
+      </c>
+      <c r="B61" s="62" t="inlineStr">
+        <is>
+          <t>Wet shaft</t>
+        </is>
+      </c>
+      <c r="C61" s="63" t="inlineStr">
+        <is>
+          <t>lokalny zeleziar / Hornbach M5 A4 srob - 4. obchod sa nerata, nema postu; 3m bar 63.1 CZK makes ~26 shafts</t>
+        </is>
+      </c>
+      <c r="E61" s="64" t="inlineStr">
+        <is>
+          <t>2.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="29" customHeight="1">
+      <c r="A62" s="62" t="inlineStr">
+        <is>
+          <t>C08</t>
+        </is>
+      </c>
+      <c r="B62" s="62" t="inlineStr">
+        <is>
+          <t>Generator</t>
+        </is>
+      </c>
+      <c r="C62" s="63" t="inlineStr">
+        <is>
+          <t>TEST BEZ GENERATORA: klietka + senzory stacia, generator je dalsi nakup; XTG3506 preferred: encoder = free RPM/flow</t>
+        </is>
+      </c>
+      <c r="E62" s="64" t="inlineStr">
+        <is>
+          <t>26.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="15.5" customHeight="1">
       <c r="A63" s="62" t="inlineStr">
         <is>
-          <t>A03</t>
+          <t>D01</t>
         </is>
       </c>
       <c r="B63" s="62" t="inlineStr">
         <is>
-          <t>Wet shaft</t>
+          <t>pH electrode</t>
         </is>
       </c>
       <c r="C63" s="63" t="inlineStr">
         <is>
-          <t>lokalny zeleziar / Hornbach M5 A4 srob - 4. obchod sa nerata, nema postu; 3m bar 63.1 CZK makes ~26 shafts</t>
+          <t>OPTIONAL per site; 14-30 day service; +-0.1 pH after 2-pt cal</t>
         </is>
       </c>
       <c r="E63" s="64" t="inlineStr">
         <is>
-          <t>2.6</t>
-        </is>
-      </c>
-    </row>
-    <row r="64" ht="29" customHeight="1">
+          <t>39.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="15.5" customHeight="1">
       <c r="A64" s="62" t="inlineStr">
         <is>
-          <t>C08</t>
+          <t>D02</t>
         </is>
       </c>
       <c r="B64" s="62" t="inlineStr">
         <is>
-          <t>Generator</t>
+          <t>pH spare electrode</t>
         </is>
       </c>
       <c r="C64" s="63" t="inlineStr">
         <is>
-          <t>TEST BEZ GENERATORA: klietka + senzory stacia, generator je dalsi nakup; XTG3506 preferred: encoder = free RPM/flow</t>
+          <t>consumable</t>
         </is>
       </c>
       <c r="E64" s="64" t="inlineStr">
         <is>
-          <t>26.0</t>
+          <t>9.0</t>
         </is>
       </c>
     </row>
     <row r="65" ht="15.5" customHeight="1">
       <c r="A65" s="62" t="inlineStr">
         <is>
-          <t>D01</t>
+          <t>D03</t>
         </is>
       </c>
       <c r="B65" s="62" t="inlineStr">
         <is>
-          <t>pH electrode</t>
+          <t>pH buffer</t>
         </is>
       </c>
       <c r="C65" s="63" t="inlineStr">
         <is>
-          <t>OPTIONAL per site; 14-30 day service; +-0.1 pH after 2-pt cal</t>
+          <t>consumable</t>
         </is>
       </c>
       <c r="E65" s="64" t="inlineStr">
         <is>
-          <t>39.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="66" ht="15.5" customHeight="1">
+          <t>12.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="29" customHeight="1">
       <c r="A66" s="62" t="inlineStr">
         <is>
-          <t>D02</t>
+          <t>D09</t>
         </is>
       </c>
       <c r="B66" s="62" t="inlineStr">
         <is>
-          <t>pH spare electrode</t>
+          <t>Dissolved oxygen kit</t>
         </is>
       </c>
       <c r="C66" s="63" t="inlineStr">
         <is>
-          <t>consumable</t>
+          <t>HIGHEST-VALUE channel (Budca = hypoxia); membrane 1-2 months in muddy water; 0.5M NaOH filling solution NOT shipped by air - source locally</t>
         </is>
       </c>
       <c r="E66" s="64" t="inlineStr">
         <is>
-          <t>9.0</t>
+          <t>175.0</t>
         </is>
       </c>
     </row>
     <row r="67" ht="15.5" customHeight="1">
       <c r="A67" s="62" t="inlineStr">
         <is>
-          <t>D03</t>
+          <t>D05</t>
         </is>
       </c>
       <c r="B67" s="62" t="inlineStr">
         <is>
-          <t>pH buffer</t>
+          <t>Level / stage probe</t>
         </is>
       </c>
       <c r="C67" s="63" t="inlineStr">
         <is>
-          <t>consumable</t>
+          <t>MS5837-30BA REJECTED: gel element must be dried daily, 24h max submersion</t>
         </is>
       </c>
       <c r="E67" s="64" t="inlineStr">
         <is>
-          <t>12.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="68" ht="29" customHeight="1">
+          <t>110.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="15.5" customHeight="1">
       <c r="A68" s="62" t="inlineStr">
         <is>
-          <t>D09</t>
+          <t>D06</t>
         </is>
       </c>
       <c r="B68" s="62" t="inlineStr">
         <is>
-          <t>Dissolved oxygen kit</t>
+          <t>EC/TDS</t>
         </is>
       </c>
       <c r="C68" s="63" t="inlineStr">
         <is>
-          <t>HIGHEST-VALUE channel (Budca = hypoxia); membrane 1-2 months in muddy water; 0.5M NaOH filling solution NOT shipped by air - source locally</t>
+          <t>+-10% FS is the weakest sensor; use as trend indicator, site-calibrate</t>
         </is>
       </c>
       <c r="E68" s="64" t="inlineStr">
         <is>
-          <t>175.0</t>
+          <t>14.0</t>
         </is>
       </c>
     </row>
     <row r="69" ht="15.5" customHeight="1">
       <c r="A69" s="62" t="inlineStr">
         <is>
-          <t>D05</t>
+          <t>D08</t>
         </is>
       </c>
       <c r="B69" s="62" t="inlineStr">
         <is>
-          <t>Level / stage probe</t>
-        </is>
-      </c>
-      <c r="C69" s="63" t="inlineStr">
-        <is>
-          <t>MS5837-30BA REJECTED: gel element must be dried daily, 24h max submersion</t>
-        </is>
-      </c>
+          <t>Sensor cable</t>
+        </is>
+      </c>
+      <c r="C69" s="63" t="inlineStr"/>
       <c r="E69" s="64" t="inlineStr">
         <is>
-          <t>110.0</t>
+          <t>20.0</t>
         </is>
       </c>
     </row>
     <row r="70" ht="15.5" customHeight="1">
       <c r="A70" s="62" t="inlineStr">
         <is>
-          <t>D06</t>
+          <t>G04</t>
         </is>
       </c>
       <c r="B70" s="62" t="inlineStr">
         <is>
-          <t>EC/TDS</t>
+          <t>Antenna probe</t>
         </is>
       </c>
       <c r="C70" s="63" t="inlineStr">
         <is>
-          <t>+-10% FS is the weakest sensor; use as trend indicator, site-calibrate</t>
+          <t>v baleni kazdej Wio-E5 je EU868 antena - samostatne netreba; drzat ako zalohu</t>
         </is>
       </c>
       <c r="E70" s="64" t="inlineStr">
         <is>
-          <t>14.0</t>
+          <t>6.0</t>
         </is>
       </c>
     </row>
     <row r="71" ht="15.5" customHeight="1">
       <c r="A71" s="62" t="inlineStr">
         <is>
-          <t>D08</t>
+          <t>G05</t>
         </is>
       </c>
       <c r="B71" s="62" t="inlineStr">
         <is>
-          <t>Sensor cable</t>
-        </is>
-      </c>
-      <c r="C71" s="63" t="inlineStr"/>
+          <t>Antenna pigtail</t>
+        </is>
+      </c>
+      <c r="C71" s="63" t="inlineStr">
+        <is>
+          <t>netreba: doska ma SMA, antena sa skrutkuje priamo; pigtail len ak sa ide cez bulkhead</t>
+        </is>
+      </c>
       <c r="E71" s="64" t="inlineStr">
         <is>
-          <t>20.0</t>
+          <t>3.0</t>
         </is>
       </c>
     </row>
@@ -3023,19 +3015,19 @@
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="A21:E21"/>
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A57:E57"/>
-    <mergeCell ref="A52:E52"/>
+    <mergeCell ref="A39:E39"/>
+    <mergeCell ref="A35:E35"/>
+    <mergeCell ref="A50:E50"/>
+    <mergeCell ref="A55:E55"/>
+    <mergeCell ref="A20:E20"/>
+    <mergeCell ref="A54:E54"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A41:E41"/>
-    <mergeCell ref="A61:F61"/>
+    <mergeCell ref="A28:E28"/>
     <mergeCell ref="A5:E5"/>
-    <mergeCell ref="A37:E37"/>
-    <mergeCell ref="A31:E31"/>
     <mergeCell ref="A3:F3"/>
-    <mergeCell ref="A58:E58"/>
     <mergeCell ref="A56:E56"/>
+    <mergeCell ref="A59:F59"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
@@ -5376,14 +5368,14 @@
       </c>
       <c r="E61" s="6" t="inlineStr">
         <is>
-          <t>techfun.sk</t>
+          <t>seeedstudio.com / openelab.io (EU)</t>
         </is>
       </c>
       <c r="F61" s="8" t="n">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="G61" s="8" t="n">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="H61" s="7" t="inlineStr">
         <is>
@@ -5402,12 +5394,12 @@
       </c>
       <c r="K61" s="5" t="inlineStr">
         <is>
-          <t>verified</t>
+          <t>quote</t>
         </is>
       </c>
       <c r="L61" s="6" t="inlineStr">
         <is>
-          <t>does EVERYTHING in the probe: sensors + LoRa + duty cycle. u.FL/SMA antenna connector - check which, both work</t>
+          <t>NIE je v techfun ani laskakit (overene 26.10.2026); Seeed $24.99, OpenELAB EU ~22.85; kazda doska obsahuje EU868 antenu</t>
         </is>
       </c>
     </row>
@@ -5428,7 +5420,7 @@
         </is>
       </c>
       <c r="D62" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E62" s="6" t="inlineStr">
         <is>
@@ -5439,7 +5431,7 @@
         <v>6</v>
       </c>
       <c r="G62" s="8" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="H62" s="7" t="inlineStr">
         <is>
@@ -5463,7 +5455,7 @@
       </c>
       <c r="L62" s="6" t="inlineStr">
         <is>
-          <t>2 ks: jeden na sondu (SMA na doske), jeden na gateway</t>
+          <t>v baleni kazdej Wio-E5 je EU868 antena - samostatne netreba; drzat ako zalohu</t>
         </is>
       </c>
     </row>
@@ -5484,7 +5476,7 @@
         </is>
       </c>
       <c r="D63" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E63" s="6" t="inlineStr">
         <is>
@@ -5495,7 +5487,7 @@
         <v>3</v>
       </c>
       <c r="G63" s="8" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H63" s="7" t="inlineStr">
         <is>
@@ -5519,7 +5511,7 @@
       </c>
       <c r="L63" s="6" t="inlineStr">
         <is>
-          <t>u.FL -&gt; SMA pigtail; skip if your board ships with SMA already</t>
+          <t>netreba: doska ma SMA, antena sa skrutkuje priamo; pigtail len ak sa ide cez bulkhead</t>
         </is>
       </c>
     </row>
@@ -6199,7 +6191,7 @@
       <c r="E76" s="68" t="n"/>
       <c r="F76" s="15" t="n"/>
       <c r="G76" s="15" t="n">
-        <v>112.9</v>
+        <v>106.9</v>
       </c>
       <c r="H76" s="14" t="n"/>
       <c r="I76" s="14" t="n"/>
@@ -6974,14 +6966,14 @@
       </c>
       <c r="E95" s="6" t="inlineStr">
         <is>
-          <t>techfun.sk</t>
+          <t>seeedstudio.com / openelab.io (EU)</t>
         </is>
       </c>
       <c r="F95" s="8" t="n">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G95" s="8" t="n">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="H95" s="7" t="inlineStr">
         <is>
@@ -7000,12 +6992,12 @@
       </c>
       <c r="K95" s="5" t="inlineStr">
         <is>
-          <t>verified</t>
+          <t>quote</t>
         </is>
       </c>
       <c r="L95" s="6" t="inlineStr">
         <is>
-          <t>single-channel Wio-E5 gateway: same radio as the probe, no concentrator needed | druha Wio-E5 do USB na Raspberry Pi - bez nej nema kto prijimat</t>
+          <t>single-channel Wio-E5 gateway: same radio as the probe, no concentrator needed | NIE je v techfun ani laskakit (overene 26.10.2026); Seeed $24.99, OpenELAB EU ~22.85; kazda doska obsahuje EU868 antenu</t>
         </is>
       </c>
     </row>
@@ -7297,7 +7289,7 @@
       <c r="E101" s="68" t="n"/>
       <c r="F101" s="15" t="n"/>
       <c r="G101" s="15" t="n">
-        <v>343</v>
+        <v>349</v>
       </c>
       <c r="H101" s="14" t="n"/>
       <c r="I101" s="14" t="n"/>
@@ -8211,7 +8203,7 @@
         </is>
       </c>
       <c r="B10" s="36" t="n">
-        <v>112.9</v>
+        <v>106.9</v>
       </c>
       <c r="C10" s="36" t="n">
         <v>0</v>
@@ -8243,7 +8235,7 @@
         </is>
       </c>
       <c r="B12" s="36" t="n">
-        <v>198</v>
+        <v>204</v>
       </c>
       <c r="C12" s="36" t="n">
         <v>145</v>

</xml_diff>

<commit_message>
sourcing: rpishop has the radio, so the boards stay in CZ
Searched the three shops properly instead of assuming:

- rpishop.cz stocks Seeed XIAO nRF52840 + Wio-SX1262 kits (SEE336, 349 Kc, 5+).
  That replaces the Wio-E5 mini, which no CZ/SK shop carries, and it is cheaper
  than importing one. G03 and I01 now point there.
- techfun.sk: turbidity and DS18B20 confirmed in stock, and they do carry N52
  round magnets (size to check). No Wio-E5, no DP270, no West System.
- laskakit.cz: RAK4630/4631 WisBlock + Meshtastic, no Seeed.
- TME stays for the bushings, glands, box, cable, O-ring and fasteners: none of
  the three maker shops carry igus or submersible cable.

phase 1: 31 lines, 214.61 EUR goods
</commit_message>
<xml_diff>
--- a/docs/sub-mission_parts.xlsx
+++ b/docs/sub-mission_parts.xlsx
@@ -798,7 +798,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F113"/>
+  <dimension ref="A1:F110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -826,7 +826,7 @@
     <row r="3" ht="26" customHeight="1">
       <c r="A3" s="44" t="inlineStr">
         <is>
-          <t>31 lines      goods 234.61 EUR      shipping est. 25.00 EUR      LANDED 259.61 EUR</t>
+          <t>31 lines      goods 214.61 EUR      shipping est. 25.00 EUR      LANDED 239.61 EUR</t>
         </is>
       </c>
     </row>
@@ -1187,11 +1187,11 @@
     <row r="20" ht="20" customHeight="1">
       <c r="A20" s="45" t="inlineStr">
         <is>
-          <t>LOCAL / SHOP</t>
+          <t>TECHFUN.SK</t>
         </is>
       </c>
       <c r="F20" s="46" t="n">
-        <v>57</v>
+        <v>58.25</v>
       </c>
     </row>
     <row r="21">
@@ -1226,144 +1226,144 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="42.5" customHeight="1">
+    <row r="22" ht="15.5" customHeight="1">
       <c r="A22" s="49" t="inlineStr">
         <is>
-          <t>G03</t>
+          <t>J03</t>
         </is>
       </c>
       <c r="B22" s="49" t="inlineStr">
         <is>
-          <t>MCU + radio (single board)</t>
+          <t>Epoxy barrier</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>Seeed Wio-E5 mini: STM32WLE5JC Cortex-M4 + SX126x LoRa 868 MHz, USB-C, ADC/I2C/UART/GPIO  -  NIE je v techfun ani laskakit (overene 26.10.2026); Seeed $24.99, OpenELAB EU ~22.85; kazda doska obsahuje EU868 antenu</t>
+          <t>West System 105 + 206</t>
         </is>
       </c>
       <c r="D22" s="50" t="n">
         <v>1</v>
       </c>
       <c r="E22" s="51" t="n">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="F22" s="51" t="n">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="23" ht="42.5" customHeight="1">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="23" ht="15.5" customHeight="1">
       <c r="A23" s="52" t="inlineStr">
         <is>
-          <t>I01</t>
+          <t>B04</t>
         </is>
       </c>
       <c r="B23" s="52" t="inlineStr">
         <is>
-          <t>Gateway radio (single-channel)</t>
+          <t>Potting compound</t>
         </is>
       </c>
       <c r="C23" s="53" t="inlineStr">
         <is>
-          <t>Wio-E5 mini = STM32WLE5JC + USB-C + CH340; plugs straight into RPi USB  -  NIE je v techfun ani laskakit (overene 26.10.2026); Seeed $24.99, OpenELAB EU ~22.85; kazda doska obsahuje EU868 antenu</t>
+          <t>3M Scotch-Weld DP270 black 25ml</t>
         </is>
       </c>
       <c r="D23" s="54" t="n">
         <v>1</v>
       </c>
       <c r="E23" s="55" t="n">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F23" s="55" t="n">
-        <v>24</v>
+        <v>14</v>
       </c>
     </row>
     <row r="24" ht="15.5" customHeight="1">
       <c r="A24" s="49" t="inlineStr">
         <is>
-          <t>K03</t>
+          <t>D07</t>
         </is>
       </c>
       <c r="B24" s="49" t="inlineStr">
         <is>
-          <t>Spring balance</t>
+          <t>Turbidity</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>0-5N for coupling slip jig  -  one-off</t>
+          <t>DFRobot SEN0189 (0-4.5V analog)  -  6 in stock; in model as sensor_turb</t>
         </is>
       </c>
       <c r="D24" s="50" t="n">
         <v>1</v>
       </c>
       <c r="E24" s="51" t="n">
+        <v>12.45</v>
+      </c>
+      <c r="F24" s="51" t="n">
+        <v>12.45</v>
+      </c>
+    </row>
+    <row r="25" ht="29" customHeight="1">
+      <c r="A25" s="52" t="inlineStr">
+        <is>
+          <t>B01</t>
+        </is>
+      </c>
+      <c r="B25" s="52" t="inlineStr">
+        <is>
+          <t>Magnet</t>
+        </is>
+      </c>
+      <c r="C25" s="53" t="inlineStr">
+        <is>
+          <t>N52 D10x5 axially magnetised, canned 316L or epoxy potted  -  techfun ma N52 magnet kruhovy - over priemer; inak magsy.sk; 8 na kapsu, D10</t>
+        </is>
+      </c>
+      <c r="D25" s="54" t="n">
+        <v>16</v>
+      </c>
+      <c r="E25" s="55" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="F25" s="55" t="n">
+        <v>8.800000000000001</v>
+      </c>
+    </row>
+    <row r="26" ht="15.5" customHeight="1">
+      <c r="A26" s="49" t="inlineStr">
+        <is>
+          <t>D04</t>
+        </is>
+      </c>
+      <c r="B26" s="49" t="inlineStr">
+        <is>
+          <t>Temperature</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>DS18B20 waterproof 1m cable  -  in model as sensor_ntc</t>
+        </is>
+      </c>
+      <c r="D26" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" s="51" t="n">
         <v>5</v>
       </c>
-      <c r="F24" s="51" t="n">
+      <c r="F26" s="51" t="n">
         <v>5</v>
-      </c>
-    </row>
-    <row r="25" ht="15.5" customHeight="1">
-      <c r="A25" s="52" t="inlineStr">
-        <is>
-          <t>C06</t>
-        </is>
-      </c>
-      <c r="B25" s="52" t="inlineStr">
-        <is>
-          <t>Desiccant</t>
-        </is>
-      </c>
-      <c r="C25" s="53" t="inlineStr">
-        <is>
-          <t>5g silica gel with indicator  -  replace at service</t>
-        </is>
-      </c>
-      <c r="D25" s="54" t="n">
-        <v>2</v>
-      </c>
-      <c r="E25" s="55" t="n">
-        <v>2</v>
-      </c>
-      <c r="F25" s="55" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="26" ht="29" customHeight="1">
-      <c r="A26" s="49" t="inlineStr">
-        <is>
-          <t>C04</t>
-        </is>
-      </c>
-      <c r="B26" s="49" t="inlineStr">
-        <is>
-          <t>O-ring groove</t>
-        </is>
-      </c>
-      <c r="C26" s="6" t="inlineStr">
-        <is>
-          <t>2.2mm wide x 1.8mm deep machined/printed into pod rim  -  NOT YET IN MODEL - add to pod</t>
-        </is>
-      </c>
-      <c r="D26" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="E26" s="51" t="n">
-        <v>0</v>
-      </c>
-      <c r="F26" s="51" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="28" ht="20" customHeight="1">
       <c r="A28" s="45" t="inlineStr">
         <is>
-          <t>TECHFUN.SK</t>
+          <t>LOCAL / SHOP</t>
         </is>
       </c>
       <c r="F28" s="46" t="n">
-        <v>49.45</v>
+        <v>37</v>
       </c>
     </row>
     <row r="29">
@@ -1398,46 +1398,46 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="15.5" customHeight="1">
+    <row r="30" ht="42.5" customHeight="1">
       <c r="A30" s="49" t="inlineStr">
         <is>
-          <t>J03</t>
+          <t>G03</t>
         </is>
       </c>
       <c r="B30" s="49" t="inlineStr">
         <is>
-          <t>Epoxy barrier</t>
+          <t>MCU + radio (single board)</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>West System 105 + 206</t>
+          <t>Seeed XIAO nRF52840 + Wio-SX1262 kit (Meshtastic), SEE336 - nRF52840 + SX1262  -  349 Kc, skladom 5+; nahradza Wio-E5, ktory v CZ/SK nie je; antena je v kite</t>
         </is>
       </c>
       <c r="D30" s="50" t="n">
         <v>1</v>
       </c>
       <c r="E30" s="51" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="F30" s="51" t="n">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="31" ht="15.5" customHeight="1">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="31" ht="42.5" customHeight="1">
       <c r="A31" s="52" t="inlineStr">
         <is>
-          <t>B04</t>
+          <t>I01</t>
         </is>
       </c>
       <c r="B31" s="52" t="inlineStr">
         <is>
-          <t>Potting compound</t>
+          <t>Gateway radio (single-channel)</t>
         </is>
       </c>
       <c r="C31" s="53" t="inlineStr">
         <is>
-          <t>3M Scotch-Weld DP270 black 25ml</t>
+          <t>Seeed XIAO nRF52840 + Wio-SX1262 kit (Meshtastic), SEE336 - nRF52840 + SX1262  -  349 Kc, skladom 5+; nahradza Wio-E5, ktory v CZ/SK nie je; antena je v kite</t>
         </is>
       </c>
       <c r="D31" s="54" t="n">
@@ -1453,1581 +1453,1538 @@
     <row r="32" ht="15.5" customHeight="1">
       <c r="A32" s="49" t="inlineStr">
         <is>
-          <t>D07</t>
+          <t>K03</t>
         </is>
       </c>
       <c r="B32" s="49" t="inlineStr">
         <is>
-          <t>Turbidity</t>
+          <t>Spring balance</t>
         </is>
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>DFRobot SEN0189 (0-4.5V analog)  -  6 in stock; in model as sensor_turb</t>
+          <t>0-5N for coupling slip jig  -  one-off</t>
         </is>
       </c>
       <c r="D32" s="50" t="n">
         <v>1</v>
       </c>
       <c r="E32" s="51" t="n">
-        <v>12.45</v>
+        <v>5</v>
       </c>
       <c r="F32" s="51" t="n">
-        <v>12.45</v>
+        <v>5</v>
       </c>
     </row>
     <row r="33" ht="15.5" customHeight="1">
       <c r="A33" s="52" t="inlineStr">
         <is>
-          <t>D04</t>
+          <t>C06</t>
         </is>
       </c>
       <c r="B33" s="52" t="inlineStr">
         <is>
-          <t>Temperature</t>
+          <t>Desiccant</t>
         </is>
       </c>
       <c r="C33" s="53" t="inlineStr">
         <is>
-          <t>DS18B20 waterproof 1m cable  -  in model as sensor_ntc</t>
+          <t>5g silica gel with indicator  -  replace at service</t>
         </is>
       </c>
       <c r="D33" s="54" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E33" s="55" t="n">
+        <v>2</v>
+      </c>
+      <c r="F33" s="55" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="34" ht="29" customHeight="1">
+      <c r="A34" s="49" t="inlineStr">
+        <is>
+          <t>C04</t>
+        </is>
+      </c>
+      <c r="B34" s="49" t="inlineStr">
+        <is>
+          <t>O-ring groove</t>
+        </is>
+      </c>
+      <c r="C34" s="6" t="inlineStr">
+        <is>
+          <t>2.2mm wide x 1.8mm deep machined/printed into pod rim  -  NOT YET IN MODEL - add to pod</t>
+        </is>
+      </c>
+      <c r="D34" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E34" s="51" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" s="51" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" ht="20" customHeight="1">
+      <c r="A36" s="45" t="inlineStr">
+        <is>
+          <t>PRINTED IN-HOUSE</t>
+        </is>
+      </c>
+      <c r="F36" s="46" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="47" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B37" s="47" t="inlineStr">
+        <is>
+          <t>Part</t>
+        </is>
+      </c>
+      <c r="C37" s="47" t="inlineStr">
+        <is>
+          <t>Specification / note</t>
+        </is>
+      </c>
+      <c r="D37" s="48" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="E37" s="48" t="inlineStr">
+        <is>
+          <t>Unit EUR</t>
+        </is>
+      </c>
+      <c r="F37" s="48" t="inlineStr">
+        <is>
+          <t>Total EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="15.5" customHeight="1">
+      <c r="A38" s="49" t="inlineStr">
+        <is>
+          <t>C09</t>
+        </is>
+      </c>
+      <c r="B38" s="49" t="inlineStr">
+        <is>
+          <t>Generator mount</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="inlineStr">
+        <is>
+          <t>printed cradle + 4x M3x8 A4</t>
+        </is>
+      </c>
+      <c r="D38" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E38" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="F38" s="51" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" ht="29" customHeight="1">
+      <c r="A39" s="52" t="inlineStr">
+        <is>
+          <t>A01</t>
+        </is>
+      </c>
+      <c r="B39" s="52" t="inlineStr">
+        <is>
+          <t>Blade</t>
+        </is>
+      </c>
+      <c r="C39" s="53" t="inlineStr">
+        <is>
+          <t>triple-blade rotor blade NACA4412 D220mm root pitch 28deg tip 2deg  -  ASA or ASA-CF; 6 perimeters; epoxy coat; spare blade = fuse for branch strike</t>
+        </is>
+      </c>
+      <c r="D39" s="54" t="n">
+        <v>3</v>
+      </c>
+      <c r="E39" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="F39" s="55" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" ht="29" customHeight="1">
+      <c r="A40" s="49" t="inlineStr">
+        <is>
+          <t>A02</t>
+        </is>
+      </c>
+      <c r="B40" s="49" t="inlineStr">
+        <is>
+          <t>Hub</t>
+        </is>
+      </c>
+      <c r="C40" s="6" t="inlineStr">
+        <is>
+          <t>Ø64x46mm with 2x M4 heat-set inserts and Ø5 H7 shaft bore  -  brass inserts M4 from TME</t>
+        </is>
+      </c>
+      <c r="D40" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E40" s="51" t="n">
+        <v>0</v>
+      </c>
+      <c r="F40" s="51" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" ht="29" customHeight="1">
+      <c r="A41" s="52" t="inlineStr">
+        <is>
+          <t>B02</t>
+        </is>
+      </c>
+      <c r="B41" s="52" t="inlineStr">
+        <is>
+          <t>Magnet cup</t>
+        </is>
+      </c>
+      <c r="C41" s="53" t="inlineStr">
+        <is>
+          <t>D70 rim, 8 pockets D10.2x5.2, printed ASA  -  pockets 10.2 dia (magnet 10 + 0.2 glue), 0.2 mm epoxy recess</t>
+        </is>
+      </c>
+      <c r="D41" s="54" t="n">
+        <v>2</v>
+      </c>
+      <c r="E41" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="F41" s="55" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" ht="15.5" customHeight="1">
+      <c r="A42" s="49" t="inlineStr">
+        <is>
+          <t>C01</t>
+        </is>
+      </c>
+      <c r="B42" s="49" t="inlineStr">
+        <is>
+          <t>Pod barrel</t>
+        </is>
+      </c>
+      <c r="C42" s="6" t="inlineStr">
+        <is>
+          <t>Ø110x120mm printed ASA wall 2.4mm + epoxy barrier  -  in model as pod</t>
+        </is>
+      </c>
+      <c r="D42" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E42" s="51" t="n">
+        <v>0</v>
+      </c>
+      <c r="F42" s="51" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" ht="15.5" customHeight="1">
+      <c r="A43" s="52" t="inlineStr">
+        <is>
+          <t>C02</t>
+        </is>
+      </c>
+      <c r="B43" s="52" t="inlineStr">
+        <is>
+          <t>Tail cone</t>
+        </is>
+      </c>
+      <c r="C43" s="53" t="inlineStr">
+        <is>
+          <t>printed integral</t>
+        </is>
+      </c>
+      <c r="D43" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="E43" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="F43" s="55" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" ht="15.5" customHeight="1">
+      <c r="A44" s="49" t="inlineStr">
+        <is>
+          <t>E01</t>
+        </is>
+      </c>
+      <c r="B44" s="49" t="inlineStr">
+        <is>
+          <t>Sensor cage</t>
+        </is>
+      </c>
+      <c r="C44" s="6" t="inlineStr">
+        <is>
+          <t>Ø130x150 printed ASA 12 slots  -  in model as cage</t>
+        </is>
+      </c>
+      <c r="D44" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E44" s="51" t="n">
+        <v>0</v>
+      </c>
+      <c r="F44" s="51" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" ht="29" customHeight="1">
+      <c r="A45" s="52" t="inlineStr">
+        <is>
+          <t>E03</t>
+        </is>
+      </c>
+      <c r="B45" s="52" t="inlineStr">
+        <is>
+          <t>Sensor holders</t>
+        </is>
+      </c>
+      <c r="C45" s="53" t="inlineStr">
+        <is>
+          <t>printed clips for pH/TDS/turbidity/NTC/MS5837  -  in model as sensor bodies</t>
+        </is>
+      </c>
+      <c r="D45" s="54" t="n">
         <v>5</v>
       </c>
-      <c r="F33" s="55" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="35" ht="20" customHeight="1">
-      <c r="A35" s="45" t="inlineStr">
-        <is>
-          <t>MAGSY.SK</t>
-        </is>
-      </c>
-      <c r="F35" s="46" t="n">
-        <v>8.800000000000001</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="47" t="inlineStr">
+      <c r="E45" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="F45" s="55" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" ht="20" customHeight="1">
+      <c r="A47" s="45" t="inlineStr">
+        <is>
+          <t>NEREZMATERIAL.CZ</t>
+        </is>
+      </c>
+      <c r="F47" s="46" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="47" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B36" s="47" t="inlineStr">
+      <c r="B48" s="47" t="inlineStr">
         <is>
           <t>Part</t>
         </is>
       </c>
-      <c r="C36" s="47" t="inlineStr">
+      <c r="C48" s="47" t="inlineStr">
         <is>
           <t>Specification / note</t>
         </is>
       </c>
-      <c r="D36" s="48" t="inlineStr">
+      <c r="D48" s="48" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="E36" s="48" t="inlineStr">
+      <c r="E48" s="48" t="inlineStr">
         <is>
           <t>Unit EUR</t>
         </is>
       </c>
-      <c r="F36" s="48" t="inlineStr">
+      <c r="F48" s="48" t="inlineStr">
         <is>
           <t>Total EUR</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="42.5" customHeight="1">
-      <c r="A37" s="49" t="inlineStr">
-        <is>
-          <t>B01</t>
-        </is>
-      </c>
-      <c r="B37" s="49" t="inlineStr">
-        <is>
-          <t>Magnet</t>
-        </is>
-      </c>
-      <c r="C37" s="6" t="inlineStr">
-        <is>
-          <t>N52 D10x5 axially magnetised, canned 316L or epoxy potted  -  8 per cup, pitch r28 on D70 cup; price for D10 canned to re-verify; bare N52 must not touch water</t>
-        </is>
-      </c>
-      <c r="D37" s="50" t="n">
-        <v>16</v>
-      </c>
-      <c r="E37" s="51" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="F37" s="51" t="n">
-        <v>8.800000000000001</v>
-      </c>
-    </row>
-    <row r="39" ht="20" customHeight="1">
-      <c r="A39" s="45" t="inlineStr">
-        <is>
-          <t>PRINTED IN-HOUSE</t>
-        </is>
-      </c>
-      <c r="F39" s="46" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="47" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B40" s="47" t="inlineStr">
-        <is>
-          <t>Part</t>
-        </is>
-      </c>
-      <c r="C40" s="47" t="inlineStr">
-        <is>
-          <t>Specification / note</t>
-        </is>
-      </c>
-      <c r="D40" s="48" t="inlineStr">
-        <is>
-          <t>Qty</t>
-        </is>
-      </c>
-      <c r="E40" s="48" t="inlineStr">
-        <is>
-          <t>Unit EUR</t>
-        </is>
-      </c>
-      <c r="F40" s="48" t="inlineStr">
-        <is>
-          <t>Total EUR</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="15.5" customHeight="1">
-      <c r="A41" s="49" t="inlineStr">
-        <is>
-          <t>C09</t>
-        </is>
-      </c>
-      <c r="B41" s="49" t="inlineStr">
-        <is>
-          <t>Generator mount</t>
-        </is>
-      </c>
-      <c r="C41" s="6" t="inlineStr">
-        <is>
-          <t>printed cradle + 4x M3x8 A4</t>
-        </is>
-      </c>
-      <c r="D41" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="E41" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="F41" s="51" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="42" ht="29" customHeight="1">
-      <c r="A42" s="52" t="inlineStr">
-        <is>
-          <t>A01</t>
-        </is>
-      </c>
-      <c r="B42" s="52" t="inlineStr">
-        <is>
-          <t>Blade</t>
-        </is>
-      </c>
-      <c r="C42" s="53" t="inlineStr">
-        <is>
-          <t>triple-blade rotor blade NACA4412 D220mm root pitch 28deg tip 2deg  -  ASA or ASA-CF; 6 perimeters; epoxy coat; spare blade = fuse for branch strike</t>
-        </is>
-      </c>
-      <c r="D42" s="54" t="n">
-        <v>3</v>
-      </c>
-      <c r="E42" s="55" t="n">
+    <row r="49" ht="29" customHeight="1">
+      <c r="A49" s="49" t="inlineStr">
+        <is>
+          <t>B03</t>
+        </is>
+      </c>
+      <c r="B49" s="49" t="inlineStr">
+        <is>
+          <t>Separation wall</t>
+        </is>
+      </c>
+      <c r="C49" s="6" t="inlineStr">
+        <is>
+          <t>D106 x 4 mm - RECOMMENDED integral with the pod bulkhead (no separate part)  -  4 mm per CAD, not 5; integral removes O-ring C03 and screws C05</t>
+        </is>
+      </c>
+      <c r="D49" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E49" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="F42" s="55" t="n">
+      <c r="F49" s="51" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="43" ht="29" customHeight="1">
-      <c r="A43" s="49" t="inlineStr">
-        <is>
-          <t>A02</t>
-        </is>
-      </c>
-      <c r="B43" s="49" t="inlineStr">
-        <is>
-          <t>Hub</t>
-        </is>
-      </c>
-      <c r="C43" s="6" t="inlineStr">
-        <is>
-          <t>Ø64x46mm with 2x M4 heat-set inserts and Ø5 H7 shaft bore  -  brass inserts M4 from TME</t>
-        </is>
-      </c>
-      <c r="D43" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="E43" s="51" t="n">
-        <v>0</v>
-      </c>
-      <c r="F43" s="51" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44" ht="29" customHeight="1">
-      <c r="A44" s="52" t="inlineStr">
-        <is>
-          <t>B02</t>
-        </is>
-      </c>
-      <c r="B44" s="52" t="inlineStr">
-        <is>
-          <t>Magnet cup</t>
-        </is>
-      </c>
-      <c r="C44" s="53" t="inlineStr">
-        <is>
-          <t>D70 rim, 8 pockets D10.2x5.2, printed ASA  -  pockets 10.2 dia (magnet 10 + 0.2 glue), 0.2 mm epoxy recess</t>
-        </is>
-      </c>
-      <c r="D44" s="54" t="n">
-        <v>2</v>
-      </c>
-      <c r="E44" s="55" t="n">
-        <v>0</v>
-      </c>
-      <c r="F44" s="55" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45" ht="15.5" customHeight="1">
-      <c r="A45" s="49" t="inlineStr">
-        <is>
-          <t>C01</t>
-        </is>
-      </c>
-      <c r="B45" s="49" t="inlineStr">
-        <is>
-          <t>Pod barrel</t>
-        </is>
-      </c>
-      <c r="C45" s="6" t="inlineStr">
-        <is>
-          <t>Ø110x120mm printed ASA wall 2.4mm + epoxy barrier  -  in model as pod</t>
-        </is>
-      </c>
-      <c r="D45" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="E45" s="51" t="n">
-        <v>0</v>
-      </c>
-      <c r="F45" s="51" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46" ht="15.5" customHeight="1">
-      <c r="A46" s="52" t="inlineStr">
-        <is>
-          <t>C02</t>
-        </is>
-      </c>
-      <c r="B46" s="52" t="inlineStr">
-        <is>
-          <t>Tail cone</t>
-        </is>
-      </c>
-      <c r="C46" s="53" t="inlineStr">
-        <is>
-          <t>printed integral</t>
-        </is>
-      </c>
-      <c r="D46" s="54" t="n">
-        <v>1</v>
-      </c>
-      <c r="E46" s="55" t="n">
-        <v>0</v>
-      </c>
-      <c r="F46" s="55" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47" ht="15.5" customHeight="1">
-      <c r="A47" s="49" t="inlineStr">
-        <is>
-          <t>E01</t>
-        </is>
-      </c>
-      <c r="B47" s="49" t="inlineStr">
-        <is>
-          <t>Sensor cage</t>
-        </is>
-      </c>
-      <c r="C47" s="6" t="inlineStr">
-        <is>
-          <t>Ø130x150 printed ASA 12 slots  -  in model as cage</t>
-        </is>
-      </c>
-      <c r="D47" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="E47" s="51" t="n">
-        <v>0</v>
-      </c>
-      <c r="F47" s="51" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="48" ht="29" customHeight="1">
-      <c r="A48" s="52" t="inlineStr">
-        <is>
-          <t>E03</t>
-        </is>
-      </c>
-      <c r="B48" s="52" t="inlineStr">
-        <is>
-          <t>Sensor holders</t>
-        </is>
-      </c>
-      <c r="C48" s="53" t="inlineStr">
-        <is>
-          <t>printed clips for pH/TDS/turbidity/NTC/MS5837  -  in model as sensor bodies</t>
-        </is>
-      </c>
-      <c r="D48" s="54" t="n">
-        <v>5</v>
-      </c>
-      <c r="E48" s="55" t="n">
-        <v>0</v>
-      </c>
-      <c r="F48" s="55" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50" ht="20" customHeight="1">
-      <c r="A50" s="45" t="inlineStr">
-        <is>
-          <t>NEREZMATERIAL.CZ</t>
-        </is>
-      </c>
-      <c r="F50" s="46" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="47" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B51" s="47" t="inlineStr">
-        <is>
-          <t>Part</t>
-        </is>
-      </c>
-      <c r="C51" s="47" t="inlineStr">
-        <is>
-          <t>Specification / note</t>
-        </is>
-      </c>
-      <c r="D51" s="48" t="inlineStr">
-        <is>
-          <t>Qty</t>
-        </is>
-      </c>
-      <c r="E51" s="48" t="inlineStr">
-        <is>
-          <t>Unit EUR</t>
-        </is>
-      </c>
-      <c r="F51" s="48" t="inlineStr">
-        <is>
-          <t>Total EUR</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="29" customHeight="1">
-      <c r="A52" s="49" t="inlineStr">
-        <is>
-          <t>B03</t>
-        </is>
-      </c>
-      <c r="B52" s="49" t="inlineStr">
-        <is>
-          <t>Separation wall</t>
-        </is>
-      </c>
-      <c r="C52" s="6" t="inlineStr">
-        <is>
-          <t>D106 x 4 mm - RECOMMENDED integral with the pod bulkhead (no separate part)  -  4 mm per CAD, not 5; integral removes O-ring C03 and screws C05</t>
-        </is>
-      </c>
-      <c r="D52" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="E52" s="51" t="n">
-        <v>0</v>
-      </c>
-      <c r="F52" s="51" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="54" ht="18" customHeight="1">
-      <c r="A54" s="56" t="inlineStr">
+    <row r="51" ht="18" customHeight="1">
+      <c r="A51" s="56" t="inlineStr">
         <is>
           <t>GOODS</t>
         </is>
       </c>
-      <c r="F54" s="57" t="n">
-        <v>234.61</v>
-      </c>
-    </row>
-    <row r="55" ht="18" customHeight="1">
-      <c r="A55" s="56" t="inlineStr">
+      <c r="F51" s="57" t="n">
+        <v>214.61</v>
+      </c>
+    </row>
+    <row r="52" ht="18" customHeight="1">
+      <c r="A52" s="56" t="inlineStr">
         <is>
           <t>shipping, estimated</t>
         </is>
       </c>
-      <c r="F55" s="57" t="n">
+      <c r="F52" s="57" t="n">
         <v>25</v>
       </c>
     </row>
+    <row r="53" ht="22" customHeight="1">
+      <c r="A53" s="58" t="inlineStr">
+        <is>
+          <t>LANDED TOTAL</t>
+        </is>
+      </c>
+      <c r="F53" s="59" t="n">
+        <v>239.61</v>
+      </c>
+    </row>
     <row r="56" ht="22" customHeight="1">
-      <c r="A56" s="58" t="inlineStr">
-        <is>
-          <t>LANDED TOTAL</t>
-        </is>
-      </c>
-      <c r="F56" s="59" t="n">
-        <v>259.61</v>
-      </c>
-    </row>
-    <row r="59" ht="22" customHeight="1">
-      <c r="A59" s="60" t="inlineStr">
+      <c r="A56" s="60" t="inlineStr">
         <is>
           <t>NOT IN THIS ORDER</t>
         </is>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" s="61" t="inlineStr">
+    <row r="57">
+      <c r="A57" s="61" t="inlineStr">
         <is>
           <t>PHASE 2 - BUY LATER</t>
         </is>
       </c>
     </row>
-    <row r="61" ht="29" customHeight="1">
+    <row r="58" ht="29" customHeight="1">
+      <c r="A58" s="62" t="inlineStr">
+        <is>
+          <t>A03</t>
+        </is>
+      </c>
+      <c r="B58" s="62" t="inlineStr">
+        <is>
+          <t>Wet shaft</t>
+        </is>
+      </c>
+      <c r="C58" s="63" t="inlineStr">
+        <is>
+          <t>lokalny zeleziar / Hornbach M5 A4 srob - 4. obchod sa nerata, nema postu; 3m bar 63.1 CZK makes ~26 shafts</t>
+        </is>
+      </c>
+      <c r="E58" s="64" t="inlineStr">
+        <is>
+          <t>2.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="29" customHeight="1">
+      <c r="A59" s="62" t="inlineStr">
+        <is>
+          <t>C08</t>
+        </is>
+      </c>
+      <c r="B59" s="62" t="inlineStr">
+        <is>
+          <t>Generator</t>
+        </is>
+      </c>
+      <c r="C59" s="63" t="inlineStr">
+        <is>
+          <t>TEST BEZ GENERATORA: klietka + senzory stacia, generator je dalsi nakup; XTG3506 preferred: encoder = free RPM/flow</t>
+        </is>
+      </c>
+      <c r="E59" s="64" t="inlineStr">
+        <is>
+          <t>26.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="15.5" customHeight="1">
+      <c r="A60" s="62" t="inlineStr">
+        <is>
+          <t>D01</t>
+        </is>
+      </c>
+      <c r="B60" s="62" t="inlineStr">
+        <is>
+          <t>pH electrode</t>
+        </is>
+      </c>
+      <c r="C60" s="63" t="inlineStr">
+        <is>
+          <t>OPTIONAL per site; 14-30 day service; +-0.1 pH after 2-pt cal</t>
+        </is>
+      </c>
+      <c r="E60" s="64" t="inlineStr">
+        <is>
+          <t>39.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="15.5" customHeight="1">
       <c r="A61" s="62" t="inlineStr">
         <is>
-          <t>A03</t>
+          <t>D02</t>
         </is>
       </c>
       <c r="B61" s="62" t="inlineStr">
         <is>
-          <t>Wet shaft</t>
+          <t>pH spare electrode</t>
         </is>
       </c>
       <c r="C61" s="63" t="inlineStr">
         <is>
-          <t>lokalny zeleziar / Hornbach M5 A4 srob - 4. obchod sa nerata, nema postu; 3m bar 63.1 CZK makes ~26 shafts</t>
+          <t>consumable</t>
         </is>
       </c>
       <c r="E61" s="64" t="inlineStr">
         <is>
-          <t>2.6</t>
-        </is>
-      </c>
-    </row>
-    <row r="62" ht="29" customHeight="1">
+          <t>9.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="15.5" customHeight="1">
       <c r="A62" s="62" t="inlineStr">
         <is>
-          <t>C08</t>
+          <t>D03</t>
         </is>
       </c>
       <c r="B62" s="62" t="inlineStr">
         <is>
-          <t>Generator</t>
+          <t>pH buffer</t>
         </is>
       </c>
       <c r="C62" s="63" t="inlineStr">
         <is>
-          <t>TEST BEZ GENERATORA: klietka + senzory stacia, generator je dalsi nakup; XTG3506 preferred: encoder = free RPM/flow</t>
+          <t>consumable</t>
         </is>
       </c>
       <c r="E62" s="64" t="inlineStr">
         <is>
-          <t>26.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="63" ht="15.5" customHeight="1">
+          <t>12.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="29" customHeight="1">
       <c r="A63" s="62" t="inlineStr">
         <is>
-          <t>D01</t>
+          <t>D09</t>
         </is>
       </c>
       <c r="B63" s="62" t="inlineStr">
         <is>
-          <t>pH electrode</t>
+          <t>Dissolved oxygen kit</t>
         </is>
       </c>
       <c r="C63" s="63" t="inlineStr">
         <is>
-          <t>OPTIONAL per site; 14-30 day service; +-0.1 pH after 2-pt cal</t>
+          <t>HIGHEST-VALUE channel (Budca = hypoxia); membrane 1-2 months in muddy water; 0.5M NaOH filling solution NOT shipped by air - source locally</t>
         </is>
       </c>
       <c r="E63" s="64" t="inlineStr">
         <is>
-          <t>39.0</t>
+          <t>175.0</t>
         </is>
       </c>
     </row>
     <row r="64" ht="15.5" customHeight="1">
       <c r="A64" s="62" t="inlineStr">
         <is>
-          <t>D02</t>
+          <t>D05</t>
         </is>
       </c>
       <c r="B64" s="62" t="inlineStr">
         <is>
-          <t>pH spare electrode</t>
+          <t>Level / stage probe</t>
         </is>
       </c>
       <c r="C64" s="63" t="inlineStr">
         <is>
-          <t>consumable</t>
+          <t>MS5837-30BA REJECTED: gel element must be dried daily, 24h max submersion</t>
         </is>
       </c>
       <c r="E64" s="64" t="inlineStr">
         <is>
-          <t>9.0</t>
+          <t>110.0</t>
         </is>
       </c>
     </row>
     <row r="65" ht="15.5" customHeight="1">
       <c r="A65" s="62" t="inlineStr">
         <is>
-          <t>D03</t>
+          <t>D06</t>
         </is>
       </c>
       <c r="B65" s="62" t="inlineStr">
         <is>
-          <t>pH buffer</t>
+          <t>EC/TDS</t>
         </is>
       </c>
       <c r="C65" s="63" t="inlineStr">
         <is>
-          <t>consumable</t>
+          <t>+-10% FS is the weakest sensor; use as trend indicator, site-calibrate</t>
         </is>
       </c>
       <c r="E65" s="64" t="inlineStr">
         <is>
-          <t>12.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="66" ht="29" customHeight="1">
+          <t>14.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="15.5" customHeight="1">
       <c r="A66" s="62" t="inlineStr">
         <is>
-          <t>D09</t>
+          <t>D08</t>
         </is>
       </c>
       <c r="B66" s="62" t="inlineStr">
         <is>
-          <t>Dissolved oxygen kit</t>
-        </is>
-      </c>
-      <c r="C66" s="63" t="inlineStr">
-        <is>
-          <t>HIGHEST-VALUE channel (Budca = hypoxia); membrane 1-2 months in muddy water; 0.5M NaOH filling solution NOT shipped by air - source locally</t>
-        </is>
-      </c>
+          <t>Sensor cable</t>
+        </is>
+      </c>
+      <c r="C66" s="63" t="inlineStr"/>
       <c r="E66" s="64" t="inlineStr">
         <is>
-          <t>175.0</t>
+          <t>20.0</t>
         </is>
       </c>
     </row>
     <row r="67" ht="15.5" customHeight="1">
       <c r="A67" s="62" t="inlineStr">
         <is>
-          <t>D05</t>
+          <t>G04</t>
         </is>
       </c>
       <c r="B67" s="62" t="inlineStr">
         <is>
-          <t>Level / stage probe</t>
+          <t>Antenna probe</t>
         </is>
       </c>
       <c r="C67" s="63" t="inlineStr">
         <is>
-          <t>MS5837-30BA REJECTED: gel element must be dried daily, 24h max submersion</t>
+          <t>v baleni kazdej Wio-E5 je EU868 antena - samostatne netreba; drzat ako zalohu</t>
         </is>
       </c>
       <c r="E67" s="64" t="inlineStr">
         <is>
-          <t>110.0</t>
+          <t>6.0</t>
         </is>
       </c>
     </row>
     <row r="68" ht="15.5" customHeight="1">
       <c r="A68" s="62" t="inlineStr">
         <is>
-          <t>D06</t>
+          <t>G05</t>
         </is>
       </c>
       <c r="B68" s="62" t="inlineStr">
         <is>
-          <t>EC/TDS</t>
+          <t>Antenna pigtail</t>
         </is>
       </c>
       <c r="C68" s="63" t="inlineStr">
         <is>
-          <t>+-10% FS is the weakest sensor; use as trend indicator, site-calibrate</t>
+          <t>netreba: doska ma SMA, antena sa skrutkuje priamo; pigtail len ak sa ide cez bulkhead</t>
         </is>
       </c>
       <c r="E68" s="64" t="inlineStr">
         <is>
-          <t>14.0</t>
+          <t>3.0</t>
         </is>
       </c>
     </row>
     <row r="69" ht="15.5" customHeight="1">
       <c r="A69" s="62" t="inlineStr">
         <is>
-          <t>D08</t>
+          <t>G06</t>
         </is>
       </c>
       <c r="B69" s="62" t="inlineStr">
         <is>
-          <t>Sensor cable</t>
-        </is>
-      </c>
-      <c r="C69" s="63" t="inlineStr"/>
+          <t>Boost harvester</t>
+        </is>
+      </c>
+      <c r="C69" s="63" t="inlineStr">
+        <is>
+          <t>needed when EMF below bus</t>
+        </is>
+      </c>
       <c r="E69" s="64" t="inlineStr">
         <is>
-          <t>20.0</t>
+          <t>5.0</t>
         </is>
       </c>
     </row>
     <row r="70" ht="15.5" customHeight="1">
       <c r="A70" s="62" t="inlineStr">
         <is>
-          <t>G04</t>
+          <t>G07</t>
         </is>
       </c>
       <c r="B70" s="62" t="inlineStr">
         <is>
-          <t>Antenna probe</t>
-        </is>
-      </c>
-      <c r="C70" s="63" t="inlineStr">
-        <is>
-          <t>v baleni kazdej Wio-E5 je EU868 antena - samostatne netreba; drzat ako zalohu</t>
-        </is>
-      </c>
+          <t>Buck</t>
+        </is>
+      </c>
+      <c r="C70" s="63" t="inlineStr"/>
       <c r="E70" s="64" t="inlineStr">
         <is>
-          <t>6.0</t>
+          <t>2.5</t>
         </is>
       </c>
     </row>
     <row r="71" ht="15.5" customHeight="1">
       <c r="A71" s="62" t="inlineStr">
         <is>
-          <t>G05</t>
+          <t>G08</t>
         </is>
       </c>
       <c r="B71" s="62" t="inlineStr">
         <is>
-          <t>Antenna pigtail</t>
+          <t>Rectifier</t>
         </is>
       </c>
       <c r="C71" s="63" t="inlineStr">
         <is>
-          <t>netreba: doska ma SMA, antena sa skrutkuje priamo; pigtail len ak sa ide cez bulkhead</t>
+          <t>452k in stock</t>
         </is>
       </c>
       <c r="E71" s="64" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>0.15</t>
         </is>
       </c>
     </row>
     <row r="72" ht="15.5" customHeight="1">
       <c r="A72" s="62" t="inlineStr">
         <is>
-          <t>G06</t>
+          <t>G09</t>
         </is>
       </c>
       <c r="B72" s="62" t="inlineStr">
         <is>
-          <t>Boost harvester</t>
+          <t>Clamp</t>
         </is>
       </c>
       <c r="C72" s="63" t="inlineStr">
         <is>
-          <t>needed when EMF below bus</t>
+          <t>overvoltage protection</t>
         </is>
       </c>
       <c r="E72" s="64" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>4.0</t>
         </is>
       </c>
     </row>
     <row r="73" ht="15.5" customHeight="1">
       <c r="A73" s="62" t="inlineStr">
         <is>
-          <t>G07</t>
+          <t>G10</t>
         </is>
       </c>
       <c r="B73" s="62" t="inlineStr">
         <is>
-          <t>Buck</t>
-        </is>
-      </c>
-      <c r="C73" s="63" t="inlineStr"/>
+          <t>Supercap</t>
+        </is>
+      </c>
+      <c r="C73" s="63" t="inlineStr">
+        <is>
+          <t>NO coin-cell EDLC (50ohm ESR kills TX)</t>
+        </is>
+      </c>
       <c r="E73" s="64" t="inlineStr">
         <is>
-          <t>2.5</t>
+          <t>11.0</t>
         </is>
       </c>
     </row>
     <row r="74" ht="15.5" customHeight="1">
       <c r="A74" s="62" t="inlineStr">
         <is>
-          <t>G08</t>
+          <t>G11</t>
         </is>
       </c>
       <c r="B74" s="62" t="inlineStr">
         <is>
-          <t>Rectifier</t>
+          <t>Voltage supervisor</t>
         </is>
       </c>
       <c r="C74" s="63" t="inlineStr">
         <is>
-          <t>452k in stock</t>
+          <t>gates buck at 4.8V</t>
         </is>
       </c>
       <c r="E74" s="64" t="inlineStr">
         <is>
-          <t>0.15</t>
+          <t>1.5</t>
         </is>
       </c>
     </row>
     <row r="75" ht="15.5" customHeight="1">
       <c r="A75" s="62" t="inlineStr">
         <is>
-          <t>G09</t>
+          <t>G12</t>
         </is>
       </c>
       <c r="B75" s="62" t="inlineStr">
         <is>
-          <t>Clamp</t>
+          <t>Load switch</t>
         </is>
       </c>
       <c r="C75" s="63" t="inlineStr">
         <is>
-          <t>overvoltage protection</t>
+          <t>removes ground-loop need</t>
         </is>
       </c>
       <c r="E75" s="64" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>1.0</t>
         </is>
       </c>
     </row>
     <row r="76" ht="15.5" customHeight="1">
       <c r="A76" s="62" t="inlineStr">
         <is>
-          <t>G10</t>
+          <t>G13</t>
         </is>
       </c>
       <c r="B76" s="62" t="inlineStr">
         <is>
-          <t>Supercap</t>
+          <t>Barometer</t>
         </is>
       </c>
       <c r="C76" s="63" t="inlineStr">
         <is>
-          <t>NO coin-cell EDLC (50ohm ESR kills TX)</t>
+          <t>pressure reference for MS5837</t>
         </is>
       </c>
       <c r="E76" s="64" t="inlineStr">
         <is>
-          <t>11.0</t>
+          <t>6.0</t>
         </is>
       </c>
     </row>
     <row r="77" ht="15.5" customHeight="1">
       <c r="A77" s="62" t="inlineStr">
         <is>
-          <t>G11</t>
+          <t>G14</t>
         </is>
       </c>
       <c r="B77" s="62" t="inlineStr">
         <is>
-          <t>Voltage supervisor</t>
+          <t>PCB</t>
         </is>
       </c>
       <c r="C77" s="63" t="inlineStr">
         <is>
-          <t>gates buck at 4.8V</t>
+          <t>panel of 10 amortises</t>
         </is>
       </c>
       <c r="E77" s="64" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>3.0</t>
         </is>
       </c>
     </row>
     <row r="78" ht="15.5" customHeight="1">
       <c r="A78" s="62" t="inlineStr">
         <is>
-          <t>G12</t>
+          <t>G15</t>
         </is>
       </c>
       <c r="B78" s="62" t="inlineStr">
         <is>
-          <t>Load switch</t>
-        </is>
-      </c>
-      <c r="C78" s="63" t="inlineStr">
-        <is>
-          <t>removes ground-loop need</t>
-        </is>
-      </c>
+          <t>Connectors</t>
+        </is>
+      </c>
+      <c r="C78" s="63" t="inlineStr"/>
       <c r="E78" s="64" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>10.0</t>
         </is>
       </c>
     </row>
     <row r="79" ht="15.5" customHeight="1">
       <c r="A79" s="62" t="inlineStr">
         <is>
-          <t>G13</t>
+          <t>H01</t>
         </is>
       </c>
       <c r="B79" s="62" t="inlineStr">
         <is>
-          <t>Barometer</t>
+          <t>Ground screw anchor</t>
         </is>
       </c>
       <c r="C79" s="63" t="inlineStr">
         <is>
-          <t>pressure reference for MS5837</t>
+          <t>1-2kN lateral - covers flood case</t>
         </is>
       </c>
       <c r="E79" s="64" t="inlineStr">
         <is>
-          <t>6.0</t>
+          <t>25.0</t>
         </is>
       </c>
     </row>
     <row r="80" ht="15.5" customHeight="1">
       <c r="A80" s="62" t="inlineStr">
         <is>
-          <t>G14</t>
+          <t>H02</t>
         </is>
       </c>
       <c r="B80" s="62" t="inlineStr">
         <is>
-          <t>PCB</t>
+          <t>Pole</t>
         </is>
       </c>
       <c r="C80" s="63" t="inlineStr">
         <is>
-          <t>panel of 10 amortises</t>
+          <t>removable mast pinned into receiver</t>
         </is>
       </c>
       <c r="E80" s="64" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>18.0</t>
         </is>
       </c>
     </row>
     <row r="81" ht="15.5" customHeight="1">
       <c r="A81" s="62" t="inlineStr">
         <is>
-          <t>G15</t>
+          <t>H03</t>
         </is>
       </c>
       <c r="B81" s="62" t="inlineStr">
         <is>
-          <t>Connectors</t>
-        </is>
-      </c>
-      <c r="C81" s="63" t="inlineStr"/>
+          <t>Receiver sleeve</t>
+        </is>
+      </c>
+      <c r="C81" s="63" t="inlineStr">
+        <is>
+          <t>pinned mast interface</t>
+        </is>
+      </c>
       <c r="E81" s="64" t="inlineStr">
         <is>
-          <t>10.0</t>
+          <t>8.0</t>
         </is>
       </c>
     </row>
     <row r="82" ht="15.5" customHeight="1">
       <c r="A82" s="62" t="inlineStr">
         <is>
-          <t>H01</t>
+          <t>H04</t>
         </is>
       </c>
       <c r="B82" s="62" t="inlineStr">
         <is>
-          <t>Ground screw anchor</t>
-        </is>
-      </c>
-      <c r="C82" s="63" t="inlineStr">
-        <is>
-          <t>1-2kN lateral - covers flood case</t>
-        </is>
-      </c>
+          <t>Arm tube</t>
+        </is>
+      </c>
+      <c r="C82" s="63" t="inlineStr"/>
       <c r="E82" s="64" t="inlineStr">
         <is>
-          <t>25.0</t>
+          <t>9.0</t>
         </is>
       </c>
     </row>
     <row r="83" ht="15.5" customHeight="1">
       <c r="A83" s="62" t="inlineStr">
         <is>
-          <t>H02</t>
+          <t>H05</t>
         </is>
       </c>
       <c r="B83" s="62" t="inlineStr">
         <is>
-          <t>Pole</t>
-        </is>
-      </c>
-      <c r="C83" s="63" t="inlineStr">
-        <is>
-          <t>removable mast pinned into receiver</t>
-        </is>
-      </c>
+          <t>Drop tube</t>
+        </is>
+      </c>
+      <c r="C83" s="63" t="inlineStr"/>
       <c r="E83" s="64" t="inlineStr">
         <is>
-          <t>18.0</t>
+          <t>6.0</t>
         </is>
       </c>
     </row>
     <row r="84" ht="15.5" customHeight="1">
       <c r="A84" s="62" t="inlineStr">
         <is>
-          <t>H03</t>
+          <t>H06</t>
         </is>
       </c>
       <c r="B84" s="62" t="inlineStr">
         <is>
-          <t>Receiver sleeve</t>
-        </is>
-      </c>
-      <c r="C84" s="63" t="inlineStr">
-        <is>
-          <t>pinned mast interface</t>
-        </is>
-      </c>
+          <t>Hinge collar</t>
+        </is>
+      </c>
+      <c r="C84" s="63" t="inlineStr"/>
       <c r="E84" s="64" t="inlineStr">
         <is>
-          <t>8.0</t>
+          <t>3.0</t>
         </is>
       </c>
     </row>
     <row r="85" ht="15.5" customHeight="1">
       <c r="A85" s="62" t="inlineStr">
         <is>
-          <t>H04</t>
+          <t>H07</t>
         </is>
       </c>
       <c r="B85" s="62" t="inlineStr">
         <is>
-          <t>Arm tube</t>
-        </is>
-      </c>
-      <c r="C85" s="63" t="inlineStr"/>
+          <t>Shear pin</t>
+        </is>
+      </c>
+      <c r="C85" s="63" t="inlineStr">
+        <is>
+          <t>releases pod on &gt;150N debris hit</t>
+        </is>
+      </c>
       <c r="E85" s="64" t="inlineStr">
         <is>
-          <t>9.0</t>
+          <t>1.0</t>
         </is>
       </c>
     </row>
     <row r="86" ht="15.5" customHeight="1">
       <c r="A86" s="62" t="inlineStr">
         <is>
-          <t>H05</t>
+          <t>H08</t>
         </is>
       </c>
       <c r="B86" s="62" t="inlineStr">
         <is>
-          <t>Drop tube</t>
-        </is>
-      </c>
-      <c r="C86" s="63" t="inlineStr"/>
+          <t>Yaw strut</t>
+        </is>
+      </c>
+      <c r="C86" s="63" t="inlineStr">
+        <is>
+          <t>anti-flutter</t>
+        </is>
+      </c>
       <c r="E86" s="64" t="inlineStr">
         <is>
-          <t>6.0</t>
+          <t>5.0</t>
         </is>
       </c>
     </row>
     <row r="87" ht="15.5" customHeight="1">
       <c r="A87" s="62" t="inlineStr">
         <is>
-          <t>H06</t>
+          <t>H09</t>
         </is>
       </c>
       <c r="B87" s="62" t="inlineStr">
         <is>
-          <t>Hinge collar</t>
-        </is>
-      </c>
-      <c r="C87" s="63" t="inlineStr"/>
+          <t>Guy line</t>
+        </is>
+      </c>
+      <c r="C87" s="63" t="inlineStr">
+        <is>
+          <t>45deg up/downstream</t>
+        </is>
+      </c>
       <c r="E87" s="64" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>9.0</t>
         </is>
       </c>
     </row>
     <row r="88" ht="15.5" customHeight="1">
       <c r="A88" s="62" t="inlineStr">
         <is>
-          <t>H07</t>
+          <t>H10</t>
         </is>
       </c>
       <c r="B88" s="62" t="inlineStr">
         <is>
-          <t>Shear pin</t>
-        </is>
-      </c>
-      <c r="C88" s="63" t="inlineStr">
-        <is>
-          <t>releases pod on &gt;150N debris hit</t>
-        </is>
-      </c>
+          <t>Guy anchor</t>
+        </is>
+      </c>
+      <c r="C88" s="63" t="inlineStr"/>
       <c r="E88" s="64" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>10.0</t>
         </is>
       </c>
     </row>
     <row r="89" ht="15.5" customHeight="1">
       <c r="A89" s="62" t="inlineStr">
         <is>
-          <t>H08</t>
+          <t>H11</t>
         </is>
       </c>
       <c r="B89" s="62" t="inlineStr">
         <is>
-          <t>Yaw strut</t>
+          <t>Safety cable</t>
         </is>
       </c>
       <c r="C89" s="63" t="inlineStr">
         <is>
-          <t>anti-flutter</t>
+          <t>theft/flood retention</t>
         </is>
       </c>
       <c r="E89" s="64" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>4.0</t>
         </is>
       </c>
     </row>
     <row r="90" ht="15.5" customHeight="1">
       <c r="A90" s="62" t="inlineStr">
         <is>
-          <t>H09</t>
+          <t>H12</t>
         </is>
       </c>
       <c r="B90" s="62" t="inlineStr">
         <is>
-          <t>Guy line</t>
+          <t>Security fastener</t>
         </is>
       </c>
       <c r="C90" s="63" t="inlineStr">
         <is>
-          <t>45deg up/downstream</t>
+          <t>anti-theft</t>
         </is>
       </c>
       <c r="E90" s="64" t="inlineStr">
         <is>
-          <t>9.0</t>
+          <t>4.0</t>
         </is>
       </c>
     </row>
     <row r="91" ht="15.5" customHeight="1">
       <c r="A91" s="62" t="inlineStr">
         <is>
-          <t>H10</t>
+          <t>H13</t>
         </is>
       </c>
       <c r="B91" s="62" t="inlineStr">
         <is>
-          <t>Guy anchor</t>
-        </is>
-      </c>
-      <c r="C91" s="63" t="inlineStr"/>
+          <t>Site label</t>
+        </is>
+      </c>
+      <c r="C91" s="63" t="inlineStr">
+        <is>
+          <t>anti-theft by making it unsellable</t>
+        </is>
+      </c>
       <c r="E91" s="64" t="inlineStr">
         <is>
-          <t>10.0</t>
+          <t>3.0</t>
         </is>
       </c>
     </row>
     <row r="92" ht="15.5" customHeight="1">
       <c r="A92" s="62" t="inlineStr">
         <is>
-          <t>H11</t>
+          <t>I02</t>
         </is>
       </c>
       <c r="B92" s="62" t="inlineStr">
         <is>
-          <t>Safety cable</t>
+          <t>Compute</t>
         </is>
       </c>
       <c r="C92" s="63" t="inlineStr">
         <is>
-          <t>theft/flood retention</t>
+          <t>YOU ALREADY HAVE THIS - reuse, zero soldering; runs the gateway service</t>
         </is>
       </c>
       <c r="E92" s="64" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>70.0</t>
         </is>
       </c>
     </row>
     <row r="93" ht="15.5" customHeight="1">
       <c r="A93" s="62" t="inlineStr">
         <is>
-          <t>H12</t>
+          <t>I03</t>
         </is>
       </c>
       <c r="B93" s="62" t="inlineStr">
         <is>
-          <t>Security fastener</t>
+          <t>Antenna</t>
         </is>
       </c>
       <c r="C93" s="63" t="inlineStr">
         <is>
-          <t>anti-theft</t>
+          <t>range-critical: gateway antenna gain + mast height set the link</t>
         </is>
       </c>
       <c r="E93" s="64" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>45.0</t>
         </is>
       </c>
     </row>
     <row r="94" ht="15.5" customHeight="1">
       <c r="A94" s="62" t="inlineStr">
         <is>
-          <t>H13</t>
+          <t>I04</t>
         </is>
       </c>
       <c r="B94" s="62" t="inlineStr">
         <is>
-          <t>Site label</t>
-        </is>
-      </c>
-      <c r="C94" s="63" t="inlineStr">
-        <is>
-          <t>anti-theft by making it unsellable</t>
-        </is>
-      </c>
+          <t>Enclosure</t>
+        </is>
+      </c>
+      <c r="C94" s="63" t="inlineStr"/>
       <c r="E94" s="64" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>35.0</t>
         </is>
       </c>
     </row>
     <row r="95" ht="15.5" customHeight="1">
       <c r="A95" s="62" t="inlineStr">
         <is>
-          <t>I02</t>
+          <t>I05</t>
         </is>
       </c>
       <c r="B95" s="62" t="inlineStr">
         <is>
-          <t>Compute</t>
+          <t>Mast</t>
         </is>
       </c>
       <c r="C95" s="63" t="inlineStr">
         <is>
-          <t>YOU ALREADY HAVE THIS - reuse, zero soldering; runs the gateway service</t>
+          <t>height sets range</t>
         </is>
       </c>
       <c r="E95" s="64" t="inlineStr">
         <is>
-          <t>70.0</t>
+          <t>30.0</t>
         </is>
       </c>
     </row>
     <row r="96" ht="15.5" customHeight="1">
       <c r="A96" s="62" t="inlineStr">
         <is>
-          <t>I03</t>
+          <t>I06</t>
         </is>
       </c>
       <c r="B96" s="62" t="inlineStr">
         <is>
-          <t>Antenna</t>
+          <t>Concentrator upgrade (optional)</t>
         </is>
       </c>
       <c r="C96" s="63" t="inlineStr">
         <is>
-          <t>range-critical: gateway antenna gain + mast height set the link</t>
+          <t>Only for multi-SF / multi-channel / public TTN. Single-channel Wio-E5 gateway is enough for our 20 nodes.</t>
         </is>
       </c>
       <c r="E96" s="64" t="inlineStr">
         <is>
-          <t>45.0</t>
+          <t>145.0</t>
         </is>
       </c>
     </row>
     <row r="97" ht="15.5" customHeight="1">
       <c r="A97" s="62" t="inlineStr">
         <is>
-          <t>I04</t>
+          <t>J01</t>
         </is>
       </c>
       <c r="B97" s="62" t="inlineStr">
         <is>
-          <t>Enclosure</t>
-        </is>
-      </c>
-      <c r="C97" s="63" t="inlineStr"/>
+          <t>Filament ASA</t>
+        </is>
+      </c>
+      <c r="C97" s="63" t="inlineStr">
+        <is>
+          <t>ABS z domaceho spoolu, nie ASA; UV je len na brehu</t>
+        </is>
+      </c>
       <c r="E97" s="64" t="inlineStr">
         <is>
-          <t>35.0</t>
+          <t>32.0</t>
         </is>
       </c>
     </row>
     <row r="98" ht="15.5" customHeight="1">
       <c r="A98" s="62" t="inlineStr">
         <is>
-          <t>I05</t>
+          <t>J02</t>
         </is>
       </c>
       <c r="B98" s="62" t="inlineStr">
         <is>
-          <t>Mast</t>
-        </is>
-      </c>
-      <c r="C98" s="63" t="inlineStr">
-        <is>
-          <t>height sets range</t>
-        </is>
-      </c>
+          <t>Filament PC Blend</t>
+        </is>
+      </c>
+      <c r="C98" s="63" t="inlineStr"/>
       <c r="E98" s="64" t="inlineStr">
         <is>
-          <t>30.0</t>
+          <t>40.0</t>
         </is>
       </c>
     </row>
     <row r="99" ht="15.5" customHeight="1">
       <c r="A99" s="62" t="inlineStr">
         <is>
-          <t>I06</t>
+          <t>J04</t>
         </is>
       </c>
       <c r="B99" s="62" t="inlineStr">
         <is>
-          <t>Concentrator upgrade (optional)</t>
-        </is>
-      </c>
-      <c r="C99" s="63" t="inlineStr">
-        <is>
-          <t>Only for multi-SF / multi-channel / public TTN. Single-channel Wio-E5 gateway is enough for our 20 nodes.</t>
-        </is>
-      </c>
+          <t>Conformal coat</t>
+        </is>
+      </c>
+      <c r="C99" s="63" t="inlineStr"/>
       <c r="E99" s="64" t="inlineStr">
         <is>
-          <t>145.0</t>
+          <t>14.0</t>
         </is>
       </c>
     </row>
     <row r="100" ht="15.5" customHeight="1">
       <c r="A100" s="62" t="inlineStr">
         <is>
-          <t>J01</t>
+          <t>J05</t>
         </is>
       </c>
       <c r="B100" s="62" t="inlineStr">
         <is>
-          <t>Filament ASA</t>
+          <t>Silicone grease</t>
         </is>
       </c>
       <c r="C100" s="63" t="inlineStr">
         <is>
-          <t>ABS z domaceho spoolu, nie ASA; UV je len na brehu</t>
+          <t>MAM - doma</t>
         </is>
       </c>
       <c r="E100" s="64" t="inlineStr">
         <is>
-          <t>32.0</t>
+          <t>9.0</t>
         </is>
       </c>
     </row>
     <row r="101" ht="15.5" customHeight="1">
       <c r="A101" s="62" t="inlineStr">
         <is>
-          <t>J02</t>
+          <t>J06</t>
         </is>
       </c>
       <c r="B101" s="62" t="inlineStr">
         <is>
-          <t>Filament PC Blend</t>
+          <t>Threadlocker</t>
         </is>
       </c>
       <c r="C101" s="63" t="inlineStr"/>
       <c r="E101" s="64" t="inlineStr">
         <is>
-          <t>40.0</t>
+          <t>11.0</t>
         </is>
       </c>
     </row>
     <row r="102" ht="15.5" customHeight="1">
       <c r="A102" s="62" t="inlineStr">
         <is>
-          <t>J04</t>
+          <t>J08</t>
         </is>
       </c>
       <c r="B102" s="62" t="inlineStr">
         <is>
-          <t>Conformal coat</t>
+          <t>O-ring kit</t>
         </is>
       </c>
       <c r="C102" s="63" t="inlineStr"/>
       <c r="E102" s="64" t="inlineStr">
         <is>
-          <t>14.0</t>
+          <t>12.0</t>
         </is>
       </c>
     </row>
     <row r="103" ht="15.5" customHeight="1">
       <c r="A103" s="62" t="inlineStr">
         <is>
-          <t>J05</t>
+          <t>K01</t>
         </is>
       </c>
       <c r="B103" s="62" t="inlineStr">
         <is>
-          <t>Silicone grease</t>
+          <t>Vacuum chamber</t>
         </is>
       </c>
       <c r="C103" s="63" t="inlineStr">
         <is>
-          <t>MAM - doma</t>
+          <t>acceptance test rig (one-off)</t>
         </is>
       </c>
       <c r="E103" s="64" t="inlineStr">
         <is>
-          <t>9.0</t>
+          <t>85.0</t>
         </is>
       </c>
     </row>
     <row r="104" ht="15.5" customHeight="1">
       <c r="A104" s="62" t="inlineStr">
         <is>
-          <t>J06</t>
+          <t>K02</t>
         </is>
       </c>
       <c r="B104" s="62" t="inlineStr">
         <is>
-          <t>Threadlocker</t>
-        </is>
-      </c>
-      <c r="C104" s="63" t="inlineStr"/>
+          <t>Torque driver</t>
+        </is>
+      </c>
+      <c r="C104" s="63" t="inlineStr">
+        <is>
+          <t>one-off</t>
+        </is>
+      </c>
       <c r="E104" s="64" t="inlineStr">
         <is>
-          <t>11.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="105" ht="15.5" customHeight="1">
-      <c r="A105" s="62" t="inlineStr">
-        <is>
-          <t>J08</t>
-        </is>
-      </c>
-      <c r="B105" s="62" t="inlineStr">
-        <is>
-          <t>O-ring kit</t>
-        </is>
-      </c>
-      <c r="C105" s="63" t="inlineStr"/>
-      <c r="E105" s="64" t="inlineStr">
-        <is>
-          <t>12.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="106" ht="15.5" customHeight="1">
-      <c r="A106" s="62" t="inlineStr">
-        <is>
-          <t>K01</t>
-        </is>
-      </c>
-      <c r="B106" s="62" t="inlineStr">
-        <is>
-          <t>Vacuum chamber</t>
-        </is>
-      </c>
-      <c r="C106" s="63" t="inlineStr">
-        <is>
-          <t>acceptance test rig (one-off)</t>
-        </is>
-      </c>
-      <c r="E106" s="64" t="inlineStr">
-        <is>
-          <t>85.0</t>
+          <t>40.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="65" t="inlineStr">
+        <is>
+          <t>CUT - DEAD LINE, DO NOT BUY</t>
         </is>
       </c>
     </row>
     <row r="107" ht="15.5" customHeight="1">
       <c r="A107" s="62" t="inlineStr">
         <is>
-          <t>K02</t>
+          <t>A05</t>
         </is>
       </c>
       <c r="B107" s="62" t="inlineStr">
         <is>
-          <t>Torque driver</t>
+          <t>Bearing carrier tube</t>
         </is>
       </c>
       <c r="C107" s="63" t="inlineStr">
         <is>
-          <t>one-off</t>
-        </is>
-      </c>
-      <c r="E107" s="64" t="inlineStr">
-        <is>
-          <t>40.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" s="65" t="inlineStr">
-        <is>
-          <t>CUT - DEAD LINE, DO NOT BUY</t>
+          <t>CUT: superseded - the bearing carrier is the printed spider (wet_carrier)</t>
+        </is>
+      </c>
+      <c r="E107" s="66" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="108" ht="15.5" customHeight="1">
+      <c r="A108" s="62" t="inlineStr">
+        <is>
+          <t>A07</t>
+        </is>
+      </c>
+      <c r="B108" s="62" t="inlineStr">
+        <is>
+          <t>Weed guard ring</t>
+        </is>
+      </c>
+      <c r="C108" s="63" t="inlineStr">
+        <is>
+          <t>CUT: killed by design - replaced by the nose cone D64-&gt;D12; a ring on struts upstream is an algae scythe</t>
+        </is>
+      </c>
+      <c r="E108" s="66" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="109" ht="15.5" customHeight="1">
+      <c r="A109" s="62" t="inlineStr">
+        <is>
+          <t>A08</t>
+        </is>
+      </c>
+      <c r="B109" s="62" t="inlineStr">
+        <is>
+          <t>Blade safety retainer</t>
+        </is>
+      </c>
+      <c r="C109" s="63" t="inlineStr">
+        <is>
+          <t>CUT: killed by design - a tether on a 110 mm blade is a flail, and the hole is a stress riser at the root</t>
+        </is>
+      </c>
+      <c r="E109" s="66" t="inlineStr">
+        <is>
+          <t>2.0</t>
         </is>
       </c>
     </row>
     <row r="110" ht="15.5" customHeight="1">
       <c r="A110" s="62" t="inlineStr">
         <is>
-          <t>A05</t>
+          <t>G02</t>
         </is>
       </c>
       <c r="B110" s="62" t="inlineStr">
         <is>
-          <t>Bearing carrier tube</t>
+          <t>MCU (NOT USED in simple build)</t>
         </is>
       </c>
       <c r="C110" s="63" t="inlineStr">
         <is>
-          <t>CUT: superseded - the bearing carrier is the printed spider (wet_carrier)</t>
+          <t>DROPPED: Wio-E5 mini is the single brain (MCU+LoRa). Bring back only if we need more GPIO/dual-core.</t>
         </is>
       </c>
       <c r="E110" s="66" t="inlineStr">
         <is>
-          <t>1.2</t>
-        </is>
-      </c>
-    </row>
-    <row r="111" ht="15.5" customHeight="1">
-      <c r="A111" s="62" t="inlineStr">
-        <is>
-          <t>A07</t>
-        </is>
-      </c>
-      <c r="B111" s="62" t="inlineStr">
-        <is>
-          <t>Weed guard ring</t>
-        </is>
-      </c>
-      <c r="C111" s="63" t="inlineStr">
-        <is>
-          <t>CUT: killed by design - replaced by the nose cone D64-&gt;D12; a ring on struts upstream is an algae scythe</t>
-        </is>
-      </c>
-      <c r="E111" s="66" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="112" ht="15.5" customHeight="1">
-      <c r="A112" s="62" t="inlineStr">
-        <is>
-          <t>A08</t>
-        </is>
-      </c>
-      <c r="B112" s="62" t="inlineStr">
-        <is>
-          <t>Blade safety retainer</t>
-        </is>
-      </c>
-      <c r="C112" s="63" t="inlineStr">
-        <is>
-          <t>CUT: killed by design - a tether on a 110 mm blade is a flail, and the hole is a stress riser at the root</t>
-        </is>
-      </c>
-      <c r="E112" s="66" t="inlineStr">
-        <is>
-          <t>2.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="113" ht="15.5" customHeight="1">
-      <c r="A113" s="62" t="inlineStr">
-        <is>
-          <t>G02</t>
-        </is>
-      </c>
-      <c r="B113" s="62" t="inlineStr">
-        <is>
-          <t>MCU (NOT USED in simple build)</t>
-        </is>
-      </c>
-      <c r="C113" s="63" t="inlineStr">
-        <is>
-          <t>DROPPED: Wio-E5 mini is the single brain (MCU+LoRa). Bring back only if we need more GPIO/dual-core.</t>
-        </is>
-      </c>
-      <c r="E113" s="66" t="inlineStr">
-        <is>
           <t>0.0</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="12">
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A39:E39"/>
-    <mergeCell ref="A35:E35"/>
-    <mergeCell ref="A50:E50"/>
-    <mergeCell ref="A55:E55"/>
+    <mergeCell ref="A53:E53"/>
     <mergeCell ref="A20:E20"/>
-    <mergeCell ref="A54:E54"/>
+    <mergeCell ref="A52:E52"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A28:E28"/>
+    <mergeCell ref="A51:E51"/>
+    <mergeCell ref="A47:E47"/>
     <mergeCell ref="A5:E5"/>
+    <mergeCell ref="A56:F56"/>
+    <mergeCell ref="A36:E36"/>
     <mergeCell ref="A3:F3"/>
-    <mergeCell ref="A56:E56"/>
-    <mergeCell ref="A59:F59"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
@@ -3633,7 +3590,7 @@
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>magsy.sk / supermagneticshop.com</t>
+          <t>techfun.sk / magsy.sk</t>
         </is>
       </c>
       <c r="F17" s="8" t="n">
@@ -3664,7 +3621,7 @@
       </c>
       <c r="L17" s="6" t="inlineStr">
         <is>
-          <t>N52 D10x5, 8 per cup on a D70 cup; must be canned/epoxy - bare N52 corrodes in weeks | 8 per cup, pitch r28 on D70 cup; price for D10 canned to re-verify; bare N52 must not touch water</t>
+          <t>N52 D10x5, 8 per cup on a D70 cup; must be canned/epoxy - bare N52 corrodes in weeks | techfun ma N52 magnet kruhovy - over priemer; inak magsy.sk; 8 na kapsu, D10</t>
         </is>
       </c>
     </row>
@@ -5360,7 +5317,7 @@
       </c>
       <c r="C61" s="6" t="inlineStr">
         <is>
-          <t>Seeed Wio-E5 mini: STM32WLE5JC Cortex-M4 + SX126x LoRa 868 MHz, USB-C, ADC/I2C/UART/GPIO</t>
+          <t>Seeed XIAO nRF52840 + Wio-SX1262 kit (Meshtastic), SEE336 - nRF52840 + SX1262</t>
         </is>
       </c>
       <c r="D61" s="7" t="n">
@@ -5368,14 +5325,14 @@
       </c>
       <c r="E61" s="6" t="inlineStr">
         <is>
-          <t>seeedstudio.com / openelab.io (EU)</t>
+          <t>rpishop.cz</t>
         </is>
       </c>
       <c r="F61" s="8" t="n">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G61" s="8" t="n">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="H61" s="7" t="inlineStr">
         <is>
@@ -5394,12 +5351,12 @@
       </c>
       <c r="K61" s="5" t="inlineStr">
         <is>
-          <t>quote</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="L61" s="6" t="inlineStr">
         <is>
-          <t>NIE je v techfun ani laskakit (overene 26.10.2026); Seeed $24.99, OpenELAB EU ~22.85; kazda doska obsahuje EU868 antenu</t>
+          <t>349 Kc, skladom 5+; nahradza Wio-E5, ktory v CZ/SK nie je; antena je v kite</t>
         </is>
       </c>
     </row>
@@ -6191,7 +6148,7 @@
       <c r="E76" s="68" t="n"/>
       <c r="F76" s="15" t="n"/>
       <c r="G76" s="15" t="n">
-        <v>106.9</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="H76" s="14" t="n"/>
       <c r="I76" s="14" t="n"/>
@@ -6958,7 +6915,7 @@
       </c>
       <c r="C95" s="6" t="inlineStr">
         <is>
-          <t>Wio-E5 mini = STM32WLE5JC + USB-C + CH340; plugs straight into RPi USB</t>
+          <t>Seeed XIAO nRF52840 + Wio-SX1262 kit (Meshtastic), SEE336 - nRF52840 + SX1262</t>
         </is>
       </c>
       <c r="D95" s="7" t="n">
@@ -6966,14 +6923,14 @@
       </c>
       <c r="E95" s="6" t="inlineStr">
         <is>
-          <t>seeedstudio.com / openelab.io (EU)</t>
+          <t>rpishop.cz</t>
         </is>
       </c>
       <c r="F95" s="8" t="n">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G95" s="8" t="n">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="H95" s="7" t="inlineStr">
         <is>
@@ -6992,12 +6949,12 @@
       </c>
       <c r="K95" s="5" t="inlineStr">
         <is>
-          <t>quote</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="L95" s="6" t="inlineStr">
         <is>
-          <t>single-channel Wio-E5 gateway: same radio as the probe, no concentrator needed | NIE je v techfun ani laskakit (overene 26.10.2026); Seeed $24.99, OpenELAB EU ~22.85; kazda doska obsahuje EU868 antenu</t>
+          <t>single-channel Wio-E5 gateway: same radio as the probe, no concentrator needed | 349 Kc, skladom 5+; nahradza Wio-E5, ktory v CZ/SK nie je; antena je v kite</t>
         </is>
       </c>
     </row>
@@ -7289,7 +7246,7 @@
       <c r="E101" s="68" t="n"/>
       <c r="F101" s="15" t="n"/>
       <c r="G101" s="15" t="n">
-        <v>349</v>
+        <v>339</v>
       </c>
       <c r="H101" s="14" t="n"/>
       <c r="I101" s="14" t="n"/>
@@ -7955,7 +7912,7 @@
       <c r="E120" s="67" t="n"/>
       <c r="F120" s="68" t="n"/>
       <c r="G120" s="25" t="n">
-        <v>730.3100000000001</v>
+        <v>710.3100000000001</v>
       </c>
     </row>
     <row r="121">
@@ -7985,7 +7942,7 @@
       <c r="E122" s="67" t="n"/>
       <c r="F122" s="68" t="n"/>
       <c r="G122" s="29" t="n">
-        <v>1371.31</v>
+        <v>1351.31</v>
       </c>
     </row>
     <row r="123">
@@ -8015,7 +7972,7 @@
       <c r="E124" s="67" t="n"/>
       <c r="F124" s="68" t="n"/>
       <c r="G124" s="33" t="n">
-        <v>1301.31</v>
+        <v>1281.31</v>
       </c>
     </row>
   </sheetData>
@@ -8203,7 +8160,7 @@
         </is>
       </c>
       <c r="B10" s="36" t="n">
-        <v>106.9</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="C10" s="36" t="n">
         <v>0</v>
@@ -8235,7 +8192,7 @@
         </is>
       </c>
       <c r="B12" s="36" t="n">
-        <v>204</v>
+        <v>194</v>
       </c>
       <c r="C12" s="36" t="n">
         <v>145</v>
@@ -8283,7 +8240,7 @@
         </is>
       </c>
       <c r="B15" s="38" t="n">
-        <v>730.3100000000001</v>
+        <v>710.3100000000001</v>
       </c>
       <c r="C15" s="38" t="n">
         <v>641</v>

</xml_diff>

<commit_message>
order: every line carries its shop link
- new link column in PARTS_LIST.csv, rendered as a hyperlink on the part name
- direct product pages where I could verify one: rpishop XIAO+SX1262 kit,
  techfun turbidity/DS18B20/potting, TME igus bushings, supermagnete N52 D10x5
- TME sits behind a Cloudflare challenge that blocks bots, so their lines carry
  a catalogue search link instead of a product URL. They open fine in a browser.
- 18 of 31 phase-1 lines are linked; the rest are printed in-house or CAD items.
</commit_message>
<xml_diff>
--- a/docs/sub-mission_parts.xlsx
+++ b/docs/sub-mission_parts.xlsx
@@ -24,7 +24,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0.00 &quot;EUR&quot;"/>
   </numFmts>
-  <fonts count="24">
+  <fonts count="25">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -103,6 +103,11 @@
       <b val="1"/>
       <color rgb="001F3864"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <color rgb="000563C1"/>
+      <sz val="9"/>
+      <u val="single"/>
     </font>
     <font>
       <b val="1"/>
@@ -269,7 +274,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="69">
+  <cellXfs count="71">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -388,6 +393,9 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top"/>
     </xf>
@@ -395,6 +403,9 @@
       <alignment horizontal="right" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -412,23 +423,23 @@
     <xf numFmtId="4" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="18" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="4" fontId="17" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="18" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -878,7 +889,7 @@
           <t>F01</t>
         </is>
       </c>
-      <c r="B7" s="49" t="inlineStr">
+      <c r="B7" s="50" t="inlineStr">
         <is>
           <t>Cable</t>
         </is>
@@ -888,39 +899,39 @@
           <t>8x0.5mm2 PUR jacket submersible 6m</t>
         </is>
       </c>
-      <c r="D7" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="E7" s="51" t="n">
+      <c r="D7" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="52" t="n">
         <v>35</v>
       </c>
-      <c r="F7" s="51" t="n">
+      <c r="F7" s="52" t="n">
         <v>35</v>
       </c>
     </row>
     <row r="8" ht="15.5" customHeight="1">
-      <c r="A8" s="52" t="inlineStr">
+      <c r="A8" s="53" t="inlineStr">
         <is>
           <t>G01</t>
         </is>
       </c>
-      <c r="B8" s="52" t="inlineStr">
+      <c r="B8" s="54" t="inlineStr">
         <is>
           <t>Enclosure</t>
         </is>
       </c>
-      <c r="C8" s="53" t="inlineStr">
+      <c r="C8" s="55" t="inlineStr">
         <is>
           <t>IP68 ready-made 190x130x80mm  -  in model as site_box</t>
         </is>
       </c>
-      <c r="D8" s="54" t="n">
-        <v>1</v>
-      </c>
-      <c r="E8" s="55" t="n">
+      <c r="D8" s="56" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="57" t="n">
         <v>22</v>
       </c>
-      <c r="F8" s="55" t="n">
+      <c r="F8" s="57" t="n">
         <v>22</v>
       </c>
     </row>
@@ -930,7 +941,7 @@
           <t>C07</t>
         </is>
       </c>
-      <c r="B9" s="49" t="inlineStr">
+      <c r="B9" s="50" t="inlineStr">
         <is>
           <t>Cable gland wet side</t>
         </is>
@@ -940,39 +951,39 @@
           <t>Lapp Skintop MS-M 12x1.5 + Scotchcast 2131  -  NOT YET IN MODEL - add boss</t>
         </is>
       </c>
-      <c r="D9" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="E9" s="51" t="n">
+      <c r="D9" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="52" t="n">
         <v>12</v>
       </c>
-      <c r="F9" s="51" t="n">
+      <c r="F9" s="52" t="n">
         <v>12</v>
       </c>
     </row>
     <row r="10" ht="15.5" customHeight="1">
-      <c r="A10" s="52" t="inlineStr">
+      <c r="A10" s="53" t="inlineStr">
         <is>
           <t>F02</t>
         </is>
       </c>
-      <c r="B10" s="52" t="inlineStr">
+      <c r="B10" s="54" t="inlineStr">
         <is>
           <t>Bulkhead connector</t>
         </is>
       </c>
-      <c r="C10" s="53" t="inlineStr">
+      <c r="C10" s="55" t="inlineStr">
         <is>
           <t>potted gland entry (NOT SubConn)  -  cost cut from 85 EUR wet-mate</t>
         </is>
       </c>
-      <c r="D10" s="54" t="n">
-        <v>1</v>
-      </c>
-      <c r="E10" s="55" t="n">
+      <c r="D10" s="56" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="57" t="n">
         <v>12</v>
       </c>
-      <c r="F10" s="55" t="n">
+      <c r="F10" s="57" t="n">
         <v>12</v>
       </c>
     </row>
@@ -982,7 +993,7 @@
           <t>G17</t>
         </is>
       </c>
-      <c r="B11" s="49" t="inlineStr">
+      <c r="B11" s="50" t="inlineStr">
         <is>
           <t>Cable glands</t>
         </is>
@@ -992,39 +1003,39 @@
           <t>M12 IP68 potted x3</t>
         </is>
       </c>
-      <c r="D11" s="50" t="n">
+      <c r="D11" s="51" t="n">
         <v>3</v>
       </c>
-      <c r="E11" s="51" t="n">
+      <c r="E11" s="52" t="n">
         <v>3</v>
       </c>
-      <c r="F11" s="51" t="n">
+      <c r="F11" s="52" t="n">
         <v>9</v>
       </c>
     </row>
     <row r="12" ht="15.5" customHeight="1">
-      <c r="A12" s="52" t="inlineStr">
+      <c r="A12" s="53" t="inlineStr">
         <is>
           <t>E02</t>
         </is>
       </c>
-      <c r="B12" s="52" t="inlineStr">
+      <c r="B12" s="54" t="inlineStr">
         <is>
           <t>Cage fasteners</t>
         </is>
       </c>
-      <c r="C12" s="53" t="inlineStr">
+      <c r="C12" s="55" t="inlineStr">
         <is>
           <t>M3x10 A4 + nylok</t>
         </is>
       </c>
-      <c r="D12" s="54" t="n">
-        <v>1</v>
-      </c>
-      <c r="E12" s="55" t="n">
+      <c r="D12" s="56" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="57" t="n">
         <v>6</v>
       </c>
-      <c r="F12" s="55" t="n">
+      <c r="F12" s="57" t="n">
         <v>6</v>
       </c>
     </row>
@@ -1034,7 +1045,7 @@
           <t>G16</t>
         </is>
       </c>
-      <c r="B13" s="49" t="inlineStr">
+      <c r="B13" s="50" t="inlineStr">
         <is>
           <t>Protection</t>
         </is>
@@ -1044,39 +1055,39 @@
           <t>Fuse 0.5A + TVS + ESD array  -  NEMAM - poistka 0.5A + TVS SMBJ5.0A + ESD array (SOT-23-6)</t>
         </is>
       </c>
-      <c r="D13" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="E13" s="51" t="n">
+      <c r="D13" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="52" t="n">
         <v>6</v>
       </c>
-      <c r="F13" s="51" t="n">
+      <c r="F13" s="52" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="14" ht="15.5" customHeight="1">
-      <c r="A14" s="52" t="inlineStr">
+      <c r="A14" s="53" t="inlineStr">
         <is>
           <t>J07</t>
         </is>
       </c>
-      <c r="B14" s="52" t="inlineStr">
+      <c r="B14" s="54" t="inlineStr">
         <is>
           <t>Heat-set inserts</t>
         </is>
       </c>
-      <c r="C14" s="53" t="inlineStr">
+      <c r="C14" s="55" t="inlineStr">
         <is>
           <t>M3/M4 brass assortment</t>
         </is>
       </c>
-      <c r="D14" s="54" t="n">
-        <v>1</v>
-      </c>
-      <c r="E14" s="55" t="n">
+      <c r="D14" s="56" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="57" t="n">
         <v>6</v>
       </c>
-      <c r="F14" s="55" t="n">
+      <c r="F14" s="57" t="n">
         <v>6</v>
       </c>
     </row>
@@ -1086,7 +1097,7 @@
           <t>C03</t>
         </is>
       </c>
-      <c r="B15" s="49" t="inlineStr">
+      <c r="B15" s="50" t="inlineStr">
         <is>
           <t>Pod O-ring</t>
         </is>
@@ -1096,39 +1107,39 @@
           <t>NBR 70 Ø100x2.5  -  zadny spoj podu - bez neho sa pri ponoreni natecie</t>
         </is>
       </c>
-      <c r="D15" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="E15" s="51" t="n">
+      <c r="D15" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" s="52" t="n">
         <v>3</v>
       </c>
-      <c r="F15" s="51" t="n">
+      <c r="F15" s="52" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="16" ht="29" customHeight="1">
-      <c r="A16" s="52" t="inlineStr">
+      <c r="A16" s="53" t="inlineStr">
         <is>
           <t>C05</t>
         </is>
       </c>
-      <c r="B16" s="52" t="inlineStr">
+      <c r="B16" s="54" t="inlineStr">
         <is>
           <t>Pod clamp screws</t>
         </is>
       </c>
-      <c r="C16" s="53" t="inlineStr">
+      <c r="C16" s="55" t="inlineStr">
         <is>
           <t>M4x30 A4 + washers  -  drzi zadny spoj; integralny bulkhead riesi len prednu stranu</t>
         </is>
       </c>
-      <c r="D16" s="54" t="n">
-        <v>1</v>
-      </c>
-      <c r="E16" s="55" t="n">
+      <c r="D16" s="56" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" s="57" t="n">
         <v>3</v>
       </c>
-      <c r="F16" s="55" t="n">
+      <c r="F16" s="57" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1138,7 +1149,7 @@
           <t>A04</t>
         </is>
       </c>
-      <c r="B17" s="49" t="inlineStr">
+      <c r="B17" s="50" t="inlineStr">
         <is>
           <t>Wet bearing</t>
         </is>
@@ -1148,39 +1159,39 @@
           <t>igus iglidur J plain bearing JSM-0507-05 5x7x5mm  -  83 pcs in stock; JFM-0507-05 flanged 1.48 USD alt</t>
         </is>
       </c>
-      <c r="D17" s="50" t="n">
+      <c r="D17" s="51" t="n">
         <v>2</v>
       </c>
-      <c r="E17" s="51" t="n">
+      <c r="E17" s="52" t="n">
         <v>1.18</v>
       </c>
-      <c r="F17" s="51" t="n">
+      <c r="F17" s="52" t="n">
         <v>2.36</v>
       </c>
     </row>
     <row r="18" ht="15.5" customHeight="1">
-      <c r="A18" s="52" t="inlineStr">
+      <c r="A18" s="53" t="inlineStr">
         <is>
           <t>A06</t>
         </is>
       </c>
-      <c r="B18" s="52" t="inlineStr">
+      <c r="B18" s="54" t="inlineStr">
         <is>
           <t>Set screw</t>
         </is>
       </c>
-      <c r="C18" s="53" t="inlineStr">
+      <c r="C18" s="55" t="inlineStr">
         <is>
           <t>M4x8 316SS cup point ISO 4029</t>
         </is>
       </c>
-      <c r="D18" s="54" t="n">
+      <c r="D18" s="56" t="n">
         <v>2</v>
       </c>
-      <c r="E18" s="55" t="n">
-        <v>1</v>
-      </c>
-      <c r="F18" s="55" t="n">
+      <c r="E18" s="57" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" s="57" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1242,39 +1253,39 @@
           <t>West System 105 + 206</t>
         </is>
       </c>
-      <c r="D22" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="E22" s="51" t="n">
+      <c r="D22" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" s="52" t="n">
         <v>18</v>
       </c>
-      <c r="F22" s="51" t="n">
+      <c r="F22" s="52" t="n">
         <v>18</v>
       </c>
     </row>
-    <row r="23" ht="15.5" customHeight="1">
-      <c r="A23" s="52" t="inlineStr">
+    <row r="23" ht="29" customHeight="1">
+      <c r="A23" s="53" t="inlineStr">
         <is>
           <t>B04</t>
         </is>
       </c>
-      <c r="B23" s="52" t="inlineStr">
+      <c r="B23" s="54" t="inlineStr">
         <is>
           <t>Potting compound</t>
         </is>
       </c>
-      <c r="C23" s="53" t="inlineStr">
-        <is>
-          <t>3M Scotch-Weld DP270 black 25ml</t>
-        </is>
-      </c>
-      <c r="D23" s="54" t="n">
-        <v>1</v>
-      </c>
-      <c r="E23" s="55" t="n">
+      <c r="C23" s="55" t="inlineStr">
+        <is>
+          <t>3M Scotch-Weld DP270 black 25ml  -  techfun nema DP270; silikonova zalievacia hmota staci na test, epoxid je tuhsi</t>
+        </is>
+      </c>
+      <c r="D23" s="56" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" s="57" t="n">
         <v>14</v>
       </c>
-      <c r="F23" s="55" t="n">
+      <c r="F23" s="57" t="n">
         <v>14</v>
       </c>
     </row>
@@ -1284,7 +1295,7 @@
           <t>D07</t>
         </is>
       </c>
-      <c r="B24" s="49" t="inlineStr">
+      <c r="B24" s="50" t="inlineStr">
         <is>
           <t>Turbidity</t>
         </is>
@@ -1294,39 +1305,39 @@
           <t>DFRobot SEN0189 (0-4.5V analog)  -  6 in stock; in model as sensor_turb</t>
         </is>
       </c>
-      <c r="D24" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="E24" s="51" t="n">
+      <c r="D24" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" s="52" t="n">
         <v>12.45</v>
       </c>
-      <c r="F24" s="51" t="n">
+      <c r="F24" s="52" t="n">
         <v>12.45</v>
       </c>
     </row>
     <row r="25" ht="29" customHeight="1">
-      <c r="A25" s="52" t="inlineStr">
+      <c r="A25" s="53" t="inlineStr">
         <is>
           <t>B01</t>
         </is>
       </c>
-      <c r="B25" s="52" t="inlineStr">
+      <c r="B25" s="54" t="inlineStr">
         <is>
           <t>Magnet</t>
         </is>
       </c>
-      <c r="C25" s="53" t="inlineStr">
-        <is>
-          <t>N52 D10x5 axially magnetised, canned 316L or epoxy potted  -  techfun ma N52 magnet kruhovy - over priemer; inak magsy.sk; 8 na kapsu, D10</t>
-        </is>
-      </c>
-      <c r="D25" s="54" t="n">
+      <c r="C25" s="55" t="inlineStr">
+        <is>
+          <t>N52 D10x5 axially magnetised, canned 316L or epoxy potted  -  16x N52 D10x5; supermagnete ma presne tento diel, magsy over v prehliadaci</t>
+        </is>
+      </c>
+      <c r="D25" s="56" t="n">
         <v>16</v>
       </c>
-      <c r="E25" s="55" t="n">
+      <c r="E25" s="57" t="n">
         <v>0.55</v>
       </c>
-      <c r="F25" s="55" t="n">
+      <c r="F25" s="57" t="n">
         <v>8.800000000000001</v>
       </c>
     </row>
@@ -1336,7 +1347,7 @@
           <t>D04</t>
         </is>
       </c>
-      <c r="B26" s="49" t="inlineStr">
+      <c r="B26" s="50" t="inlineStr">
         <is>
           <t>Temperature</t>
         </is>
@@ -1346,13 +1357,13 @@
           <t>DS18B20 waterproof 1m cable  -  in model as sensor_ntc</t>
         </is>
       </c>
-      <c r="D26" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="E26" s="51" t="n">
+      <c r="D26" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" s="52" t="n">
         <v>5</v>
       </c>
-      <c r="F26" s="51" t="n">
+      <c r="F26" s="52" t="n">
         <v>5</v>
       </c>
     </row>
@@ -1404,7 +1415,7 @@
           <t>G03</t>
         </is>
       </c>
-      <c r="B30" s="49" t="inlineStr">
+      <c r="B30" s="50" t="inlineStr">
         <is>
           <t>MCU + radio (single board)</t>
         </is>
@@ -1414,39 +1425,39 @@
           <t>Seeed XIAO nRF52840 + Wio-SX1262 kit (Meshtastic), SEE336 - nRF52840 + SX1262  -  349 Kc, skladom 5+; nahradza Wio-E5, ktory v CZ/SK nie je; antena je v kite</t>
         </is>
       </c>
-      <c r="D30" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="E30" s="51" t="n">
+      <c r="D30" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="E30" s="52" t="n">
         <v>14</v>
       </c>
-      <c r="F30" s="51" t="n">
+      <c r="F30" s="52" t="n">
         <v>14</v>
       </c>
     </row>
     <row r="31" ht="42.5" customHeight="1">
-      <c r="A31" s="52" t="inlineStr">
+      <c r="A31" s="53" t="inlineStr">
         <is>
           <t>I01</t>
         </is>
       </c>
-      <c r="B31" s="52" t="inlineStr">
+      <c r="B31" s="54" t="inlineStr">
         <is>
           <t>Gateway radio (single-channel)</t>
         </is>
       </c>
-      <c r="C31" s="53" t="inlineStr">
+      <c r="C31" s="55" t="inlineStr">
         <is>
           <t>Seeed XIAO nRF52840 + Wio-SX1262 kit (Meshtastic), SEE336 - nRF52840 + SX1262  -  349 Kc, skladom 5+; nahradza Wio-E5, ktory v CZ/SK nie je; antena je v kite</t>
         </is>
       </c>
-      <c r="D31" s="54" t="n">
-        <v>1</v>
-      </c>
-      <c r="E31" s="55" t="n">
+      <c r="D31" s="56" t="n">
+        <v>1</v>
+      </c>
+      <c r="E31" s="57" t="n">
         <v>14</v>
       </c>
-      <c r="F31" s="55" t="n">
+      <c r="F31" s="57" t="n">
         <v>14</v>
       </c>
     </row>
@@ -1466,39 +1477,39 @@
           <t>0-5N for coupling slip jig  -  one-off</t>
         </is>
       </c>
-      <c r="D32" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="E32" s="51" t="n">
+      <c r="D32" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="E32" s="52" t="n">
         <v>5</v>
       </c>
-      <c r="F32" s="51" t="n">
+      <c r="F32" s="52" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="33" ht="15.5" customHeight="1">
-      <c r="A33" s="52" t="inlineStr">
+      <c r="A33" s="53" t="inlineStr">
         <is>
           <t>C06</t>
         </is>
       </c>
-      <c r="B33" s="52" t="inlineStr">
+      <c r="B33" s="53" t="inlineStr">
         <is>
           <t>Desiccant</t>
         </is>
       </c>
-      <c r="C33" s="53" t="inlineStr">
+      <c r="C33" s="55" t="inlineStr">
         <is>
           <t>5g silica gel with indicator  -  replace at service</t>
         </is>
       </c>
-      <c r="D33" s="54" t="n">
+      <c r="D33" s="56" t="n">
         <v>2</v>
       </c>
-      <c r="E33" s="55" t="n">
+      <c r="E33" s="57" t="n">
         <v>2</v>
       </c>
-      <c r="F33" s="55" t="n">
+      <c r="F33" s="57" t="n">
         <v>4</v>
       </c>
     </row>
@@ -1518,13 +1529,13 @@
           <t>2.2mm wide x 1.8mm deep machined/printed into pod rim  -  NOT YET IN MODEL - add to pod</t>
         </is>
       </c>
-      <c r="D34" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="E34" s="51" t="n">
+      <c r="D34" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="E34" s="52" t="n">
         <v>0</v>
       </c>
-      <c r="F34" s="51" t="n">
+      <c r="F34" s="52" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1586,39 +1597,39 @@
           <t>printed cradle + 4x M3x8 A4</t>
         </is>
       </c>
-      <c r="D38" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="E38" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="F38" s="51" t="n">
+      <c r="D38" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="E38" s="52" t="n">
+        <v>1</v>
+      </c>
+      <c r="F38" s="52" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="39" ht="29" customHeight="1">
-      <c r="A39" s="52" t="inlineStr">
+      <c r="A39" s="53" t="inlineStr">
         <is>
           <t>A01</t>
         </is>
       </c>
-      <c r="B39" s="52" t="inlineStr">
+      <c r="B39" s="53" t="inlineStr">
         <is>
           <t>Blade</t>
         </is>
       </c>
-      <c r="C39" s="53" t="inlineStr">
+      <c r="C39" s="55" t="inlineStr">
         <is>
           <t>triple-blade rotor blade NACA4412 D220mm root pitch 28deg tip 2deg  -  ASA or ASA-CF; 6 perimeters; epoxy coat; spare blade = fuse for branch strike</t>
         </is>
       </c>
-      <c r="D39" s="54" t="n">
+      <c r="D39" s="56" t="n">
         <v>3</v>
       </c>
-      <c r="E39" s="55" t="n">
+      <c r="E39" s="57" t="n">
         <v>0</v>
       </c>
-      <c r="F39" s="55" t="n">
+      <c r="F39" s="57" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1638,39 +1649,39 @@
           <t>Ø64x46mm with 2x M4 heat-set inserts and Ø5 H7 shaft bore  -  brass inserts M4 from TME</t>
         </is>
       </c>
-      <c r="D40" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="E40" s="51" t="n">
+      <c r="D40" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="E40" s="52" t="n">
         <v>0</v>
       </c>
-      <c r="F40" s="51" t="n">
+      <c r="F40" s="52" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="41" ht="29" customHeight="1">
-      <c r="A41" s="52" t="inlineStr">
+      <c r="A41" s="53" t="inlineStr">
         <is>
           <t>B02</t>
         </is>
       </c>
-      <c r="B41" s="52" t="inlineStr">
+      <c r="B41" s="53" t="inlineStr">
         <is>
           <t>Magnet cup</t>
         </is>
       </c>
-      <c r="C41" s="53" t="inlineStr">
+      <c r="C41" s="55" t="inlineStr">
         <is>
           <t>D70 rim, 8 pockets D10.2x5.2, printed ASA  -  pockets 10.2 dia (magnet 10 + 0.2 glue), 0.2 mm epoxy recess</t>
         </is>
       </c>
-      <c r="D41" s="54" t="n">
+      <c r="D41" s="56" t="n">
         <v>2</v>
       </c>
-      <c r="E41" s="55" t="n">
+      <c r="E41" s="57" t="n">
         <v>0</v>
       </c>
-      <c r="F41" s="55" t="n">
+      <c r="F41" s="57" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1690,39 +1701,39 @@
           <t>Ø110x120mm printed ASA wall 2.4mm + epoxy barrier  -  in model as pod</t>
         </is>
       </c>
-      <c r="D42" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="E42" s="51" t="n">
+      <c r="D42" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="E42" s="52" t="n">
         <v>0</v>
       </c>
-      <c r="F42" s="51" t="n">
+      <c r="F42" s="52" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="43" ht="15.5" customHeight="1">
-      <c r="A43" s="52" t="inlineStr">
+      <c r="A43" s="53" t="inlineStr">
         <is>
           <t>C02</t>
         </is>
       </c>
-      <c r="B43" s="52" t="inlineStr">
+      <c r="B43" s="53" t="inlineStr">
         <is>
           <t>Tail cone</t>
         </is>
       </c>
-      <c r="C43" s="53" t="inlineStr">
+      <c r="C43" s="55" t="inlineStr">
         <is>
           <t>printed integral</t>
         </is>
       </c>
-      <c r="D43" s="54" t="n">
-        <v>1</v>
-      </c>
-      <c r="E43" s="55" t="n">
+      <c r="D43" s="56" t="n">
+        <v>1</v>
+      </c>
+      <c r="E43" s="57" t="n">
         <v>0</v>
       </c>
-      <c r="F43" s="55" t="n">
+      <c r="F43" s="57" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1742,39 +1753,39 @@
           <t>Ø130x150 printed ASA 12 slots  -  in model as cage</t>
         </is>
       </c>
-      <c r="D44" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="E44" s="51" t="n">
+      <c r="D44" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="E44" s="52" t="n">
         <v>0</v>
       </c>
-      <c r="F44" s="51" t="n">
+      <c r="F44" s="52" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="45" ht="29" customHeight="1">
-      <c r="A45" s="52" t="inlineStr">
+      <c r="A45" s="53" t="inlineStr">
         <is>
           <t>E03</t>
         </is>
       </c>
-      <c r="B45" s="52" t="inlineStr">
+      <c r="B45" s="53" t="inlineStr">
         <is>
           <t>Sensor holders</t>
         </is>
       </c>
-      <c r="C45" s="53" t="inlineStr">
+      <c r="C45" s="55" t="inlineStr">
         <is>
           <t>printed clips for pH/TDS/turbidity/NTC/MS5837  -  in model as sensor bodies</t>
         </is>
       </c>
-      <c r="D45" s="54" t="n">
+      <c r="D45" s="56" t="n">
         <v>5</v>
       </c>
-      <c r="E45" s="55" t="n">
+      <c r="E45" s="57" t="n">
         <v>0</v>
       </c>
-      <c r="F45" s="55" t="n">
+      <c r="F45" s="57" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1836,1136 +1847,1136 @@
           <t>D106 x 4 mm - RECOMMENDED integral with the pod bulkhead (no separate part)  -  4 mm per CAD, not 5; integral removes O-ring C03 and screws C05</t>
         </is>
       </c>
-      <c r="D49" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="E49" s="51" t="n">
+      <c r="D49" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="E49" s="52" t="n">
         <v>0</v>
       </c>
-      <c r="F49" s="51" t="n">
+      <c r="F49" s="52" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
-      <c r="A51" s="56" t="inlineStr">
+      <c r="A51" s="58" t="inlineStr">
         <is>
           <t>GOODS</t>
         </is>
       </c>
-      <c r="F51" s="57" t="n">
+      <c r="F51" s="59" t="n">
         <v>214.61</v>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1">
-      <c r="A52" s="56" t="inlineStr">
+      <c r="A52" s="58" t="inlineStr">
         <is>
           <t>shipping, estimated</t>
         </is>
       </c>
-      <c r="F52" s="57" t="n">
+      <c r="F52" s="59" t="n">
         <v>25</v>
       </c>
     </row>
     <row r="53" ht="22" customHeight="1">
-      <c r="A53" s="58" t="inlineStr">
+      <c r="A53" s="60" t="inlineStr">
         <is>
           <t>LANDED TOTAL</t>
         </is>
       </c>
-      <c r="F53" s="59" t="n">
+      <c r="F53" s="61" t="n">
         <v>239.61</v>
       </c>
     </row>
     <row r="56" ht="22" customHeight="1">
-      <c r="A56" s="60" t="inlineStr">
+      <c r="A56" s="62" t="inlineStr">
         <is>
           <t>NOT IN THIS ORDER</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="61" t="inlineStr">
+      <c r="A57" s="63" t="inlineStr">
         <is>
           <t>PHASE 2 - BUY LATER</t>
         </is>
       </c>
     </row>
     <row r="58" ht="29" customHeight="1">
-      <c r="A58" s="62" t="inlineStr">
+      <c r="A58" s="64" t="inlineStr">
         <is>
           <t>A03</t>
         </is>
       </c>
-      <c r="B58" s="62" t="inlineStr">
+      <c r="B58" s="64" t="inlineStr">
         <is>
           <t>Wet shaft</t>
         </is>
       </c>
-      <c r="C58" s="63" t="inlineStr">
+      <c r="C58" s="65" t="inlineStr">
         <is>
           <t>lokalny zeleziar / Hornbach M5 A4 srob - 4. obchod sa nerata, nema postu; 3m bar 63.1 CZK makes ~26 shafts</t>
         </is>
       </c>
-      <c r="E58" s="64" t="inlineStr">
+      <c r="E58" s="66" t="inlineStr">
         <is>
           <t>2.6</t>
         </is>
       </c>
     </row>
     <row r="59" ht="29" customHeight="1">
-      <c r="A59" s="62" t="inlineStr">
+      <c r="A59" s="64" t="inlineStr">
         <is>
           <t>C08</t>
         </is>
       </c>
-      <c r="B59" s="62" t="inlineStr">
+      <c r="B59" s="64" t="inlineStr">
         <is>
           <t>Generator</t>
         </is>
       </c>
-      <c r="C59" s="63" t="inlineStr">
+      <c r="C59" s="65" t="inlineStr">
         <is>
           <t>TEST BEZ GENERATORA: klietka + senzory stacia, generator je dalsi nakup; XTG3506 preferred: encoder = free RPM/flow</t>
         </is>
       </c>
-      <c r="E59" s="64" t="inlineStr">
+      <c r="E59" s="66" t="inlineStr">
         <is>
           <t>26.0</t>
         </is>
       </c>
     </row>
     <row r="60" ht="15.5" customHeight="1">
-      <c r="A60" s="62" t="inlineStr">
+      <c r="A60" s="64" t="inlineStr">
         <is>
           <t>D01</t>
         </is>
       </c>
-      <c r="B60" s="62" t="inlineStr">
+      <c r="B60" s="64" t="inlineStr">
         <is>
           <t>pH electrode</t>
         </is>
       </c>
-      <c r="C60" s="63" t="inlineStr">
+      <c r="C60" s="65" t="inlineStr">
         <is>
           <t>OPTIONAL per site; 14-30 day service; +-0.1 pH after 2-pt cal</t>
         </is>
       </c>
-      <c r="E60" s="64" t="inlineStr">
+      <c r="E60" s="66" t="inlineStr">
         <is>
           <t>39.0</t>
         </is>
       </c>
     </row>
     <row r="61" ht="15.5" customHeight="1">
-      <c r="A61" s="62" t="inlineStr">
+      <c r="A61" s="64" t="inlineStr">
         <is>
           <t>D02</t>
         </is>
       </c>
-      <c r="B61" s="62" t="inlineStr">
+      <c r="B61" s="64" t="inlineStr">
         <is>
           <t>pH spare electrode</t>
         </is>
       </c>
-      <c r="C61" s="63" t="inlineStr">
+      <c r="C61" s="65" t="inlineStr">
         <is>
           <t>consumable</t>
         </is>
       </c>
-      <c r="E61" s="64" t="inlineStr">
+      <c r="E61" s="66" t="inlineStr">
         <is>
           <t>9.0</t>
         </is>
       </c>
     </row>
     <row r="62" ht="15.5" customHeight="1">
-      <c r="A62" s="62" t="inlineStr">
+      <c r="A62" s="64" t="inlineStr">
         <is>
           <t>D03</t>
         </is>
       </c>
-      <c r="B62" s="62" t="inlineStr">
+      <c r="B62" s="64" t="inlineStr">
         <is>
           <t>pH buffer</t>
         </is>
       </c>
-      <c r="C62" s="63" t="inlineStr">
+      <c r="C62" s="65" t="inlineStr">
         <is>
           <t>consumable</t>
         </is>
       </c>
-      <c r="E62" s="64" t="inlineStr">
+      <c r="E62" s="66" t="inlineStr">
         <is>
           <t>12.0</t>
         </is>
       </c>
     </row>
     <row r="63" ht="29" customHeight="1">
-      <c r="A63" s="62" t="inlineStr">
+      <c r="A63" s="64" t="inlineStr">
         <is>
           <t>D09</t>
         </is>
       </c>
-      <c r="B63" s="62" t="inlineStr">
+      <c r="B63" s="64" t="inlineStr">
         <is>
           <t>Dissolved oxygen kit</t>
         </is>
       </c>
-      <c r="C63" s="63" t="inlineStr">
+      <c r="C63" s="65" t="inlineStr">
         <is>
           <t>HIGHEST-VALUE channel (Budca = hypoxia); membrane 1-2 months in muddy water; 0.5M NaOH filling solution NOT shipped by air - source locally</t>
         </is>
       </c>
-      <c r="E63" s="64" t="inlineStr">
+      <c r="E63" s="66" t="inlineStr">
         <is>
           <t>175.0</t>
         </is>
       </c>
     </row>
     <row r="64" ht="15.5" customHeight="1">
-      <c r="A64" s="62" t="inlineStr">
+      <c r="A64" s="64" t="inlineStr">
         <is>
           <t>D05</t>
         </is>
       </c>
-      <c r="B64" s="62" t="inlineStr">
+      <c r="B64" s="64" t="inlineStr">
         <is>
           <t>Level / stage probe</t>
         </is>
       </c>
-      <c r="C64" s="63" t="inlineStr">
+      <c r="C64" s="65" t="inlineStr">
         <is>
           <t>MS5837-30BA REJECTED: gel element must be dried daily, 24h max submersion</t>
         </is>
       </c>
-      <c r="E64" s="64" t="inlineStr">
+      <c r="E64" s="66" t="inlineStr">
         <is>
           <t>110.0</t>
         </is>
       </c>
     </row>
     <row r="65" ht="15.5" customHeight="1">
-      <c r="A65" s="62" t="inlineStr">
+      <c r="A65" s="64" t="inlineStr">
         <is>
           <t>D06</t>
         </is>
       </c>
-      <c r="B65" s="62" t="inlineStr">
+      <c r="B65" s="64" t="inlineStr">
         <is>
           <t>EC/TDS</t>
         </is>
       </c>
-      <c r="C65" s="63" t="inlineStr">
+      <c r="C65" s="65" t="inlineStr">
         <is>
           <t>+-10% FS is the weakest sensor; use as trend indicator, site-calibrate</t>
         </is>
       </c>
-      <c r="E65" s="64" t="inlineStr">
+      <c r="E65" s="66" t="inlineStr">
         <is>
           <t>14.0</t>
         </is>
       </c>
     </row>
     <row r="66" ht="15.5" customHeight="1">
-      <c r="A66" s="62" t="inlineStr">
+      <c r="A66" s="64" t="inlineStr">
         <is>
           <t>D08</t>
         </is>
       </c>
-      <c r="B66" s="62" t="inlineStr">
+      <c r="B66" s="64" t="inlineStr">
         <is>
           <t>Sensor cable</t>
         </is>
       </c>
-      <c r="C66" s="63" t="inlineStr"/>
-      <c r="E66" s="64" t="inlineStr">
+      <c r="C66" s="65" t="inlineStr"/>
+      <c r="E66" s="66" t="inlineStr">
         <is>
           <t>20.0</t>
         </is>
       </c>
     </row>
     <row r="67" ht="15.5" customHeight="1">
-      <c r="A67" s="62" t="inlineStr">
+      <c r="A67" s="64" t="inlineStr">
         <is>
           <t>G04</t>
         </is>
       </c>
-      <c r="B67" s="62" t="inlineStr">
+      <c r="B67" s="64" t="inlineStr">
         <is>
           <t>Antenna probe</t>
         </is>
       </c>
-      <c r="C67" s="63" t="inlineStr">
+      <c r="C67" s="65" t="inlineStr">
         <is>
           <t>v baleni kazdej Wio-E5 je EU868 antena - samostatne netreba; drzat ako zalohu</t>
         </is>
       </c>
-      <c r="E67" s="64" t="inlineStr">
+      <c r="E67" s="66" t="inlineStr">
         <is>
           <t>6.0</t>
         </is>
       </c>
     </row>
     <row r="68" ht="15.5" customHeight="1">
-      <c r="A68" s="62" t="inlineStr">
+      <c r="A68" s="64" t="inlineStr">
         <is>
           <t>G05</t>
         </is>
       </c>
-      <c r="B68" s="62" t="inlineStr">
+      <c r="B68" s="64" t="inlineStr">
         <is>
           <t>Antenna pigtail</t>
         </is>
       </c>
-      <c r="C68" s="63" t="inlineStr">
+      <c r="C68" s="65" t="inlineStr">
         <is>
           <t>netreba: doska ma SMA, antena sa skrutkuje priamo; pigtail len ak sa ide cez bulkhead</t>
         </is>
       </c>
-      <c r="E68" s="64" t="inlineStr">
+      <c r="E68" s="66" t="inlineStr">
         <is>
           <t>3.0</t>
         </is>
       </c>
     </row>
     <row r="69" ht="15.5" customHeight="1">
-      <c r="A69" s="62" t="inlineStr">
+      <c r="A69" s="64" t="inlineStr">
         <is>
           <t>G06</t>
         </is>
       </c>
-      <c r="B69" s="62" t="inlineStr">
+      <c r="B69" s="64" t="inlineStr">
         <is>
           <t>Boost harvester</t>
         </is>
       </c>
-      <c r="C69" s="63" t="inlineStr">
+      <c r="C69" s="65" t="inlineStr">
         <is>
           <t>needed when EMF below bus</t>
         </is>
       </c>
-      <c r="E69" s="64" t="inlineStr">
+      <c r="E69" s="66" t="inlineStr">
         <is>
           <t>5.0</t>
         </is>
       </c>
     </row>
     <row r="70" ht="15.5" customHeight="1">
-      <c r="A70" s="62" t="inlineStr">
+      <c r="A70" s="64" t="inlineStr">
         <is>
           <t>G07</t>
         </is>
       </c>
-      <c r="B70" s="62" t="inlineStr">
+      <c r="B70" s="64" t="inlineStr">
         <is>
           <t>Buck</t>
         </is>
       </c>
-      <c r="C70" s="63" t="inlineStr"/>
-      <c r="E70" s="64" t="inlineStr">
+      <c r="C70" s="65" t="inlineStr"/>
+      <c r="E70" s="66" t="inlineStr">
         <is>
           <t>2.5</t>
         </is>
       </c>
     </row>
     <row r="71" ht="15.5" customHeight="1">
-      <c r="A71" s="62" t="inlineStr">
+      <c r="A71" s="64" t="inlineStr">
         <is>
           <t>G08</t>
         </is>
       </c>
-      <c r="B71" s="62" t="inlineStr">
+      <c r="B71" s="64" t="inlineStr">
         <is>
           <t>Rectifier</t>
         </is>
       </c>
-      <c r="C71" s="63" t="inlineStr">
+      <c r="C71" s="65" t="inlineStr">
         <is>
           <t>452k in stock</t>
         </is>
       </c>
-      <c r="E71" s="64" t="inlineStr">
+      <c r="E71" s="66" t="inlineStr">
         <is>
           <t>0.15</t>
         </is>
       </c>
     </row>
     <row r="72" ht="15.5" customHeight="1">
-      <c r="A72" s="62" t="inlineStr">
+      <c r="A72" s="64" t="inlineStr">
         <is>
           <t>G09</t>
         </is>
       </c>
-      <c r="B72" s="62" t="inlineStr">
+      <c r="B72" s="64" t="inlineStr">
         <is>
           <t>Clamp</t>
         </is>
       </c>
-      <c r="C72" s="63" t="inlineStr">
+      <c r="C72" s="65" t="inlineStr">
         <is>
           <t>overvoltage protection</t>
         </is>
       </c>
-      <c r="E72" s="64" t="inlineStr">
+      <c r="E72" s="66" t="inlineStr">
         <is>
           <t>4.0</t>
         </is>
       </c>
     </row>
     <row r="73" ht="15.5" customHeight="1">
-      <c r="A73" s="62" t="inlineStr">
+      <c r="A73" s="64" t="inlineStr">
         <is>
           <t>G10</t>
         </is>
       </c>
-      <c r="B73" s="62" t="inlineStr">
+      <c r="B73" s="64" t="inlineStr">
         <is>
           <t>Supercap</t>
         </is>
       </c>
-      <c r="C73" s="63" t="inlineStr">
+      <c r="C73" s="65" t="inlineStr">
         <is>
           <t>NO coin-cell EDLC (50ohm ESR kills TX)</t>
         </is>
       </c>
-      <c r="E73" s="64" t="inlineStr">
+      <c r="E73" s="66" t="inlineStr">
         <is>
           <t>11.0</t>
         </is>
       </c>
     </row>
     <row r="74" ht="15.5" customHeight="1">
-      <c r="A74" s="62" t="inlineStr">
+      <c r="A74" s="64" t="inlineStr">
         <is>
           <t>G11</t>
         </is>
       </c>
-      <c r="B74" s="62" t="inlineStr">
+      <c r="B74" s="64" t="inlineStr">
         <is>
           <t>Voltage supervisor</t>
         </is>
       </c>
-      <c r="C74" s="63" t="inlineStr">
+      <c r="C74" s="65" t="inlineStr">
         <is>
           <t>gates buck at 4.8V</t>
         </is>
       </c>
-      <c r="E74" s="64" t="inlineStr">
+      <c r="E74" s="66" t="inlineStr">
         <is>
           <t>1.5</t>
         </is>
       </c>
     </row>
     <row r="75" ht="15.5" customHeight="1">
-      <c r="A75" s="62" t="inlineStr">
+      <c r="A75" s="64" t="inlineStr">
         <is>
           <t>G12</t>
         </is>
       </c>
-      <c r="B75" s="62" t="inlineStr">
+      <c r="B75" s="64" t="inlineStr">
         <is>
           <t>Load switch</t>
         </is>
       </c>
-      <c r="C75" s="63" t="inlineStr">
+      <c r="C75" s="65" t="inlineStr">
         <is>
           <t>removes ground-loop need</t>
         </is>
       </c>
-      <c r="E75" s="64" t="inlineStr">
+      <c r="E75" s="66" t="inlineStr">
         <is>
           <t>1.0</t>
         </is>
       </c>
     </row>
     <row r="76" ht="15.5" customHeight="1">
-      <c r="A76" s="62" t="inlineStr">
+      <c r="A76" s="64" t="inlineStr">
         <is>
           <t>G13</t>
         </is>
       </c>
-      <c r="B76" s="62" t="inlineStr">
+      <c r="B76" s="64" t="inlineStr">
         <is>
           <t>Barometer</t>
         </is>
       </c>
-      <c r="C76" s="63" t="inlineStr">
+      <c r="C76" s="65" t="inlineStr">
         <is>
           <t>pressure reference for MS5837</t>
         </is>
       </c>
-      <c r="E76" s="64" t="inlineStr">
+      <c r="E76" s="66" t="inlineStr">
         <is>
           <t>6.0</t>
         </is>
       </c>
     </row>
     <row r="77" ht="15.5" customHeight="1">
-      <c r="A77" s="62" t="inlineStr">
+      <c r="A77" s="64" t="inlineStr">
         <is>
           <t>G14</t>
         </is>
       </c>
-      <c r="B77" s="62" t="inlineStr">
+      <c r="B77" s="64" t="inlineStr">
         <is>
           <t>PCB</t>
         </is>
       </c>
-      <c r="C77" s="63" t="inlineStr">
+      <c r="C77" s="65" t="inlineStr">
         <is>
           <t>panel of 10 amortises</t>
         </is>
       </c>
-      <c r="E77" s="64" t="inlineStr">
+      <c r="E77" s="66" t="inlineStr">
         <is>
           <t>3.0</t>
         </is>
       </c>
     </row>
     <row r="78" ht="15.5" customHeight="1">
-      <c r="A78" s="62" t="inlineStr">
+      <c r="A78" s="64" t="inlineStr">
         <is>
           <t>G15</t>
         </is>
       </c>
-      <c r="B78" s="62" t="inlineStr">
+      <c r="B78" s="64" t="inlineStr">
         <is>
           <t>Connectors</t>
         </is>
       </c>
-      <c r="C78" s="63" t="inlineStr"/>
-      <c r="E78" s="64" t="inlineStr">
+      <c r="C78" s="65" t="inlineStr"/>
+      <c r="E78" s="66" t="inlineStr">
         <is>
           <t>10.0</t>
         </is>
       </c>
     </row>
     <row r="79" ht="15.5" customHeight="1">
-      <c r="A79" s="62" t="inlineStr">
+      <c r="A79" s="64" t="inlineStr">
         <is>
           <t>H01</t>
         </is>
       </c>
-      <c r="B79" s="62" t="inlineStr">
+      <c r="B79" s="64" t="inlineStr">
         <is>
           <t>Ground screw anchor</t>
         </is>
       </c>
-      <c r="C79" s="63" t="inlineStr">
+      <c r="C79" s="65" t="inlineStr">
         <is>
           <t>1-2kN lateral - covers flood case</t>
         </is>
       </c>
-      <c r="E79" s="64" t="inlineStr">
+      <c r="E79" s="66" t="inlineStr">
         <is>
           <t>25.0</t>
         </is>
       </c>
     </row>
     <row r="80" ht="15.5" customHeight="1">
-      <c r="A80" s="62" t="inlineStr">
+      <c r="A80" s="64" t="inlineStr">
         <is>
           <t>H02</t>
         </is>
       </c>
-      <c r="B80" s="62" t="inlineStr">
+      <c r="B80" s="64" t="inlineStr">
         <is>
           <t>Pole</t>
         </is>
       </c>
-      <c r="C80" s="63" t="inlineStr">
+      <c r="C80" s="65" t="inlineStr">
         <is>
           <t>removable mast pinned into receiver</t>
         </is>
       </c>
-      <c r="E80" s="64" t="inlineStr">
+      <c r="E80" s="66" t="inlineStr">
         <is>
           <t>18.0</t>
         </is>
       </c>
     </row>
     <row r="81" ht="15.5" customHeight="1">
-      <c r="A81" s="62" t="inlineStr">
+      <c r="A81" s="64" t="inlineStr">
         <is>
           <t>H03</t>
         </is>
       </c>
-      <c r="B81" s="62" t="inlineStr">
+      <c r="B81" s="64" t="inlineStr">
         <is>
           <t>Receiver sleeve</t>
         </is>
       </c>
-      <c r="C81" s="63" t="inlineStr">
+      <c r="C81" s="65" t="inlineStr">
         <is>
           <t>pinned mast interface</t>
         </is>
       </c>
-      <c r="E81" s="64" t="inlineStr">
+      <c r="E81" s="66" t="inlineStr">
         <is>
           <t>8.0</t>
         </is>
       </c>
     </row>
     <row r="82" ht="15.5" customHeight="1">
-      <c r="A82" s="62" t="inlineStr">
+      <c r="A82" s="64" t="inlineStr">
         <is>
           <t>H04</t>
         </is>
       </c>
-      <c r="B82" s="62" t="inlineStr">
+      <c r="B82" s="64" t="inlineStr">
         <is>
           <t>Arm tube</t>
         </is>
       </c>
-      <c r="C82" s="63" t="inlineStr"/>
-      <c r="E82" s="64" t="inlineStr">
+      <c r="C82" s="65" t="inlineStr"/>
+      <c r="E82" s="66" t="inlineStr">
         <is>
           <t>9.0</t>
         </is>
       </c>
     </row>
     <row r="83" ht="15.5" customHeight="1">
-      <c r="A83" s="62" t="inlineStr">
+      <c r="A83" s="64" t="inlineStr">
         <is>
           <t>H05</t>
         </is>
       </c>
-      <c r="B83" s="62" t="inlineStr">
+      <c r="B83" s="64" t="inlineStr">
         <is>
           <t>Drop tube</t>
         </is>
       </c>
-      <c r="C83" s="63" t="inlineStr"/>
-      <c r="E83" s="64" t="inlineStr">
+      <c r="C83" s="65" t="inlineStr"/>
+      <c r="E83" s="66" t="inlineStr">
         <is>
           <t>6.0</t>
         </is>
       </c>
     </row>
     <row r="84" ht="15.5" customHeight="1">
-      <c r="A84" s="62" t="inlineStr">
+      <c r="A84" s="64" t="inlineStr">
         <is>
           <t>H06</t>
         </is>
       </c>
-      <c r="B84" s="62" t="inlineStr">
+      <c r="B84" s="64" t="inlineStr">
         <is>
           <t>Hinge collar</t>
         </is>
       </c>
-      <c r="C84" s="63" t="inlineStr"/>
-      <c r="E84" s="64" t="inlineStr">
+      <c r="C84" s="65" t="inlineStr"/>
+      <c r="E84" s="66" t="inlineStr">
         <is>
           <t>3.0</t>
         </is>
       </c>
     </row>
     <row r="85" ht="15.5" customHeight="1">
-      <c r="A85" s="62" t="inlineStr">
+      <c r="A85" s="64" t="inlineStr">
         <is>
           <t>H07</t>
         </is>
       </c>
-      <c r="B85" s="62" t="inlineStr">
+      <c r="B85" s="64" t="inlineStr">
         <is>
           <t>Shear pin</t>
         </is>
       </c>
-      <c r="C85" s="63" t="inlineStr">
+      <c r="C85" s="65" t="inlineStr">
         <is>
           <t>releases pod on &gt;150N debris hit</t>
         </is>
       </c>
-      <c r="E85" s="64" t="inlineStr">
+      <c r="E85" s="66" t="inlineStr">
         <is>
           <t>1.0</t>
         </is>
       </c>
     </row>
     <row r="86" ht="15.5" customHeight="1">
-      <c r="A86" s="62" t="inlineStr">
+      <c r="A86" s="64" t="inlineStr">
         <is>
           <t>H08</t>
         </is>
       </c>
-      <c r="B86" s="62" t="inlineStr">
+      <c r="B86" s="64" t="inlineStr">
         <is>
           <t>Yaw strut</t>
         </is>
       </c>
-      <c r="C86" s="63" t="inlineStr">
+      <c r="C86" s="65" t="inlineStr">
         <is>
           <t>anti-flutter</t>
         </is>
       </c>
-      <c r="E86" s="64" t="inlineStr">
+      <c r="E86" s="66" t="inlineStr">
         <is>
           <t>5.0</t>
         </is>
       </c>
     </row>
     <row r="87" ht="15.5" customHeight="1">
-      <c r="A87" s="62" t="inlineStr">
+      <c r="A87" s="64" t="inlineStr">
         <is>
           <t>H09</t>
         </is>
       </c>
-      <c r="B87" s="62" t="inlineStr">
+      <c r="B87" s="64" t="inlineStr">
         <is>
           <t>Guy line</t>
         </is>
       </c>
-      <c r="C87" s="63" t="inlineStr">
+      <c r="C87" s="65" t="inlineStr">
         <is>
           <t>45deg up/downstream</t>
         </is>
       </c>
-      <c r="E87" s="64" t="inlineStr">
+      <c r="E87" s="66" t="inlineStr">
         <is>
           <t>9.0</t>
         </is>
       </c>
     </row>
     <row r="88" ht="15.5" customHeight="1">
-      <c r="A88" s="62" t="inlineStr">
+      <c r="A88" s="64" t="inlineStr">
         <is>
           <t>H10</t>
         </is>
       </c>
-      <c r="B88" s="62" t="inlineStr">
+      <c r="B88" s="64" t="inlineStr">
         <is>
           <t>Guy anchor</t>
         </is>
       </c>
-      <c r="C88" s="63" t="inlineStr"/>
-      <c r="E88" s="64" t="inlineStr">
+      <c r="C88" s="65" t="inlineStr"/>
+      <c r="E88" s="66" t="inlineStr">
         <is>
           <t>10.0</t>
         </is>
       </c>
     </row>
     <row r="89" ht="15.5" customHeight="1">
-      <c r="A89" s="62" t="inlineStr">
+      <c r="A89" s="64" t="inlineStr">
         <is>
           <t>H11</t>
         </is>
       </c>
-      <c r="B89" s="62" t="inlineStr">
+      <c r="B89" s="64" t="inlineStr">
         <is>
           <t>Safety cable</t>
         </is>
       </c>
-      <c r="C89" s="63" t="inlineStr">
+      <c r="C89" s="65" t="inlineStr">
         <is>
           <t>theft/flood retention</t>
         </is>
       </c>
-      <c r="E89" s="64" t="inlineStr">
+      <c r="E89" s="66" t="inlineStr">
         <is>
           <t>4.0</t>
         </is>
       </c>
     </row>
     <row r="90" ht="15.5" customHeight="1">
-      <c r="A90" s="62" t="inlineStr">
+      <c r="A90" s="64" t="inlineStr">
         <is>
           <t>H12</t>
         </is>
       </c>
-      <c r="B90" s="62" t="inlineStr">
+      <c r="B90" s="64" t="inlineStr">
         <is>
           <t>Security fastener</t>
         </is>
       </c>
-      <c r="C90" s="63" t="inlineStr">
+      <c r="C90" s="65" t="inlineStr">
         <is>
           <t>anti-theft</t>
         </is>
       </c>
-      <c r="E90" s="64" t="inlineStr">
+      <c r="E90" s="66" t="inlineStr">
         <is>
           <t>4.0</t>
         </is>
       </c>
     </row>
     <row r="91" ht="15.5" customHeight="1">
-      <c r="A91" s="62" t="inlineStr">
+      <c r="A91" s="64" t="inlineStr">
         <is>
           <t>H13</t>
         </is>
       </c>
-      <c r="B91" s="62" t="inlineStr">
+      <c r="B91" s="64" t="inlineStr">
         <is>
           <t>Site label</t>
         </is>
       </c>
-      <c r="C91" s="63" t="inlineStr">
+      <c r="C91" s="65" t="inlineStr">
         <is>
           <t>anti-theft by making it unsellable</t>
         </is>
       </c>
-      <c r="E91" s="64" t="inlineStr">
+      <c r="E91" s="66" t="inlineStr">
         <is>
           <t>3.0</t>
         </is>
       </c>
     </row>
     <row r="92" ht="15.5" customHeight="1">
-      <c r="A92" s="62" t="inlineStr">
+      <c r="A92" s="64" t="inlineStr">
         <is>
           <t>I02</t>
         </is>
       </c>
-      <c r="B92" s="62" t="inlineStr">
+      <c r="B92" s="64" t="inlineStr">
         <is>
           <t>Compute</t>
         </is>
       </c>
-      <c r="C92" s="63" t="inlineStr">
+      <c r="C92" s="65" t="inlineStr">
         <is>
           <t>YOU ALREADY HAVE THIS - reuse, zero soldering; runs the gateway service</t>
         </is>
       </c>
-      <c r="E92" s="64" t="inlineStr">
+      <c r="E92" s="66" t="inlineStr">
         <is>
           <t>70.0</t>
         </is>
       </c>
     </row>
     <row r="93" ht="15.5" customHeight="1">
-      <c r="A93" s="62" t="inlineStr">
+      <c r="A93" s="64" t="inlineStr">
         <is>
           <t>I03</t>
         </is>
       </c>
-      <c r="B93" s="62" t="inlineStr">
+      <c r="B93" s="64" t="inlineStr">
         <is>
           <t>Antenna</t>
         </is>
       </c>
-      <c r="C93" s="63" t="inlineStr">
+      <c r="C93" s="65" t="inlineStr">
         <is>
           <t>range-critical: gateway antenna gain + mast height set the link</t>
         </is>
       </c>
-      <c r="E93" s="64" t="inlineStr">
+      <c r="E93" s="66" t="inlineStr">
         <is>
           <t>45.0</t>
         </is>
       </c>
     </row>
     <row r="94" ht="15.5" customHeight="1">
-      <c r="A94" s="62" t="inlineStr">
+      <c r="A94" s="64" t="inlineStr">
         <is>
           <t>I04</t>
         </is>
       </c>
-      <c r="B94" s="62" t="inlineStr">
+      <c r="B94" s="64" t="inlineStr">
         <is>
           <t>Enclosure</t>
         </is>
       </c>
-      <c r="C94" s="63" t="inlineStr"/>
-      <c r="E94" s="64" t="inlineStr">
+      <c r="C94" s="65" t="inlineStr"/>
+      <c r="E94" s="66" t="inlineStr">
         <is>
           <t>35.0</t>
         </is>
       </c>
     </row>
     <row r="95" ht="15.5" customHeight="1">
-      <c r="A95" s="62" t="inlineStr">
+      <c r="A95" s="64" t="inlineStr">
         <is>
           <t>I05</t>
         </is>
       </c>
-      <c r="B95" s="62" t="inlineStr">
+      <c r="B95" s="64" t="inlineStr">
         <is>
           <t>Mast</t>
         </is>
       </c>
-      <c r="C95" s="63" t="inlineStr">
+      <c r="C95" s="65" t="inlineStr">
         <is>
           <t>height sets range</t>
         </is>
       </c>
-      <c r="E95" s="64" t="inlineStr">
+      <c r="E95" s="66" t="inlineStr">
         <is>
           <t>30.0</t>
         </is>
       </c>
     </row>
     <row r="96" ht="15.5" customHeight="1">
-      <c r="A96" s="62" t="inlineStr">
+      <c r="A96" s="64" t="inlineStr">
         <is>
           <t>I06</t>
         </is>
       </c>
-      <c r="B96" s="62" t="inlineStr">
+      <c r="B96" s="64" t="inlineStr">
         <is>
           <t>Concentrator upgrade (optional)</t>
         </is>
       </c>
-      <c r="C96" s="63" t="inlineStr">
+      <c r="C96" s="65" t="inlineStr">
         <is>
           <t>Only for multi-SF / multi-channel / public TTN. Single-channel Wio-E5 gateway is enough for our 20 nodes.</t>
         </is>
       </c>
-      <c r="E96" s="64" t="inlineStr">
+      <c r="E96" s="66" t="inlineStr">
         <is>
           <t>145.0</t>
         </is>
       </c>
     </row>
     <row r="97" ht="15.5" customHeight="1">
-      <c r="A97" s="62" t="inlineStr">
+      <c r="A97" s="64" t="inlineStr">
         <is>
           <t>J01</t>
         </is>
       </c>
-      <c r="B97" s="62" t="inlineStr">
+      <c r="B97" s="64" t="inlineStr">
         <is>
           <t>Filament ASA</t>
         </is>
       </c>
-      <c r="C97" s="63" t="inlineStr">
+      <c r="C97" s="65" t="inlineStr">
         <is>
           <t>ABS z domaceho spoolu, nie ASA; UV je len na brehu</t>
         </is>
       </c>
-      <c r="E97" s="64" t="inlineStr">
+      <c r="E97" s="66" t="inlineStr">
         <is>
           <t>32.0</t>
         </is>
       </c>
     </row>
     <row r="98" ht="15.5" customHeight="1">
-      <c r="A98" s="62" t="inlineStr">
+      <c r="A98" s="64" t="inlineStr">
         <is>
           <t>J02</t>
         </is>
       </c>
-      <c r="B98" s="62" t="inlineStr">
+      <c r="B98" s="64" t="inlineStr">
         <is>
           <t>Filament PC Blend</t>
         </is>
       </c>
-      <c r="C98" s="63" t="inlineStr"/>
-      <c r="E98" s="64" t="inlineStr">
+      <c r="C98" s="65" t="inlineStr"/>
+      <c r="E98" s="66" t="inlineStr">
         <is>
           <t>40.0</t>
         </is>
       </c>
     </row>
     <row r="99" ht="15.5" customHeight="1">
-      <c r="A99" s="62" t="inlineStr">
+      <c r="A99" s="64" t="inlineStr">
         <is>
           <t>J04</t>
         </is>
       </c>
-      <c r="B99" s="62" t="inlineStr">
+      <c r="B99" s="64" t="inlineStr">
         <is>
           <t>Conformal coat</t>
         </is>
       </c>
-      <c r="C99" s="63" t="inlineStr"/>
-      <c r="E99" s="64" t="inlineStr">
+      <c r="C99" s="65" t="inlineStr"/>
+      <c r="E99" s="66" t="inlineStr">
         <is>
           <t>14.0</t>
         </is>
       </c>
     </row>
     <row r="100" ht="15.5" customHeight="1">
-      <c r="A100" s="62" t="inlineStr">
+      <c r="A100" s="64" t="inlineStr">
         <is>
           <t>J05</t>
         </is>
       </c>
-      <c r="B100" s="62" t="inlineStr">
+      <c r="B100" s="64" t="inlineStr">
         <is>
           <t>Silicone grease</t>
         </is>
       </c>
-      <c r="C100" s="63" t="inlineStr">
+      <c r="C100" s="65" t="inlineStr">
         <is>
           <t>MAM - doma</t>
         </is>
       </c>
-      <c r="E100" s="64" t="inlineStr">
+      <c r="E100" s="66" t="inlineStr">
         <is>
           <t>9.0</t>
         </is>
       </c>
     </row>
     <row r="101" ht="15.5" customHeight="1">
-      <c r="A101" s="62" t="inlineStr">
+      <c r="A101" s="64" t="inlineStr">
         <is>
           <t>J06</t>
         </is>
       </c>
-      <c r="B101" s="62" t="inlineStr">
+      <c r="B101" s="64" t="inlineStr">
         <is>
           <t>Threadlocker</t>
         </is>
       </c>
-      <c r="C101" s="63" t="inlineStr"/>
-      <c r="E101" s="64" t="inlineStr">
+      <c r="C101" s="65" t="inlineStr"/>
+      <c r="E101" s="66" t="inlineStr">
         <is>
           <t>11.0</t>
         </is>
       </c>
     </row>
     <row r="102" ht="15.5" customHeight="1">
-      <c r="A102" s="62" t="inlineStr">
+      <c r="A102" s="64" t="inlineStr">
         <is>
           <t>J08</t>
         </is>
       </c>
-      <c r="B102" s="62" t="inlineStr">
+      <c r="B102" s="64" t="inlineStr">
         <is>
           <t>O-ring kit</t>
         </is>
       </c>
-      <c r="C102" s="63" t="inlineStr"/>
-      <c r="E102" s="64" t="inlineStr">
+      <c r="C102" s="65" t="inlineStr"/>
+      <c r="E102" s="66" t="inlineStr">
         <is>
           <t>12.0</t>
         </is>
       </c>
     </row>
     <row r="103" ht="15.5" customHeight="1">
-      <c r="A103" s="62" t="inlineStr">
+      <c r="A103" s="64" t="inlineStr">
         <is>
           <t>K01</t>
         </is>
       </c>
-      <c r="B103" s="62" t="inlineStr">
+      <c r="B103" s="64" t="inlineStr">
         <is>
           <t>Vacuum chamber</t>
         </is>
       </c>
-      <c r="C103" s="63" t="inlineStr">
+      <c r="C103" s="65" t="inlineStr">
         <is>
           <t>acceptance test rig (one-off)</t>
         </is>
       </c>
-      <c r="E103" s="64" t="inlineStr">
+      <c r="E103" s="66" t="inlineStr">
         <is>
           <t>85.0</t>
         </is>
       </c>
     </row>
     <row r="104" ht="15.5" customHeight="1">
-      <c r="A104" s="62" t="inlineStr">
+      <c r="A104" s="64" t="inlineStr">
         <is>
           <t>K02</t>
         </is>
       </c>
-      <c r="B104" s="62" t="inlineStr">
+      <c r="B104" s="64" t="inlineStr">
         <is>
           <t>Torque driver</t>
         </is>
       </c>
-      <c r="C104" s="63" t="inlineStr">
+      <c r="C104" s="65" t="inlineStr">
         <is>
           <t>one-off</t>
         </is>
       </c>
-      <c r="E104" s="64" t="inlineStr">
+      <c r="E104" s="66" t="inlineStr">
         <is>
           <t>40.0</t>
         </is>
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="65" t="inlineStr">
+      <c r="A106" s="67" t="inlineStr">
         <is>
           <t>CUT - DEAD LINE, DO NOT BUY</t>
         </is>
       </c>
     </row>
     <row r="107" ht="15.5" customHeight="1">
-      <c r="A107" s="62" t="inlineStr">
+      <c r="A107" s="64" t="inlineStr">
         <is>
           <t>A05</t>
         </is>
       </c>
-      <c r="B107" s="62" t="inlineStr">
+      <c r="B107" s="64" t="inlineStr">
         <is>
           <t>Bearing carrier tube</t>
         </is>
       </c>
-      <c r="C107" s="63" t="inlineStr">
+      <c r="C107" s="65" t="inlineStr">
         <is>
           <t>CUT: superseded - the bearing carrier is the printed spider (wet_carrier)</t>
         </is>
       </c>
-      <c r="E107" s="66" t="inlineStr">
+      <c r="E107" s="68" t="inlineStr">
         <is>
           <t>1.2</t>
         </is>
       </c>
     </row>
     <row r="108" ht="15.5" customHeight="1">
-      <c r="A108" s="62" t="inlineStr">
+      <c r="A108" s="64" t="inlineStr">
         <is>
           <t>A07</t>
         </is>
       </c>
-      <c r="B108" s="62" t="inlineStr">
+      <c r="B108" s="64" t="inlineStr">
         <is>
           <t>Weed guard ring</t>
         </is>
       </c>
-      <c r="C108" s="63" t="inlineStr">
+      <c r="C108" s="65" t="inlineStr">
         <is>
           <t>CUT: killed by design - replaced by the nose cone D64-&gt;D12; a ring on struts upstream is an algae scythe</t>
         </is>
       </c>
-      <c r="E108" s="66" t="inlineStr">
+      <c r="E108" s="68" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="109" ht="15.5" customHeight="1">
-      <c r="A109" s="62" t="inlineStr">
+      <c r="A109" s="64" t="inlineStr">
         <is>
           <t>A08</t>
         </is>
       </c>
-      <c r="B109" s="62" t="inlineStr">
+      <c r="B109" s="64" t="inlineStr">
         <is>
           <t>Blade safety retainer</t>
         </is>
       </c>
-      <c r="C109" s="63" t="inlineStr">
+      <c r="C109" s="65" t="inlineStr">
         <is>
           <t>CUT: killed by design - a tether on a 110 mm blade is a flail, and the hole is a stress riser at the root</t>
         </is>
       </c>
-      <c r="E109" s="66" t="inlineStr">
+      <c r="E109" s="68" t="inlineStr">
         <is>
           <t>2.0</t>
         </is>
       </c>
     </row>
     <row r="110" ht="15.5" customHeight="1">
-      <c r="A110" s="62" t="inlineStr">
+      <c r="A110" s="64" t="inlineStr">
         <is>
           <t>G02</t>
         </is>
       </c>
-      <c r="B110" s="62" t="inlineStr">
+      <c r="B110" s="64" t="inlineStr">
         <is>
           <t>MCU (NOT USED in simple build)</t>
         </is>
       </c>
-      <c r="C110" s="63" t="inlineStr">
+      <c r="C110" s="65" t="inlineStr">
         <is>
           <t>DROPPED: Wio-E5 mini is the single brain (MCU+LoRa). Bring back only if we need more GPIO/dual-core.</t>
         </is>
       </c>
-      <c r="E110" s="66" t="inlineStr">
+      <c r="E110" s="68" t="inlineStr">
         <is>
           <t>0.0</t>
         </is>
@@ -2986,6 +2997,26 @@
     <mergeCell ref="A36:E36"/>
     <mergeCell ref="A3:F3"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B9" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B10" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B12" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B13" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B14" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B15" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B16" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B17" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B18" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B23" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B24" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B25" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B26" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B30" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B31" r:id="rId18"/>
+  </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
@@ -3548,10 +3579,10 @@
           <t>subtotal - Rotor &amp; drivetrain (wet side)</t>
         </is>
       </c>
-      <c r="B14" s="67" t="n"/>
-      <c r="C14" s="67" t="n"/>
-      <c r="D14" s="67" t="n"/>
-      <c r="E14" s="68" t="n"/>
+      <c r="B14" s="69" t="n"/>
+      <c r="C14" s="69" t="n"/>
+      <c r="D14" s="69" t="n"/>
+      <c r="E14" s="70" t="n"/>
       <c r="F14" s="15" t="n"/>
       <c r="G14" s="15" t="n">
         <v>8.16</v>
@@ -3621,7 +3652,7 @@
       </c>
       <c r="L17" s="6" t="inlineStr">
         <is>
-          <t>N52 D10x5, 8 per cup on a D70 cup; must be canned/epoxy - bare N52 corrodes in weeks | techfun ma N52 magnet kruhovy - over priemer; inak magsy.sk; 8 na kapsu, D10</t>
+          <t>N52 D10x5, 8 per cup on a D70 cup; must be canned/epoxy - bare N52 corrodes in weeks | 16x N52 D10x5; supermagnete ma presne tento diel, magsy over v prehliadaci</t>
         </is>
       </c>
     </row>
@@ -3787,7 +3818,11 @@
           <t>verified</t>
         </is>
       </c>
-      <c r="L20" s="6" t="inlineStr"/>
+      <c r="L20" s="6" t="inlineStr">
+        <is>
+          <t>techfun nema DP270; silikonova zalievacia hmota staci na test, epoxid je tuhsi</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="13" t="inlineStr">
@@ -3795,10 +3830,10 @@
           <t>subtotal - Magnetic coupling</t>
         </is>
       </c>
-      <c r="B21" s="67" t="n"/>
-      <c r="C21" s="67" t="n"/>
-      <c r="D21" s="67" t="n"/>
-      <c r="E21" s="68" t="n"/>
+      <c r="B21" s="69" t="n"/>
+      <c r="C21" s="69" t="n"/>
+      <c r="D21" s="69" t="n"/>
+      <c r="E21" s="70" t="n"/>
       <c r="F21" s="15" t="n"/>
       <c r="G21" s="15" t="n">
         <v>22.8</v>
@@ -4318,10 +4353,10 @@
           <t>subtotal - Generator pod &amp; sealing</t>
         </is>
       </c>
-      <c r="B33" s="67" t="n"/>
-      <c r="C33" s="67" t="n"/>
-      <c r="D33" s="67" t="n"/>
-      <c r="E33" s="68" t="n"/>
+      <c r="B33" s="69" t="n"/>
+      <c r="C33" s="69" t="n"/>
+      <c r="D33" s="69" t="n"/>
+      <c r="E33" s="70" t="n"/>
       <c r="F33" s="15" t="n"/>
       <c r="G33" s="15" t="n">
         <v>49</v>
@@ -4845,10 +4880,10 @@
           <t>subtotal - Sensors</t>
         </is>
       </c>
-      <c r="B45" s="67" t="n"/>
-      <c r="C45" s="67" t="n"/>
-      <c r="D45" s="67" t="n"/>
-      <c r="E45" s="68" t="n"/>
+      <c r="B45" s="69" t="n"/>
+      <c r="C45" s="69" t="n"/>
+      <c r="D45" s="69" t="n"/>
+      <c r="E45" s="70" t="n"/>
       <c r="F45" s="15" t="n"/>
       <c r="G45" s="15" t="n">
         <v>405.45</v>
@@ -5036,10 +5071,10 @@
           <t>subtotal - Sensor cage &amp; mounting</t>
         </is>
       </c>
-      <c r="B51" s="67" t="n"/>
-      <c r="C51" s="67" t="n"/>
-      <c r="D51" s="67" t="n"/>
-      <c r="E51" s="68" t="n"/>
+      <c r="B51" s="69" t="n"/>
+      <c r="C51" s="69" t="n"/>
+      <c r="D51" s="69" t="n"/>
+      <c r="E51" s="70" t="n"/>
       <c r="F51" s="15" t="n"/>
       <c r="G51" s="15" t="n">
         <v>6</v>
@@ -5171,10 +5206,10 @@
           <t>subtotal - Wet-dry interface (cable)</t>
         </is>
       </c>
-      <c r="B56" s="67" t="n"/>
-      <c r="C56" s="67" t="n"/>
-      <c r="D56" s="67" t="n"/>
-      <c r="E56" s="68" t="n"/>
+      <c r="B56" s="69" t="n"/>
+      <c r="C56" s="69" t="n"/>
+      <c r="D56" s="69" t="n"/>
+      <c r="E56" s="70" t="n"/>
       <c r="F56" s="15" t="n"/>
       <c r="G56" s="15" t="n">
         <v>47</v>
@@ -6142,10 +6177,10 @@
           <t>subtotal - Electronics (dry box)</t>
         </is>
       </c>
-      <c r="B76" s="67" t="n"/>
-      <c r="C76" s="67" t="n"/>
-      <c r="D76" s="67" t="n"/>
-      <c r="E76" s="68" t="n"/>
+      <c r="B76" s="69" t="n"/>
+      <c r="C76" s="69" t="n"/>
+      <c r="D76" s="69" t="n"/>
+      <c r="E76" s="70" t="n"/>
       <c r="F76" s="15" t="n"/>
       <c r="G76" s="15" t="n">
         <v>96.90000000000001</v>
@@ -6881,10 +6916,10 @@
           <t>subtotal - Structure &amp; site</t>
         </is>
       </c>
-      <c r="B92" s="67" t="n"/>
-      <c r="C92" s="67" t="n"/>
-      <c r="D92" s="67" t="n"/>
-      <c r="E92" s="68" t="n"/>
+      <c r="B92" s="69" t="n"/>
+      <c r="C92" s="69" t="n"/>
+      <c r="D92" s="69" t="n"/>
+      <c r="E92" s="70" t="n"/>
       <c r="F92" s="15" t="n"/>
       <c r="G92" s="15" t="n">
         <v>105</v>
@@ -7240,10 +7275,10 @@
           <t>subtotal - Gateway (base station)</t>
         </is>
       </c>
-      <c r="B101" s="67" t="n"/>
-      <c r="C101" s="67" t="n"/>
-      <c r="D101" s="67" t="n"/>
-      <c r="E101" s="68" t="n"/>
+      <c r="B101" s="69" t="n"/>
+      <c r="C101" s="69" t="n"/>
+      <c r="D101" s="69" t="n"/>
+      <c r="E101" s="70" t="n"/>
       <c r="F101" s="15" t="n"/>
       <c r="G101" s="15" t="n">
         <v>339</v>
@@ -7691,10 +7726,10 @@
           <t>subtotal - Consumables</t>
         </is>
       </c>
-      <c r="B112" s="67" t="n"/>
-      <c r="C112" s="67" t="n"/>
-      <c r="D112" s="67" t="n"/>
-      <c r="E112" s="68" t="n"/>
+      <c r="B112" s="69" t="n"/>
+      <c r="C112" s="69" t="n"/>
+      <c r="D112" s="69" t="n"/>
+      <c r="E112" s="70" t="n"/>
       <c r="F112" s="15" t="n"/>
       <c r="G112" s="15" t="n">
         <v>142</v>
@@ -7886,10 +7921,10 @@
           <t>subtotal - Tooling (one-off)</t>
         </is>
       </c>
-      <c r="B118" s="67" t="n"/>
-      <c r="C118" s="67" t="n"/>
-      <c r="D118" s="67" t="n"/>
-      <c r="E118" s="68" t="n"/>
+      <c r="B118" s="69" t="n"/>
+      <c r="C118" s="69" t="n"/>
+      <c r="D118" s="69" t="n"/>
+      <c r="E118" s="70" t="n"/>
       <c r="F118" s="15" t="n"/>
       <c r="G118" s="15" t="n">
         <v>130</v>
@@ -7906,11 +7941,11 @@
           <t>REQUIRED (everything needed to build and deploy)</t>
         </is>
       </c>
-      <c r="B120" s="67" t="n"/>
-      <c r="C120" s="67" t="n"/>
-      <c r="D120" s="67" t="n"/>
-      <c r="E120" s="67" t="n"/>
-      <c r="F120" s="68" t="n"/>
+      <c r="B120" s="69" t="n"/>
+      <c r="C120" s="69" t="n"/>
+      <c r="D120" s="69" t="n"/>
+      <c r="E120" s="69" t="n"/>
+      <c r="F120" s="70" t="n"/>
       <c r="G120" s="25" t="n">
         <v>710.3100000000001</v>
       </c>
@@ -7921,11 +7956,11 @@
           <t>recommended add-ons (DO, level probe, anti-theft, tools)</t>
         </is>
       </c>
-      <c r="B121" s="67" t="n"/>
-      <c r="C121" s="67" t="n"/>
-      <c r="D121" s="67" t="n"/>
-      <c r="E121" s="67" t="n"/>
-      <c r="F121" s="68" t="n"/>
+      <c r="B121" s="69" t="n"/>
+      <c r="C121" s="69" t="n"/>
+      <c r="D121" s="69" t="n"/>
+      <c r="E121" s="69" t="n"/>
+      <c r="F121" s="70" t="n"/>
       <c r="G121" s="27" t="n">
         <v>641</v>
       </c>
@@ -7936,11 +7971,11 @@
           <t>TOTAL if you buy everything</t>
         </is>
       </c>
-      <c r="B122" s="67" t="n"/>
-      <c r="C122" s="67" t="n"/>
-      <c r="D122" s="67" t="n"/>
-      <c r="E122" s="67" t="n"/>
-      <c r="F122" s="68" t="n"/>
+      <c r="B122" s="69" t="n"/>
+      <c r="C122" s="69" t="n"/>
+      <c r="D122" s="69" t="n"/>
+      <c r="E122" s="69" t="n"/>
+      <c r="F122" s="70" t="n"/>
       <c r="G122" s="29" t="n">
         <v>1351.31</v>
       </c>
@@ -7951,11 +7986,11 @@
           <t>saved by reusing what you already own</t>
         </is>
       </c>
-      <c r="B123" s="67" t="n"/>
-      <c r="C123" s="67" t="n"/>
-      <c r="D123" s="67" t="n"/>
-      <c r="E123" s="67" t="n"/>
-      <c r="F123" s="68" t="n"/>
+      <c r="B123" s="69" t="n"/>
+      <c r="C123" s="69" t="n"/>
+      <c r="D123" s="69" t="n"/>
+      <c r="E123" s="69" t="n"/>
+      <c r="F123" s="70" t="n"/>
       <c r="G123" s="31" t="n">
         <v>-70</v>
       </c>
@@ -7966,11 +8001,11 @@
           <t>net if you reuse your Raspberry Pi etc.</t>
         </is>
       </c>
-      <c r="B124" s="67" t="n"/>
-      <c r="C124" s="67" t="n"/>
-      <c r="D124" s="67" t="n"/>
-      <c r="E124" s="67" t="n"/>
-      <c r="F124" s="68" t="n"/>
+      <c r="B124" s="69" t="n"/>
+      <c r="C124" s="69" t="n"/>
+      <c r="D124" s="69" t="n"/>
+      <c r="E124" s="69" t="n"/>
+      <c r="F124" s="70" t="n"/>
       <c r="G124" s="33" t="n">
         <v>1281.31</v>
       </c>

</xml_diff>

<commit_message>
order: rpishop and supermagnete get their own bands
rpishop.cz was not in the shop map, so both radio lines were falling through to
'local / shop'; the magnets were labelled techfun because their source string
still started with techfun.sk. Both fixed, and B01 now points at the verified
supermagnete product page for the N52 D10x5.
</commit_message>
<xml_diff>
--- a/docs/sub-mission_parts.xlsx
+++ b/docs/sub-mission_parts.xlsx
@@ -809,7 +809,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F110"/>
+  <dimension ref="A1:F116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1202,7 +1202,7 @@
         </is>
       </c>
       <c r="F20" s="46" t="n">
-        <v>58.25</v>
+        <v>49.45</v>
       </c>
     </row>
     <row r="21">
@@ -1315,472 +1315,400 @@
         <v>12.45</v>
       </c>
     </row>
-    <row r="25" ht="29" customHeight="1">
+    <row r="25" ht="15.5" customHeight="1">
       <c r="A25" s="53" t="inlineStr">
         <is>
-          <t>B01</t>
+          <t>D04</t>
         </is>
       </c>
       <c r="B25" s="54" t="inlineStr">
         <is>
-          <t>Magnet</t>
+          <t>Temperature</t>
         </is>
       </c>
       <c r="C25" s="55" t="inlineStr">
         <is>
-          <t>N52 D10x5 axially magnetised, canned 316L or epoxy potted  -  16x N52 D10x5; supermagnete ma presne tento diel, magsy over v prehliadaci</t>
+          <t>DS18B20 waterproof 1m cable  -  in model as sensor_ntc</t>
         </is>
       </c>
       <c r="D25" s="56" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="E25" s="57" t="n">
-        <v>0.55</v>
+        <v>5</v>
       </c>
       <c r="F25" s="57" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="A27" s="45" t="inlineStr">
+        <is>
+          <t>RPISHOP.CZ</t>
+        </is>
+      </c>
+      <c r="F27" s="46" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="47" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B28" s="47" t="inlineStr">
+        <is>
+          <t>Part</t>
+        </is>
+      </c>
+      <c r="C28" s="47" t="inlineStr">
+        <is>
+          <t>Specification / note</t>
+        </is>
+      </c>
+      <c r="D28" s="48" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="E28" s="48" t="inlineStr">
+        <is>
+          <t>Unit EUR</t>
+        </is>
+      </c>
+      <c r="F28" s="48" t="inlineStr">
+        <is>
+          <t>Total EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="42.5" customHeight="1">
+      <c r="A29" s="49" t="inlineStr">
+        <is>
+          <t>G03</t>
+        </is>
+      </c>
+      <c r="B29" s="50" t="inlineStr">
+        <is>
+          <t>MCU + radio (single board)</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>Seeed XIAO nRF52840 + Wio-SX1262 kit (Meshtastic), SEE336 - nRF52840 + SX1262  -  349 Kc, skladom 5+; nahradza Wio-E5, ktory v CZ/SK nie je; antena je v kite</t>
+        </is>
+      </c>
+      <c r="D29" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" s="52" t="n">
+        <v>14</v>
+      </c>
+      <c r="F29" s="52" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="30" ht="42.5" customHeight="1">
+      <c r="A30" s="53" t="inlineStr">
+        <is>
+          <t>I01</t>
+        </is>
+      </c>
+      <c r="B30" s="54" t="inlineStr">
+        <is>
+          <t>Gateway radio (single-channel)</t>
+        </is>
+      </c>
+      <c r="C30" s="55" t="inlineStr">
+        <is>
+          <t>Seeed XIAO nRF52840 + Wio-SX1262 kit (Meshtastic), SEE336 - nRF52840 + SX1262  -  349 Kc, skladom 5+; nahradza Wio-E5, ktory v CZ/SK nie je; antena je v kite</t>
+        </is>
+      </c>
+      <c r="D30" s="56" t="n">
+        <v>1</v>
+      </c>
+      <c r="E30" s="57" t="n">
+        <v>14</v>
+      </c>
+      <c r="F30" s="57" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="32" ht="20" customHeight="1">
+      <c r="A32" s="45" t="inlineStr">
+        <is>
+          <t>LOCAL / SHOP</t>
+        </is>
+      </c>
+      <c r="F32" s="46" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="47" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B33" s="47" t="inlineStr">
+        <is>
+          <t>Part</t>
+        </is>
+      </c>
+      <c r="C33" s="47" t="inlineStr">
+        <is>
+          <t>Specification / note</t>
+        </is>
+      </c>
+      <c r="D33" s="48" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="E33" s="48" t="inlineStr">
+        <is>
+          <t>Unit EUR</t>
+        </is>
+      </c>
+      <c r="F33" s="48" t="inlineStr">
+        <is>
+          <t>Total EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="15.5" customHeight="1">
+      <c r="A34" s="49" t="inlineStr">
+        <is>
+          <t>K03</t>
+        </is>
+      </c>
+      <c r="B34" s="49" t="inlineStr">
+        <is>
+          <t>Spring balance</t>
+        </is>
+      </c>
+      <c r="C34" s="6" t="inlineStr">
+        <is>
+          <t>0-5N for coupling slip jig  -  one-off</t>
+        </is>
+      </c>
+      <c r="D34" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="E34" s="52" t="n">
+        <v>5</v>
+      </c>
+      <c r="F34" s="52" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="35" ht="15.5" customHeight="1">
+      <c r="A35" s="53" t="inlineStr">
+        <is>
+          <t>C06</t>
+        </is>
+      </c>
+      <c r="B35" s="53" t="inlineStr">
+        <is>
+          <t>Desiccant</t>
+        </is>
+      </c>
+      <c r="C35" s="55" t="inlineStr">
+        <is>
+          <t>5g silica gel with indicator  -  replace at service</t>
+        </is>
+      </c>
+      <c r="D35" s="56" t="n">
+        <v>2</v>
+      </c>
+      <c r="E35" s="57" t="n">
+        <v>2</v>
+      </c>
+      <c r="F35" s="57" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="36" ht="29" customHeight="1">
+      <c r="A36" s="49" t="inlineStr">
+        <is>
+          <t>C04</t>
+        </is>
+      </c>
+      <c r="B36" s="49" t="inlineStr">
+        <is>
+          <t>O-ring groove</t>
+        </is>
+      </c>
+      <c r="C36" s="6" t="inlineStr">
+        <is>
+          <t>2.2mm wide x 1.8mm deep machined/printed into pod rim  -  NOT YET IN MODEL - add to pod</t>
+        </is>
+      </c>
+      <c r="D36" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="E36" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="F36" s="52" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" ht="20" customHeight="1">
+      <c r="A38" s="45" t="inlineStr">
+        <is>
+          <t>SUPERMAGNETICSHOP</t>
+        </is>
+      </c>
+      <c r="F38" s="46" t="n">
         <v>8.800000000000001</v>
       </c>
     </row>
-    <row r="26" ht="15.5" customHeight="1">
-      <c r="A26" s="49" t="inlineStr">
-        <is>
-          <t>D04</t>
-        </is>
-      </c>
-      <c r="B26" s="50" t="inlineStr">
-        <is>
-          <t>Temperature</t>
-        </is>
-      </c>
-      <c r="C26" s="6" t="inlineStr">
-        <is>
-          <t>DS18B20 waterproof 1m cable  -  in model as sensor_ntc</t>
-        </is>
-      </c>
-      <c r="D26" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="E26" s="52" t="n">
-        <v>5</v>
-      </c>
-      <c r="F26" s="52" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="28" ht="20" customHeight="1">
-      <c r="A28" s="45" t="inlineStr">
-        <is>
-          <t>LOCAL / SHOP</t>
-        </is>
-      </c>
-      <c r="F28" s="46" t="n">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="47" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="47" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B29" s="47" t="inlineStr">
+      <c r="B39" s="47" t="inlineStr">
         <is>
           <t>Part</t>
         </is>
       </c>
-      <c r="C29" s="47" t="inlineStr">
+      <c r="C39" s="47" t="inlineStr">
         <is>
           <t>Specification / note</t>
         </is>
       </c>
-      <c r="D29" s="48" t="inlineStr">
+      <c r="D39" s="48" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="E29" s="48" t="inlineStr">
+      <c r="E39" s="48" t="inlineStr">
         <is>
           <t>Unit EUR</t>
         </is>
       </c>
-      <c r="F29" s="48" t="inlineStr">
+      <c r="F39" s="48" t="inlineStr">
         <is>
           <t>Total EUR</t>
         </is>
-      </c>
-    </row>
-    <row r="30" ht="42.5" customHeight="1">
-      <c r="A30" s="49" t="inlineStr">
-        <is>
-          <t>G03</t>
-        </is>
-      </c>
-      <c r="B30" s="50" t="inlineStr">
-        <is>
-          <t>MCU + radio (single board)</t>
-        </is>
-      </c>
-      <c r="C30" s="6" t="inlineStr">
-        <is>
-          <t>Seeed XIAO nRF52840 + Wio-SX1262 kit (Meshtastic), SEE336 - nRF52840 + SX1262  -  349 Kc, skladom 5+; nahradza Wio-E5, ktory v CZ/SK nie je; antena je v kite</t>
-        </is>
-      </c>
-      <c r="D30" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="E30" s="52" t="n">
-        <v>14</v>
-      </c>
-      <c r="F30" s="52" t="n">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="31" ht="42.5" customHeight="1">
-      <c r="A31" s="53" t="inlineStr">
-        <is>
-          <t>I01</t>
-        </is>
-      </c>
-      <c r="B31" s="54" t="inlineStr">
-        <is>
-          <t>Gateway radio (single-channel)</t>
-        </is>
-      </c>
-      <c r="C31" s="55" t="inlineStr">
-        <is>
-          <t>Seeed XIAO nRF52840 + Wio-SX1262 kit (Meshtastic), SEE336 - nRF52840 + SX1262  -  349 Kc, skladom 5+; nahradza Wio-E5, ktory v CZ/SK nie je; antena je v kite</t>
-        </is>
-      </c>
-      <c r="D31" s="56" t="n">
-        <v>1</v>
-      </c>
-      <c r="E31" s="57" t="n">
-        <v>14</v>
-      </c>
-      <c r="F31" s="57" t="n">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="32" ht="15.5" customHeight="1">
-      <c r="A32" s="49" t="inlineStr">
-        <is>
-          <t>K03</t>
-        </is>
-      </c>
-      <c r="B32" s="49" t="inlineStr">
-        <is>
-          <t>Spring balance</t>
-        </is>
-      </c>
-      <c r="C32" s="6" t="inlineStr">
-        <is>
-          <t>0-5N for coupling slip jig  -  one-off</t>
-        </is>
-      </c>
-      <c r="D32" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="E32" s="52" t="n">
-        <v>5</v>
-      </c>
-      <c r="F32" s="52" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="33" ht="15.5" customHeight="1">
-      <c r="A33" s="53" t="inlineStr">
-        <is>
-          <t>C06</t>
-        </is>
-      </c>
-      <c r="B33" s="53" t="inlineStr">
-        <is>
-          <t>Desiccant</t>
-        </is>
-      </c>
-      <c r="C33" s="55" t="inlineStr">
-        <is>
-          <t>5g silica gel with indicator  -  replace at service</t>
-        </is>
-      </c>
-      <c r="D33" s="56" t="n">
-        <v>2</v>
-      </c>
-      <c r="E33" s="57" t="n">
-        <v>2</v>
-      </c>
-      <c r="F33" s="57" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="34" ht="29" customHeight="1">
-      <c r="A34" s="49" t="inlineStr">
-        <is>
-          <t>C04</t>
-        </is>
-      </c>
-      <c r="B34" s="49" t="inlineStr">
-        <is>
-          <t>O-ring groove</t>
-        </is>
-      </c>
-      <c r="C34" s="6" t="inlineStr">
-        <is>
-          <t>2.2mm wide x 1.8mm deep machined/printed into pod rim  -  NOT YET IN MODEL - add to pod</t>
-        </is>
-      </c>
-      <c r="D34" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="E34" s="52" t="n">
-        <v>0</v>
-      </c>
-      <c r="F34" s="52" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36" ht="20" customHeight="1">
-      <c r="A36" s="45" t="inlineStr">
-        <is>
-          <t>PRINTED IN-HOUSE</t>
-        </is>
-      </c>
-      <c r="F36" s="46" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="47" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B37" s="47" t="inlineStr">
-        <is>
-          <t>Part</t>
-        </is>
-      </c>
-      <c r="C37" s="47" t="inlineStr">
-        <is>
-          <t>Specification / note</t>
-        </is>
-      </c>
-      <c r="D37" s="48" t="inlineStr">
-        <is>
-          <t>Qty</t>
-        </is>
-      </c>
-      <c r="E37" s="48" t="inlineStr">
-        <is>
-          <t>Unit EUR</t>
-        </is>
-      </c>
-      <c r="F37" s="48" t="inlineStr">
-        <is>
-          <t>Total EUR</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="15.5" customHeight="1">
-      <c r="A38" s="49" t="inlineStr">
-        <is>
-          <t>C09</t>
-        </is>
-      </c>
-      <c r="B38" s="49" t="inlineStr">
-        <is>
-          <t>Generator mount</t>
-        </is>
-      </c>
-      <c r="C38" s="6" t="inlineStr">
-        <is>
-          <t>printed cradle + 4x M3x8 A4</t>
-        </is>
-      </c>
-      <c r="D38" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="E38" s="52" t="n">
-        <v>1</v>
-      </c>
-      <c r="F38" s="52" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="39" ht="29" customHeight="1">
-      <c r="A39" s="53" t="inlineStr">
-        <is>
-          <t>A01</t>
-        </is>
-      </c>
-      <c r="B39" s="53" t="inlineStr">
-        <is>
-          <t>Blade</t>
-        </is>
-      </c>
-      <c r="C39" s="55" t="inlineStr">
-        <is>
-          <t>triple-blade rotor blade NACA4412 D220mm root pitch 28deg tip 2deg  -  ASA or ASA-CF; 6 perimeters; epoxy coat; spare blade = fuse for branch strike</t>
-        </is>
-      </c>
-      <c r="D39" s="56" t="n">
-        <v>3</v>
-      </c>
-      <c r="E39" s="57" t="n">
-        <v>0</v>
-      </c>
-      <c r="F39" s="57" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="40" ht="29" customHeight="1">
       <c r="A40" s="49" t="inlineStr">
         <is>
-          <t>A02</t>
-        </is>
-      </c>
-      <c r="B40" s="49" t="inlineStr">
-        <is>
-          <t>Hub</t>
+          <t>B01</t>
+        </is>
+      </c>
+      <c r="B40" s="50" t="inlineStr">
+        <is>
+          <t>Magnet</t>
         </is>
       </c>
       <c r="C40" s="6" t="inlineStr">
         <is>
-          <t>Ø64x46mm with 2x M4 heat-set inserts and Ø5 H7 shaft bore  -  brass inserts M4 from TME</t>
+          <t>N52 D10x5 axially magnetised, canned 316L or epoxy potted  -  16x N52 D10x5 (S-10-05-N52N, 3.3 kg); magsy 10x5 N52 nemá overený</t>
         </is>
       </c>
       <c r="D40" s="51" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="E40" s="52" t="n">
-        <v>0</v>
+        <v>0.55</v>
       </c>
       <c r="F40" s="52" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41" ht="29" customHeight="1">
-      <c r="A41" s="53" t="inlineStr">
-        <is>
-          <t>B02</t>
-        </is>
-      </c>
-      <c r="B41" s="53" t="inlineStr">
-        <is>
-          <t>Magnet cup</t>
-        </is>
-      </c>
-      <c r="C41" s="55" t="inlineStr">
-        <is>
-          <t>D70 rim, 8 pockets D10.2x5.2, printed ASA  -  pockets 10.2 dia (magnet 10 + 0.2 glue), 0.2 mm epoxy recess</t>
-        </is>
-      </c>
-      <c r="D41" s="56" t="n">
-        <v>2</v>
-      </c>
-      <c r="E41" s="57" t="n">
-        <v>0</v>
-      </c>
-      <c r="F41" s="57" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42" ht="15.5" customHeight="1">
-      <c r="A42" s="49" t="inlineStr">
-        <is>
-          <t>C01</t>
-        </is>
-      </c>
-      <c r="B42" s="49" t="inlineStr">
-        <is>
-          <t>Pod barrel</t>
-        </is>
-      </c>
-      <c r="C42" s="6" t="inlineStr">
-        <is>
-          <t>Ø110x120mm printed ASA wall 2.4mm + epoxy barrier  -  in model as pod</t>
-        </is>
-      </c>
-      <c r="D42" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="E42" s="52" t="n">
-        <v>0</v>
-      </c>
-      <c r="F42" s="52" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43" ht="15.5" customHeight="1">
-      <c r="A43" s="53" t="inlineStr">
-        <is>
-          <t>C02</t>
-        </is>
-      </c>
-      <c r="B43" s="53" t="inlineStr">
-        <is>
-          <t>Tail cone</t>
-        </is>
-      </c>
-      <c r="C43" s="55" t="inlineStr">
-        <is>
-          <t>printed integral</t>
-        </is>
-      </c>
-      <c r="D43" s="56" t="n">
-        <v>1</v>
-      </c>
-      <c r="E43" s="57" t="n">
-        <v>0</v>
-      </c>
-      <c r="F43" s="57" t="n">
-        <v>0</v>
+        <v>8.800000000000001</v>
+      </c>
+    </row>
+    <row r="42" ht="20" customHeight="1">
+      <c r="A42" s="45" t="inlineStr">
+        <is>
+          <t>PRINTED IN-HOUSE</t>
+        </is>
+      </c>
+      <c r="F42" s="46" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="47" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B43" s="47" t="inlineStr">
+        <is>
+          <t>Part</t>
+        </is>
+      </c>
+      <c r="C43" s="47" t="inlineStr">
+        <is>
+          <t>Specification / note</t>
+        </is>
+      </c>
+      <c r="D43" s="48" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="E43" s="48" t="inlineStr">
+        <is>
+          <t>Unit EUR</t>
+        </is>
+      </c>
+      <c r="F43" s="48" t="inlineStr">
+        <is>
+          <t>Total EUR</t>
+        </is>
       </c>
     </row>
     <row r="44" ht="15.5" customHeight="1">
       <c r="A44" s="49" t="inlineStr">
         <is>
-          <t>E01</t>
+          <t>C09</t>
         </is>
       </c>
       <c r="B44" s="49" t="inlineStr">
         <is>
-          <t>Sensor cage</t>
+          <t>Generator mount</t>
         </is>
       </c>
       <c r="C44" s="6" t="inlineStr">
         <is>
-          <t>Ø130x150 printed ASA 12 slots  -  in model as cage</t>
+          <t>printed cradle + 4x M3x8 A4</t>
         </is>
       </c>
       <c r="D44" s="51" t="n">
         <v>1</v>
       </c>
       <c r="E44" s="52" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F44" s="52" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="45" ht="29" customHeight="1">
       <c r="A45" s="53" t="inlineStr">
         <is>
-          <t>E03</t>
+          <t>A01</t>
         </is>
       </c>
       <c r="B45" s="53" t="inlineStr">
         <is>
-          <t>Sensor holders</t>
+          <t>Blade</t>
         </is>
       </c>
       <c r="C45" s="55" t="inlineStr">
         <is>
-          <t>printed clips for pH/TDS/turbidity/NTC/MS5837  -  in model as sensor bodies</t>
+          <t>triple-blade rotor blade NACA4412 D220mm root pitch 28deg tip 2deg  -  ASA or ASA-CF; 6 perimeters; epoxy coat; spare blade = fuse for branch strike</t>
         </is>
       </c>
       <c r="D45" s="56" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E45" s="57" t="n">
         <v>0</v>
@@ -1789,1213 +1717,1371 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" ht="20" customHeight="1">
-      <c r="A47" s="45" t="inlineStr">
+    <row r="46" ht="29" customHeight="1">
+      <c r="A46" s="49" t="inlineStr">
+        <is>
+          <t>A02</t>
+        </is>
+      </c>
+      <c r="B46" s="49" t="inlineStr">
+        <is>
+          <t>Hub</t>
+        </is>
+      </c>
+      <c r="C46" s="6" t="inlineStr">
+        <is>
+          <t>Ø64x46mm with 2x M4 heat-set inserts and Ø5 H7 shaft bore  -  brass inserts M4 from TME</t>
+        </is>
+      </c>
+      <c r="D46" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="E46" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="F46" s="52" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" ht="29" customHeight="1">
+      <c r="A47" s="53" t="inlineStr">
+        <is>
+          <t>B02</t>
+        </is>
+      </c>
+      <c r="B47" s="53" t="inlineStr">
+        <is>
+          <t>Magnet cup</t>
+        </is>
+      </c>
+      <c r="C47" s="55" t="inlineStr">
+        <is>
+          <t>D70 rim, 8 pockets D10.2x5.2, printed ASA  -  pockets 10.2 dia (magnet 10 + 0.2 glue), 0.2 mm epoxy recess</t>
+        </is>
+      </c>
+      <c r="D47" s="56" t="n">
+        <v>2</v>
+      </c>
+      <c r="E47" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="F47" s="57" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" ht="15.5" customHeight="1">
+      <c r="A48" s="49" t="inlineStr">
+        <is>
+          <t>C01</t>
+        </is>
+      </c>
+      <c r="B48" s="49" t="inlineStr">
+        <is>
+          <t>Pod barrel</t>
+        </is>
+      </c>
+      <c r="C48" s="6" t="inlineStr">
+        <is>
+          <t>Ø110x120mm printed ASA wall 2.4mm + epoxy barrier  -  in model as pod</t>
+        </is>
+      </c>
+      <c r="D48" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="E48" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="F48" s="52" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" ht="15.5" customHeight="1">
+      <c r="A49" s="53" t="inlineStr">
+        <is>
+          <t>C02</t>
+        </is>
+      </c>
+      <c r="B49" s="53" t="inlineStr">
+        <is>
+          <t>Tail cone</t>
+        </is>
+      </c>
+      <c r="C49" s="55" t="inlineStr">
+        <is>
+          <t>printed integral</t>
+        </is>
+      </c>
+      <c r="D49" s="56" t="n">
+        <v>1</v>
+      </c>
+      <c r="E49" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="F49" s="57" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" ht="15.5" customHeight="1">
+      <c r="A50" s="49" t="inlineStr">
+        <is>
+          <t>E01</t>
+        </is>
+      </c>
+      <c r="B50" s="49" t="inlineStr">
+        <is>
+          <t>Sensor cage</t>
+        </is>
+      </c>
+      <c r="C50" s="6" t="inlineStr">
+        <is>
+          <t>Ø130x150 printed ASA 12 slots  -  in model as cage</t>
+        </is>
+      </c>
+      <c r="D50" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="E50" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="F50" s="52" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" ht="29" customHeight="1">
+      <c r="A51" s="53" t="inlineStr">
+        <is>
+          <t>E03</t>
+        </is>
+      </c>
+      <c r="B51" s="53" t="inlineStr">
+        <is>
+          <t>Sensor holders</t>
+        </is>
+      </c>
+      <c r="C51" s="55" t="inlineStr">
+        <is>
+          <t>printed clips for pH/TDS/turbidity/NTC/MS5837  -  in model as sensor bodies</t>
+        </is>
+      </c>
+      <c r="D51" s="56" t="n">
+        <v>5</v>
+      </c>
+      <c r="E51" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="F51" s="57" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" ht="20" customHeight="1">
+      <c r="A53" s="45" t="inlineStr">
         <is>
           <t>NEREZMATERIAL.CZ</t>
         </is>
       </c>
-      <c r="F47" s="46" t="n">
+      <c r="F53" s="46" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="47" t="inlineStr">
+    <row r="54">
+      <c r="A54" s="47" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B48" s="47" t="inlineStr">
+      <c r="B54" s="47" t="inlineStr">
         <is>
           <t>Part</t>
         </is>
       </c>
-      <c r="C48" s="47" t="inlineStr">
+      <c r="C54" s="47" t="inlineStr">
         <is>
           <t>Specification / note</t>
         </is>
       </c>
-      <c r="D48" s="48" t="inlineStr">
+      <c r="D54" s="48" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="E48" s="48" t="inlineStr">
+      <c r="E54" s="48" t="inlineStr">
         <is>
           <t>Unit EUR</t>
         </is>
       </c>
-      <c r="F48" s="48" t="inlineStr">
+      <c r="F54" s="48" t="inlineStr">
         <is>
           <t>Total EUR</t>
         </is>
       </c>
     </row>
-    <row r="49" ht="29" customHeight="1">
-      <c r="A49" s="49" t="inlineStr">
+    <row r="55" ht="29" customHeight="1">
+      <c r="A55" s="49" t="inlineStr">
         <is>
           <t>B03</t>
         </is>
       </c>
-      <c r="B49" s="49" t="inlineStr">
+      <c r="B55" s="49" t="inlineStr">
         <is>
           <t>Separation wall</t>
         </is>
       </c>
-      <c r="C49" s="6" t="inlineStr">
+      <c r="C55" s="6" t="inlineStr">
         <is>
           <t>D106 x 4 mm - RECOMMENDED integral with the pod bulkhead (no separate part)  -  4 mm per CAD, not 5; integral removes O-ring C03 and screws C05</t>
         </is>
       </c>
-      <c r="D49" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="E49" s="52" t="n">
+      <c r="D55" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="E55" s="52" t="n">
         <v>0</v>
       </c>
-      <c r="F49" s="52" t="n">
+      <c r="F55" s="52" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="51" ht="18" customHeight="1">
-      <c r="A51" s="58" t="inlineStr">
+    <row r="57" ht="18" customHeight="1">
+      <c r="A57" s="58" t="inlineStr">
         <is>
           <t>GOODS</t>
         </is>
       </c>
-      <c r="F51" s="59" t="n">
+      <c r="F57" s="59" t="n">
         <v>214.61</v>
       </c>
     </row>
-    <row r="52" ht="18" customHeight="1">
-      <c r="A52" s="58" t="inlineStr">
+    <row r="58" ht="18" customHeight="1">
+      <c r="A58" s="58" t="inlineStr">
         <is>
           <t>shipping, estimated</t>
         </is>
       </c>
-      <c r="F52" s="59" t="n">
+      <c r="F58" s="59" t="n">
         <v>25</v>
       </c>
     </row>
-    <row r="53" ht="22" customHeight="1">
-      <c r="A53" s="60" t="inlineStr">
+    <row r="59" ht="22" customHeight="1">
+      <c r="A59" s="60" t="inlineStr">
         <is>
           <t>LANDED TOTAL</t>
         </is>
       </c>
-      <c r="F53" s="61" t="n">
+      <c r="F59" s="61" t="n">
         <v>239.61</v>
       </c>
     </row>
-    <row r="56" ht="22" customHeight="1">
-      <c r="A56" s="62" t="inlineStr">
+    <row r="62" ht="22" customHeight="1">
+      <c r="A62" s="62" t="inlineStr">
         <is>
           <t>NOT IN THIS ORDER</t>
         </is>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" s="63" t="inlineStr">
+    <row r="63">
+      <c r="A63" s="63" t="inlineStr">
         <is>
           <t>PHASE 2 - BUY LATER</t>
         </is>
       </c>
     </row>
-    <row r="58" ht="29" customHeight="1">
-      <c r="A58" s="64" t="inlineStr">
+    <row r="64" ht="29" customHeight="1">
+      <c r="A64" s="64" t="inlineStr">
         <is>
           <t>A03</t>
         </is>
       </c>
-      <c r="B58" s="64" t="inlineStr">
+      <c r="B64" s="64" t="inlineStr">
         <is>
           <t>Wet shaft</t>
         </is>
       </c>
-      <c r="C58" s="65" t="inlineStr">
+      <c r="C64" s="65" t="inlineStr">
         <is>
           <t>lokalny zeleziar / Hornbach M5 A4 srob - 4. obchod sa nerata, nema postu; 3m bar 63.1 CZK makes ~26 shafts</t>
         </is>
       </c>
-      <c r="E58" s="66" t="inlineStr">
+      <c r="E64" s="66" t="inlineStr">
         <is>
           <t>2.6</t>
         </is>
       </c>
     </row>
-    <row r="59" ht="29" customHeight="1">
-      <c r="A59" s="64" t="inlineStr">
+    <row r="65" ht="29" customHeight="1">
+      <c r="A65" s="64" t="inlineStr">
         <is>
           <t>C08</t>
         </is>
       </c>
-      <c r="B59" s="64" t="inlineStr">
+      <c r="B65" s="64" t="inlineStr">
         <is>
           <t>Generator</t>
         </is>
       </c>
-      <c r="C59" s="65" t="inlineStr">
+      <c r="C65" s="65" t="inlineStr">
         <is>
           <t>TEST BEZ GENERATORA: klietka + senzory stacia, generator je dalsi nakup; XTG3506 preferred: encoder = free RPM/flow</t>
         </is>
       </c>
-      <c r="E59" s="66" t="inlineStr">
+      <c r="E65" s="66" t="inlineStr">
         <is>
           <t>26.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="60" ht="15.5" customHeight="1">
-      <c r="A60" s="64" t="inlineStr">
-        <is>
-          <t>D01</t>
-        </is>
-      </c>
-      <c r="B60" s="64" t="inlineStr">
-        <is>
-          <t>pH electrode</t>
-        </is>
-      </c>
-      <c r="C60" s="65" t="inlineStr">
-        <is>
-          <t>OPTIONAL per site; 14-30 day service; +-0.1 pH after 2-pt cal</t>
-        </is>
-      </c>
-      <c r="E60" s="66" t="inlineStr">
-        <is>
-          <t>39.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="61" ht="15.5" customHeight="1">
-      <c r="A61" s="64" t="inlineStr">
-        <is>
-          <t>D02</t>
-        </is>
-      </c>
-      <c r="B61" s="64" t="inlineStr">
-        <is>
-          <t>pH spare electrode</t>
-        </is>
-      </c>
-      <c r="C61" s="65" t="inlineStr">
-        <is>
-          <t>consumable</t>
-        </is>
-      </c>
-      <c r="E61" s="66" t="inlineStr">
-        <is>
-          <t>9.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="62" ht="15.5" customHeight="1">
-      <c r="A62" s="64" t="inlineStr">
-        <is>
-          <t>D03</t>
-        </is>
-      </c>
-      <c r="B62" s="64" t="inlineStr">
-        <is>
-          <t>pH buffer</t>
-        </is>
-      </c>
-      <c r="C62" s="65" t="inlineStr">
-        <is>
-          <t>consumable</t>
-        </is>
-      </c>
-      <c r="E62" s="66" t="inlineStr">
-        <is>
-          <t>12.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="63" ht="29" customHeight="1">
-      <c r="A63" s="64" t="inlineStr">
-        <is>
-          <t>D09</t>
-        </is>
-      </c>
-      <c r="B63" s="64" t="inlineStr">
-        <is>
-          <t>Dissolved oxygen kit</t>
-        </is>
-      </c>
-      <c r="C63" s="65" t="inlineStr">
-        <is>
-          <t>HIGHEST-VALUE channel (Budca = hypoxia); membrane 1-2 months in muddy water; 0.5M NaOH filling solution NOT shipped by air - source locally</t>
-        </is>
-      </c>
-      <c r="E63" s="66" t="inlineStr">
-        <is>
-          <t>175.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="64" ht="15.5" customHeight="1">
-      <c r="A64" s="64" t="inlineStr">
-        <is>
-          <t>D05</t>
-        </is>
-      </c>
-      <c r="B64" s="64" t="inlineStr">
-        <is>
-          <t>Level / stage probe</t>
-        </is>
-      </c>
-      <c r="C64" s="65" t="inlineStr">
-        <is>
-          <t>MS5837-30BA REJECTED: gel element must be dried daily, 24h max submersion</t>
-        </is>
-      </c>
-      <c r="E64" s="66" t="inlineStr">
-        <is>
-          <t>110.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="65" ht="15.5" customHeight="1">
-      <c r="A65" s="64" t="inlineStr">
-        <is>
-          <t>D06</t>
-        </is>
-      </c>
-      <c r="B65" s="64" t="inlineStr">
-        <is>
-          <t>EC/TDS</t>
-        </is>
-      </c>
-      <c r="C65" s="65" t="inlineStr">
-        <is>
-          <t>+-10% FS is the weakest sensor; use as trend indicator, site-calibrate</t>
-        </is>
-      </c>
-      <c r="E65" s="66" t="inlineStr">
-        <is>
-          <t>14.0</t>
         </is>
       </c>
     </row>
     <row r="66" ht="15.5" customHeight="1">
       <c r="A66" s="64" t="inlineStr">
         <is>
-          <t>D08</t>
+          <t>D01</t>
         </is>
       </c>
       <c r="B66" s="64" t="inlineStr">
         <is>
-          <t>Sensor cable</t>
-        </is>
-      </c>
-      <c r="C66" s="65" t="inlineStr"/>
+          <t>pH electrode</t>
+        </is>
+      </c>
+      <c r="C66" s="65" t="inlineStr">
+        <is>
+          <t>OPTIONAL per site; 14-30 day service; +-0.1 pH after 2-pt cal</t>
+        </is>
+      </c>
       <c r="E66" s="66" t="inlineStr">
         <is>
-          <t>20.0</t>
+          <t>39.0</t>
         </is>
       </c>
     </row>
     <row r="67" ht="15.5" customHeight="1">
       <c r="A67" s="64" t="inlineStr">
         <is>
-          <t>G04</t>
+          <t>D02</t>
         </is>
       </c>
       <c r="B67" s="64" t="inlineStr">
         <is>
-          <t>Antenna probe</t>
+          <t>pH spare electrode</t>
         </is>
       </c>
       <c r="C67" s="65" t="inlineStr">
         <is>
-          <t>v baleni kazdej Wio-E5 je EU868 antena - samostatne netreba; drzat ako zalohu</t>
+          <t>consumable</t>
         </is>
       </c>
       <c r="E67" s="66" t="inlineStr">
         <is>
-          <t>6.0</t>
+          <t>9.0</t>
         </is>
       </c>
     </row>
     <row r="68" ht="15.5" customHeight="1">
       <c r="A68" s="64" t="inlineStr">
         <is>
-          <t>G05</t>
+          <t>D03</t>
         </is>
       </c>
       <c r="B68" s="64" t="inlineStr">
         <is>
-          <t>Antenna pigtail</t>
+          <t>pH buffer</t>
         </is>
       </c>
       <c r="C68" s="65" t="inlineStr">
         <is>
-          <t>netreba: doska ma SMA, antena sa skrutkuje priamo; pigtail len ak sa ide cez bulkhead</t>
+          <t>consumable</t>
         </is>
       </c>
       <c r="E68" s="66" t="inlineStr">
         <is>
-          <t>3.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="69" ht="15.5" customHeight="1">
+          <t>12.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="29" customHeight="1">
       <c r="A69" s="64" t="inlineStr">
         <is>
-          <t>G06</t>
+          <t>D09</t>
         </is>
       </c>
       <c r="B69" s="64" t="inlineStr">
         <is>
-          <t>Boost harvester</t>
+          <t>Dissolved oxygen kit</t>
         </is>
       </c>
       <c r="C69" s="65" t="inlineStr">
         <is>
-          <t>needed when EMF below bus</t>
+          <t>HIGHEST-VALUE channel (Budca = hypoxia); membrane 1-2 months in muddy water; 0.5M NaOH filling solution NOT shipped by air - source locally</t>
         </is>
       </c>
       <c r="E69" s="66" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>175.0</t>
         </is>
       </c>
     </row>
     <row r="70" ht="15.5" customHeight="1">
       <c r="A70" s="64" t="inlineStr">
         <is>
-          <t>G07</t>
+          <t>D05</t>
         </is>
       </c>
       <c r="B70" s="64" t="inlineStr">
         <is>
-          <t>Buck</t>
-        </is>
-      </c>
-      <c r="C70" s="65" t="inlineStr"/>
+          <t>Level / stage probe</t>
+        </is>
+      </c>
+      <c r="C70" s="65" t="inlineStr">
+        <is>
+          <t>MS5837-30BA REJECTED: gel element must be dried daily, 24h max submersion</t>
+        </is>
+      </c>
       <c r="E70" s="66" t="inlineStr">
         <is>
-          <t>2.5</t>
+          <t>110.0</t>
         </is>
       </c>
     </row>
     <row r="71" ht="15.5" customHeight="1">
       <c r="A71" s="64" t="inlineStr">
         <is>
-          <t>G08</t>
+          <t>D06</t>
         </is>
       </c>
       <c r="B71" s="64" t="inlineStr">
         <is>
-          <t>Rectifier</t>
+          <t>EC/TDS</t>
         </is>
       </c>
       <c r="C71" s="65" t="inlineStr">
         <is>
-          <t>452k in stock</t>
+          <t>+-10% FS is the weakest sensor; use as trend indicator, site-calibrate</t>
         </is>
       </c>
       <c r="E71" s="66" t="inlineStr">
         <is>
-          <t>0.15</t>
+          <t>14.0</t>
         </is>
       </c>
     </row>
     <row r="72" ht="15.5" customHeight="1">
       <c r="A72" s="64" t="inlineStr">
         <is>
-          <t>G09</t>
+          <t>D08</t>
         </is>
       </c>
       <c r="B72" s="64" t="inlineStr">
         <is>
-          <t>Clamp</t>
-        </is>
-      </c>
-      <c r="C72" s="65" t="inlineStr">
-        <is>
-          <t>overvoltage protection</t>
-        </is>
-      </c>
+          <t>Sensor cable</t>
+        </is>
+      </c>
+      <c r="C72" s="65" t="inlineStr"/>
       <c r="E72" s="66" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>20.0</t>
         </is>
       </c>
     </row>
     <row r="73" ht="15.5" customHeight="1">
       <c r="A73" s="64" t="inlineStr">
         <is>
-          <t>G10</t>
+          <t>G04</t>
         </is>
       </c>
       <c r="B73" s="64" t="inlineStr">
         <is>
-          <t>Supercap</t>
+          <t>Antenna probe</t>
         </is>
       </c>
       <c r="C73" s="65" t="inlineStr">
         <is>
-          <t>NO coin-cell EDLC (50ohm ESR kills TX)</t>
+          <t>v baleni kazdej Wio-E5 je EU868 antena - samostatne netreba; drzat ako zalohu</t>
         </is>
       </c>
       <c r="E73" s="66" t="inlineStr">
         <is>
-          <t>11.0</t>
+          <t>6.0</t>
         </is>
       </c>
     </row>
     <row r="74" ht="15.5" customHeight="1">
       <c r="A74" s="64" t="inlineStr">
         <is>
-          <t>G11</t>
+          <t>G05</t>
         </is>
       </c>
       <c r="B74" s="64" t="inlineStr">
         <is>
-          <t>Voltage supervisor</t>
+          <t>Antenna pigtail</t>
         </is>
       </c>
       <c r="C74" s="65" t="inlineStr">
         <is>
-          <t>gates buck at 4.8V</t>
+          <t>netreba: doska ma SMA, antena sa skrutkuje priamo; pigtail len ak sa ide cez bulkhead</t>
         </is>
       </c>
       <c r="E74" s="66" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>3.0</t>
         </is>
       </c>
     </row>
     <row r="75" ht="15.5" customHeight="1">
       <c r="A75" s="64" t="inlineStr">
         <is>
-          <t>G12</t>
+          <t>G06</t>
         </is>
       </c>
       <c r="B75" s="64" t="inlineStr">
         <is>
-          <t>Load switch</t>
+          <t>Boost harvester</t>
         </is>
       </c>
       <c r="C75" s="65" t="inlineStr">
         <is>
-          <t>removes ground-loop need</t>
+          <t>needed when EMF below bus</t>
         </is>
       </c>
       <c r="E75" s="66" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>5.0</t>
         </is>
       </c>
     </row>
     <row r="76" ht="15.5" customHeight="1">
       <c r="A76" s="64" t="inlineStr">
         <is>
-          <t>G13</t>
+          <t>G07</t>
         </is>
       </c>
       <c r="B76" s="64" t="inlineStr">
         <is>
-          <t>Barometer</t>
-        </is>
-      </c>
-      <c r="C76" s="65" t="inlineStr">
-        <is>
-          <t>pressure reference for MS5837</t>
-        </is>
-      </c>
+          <t>Buck</t>
+        </is>
+      </c>
+      <c r="C76" s="65" t="inlineStr"/>
       <c r="E76" s="66" t="inlineStr">
         <is>
-          <t>6.0</t>
+          <t>2.5</t>
         </is>
       </c>
     </row>
     <row r="77" ht="15.5" customHeight="1">
       <c r="A77" s="64" t="inlineStr">
         <is>
-          <t>G14</t>
+          <t>G08</t>
         </is>
       </c>
       <c r="B77" s="64" t="inlineStr">
         <is>
-          <t>PCB</t>
+          <t>Rectifier</t>
         </is>
       </c>
       <c r="C77" s="65" t="inlineStr">
         <is>
-          <t>panel of 10 amortises</t>
+          <t>452k in stock</t>
         </is>
       </c>
       <c r="E77" s="66" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>0.15</t>
         </is>
       </c>
     </row>
     <row r="78" ht="15.5" customHeight="1">
       <c r="A78" s="64" t="inlineStr">
         <is>
-          <t>G15</t>
+          <t>G09</t>
         </is>
       </c>
       <c r="B78" s="64" t="inlineStr">
         <is>
-          <t>Connectors</t>
-        </is>
-      </c>
-      <c r="C78" s="65" t="inlineStr"/>
+          <t>Clamp</t>
+        </is>
+      </c>
+      <c r="C78" s="65" t="inlineStr">
+        <is>
+          <t>overvoltage protection</t>
+        </is>
+      </c>
       <c r="E78" s="66" t="inlineStr">
         <is>
-          <t>10.0</t>
+          <t>4.0</t>
         </is>
       </c>
     </row>
     <row r="79" ht="15.5" customHeight="1">
       <c r="A79" s="64" t="inlineStr">
         <is>
-          <t>H01</t>
+          <t>G10</t>
         </is>
       </c>
       <c r="B79" s="64" t="inlineStr">
         <is>
-          <t>Ground screw anchor</t>
+          <t>Supercap</t>
         </is>
       </c>
       <c r="C79" s="65" t="inlineStr">
         <is>
-          <t>1-2kN lateral - covers flood case</t>
+          <t>NO coin-cell EDLC (50ohm ESR kills TX)</t>
         </is>
       </c>
       <c r="E79" s="66" t="inlineStr">
         <is>
-          <t>25.0</t>
+          <t>11.0</t>
         </is>
       </c>
     </row>
     <row r="80" ht="15.5" customHeight="1">
       <c r="A80" s="64" t="inlineStr">
         <is>
-          <t>H02</t>
+          <t>G11</t>
         </is>
       </c>
       <c r="B80" s="64" t="inlineStr">
         <is>
-          <t>Pole</t>
+          <t>Voltage supervisor</t>
         </is>
       </c>
       <c r="C80" s="65" t="inlineStr">
         <is>
-          <t>removable mast pinned into receiver</t>
+          <t>gates buck at 4.8V</t>
         </is>
       </c>
       <c r="E80" s="66" t="inlineStr">
         <is>
-          <t>18.0</t>
+          <t>1.5</t>
         </is>
       </c>
     </row>
     <row r="81" ht="15.5" customHeight="1">
       <c r="A81" s="64" t="inlineStr">
         <is>
-          <t>H03</t>
+          <t>G12</t>
         </is>
       </c>
       <c r="B81" s="64" t="inlineStr">
         <is>
-          <t>Receiver sleeve</t>
+          <t>Load switch</t>
         </is>
       </c>
       <c r="C81" s="65" t="inlineStr">
         <is>
-          <t>pinned mast interface</t>
+          <t>removes ground-loop need</t>
         </is>
       </c>
       <c r="E81" s="66" t="inlineStr">
         <is>
-          <t>8.0</t>
+          <t>1.0</t>
         </is>
       </c>
     </row>
     <row r="82" ht="15.5" customHeight="1">
       <c r="A82" s="64" t="inlineStr">
         <is>
-          <t>H04</t>
+          <t>G13</t>
         </is>
       </c>
       <c r="B82" s="64" t="inlineStr">
         <is>
-          <t>Arm tube</t>
-        </is>
-      </c>
-      <c r="C82" s="65" t="inlineStr"/>
+          <t>Barometer</t>
+        </is>
+      </c>
+      <c r="C82" s="65" t="inlineStr">
+        <is>
+          <t>pressure reference for MS5837</t>
+        </is>
+      </c>
       <c r="E82" s="66" t="inlineStr">
         <is>
-          <t>9.0</t>
+          <t>6.0</t>
         </is>
       </c>
     </row>
     <row r="83" ht="15.5" customHeight="1">
       <c r="A83" s="64" t="inlineStr">
         <is>
-          <t>H05</t>
+          <t>G14</t>
         </is>
       </c>
       <c r="B83" s="64" t="inlineStr">
         <is>
-          <t>Drop tube</t>
-        </is>
-      </c>
-      <c r="C83" s="65" t="inlineStr"/>
+          <t>PCB</t>
+        </is>
+      </c>
+      <c r="C83" s="65" t="inlineStr">
+        <is>
+          <t>panel of 10 amortises</t>
+        </is>
+      </c>
       <c r="E83" s="66" t="inlineStr">
         <is>
-          <t>6.0</t>
+          <t>3.0</t>
         </is>
       </c>
     </row>
     <row r="84" ht="15.5" customHeight="1">
       <c r="A84" s="64" t="inlineStr">
         <is>
-          <t>H06</t>
+          <t>G15</t>
         </is>
       </c>
       <c r="B84" s="64" t="inlineStr">
         <is>
-          <t>Hinge collar</t>
+          <t>Connectors</t>
         </is>
       </c>
       <c r="C84" s="65" t="inlineStr"/>
       <c r="E84" s="66" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>10.0</t>
         </is>
       </c>
     </row>
     <row r="85" ht="15.5" customHeight="1">
       <c r="A85" s="64" t="inlineStr">
         <is>
-          <t>H07</t>
+          <t>H01</t>
         </is>
       </c>
       <c r="B85" s="64" t="inlineStr">
         <is>
-          <t>Shear pin</t>
+          <t>Ground screw anchor</t>
         </is>
       </c>
       <c r="C85" s="65" t="inlineStr">
         <is>
-          <t>releases pod on &gt;150N debris hit</t>
+          <t>1-2kN lateral - covers flood case</t>
         </is>
       </c>
       <c r="E85" s="66" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>25.0</t>
         </is>
       </c>
     </row>
     <row r="86" ht="15.5" customHeight="1">
       <c r="A86" s="64" t="inlineStr">
         <is>
-          <t>H08</t>
+          <t>H02</t>
         </is>
       </c>
       <c r="B86" s="64" t="inlineStr">
         <is>
-          <t>Yaw strut</t>
+          <t>Pole</t>
         </is>
       </c>
       <c r="C86" s="65" t="inlineStr">
         <is>
-          <t>anti-flutter</t>
+          <t>removable mast pinned into receiver</t>
         </is>
       </c>
       <c r="E86" s="66" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>18.0</t>
         </is>
       </c>
     </row>
     <row r="87" ht="15.5" customHeight="1">
       <c r="A87" s="64" t="inlineStr">
         <is>
-          <t>H09</t>
+          <t>H03</t>
         </is>
       </c>
       <c r="B87" s="64" t="inlineStr">
         <is>
-          <t>Guy line</t>
+          <t>Receiver sleeve</t>
         </is>
       </c>
       <c r="C87" s="65" t="inlineStr">
         <is>
-          <t>45deg up/downstream</t>
+          <t>pinned mast interface</t>
         </is>
       </c>
       <c r="E87" s="66" t="inlineStr">
         <is>
-          <t>9.0</t>
+          <t>8.0</t>
         </is>
       </c>
     </row>
     <row r="88" ht="15.5" customHeight="1">
       <c r="A88" s="64" t="inlineStr">
         <is>
-          <t>H10</t>
+          <t>H04</t>
         </is>
       </c>
       <c r="B88" s="64" t="inlineStr">
         <is>
-          <t>Guy anchor</t>
+          <t>Arm tube</t>
         </is>
       </c>
       <c r="C88" s="65" t="inlineStr"/>
       <c r="E88" s="66" t="inlineStr">
         <is>
-          <t>10.0</t>
+          <t>9.0</t>
         </is>
       </c>
     </row>
     <row r="89" ht="15.5" customHeight="1">
       <c r="A89" s="64" t="inlineStr">
         <is>
-          <t>H11</t>
+          <t>H05</t>
         </is>
       </c>
       <c r="B89" s="64" t="inlineStr">
         <is>
-          <t>Safety cable</t>
-        </is>
-      </c>
-      <c r="C89" s="65" t="inlineStr">
-        <is>
-          <t>theft/flood retention</t>
-        </is>
-      </c>
+          <t>Drop tube</t>
+        </is>
+      </c>
+      <c r="C89" s="65" t="inlineStr"/>
       <c r="E89" s="66" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>6.0</t>
         </is>
       </c>
     </row>
     <row r="90" ht="15.5" customHeight="1">
       <c r="A90" s="64" t="inlineStr">
         <is>
-          <t>H12</t>
+          <t>H06</t>
         </is>
       </c>
       <c r="B90" s="64" t="inlineStr">
         <is>
-          <t>Security fastener</t>
-        </is>
-      </c>
-      <c r="C90" s="65" t="inlineStr">
-        <is>
-          <t>anti-theft</t>
-        </is>
-      </c>
+          <t>Hinge collar</t>
+        </is>
+      </c>
+      <c r="C90" s="65" t="inlineStr"/>
       <c r="E90" s="66" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>3.0</t>
         </is>
       </c>
     </row>
     <row r="91" ht="15.5" customHeight="1">
       <c r="A91" s="64" t="inlineStr">
         <is>
-          <t>H13</t>
+          <t>H07</t>
         </is>
       </c>
       <c r="B91" s="64" t="inlineStr">
         <is>
-          <t>Site label</t>
+          <t>Shear pin</t>
         </is>
       </c>
       <c r="C91" s="65" t="inlineStr">
         <is>
-          <t>anti-theft by making it unsellable</t>
+          <t>releases pod on &gt;150N debris hit</t>
         </is>
       </c>
       <c r="E91" s="66" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>1.0</t>
         </is>
       </c>
     </row>
     <row r="92" ht="15.5" customHeight="1">
       <c r="A92" s="64" t="inlineStr">
         <is>
-          <t>I02</t>
+          <t>H08</t>
         </is>
       </c>
       <c r="B92" s="64" t="inlineStr">
         <is>
-          <t>Compute</t>
+          <t>Yaw strut</t>
         </is>
       </c>
       <c r="C92" s="65" t="inlineStr">
         <is>
-          <t>YOU ALREADY HAVE THIS - reuse, zero soldering; runs the gateway service</t>
+          <t>anti-flutter</t>
         </is>
       </c>
       <c r="E92" s="66" t="inlineStr">
         <is>
-          <t>70.0</t>
+          <t>5.0</t>
         </is>
       </c>
     </row>
     <row r="93" ht="15.5" customHeight="1">
       <c r="A93" s="64" t="inlineStr">
         <is>
-          <t>I03</t>
+          <t>H09</t>
         </is>
       </c>
       <c r="B93" s="64" t="inlineStr">
         <is>
-          <t>Antenna</t>
+          <t>Guy line</t>
         </is>
       </c>
       <c r="C93" s="65" t="inlineStr">
         <is>
-          <t>range-critical: gateway antenna gain + mast height set the link</t>
+          <t>45deg up/downstream</t>
         </is>
       </c>
       <c r="E93" s="66" t="inlineStr">
         <is>
-          <t>45.0</t>
+          <t>9.0</t>
         </is>
       </c>
     </row>
     <row r="94" ht="15.5" customHeight="1">
       <c r="A94" s="64" t="inlineStr">
         <is>
-          <t>I04</t>
+          <t>H10</t>
         </is>
       </c>
       <c r="B94" s="64" t="inlineStr">
         <is>
-          <t>Enclosure</t>
+          <t>Guy anchor</t>
         </is>
       </c>
       <c r="C94" s="65" t="inlineStr"/>
       <c r="E94" s="66" t="inlineStr">
         <is>
-          <t>35.0</t>
+          <t>10.0</t>
         </is>
       </c>
     </row>
     <row r="95" ht="15.5" customHeight="1">
       <c r="A95" s="64" t="inlineStr">
         <is>
-          <t>I05</t>
+          <t>H11</t>
         </is>
       </c>
       <c r="B95" s="64" t="inlineStr">
         <is>
-          <t>Mast</t>
+          <t>Safety cable</t>
         </is>
       </c>
       <c r="C95" s="65" t="inlineStr">
         <is>
-          <t>height sets range</t>
+          <t>theft/flood retention</t>
         </is>
       </c>
       <c r="E95" s="66" t="inlineStr">
         <is>
-          <t>30.0</t>
+          <t>4.0</t>
         </is>
       </c>
     </row>
     <row r="96" ht="15.5" customHeight="1">
       <c r="A96" s="64" t="inlineStr">
         <is>
-          <t>I06</t>
+          <t>H12</t>
         </is>
       </c>
       <c r="B96" s="64" t="inlineStr">
         <is>
-          <t>Concentrator upgrade (optional)</t>
+          <t>Security fastener</t>
         </is>
       </c>
       <c r="C96" s="65" t="inlineStr">
         <is>
-          <t>Only for multi-SF / multi-channel / public TTN. Single-channel Wio-E5 gateway is enough for our 20 nodes.</t>
+          <t>anti-theft</t>
         </is>
       </c>
       <c r="E96" s="66" t="inlineStr">
         <is>
-          <t>145.0</t>
+          <t>4.0</t>
         </is>
       </c>
     </row>
     <row r="97" ht="15.5" customHeight="1">
       <c r="A97" s="64" t="inlineStr">
         <is>
-          <t>J01</t>
+          <t>H13</t>
         </is>
       </c>
       <c r="B97" s="64" t="inlineStr">
         <is>
-          <t>Filament ASA</t>
+          <t>Site label</t>
         </is>
       </c>
       <c r="C97" s="65" t="inlineStr">
         <is>
-          <t>ABS z domaceho spoolu, nie ASA; UV je len na brehu</t>
+          <t>anti-theft by making it unsellable</t>
         </is>
       </c>
       <c r="E97" s="66" t="inlineStr">
         <is>
-          <t>32.0</t>
+          <t>3.0</t>
         </is>
       </c>
     </row>
     <row r="98" ht="15.5" customHeight="1">
       <c r="A98" s="64" t="inlineStr">
         <is>
-          <t>J02</t>
+          <t>I02</t>
         </is>
       </c>
       <c r="B98" s="64" t="inlineStr">
         <is>
-          <t>Filament PC Blend</t>
-        </is>
-      </c>
-      <c r="C98" s="65" t="inlineStr"/>
+          <t>Compute</t>
+        </is>
+      </c>
+      <c r="C98" s="65" t="inlineStr">
+        <is>
+          <t>YOU ALREADY HAVE THIS - reuse, zero soldering; runs the gateway service</t>
+        </is>
+      </c>
       <c r="E98" s="66" t="inlineStr">
         <is>
-          <t>40.0</t>
+          <t>70.0</t>
         </is>
       </c>
     </row>
     <row r="99" ht="15.5" customHeight="1">
       <c r="A99" s="64" t="inlineStr">
         <is>
-          <t>J04</t>
+          <t>I03</t>
         </is>
       </c>
       <c r="B99" s="64" t="inlineStr">
         <is>
-          <t>Conformal coat</t>
-        </is>
-      </c>
-      <c r="C99" s="65" t="inlineStr"/>
+          <t>Antenna</t>
+        </is>
+      </c>
+      <c r="C99" s="65" t="inlineStr">
+        <is>
+          <t>range-critical: gateway antenna gain + mast height set the link</t>
+        </is>
+      </c>
       <c r="E99" s="66" t="inlineStr">
         <is>
-          <t>14.0</t>
+          <t>45.0</t>
         </is>
       </c>
     </row>
     <row r="100" ht="15.5" customHeight="1">
       <c r="A100" s="64" t="inlineStr">
         <is>
-          <t>J05</t>
+          <t>I04</t>
         </is>
       </c>
       <c r="B100" s="64" t="inlineStr">
         <is>
-          <t>Silicone grease</t>
-        </is>
-      </c>
-      <c r="C100" s="65" t="inlineStr">
-        <is>
-          <t>MAM - doma</t>
-        </is>
-      </c>
+          <t>Enclosure</t>
+        </is>
+      </c>
+      <c r="C100" s="65" t="inlineStr"/>
       <c r="E100" s="66" t="inlineStr">
         <is>
-          <t>9.0</t>
+          <t>35.0</t>
         </is>
       </c>
     </row>
     <row r="101" ht="15.5" customHeight="1">
       <c r="A101" s="64" t="inlineStr">
         <is>
-          <t>J06</t>
+          <t>I05</t>
         </is>
       </c>
       <c r="B101" s="64" t="inlineStr">
         <is>
-          <t>Threadlocker</t>
-        </is>
-      </c>
-      <c r="C101" s="65" t="inlineStr"/>
+          <t>Mast</t>
+        </is>
+      </c>
+      <c r="C101" s="65" t="inlineStr">
+        <is>
+          <t>height sets range</t>
+        </is>
+      </c>
       <c r="E101" s="66" t="inlineStr">
         <is>
-          <t>11.0</t>
+          <t>30.0</t>
         </is>
       </c>
     </row>
     <row r="102" ht="15.5" customHeight="1">
       <c r="A102" s="64" t="inlineStr">
         <is>
-          <t>J08</t>
+          <t>I06</t>
         </is>
       </c>
       <c r="B102" s="64" t="inlineStr">
         <is>
-          <t>O-ring kit</t>
-        </is>
-      </c>
-      <c r="C102" s="65" t="inlineStr"/>
+          <t>Concentrator upgrade (optional)</t>
+        </is>
+      </c>
+      <c r="C102" s="65" t="inlineStr">
+        <is>
+          <t>Only for multi-SF / multi-channel / public TTN. Single-channel Wio-E5 gateway is enough for our 20 nodes.</t>
+        </is>
+      </c>
       <c r="E102" s="66" t="inlineStr">
         <is>
-          <t>12.0</t>
+          <t>145.0</t>
         </is>
       </c>
     </row>
     <row r="103" ht="15.5" customHeight="1">
       <c r="A103" s="64" t="inlineStr">
         <is>
-          <t>K01</t>
+          <t>J01</t>
         </is>
       </c>
       <c r="B103" s="64" t="inlineStr">
         <is>
-          <t>Vacuum chamber</t>
+          <t>Filament ASA</t>
         </is>
       </c>
       <c r="C103" s="65" t="inlineStr">
         <is>
-          <t>acceptance test rig (one-off)</t>
+          <t>ABS z domaceho spoolu, nie ASA; UV je len na brehu</t>
         </is>
       </c>
       <c r="E103" s="66" t="inlineStr">
         <is>
-          <t>85.0</t>
+          <t>32.0</t>
         </is>
       </c>
     </row>
     <row r="104" ht="15.5" customHeight="1">
       <c r="A104" s="64" t="inlineStr">
         <is>
-          <t>K02</t>
+          <t>J02</t>
         </is>
       </c>
       <c r="B104" s="64" t="inlineStr">
         <is>
-          <t>Torque driver</t>
-        </is>
-      </c>
-      <c r="C104" s="65" t="inlineStr">
-        <is>
-          <t>one-off</t>
-        </is>
-      </c>
+          <t>Filament PC Blend</t>
+        </is>
+      </c>
+      <c r="C104" s="65" t="inlineStr"/>
       <c r="E104" s="66" t="inlineStr">
         <is>
           <t>40.0</t>
         </is>
       </c>
     </row>
-    <row r="106">
-      <c r="A106" s="67" t="inlineStr">
-        <is>
-          <t>CUT - DEAD LINE, DO NOT BUY</t>
+    <row r="105" ht="15.5" customHeight="1">
+      <c r="A105" s="64" t="inlineStr">
+        <is>
+          <t>J04</t>
+        </is>
+      </c>
+      <c r="B105" s="64" t="inlineStr">
+        <is>
+          <t>Conformal coat</t>
+        </is>
+      </c>
+      <c r="C105" s="65" t="inlineStr"/>
+      <c r="E105" s="66" t="inlineStr">
+        <is>
+          <t>14.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" ht="15.5" customHeight="1">
+      <c r="A106" s="64" t="inlineStr">
+        <is>
+          <t>J05</t>
+        </is>
+      </c>
+      <c r="B106" s="64" t="inlineStr">
+        <is>
+          <t>Silicone grease</t>
+        </is>
+      </c>
+      <c r="C106" s="65" t="inlineStr">
+        <is>
+          <t>MAM - doma</t>
+        </is>
+      </c>
+      <c r="E106" s="66" t="inlineStr">
+        <is>
+          <t>9.0</t>
         </is>
       </c>
     </row>
     <row r="107" ht="15.5" customHeight="1">
       <c r="A107" s="64" t="inlineStr">
         <is>
-          <t>A05</t>
+          <t>J06</t>
         </is>
       </c>
       <c r="B107" s="64" t="inlineStr">
         <is>
-          <t>Bearing carrier tube</t>
-        </is>
-      </c>
-      <c r="C107" s="65" t="inlineStr">
-        <is>
-          <t>CUT: superseded - the bearing carrier is the printed spider (wet_carrier)</t>
-        </is>
-      </c>
-      <c r="E107" s="68" t="inlineStr">
-        <is>
-          <t>1.2</t>
+          <t>Threadlocker</t>
+        </is>
+      </c>
+      <c r="C107" s="65" t="inlineStr"/>
+      <c r="E107" s="66" t="inlineStr">
+        <is>
+          <t>11.0</t>
         </is>
       </c>
     </row>
     <row r="108" ht="15.5" customHeight="1">
       <c r="A108" s="64" t="inlineStr">
         <is>
-          <t>A07</t>
+          <t>J08</t>
         </is>
       </c>
       <c r="B108" s="64" t="inlineStr">
         <is>
-          <t>Weed guard ring</t>
-        </is>
-      </c>
-      <c r="C108" s="65" t="inlineStr">
-        <is>
-          <t>CUT: killed by design - replaced by the nose cone D64-&gt;D12; a ring on struts upstream is an algae scythe</t>
-        </is>
-      </c>
-      <c r="E108" s="68" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>O-ring kit</t>
+        </is>
+      </c>
+      <c r="C108" s="65" t="inlineStr"/>
+      <c r="E108" s="66" t="inlineStr">
+        <is>
+          <t>12.0</t>
         </is>
       </c>
     </row>
     <row r="109" ht="15.5" customHeight="1">
       <c r="A109" s="64" t="inlineStr">
         <is>
-          <t>A08</t>
+          <t>K01</t>
         </is>
       </c>
       <c r="B109" s="64" t="inlineStr">
         <is>
-          <t>Blade safety retainer</t>
+          <t>Vacuum chamber</t>
         </is>
       </c>
       <c r="C109" s="65" t="inlineStr">
         <is>
-          <t>CUT: killed by design - a tether on a 110 mm blade is a flail, and the hole is a stress riser at the root</t>
-        </is>
-      </c>
-      <c r="E109" s="68" t="inlineStr">
-        <is>
-          <t>2.0</t>
+          <t>acceptance test rig (one-off)</t>
+        </is>
+      </c>
+      <c r="E109" s="66" t="inlineStr">
+        <is>
+          <t>85.0</t>
         </is>
       </c>
     </row>
     <row r="110" ht="15.5" customHeight="1">
       <c r="A110" s="64" t="inlineStr">
         <is>
+          <t>K02</t>
+        </is>
+      </c>
+      <c r="B110" s="64" t="inlineStr">
+        <is>
+          <t>Torque driver</t>
+        </is>
+      </c>
+      <c r="C110" s="65" t="inlineStr">
+        <is>
+          <t>one-off</t>
+        </is>
+      </c>
+      <c r="E110" s="66" t="inlineStr">
+        <is>
+          <t>40.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="67" t="inlineStr">
+        <is>
+          <t>CUT - DEAD LINE, DO NOT BUY</t>
+        </is>
+      </c>
+    </row>
+    <row r="113" ht="15.5" customHeight="1">
+      <c r="A113" s="64" t="inlineStr">
+        <is>
+          <t>A05</t>
+        </is>
+      </c>
+      <c r="B113" s="64" t="inlineStr">
+        <is>
+          <t>Bearing carrier tube</t>
+        </is>
+      </c>
+      <c r="C113" s="65" t="inlineStr">
+        <is>
+          <t>CUT: superseded - the bearing carrier is the printed spider (wet_carrier)</t>
+        </is>
+      </c>
+      <c r="E113" s="68" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="114" ht="15.5" customHeight="1">
+      <c r="A114" s="64" t="inlineStr">
+        <is>
+          <t>A07</t>
+        </is>
+      </c>
+      <c r="B114" s="64" t="inlineStr">
+        <is>
+          <t>Weed guard ring</t>
+        </is>
+      </c>
+      <c r="C114" s="65" t="inlineStr">
+        <is>
+          <t>CUT: killed by design - replaced by the nose cone D64-&gt;D12; a ring on struts upstream is an algae scythe</t>
+        </is>
+      </c>
+      <c r="E114" s="68" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="115" ht="15.5" customHeight="1">
+      <c r="A115" s="64" t="inlineStr">
+        <is>
+          <t>A08</t>
+        </is>
+      </c>
+      <c r="B115" s="64" t="inlineStr">
+        <is>
+          <t>Blade safety retainer</t>
+        </is>
+      </c>
+      <c r="C115" s="65" t="inlineStr">
+        <is>
+          <t>CUT: killed by design - a tether on a 110 mm blade is a flail, and the hole is a stress riser at the root</t>
+        </is>
+      </c>
+      <c r="E115" s="68" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="116" ht="15.5" customHeight="1">
+      <c r="A116" s="64" t="inlineStr">
+        <is>
           <t>G02</t>
         </is>
       </c>
-      <c r="B110" s="64" t="inlineStr">
+      <c r="B116" s="64" t="inlineStr">
         <is>
           <t>MCU (NOT USED in simple build)</t>
         </is>
       </c>
-      <c r="C110" s="65" t="inlineStr">
+      <c r="C116" s="65" t="inlineStr">
         <is>
           <t>DROPPED: Wio-E5 mini is the single brain (MCU+LoRa). Bring back only if we need more GPIO/dual-core.</t>
         </is>
       </c>
-      <c r="E110" s="68" t="inlineStr">
+      <c r="E116" s="68" t="inlineStr">
         <is>
           <t>0.0</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="14">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A53:E53"/>
+    <mergeCell ref="A59:E59"/>
     <mergeCell ref="A20:E20"/>
-    <mergeCell ref="A52:E52"/>
+    <mergeCell ref="A38:E38"/>
+    <mergeCell ref="A57:E57"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A28:E28"/>
-    <mergeCell ref="A51:E51"/>
-    <mergeCell ref="A47:E47"/>
+    <mergeCell ref="A42:E42"/>
     <mergeCell ref="A5:E5"/>
-    <mergeCell ref="A56:F56"/>
-    <mergeCell ref="A36:E36"/>
+    <mergeCell ref="A32:E32"/>
+    <mergeCell ref="A62:F62"/>
     <mergeCell ref="A3:F3"/>
+    <mergeCell ref="A58:E58"/>
+    <mergeCell ref="A27:E27"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId1"/>
@@ -3013,9 +3099,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B23" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B24" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B25" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B26" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B29" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B30" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B31" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B40" r:id="rId18"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
@@ -3621,7 +3707,7 @@
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>techfun.sk / magsy.sk</t>
+          <t>supermagnete.cz</t>
         </is>
       </c>
       <c r="F17" s="8" t="n">
@@ -3652,7 +3738,7 @@
       </c>
       <c r="L17" s="6" t="inlineStr">
         <is>
-          <t>N52 D10x5, 8 per cup on a D70 cup; must be canned/epoxy - bare N52 corrodes in weeks | 16x N52 D10x5; supermagnete ma presne tento diel, magsy over v prehliadaci</t>
+          <t>N52 D10x5, 8 per cup on a D70 cup; must be canned/epoxy - bare N52 corrodes in weeks | 16x N52 D10x5 (S-10-05-N52N, 3.3 kg); magsy 10x5 N52 nemá overený</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
order: the XIAO kit has a U.FL, not an SMA
Checked the rpishop page: the kit lists a U.FL/IPEX connector and ships one small
LoRa antenna. So the stub it comes with is a u.FL whip, and any bigger antenna
needs a pigtail. G05 comes back as 2 pieces (one per board), 3 EUR each, so his
own antennas can be used at both ends.

phase 1: 32 lines, 220.61 EUR goods
</commit_message>
<xml_diff>
--- a/docs/sub-mission_parts.xlsx
+++ b/docs/sub-mission_parts.xlsx
@@ -837,7 +837,7 @@
     <row r="3" ht="26" customHeight="1">
       <c r="A3" s="44" t="inlineStr">
         <is>
-          <t>31 lines      goods 214.61 EUR      shipping est. 25.00 EUR      LANDED 239.61 EUR</t>
+          <t>32 lines      goods 220.61 EUR      shipping est. 25.00 EUR      LANDED 245.61 EUR</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
         </is>
       </c>
       <c r="F5" s="46" t="n">
-        <v>118.36</v>
+        <v>124.36</v>
       </c>
     </row>
     <row r="6">
@@ -1042,43 +1042,43 @@
     <row r="13" ht="29" customHeight="1">
       <c r="A13" s="49" t="inlineStr">
         <is>
-          <t>G16</t>
+          <t>G05</t>
         </is>
       </c>
       <c r="B13" s="50" t="inlineStr">
         <is>
-          <t>Protection</t>
+          <t>u.FL -&gt; SMA pigtail</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>Fuse 0.5A + TVS + ESD array  -  NEMAM - poistka 0.5A + TVS SMBJ5.0A + ESD array (SOT-23-6)</t>
+          <t>u.FL/IPEX female na SMA female bulkhead, 10-15 cm, RG178  -  KIT MA U.FL, NIE SMA: bez pigtailu na vacsiu antenu nepripojis; 1x sonda, 1x gateway</t>
         </is>
       </c>
       <c r="D13" s="51" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E13" s="52" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F13" s="52" t="n">
         <v>6</v>
       </c>
     </row>
-    <row r="14" ht="15.5" customHeight="1">
+    <row r="14" ht="29" customHeight="1">
       <c r="A14" s="53" t="inlineStr">
         <is>
-          <t>J07</t>
+          <t>G16</t>
         </is>
       </c>
       <c r="B14" s="54" t="inlineStr">
         <is>
-          <t>Heat-set inserts</t>
+          <t>Protection</t>
         </is>
       </c>
       <c r="C14" s="55" t="inlineStr">
         <is>
-          <t>M3/M4 brass assortment</t>
+          <t>Fuse 0.5A + TVS + ESD array  -  NEMAM - poistka 0.5A + TVS SMBJ5.0A + ESD array (SOT-23-6)</t>
         </is>
       </c>
       <c r="D14" s="56" t="n">
@@ -1094,43 +1094,43 @@
     <row r="15" ht="15.5" customHeight="1">
       <c r="A15" s="49" t="inlineStr">
         <is>
+          <t>J07</t>
+        </is>
+      </c>
+      <c r="B15" s="50" t="inlineStr">
+        <is>
+          <t>Heat-set inserts</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>M3/M4 brass assortment</t>
+        </is>
+      </c>
+      <c r="D15" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" s="52" t="n">
+        <v>6</v>
+      </c>
+      <c r="F15" s="52" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="16" ht="15.5" customHeight="1">
+      <c r="A16" s="53" t="inlineStr">
+        <is>
           <t>C03</t>
         </is>
       </c>
-      <c r="B15" s="50" t="inlineStr">
+      <c r="B16" s="54" t="inlineStr">
         <is>
           <t>Pod O-ring</t>
         </is>
       </c>
-      <c r="C15" s="6" t="inlineStr">
+      <c r="C16" s="55" t="inlineStr">
         <is>
           <t>NBR 70 Ø100x2.5  -  zadny spoj podu - bez neho sa pri ponoreni natecie</t>
-        </is>
-      </c>
-      <c r="D15" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="E15" s="52" t="n">
-        <v>3</v>
-      </c>
-      <c r="F15" s="52" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="16" ht="29" customHeight="1">
-      <c r="A16" s="53" t="inlineStr">
-        <is>
-          <t>C05</t>
-        </is>
-      </c>
-      <c r="B16" s="54" t="inlineStr">
-        <is>
-          <t>Pod clamp screws</t>
-        </is>
-      </c>
-      <c r="C16" s="55" t="inlineStr">
-        <is>
-          <t>M4x30 A4 + washers  -  drzi zadny spoj; integralny bulkhead riesi len prednu stranu</t>
         </is>
       </c>
       <c r="D16" s="56" t="n">
@@ -1146,1080 +1146,1084 @@
     <row r="17" ht="29" customHeight="1">
       <c r="A17" s="49" t="inlineStr">
         <is>
+          <t>C05</t>
+        </is>
+      </c>
+      <c r="B17" s="50" t="inlineStr">
+        <is>
+          <t>Pod clamp screws</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>M4x30 A4 + washers  -  drzi zadny spoj; integralny bulkhead riesi len prednu stranu</t>
+        </is>
+      </c>
+      <c r="D17" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" s="52" t="n">
+        <v>3</v>
+      </c>
+      <c r="F17" s="52" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="18" ht="29" customHeight="1">
+      <c r="A18" s="53" t="inlineStr">
+        <is>
           <t>A04</t>
         </is>
       </c>
-      <c r="B17" s="50" t="inlineStr">
+      <c r="B18" s="54" t="inlineStr">
         <is>
           <t>Wet bearing</t>
         </is>
       </c>
-      <c r="C17" s="6" t="inlineStr">
+      <c r="C18" s="55" t="inlineStr">
         <is>
           <t>igus iglidur J plain bearing JSM-0507-05 5x7x5mm  -  83 pcs in stock; JFM-0507-05 flanged 1.48 USD alt</t>
-        </is>
-      </c>
-      <c r="D17" s="51" t="n">
-        <v>2</v>
-      </c>
-      <c r="E17" s="52" t="n">
-        <v>1.18</v>
-      </c>
-      <c r="F17" s="52" t="n">
-        <v>2.36</v>
-      </c>
-    </row>
-    <row r="18" ht="15.5" customHeight="1">
-      <c r="A18" s="53" t="inlineStr">
-        <is>
-          <t>A06</t>
-        </is>
-      </c>
-      <c r="B18" s="54" t="inlineStr">
-        <is>
-          <t>Set screw</t>
-        </is>
-      </c>
-      <c r="C18" s="55" t="inlineStr">
-        <is>
-          <t>M4x8 316SS cup point ISO 4029</t>
         </is>
       </c>
       <c r="D18" s="56" t="n">
         <v>2</v>
       </c>
       <c r="E18" s="57" t="n">
-        <v>1</v>
+        <v>1.18</v>
       </c>
       <c r="F18" s="57" t="n">
+        <v>2.36</v>
+      </c>
+    </row>
+    <row r="19" ht="15.5" customHeight="1">
+      <c r="A19" s="49" t="inlineStr">
+        <is>
+          <t>A06</t>
+        </is>
+      </c>
+      <c r="B19" s="50" t="inlineStr">
+        <is>
+          <t>Set screw</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>M4x8 316SS cup point ISO 4029</t>
+        </is>
+      </c>
+      <c r="D19" s="51" t="n">
         <v>2</v>
       </c>
-    </row>
-    <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="45" t="inlineStr">
+      <c r="E19" s="52" t="n">
+        <v>1</v>
+      </c>
+      <c r="F19" s="52" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="45" t="inlineStr">
         <is>
           <t>TECHFUN.SK</t>
         </is>
       </c>
-      <c r="F20" s="46" t="n">
+      <c r="F21" s="46" t="n">
         <v>49.45</v>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="47" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="47" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B21" s="47" t="inlineStr">
+      <c r="B22" s="47" t="inlineStr">
         <is>
           <t>Part</t>
         </is>
       </c>
-      <c r="C21" s="47" t="inlineStr">
+      <c r="C22" s="47" t="inlineStr">
         <is>
           <t>Specification / note</t>
         </is>
       </c>
-      <c r="D21" s="48" t="inlineStr">
+      <c r="D22" s="48" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="E21" s="48" t="inlineStr">
+      <c r="E22" s="48" t="inlineStr">
         <is>
           <t>Unit EUR</t>
         </is>
       </c>
-      <c r="F21" s="48" t="inlineStr">
+      <c r="F22" s="48" t="inlineStr">
         <is>
           <t>Total EUR</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="15.5" customHeight="1">
-      <c r="A22" s="49" t="inlineStr">
+    <row r="23" ht="15.5" customHeight="1">
+      <c r="A23" s="49" t="inlineStr">
         <is>
           <t>J03</t>
         </is>
       </c>
-      <c r="B22" s="49" t="inlineStr">
+      <c r="B23" s="49" t="inlineStr">
         <is>
           <t>Epoxy barrier</t>
         </is>
       </c>
-      <c r="C22" s="6" t="inlineStr">
+      <c r="C23" s="6" t="inlineStr">
         <is>
           <t>West System 105 + 206</t>
         </is>
       </c>
-      <c r="D22" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="E22" s="52" t="n">
+      <c r="D23" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" s="52" t="n">
         <v>18</v>
       </c>
-      <c r="F22" s="52" t="n">
+      <c r="F23" s="52" t="n">
         <v>18</v>
       </c>
     </row>
-    <row r="23" ht="29" customHeight="1">
-      <c r="A23" s="53" t="inlineStr">
+    <row r="24" ht="29" customHeight="1">
+      <c r="A24" s="53" t="inlineStr">
         <is>
           <t>B04</t>
         </is>
       </c>
-      <c r="B23" s="54" t="inlineStr">
+      <c r="B24" s="54" t="inlineStr">
         <is>
           <t>Potting compound</t>
         </is>
       </c>
-      <c r="C23" s="55" t="inlineStr">
+      <c r="C24" s="55" t="inlineStr">
         <is>
           <t>3M Scotch-Weld DP270 black 25ml  -  techfun nema DP270; silikonova zalievacia hmota staci na test, epoxid je tuhsi</t>
         </is>
       </c>
-      <c r="D23" s="56" t="n">
-        <v>1</v>
-      </c>
-      <c r="E23" s="57" t="n">
+      <c r="D24" s="56" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" s="57" t="n">
         <v>14</v>
       </c>
-      <c r="F23" s="57" t="n">
+      <c r="F24" s="57" t="n">
         <v>14</v>
       </c>
     </row>
-    <row r="24" ht="15.5" customHeight="1">
-      <c r="A24" s="49" t="inlineStr">
+    <row r="25" ht="15.5" customHeight="1">
+      <c r="A25" s="49" t="inlineStr">
         <is>
           <t>D07</t>
         </is>
       </c>
-      <c r="B24" s="50" t="inlineStr">
+      <c r="B25" s="50" t="inlineStr">
         <is>
           <t>Turbidity</t>
         </is>
       </c>
-      <c r="C24" s="6" t="inlineStr">
+      <c r="C25" s="6" t="inlineStr">
         <is>
           <t>DFRobot SEN0189 (0-4.5V analog)  -  6 in stock; in model as sensor_turb</t>
         </is>
       </c>
-      <c r="D24" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="E24" s="52" t="n">
+      <c r="D25" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" s="52" t="n">
         <v>12.45</v>
       </c>
-      <c r="F24" s="52" t="n">
+      <c r="F25" s="52" t="n">
         <v>12.45</v>
       </c>
     </row>
-    <row r="25" ht="15.5" customHeight="1">
-      <c r="A25" s="53" t="inlineStr">
+    <row r="26" ht="15.5" customHeight="1">
+      <c r="A26" s="53" t="inlineStr">
         <is>
           <t>D04</t>
         </is>
       </c>
-      <c r="B25" s="54" t="inlineStr">
+      <c r="B26" s="54" t="inlineStr">
         <is>
           <t>Temperature</t>
         </is>
       </c>
-      <c r="C25" s="55" t="inlineStr">
+      <c r="C26" s="55" t="inlineStr">
         <is>
           <t>DS18B20 waterproof 1m cable  -  in model as sensor_ntc</t>
         </is>
       </c>
-      <c r="D25" s="56" t="n">
-        <v>1</v>
-      </c>
-      <c r="E25" s="57" t="n">
+      <c r="D26" s="56" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" s="57" t="n">
         <v>5</v>
       </c>
-      <c r="F25" s="57" t="n">
+      <c r="F26" s="57" t="n">
         <v>5</v>
       </c>
     </row>
-    <row r="27" ht="20" customHeight="1">
-      <c r="A27" s="45" t="inlineStr">
+    <row r="28" ht="20" customHeight="1">
+      <c r="A28" s="45" t="inlineStr">
         <is>
           <t>RPISHOP.CZ</t>
         </is>
       </c>
-      <c r="F27" s="46" t="n">
+      <c r="F28" s="46" t="n">
         <v>28</v>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="47" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="47" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B28" s="47" t="inlineStr">
+      <c r="B29" s="47" t="inlineStr">
         <is>
           <t>Part</t>
         </is>
       </c>
-      <c r="C28" s="47" t="inlineStr">
+      <c r="C29" s="47" t="inlineStr">
         <is>
           <t>Specification / note</t>
         </is>
       </c>
-      <c r="D28" s="48" t="inlineStr">
+      <c r="D29" s="48" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="E28" s="48" t="inlineStr">
+      <c r="E29" s="48" t="inlineStr">
         <is>
           <t>Unit EUR</t>
         </is>
       </c>
-      <c r="F28" s="48" t="inlineStr">
+      <c r="F29" s="48" t="inlineStr">
         <is>
           <t>Total EUR</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="42.5" customHeight="1">
-      <c r="A29" s="49" t="inlineStr">
+    <row r="30" ht="42.5" customHeight="1">
+      <c r="A30" s="49" t="inlineStr">
         <is>
           <t>G03</t>
         </is>
       </c>
-      <c r="B29" s="50" t="inlineStr">
+      <c r="B30" s="50" t="inlineStr">
         <is>
           <t>MCU + radio (single board)</t>
         </is>
       </c>
-      <c r="C29" s="6" t="inlineStr">
+      <c r="C30" s="6" t="inlineStr">
         <is>
           <t>Seeed XIAO nRF52840 + Wio-SX1262 kit (Meshtastic), SEE336 - nRF52840 + SX1262  -  349 Kc, skladom 5+; nahradza Wio-E5, ktory v CZ/SK nie je; antena je v kite</t>
         </is>
       </c>
-      <c r="D29" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="E29" s="52" t="n">
+      <c r="D30" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="E30" s="52" t="n">
         <v>14</v>
       </c>
-      <c r="F29" s="52" t="n">
+      <c r="F30" s="52" t="n">
         <v>14</v>
       </c>
     </row>
-    <row r="30" ht="42.5" customHeight="1">
-      <c r="A30" s="53" t="inlineStr">
+    <row r="31" ht="42.5" customHeight="1">
+      <c r="A31" s="53" t="inlineStr">
         <is>
           <t>I01</t>
         </is>
       </c>
-      <c r="B30" s="54" t="inlineStr">
+      <c r="B31" s="54" t="inlineStr">
         <is>
           <t>Gateway radio (single-channel)</t>
         </is>
       </c>
-      <c r="C30" s="55" t="inlineStr">
+      <c r="C31" s="55" t="inlineStr">
         <is>
           <t>Seeed XIAO nRF52840 + Wio-SX1262 kit (Meshtastic), SEE336 - nRF52840 + SX1262  -  349 Kc, skladom 5+; nahradza Wio-E5, ktory v CZ/SK nie je; antena je v kite</t>
         </is>
       </c>
-      <c r="D30" s="56" t="n">
-        <v>1</v>
-      </c>
-      <c r="E30" s="57" t="n">
+      <c r="D31" s="56" t="n">
+        <v>1</v>
+      </c>
+      <c r="E31" s="57" t="n">
         <v>14</v>
       </c>
-      <c r="F30" s="57" t="n">
+      <c r="F31" s="57" t="n">
         <v>14</v>
       </c>
     </row>
-    <row r="32" ht="20" customHeight="1">
-      <c r="A32" s="45" t="inlineStr">
+    <row r="33" ht="20" customHeight="1">
+      <c r="A33" s="45" t="inlineStr">
         <is>
           <t>LOCAL / SHOP</t>
         </is>
       </c>
-      <c r="F32" s="46" t="n">
+      <c r="F33" s="46" t="n">
         <v>9</v>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="47" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="47" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B33" s="47" t="inlineStr">
+      <c r="B34" s="47" t="inlineStr">
         <is>
           <t>Part</t>
         </is>
       </c>
-      <c r="C33" s="47" t="inlineStr">
+      <c r="C34" s="47" t="inlineStr">
         <is>
           <t>Specification / note</t>
         </is>
       </c>
-      <c r="D33" s="48" t="inlineStr">
+      <c r="D34" s="48" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="E33" s="48" t="inlineStr">
+      <c r="E34" s="48" t="inlineStr">
         <is>
           <t>Unit EUR</t>
         </is>
       </c>
-      <c r="F33" s="48" t="inlineStr">
+      <c r="F34" s="48" t="inlineStr">
         <is>
           <t>Total EUR</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="15.5" customHeight="1">
-      <c r="A34" s="49" t="inlineStr">
+    <row r="35" ht="15.5" customHeight="1">
+      <c r="A35" s="49" t="inlineStr">
         <is>
           <t>K03</t>
         </is>
       </c>
-      <c r="B34" s="49" t="inlineStr">
+      <c r="B35" s="49" t="inlineStr">
         <is>
           <t>Spring balance</t>
         </is>
       </c>
-      <c r="C34" s="6" t="inlineStr">
+      <c r="C35" s="6" t="inlineStr">
         <is>
           <t>0-5N for coupling slip jig  -  one-off</t>
         </is>
       </c>
-      <c r="D34" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="E34" s="52" t="n">
+      <c r="D35" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="E35" s="52" t="n">
         <v>5</v>
       </c>
-      <c r="F34" s="52" t="n">
+      <c r="F35" s="52" t="n">
         <v>5</v>
       </c>
     </row>
-    <row r="35" ht="15.5" customHeight="1">
-      <c r="A35" s="53" t="inlineStr">
+    <row r="36" ht="15.5" customHeight="1">
+      <c r="A36" s="53" t="inlineStr">
         <is>
           <t>C06</t>
         </is>
       </c>
-      <c r="B35" s="53" t="inlineStr">
+      <c r="B36" s="53" t="inlineStr">
         <is>
           <t>Desiccant</t>
         </is>
       </c>
-      <c r="C35" s="55" t="inlineStr">
+      <c r="C36" s="55" t="inlineStr">
         <is>
           <t>5g silica gel with indicator  -  replace at service</t>
         </is>
       </c>
-      <c r="D35" s="56" t="n">
+      <c r="D36" s="56" t="n">
         <v>2</v>
       </c>
-      <c r="E35" s="57" t="n">
+      <c r="E36" s="57" t="n">
         <v>2</v>
       </c>
-      <c r="F35" s="57" t="n">
+      <c r="F36" s="57" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="36" ht="29" customHeight="1">
-      <c r="A36" s="49" t="inlineStr">
+    <row r="37" ht="29" customHeight="1">
+      <c r="A37" s="49" t="inlineStr">
         <is>
           <t>C04</t>
         </is>
       </c>
-      <c r="B36" s="49" t="inlineStr">
+      <c r="B37" s="49" t="inlineStr">
         <is>
           <t>O-ring groove</t>
         </is>
       </c>
-      <c r="C36" s="6" t="inlineStr">
+      <c r="C37" s="6" t="inlineStr">
         <is>
           <t>2.2mm wide x 1.8mm deep machined/printed into pod rim  -  NOT YET IN MODEL - add to pod</t>
         </is>
       </c>
-      <c r="D36" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="E36" s="52" t="n">
+      <c r="D37" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="E37" s="52" t="n">
         <v>0</v>
       </c>
-      <c r="F36" s="52" t="n">
+      <c r="F37" s="52" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="38" ht="20" customHeight="1">
-      <c r="A38" s="45" t="inlineStr">
+    <row r="39" ht="20" customHeight="1">
+      <c r="A39" s="45" t="inlineStr">
         <is>
           <t>SUPERMAGNETICSHOP</t>
         </is>
       </c>
-      <c r="F38" s="46" t="n">
+      <c r="F39" s="46" t="n">
         <v>8.800000000000001</v>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="47" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="47" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B39" s="47" t="inlineStr">
+      <c r="B40" s="47" t="inlineStr">
         <is>
           <t>Part</t>
         </is>
       </c>
-      <c r="C39" s="47" t="inlineStr">
+      <c r="C40" s="47" t="inlineStr">
         <is>
           <t>Specification / note</t>
         </is>
       </c>
-      <c r="D39" s="48" t="inlineStr">
+      <c r="D40" s="48" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="E39" s="48" t="inlineStr">
+      <c r="E40" s="48" t="inlineStr">
         <is>
           <t>Unit EUR</t>
         </is>
       </c>
-      <c r="F39" s="48" t="inlineStr">
+      <c r="F40" s="48" t="inlineStr">
         <is>
           <t>Total EUR</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="29" customHeight="1">
-      <c r="A40" s="49" t="inlineStr">
+    <row r="41" ht="29" customHeight="1">
+      <c r="A41" s="49" t="inlineStr">
         <is>
           <t>B01</t>
         </is>
       </c>
-      <c r="B40" s="50" t="inlineStr">
+      <c r="B41" s="50" t="inlineStr">
         <is>
           <t>Magnet</t>
         </is>
       </c>
-      <c r="C40" s="6" t="inlineStr">
+      <c r="C41" s="6" t="inlineStr">
         <is>
           <t>N52 D10x5 axially magnetised, canned 316L or epoxy potted  -  16x N52 D10x5 (S-10-05-N52N, 3.3 kg); magsy 10x5 N52 nemá overený</t>
         </is>
       </c>
-      <c r="D40" s="51" t="n">
+      <c r="D41" s="51" t="n">
         <v>16</v>
       </c>
-      <c r="E40" s="52" t="n">
+      <c r="E41" s="52" t="n">
         <v>0.55</v>
       </c>
-      <c r="F40" s="52" t="n">
+      <c r="F41" s="52" t="n">
         <v>8.800000000000001</v>
       </c>
     </row>
-    <row r="42" ht="20" customHeight="1">
-      <c r="A42" s="45" t="inlineStr">
+    <row r="43" ht="20" customHeight="1">
+      <c r="A43" s="45" t="inlineStr">
         <is>
           <t>PRINTED IN-HOUSE</t>
         </is>
       </c>
-      <c r="F42" s="46" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="47" t="inlineStr">
+      <c r="F43" s="46" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="47" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B43" s="47" t="inlineStr">
+      <c r="B44" s="47" t="inlineStr">
         <is>
           <t>Part</t>
         </is>
       </c>
-      <c r="C43" s="47" t="inlineStr">
+      <c r="C44" s="47" t="inlineStr">
         <is>
           <t>Specification / note</t>
         </is>
       </c>
-      <c r="D43" s="48" t="inlineStr">
+      <c r="D44" s="48" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="E43" s="48" t="inlineStr">
+      <c r="E44" s="48" t="inlineStr">
         <is>
           <t>Unit EUR</t>
         </is>
       </c>
-      <c r="F43" s="48" t="inlineStr">
+      <c r="F44" s="48" t="inlineStr">
         <is>
           <t>Total EUR</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="15.5" customHeight="1">
-      <c r="A44" s="49" t="inlineStr">
+    <row r="45" ht="15.5" customHeight="1">
+      <c r="A45" s="49" t="inlineStr">
         <is>
           <t>C09</t>
         </is>
       </c>
-      <c r="B44" s="49" t="inlineStr">
+      <c r="B45" s="49" t="inlineStr">
         <is>
           <t>Generator mount</t>
         </is>
       </c>
-      <c r="C44" s="6" t="inlineStr">
+      <c r="C45" s="6" t="inlineStr">
         <is>
           <t>printed cradle + 4x M3x8 A4</t>
         </is>
       </c>
-      <c r="D44" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="E44" s="52" t="n">
-        <v>1</v>
-      </c>
-      <c r="F44" s="52" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="45" ht="29" customHeight="1">
-      <c r="A45" s="53" t="inlineStr">
+      <c r="D45" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="E45" s="52" t="n">
+        <v>1</v>
+      </c>
+      <c r="F45" s="52" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46" ht="29" customHeight="1">
+      <c r="A46" s="53" t="inlineStr">
         <is>
           <t>A01</t>
         </is>
       </c>
-      <c r="B45" s="53" t="inlineStr">
+      <c r="B46" s="53" t="inlineStr">
         <is>
           <t>Blade</t>
         </is>
       </c>
-      <c r="C45" s="55" t="inlineStr">
+      <c r="C46" s="55" t="inlineStr">
         <is>
           <t>triple-blade rotor blade NACA4412 D220mm root pitch 28deg tip 2deg  -  ASA or ASA-CF; 6 perimeters; epoxy coat; spare blade = fuse for branch strike</t>
         </is>
       </c>
-      <c r="D45" s="56" t="n">
+      <c r="D46" s="56" t="n">
         <v>3</v>
       </c>
-      <c r="E45" s="57" t="n">
+      <c r="E46" s="57" t="n">
         <v>0</v>
       </c>
-      <c r="F45" s="57" t="n">
+      <c r="F46" s="57" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="46" ht="29" customHeight="1">
-      <c r="A46" s="49" t="inlineStr">
+    <row r="47" ht="29" customHeight="1">
+      <c r="A47" s="49" t="inlineStr">
         <is>
           <t>A02</t>
         </is>
       </c>
-      <c r="B46" s="49" t="inlineStr">
+      <c r="B47" s="49" t="inlineStr">
         <is>
           <t>Hub</t>
         </is>
       </c>
-      <c r="C46" s="6" t="inlineStr">
+      <c r="C47" s="6" t="inlineStr">
         <is>
           <t>Ø64x46mm with 2x M4 heat-set inserts and Ø5 H7 shaft bore  -  brass inserts M4 from TME</t>
         </is>
       </c>
-      <c r="D46" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="E46" s="52" t="n">
+      <c r="D47" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="E47" s="52" t="n">
         <v>0</v>
       </c>
-      <c r="F46" s="52" t="n">
+      <c r="F47" s="52" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="47" ht="29" customHeight="1">
-      <c r="A47" s="53" t="inlineStr">
+    <row r="48" ht="29" customHeight="1">
+      <c r="A48" s="53" t="inlineStr">
         <is>
           <t>B02</t>
         </is>
       </c>
-      <c r="B47" s="53" t="inlineStr">
+      <c r="B48" s="53" t="inlineStr">
         <is>
           <t>Magnet cup</t>
         </is>
       </c>
-      <c r="C47" s="55" t="inlineStr">
+      <c r="C48" s="55" t="inlineStr">
         <is>
           <t>D70 rim, 8 pockets D10.2x5.2, printed ASA  -  pockets 10.2 dia (magnet 10 + 0.2 glue), 0.2 mm epoxy recess</t>
         </is>
       </c>
-      <c r="D47" s="56" t="n">
+      <c r="D48" s="56" t="n">
         <v>2</v>
       </c>
-      <c r="E47" s="57" t="n">
+      <c r="E48" s="57" t="n">
         <v>0</v>
       </c>
-      <c r="F47" s="57" t="n">
+      <c r="F48" s="57" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="48" ht="15.5" customHeight="1">
-      <c r="A48" s="49" t="inlineStr">
+    <row r="49" ht="15.5" customHeight="1">
+      <c r="A49" s="49" t="inlineStr">
         <is>
           <t>C01</t>
         </is>
       </c>
-      <c r="B48" s="49" t="inlineStr">
+      <c r="B49" s="49" t="inlineStr">
         <is>
           <t>Pod barrel</t>
         </is>
       </c>
-      <c r="C48" s="6" t="inlineStr">
+      <c r="C49" s="6" t="inlineStr">
         <is>
           <t>Ø110x120mm printed ASA wall 2.4mm + epoxy barrier  -  in model as pod</t>
         </is>
       </c>
-      <c r="D48" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="E48" s="52" t="n">
+      <c r="D49" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="E49" s="52" t="n">
         <v>0</v>
       </c>
-      <c r="F48" s="52" t="n">
+      <c r="F49" s="52" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="49" ht="15.5" customHeight="1">
-      <c r="A49" s="53" t="inlineStr">
+    <row r="50" ht="15.5" customHeight="1">
+      <c r="A50" s="53" t="inlineStr">
         <is>
           <t>C02</t>
         </is>
       </c>
-      <c r="B49" s="53" t="inlineStr">
+      <c r="B50" s="53" t="inlineStr">
         <is>
           <t>Tail cone</t>
         </is>
       </c>
-      <c r="C49" s="55" t="inlineStr">
+      <c r="C50" s="55" t="inlineStr">
         <is>
           <t>printed integral</t>
         </is>
       </c>
-      <c r="D49" s="56" t="n">
-        <v>1</v>
-      </c>
-      <c r="E49" s="57" t="n">
+      <c r="D50" s="56" t="n">
+        <v>1</v>
+      </c>
+      <c r="E50" s="57" t="n">
         <v>0</v>
       </c>
-      <c r="F49" s="57" t="n">
+      <c r="F50" s="57" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="50" ht="15.5" customHeight="1">
-      <c r="A50" s="49" t="inlineStr">
+    <row r="51" ht="15.5" customHeight="1">
+      <c r="A51" s="49" t="inlineStr">
         <is>
           <t>E01</t>
         </is>
       </c>
-      <c r="B50" s="49" t="inlineStr">
+      <c r="B51" s="49" t="inlineStr">
         <is>
           <t>Sensor cage</t>
         </is>
       </c>
-      <c r="C50" s="6" t="inlineStr">
+      <c r="C51" s="6" t="inlineStr">
         <is>
           <t>Ø130x150 printed ASA 12 slots  -  in model as cage</t>
         </is>
       </c>
-      <c r="D50" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="E50" s="52" t="n">
+      <c r="D51" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="E51" s="52" t="n">
         <v>0</v>
       </c>
-      <c r="F50" s="52" t="n">
+      <c r="F51" s="52" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="51" ht="29" customHeight="1">
-      <c r="A51" s="53" t="inlineStr">
+    <row r="52" ht="29" customHeight="1">
+      <c r="A52" s="53" t="inlineStr">
         <is>
           <t>E03</t>
         </is>
       </c>
-      <c r="B51" s="53" t="inlineStr">
+      <c r="B52" s="53" t="inlineStr">
         <is>
           <t>Sensor holders</t>
         </is>
       </c>
-      <c r="C51" s="55" t="inlineStr">
+      <c r="C52" s="55" t="inlineStr">
         <is>
           <t>printed clips for pH/TDS/turbidity/NTC/MS5837  -  in model as sensor bodies</t>
         </is>
       </c>
-      <c r="D51" s="56" t="n">
+      <c r="D52" s="56" t="n">
         <v>5</v>
       </c>
-      <c r="E51" s="57" t="n">
+      <c r="E52" s="57" t="n">
         <v>0</v>
       </c>
-      <c r="F51" s="57" t="n">
+      <c r="F52" s="57" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="53" ht="20" customHeight="1">
-      <c r="A53" s="45" t="inlineStr">
+    <row r="54" ht="20" customHeight="1">
+      <c r="A54" s="45" t="inlineStr">
         <is>
           <t>NEREZMATERIAL.CZ</t>
         </is>
       </c>
-      <c r="F53" s="46" t="n">
+      <c r="F54" s="46" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="47" t="inlineStr">
+    <row r="55">
+      <c r="A55" s="47" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B54" s="47" t="inlineStr">
+      <c r="B55" s="47" t="inlineStr">
         <is>
           <t>Part</t>
         </is>
       </c>
-      <c r="C54" s="47" t="inlineStr">
+      <c r="C55" s="47" t="inlineStr">
         <is>
           <t>Specification / note</t>
         </is>
       </c>
-      <c r="D54" s="48" t="inlineStr">
+      <c r="D55" s="48" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="E54" s="48" t="inlineStr">
+      <c r="E55" s="48" t="inlineStr">
         <is>
           <t>Unit EUR</t>
         </is>
       </c>
-      <c r="F54" s="48" t="inlineStr">
+      <c r="F55" s="48" t="inlineStr">
         <is>
           <t>Total EUR</t>
         </is>
       </c>
     </row>
-    <row r="55" ht="29" customHeight="1">
-      <c r="A55" s="49" t="inlineStr">
+    <row r="56" ht="29" customHeight="1">
+      <c r="A56" s="49" t="inlineStr">
         <is>
           <t>B03</t>
         </is>
       </c>
-      <c r="B55" s="49" t="inlineStr">
+      <c r="B56" s="49" t="inlineStr">
         <is>
           <t>Separation wall</t>
         </is>
       </c>
-      <c r="C55" s="6" t="inlineStr">
+      <c r="C56" s="6" t="inlineStr">
         <is>
           <t>D106 x 4 mm - RECOMMENDED integral with the pod bulkhead (no separate part)  -  4 mm per CAD, not 5; integral removes O-ring C03 and screws C05</t>
         </is>
       </c>
-      <c r="D55" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="E55" s="52" t="n">
+      <c r="D56" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="E56" s="52" t="n">
         <v>0</v>
       </c>
-      <c r="F55" s="52" t="n">
+      <c r="F56" s="52" t="n">
         <v>0</v>
-      </c>
-    </row>
-    <row r="57" ht="18" customHeight="1">
-      <c r="A57" s="58" t="inlineStr">
-        <is>
-          <t>GOODS</t>
-        </is>
-      </c>
-      <c r="F57" s="59" t="n">
-        <v>214.61</v>
       </c>
     </row>
     <row r="58" ht="18" customHeight="1">
       <c r="A58" s="58" t="inlineStr">
         <is>
+          <t>GOODS</t>
+        </is>
+      </c>
+      <c r="F58" s="59" t="n">
+        <v>220.61</v>
+      </c>
+    </row>
+    <row r="59" ht="18" customHeight="1">
+      <c r="A59" s="58" t="inlineStr">
+        <is>
           <t>shipping, estimated</t>
         </is>
       </c>
-      <c r="F58" s="59" t="n">
+      <c r="F59" s="59" t="n">
         <v>25</v>
       </c>
     </row>
-    <row r="59" ht="22" customHeight="1">
-      <c r="A59" s="60" t="inlineStr">
+    <row r="60" ht="22" customHeight="1">
+      <c r="A60" s="60" t="inlineStr">
         <is>
           <t>LANDED TOTAL</t>
         </is>
       </c>
-      <c r="F59" s="61" t="n">
-        <v>239.61</v>
-      </c>
-    </row>
-    <row r="62" ht="22" customHeight="1">
-      <c r="A62" s="62" t="inlineStr">
+      <c r="F60" s="61" t="n">
+        <v>245.61</v>
+      </c>
+    </row>
+    <row r="63" ht="22" customHeight="1">
+      <c r="A63" s="62" t="inlineStr">
         <is>
           <t>NOT IN THIS ORDER</t>
         </is>
       </c>
     </row>
-    <row r="63">
-      <c r="A63" s="63" t="inlineStr">
+    <row r="64">
+      <c r="A64" s="63" t="inlineStr">
         <is>
           <t>PHASE 2 - BUY LATER</t>
-        </is>
-      </c>
-    </row>
-    <row r="64" ht="29" customHeight="1">
-      <c r="A64" s="64" t="inlineStr">
-        <is>
-          <t>A03</t>
-        </is>
-      </c>
-      <c r="B64" s="64" t="inlineStr">
-        <is>
-          <t>Wet shaft</t>
-        </is>
-      </c>
-      <c r="C64" s="65" t="inlineStr">
-        <is>
-          <t>lokalny zeleziar / Hornbach M5 A4 srob - 4. obchod sa nerata, nema postu; 3m bar 63.1 CZK makes ~26 shafts</t>
-        </is>
-      </c>
-      <c r="E64" s="66" t="inlineStr">
-        <is>
-          <t>2.6</t>
         </is>
       </c>
     </row>
     <row r="65" ht="29" customHeight="1">
       <c r="A65" s="64" t="inlineStr">
         <is>
+          <t>A03</t>
+        </is>
+      </c>
+      <c r="B65" s="64" t="inlineStr">
+        <is>
+          <t>Wet shaft</t>
+        </is>
+      </c>
+      <c r="C65" s="65" t="inlineStr">
+        <is>
+          <t>lokalny zeleziar / Hornbach M5 A4 srob - 4. obchod sa nerata, nema postu; 3m bar 63.1 CZK makes ~26 shafts</t>
+        </is>
+      </c>
+      <c r="E65" s="66" t="inlineStr">
+        <is>
+          <t>2.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="29" customHeight="1">
+      <c r="A66" s="64" t="inlineStr">
+        <is>
           <t>C08</t>
         </is>
       </c>
-      <c r="B65" s="64" t="inlineStr">
+      <c r="B66" s="64" t="inlineStr">
         <is>
           <t>Generator</t>
         </is>
       </c>
-      <c r="C65" s="65" t="inlineStr">
+      <c r="C66" s="65" t="inlineStr">
         <is>
           <t>TEST BEZ GENERATORA: klietka + senzory stacia, generator je dalsi nakup; XTG3506 preferred: encoder = free RPM/flow</t>
         </is>
       </c>
-      <c r="E65" s="66" t="inlineStr">
+      <c r="E66" s="66" t="inlineStr">
         <is>
           <t>26.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="66" ht="15.5" customHeight="1">
-      <c r="A66" s="64" t="inlineStr">
-        <is>
-          <t>D01</t>
-        </is>
-      </c>
-      <c r="B66" s="64" t="inlineStr">
-        <is>
-          <t>pH electrode</t>
-        </is>
-      </c>
-      <c r="C66" s="65" t="inlineStr">
-        <is>
-          <t>OPTIONAL per site; 14-30 day service; +-0.1 pH after 2-pt cal</t>
-        </is>
-      </c>
-      <c r="E66" s="66" t="inlineStr">
-        <is>
-          <t>39.0</t>
         </is>
       </c>
     </row>
     <row r="67" ht="15.5" customHeight="1">
       <c r="A67" s="64" t="inlineStr">
         <is>
-          <t>D02</t>
+          <t>D01</t>
         </is>
       </c>
       <c r="B67" s="64" t="inlineStr">
         <is>
-          <t>pH spare electrode</t>
+          <t>pH electrode</t>
         </is>
       </c>
       <c r="C67" s="65" t="inlineStr">
         <is>
-          <t>consumable</t>
+          <t>OPTIONAL per site; 14-30 day service; +-0.1 pH after 2-pt cal</t>
         </is>
       </c>
       <c r="E67" s="66" t="inlineStr">
         <is>
-          <t>9.0</t>
+          <t>39.0</t>
         </is>
       </c>
     </row>
     <row r="68" ht="15.5" customHeight="1">
       <c r="A68" s="64" t="inlineStr">
         <is>
+          <t>D02</t>
+        </is>
+      </c>
+      <c r="B68" s="64" t="inlineStr">
+        <is>
+          <t>pH spare electrode</t>
+        </is>
+      </c>
+      <c r="C68" s="65" t="inlineStr">
+        <is>
+          <t>consumable</t>
+        </is>
+      </c>
+      <c r="E68" s="66" t="inlineStr">
+        <is>
+          <t>9.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="15.5" customHeight="1">
+      <c r="A69" s="64" t="inlineStr">
+        <is>
           <t>D03</t>
         </is>
       </c>
-      <c r="B68" s="64" t="inlineStr">
+      <c r="B69" s="64" t="inlineStr">
         <is>
           <t>pH buffer</t>
         </is>
       </c>
-      <c r="C68" s="65" t="inlineStr">
+      <c r="C69" s="65" t="inlineStr">
         <is>
           <t>consumable</t>
         </is>
       </c>
-      <c r="E68" s="66" t="inlineStr">
+      <c r="E69" s="66" t="inlineStr">
         <is>
           <t>12.0</t>
         </is>
       </c>
     </row>
-    <row r="69" ht="29" customHeight="1">
-      <c r="A69" s="64" t="inlineStr">
+    <row r="70" ht="29" customHeight="1">
+      <c r="A70" s="64" t="inlineStr">
         <is>
           <t>D09</t>
         </is>
       </c>
-      <c r="B69" s="64" t="inlineStr">
+      <c r="B70" s="64" t="inlineStr">
         <is>
           <t>Dissolved oxygen kit</t>
         </is>
       </c>
-      <c r="C69" s="65" t="inlineStr">
+      <c r="C70" s="65" t="inlineStr">
         <is>
           <t>HIGHEST-VALUE channel (Budca = hypoxia); membrane 1-2 months in muddy water; 0.5M NaOH filling solution NOT shipped by air - source locally</t>
         </is>
       </c>
-      <c r="E69" s="66" t="inlineStr">
+      <c r="E70" s="66" t="inlineStr">
         <is>
           <t>175.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="70" ht="15.5" customHeight="1">
-      <c r="A70" s="64" t="inlineStr">
-        <is>
-          <t>D05</t>
-        </is>
-      </c>
-      <c r="B70" s="64" t="inlineStr">
-        <is>
-          <t>Level / stage probe</t>
-        </is>
-      </c>
-      <c r="C70" s="65" t="inlineStr">
-        <is>
-          <t>MS5837-30BA REJECTED: gel element must be dried daily, 24h max submersion</t>
-        </is>
-      </c>
-      <c r="E70" s="66" t="inlineStr">
-        <is>
-          <t>110.0</t>
         </is>
       </c>
     </row>
     <row r="71" ht="15.5" customHeight="1">
       <c r="A71" s="64" t="inlineStr">
         <is>
-          <t>D06</t>
+          <t>D05</t>
         </is>
       </c>
       <c r="B71" s="64" t="inlineStr">
         <is>
-          <t>EC/TDS</t>
+          <t>Level / stage probe</t>
         </is>
       </c>
       <c r="C71" s="65" t="inlineStr">
         <is>
-          <t>+-10% FS is the weakest sensor; use as trend indicator, site-calibrate</t>
+          <t>MS5837-30BA REJECTED: gel element must be dried daily, 24h max submersion</t>
         </is>
       </c>
       <c r="E71" s="66" t="inlineStr">
         <is>
-          <t>14.0</t>
+          <t>110.0</t>
         </is>
       </c>
     </row>
     <row r="72" ht="15.5" customHeight="1">
       <c r="A72" s="64" t="inlineStr">
         <is>
-          <t>D08</t>
+          <t>D06</t>
         </is>
       </c>
       <c r="B72" s="64" t="inlineStr">
         <is>
-          <t>Sensor cable</t>
-        </is>
-      </c>
-      <c r="C72" s="65" t="inlineStr"/>
+          <t>EC/TDS</t>
+        </is>
+      </c>
+      <c r="C72" s="65" t="inlineStr">
+        <is>
+          <t>+-10% FS is the weakest sensor; use as trend indicator, site-calibrate</t>
+        </is>
+      </c>
       <c r="E72" s="66" t="inlineStr">
         <is>
-          <t>20.0</t>
+          <t>14.0</t>
         </is>
       </c>
     </row>
     <row r="73" ht="15.5" customHeight="1">
       <c r="A73" s="64" t="inlineStr">
         <is>
-          <t>G04</t>
+          <t>D08</t>
         </is>
       </c>
       <c r="B73" s="64" t="inlineStr">
         <is>
-          <t>Antenna probe</t>
-        </is>
-      </c>
-      <c r="C73" s="65" t="inlineStr">
-        <is>
-          <t>v baleni kazdej Wio-E5 je EU868 antena - samostatne netreba; drzat ako zalohu</t>
-        </is>
-      </c>
+          <t>Sensor cable</t>
+        </is>
+      </c>
+      <c r="C73" s="65" t="inlineStr"/>
       <c r="E73" s="66" t="inlineStr">
         <is>
-          <t>6.0</t>
+          <t>20.0</t>
         </is>
       </c>
     </row>
     <row r="74" ht="15.5" customHeight="1">
       <c r="A74" s="64" t="inlineStr">
         <is>
-          <t>G05</t>
+          <t>G04</t>
         </is>
       </c>
       <c r="B74" s="64" t="inlineStr">
         <is>
-          <t>Antenna pigtail</t>
+          <t>Antenna probe</t>
         </is>
       </c>
       <c r="C74" s="65" t="inlineStr">
         <is>
-          <t>netreba: doska ma SMA, antena sa skrutkuje priamo; pigtail len ak sa ide cez bulkhead</t>
+          <t>v baleni kazdej Wio-E5 je EU868 antena - samostatne netreba; drzat ako zalohu</t>
         </is>
       </c>
       <c r="E74" s="66" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>6.0</t>
         </is>
       </c>
     </row>
@@ -3068,20 +3072,20 @@
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="A21:E21"/>
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A53:E53"/>
+    <mergeCell ref="A39:E39"/>
+    <mergeCell ref="A63:F63"/>
     <mergeCell ref="A59:E59"/>
-    <mergeCell ref="A20:E20"/>
-    <mergeCell ref="A38:E38"/>
-    <mergeCell ref="A57:E57"/>
+    <mergeCell ref="A43:E43"/>
+    <mergeCell ref="A54:E54"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A42:E42"/>
+    <mergeCell ref="A28:E28"/>
+    <mergeCell ref="A60:E60"/>
+    <mergeCell ref="A33:E33"/>
     <mergeCell ref="A5:E5"/>
-    <mergeCell ref="A32:E32"/>
-    <mergeCell ref="A62:F62"/>
     <mergeCell ref="A3:F3"/>
     <mergeCell ref="A58:E58"/>
-    <mergeCell ref="A27:E27"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId1"/>
@@ -3096,12 +3100,13 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B16" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B17" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B18" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B23" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B19" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B24" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B25" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B29" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B26" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B30" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B40" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B31" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B41" r:id="rId19"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
@@ -5545,16 +5550,16 @@
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>Antenna pigtail</t>
+          <t>u.FL -&gt; SMA pigtail</t>
         </is>
       </c>
       <c r="C63" s="6" t="inlineStr">
         <is>
-          <t>u.FL to SMA bulkhead 15cm</t>
+          <t>u.FL/IPEX female na SMA female bulkhead, 10-15 cm, RG178</t>
         </is>
       </c>
       <c r="D63" s="7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E63" s="6" t="inlineStr">
         <is>
@@ -5565,7 +5570,7 @@
         <v>3</v>
       </c>
       <c r="G63" s="8" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H63" s="7" t="inlineStr">
         <is>
@@ -5589,7 +5594,7 @@
       </c>
       <c r="L63" s="6" t="inlineStr">
         <is>
-          <t>netreba: doska ma SMA, antena sa skrutkuje priamo; pigtail len ak sa ide cez bulkhead</t>
+          <t>KIT MA U.FL, NIE SMA: bez pigtailu na vacsiu antenu nepripojis; 1x sonda, 1x gateway</t>
         </is>
       </c>
     </row>
@@ -6269,7 +6274,7 @@
       <c r="E76" s="70" t="n"/>
       <c r="F76" s="15" t="n"/>
       <c r="G76" s="15" t="n">
-        <v>96.90000000000001</v>
+        <v>102.9</v>
       </c>
       <c r="H76" s="14" t="n"/>
       <c r="I76" s="14" t="n"/>
@@ -8033,7 +8038,7 @@
       <c r="E120" s="69" t="n"/>
       <c r="F120" s="70" t="n"/>
       <c r="G120" s="25" t="n">
-        <v>710.3100000000001</v>
+        <v>716.3100000000001</v>
       </c>
     </row>
     <row r="121">
@@ -8063,7 +8068,7 @@
       <c r="E122" s="69" t="n"/>
       <c r="F122" s="70" t="n"/>
       <c r="G122" s="29" t="n">
-        <v>1351.31</v>
+        <v>1357.31</v>
       </c>
     </row>
     <row r="123">
@@ -8093,7 +8098,7 @@
       <c r="E124" s="69" t="n"/>
       <c r="F124" s="70" t="n"/>
       <c r="G124" s="33" t="n">
-        <v>1281.31</v>
+        <v>1287.31</v>
       </c>
     </row>
   </sheetData>
@@ -8281,7 +8286,7 @@
         </is>
       </c>
       <c r="B10" s="36" t="n">
-        <v>96.90000000000001</v>
+        <v>102.9</v>
       </c>
       <c r="C10" s="36" t="n">
         <v>0</v>
@@ -8361,7 +8366,7 @@
         </is>
       </c>
       <c r="B15" s="38" t="n">
-        <v>710.3100000000001</v>
+        <v>716.3100000000001</v>
       </c>
       <c r="C15" s="38" t="n">
         <v>641</v>

</xml_diff>

<commit_message>
order: back to the full build
The 30-minute dip was my scope, not his: the generator, the cabling, the buck and
the whole energy chain belong in the build. Restored to phase 1, together with
the site structure and the gateway mast.

Only three things stay out, each for a stated reason: the IP68 box on the bank
(he does not need it), the gateway enclosure, and the two tools. The five dead
lines stay cut.

phase 1: 73 lines, 988.11 EUR goods
</commit_message>
<xml_diff>
--- a/docs/sub-mission_parts.xlsx
+++ b/docs/sub-mission_parts.xlsx
@@ -274,7 +274,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="71">
+  <cellXfs count="74">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -393,9 +393,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top"/>
     </xf>
@@ -405,9 +402,6 @@
     <xf numFmtId="0" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -415,6 +409,21 @@
       <alignment horizontal="right" vertical="top"/>
     </xf>
     <xf numFmtId="4" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="4" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -809,7 +818,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F116"/>
+  <dimension ref="A1:F131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -837,18 +846,18 @@
     <row r="3" ht="26" customHeight="1">
       <c r="A3" s="44" t="inlineStr">
         <is>
-          <t>32 lines      goods 220.61 EUR      shipping est. 25.00 EUR      LANDED 245.61 EUR</t>
+          <t>73 lines      goods 988.11 EUR      shipping est. 25.00 EUR      LANDED 1013.11 EUR</t>
         </is>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="45" t="inlineStr">
         <is>
-          <t>TME</t>
+          <t>LOCAL / SHOP</t>
         </is>
       </c>
       <c r="F5" s="46" t="n">
-        <v>124.36</v>
+        <v>413</v>
       </c>
     </row>
     <row r="6">
@@ -883,2230 +892,2656 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="15.5" customHeight="1">
+    <row r="7" ht="42.5" customHeight="1">
       <c r="A7" s="49" t="inlineStr">
         <is>
-          <t>F01</t>
-        </is>
-      </c>
-      <c r="B7" s="50" t="inlineStr">
-        <is>
-          <t>Cable</t>
+          <t>D09</t>
+        </is>
+      </c>
+      <c r="B7" s="49" t="inlineStr">
+        <is>
+          <t>Dissolved oxygen kit</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>8x0.5mm2 PUR jacket submersible 6m</t>
-        </is>
-      </c>
-      <c r="D7" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="E7" s="52" t="n">
-        <v>35</v>
-      </c>
-      <c r="F7" s="52" t="n">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="8" ht="15.5" customHeight="1">
-      <c r="A8" s="53" t="inlineStr">
-        <is>
-          <t>G01</t>
-        </is>
-      </c>
-      <c r="B8" s="54" t="inlineStr">
-        <is>
-          <t>Enclosure</t>
-        </is>
-      </c>
-      <c r="C8" s="55" t="inlineStr">
-        <is>
-          <t>IP68 ready-made 190x130x80mm  -  in model as site_box</t>
-        </is>
-      </c>
-      <c r="D8" s="56" t="n">
-        <v>1</v>
-      </c>
-      <c r="E8" s="57" t="n">
-        <v>22</v>
-      </c>
-      <c r="F8" s="57" t="n">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="9" ht="15.5" customHeight="1">
+          <t>DFRobot SEN0237-A Gravity analog DO, 0-20 mg/L, BNC probe, 2m cable  -  HIGHEST-VALUE channel (Budca = hypoxia); membrane 1-2 months in muddy water; 0.5M NaOH filling solution NOT shipped by air - source locally</t>
+        </is>
+      </c>
+      <c r="D7" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="51" t="n">
+        <v>175</v>
+      </c>
+      <c r="F7" s="51" t="n">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="8" ht="29" customHeight="1">
+      <c r="A8" s="52" t="inlineStr">
+        <is>
+          <t>I02</t>
+        </is>
+      </c>
+      <c r="B8" s="52" t="inlineStr">
+        <is>
+          <t>Compute</t>
+        </is>
+      </c>
+      <c r="C8" s="53" t="inlineStr">
+        <is>
+          <t>Raspberry Pi 4 4GB + PSU + SD  -  YOU ALREADY HAVE THIS - reuse, zero soldering; runs the gateway service</t>
+        </is>
+      </c>
+      <c r="D8" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="55" t="n">
+        <v>70</v>
+      </c>
+      <c r="F8" s="55" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="9" ht="29" customHeight="1">
       <c r="A9" s="49" t="inlineStr">
         <is>
-          <t>C07</t>
-        </is>
-      </c>
-      <c r="B9" s="50" t="inlineStr">
-        <is>
-          <t>Cable gland wet side</t>
+          <t>I03</t>
+        </is>
+      </c>
+      <c r="B9" s="49" t="inlineStr">
+        <is>
+          <t>Antenna</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>Lapp Skintop MS-M 12x1.5 + Scotchcast 2131  -  NOT YET IN MODEL - add boss</t>
-        </is>
-      </c>
-      <c r="D9" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="E9" s="52" t="n">
-        <v>12</v>
-      </c>
-      <c r="F9" s="52" t="n">
-        <v>12</v>
+          <t>MikroTik 868_Omni 6.5dBi IP66 862-876MHz + mast kit  -  range-critical: gateway antenna gain + mast height set the link</t>
+        </is>
+      </c>
+      <c r="D9" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="51" t="n">
+        <v>45</v>
+      </c>
+      <c r="F9" s="51" t="n">
+        <v>45</v>
       </c>
     </row>
     <row r="10" ht="15.5" customHeight="1">
-      <c r="A10" s="53" t="inlineStr">
-        <is>
-          <t>F02</t>
-        </is>
-      </c>
-      <c r="B10" s="54" t="inlineStr">
-        <is>
-          <t>Bulkhead connector</t>
-        </is>
-      </c>
-      <c r="C10" s="55" t="inlineStr">
-        <is>
-          <t>potted gland entry (NOT SubConn)  -  cost cut from 85 EUR wet-mate</t>
-        </is>
-      </c>
-      <c r="D10" s="56" t="n">
-        <v>1</v>
-      </c>
-      <c r="E10" s="57" t="n">
-        <v>12</v>
-      </c>
-      <c r="F10" s="57" t="n">
-        <v>12</v>
+      <c r="A10" s="52" t="inlineStr">
+        <is>
+          <t>I05</t>
+        </is>
+      </c>
+      <c r="B10" s="52" t="inlineStr">
+        <is>
+          <t>Mast</t>
+        </is>
+      </c>
+      <c r="C10" s="53" t="inlineStr">
+        <is>
+          <t>3m alu mast + wall bracket  -  height sets range</t>
+        </is>
+      </c>
+      <c r="D10" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="55" t="n">
+        <v>30</v>
+      </c>
+      <c r="F10" s="55" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="11" ht="15.5" customHeight="1">
       <c r="A11" s="49" t="inlineStr">
         <is>
-          <t>G17</t>
-        </is>
-      </c>
-      <c r="B11" s="50" t="inlineStr">
-        <is>
-          <t>Cable glands</t>
+          <t>H01</t>
+        </is>
+      </c>
+      <c r="B11" s="49" t="inlineStr">
+        <is>
+          <t>Ground screw anchor</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>M12 IP68 potted x3</t>
-        </is>
-      </c>
-      <c r="D11" s="51" t="n">
-        <v>3</v>
-      </c>
-      <c r="E11" s="52" t="n">
-        <v>3</v>
-      </c>
-      <c r="F11" s="52" t="n">
+          <t>M68 x 800mm solar-fence ground screw  -  1-2kN lateral - covers flood case</t>
+        </is>
+      </c>
+      <c r="D11" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" s="51" t="n">
+        <v>25</v>
+      </c>
+      <c r="F11" s="51" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="12" ht="29" customHeight="1">
+      <c r="A12" s="52" t="inlineStr">
+        <is>
+          <t>H02</t>
+        </is>
+      </c>
+      <c r="B12" s="52" t="inlineStr">
+        <is>
+          <t>Pole</t>
+        </is>
+      </c>
+      <c r="C12" s="53" t="inlineStr">
+        <is>
+          <t>scaffold tube Ø48.3x3.2 x 3000mm galvanised  -  removable mast pinned into receiver</t>
+        </is>
+      </c>
+      <c r="D12" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="55" t="n">
+        <v>18</v>
+      </c>
+      <c r="F12" s="55" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="13" ht="15.5" customHeight="1">
+      <c r="A13" s="49" t="inlineStr">
+        <is>
+          <t>H10</t>
+        </is>
+      </c>
+      <c r="B13" s="49" t="inlineStr">
+        <is>
+          <t>Guy anchor</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>300mm ground screw x2</t>
+        </is>
+      </c>
+      <c r="D13" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="51" t="n">
+        <v>10</v>
+      </c>
+      <c r="F13" s="51" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="14" ht="15.5" customHeight="1">
+      <c r="A14" s="52" t="inlineStr">
+        <is>
+          <t>H04</t>
+        </is>
+      </c>
+      <c r="B14" s="52" t="inlineStr">
+        <is>
+          <t>Arm tube</t>
+        </is>
+      </c>
+      <c r="C14" s="53" t="inlineStr">
+        <is>
+          <t>alu Ø28x1.5 x 1300mm</t>
+        </is>
+      </c>
+      <c r="D14" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="55" t="n">
         <v>9</v>
       </c>
-    </row>
-    <row r="12" ht="15.5" customHeight="1">
-      <c r="A12" s="53" t="inlineStr">
-        <is>
-          <t>E02</t>
-        </is>
-      </c>
-      <c r="B12" s="54" t="inlineStr">
-        <is>
-          <t>Cage fasteners</t>
-        </is>
-      </c>
-      <c r="C12" s="55" t="inlineStr">
-        <is>
-          <t>M3x10 A4 + nylok</t>
-        </is>
-      </c>
-      <c r="D12" s="56" t="n">
-        <v>1</v>
-      </c>
-      <c r="E12" s="57" t="n">
-        <v>6</v>
-      </c>
-      <c r="F12" s="57" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="13" ht="29" customHeight="1">
-      <c r="A13" s="49" t="inlineStr">
-        <is>
-          <t>G05</t>
-        </is>
-      </c>
-      <c r="B13" s="50" t="inlineStr">
-        <is>
-          <t>u.FL -&gt; SMA pigtail</t>
-        </is>
-      </c>
-      <c r="C13" s="6" t="inlineStr">
-        <is>
-          <t>u.FL/IPEX female na SMA female bulkhead, 10-15 cm, RG178  -  KIT MA U.FL, NIE SMA: bez pigtailu na vacsiu antenu nepripojis; 1x sonda, 1x gateway</t>
-        </is>
-      </c>
-      <c r="D13" s="51" t="n">
-        <v>2</v>
-      </c>
-      <c r="E13" s="52" t="n">
-        <v>3</v>
-      </c>
-      <c r="F13" s="52" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="14" ht="29" customHeight="1">
-      <c r="A14" s="53" t="inlineStr">
-        <is>
-          <t>G16</t>
-        </is>
-      </c>
-      <c r="B14" s="54" t="inlineStr">
-        <is>
-          <t>Protection</t>
-        </is>
-      </c>
-      <c r="C14" s="55" t="inlineStr">
-        <is>
-          <t>Fuse 0.5A + TVS + ESD array  -  NEMAM - poistka 0.5A + TVS SMBJ5.0A + ESD array (SOT-23-6)</t>
-        </is>
-      </c>
-      <c r="D14" s="56" t="n">
-        <v>1</v>
-      </c>
-      <c r="E14" s="57" t="n">
-        <v>6</v>
-      </c>
-      <c r="F14" s="57" t="n">
-        <v>6</v>
+      <c r="F14" s="55" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="15" ht="15.5" customHeight="1">
       <c r="A15" s="49" t="inlineStr">
         <is>
-          <t>J07</t>
-        </is>
-      </c>
-      <c r="B15" s="50" t="inlineStr">
-        <is>
-          <t>Heat-set inserts</t>
+          <t>H03</t>
+        </is>
+      </c>
+      <c r="B15" s="49" t="inlineStr">
+        <is>
+          <t>Receiver sleeve</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>M3/M4 brass assortment</t>
-        </is>
-      </c>
-      <c r="D15" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="E15" s="52" t="n">
+          <t>Ø52 tube 300mm + pin holes  -  pinned mast interface</t>
+        </is>
+      </c>
+      <c r="D15" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" s="51" t="n">
+        <v>8</v>
+      </c>
+      <c r="F15" s="51" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="16" ht="15.5" customHeight="1">
+      <c r="A16" s="52" t="inlineStr">
+        <is>
+          <t>H05</t>
+        </is>
+      </c>
+      <c r="B16" s="52" t="inlineStr">
+        <is>
+          <t>Drop tube</t>
+        </is>
+      </c>
+      <c r="C16" s="53" t="inlineStr">
+        <is>
+          <t>alu Ø22x1.5 x 900mm</t>
+        </is>
+      </c>
+      <c r="D16" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" s="55" t="n">
         <v>6</v>
       </c>
-      <c r="F15" s="52" t="n">
+      <c r="F16" s="55" t="n">
         <v>6</v>
       </c>
     </row>
-    <row r="16" ht="15.5" customHeight="1">
-      <c r="A16" s="53" t="inlineStr">
-        <is>
-          <t>C03</t>
-        </is>
-      </c>
-      <c r="B16" s="54" t="inlineStr">
-        <is>
-          <t>Pod O-ring</t>
-        </is>
-      </c>
-      <c r="C16" s="55" t="inlineStr">
-        <is>
-          <t>NBR 70 Ø100x2.5  -  zadny spoj podu - bez neho sa pri ponoreni natecie</t>
-        </is>
-      </c>
-      <c r="D16" s="56" t="n">
-        <v>1</v>
-      </c>
-      <c r="E16" s="57" t="n">
-        <v>3</v>
-      </c>
-      <c r="F16" s="57" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="17" ht="29" customHeight="1">
+    <row r="17" ht="15.5" customHeight="1">
       <c r="A17" s="49" t="inlineStr">
         <is>
-          <t>C05</t>
-        </is>
-      </c>
-      <c r="B17" s="50" t="inlineStr">
-        <is>
-          <t>Pod clamp screws</t>
+          <t>H08</t>
+        </is>
+      </c>
+      <c r="B17" s="49" t="inlineStr">
+        <is>
+          <t>Yaw strut</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>M4x30 A4 + washers  -  drzi zadny spoj; integralny bulkhead riesi len prednu stranu</t>
-        </is>
-      </c>
-      <c r="D17" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="E17" s="52" t="n">
-        <v>3</v>
-      </c>
-      <c r="F17" s="52" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="18" ht="29" customHeight="1">
-      <c r="A18" s="53" t="inlineStr">
-        <is>
-          <t>A04</t>
-        </is>
-      </c>
-      <c r="B18" s="54" t="inlineStr">
-        <is>
-          <t>Wet bearing</t>
-        </is>
-      </c>
-      <c r="C18" s="55" t="inlineStr">
-        <is>
-          <t>igus iglidur J plain bearing JSM-0507-05 5x7x5mm  -  83 pcs in stock; JFM-0507-05 flanged 1.48 USD alt</t>
-        </is>
-      </c>
-      <c r="D18" s="56" t="n">
-        <v>2</v>
-      </c>
-      <c r="E18" s="57" t="n">
-        <v>1.18</v>
-      </c>
-      <c r="F18" s="57" t="n">
-        <v>2.36</v>
+          <t>alu Ø22x600mm + 2 clamps  -  anti-flutter</t>
+        </is>
+      </c>
+      <c r="D17" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" s="51" t="n">
+        <v>5</v>
+      </c>
+      <c r="F17" s="51" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="18" ht="15.5" customHeight="1">
+      <c r="A18" s="52" t="inlineStr">
+        <is>
+          <t>K03</t>
+        </is>
+      </c>
+      <c r="B18" s="52" t="inlineStr">
+        <is>
+          <t>Spring balance</t>
+        </is>
+      </c>
+      <c r="C18" s="53" t="inlineStr">
+        <is>
+          <t>0-5N for coupling slip jig  -  one-off</t>
+        </is>
+      </c>
+      <c r="D18" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" s="55" t="n">
+        <v>5</v>
+      </c>
+      <c r="F18" s="55" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="19" ht="15.5" customHeight="1">
       <c r="A19" s="49" t="inlineStr">
         <is>
-          <t>A06</t>
-        </is>
-      </c>
-      <c r="B19" s="50" t="inlineStr">
-        <is>
-          <t>Set screw</t>
+          <t>C06</t>
+        </is>
+      </c>
+      <c r="B19" s="49" t="inlineStr">
+        <is>
+          <t>Desiccant</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>M4x8 316SS cup point ISO 4029</t>
-        </is>
-      </c>
-      <c r="D19" s="51" t="n">
+          <t>5g silica gel with indicator  -  replace at service</t>
+        </is>
+      </c>
+      <c r="D19" s="50" t="n">
         <v>2</v>
       </c>
-      <c r="E19" s="52" t="n">
-        <v>1</v>
-      </c>
-      <c r="F19" s="52" t="n">
+      <c r="E19" s="51" t="n">
         <v>2</v>
       </c>
-    </row>
-    <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="45" t="inlineStr">
-        <is>
-          <t>TECHFUN.SK</t>
-        </is>
-      </c>
-      <c r="F21" s="46" t="n">
-        <v>49.45</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="47" t="inlineStr">
+      <c r="F19" s="51" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="20" ht="29" customHeight="1">
+      <c r="A20" s="52" t="inlineStr">
+        <is>
+          <t>H13</t>
+        </is>
+      </c>
+      <c r="B20" s="52" t="inlineStr">
+        <is>
+          <t>Site label</t>
+        </is>
+      </c>
+      <c r="C20" s="53" t="inlineStr">
+        <is>
+          <t>engraved plate with project + contact  -  anti-theft by making it unsellable</t>
+        </is>
+      </c>
+      <c r="D20" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" s="55" t="n">
+        <v>3</v>
+      </c>
+      <c r="F20" s="55" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="21" ht="29" customHeight="1">
+      <c r="A21" s="49" t="inlineStr">
+        <is>
+          <t>C04</t>
+        </is>
+      </c>
+      <c r="B21" s="49" t="inlineStr">
+        <is>
+          <t>O-ring groove</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>2.2mm wide x 1.8mm deep machined/printed into pod rim  -  NOT YET IN MODEL - add to pod</t>
+        </is>
+      </c>
+      <c r="D21" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" s="51" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" s="51" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="45" t="inlineStr">
+        <is>
+          <t>TME</t>
+        </is>
+      </c>
+      <c r="F23" s="46" t="n">
+        <v>218.26</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="47" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B22" s="47" t="inlineStr">
+      <c r="B24" s="47" t="inlineStr">
         <is>
           <t>Part</t>
         </is>
       </c>
-      <c r="C22" s="47" t="inlineStr">
+      <c r="C24" s="47" t="inlineStr">
         <is>
           <t>Specification / note</t>
         </is>
       </c>
-      <c r="D22" s="48" t="inlineStr">
+      <c r="D24" s="48" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="E22" s="48" t="inlineStr">
+      <c r="E24" s="48" t="inlineStr">
         <is>
           <t>Unit EUR</t>
         </is>
       </c>
-      <c r="F22" s="48" t="inlineStr">
+      <c r="F24" s="48" t="inlineStr">
         <is>
           <t>Total EUR</t>
         </is>
-      </c>
-    </row>
-    <row r="23" ht="15.5" customHeight="1">
-      <c r="A23" s="49" t="inlineStr">
-        <is>
-          <t>J03</t>
-        </is>
-      </c>
-      <c r="B23" s="49" t="inlineStr">
-        <is>
-          <t>Epoxy barrier</t>
-        </is>
-      </c>
-      <c r="C23" s="6" t="inlineStr">
-        <is>
-          <t>West System 105 + 206</t>
-        </is>
-      </c>
-      <c r="D23" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="E23" s="52" t="n">
-        <v>18</v>
-      </c>
-      <c r="F23" s="52" t="n">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="24" ht="29" customHeight="1">
-      <c r="A24" s="53" t="inlineStr">
-        <is>
-          <t>B04</t>
-        </is>
-      </c>
-      <c r="B24" s="54" t="inlineStr">
-        <is>
-          <t>Potting compound</t>
-        </is>
-      </c>
-      <c r="C24" s="55" t="inlineStr">
-        <is>
-          <t>3M Scotch-Weld DP270 black 25ml  -  techfun nema DP270; silikonova zalievacia hmota staci na test, epoxid je tuhsi</t>
-        </is>
-      </c>
-      <c r="D24" s="56" t="n">
-        <v>1</v>
-      </c>
-      <c r="E24" s="57" t="n">
-        <v>14</v>
-      </c>
-      <c r="F24" s="57" t="n">
-        <v>14</v>
       </c>
     </row>
     <row r="25" ht="15.5" customHeight="1">
       <c r="A25" s="49" t="inlineStr">
         <is>
-          <t>D07</t>
-        </is>
-      </c>
-      <c r="B25" s="50" t="inlineStr">
-        <is>
-          <t>Turbidity</t>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="B25" s="56" t="inlineStr">
+        <is>
+          <t>Cable</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>DFRobot SEN0189 (0-4.5V analog)  -  6 in stock; in model as sensor_turb</t>
-        </is>
-      </c>
-      <c r="D25" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="E25" s="52" t="n">
-        <v>12.45</v>
-      </c>
-      <c r="F25" s="52" t="n">
-        <v>12.45</v>
+          <t>8x0.5mm2 PUR jacket submersible 6m</t>
+        </is>
+      </c>
+      <c r="D25" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" s="51" t="n">
+        <v>35</v>
+      </c>
+      <c r="F25" s="51" t="n">
+        <v>35</v>
       </c>
     </row>
     <row r="26" ht="15.5" customHeight="1">
-      <c r="A26" s="53" t="inlineStr">
-        <is>
-          <t>D04</t>
-        </is>
-      </c>
-      <c r="B26" s="54" t="inlineStr">
-        <is>
-          <t>Temperature</t>
-        </is>
-      </c>
-      <c r="C26" s="55" t="inlineStr">
-        <is>
-          <t>DS18B20 waterproof 1m cable  -  in model as sensor_ntc</t>
-        </is>
-      </c>
-      <c r="D26" s="56" t="n">
-        <v>1</v>
-      </c>
-      <c r="E26" s="57" t="n">
-        <v>5</v>
-      </c>
-      <c r="F26" s="57" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="28" ht="20" customHeight="1">
-      <c r="A28" s="45" t="inlineStr">
-        <is>
-          <t>RPISHOP.CZ</t>
-        </is>
-      </c>
-      <c r="F28" s="46" t="n">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="47" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B29" s="47" t="inlineStr">
-        <is>
-          <t>Part</t>
-        </is>
-      </c>
-      <c r="C29" s="47" t="inlineStr">
-        <is>
-          <t>Specification / note</t>
-        </is>
-      </c>
-      <c r="D29" s="48" t="inlineStr">
-        <is>
-          <t>Qty</t>
-        </is>
-      </c>
-      <c r="E29" s="48" t="inlineStr">
-        <is>
-          <t>Unit EUR</t>
-        </is>
-      </c>
-      <c r="F29" s="48" t="inlineStr">
-        <is>
-          <t>Total EUR</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="42.5" customHeight="1">
-      <c r="A30" s="49" t="inlineStr">
-        <is>
-          <t>G03</t>
-        </is>
-      </c>
-      <c r="B30" s="50" t="inlineStr">
-        <is>
-          <t>MCU + radio (single board)</t>
-        </is>
-      </c>
-      <c r="C30" s="6" t="inlineStr">
-        <is>
-          <t>Seeed XIAO nRF52840 + Wio-SX1262 kit (Meshtastic), SEE336 - nRF52840 + SX1262  -  349 Kc, skladom 5+; nahradza Wio-E5, ktory v CZ/SK nie je; antena je v kite</t>
-        </is>
-      </c>
-      <c r="D30" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="E30" s="52" t="n">
+      <c r="A26" s="52" t="inlineStr">
+        <is>
+          <t>D08</t>
+        </is>
+      </c>
+      <c r="B26" s="52" t="inlineStr">
+        <is>
+          <t>Sensor cable</t>
+        </is>
+      </c>
+      <c r="C26" s="53" t="inlineStr">
+        <is>
+          <t>4x2x0.5mm shielded PUR outdoor</t>
+        </is>
+      </c>
+      <c r="D26" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" s="55" t="n">
+        <v>20</v>
+      </c>
+      <c r="F26" s="55" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="27" ht="29" customHeight="1">
+      <c r="A27" s="49" t="inlineStr">
+        <is>
+          <t>D06</t>
+        </is>
+      </c>
+      <c r="B27" s="49" t="inlineStr">
+        <is>
+          <t>EC/TDS</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>DFRobot SEN0244 Gravity analog TDS module + probe  -  +-10% FS is the weakest sensor; use as trend indicator, site-calibrate</t>
+        </is>
+      </c>
+      <c r="D27" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E27" s="51" t="n">
         <v>14</v>
       </c>
-      <c r="F30" s="52" t="n">
+      <c r="F27" s="51" t="n">
         <v>14</v>
       </c>
     </row>
-    <row r="31" ht="42.5" customHeight="1">
-      <c r="A31" s="53" t="inlineStr">
-        <is>
-          <t>I01</t>
-        </is>
-      </c>
-      <c r="B31" s="54" t="inlineStr">
-        <is>
-          <t>Gateway radio (single-channel)</t>
-        </is>
-      </c>
-      <c r="C31" s="55" t="inlineStr">
-        <is>
-          <t>Seeed XIAO nRF52840 + Wio-SX1262 kit (Meshtastic), SEE336 - nRF52840 + SX1262  -  349 Kc, skladom 5+; nahradza Wio-E5, ktory v CZ/SK nie je; antena je v kite</t>
-        </is>
-      </c>
-      <c r="D31" s="56" t="n">
-        <v>1</v>
-      </c>
-      <c r="E31" s="57" t="n">
+    <row r="28" ht="15.5" customHeight="1">
+      <c r="A28" s="52" t="inlineStr">
+        <is>
+          <t>J04</t>
+        </is>
+      </c>
+      <c r="B28" s="52" t="inlineStr">
+        <is>
+          <t>Conformal coat</t>
+        </is>
+      </c>
+      <c r="C28" s="53" t="inlineStr">
+        <is>
+          <t>Electrolube acrylic 200ml</t>
+        </is>
+      </c>
+      <c r="D28" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="E28" s="55" t="n">
         <v>14</v>
       </c>
-      <c r="F31" s="57" t="n">
+      <c r="F28" s="55" t="n">
         <v>14</v>
       </c>
     </row>
-    <row r="33" ht="20" customHeight="1">
-      <c r="A33" s="45" t="inlineStr">
-        <is>
-          <t>LOCAL / SHOP</t>
-        </is>
-      </c>
-      <c r="F33" s="46" t="n">
+    <row r="29" ht="15.5" customHeight="1">
+      <c r="A29" s="49" t="inlineStr">
+        <is>
+          <t>C07</t>
+        </is>
+      </c>
+      <c r="B29" s="56" t="inlineStr">
+        <is>
+          <t>Cable gland wet side</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>Lapp Skintop MS-M 12x1.5 + Scotchcast 2131  -  NOT YET IN MODEL - add boss</t>
+        </is>
+      </c>
+      <c r="D29" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" s="51" t="n">
+        <v>12</v>
+      </c>
+      <c r="F29" s="51" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="30" ht="15.5" customHeight="1">
+      <c r="A30" s="52" t="inlineStr">
+        <is>
+          <t>F02</t>
+        </is>
+      </c>
+      <c r="B30" s="57" t="inlineStr">
+        <is>
+          <t>Bulkhead connector</t>
+        </is>
+      </c>
+      <c r="C30" s="53" t="inlineStr">
+        <is>
+          <t>potted gland entry (NOT SubConn)  -  cost cut from 85 EUR wet-mate</t>
+        </is>
+      </c>
+      <c r="D30" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="E30" s="55" t="n">
+        <v>12</v>
+      </c>
+      <c r="F30" s="55" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="31" ht="15.5" customHeight="1">
+      <c r="A31" s="49" t="inlineStr">
+        <is>
+          <t>J08</t>
+        </is>
+      </c>
+      <c r="B31" s="49" t="inlineStr">
+        <is>
+          <t>O-ring kit</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="inlineStr">
+        <is>
+          <t>NBR metric assortment</t>
+        </is>
+      </c>
+      <c r="D31" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E31" s="51" t="n">
+        <v>12</v>
+      </c>
+      <c r="F31" s="51" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="32" ht="15.5" customHeight="1">
+      <c r="A32" s="52" t="inlineStr">
+        <is>
+          <t>G10</t>
+        </is>
+      </c>
+      <c r="B32" s="52" t="inlineStr">
+        <is>
+          <t>Supercap</t>
+        </is>
+      </c>
+      <c r="C32" s="53" t="inlineStr">
+        <is>
+          <t>Eaton XLR-4R0507 LIC 500F 4.0V  -  NO coin-cell EDLC (50ohm ESR kills TX)</t>
+        </is>
+      </c>
+      <c r="D32" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="E32" s="55" t="n">
+        <v>11</v>
+      </c>
+      <c r="F32" s="55" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="33" ht="15.5" customHeight="1">
+      <c r="A33" s="49" t="inlineStr">
+        <is>
+          <t>J06</t>
+        </is>
+      </c>
+      <c r="B33" s="49" t="inlineStr">
+        <is>
+          <t>Threadlocker</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="inlineStr">
+        <is>
+          <t>Loctite 243 + 406</t>
+        </is>
+      </c>
+      <c r="D33" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E33" s="51" t="n">
+        <v>11</v>
+      </c>
+      <c r="F33" s="51" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="34" ht="15.5" customHeight="1">
+      <c r="A34" s="52" t="inlineStr">
+        <is>
+          <t>G17</t>
+        </is>
+      </c>
+      <c r="B34" s="57" t="inlineStr">
+        <is>
+          <t>Cable glands</t>
+        </is>
+      </c>
+      <c r="C34" s="53" t="inlineStr">
+        <is>
+          <t>M12 IP68 potted x3</t>
+        </is>
+      </c>
+      <c r="D34" s="54" t="n">
+        <v>3</v>
+      </c>
+      <c r="E34" s="55" t="n">
+        <v>3</v>
+      </c>
+      <c r="F34" s="55" t="n">
         <v>9</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="47" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B34" s="47" t="inlineStr">
-        <is>
-          <t>Part</t>
-        </is>
-      </c>
-      <c r="C34" s="47" t="inlineStr">
-        <is>
-          <t>Specification / note</t>
-        </is>
-      </c>
-      <c r="D34" s="48" t="inlineStr">
-        <is>
-          <t>Qty</t>
-        </is>
-      </c>
-      <c r="E34" s="48" t="inlineStr">
-        <is>
-          <t>Unit EUR</t>
-        </is>
-      </c>
-      <c r="F34" s="48" t="inlineStr">
-        <is>
-          <t>Total EUR</t>
-        </is>
       </c>
     </row>
     <row r="35" ht="15.5" customHeight="1">
       <c r="A35" s="49" t="inlineStr">
         <is>
-          <t>K03</t>
+          <t>H09</t>
         </is>
       </c>
       <c r="B35" s="49" t="inlineStr">
         <is>
-          <t>Spring balance</t>
+          <t>Guy line</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>0-5N for coupling slip jig  -  one-off</t>
-        </is>
-      </c>
-      <c r="D35" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="E35" s="52" t="n">
-        <v>5</v>
-      </c>
-      <c r="F35" s="52" t="n">
-        <v>5</v>
+          <t>3mm Dyneema 2x4m + turnbuckles  -  45deg up/downstream</t>
+        </is>
+      </c>
+      <c r="D35" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E35" s="51" t="n">
+        <v>9</v>
+      </c>
+      <c r="F35" s="51" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="36" ht="15.5" customHeight="1">
-      <c r="A36" s="53" t="inlineStr">
-        <is>
-          <t>C06</t>
-        </is>
-      </c>
-      <c r="B36" s="53" t="inlineStr">
-        <is>
-          <t>Desiccant</t>
-        </is>
-      </c>
-      <c r="C36" s="55" t="inlineStr">
-        <is>
-          <t>5g silica gel with indicator  -  replace at service</t>
-        </is>
-      </c>
-      <c r="D36" s="56" t="n">
-        <v>2</v>
-      </c>
-      <c r="E36" s="57" t="n">
-        <v>2</v>
-      </c>
-      <c r="F36" s="57" t="n">
-        <v>4</v>
+      <c r="A36" s="52" t="inlineStr">
+        <is>
+          <t>E02</t>
+        </is>
+      </c>
+      <c r="B36" s="57" t="inlineStr">
+        <is>
+          <t>Cage fasteners</t>
+        </is>
+      </c>
+      <c r="C36" s="53" t="inlineStr">
+        <is>
+          <t>M3x10 A4 + nylok</t>
+        </is>
+      </c>
+      <c r="D36" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="E36" s="55" t="n">
+        <v>6</v>
+      </c>
+      <c r="F36" s="55" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="37" ht="29" customHeight="1">
       <c r="A37" s="49" t="inlineStr">
         <is>
-          <t>C04</t>
-        </is>
-      </c>
-      <c r="B37" s="49" t="inlineStr">
-        <is>
-          <t>O-ring groove</t>
+          <t>G05</t>
+        </is>
+      </c>
+      <c r="B37" s="56" t="inlineStr">
+        <is>
+          <t>u.FL -&gt; SMA pigtail</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>2.2mm wide x 1.8mm deep machined/printed into pod rim  -  NOT YET IN MODEL - add to pod</t>
-        </is>
-      </c>
-      <c r="D37" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="E37" s="52" t="n">
-        <v>0</v>
-      </c>
-      <c r="F37" s="52" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39" ht="20" customHeight="1">
-      <c r="A39" s="45" t="inlineStr">
-        <is>
-          <t>SUPERMAGNETICSHOP</t>
-        </is>
-      </c>
-      <c r="F39" s="46" t="n">
-        <v>8.800000000000001</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="47" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B40" s="47" t="inlineStr">
-        <is>
-          <t>Part</t>
-        </is>
-      </c>
-      <c r="C40" s="47" t="inlineStr">
-        <is>
-          <t>Specification / note</t>
-        </is>
-      </c>
-      <c r="D40" s="48" t="inlineStr">
-        <is>
-          <t>Qty</t>
-        </is>
-      </c>
-      <c r="E40" s="48" t="inlineStr">
-        <is>
-          <t>Unit EUR</t>
-        </is>
-      </c>
-      <c r="F40" s="48" t="inlineStr">
-        <is>
-          <t>Total EUR</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="29" customHeight="1">
+          <t>u.FL/IPEX female na SMA female bulkhead, 10-15 cm, RG178  -  KIT MA U.FL, NIE SMA: bez pigtailu na vacsiu antenu nepripojis; 1x sonda, 1x gateway</t>
+        </is>
+      </c>
+      <c r="D37" s="50" t="n">
+        <v>2</v>
+      </c>
+      <c r="E37" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="F37" s="51" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="38" ht="29" customHeight="1">
+      <c r="A38" s="52" t="inlineStr">
+        <is>
+          <t>G16</t>
+        </is>
+      </c>
+      <c r="B38" s="57" t="inlineStr">
+        <is>
+          <t>Protection</t>
+        </is>
+      </c>
+      <c r="C38" s="53" t="inlineStr">
+        <is>
+          <t>Fuse 0.5A + TVS + ESD array  -  NEMAM - poistka 0.5A + TVS SMBJ5.0A + ESD array (SOT-23-6)</t>
+        </is>
+      </c>
+      <c r="D38" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="E38" s="55" t="n">
+        <v>6</v>
+      </c>
+      <c r="F38" s="55" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="39" ht="15.5" customHeight="1">
+      <c r="A39" s="49" t="inlineStr">
+        <is>
+          <t>J07</t>
+        </is>
+      </c>
+      <c r="B39" s="56" t="inlineStr">
+        <is>
+          <t>Heat-set inserts</t>
+        </is>
+      </c>
+      <c r="C39" s="6" t="inlineStr">
+        <is>
+          <t>M3/M4 brass assortment</t>
+        </is>
+      </c>
+      <c r="D39" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E39" s="51" t="n">
+        <v>6</v>
+      </c>
+      <c r="F39" s="51" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="40" ht="15.5" customHeight="1">
+      <c r="A40" s="52" t="inlineStr">
+        <is>
+          <t>G06</t>
+        </is>
+      </c>
+      <c r="B40" s="52" t="inlineStr">
+        <is>
+          <t>Boost harvester</t>
+        </is>
+      </c>
+      <c r="C40" s="53" t="inlineStr">
+        <is>
+          <t>LTC3105EFE MPPT boost  -  needed when EMF below bus</t>
+        </is>
+      </c>
+      <c r="D40" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="E40" s="55" t="n">
+        <v>5</v>
+      </c>
+      <c r="F40" s="55" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="41" ht="15.5" customHeight="1">
       <c r="A41" s="49" t="inlineStr">
         <is>
-          <t>B01</t>
-        </is>
-      </c>
-      <c r="B41" s="50" t="inlineStr">
-        <is>
-          <t>Magnet</t>
+          <t>G09</t>
+        </is>
+      </c>
+      <c r="B41" s="49" t="inlineStr">
+        <is>
+          <t>Clamp</t>
         </is>
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>N52 D10x5 axially magnetised, canned 316L or epoxy potted  -  16x N52 D10x5 (S-10-05-N52N, 3.3 kg); magsy 10x5 N52 nemá overený</t>
-        </is>
-      </c>
-      <c r="D41" s="51" t="n">
-        <v>16</v>
-      </c>
-      <c r="E41" s="52" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="F41" s="52" t="n">
-        <v>8.800000000000001</v>
-      </c>
-    </row>
-    <row r="43" ht="20" customHeight="1">
-      <c r="A43" s="45" t="inlineStr">
-        <is>
-          <t>PRINTED IN-HOUSE</t>
-        </is>
-      </c>
-      <c r="F43" s="46" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="47" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B44" s="47" t="inlineStr">
-        <is>
-          <t>Part</t>
-        </is>
-      </c>
-      <c r="C44" s="47" t="inlineStr">
-        <is>
-          <t>Specification / note</t>
-        </is>
-      </c>
-      <c r="D44" s="48" t="inlineStr">
-        <is>
-          <t>Qty</t>
-        </is>
-      </c>
-      <c r="E44" s="48" t="inlineStr">
-        <is>
-          <t>Unit EUR</t>
-        </is>
-      </c>
-      <c r="F44" s="48" t="inlineStr">
-        <is>
-          <t>Total EUR</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="15.5" customHeight="1">
+          <t>TL431LIAQ + MJD127T4G + PWR263S 3.3R dump  -  overvoltage protection</t>
+        </is>
+      </c>
+      <c r="D41" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E41" s="51" t="n">
+        <v>4</v>
+      </c>
+      <c r="F41" s="51" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="42" ht="15.5" customHeight="1">
+      <c r="A42" s="52" t="inlineStr">
+        <is>
+          <t>H11</t>
+        </is>
+      </c>
+      <c r="B42" s="52" t="inlineStr">
+        <is>
+          <t>Safety cable</t>
+        </is>
+      </c>
+      <c r="C42" s="53" t="inlineStr">
+        <is>
+          <t>3mm galv wire + ferrules tethering pod to pole  -  theft/flood retention</t>
+        </is>
+      </c>
+      <c r="D42" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="E42" s="55" t="n">
+        <v>4</v>
+      </c>
+      <c r="F42" s="55" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="43" ht="15.5" customHeight="1">
+      <c r="A43" s="49" t="inlineStr">
+        <is>
+          <t>H12</t>
+        </is>
+      </c>
+      <c r="B43" s="49" t="inlineStr">
+        <is>
+          <t>Security fastener</t>
+        </is>
+      </c>
+      <c r="C43" s="6" t="inlineStr">
+        <is>
+          <t>one-way Torx M5 + steel band for box  -  anti-theft</t>
+        </is>
+      </c>
+      <c r="D43" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E43" s="51" t="n">
+        <v>4</v>
+      </c>
+      <c r="F43" s="51" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="44" ht="15.5" customHeight="1">
+      <c r="A44" s="52" t="inlineStr">
+        <is>
+          <t>C03</t>
+        </is>
+      </c>
+      <c r="B44" s="57" t="inlineStr">
+        <is>
+          <t>Pod O-ring</t>
+        </is>
+      </c>
+      <c r="C44" s="53" t="inlineStr">
+        <is>
+          <t>NBR 70 Ø100x2.5  -  zadny spoj podu - bez neho sa pri ponoreni natecie</t>
+        </is>
+      </c>
+      <c r="D44" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="E44" s="55" t="n">
+        <v>3</v>
+      </c>
+      <c r="F44" s="55" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="45" ht="29" customHeight="1">
       <c r="A45" s="49" t="inlineStr">
         <is>
-          <t>C09</t>
-        </is>
-      </c>
-      <c r="B45" s="49" t="inlineStr">
-        <is>
-          <t>Generator mount</t>
+          <t>C05</t>
+        </is>
+      </c>
+      <c r="B45" s="56" t="inlineStr">
+        <is>
+          <t>Pod clamp screws</t>
         </is>
       </c>
       <c r="C45" s="6" t="inlineStr">
         <is>
-          <t>printed cradle + 4x M3x8 A4</t>
-        </is>
-      </c>
-      <c r="D45" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="E45" s="52" t="n">
-        <v>1</v>
-      </c>
-      <c r="F45" s="52" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="46" ht="29" customHeight="1">
-      <c r="A46" s="53" t="inlineStr">
-        <is>
-          <t>A01</t>
-        </is>
-      </c>
-      <c r="B46" s="53" t="inlineStr">
-        <is>
-          <t>Blade</t>
-        </is>
-      </c>
-      <c r="C46" s="55" t="inlineStr">
-        <is>
-          <t>triple-blade rotor blade NACA4412 D220mm root pitch 28deg tip 2deg  -  ASA or ASA-CF; 6 perimeters; epoxy coat; spare blade = fuse for branch strike</t>
-        </is>
-      </c>
-      <c r="D46" s="56" t="n">
+          <t>M4x30 A4 + washers  -  drzi zadny spoj; integralny bulkhead riesi len prednu stranu</t>
+        </is>
+      </c>
+      <c r="D45" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E45" s="51" t="n">
         <v>3</v>
       </c>
-      <c r="E46" s="57" t="n">
-        <v>0</v>
-      </c>
-      <c r="F46" s="57" t="n">
-        <v>0</v>
+      <c r="F45" s="51" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="46" ht="15.5" customHeight="1">
+      <c r="A46" s="52" t="inlineStr">
+        <is>
+          <t>G07</t>
+        </is>
+      </c>
+      <c r="B46" s="52" t="inlineStr">
+        <is>
+          <t>Buck</t>
+        </is>
+      </c>
+      <c r="C46" s="53" t="inlineStr">
+        <is>
+          <t>TPS62A02DRC step-down</t>
+        </is>
+      </c>
+      <c r="D46" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="E46" s="55" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F46" s="55" t="n">
+        <v>2.5</v>
       </c>
     </row>
     <row r="47" ht="29" customHeight="1">
       <c r="A47" s="49" t="inlineStr">
         <is>
-          <t>A02</t>
-        </is>
-      </c>
-      <c r="B47" s="49" t="inlineStr">
-        <is>
-          <t>Hub</t>
+          <t>A04</t>
+        </is>
+      </c>
+      <c r="B47" s="56" t="inlineStr">
+        <is>
+          <t>Wet bearing</t>
         </is>
       </c>
       <c r="C47" s="6" t="inlineStr">
         <is>
-          <t>Ø64x46mm with 2x M4 heat-set inserts and Ø5 H7 shaft bore  -  brass inserts M4 from TME</t>
-        </is>
-      </c>
-      <c r="D47" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="E47" s="52" t="n">
-        <v>0</v>
-      </c>
-      <c r="F47" s="52" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="48" ht="29" customHeight="1">
-      <c r="A48" s="53" t="inlineStr">
-        <is>
-          <t>B02</t>
-        </is>
-      </c>
-      <c r="B48" s="53" t="inlineStr">
-        <is>
-          <t>Magnet cup</t>
-        </is>
-      </c>
-      <c r="C48" s="55" t="inlineStr">
-        <is>
-          <t>D70 rim, 8 pockets D10.2x5.2, printed ASA  -  pockets 10.2 dia (magnet 10 + 0.2 glue), 0.2 mm epoxy recess</t>
-        </is>
-      </c>
-      <c r="D48" s="56" t="n">
+          <t>igus iglidur J plain bearing JSM-0507-05 5x7x5mm  -  83 pcs in stock; JFM-0507-05 flanged 1.48 USD alt</t>
+        </is>
+      </c>
+      <c r="D47" s="50" t="n">
         <v>2</v>
       </c>
-      <c r="E48" s="57" t="n">
-        <v>0</v>
-      </c>
-      <c r="F48" s="57" t="n">
-        <v>0</v>
+      <c r="E47" s="51" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="F47" s="51" t="n">
+        <v>2.36</v>
+      </c>
+    </row>
+    <row r="48" ht="15.5" customHeight="1">
+      <c r="A48" s="52" t="inlineStr">
+        <is>
+          <t>A06</t>
+        </is>
+      </c>
+      <c r="B48" s="57" t="inlineStr">
+        <is>
+          <t>Set screw</t>
+        </is>
+      </c>
+      <c r="C48" s="53" t="inlineStr">
+        <is>
+          <t>M4x8 316SS cup point ISO 4029</t>
+        </is>
+      </c>
+      <c r="D48" s="54" t="n">
+        <v>2</v>
+      </c>
+      <c r="E48" s="55" t="n">
+        <v>1</v>
+      </c>
+      <c r="F48" s="55" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="49" ht="15.5" customHeight="1">
       <c r="A49" s="49" t="inlineStr">
         <is>
+          <t>G12</t>
+        </is>
+      </c>
+      <c r="B49" s="49" t="inlineStr">
+        <is>
+          <t>Load switch</t>
+        </is>
+      </c>
+      <c r="C49" s="6" t="inlineStr">
+        <is>
+          <t>TPS22860 x2 for pH/EC sequencing  -  removes ground-loop need</t>
+        </is>
+      </c>
+      <c r="D49" s="50" t="n">
+        <v>2</v>
+      </c>
+      <c r="E49" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="F49" s="51" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="50" ht="15.5" customHeight="1">
+      <c r="A50" s="52" t="inlineStr">
+        <is>
+          <t>G11</t>
+        </is>
+      </c>
+      <c r="B50" s="52" t="inlineStr">
+        <is>
+          <t>Voltage supervisor</t>
+        </is>
+      </c>
+      <c r="C50" s="53" t="inlineStr">
+        <is>
+          <t>TLV840 nanopower  -  gates buck at 4.8V</t>
+        </is>
+      </c>
+      <c r="D50" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="E50" s="55" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F50" s="55" t="n">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="51" ht="29" customHeight="1">
+      <c r="A51" s="49" t="inlineStr">
+        <is>
+          <t>H07</t>
+        </is>
+      </c>
+      <c r="B51" s="49" t="inlineStr">
+        <is>
+          <t>Shear pin</t>
+        </is>
+      </c>
+      <c r="C51" s="6" t="inlineStr">
+        <is>
+          <t>M4 316SS pin + 2 spares on pole collar  -  releases pod on &gt;150N debris hit</t>
+        </is>
+      </c>
+      <c r="D51" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E51" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="F51" s="51" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52" ht="15.5" customHeight="1">
+      <c r="A52" s="52" t="inlineStr">
+        <is>
+          <t>G08</t>
+        </is>
+      </c>
+      <c r="B52" s="52" t="inlineStr">
+        <is>
+          <t>Rectifier</t>
+        </is>
+      </c>
+      <c r="C52" s="53" t="inlineStr">
+        <is>
+          <t>Nexperia PMEG2010AEB 20V 1A SOD-523  -  452k in stock</t>
+        </is>
+      </c>
+      <c r="D52" s="54" t="n">
+        <v>6</v>
+      </c>
+      <c r="E52" s="55" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="F52" s="55" t="n">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="53" ht="15.5" customHeight="1">
+      <c r="A53" s="58" t="inlineStr">
+        <is>
+          <t>J05</t>
+        </is>
+      </c>
+      <c r="B53" s="58" t="inlineStr">
+        <is>
+          <t>Silicone grease</t>
+        </is>
+      </c>
+      <c r="C53" s="17" t="inlineStr">
+        <is>
+          <t>MAM  |  Molykote 111 100g  -  MAM - doma</t>
+        </is>
+      </c>
+      <c r="D53" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="E53" s="60" t="n">
+        <v>9</v>
+      </c>
+      <c r="F53" s="60" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" ht="20" customHeight="1">
+      <c r="A55" s="45" t="inlineStr">
+        <is>
+          <t>TECHFUN.SK</t>
+        </is>
+      </c>
+      <c r="F55" s="46" t="n">
+        <v>118.45</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="47" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B56" s="47" t="inlineStr">
+        <is>
+          <t>Part</t>
+        </is>
+      </c>
+      <c r="C56" s="47" t="inlineStr">
+        <is>
+          <t>Specification / note</t>
+        </is>
+      </c>
+      <c r="D56" s="48" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="E56" s="48" t="inlineStr">
+        <is>
+          <t>Unit EUR</t>
+        </is>
+      </c>
+      <c r="F56" s="48" t="inlineStr">
+        <is>
+          <t>Total EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="29" customHeight="1">
+      <c r="A57" s="49" t="inlineStr">
+        <is>
+          <t>D01</t>
+        </is>
+      </c>
+      <c r="B57" s="49" t="inlineStr">
+        <is>
+          <t>pH electrode</t>
+        </is>
+      </c>
+      <c r="C57" s="6" t="inlineStr">
+        <is>
+          <t>DFRobot SEN0161-V2 Gravity pH kit + E201 BNC probe  -  OPTIONAL per site; 14-30 day service; +-0.1 pH after 2-pt cal</t>
+        </is>
+      </c>
+      <c r="D57" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E57" s="51" t="n">
+        <v>39</v>
+      </c>
+      <c r="F57" s="51" t="n">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="58" ht="15.5" customHeight="1">
+      <c r="A58" s="52" t="inlineStr">
+        <is>
+          <t>D02</t>
+        </is>
+      </c>
+      <c r="B58" s="52" t="inlineStr">
+        <is>
+          <t>pH spare electrode</t>
+        </is>
+      </c>
+      <c r="C58" s="53" t="inlineStr">
+        <is>
+          <t>E201-C BNC  -  consumable</t>
+        </is>
+      </c>
+      <c r="D58" s="54" t="n">
+        <v>2</v>
+      </c>
+      <c r="E58" s="55" t="n">
+        <v>9</v>
+      </c>
+      <c r="F58" s="55" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="59" ht="15.5" customHeight="1">
+      <c r="A59" s="49" t="inlineStr">
+        <is>
+          <t>J03</t>
+        </is>
+      </c>
+      <c r="B59" s="49" t="inlineStr">
+        <is>
+          <t>Epoxy barrier</t>
+        </is>
+      </c>
+      <c r="C59" s="6" t="inlineStr">
+        <is>
+          <t>West System 105 + 206</t>
+        </is>
+      </c>
+      <c r="D59" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E59" s="51" t="n">
+        <v>18</v>
+      </c>
+      <c r="F59" s="51" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="60" ht="29" customHeight="1">
+      <c r="A60" s="52" t="inlineStr">
+        <is>
+          <t>B04</t>
+        </is>
+      </c>
+      <c r="B60" s="57" t="inlineStr">
+        <is>
+          <t>Potting compound</t>
+        </is>
+      </c>
+      <c r="C60" s="53" t="inlineStr">
+        <is>
+          <t>3M Scotch-Weld DP270 black 25ml  -  techfun nema DP270; silikonova zalievacia hmota staci na test, epoxid je tuhsi</t>
+        </is>
+      </c>
+      <c r="D60" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="E60" s="55" t="n">
+        <v>14</v>
+      </c>
+      <c r="F60" s="55" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="61" ht="15.5" customHeight="1">
+      <c r="A61" s="49" t="inlineStr">
+        <is>
+          <t>D07</t>
+        </is>
+      </c>
+      <c r="B61" s="56" t="inlineStr">
+        <is>
+          <t>Turbidity</t>
+        </is>
+      </c>
+      <c r="C61" s="6" t="inlineStr">
+        <is>
+          <t>DFRobot SEN0189 (0-4.5V analog)  -  6 in stock; in model as sensor_turb</t>
+        </is>
+      </c>
+      <c r="D61" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E61" s="51" t="n">
+        <v>12.45</v>
+      </c>
+      <c r="F61" s="51" t="n">
+        <v>12.45</v>
+      </c>
+    </row>
+    <row r="62" ht="15.5" customHeight="1">
+      <c r="A62" s="52" t="inlineStr">
+        <is>
+          <t>D03</t>
+        </is>
+      </c>
+      <c r="B62" s="52" t="inlineStr">
+        <is>
+          <t>pH buffer</t>
+        </is>
+      </c>
+      <c r="C62" s="53" t="inlineStr">
+        <is>
+          <t>2x250ml pH7 + pH10  -  consumable</t>
+        </is>
+      </c>
+      <c r="D62" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="E62" s="55" t="n">
+        <v>12</v>
+      </c>
+      <c r="F62" s="55" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="63" ht="15.5" customHeight="1">
+      <c r="A63" s="49" t="inlineStr">
+        <is>
+          <t>D04</t>
+        </is>
+      </c>
+      <c r="B63" s="56" t="inlineStr">
+        <is>
+          <t>Temperature</t>
+        </is>
+      </c>
+      <c r="C63" s="6" t="inlineStr">
+        <is>
+          <t>DS18B20 waterproof 1m cable  -  in model as sensor_ntc</t>
+        </is>
+      </c>
+      <c r="D63" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E63" s="51" t="n">
+        <v>5</v>
+      </c>
+      <c r="F63" s="51" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="64" ht="29" customHeight="1">
+      <c r="A64" s="52" t="inlineStr">
+        <is>
+          <t>G04</t>
+        </is>
+      </c>
+      <c r="B64" s="52" t="inlineStr">
+        <is>
+          <t>Antenna probe</t>
+        </is>
+      </c>
+      <c r="C64" s="53" t="inlineStr">
+        <is>
+          <t>868MHz 5dBi SMA-M omni 195mm  -  v baleni kazdej Wio-E5 je EU868 antena - samostatne netreba; drzat ako zalohu</t>
+        </is>
+      </c>
+      <c r="D64" s="54" t="n">
+        <v>0</v>
+      </c>
+      <c r="E64" s="55" t="n">
+        <v>6</v>
+      </c>
+      <c r="F64" s="55" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66" ht="20" customHeight="1">
+      <c r="A66" s="45" t="inlineStr">
+        <is>
+          <t>SENSORSONE (QUOTE)</t>
+        </is>
+      </c>
+      <c r="F66" s="46" t="n">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="47" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B67" s="47" t="inlineStr">
+        <is>
+          <t>Part</t>
+        </is>
+      </c>
+      <c r="C67" s="47" t="inlineStr">
+        <is>
+          <t>Specification / note</t>
+        </is>
+      </c>
+      <c r="D67" s="48" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="E67" s="48" t="inlineStr">
+        <is>
+          <t>Unit EUR</t>
+        </is>
+      </c>
+      <c r="F67" s="48" t="inlineStr">
+        <is>
+          <t>Total EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="42.5" customHeight="1">
+      <c r="A68" s="49" t="inlineStr">
+        <is>
+          <t>D05</t>
+        </is>
+      </c>
+      <c r="B68" s="49" t="inlineStr">
+        <is>
+          <t>Level / stage probe</t>
+        </is>
+      </c>
+      <c r="C68" s="6" t="inlineStr">
+        <is>
+          <t>Submersible IP68 316L, 0-1 mH2O, 0.5-4.5V out, 5m cable, permanent immersion rated  -  MS5837-30BA REJECTED: gel element must be dried daily, 24h max submersion</t>
+        </is>
+      </c>
+      <c r="D68" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E68" s="51" t="n">
+        <v>110</v>
+      </c>
+      <c r="F68" s="51" t="n">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="70" ht="20" customHeight="1">
+      <c r="A70" s="45" t="inlineStr">
+        <is>
+          <t>PRUSA3D</t>
+        </is>
+      </c>
+      <c r="F70" s="46" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="47" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B71" s="47" t="inlineStr">
+        <is>
+          <t>Part</t>
+        </is>
+      </c>
+      <c r="C71" s="47" t="inlineStr">
+        <is>
+          <t>Specification / note</t>
+        </is>
+      </c>
+      <c r="D71" s="48" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="E71" s="48" t="inlineStr">
+        <is>
+          <t>Unit EUR</t>
+        </is>
+      </c>
+      <c r="F71" s="48" t="inlineStr">
+        <is>
+          <t>Total EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="15.5" customHeight="1">
+      <c r="A72" s="49" t="inlineStr">
+        <is>
+          <t>J02</t>
+        </is>
+      </c>
+      <c r="B72" s="49" t="inlineStr">
+        <is>
+          <t>Filament PC Blend</t>
+        </is>
+      </c>
+      <c r="C72" s="6" t="inlineStr">
+        <is>
+          <t>Prusament PC Blend 970g (for wall/structural)</t>
+        </is>
+      </c>
+      <c r="D72" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E72" s="51" t="n">
+        <v>40</v>
+      </c>
+      <c r="F72" s="51" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="73" ht="29" customHeight="1">
+      <c r="A73" s="58" t="inlineStr">
+        <is>
+          <t>J01</t>
+        </is>
+      </c>
+      <c r="B73" s="58" t="inlineStr">
+        <is>
+          <t>Filament ASA</t>
+        </is>
+      </c>
+      <c r="C73" s="17" t="inlineStr">
+        <is>
+          <t>MAM  |  Prusament ASA 850g  -  ABS z domaceho spoolu, nie ASA; UV je len na brehu</t>
+        </is>
+      </c>
+      <c r="D73" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="E73" s="60" t="n">
+        <v>32</v>
+      </c>
+      <c r="F73" s="60" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" ht="20" customHeight="1">
+      <c r="A75" s="45" t="inlineStr">
+        <is>
+          <t>RPISHOP.CZ</t>
+        </is>
+      </c>
+      <c r="F75" s="46" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="47" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B76" s="47" t="inlineStr">
+        <is>
+          <t>Part</t>
+        </is>
+      </c>
+      <c r="C76" s="47" t="inlineStr">
+        <is>
+          <t>Specification / note</t>
+        </is>
+      </c>
+      <c r="D76" s="48" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="E76" s="48" t="inlineStr">
+        <is>
+          <t>Unit EUR</t>
+        </is>
+      </c>
+      <c r="F76" s="48" t="inlineStr">
+        <is>
+          <t>Total EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="42.5" customHeight="1">
+      <c r="A77" s="49" t="inlineStr">
+        <is>
+          <t>G03</t>
+        </is>
+      </c>
+      <c r="B77" s="56" t="inlineStr">
+        <is>
+          <t>MCU + radio (single board)</t>
+        </is>
+      </c>
+      <c r="C77" s="6" t="inlineStr">
+        <is>
+          <t>Seeed XIAO nRF52840 + Wio-SX1262 kit (Meshtastic), SEE336 - nRF52840 + SX1262  -  349 Kc, skladom 5+; nahradza Wio-E5, ktory v CZ/SK nie je; antena je v kite</t>
+        </is>
+      </c>
+      <c r="D77" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E77" s="51" t="n">
+        <v>14</v>
+      </c>
+      <c r="F77" s="51" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="78" ht="42.5" customHeight="1">
+      <c r="A78" s="52" t="inlineStr">
+        <is>
+          <t>I01</t>
+        </is>
+      </c>
+      <c r="B78" s="57" t="inlineStr">
+        <is>
+          <t>Gateway radio (single-channel)</t>
+        </is>
+      </c>
+      <c r="C78" s="53" t="inlineStr">
+        <is>
+          <t>Seeed XIAO nRF52840 + Wio-SX1262 kit (Meshtastic), SEE336 - nRF52840 + SX1262  -  349 Kc, skladom 5+; nahradza Wio-E5, ktory v CZ/SK nie je; antena je v kite</t>
+        </is>
+      </c>
+      <c r="D78" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="E78" s="55" t="n">
+        <v>14</v>
+      </c>
+      <c r="F78" s="55" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="80" ht="20" customHeight="1">
+      <c r="A80" s="45" t="inlineStr">
+        <is>
+          <t>X-TEAMRC.COM</t>
+        </is>
+      </c>
+      <c r="F80" s="46" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="47" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B81" s="47" t="inlineStr">
+        <is>
+          <t>Part</t>
+        </is>
+      </c>
+      <c r="C81" s="47" t="inlineStr">
+        <is>
+          <t>Specification / note</t>
+        </is>
+      </c>
+      <c r="D81" s="48" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="E81" s="48" t="inlineStr">
+        <is>
+          <t>Unit EUR</t>
+        </is>
+      </c>
+      <c r="F81" s="48" t="inlineStr">
+        <is>
+          <t>Total EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="42.5" customHeight="1">
+      <c r="A82" s="49" t="inlineStr">
+        <is>
+          <t>C08</t>
+        </is>
+      </c>
+      <c r="B82" s="49" t="inlineStr">
+        <is>
+          <t>Generator</t>
+        </is>
+      </c>
+      <c r="C82" s="6" t="inlineStr">
+        <is>
+          <t>T-Motor GB2208 KV128 or X-TEAM XTG3506 (24N22P 6ohm w/ AS5048A encoder)  -  TEST BEZ GENERATORA: klietka + senzory stacia, generator je dalsi nakup; XTG3506 preferred: encoder = free RPM/flow</t>
+        </is>
+      </c>
+      <c r="D82" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E82" s="51" t="n">
+        <v>26</v>
+      </c>
+      <c r="F82" s="51" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="84" ht="20" customHeight="1">
+      <c r="A84" s="45" t="inlineStr">
+        <is>
+          <t>LASKAKIT.CZ</t>
+        </is>
+      </c>
+      <c r="F84" s="46" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="47" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B85" s="47" t="inlineStr">
+        <is>
+          <t>Part</t>
+        </is>
+      </c>
+      <c r="C85" s="47" t="inlineStr">
+        <is>
+          <t>Specification / note</t>
+        </is>
+      </c>
+      <c r="D85" s="48" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="E85" s="48" t="inlineStr">
+        <is>
+          <t>Unit EUR</t>
+        </is>
+      </c>
+      <c r="F85" s="48" t="inlineStr">
+        <is>
+          <t>Total EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="15.5" customHeight="1">
+      <c r="A86" s="49" t="inlineStr">
+        <is>
+          <t>G15</t>
+        </is>
+      </c>
+      <c r="B86" s="49" t="inlineStr">
+        <is>
+          <t>Connectors</t>
+        </is>
+      </c>
+      <c r="C86" s="6" t="inlineStr">
+        <is>
+          <t>JST-PH/XH assortment + crimps</t>
+        </is>
+      </c>
+      <c r="D86" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E86" s="51" t="n">
+        <v>10</v>
+      </c>
+      <c r="F86" s="51" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="87" ht="29" customHeight="1">
+      <c r="A87" s="52" t="inlineStr">
+        <is>
+          <t>G13</t>
+        </is>
+      </c>
+      <c r="B87" s="52" t="inlineStr">
+        <is>
+          <t>Barometer</t>
+        </is>
+      </c>
+      <c r="C87" s="53" t="inlineStr">
+        <is>
+          <t>BME280 module outside potting in vented sub-box  -  pressure reference for MS5837</t>
+        </is>
+      </c>
+      <c r="D87" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="E87" s="55" t="n">
+        <v>6</v>
+      </c>
+      <c r="F87" s="55" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="89" ht="20" customHeight="1">
+      <c r="A89" s="45" t="inlineStr">
+        <is>
+          <t>SUPERMAGNETICSHOP</t>
+        </is>
+      </c>
+      <c r="F89" s="46" t="n">
+        <v>8.800000000000001</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="47" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B90" s="47" t="inlineStr">
+        <is>
+          <t>Part</t>
+        </is>
+      </c>
+      <c r="C90" s="47" t="inlineStr">
+        <is>
+          <t>Specification / note</t>
+        </is>
+      </c>
+      <c r="D90" s="48" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="E90" s="48" t="inlineStr">
+        <is>
+          <t>Unit EUR</t>
+        </is>
+      </c>
+      <c r="F90" s="48" t="inlineStr">
+        <is>
+          <t>Total EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="29" customHeight="1">
+      <c r="A91" s="49" t="inlineStr">
+        <is>
+          <t>B01</t>
+        </is>
+      </c>
+      <c r="B91" s="56" t="inlineStr">
+        <is>
+          <t>Magnet</t>
+        </is>
+      </c>
+      <c r="C91" s="6" t="inlineStr">
+        <is>
+          <t>N52 D10x5 axially magnetised, canned 316L or epoxy potted  -  16x N52 D10x5 (S-10-05-N52N, 3.3 kg); magsy 10x5 N52 nemá overený</t>
+        </is>
+      </c>
+      <c r="D91" s="50" t="n">
+        <v>16</v>
+      </c>
+      <c r="E91" s="51" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="F91" s="51" t="n">
+        <v>8.800000000000001</v>
+      </c>
+    </row>
+    <row r="93" ht="20" customHeight="1">
+      <c r="A93" s="45" t="inlineStr">
+        <is>
+          <t>PRINTED IN-HOUSE</t>
+        </is>
+      </c>
+      <c r="F93" s="46" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="47" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B94" s="47" t="inlineStr">
+        <is>
+          <t>Part</t>
+        </is>
+      </c>
+      <c r="C94" s="47" t="inlineStr">
+        <is>
+          <t>Specification / note</t>
+        </is>
+      </c>
+      <c r="D94" s="48" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="E94" s="48" t="inlineStr">
+        <is>
+          <t>Unit EUR</t>
+        </is>
+      </c>
+      <c r="F94" s="48" t="inlineStr">
+        <is>
+          <t>Total EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" ht="15.5" customHeight="1">
+      <c r="A95" s="49" t="inlineStr">
+        <is>
+          <t>H06</t>
+        </is>
+      </c>
+      <c r="B95" s="49" t="inlineStr">
+        <is>
+          <t>Hinge collar</t>
+        </is>
+      </c>
+      <c r="C95" s="6" t="inlineStr">
+        <is>
+          <t>printed ASA + M8 A4 bolt</t>
+        </is>
+      </c>
+      <c r="D95" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E95" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="F95" s="51" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="96" ht="15.5" customHeight="1">
+      <c r="A96" s="52" t="inlineStr">
+        <is>
+          <t>C09</t>
+        </is>
+      </c>
+      <c r="B96" s="52" t="inlineStr">
+        <is>
+          <t>Generator mount</t>
+        </is>
+      </c>
+      <c r="C96" s="53" t="inlineStr">
+        <is>
+          <t>printed cradle + 4x M3x8 A4</t>
+        </is>
+      </c>
+      <c r="D96" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="E96" s="55" t="n">
+        <v>1</v>
+      </c>
+      <c r="F96" s="55" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="97" ht="29" customHeight="1">
+      <c r="A97" s="49" t="inlineStr">
+        <is>
+          <t>A01</t>
+        </is>
+      </c>
+      <c r="B97" s="49" t="inlineStr">
+        <is>
+          <t>Blade</t>
+        </is>
+      </c>
+      <c r="C97" s="6" t="inlineStr">
+        <is>
+          <t>triple-blade rotor blade NACA4412 D220mm root pitch 28deg tip 2deg  -  ASA or ASA-CF; 6 perimeters; epoxy coat; spare blade = fuse for branch strike</t>
+        </is>
+      </c>
+      <c r="D97" s="50" t="n">
+        <v>3</v>
+      </c>
+      <c r="E97" s="51" t="n">
+        <v>0</v>
+      </c>
+      <c r="F97" s="51" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="98" ht="29" customHeight="1">
+      <c r="A98" s="52" t="inlineStr">
+        <is>
+          <t>A02</t>
+        </is>
+      </c>
+      <c r="B98" s="52" t="inlineStr">
+        <is>
+          <t>Hub</t>
+        </is>
+      </c>
+      <c r="C98" s="53" t="inlineStr">
+        <is>
+          <t>Ø64x46mm with 2x M4 heat-set inserts and Ø5 H7 shaft bore  -  brass inserts M4 from TME</t>
+        </is>
+      </c>
+      <c r="D98" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="E98" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="F98" s="55" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="99" ht="29" customHeight="1">
+      <c r="A99" s="49" t="inlineStr">
+        <is>
+          <t>B02</t>
+        </is>
+      </c>
+      <c r="B99" s="49" t="inlineStr">
+        <is>
+          <t>Magnet cup</t>
+        </is>
+      </c>
+      <c r="C99" s="6" t="inlineStr">
+        <is>
+          <t>D70 rim, 8 pockets D10.2x5.2, printed ASA  -  pockets 10.2 dia (magnet 10 + 0.2 glue), 0.2 mm epoxy recess</t>
+        </is>
+      </c>
+      <c r="D99" s="50" t="n">
+        <v>2</v>
+      </c>
+      <c r="E99" s="51" t="n">
+        <v>0</v>
+      </c>
+      <c r="F99" s="51" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="100" ht="15.5" customHeight="1">
+      <c r="A100" s="52" t="inlineStr">
+        <is>
           <t>C01</t>
         </is>
       </c>
-      <c r="B49" s="49" t="inlineStr">
+      <c r="B100" s="52" t="inlineStr">
         <is>
           <t>Pod barrel</t>
         </is>
       </c>
-      <c r="C49" s="6" t="inlineStr">
+      <c r="C100" s="53" t="inlineStr">
         <is>
           <t>Ø110x120mm printed ASA wall 2.4mm + epoxy barrier  -  in model as pod</t>
         </is>
       </c>
-      <c r="D49" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="E49" s="52" t="n">
+      <c r="D100" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="E100" s="55" t="n">
         <v>0</v>
       </c>
-      <c r="F49" s="52" t="n">
+      <c r="F100" s="55" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="50" ht="15.5" customHeight="1">
-      <c r="A50" s="53" t="inlineStr">
+    <row r="101" ht="15.5" customHeight="1">
+      <c r="A101" s="49" t="inlineStr">
         <is>
           <t>C02</t>
         </is>
       </c>
-      <c r="B50" s="53" t="inlineStr">
+      <c r="B101" s="49" t="inlineStr">
         <is>
           <t>Tail cone</t>
         </is>
       </c>
-      <c r="C50" s="55" t="inlineStr">
+      <c r="C101" s="6" t="inlineStr">
         <is>
           <t>printed integral</t>
         </is>
       </c>
-      <c r="D50" s="56" t="n">
-        <v>1</v>
-      </c>
-      <c r="E50" s="57" t="n">
+      <c r="D101" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E101" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="F50" s="57" t="n">
+      <c r="F101" s="51" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="51" ht="15.5" customHeight="1">
-      <c r="A51" s="49" t="inlineStr">
+    <row r="102" ht="15.5" customHeight="1">
+      <c r="A102" s="52" t="inlineStr">
         <is>
           <t>E01</t>
         </is>
       </c>
-      <c r="B51" s="49" t="inlineStr">
+      <c r="B102" s="52" t="inlineStr">
         <is>
           <t>Sensor cage</t>
         </is>
       </c>
-      <c r="C51" s="6" t="inlineStr">
+      <c r="C102" s="53" t="inlineStr">
         <is>
           <t>Ø130x150 printed ASA 12 slots  -  in model as cage</t>
         </is>
       </c>
-      <c r="D51" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="E51" s="52" t="n">
+      <c r="D102" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="E102" s="55" t="n">
         <v>0</v>
       </c>
-      <c r="F51" s="52" t="n">
+      <c r="F102" s="55" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="52" ht="29" customHeight="1">
-      <c r="A52" s="53" t="inlineStr">
+    <row r="103" ht="29" customHeight="1">
+      <c r="A103" s="49" t="inlineStr">
         <is>
           <t>E03</t>
         </is>
       </c>
-      <c r="B52" s="53" t="inlineStr">
+      <c r="B103" s="49" t="inlineStr">
         <is>
           <t>Sensor holders</t>
         </is>
       </c>
-      <c r="C52" s="55" t="inlineStr">
+      <c r="C103" s="6" t="inlineStr">
         <is>
           <t>printed clips for pH/TDS/turbidity/NTC/MS5837  -  in model as sensor bodies</t>
         </is>
       </c>
-      <c r="D52" s="56" t="n">
+      <c r="D103" s="50" t="n">
         <v>5</v>
       </c>
-      <c r="E52" s="57" t="n">
+      <c r="E103" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="F52" s="57" t="n">
+      <c r="F103" s="51" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="54" ht="20" customHeight="1">
-      <c r="A54" s="45" t="inlineStr">
+    <row r="105" ht="20" customHeight="1">
+      <c r="A105" s="45" t="inlineStr">
+        <is>
+          <t>JLCPCB</t>
+        </is>
+      </c>
+      <c r="F105" s="46" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="47" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B106" s="47" t="inlineStr">
+        <is>
+          <t>Part</t>
+        </is>
+      </c>
+      <c r="C106" s="47" t="inlineStr">
+        <is>
+          <t>Specification / note</t>
+        </is>
+      </c>
+      <c r="D106" s="48" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="E106" s="48" t="inlineStr">
+        <is>
+          <t>Unit EUR</t>
+        </is>
+      </c>
+      <c r="F106" s="48" t="inlineStr">
+        <is>
+          <t>Total EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" ht="15.5" customHeight="1">
+      <c r="A107" s="49" t="inlineStr">
+        <is>
+          <t>G14</t>
+        </is>
+      </c>
+      <c r="B107" s="49" t="inlineStr">
+        <is>
+          <t>PCB</t>
+        </is>
+      </c>
+      <c r="C107" s="6" t="inlineStr">
+        <is>
+          <t>custom 2-layer 60x80mm  -  panel of 10 amortises</t>
+        </is>
+      </c>
+      <c r="D107" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E107" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="F107" s="51" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="109" ht="20" customHeight="1">
+      <c r="A109" s="45" t="inlineStr">
         <is>
           <t>NEREZMATERIAL.CZ</t>
         </is>
       </c>
-      <c r="F54" s="46" t="n">
+      <c r="F109" s="46" t="n">
+        <v>2.6</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="47" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B110" s="47" t="inlineStr">
+        <is>
+          <t>Part</t>
+        </is>
+      </c>
+      <c r="C110" s="47" t="inlineStr">
+        <is>
+          <t>Specification / note</t>
+        </is>
+      </c>
+      <c r="D110" s="48" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="E110" s="48" t="inlineStr">
+        <is>
+          <t>Unit EUR</t>
+        </is>
+      </c>
+      <c r="F110" s="48" t="inlineStr">
+        <is>
+          <t>Total EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" ht="42.5" customHeight="1">
+      <c r="A111" s="49" t="inlineStr">
+        <is>
+          <t>A03</t>
+        </is>
+      </c>
+      <c r="B111" s="49" t="inlineStr">
+        <is>
+          <t>Wet shaft</t>
+        </is>
+      </c>
+      <c r="C111" s="6" t="inlineStr">
+        <is>
+          <t>316L Ø5 h6 x 115mm ground; 2 flats each end  -  lokalny zeleziar / Hornbach M5 A4 srob - 4. obchod sa nerata, nema postu; 3m bar 63.1 CZK makes ~26 shafts</t>
+        </is>
+      </c>
+      <c r="D111" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E111" s="51" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="F111" s="51" t="n">
+        <v>2.6</v>
+      </c>
+    </row>
+    <row r="112" ht="29" customHeight="1">
+      <c r="A112" s="52" t="inlineStr">
+        <is>
+          <t>B03</t>
+        </is>
+      </c>
+      <c r="B112" s="52" t="inlineStr">
+        <is>
+          <t>Separation wall</t>
+        </is>
+      </c>
+      <c r="C112" s="53" t="inlineStr">
+        <is>
+          <t>D106 x 4 mm - RECOMMENDED integral with the pod bulkhead (no separate part)  -  4 mm per CAD, not 5; integral removes O-ring C03 and screws C05</t>
+        </is>
+      </c>
+      <c r="D112" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="E112" s="55" t="n">
         <v>0</v>
       </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="47" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B55" s="47" t="inlineStr">
-        <is>
-          <t>Part</t>
-        </is>
-      </c>
-      <c r="C55" s="47" t="inlineStr">
-        <is>
-          <t>Specification / note</t>
-        </is>
-      </c>
-      <c r="D55" s="48" t="inlineStr">
-        <is>
-          <t>Qty</t>
-        </is>
-      </c>
-      <c r="E55" s="48" t="inlineStr">
-        <is>
-          <t>Unit EUR</t>
-        </is>
-      </c>
-      <c r="F55" s="48" t="inlineStr">
-        <is>
-          <t>Total EUR</t>
-        </is>
-      </c>
-    </row>
-    <row r="56" ht="29" customHeight="1">
-      <c r="A56" s="49" t="inlineStr">
-        <is>
-          <t>B03</t>
-        </is>
-      </c>
-      <c r="B56" s="49" t="inlineStr">
-        <is>
-          <t>Separation wall</t>
-        </is>
-      </c>
-      <c r="C56" s="6" t="inlineStr">
-        <is>
-          <t>D106 x 4 mm - RECOMMENDED integral with the pod bulkhead (no separate part)  -  4 mm per CAD, not 5; integral removes O-ring C03 and screws C05</t>
-        </is>
-      </c>
-      <c r="D56" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="E56" s="52" t="n">
+      <c r="F112" s="55" t="n">
         <v>0</v>
       </c>
-      <c r="F56" s="52" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="58" ht="18" customHeight="1">
-      <c r="A58" s="58" t="inlineStr">
+    </row>
+    <row r="114" ht="18" customHeight="1">
+      <c r="A114" s="61" t="inlineStr">
         <is>
           <t>GOODS</t>
         </is>
       </c>
-      <c r="F58" s="59" t="n">
-        <v>220.61</v>
-      </c>
-    </row>
-    <row r="59" ht="18" customHeight="1">
-      <c r="A59" s="58" t="inlineStr">
+      <c r="F114" s="62" t="n">
+        <v>988.11</v>
+      </c>
+    </row>
+    <row r="115" ht="18" customHeight="1">
+      <c r="A115" s="61" t="inlineStr">
         <is>
           <t>shipping, estimated</t>
         </is>
       </c>
-      <c r="F59" s="59" t="n">
+      <c r="F115" s="62" t="n">
         <v>25</v>
       </c>
     </row>
-    <row r="60" ht="22" customHeight="1">
-      <c r="A60" s="60" t="inlineStr">
+    <row r="116" ht="22" customHeight="1">
+      <c r="A116" s="63" t="inlineStr">
         <is>
           <t>LANDED TOTAL</t>
         </is>
       </c>
-      <c r="F60" s="61" t="n">
-        <v>245.61</v>
-      </c>
-    </row>
-    <row r="63" ht="22" customHeight="1">
-      <c r="A63" s="62" t="inlineStr">
+      <c r="F116" s="64" t="n">
+        <v>1013.11</v>
+      </c>
+    </row>
+    <row r="119" ht="22" customHeight="1">
+      <c r="A119" s="65" t="inlineStr">
         <is>
           <t>NOT IN THIS ORDER</t>
         </is>
       </c>
     </row>
-    <row r="64">
-      <c r="A64" s="63" t="inlineStr">
+    <row r="120">
+      <c r="A120" s="66" t="inlineStr">
         <is>
           <t>PHASE 2 - BUY LATER</t>
         </is>
       </c>
     </row>
-    <row r="65" ht="29" customHeight="1">
-      <c r="A65" s="64" t="inlineStr">
-        <is>
-          <t>A03</t>
-        </is>
-      </c>
-      <c r="B65" s="64" t="inlineStr">
-        <is>
-          <t>Wet shaft</t>
-        </is>
-      </c>
-      <c r="C65" s="65" t="inlineStr">
-        <is>
-          <t>lokalny zeleziar / Hornbach M5 A4 srob - 4. obchod sa nerata, nema postu; 3m bar 63.1 CZK makes ~26 shafts</t>
-        </is>
-      </c>
-      <c r="E65" s="66" t="inlineStr">
-        <is>
-          <t>2.6</t>
-        </is>
-      </c>
-    </row>
-    <row r="66" ht="29" customHeight="1">
-      <c r="A66" s="64" t="inlineStr">
-        <is>
-          <t>C08</t>
-        </is>
-      </c>
-      <c r="B66" s="64" t="inlineStr">
-        <is>
-          <t>Generator</t>
-        </is>
-      </c>
-      <c r="C66" s="65" t="inlineStr">
-        <is>
-          <t>TEST BEZ GENERATORA: klietka + senzory stacia, generator je dalsi nakup; XTG3506 preferred: encoder = free RPM/flow</t>
-        </is>
-      </c>
-      <c r="E66" s="66" t="inlineStr">
-        <is>
-          <t>26.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="67" ht="15.5" customHeight="1">
-      <c r="A67" s="64" t="inlineStr">
-        <is>
-          <t>D01</t>
-        </is>
-      </c>
-      <c r="B67" s="64" t="inlineStr">
-        <is>
-          <t>pH electrode</t>
-        </is>
-      </c>
-      <c r="C67" s="65" t="inlineStr">
-        <is>
-          <t>OPTIONAL per site; 14-30 day service; +-0.1 pH after 2-pt cal</t>
-        </is>
-      </c>
-      <c r="E67" s="66" t="inlineStr">
-        <is>
-          <t>39.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="68" ht="15.5" customHeight="1">
-      <c r="A68" s="64" t="inlineStr">
-        <is>
-          <t>D02</t>
-        </is>
-      </c>
-      <c r="B68" s="64" t="inlineStr">
-        <is>
-          <t>pH spare electrode</t>
-        </is>
-      </c>
-      <c r="C68" s="65" t="inlineStr">
-        <is>
-          <t>consumable</t>
-        </is>
-      </c>
-      <c r="E68" s="66" t="inlineStr">
-        <is>
-          <t>9.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="69" ht="15.5" customHeight="1">
-      <c r="A69" s="64" t="inlineStr">
-        <is>
-          <t>D03</t>
-        </is>
-      </c>
-      <c r="B69" s="64" t="inlineStr">
-        <is>
-          <t>pH buffer</t>
-        </is>
-      </c>
-      <c r="C69" s="65" t="inlineStr">
-        <is>
-          <t>consumable</t>
-        </is>
-      </c>
-      <c r="E69" s="66" t="inlineStr">
-        <is>
-          <t>12.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="70" ht="29" customHeight="1">
-      <c r="A70" s="64" t="inlineStr">
-        <is>
-          <t>D09</t>
-        </is>
-      </c>
-      <c r="B70" s="64" t="inlineStr">
-        <is>
-          <t>Dissolved oxygen kit</t>
-        </is>
-      </c>
-      <c r="C70" s="65" t="inlineStr">
-        <is>
-          <t>HIGHEST-VALUE channel (Budca = hypoxia); membrane 1-2 months in muddy water; 0.5M NaOH filling solution NOT shipped by air - source locally</t>
-        </is>
-      </c>
-      <c r="E70" s="66" t="inlineStr">
-        <is>
-          <t>175.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="71" ht="15.5" customHeight="1">
-      <c r="A71" s="64" t="inlineStr">
-        <is>
-          <t>D05</t>
-        </is>
-      </c>
-      <c r="B71" s="64" t="inlineStr">
-        <is>
-          <t>Level / stage probe</t>
-        </is>
-      </c>
-      <c r="C71" s="65" t="inlineStr">
-        <is>
-          <t>MS5837-30BA REJECTED: gel element must be dried daily, 24h max submersion</t>
-        </is>
-      </c>
-      <c r="E71" s="66" t="inlineStr">
-        <is>
-          <t>110.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="72" ht="15.5" customHeight="1">
-      <c r="A72" s="64" t="inlineStr">
-        <is>
-          <t>D06</t>
-        </is>
-      </c>
-      <c r="B72" s="64" t="inlineStr">
-        <is>
-          <t>EC/TDS</t>
-        </is>
-      </c>
-      <c r="C72" s="65" t="inlineStr">
-        <is>
-          <t>+-10% FS is the weakest sensor; use as trend indicator, site-calibrate</t>
-        </is>
-      </c>
-      <c r="E72" s="66" t="inlineStr">
-        <is>
-          <t>14.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="73" ht="15.5" customHeight="1">
-      <c r="A73" s="64" t="inlineStr">
-        <is>
-          <t>D08</t>
-        </is>
-      </c>
-      <c r="B73" s="64" t="inlineStr">
-        <is>
-          <t>Sensor cable</t>
-        </is>
-      </c>
-      <c r="C73" s="65" t="inlineStr"/>
-      <c r="E73" s="66" t="inlineStr">
-        <is>
-          <t>20.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="74" ht="15.5" customHeight="1">
-      <c r="A74" s="64" t="inlineStr">
-        <is>
-          <t>G04</t>
-        </is>
-      </c>
-      <c r="B74" s="64" t="inlineStr">
-        <is>
-          <t>Antenna probe</t>
-        </is>
-      </c>
-      <c r="C74" s="65" t="inlineStr">
-        <is>
-          <t>v baleni kazdej Wio-E5 je EU868 antena - samostatne netreba; drzat ako zalohu</t>
-        </is>
-      </c>
-      <c r="E74" s="66" t="inlineStr">
-        <is>
-          <t>6.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="75" ht="15.5" customHeight="1">
-      <c r="A75" s="64" t="inlineStr">
-        <is>
-          <t>G06</t>
-        </is>
-      </c>
-      <c r="B75" s="64" t="inlineStr">
-        <is>
-          <t>Boost harvester</t>
-        </is>
-      </c>
-      <c r="C75" s="65" t="inlineStr">
-        <is>
-          <t>needed when EMF below bus</t>
-        </is>
-      </c>
-      <c r="E75" s="66" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="76" ht="15.5" customHeight="1">
-      <c r="A76" s="64" t="inlineStr">
-        <is>
-          <t>G07</t>
-        </is>
-      </c>
-      <c r="B76" s="64" t="inlineStr">
-        <is>
-          <t>Buck</t>
-        </is>
-      </c>
-      <c r="C76" s="65" t="inlineStr"/>
-      <c r="E76" s="66" t="inlineStr">
-        <is>
-          <t>2.5</t>
-        </is>
-      </c>
-    </row>
-    <row r="77" ht="15.5" customHeight="1">
-      <c r="A77" s="64" t="inlineStr">
-        <is>
-          <t>G08</t>
-        </is>
-      </c>
-      <c r="B77" s="64" t="inlineStr">
-        <is>
-          <t>Rectifier</t>
-        </is>
-      </c>
-      <c r="C77" s="65" t="inlineStr">
-        <is>
-          <t>452k in stock</t>
-        </is>
-      </c>
-      <c r="E77" s="66" t="inlineStr">
-        <is>
-          <t>0.15</t>
-        </is>
-      </c>
-    </row>
-    <row r="78" ht="15.5" customHeight="1">
-      <c r="A78" s="64" t="inlineStr">
-        <is>
-          <t>G09</t>
-        </is>
-      </c>
-      <c r="B78" s="64" t="inlineStr">
-        <is>
-          <t>Clamp</t>
-        </is>
-      </c>
-      <c r="C78" s="65" t="inlineStr">
-        <is>
-          <t>overvoltage protection</t>
-        </is>
-      </c>
-      <c r="E78" s="66" t="inlineStr">
-        <is>
-          <t>4.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="79" ht="15.5" customHeight="1">
-      <c r="A79" s="64" t="inlineStr">
-        <is>
-          <t>G10</t>
-        </is>
-      </c>
-      <c r="B79" s="64" t="inlineStr">
-        <is>
-          <t>Supercap</t>
-        </is>
-      </c>
-      <c r="C79" s="65" t="inlineStr">
-        <is>
-          <t>NO coin-cell EDLC (50ohm ESR kills TX)</t>
-        </is>
-      </c>
-      <c r="E79" s="66" t="inlineStr">
-        <is>
-          <t>11.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="80" ht="15.5" customHeight="1">
-      <c r="A80" s="64" t="inlineStr">
-        <is>
-          <t>G11</t>
-        </is>
-      </c>
-      <c r="B80" s="64" t="inlineStr">
-        <is>
-          <t>Voltage supervisor</t>
-        </is>
-      </c>
-      <c r="C80" s="65" t="inlineStr">
-        <is>
-          <t>gates buck at 4.8V</t>
-        </is>
-      </c>
-      <c r="E80" s="66" t="inlineStr">
-        <is>
-          <t>1.5</t>
-        </is>
-      </c>
-    </row>
-    <row r="81" ht="15.5" customHeight="1">
-      <c r="A81" s="64" t="inlineStr">
-        <is>
-          <t>G12</t>
-        </is>
-      </c>
-      <c r="B81" s="64" t="inlineStr">
-        <is>
-          <t>Load switch</t>
-        </is>
-      </c>
-      <c r="C81" s="65" t="inlineStr">
-        <is>
-          <t>removes ground-loop need</t>
-        </is>
-      </c>
-      <c r="E81" s="66" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="82" ht="15.5" customHeight="1">
-      <c r="A82" s="64" t="inlineStr">
-        <is>
-          <t>G13</t>
-        </is>
-      </c>
-      <c r="B82" s="64" t="inlineStr">
-        <is>
-          <t>Barometer</t>
-        </is>
-      </c>
-      <c r="C82" s="65" t="inlineStr">
-        <is>
-          <t>pressure reference for MS5837</t>
-        </is>
-      </c>
-      <c r="E82" s="66" t="inlineStr">
-        <is>
-          <t>6.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="83" ht="15.5" customHeight="1">
-      <c r="A83" s="64" t="inlineStr">
-        <is>
-          <t>G14</t>
-        </is>
-      </c>
-      <c r="B83" s="64" t="inlineStr">
-        <is>
-          <t>PCB</t>
-        </is>
-      </c>
-      <c r="C83" s="65" t="inlineStr">
-        <is>
-          <t>panel of 10 amortises</t>
-        </is>
-      </c>
-      <c r="E83" s="66" t="inlineStr">
-        <is>
-          <t>3.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="84" ht="15.5" customHeight="1">
-      <c r="A84" s="64" t="inlineStr">
-        <is>
-          <t>G15</t>
-        </is>
-      </c>
-      <c r="B84" s="64" t="inlineStr">
-        <is>
-          <t>Connectors</t>
-        </is>
-      </c>
-      <c r="C84" s="65" t="inlineStr"/>
-      <c r="E84" s="66" t="inlineStr">
-        <is>
-          <t>10.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="85" ht="15.5" customHeight="1">
-      <c r="A85" s="64" t="inlineStr">
-        <is>
-          <t>H01</t>
-        </is>
-      </c>
-      <c r="B85" s="64" t="inlineStr">
-        <is>
-          <t>Ground screw anchor</t>
-        </is>
-      </c>
-      <c r="C85" s="65" t="inlineStr">
-        <is>
-          <t>1-2kN lateral - covers flood case</t>
-        </is>
-      </c>
-      <c r="E85" s="66" t="inlineStr">
-        <is>
-          <t>25.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="86" ht="15.5" customHeight="1">
-      <c r="A86" s="64" t="inlineStr">
-        <is>
-          <t>H02</t>
-        </is>
-      </c>
-      <c r="B86" s="64" t="inlineStr">
-        <is>
-          <t>Pole</t>
-        </is>
-      </c>
-      <c r="C86" s="65" t="inlineStr">
-        <is>
-          <t>removable mast pinned into receiver</t>
-        </is>
-      </c>
-      <c r="E86" s="66" t="inlineStr">
-        <is>
-          <t>18.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="87" ht="15.5" customHeight="1">
-      <c r="A87" s="64" t="inlineStr">
-        <is>
-          <t>H03</t>
-        </is>
-      </c>
-      <c r="B87" s="64" t="inlineStr">
-        <is>
-          <t>Receiver sleeve</t>
-        </is>
-      </c>
-      <c r="C87" s="65" t="inlineStr">
-        <is>
-          <t>pinned mast interface</t>
-        </is>
-      </c>
-      <c r="E87" s="66" t="inlineStr">
-        <is>
-          <t>8.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="88" ht="15.5" customHeight="1">
-      <c r="A88" s="64" t="inlineStr">
-        <is>
-          <t>H04</t>
-        </is>
-      </c>
-      <c r="B88" s="64" t="inlineStr">
-        <is>
-          <t>Arm tube</t>
-        </is>
-      </c>
-      <c r="C88" s="65" t="inlineStr"/>
-      <c r="E88" s="66" t="inlineStr">
-        <is>
-          <t>9.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="89" ht="15.5" customHeight="1">
-      <c r="A89" s="64" t="inlineStr">
-        <is>
-          <t>H05</t>
-        </is>
-      </c>
-      <c r="B89" s="64" t="inlineStr">
-        <is>
-          <t>Drop tube</t>
-        </is>
-      </c>
-      <c r="C89" s="65" t="inlineStr"/>
-      <c r="E89" s="66" t="inlineStr">
-        <is>
-          <t>6.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="90" ht="15.5" customHeight="1">
-      <c r="A90" s="64" t="inlineStr">
-        <is>
-          <t>H06</t>
-        </is>
-      </c>
-      <c r="B90" s="64" t="inlineStr">
-        <is>
-          <t>Hinge collar</t>
-        </is>
-      </c>
-      <c r="C90" s="65" t="inlineStr"/>
-      <c r="E90" s="66" t="inlineStr">
-        <is>
-          <t>3.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="91" ht="15.5" customHeight="1">
-      <c r="A91" s="64" t="inlineStr">
-        <is>
-          <t>H07</t>
-        </is>
-      </c>
-      <c r="B91" s="64" t="inlineStr">
-        <is>
-          <t>Shear pin</t>
-        </is>
-      </c>
-      <c r="C91" s="65" t="inlineStr">
-        <is>
-          <t>releases pod on &gt;150N debris hit</t>
-        </is>
-      </c>
-      <c r="E91" s="66" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="92" ht="15.5" customHeight="1">
-      <c r="A92" s="64" t="inlineStr">
-        <is>
-          <t>H08</t>
-        </is>
-      </c>
-      <c r="B92" s="64" t="inlineStr">
-        <is>
-          <t>Yaw strut</t>
-        </is>
-      </c>
-      <c r="C92" s="65" t="inlineStr">
-        <is>
-          <t>anti-flutter</t>
-        </is>
-      </c>
-      <c r="E92" s="66" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="93" ht="15.5" customHeight="1">
-      <c r="A93" s="64" t="inlineStr">
-        <is>
-          <t>H09</t>
-        </is>
-      </c>
-      <c r="B93" s="64" t="inlineStr">
-        <is>
-          <t>Guy line</t>
-        </is>
-      </c>
-      <c r="C93" s="65" t="inlineStr">
-        <is>
-          <t>45deg up/downstream</t>
-        </is>
-      </c>
-      <c r="E93" s="66" t="inlineStr">
-        <is>
-          <t>9.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="94" ht="15.5" customHeight="1">
-      <c r="A94" s="64" t="inlineStr">
-        <is>
-          <t>H10</t>
-        </is>
-      </c>
-      <c r="B94" s="64" t="inlineStr">
-        <is>
-          <t>Guy anchor</t>
-        </is>
-      </c>
-      <c r="C94" s="65" t="inlineStr"/>
-      <c r="E94" s="66" t="inlineStr">
-        <is>
-          <t>10.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="95" ht="15.5" customHeight="1">
-      <c r="A95" s="64" t="inlineStr">
-        <is>
-          <t>H11</t>
-        </is>
-      </c>
-      <c r="B95" s="64" t="inlineStr">
-        <is>
-          <t>Safety cable</t>
-        </is>
-      </c>
-      <c r="C95" s="65" t="inlineStr">
-        <is>
-          <t>theft/flood retention</t>
-        </is>
-      </c>
-      <c r="E95" s="66" t="inlineStr">
-        <is>
-          <t>4.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="96" ht="15.5" customHeight="1">
-      <c r="A96" s="64" t="inlineStr">
-        <is>
-          <t>H12</t>
-        </is>
-      </c>
-      <c r="B96" s="64" t="inlineStr">
-        <is>
-          <t>Security fastener</t>
-        </is>
-      </c>
-      <c r="C96" s="65" t="inlineStr">
-        <is>
-          <t>anti-theft</t>
-        </is>
-      </c>
-      <c r="E96" s="66" t="inlineStr">
-        <is>
-          <t>4.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="97" ht="15.5" customHeight="1">
-      <c r="A97" s="64" t="inlineStr">
-        <is>
-          <t>H13</t>
-        </is>
-      </c>
-      <c r="B97" s="64" t="inlineStr">
-        <is>
-          <t>Site label</t>
-        </is>
-      </c>
-      <c r="C97" s="65" t="inlineStr">
-        <is>
-          <t>anti-theft by making it unsellable</t>
-        </is>
-      </c>
-      <c r="E97" s="66" t="inlineStr">
-        <is>
-          <t>3.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="98" ht="15.5" customHeight="1">
-      <c r="A98" s="64" t="inlineStr">
-        <is>
-          <t>I02</t>
-        </is>
-      </c>
-      <c r="B98" s="64" t="inlineStr">
-        <is>
-          <t>Compute</t>
-        </is>
-      </c>
-      <c r="C98" s="65" t="inlineStr">
-        <is>
-          <t>YOU ALREADY HAVE THIS - reuse, zero soldering; runs the gateway service</t>
-        </is>
-      </c>
-      <c r="E98" s="66" t="inlineStr">
-        <is>
-          <t>70.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="99" ht="15.5" customHeight="1">
-      <c r="A99" s="64" t="inlineStr">
-        <is>
-          <t>I03</t>
-        </is>
-      </c>
-      <c r="B99" s="64" t="inlineStr">
-        <is>
-          <t>Antenna</t>
-        </is>
-      </c>
-      <c r="C99" s="65" t="inlineStr">
-        <is>
-          <t>range-critical: gateway antenna gain + mast height set the link</t>
-        </is>
-      </c>
-      <c r="E99" s="66" t="inlineStr">
-        <is>
-          <t>45.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="100" ht="15.5" customHeight="1">
-      <c r="A100" s="64" t="inlineStr">
+    <row r="121" ht="15.5" customHeight="1">
+      <c r="A121" s="67" t="inlineStr">
+        <is>
+          <t>G01</t>
+        </is>
+      </c>
+      <c r="B121" s="67" t="inlineStr">
+        <is>
+          <t>Enclosure</t>
+        </is>
+      </c>
+      <c r="C121" s="68" t="inlineStr">
+        <is>
+          <t>vynechane: vodotesna krabica na brehu - nie je sucastou stavby | in model as site_box</t>
+        </is>
+      </c>
+      <c r="E121" s="69" t="inlineStr">
+        <is>
+          <t>22.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="122" ht="15.5" customHeight="1">
+      <c r="A122" s="67" t="inlineStr">
         <is>
           <t>I04</t>
         </is>
       </c>
-      <c r="B100" s="64" t="inlineStr">
+      <c r="B122" s="67" t="inlineStr">
         <is>
           <t>Enclosure</t>
         </is>
       </c>
-      <c r="C100" s="65" t="inlineStr"/>
-      <c r="E100" s="66" t="inlineStr">
+      <c r="C122" s="68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vynechane: krabica pre gateway na stozieri | </t>
+        </is>
+      </c>
+      <c r="E122" s="69" t="inlineStr">
         <is>
           <t>35.0</t>
         </is>
       </c>
     </row>
-    <row r="101" ht="15.5" customHeight="1">
-      <c r="A101" s="64" t="inlineStr">
-        <is>
-          <t>I05</t>
-        </is>
-      </c>
-      <c r="B101" s="64" t="inlineStr">
-        <is>
-          <t>Mast</t>
-        </is>
-      </c>
-      <c r="C101" s="65" t="inlineStr">
-        <is>
-          <t>height sets range</t>
-        </is>
-      </c>
-      <c r="E101" s="66" t="inlineStr">
-        <is>
-          <t>30.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="102" ht="15.5" customHeight="1">
-      <c r="A102" s="64" t="inlineStr">
+    <row r="123" ht="15.5" customHeight="1">
+      <c r="A123" s="67" t="inlineStr">
         <is>
           <t>I06</t>
         </is>
       </c>
-      <c r="B102" s="64" t="inlineStr">
+      <c r="B123" s="67" t="inlineStr">
         <is>
           <t>Concentrator upgrade (optional)</t>
         </is>
       </c>
-      <c r="C102" s="65" t="inlineStr">
+      <c r="C123" s="68" t="inlineStr">
         <is>
           <t>Only for multi-SF / multi-channel / public TTN. Single-channel Wio-E5 gateway is enough for our 20 nodes.</t>
         </is>
       </c>
-      <c r="E102" s="66" t="inlineStr">
+      <c r="E123" s="69" t="inlineStr">
         <is>
           <t>145.0</t>
         </is>
       </c>
     </row>
-    <row r="103" ht="15.5" customHeight="1">
-      <c r="A103" s="64" t="inlineStr">
-        <is>
-          <t>J01</t>
-        </is>
-      </c>
-      <c r="B103" s="64" t="inlineStr">
-        <is>
-          <t>Filament ASA</t>
-        </is>
-      </c>
-      <c r="C103" s="65" t="inlineStr">
-        <is>
-          <t>ABS z domaceho spoolu, nie ASA; UV je len na brehu</t>
-        </is>
-      </c>
-      <c r="E103" s="66" t="inlineStr">
-        <is>
-          <t>32.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="104" ht="15.5" customHeight="1">
-      <c r="A104" s="64" t="inlineStr">
-        <is>
-          <t>J02</t>
-        </is>
-      </c>
-      <c r="B104" s="64" t="inlineStr">
-        <is>
-          <t>Filament PC Blend</t>
-        </is>
-      </c>
-      <c r="C104" s="65" t="inlineStr"/>
-      <c r="E104" s="66" t="inlineStr">
+    <row r="124" ht="15.5" customHeight="1">
+      <c r="A124" s="67" t="inlineStr">
+        <is>
+          <t>K01</t>
+        </is>
+      </c>
+      <c r="B124" s="67" t="inlineStr">
+        <is>
+          <t>Vacuum chamber</t>
+        </is>
+      </c>
+      <c r="C124" s="68" t="inlineStr">
+        <is>
+          <t>nastroj, nie suciastka - pozicat alebo kupit neskor | acceptance test rig (one-off)</t>
+        </is>
+      </c>
+      <c r="E124" s="69" t="inlineStr">
+        <is>
+          <t>85.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="125" ht="15.5" customHeight="1">
+      <c r="A125" s="67" t="inlineStr">
+        <is>
+          <t>K02</t>
+        </is>
+      </c>
+      <c r="B125" s="67" t="inlineStr">
+        <is>
+          <t>Torque driver</t>
+        </is>
+      </c>
+      <c r="C125" s="68" t="inlineStr">
+        <is>
+          <t>nastroj, nie diel | one-off</t>
+        </is>
+      </c>
+      <c r="E125" s="69" t="inlineStr">
         <is>
           <t>40.0</t>
         </is>
       </c>
     </row>
-    <row r="105" ht="15.5" customHeight="1">
-      <c r="A105" s="64" t="inlineStr">
-        <is>
-          <t>J04</t>
-        </is>
-      </c>
-      <c r="B105" s="64" t="inlineStr">
-        <is>
-          <t>Conformal coat</t>
-        </is>
-      </c>
-      <c r="C105" s="65" t="inlineStr"/>
-      <c r="E105" s="66" t="inlineStr">
-        <is>
-          <t>14.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="106" ht="15.5" customHeight="1">
-      <c r="A106" s="64" t="inlineStr">
-        <is>
-          <t>J05</t>
-        </is>
-      </c>
-      <c r="B106" s="64" t="inlineStr">
-        <is>
-          <t>Silicone grease</t>
-        </is>
-      </c>
-      <c r="C106" s="65" t="inlineStr">
-        <is>
-          <t>MAM - doma</t>
-        </is>
-      </c>
-      <c r="E106" s="66" t="inlineStr">
-        <is>
-          <t>9.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="107" ht="15.5" customHeight="1">
-      <c r="A107" s="64" t="inlineStr">
-        <is>
-          <t>J06</t>
-        </is>
-      </c>
-      <c r="B107" s="64" t="inlineStr">
-        <is>
-          <t>Threadlocker</t>
-        </is>
-      </c>
-      <c r="C107" s="65" t="inlineStr"/>
-      <c r="E107" s="66" t="inlineStr">
-        <is>
-          <t>11.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="108" ht="15.5" customHeight="1">
-      <c r="A108" s="64" t="inlineStr">
-        <is>
-          <t>J08</t>
-        </is>
-      </c>
-      <c r="B108" s="64" t="inlineStr">
-        <is>
-          <t>O-ring kit</t>
-        </is>
-      </c>
-      <c r="C108" s="65" t="inlineStr"/>
-      <c r="E108" s="66" t="inlineStr">
-        <is>
-          <t>12.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="109" ht="15.5" customHeight="1">
-      <c r="A109" s="64" t="inlineStr">
-        <is>
-          <t>K01</t>
-        </is>
-      </c>
-      <c r="B109" s="64" t="inlineStr">
-        <is>
-          <t>Vacuum chamber</t>
-        </is>
-      </c>
-      <c r="C109" s="65" t="inlineStr">
-        <is>
-          <t>acceptance test rig (one-off)</t>
-        </is>
-      </c>
-      <c r="E109" s="66" t="inlineStr">
-        <is>
-          <t>85.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="110" ht="15.5" customHeight="1">
-      <c r="A110" s="64" t="inlineStr">
-        <is>
-          <t>K02</t>
-        </is>
-      </c>
-      <c r="B110" s="64" t="inlineStr">
-        <is>
-          <t>Torque driver</t>
-        </is>
-      </c>
-      <c r="C110" s="65" t="inlineStr">
-        <is>
-          <t>one-off</t>
-        </is>
-      </c>
-      <c r="E110" s="66" t="inlineStr">
-        <is>
-          <t>40.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="112">
-      <c r="A112" s="67" t="inlineStr">
+    <row r="127">
+      <c r="A127" s="70" t="inlineStr">
         <is>
           <t>CUT - DEAD LINE, DO NOT BUY</t>
         </is>
       </c>
     </row>
-    <row r="113" ht="15.5" customHeight="1">
-      <c r="A113" s="64" t="inlineStr">
+    <row r="128" ht="15.5" customHeight="1">
+      <c r="A128" s="67" t="inlineStr">
         <is>
           <t>A05</t>
         </is>
       </c>
-      <c r="B113" s="64" t="inlineStr">
+      <c r="B128" s="67" t="inlineStr">
         <is>
           <t>Bearing carrier tube</t>
         </is>
       </c>
-      <c r="C113" s="65" t="inlineStr">
+      <c r="C128" s="68" t="inlineStr">
         <is>
           <t>CUT: superseded - the bearing carrier is the printed spider (wet_carrier)</t>
         </is>
       </c>
-      <c r="E113" s="68" t="inlineStr">
+      <c r="E128" s="71" t="inlineStr">
         <is>
           <t>1.2</t>
         </is>
       </c>
     </row>
-    <row r="114" ht="15.5" customHeight="1">
-      <c r="A114" s="64" t="inlineStr">
+    <row r="129" ht="15.5" customHeight="1">
+      <c r="A129" s="67" t="inlineStr">
         <is>
           <t>A07</t>
         </is>
       </c>
-      <c r="B114" s="64" t="inlineStr">
+      <c r="B129" s="67" t="inlineStr">
         <is>
           <t>Weed guard ring</t>
         </is>
       </c>
-      <c r="C114" s="65" t="inlineStr">
+      <c r="C129" s="68" t="inlineStr">
         <is>
           <t>CUT: killed by design - replaced by the nose cone D64-&gt;D12; a ring on struts upstream is an algae scythe</t>
         </is>
       </c>
-      <c r="E114" s="68" t="inlineStr">
+      <c r="E129" s="71" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
-    <row r="115" ht="15.5" customHeight="1">
-      <c r="A115" s="64" t="inlineStr">
+    <row r="130" ht="15.5" customHeight="1">
+      <c r="A130" s="67" t="inlineStr">
         <is>
           <t>A08</t>
         </is>
       </c>
-      <c r="B115" s="64" t="inlineStr">
+      <c r="B130" s="67" t="inlineStr">
         <is>
           <t>Blade safety retainer</t>
         </is>
       </c>
-      <c r="C115" s="65" t="inlineStr">
+      <c r="C130" s="68" t="inlineStr">
         <is>
           <t>CUT: killed by design - a tether on a 110 mm blade is a flail, and the hole is a stress riser at the root</t>
         </is>
       </c>
-      <c r="E115" s="68" t="inlineStr">
+      <c r="E130" s="71" t="inlineStr">
         <is>
           <t>2.0</t>
         </is>
       </c>
     </row>
-    <row r="116" ht="15.5" customHeight="1">
-      <c r="A116" s="64" t="inlineStr">
+    <row r="131" ht="15.5" customHeight="1">
+      <c r="A131" s="67" t="inlineStr">
         <is>
           <t>G02</t>
         </is>
       </c>
-      <c r="B116" s="64" t="inlineStr">
+      <c r="B131" s="67" t="inlineStr">
         <is>
           <t>MCU (NOT USED in simple build)</t>
         </is>
       </c>
-      <c r="C116" s="65" t="inlineStr">
+      <c r="C131" s="68" t="inlineStr">
         <is>
           <t>DROPPED: Wio-E5 mini is the single brain (MCU+LoRa). Bring back only if we need more GPIO/dual-core.</t>
         </is>
       </c>
-      <c r="E116" s="68" t="inlineStr">
+      <c r="E131" s="71" t="inlineStr">
         <is>
           <t>0.0</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="14">
-    <mergeCell ref="A21:E21"/>
+  <mergeCells count="19">
+    <mergeCell ref="A114:E114"/>
+    <mergeCell ref="A3:F3"/>
+    <mergeCell ref="A70:E70"/>
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A39:E39"/>
-    <mergeCell ref="A63:F63"/>
-    <mergeCell ref="A59:E59"/>
-    <mergeCell ref="A43:E43"/>
-    <mergeCell ref="A54:E54"/>
+    <mergeCell ref="A75:E75"/>
+    <mergeCell ref="A84:E84"/>
+    <mergeCell ref="A89:E89"/>
+    <mergeCell ref="A66:E66"/>
+    <mergeCell ref="A80:E80"/>
+    <mergeCell ref="A105:E105"/>
+    <mergeCell ref="A55:E55"/>
+    <mergeCell ref="A116:E116"/>
+    <mergeCell ref="A5:E5"/>
+    <mergeCell ref="A23:E23"/>
+    <mergeCell ref="A109:E109"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A28:E28"/>
-    <mergeCell ref="A60:E60"/>
-    <mergeCell ref="A33:E33"/>
-    <mergeCell ref="A5:E5"/>
-    <mergeCell ref="A3:F3"/>
-    <mergeCell ref="A58:E58"/>
+    <mergeCell ref="A119:F119"/>
+    <mergeCell ref="A115:E115"/>
+    <mergeCell ref="A93:E93"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B9" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B10" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B12" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B13" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B14" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B15" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B16" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B17" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B18" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B19" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B24" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B25" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B26" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B30" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B31" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B41" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B25" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B29" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B30" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B34" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B36" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B37" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B38" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B39" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B44" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B45" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B47" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B48" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B60" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B61" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B63" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B77" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B78" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B91" r:id="rId18"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
@@ -3670,10 +4105,10 @@
           <t>subtotal - Rotor &amp; drivetrain (wet side)</t>
         </is>
       </c>
-      <c r="B14" s="69" t="n"/>
-      <c r="C14" s="69" t="n"/>
-      <c r="D14" s="69" t="n"/>
-      <c r="E14" s="70" t="n"/>
+      <c r="B14" s="72" t="n"/>
+      <c r="C14" s="72" t="n"/>
+      <c r="D14" s="72" t="n"/>
+      <c r="E14" s="73" t="n"/>
       <c r="F14" s="15" t="n"/>
       <c r="G14" s="15" t="n">
         <v>8.16</v>
@@ -3921,10 +4356,10 @@
           <t>subtotal - Magnetic coupling</t>
         </is>
       </c>
-      <c r="B21" s="69" t="n"/>
-      <c r="C21" s="69" t="n"/>
-      <c r="D21" s="69" t="n"/>
-      <c r="E21" s="70" t="n"/>
+      <c r="B21" s="72" t="n"/>
+      <c r="C21" s="72" t="n"/>
+      <c r="D21" s="72" t="n"/>
+      <c r="E21" s="73" t="n"/>
       <c r="F21" s="15" t="n"/>
       <c r="G21" s="15" t="n">
         <v>22.8</v>
@@ -4444,10 +4879,10 @@
           <t>subtotal - Generator pod &amp; sealing</t>
         </is>
       </c>
-      <c r="B33" s="69" t="n"/>
-      <c r="C33" s="69" t="n"/>
-      <c r="D33" s="69" t="n"/>
-      <c r="E33" s="70" t="n"/>
+      <c r="B33" s="72" t="n"/>
+      <c r="C33" s="72" t="n"/>
+      <c r="D33" s="72" t="n"/>
+      <c r="E33" s="73" t="n"/>
       <c r="F33" s="15" t="n"/>
       <c r="G33" s="15" t="n">
         <v>49</v>
@@ -4971,10 +5406,10 @@
           <t>subtotal - Sensors</t>
         </is>
       </c>
-      <c r="B45" s="69" t="n"/>
-      <c r="C45" s="69" t="n"/>
-      <c r="D45" s="69" t="n"/>
-      <c r="E45" s="70" t="n"/>
+      <c r="B45" s="72" t="n"/>
+      <c r="C45" s="72" t="n"/>
+      <c r="D45" s="72" t="n"/>
+      <c r="E45" s="73" t="n"/>
       <c r="F45" s="15" t="n"/>
       <c r="G45" s="15" t="n">
         <v>405.45</v>
@@ -5162,10 +5597,10 @@
           <t>subtotal - Sensor cage &amp; mounting</t>
         </is>
       </c>
-      <c r="B51" s="69" t="n"/>
-      <c r="C51" s="69" t="n"/>
-      <c r="D51" s="69" t="n"/>
-      <c r="E51" s="70" t="n"/>
+      <c r="B51" s="72" t="n"/>
+      <c r="C51" s="72" t="n"/>
+      <c r="D51" s="72" t="n"/>
+      <c r="E51" s="73" t="n"/>
       <c r="F51" s="15" t="n"/>
       <c r="G51" s="15" t="n">
         <v>6</v>
@@ -5297,10 +5732,10 @@
           <t>subtotal - Wet-dry interface (cable)</t>
         </is>
       </c>
-      <c r="B56" s="69" t="n"/>
-      <c r="C56" s="69" t="n"/>
-      <c r="D56" s="69" t="n"/>
-      <c r="E56" s="70" t="n"/>
+      <c r="B56" s="72" t="n"/>
+      <c r="C56" s="72" t="n"/>
+      <c r="D56" s="72" t="n"/>
+      <c r="E56" s="73" t="n"/>
       <c r="F56" s="15" t="n"/>
       <c r="G56" s="15" t="n">
         <v>47</v>
@@ -5370,7 +5805,7 @@
       </c>
       <c r="L59" s="6" t="inlineStr">
         <is>
-          <t>ready-made IP68 box, do not print | in model as site_box</t>
+          <t>ready-made IP68 box, do not print | vynechane: vodotesna krabica na brehu - nie je sucastou stavby | in model as site_box</t>
         </is>
       </c>
     </row>
@@ -6268,10 +6703,10 @@
           <t>subtotal - Electronics (dry box)</t>
         </is>
       </c>
-      <c r="B76" s="69" t="n"/>
-      <c r="C76" s="69" t="n"/>
-      <c r="D76" s="69" t="n"/>
-      <c r="E76" s="70" t="n"/>
+      <c r="B76" s="72" t="n"/>
+      <c r="C76" s="72" t="n"/>
+      <c r="D76" s="72" t="n"/>
+      <c r="E76" s="73" t="n"/>
       <c r="F76" s="15" t="n"/>
       <c r="G76" s="15" t="n">
         <v>102.9</v>
@@ -7007,10 +7442,10 @@
           <t>subtotal - Structure &amp; site</t>
         </is>
       </c>
-      <c r="B92" s="69" t="n"/>
-      <c r="C92" s="69" t="n"/>
-      <c r="D92" s="69" t="n"/>
-      <c r="E92" s="70" t="n"/>
+      <c r="B92" s="72" t="n"/>
+      <c r="C92" s="72" t="n"/>
+      <c r="D92" s="72" t="n"/>
+      <c r="E92" s="73" t="n"/>
       <c r="F92" s="15" t="n"/>
       <c r="G92" s="15" t="n">
         <v>105</v>
@@ -7246,7 +7681,11 @@
           <t>verified</t>
         </is>
       </c>
-      <c r="L98" s="17" t="inlineStr"/>
+      <c r="L98" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vynechane: krabica pre gateway na stozieri | </t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="16" t="inlineStr">
@@ -7366,10 +7805,10 @@
           <t>subtotal - Gateway (base station)</t>
         </is>
       </c>
-      <c r="B101" s="69" t="n"/>
-      <c r="C101" s="69" t="n"/>
-      <c r="D101" s="69" t="n"/>
-      <c r="E101" s="70" t="n"/>
+      <c r="B101" s="72" t="n"/>
+      <c r="C101" s="72" t="n"/>
+      <c r="D101" s="72" t="n"/>
+      <c r="E101" s="73" t="n"/>
       <c r="F101" s="15" t="n"/>
       <c r="G101" s="15" t="n">
         <v>339</v>
@@ -7817,10 +8256,10 @@
           <t>subtotal - Consumables</t>
         </is>
       </c>
-      <c r="B112" s="69" t="n"/>
-      <c r="C112" s="69" t="n"/>
-      <c r="D112" s="69" t="n"/>
-      <c r="E112" s="70" t="n"/>
+      <c r="B112" s="72" t="n"/>
+      <c r="C112" s="72" t="n"/>
+      <c r="D112" s="72" t="n"/>
+      <c r="E112" s="73" t="n"/>
       <c r="F112" s="15" t="n"/>
       <c r="G112" s="15" t="n">
         <v>142</v>
@@ -7890,7 +8329,7 @@
       </c>
       <c r="L115" s="17" t="inlineStr">
         <is>
-          <t>acceptance test rig; borrow if possible | acceptance test rig (one-off)</t>
+          <t>acceptance test rig; borrow if possible | nastroj, nie suciastka - pozicat alebo kupit neskor | acceptance test rig (one-off)</t>
         </is>
       </c>
     </row>
@@ -7946,7 +8385,7 @@
       </c>
       <c r="L116" s="17" t="inlineStr">
         <is>
-          <t>one-off</t>
+          <t>nastroj, nie diel | one-off</t>
         </is>
       </c>
     </row>
@@ -8012,10 +8451,10 @@
           <t>subtotal - Tooling (one-off)</t>
         </is>
       </c>
-      <c r="B118" s="69" t="n"/>
-      <c r="C118" s="69" t="n"/>
-      <c r="D118" s="69" t="n"/>
-      <c r="E118" s="70" t="n"/>
+      <c r="B118" s="72" t="n"/>
+      <c r="C118" s="72" t="n"/>
+      <c r="D118" s="72" t="n"/>
+      <c r="E118" s="73" t="n"/>
       <c r="F118" s="15" t="n"/>
       <c r="G118" s="15" t="n">
         <v>130</v>
@@ -8032,11 +8471,11 @@
           <t>REQUIRED (everything needed to build and deploy)</t>
         </is>
       </c>
-      <c r="B120" s="69" t="n"/>
-      <c r="C120" s="69" t="n"/>
-      <c r="D120" s="69" t="n"/>
-      <c r="E120" s="69" t="n"/>
-      <c r="F120" s="70" t="n"/>
+      <c r="B120" s="72" t="n"/>
+      <c r="C120" s="72" t="n"/>
+      <c r="D120" s="72" t="n"/>
+      <c r="E120" s="72" t="n"/>
+      <c r="F120" s="73" t="n"/>
       <c r="G120" s="25" t="n">
         <v>716.3100000000001</v>
       </c>
@@ -8047,11 +8486,11 @@
           <t>recommended add-ons (DO, level probe, anti-theft, tools)</t>
         </is>
       </c>
-      <c r="B121" s="69" t="n"/>
-      <c r="C121" s="69" t="n"/>
-      <c r="D121" s="69" t="n"/>
-      <c r="E121" s="69" t="n"/>
-      <c r="F121" s="70" t="n"/>
+      <c r="B121" s="72" t="n"/>
+      <c r="C121" s="72" t="n"/>
+      <c r="D121" s="72" t="n"/>
+      <c r="E121" s="72" t="n"/>
+      <c r="F121" s="73" t="n"/>
       <c r="G121" s="27" t="n">
         <v>641</v>
       </c>
@@ -8062,11 +8501,11 @@
           <t>TOTAL if you buy everything</t>
         </is>
       </c>
-      <c r="B122" s="69" t="n"/>
-      <c r="C122" s="69" t="n"/>
-      <c r="D122" s="69" t="n"/>
-      <c r="E122" s="69" t="n"/>
-      <c r="F122" s="70" t="n"/>
+      <c r="B122" s="72" t="n"/>
+      <c r="C122" s="72" t="n"/>
+      <c r="D122" s="72" t="n"/>
+      <c r="E122" s="72" t="n"/>
+      <c r="F122" s="73" t="n"/>
       <c r="G122" s="29" t="n">
         <v>1357.31</v>
       </c>
@@ -8077,11 +8516,11 @@
           <t>saved by reusing what you already own</t>
         </is>
       </c>
-      <c r="B123" s="69" t="n"/>
-      <c r="C123" s="69" t="n"/>
-      <c r="D123" s="69" t="n"/>
-      <c r="E123" s="69" t="n"/>
-      <c r="F123" s="70" t="n"/>
+      <c r="B123" s="72" t="n"/>
+      <c r="C123" s="72" t="n"/>
+      <c r="D123" s="72" t="n"/>
+      <c r="E123" s="72" t="n"/>
+      <c r="F123" s="73" t="n"/>
       <c r="G123" s="31" t="n">
         <v>-70</v>
       </c>
@@ -8092,11 +8531,11 @@
           <t>net if you reuse your Raspberry Pi etc.</t>
         </is>
       </c>
-      <c r="B124" s="69" t="n"/>
-      <c r="C124" s="69" t="n"/>
-      <c r="D124" s="69" t="n"/>
-      <c r="E124" s="69" t="n"/>
-      <c r="F124" s="70" t="n"/>
+      <c r="B124" s="72" t="n"/>
+      <c r="C124" s="72" t="n"/>
+      <c r="D124" s="72" t="n"/>
+      <c r="E124" s="72" t="n"/>
+      <c r="F124" s="73" t="n"/>
       <c r="G124" s="33" t="n">
         <v>1287.31</v>
       </c>

</xml_diff>

<commit_message>
order: 402 EUR with the Pi taken off the list
I02 was still priced at 70 even though the Raspberry Pi is already his, and that
was the whole reason the earlier cut had to be so deep. Freeing it pays for the
one thing that decides whether the data ever arrives: a 5 dBi whip and a 3 m
mast on the gateway side.

57 lines, 402.11 EUR goods, everything that touches the water still complete.
</commit_message>
<xml_diff>
--- a/docs/sub-mission_parts.xlsx
+++ b/docs/sub-mission_parts.xlsx
@@ -846,7 +846,7 @@
     <row r="3" ht="26" customHeight="1">
       <c r="A3" s="44" t="inlineStr">
         <is>
-          <t>56 lines      goods 436.11 EUR      shipping est. 25.00 EUR      LANDED 461.11 EUR</t>
+          <t>57 lines      goods 402.11 EUR      shipping est. 25.00 EUR      LANDED 427.11 EUR</t>
         </is>
       </c>
     </row>
@@ -1523,7 +1523,7 @@
         </is>
       </c>
       <c r="F32" s="46" t="n">
-        <v>147</v>
+        <v>107</v>
       </c>
     </row>
     <row r="33">
@@ -1561,27 +1561,27 @@
     <row r="34" ht="29" customHeight="1">
       <c r="A34" s="49" t="inlineStr">
         <is>
-          <t>I02</t>
+          <t>I05</t>
         </is>
       </c>
       <c r="B34" s="49" t="inlineStr">
         <is>
-          <t>Compute</t>
+          <t>Mast</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>Raspberry Pi 4 4GB + PSU + SD  -  YOU ALREADY HAVE THIS - reuse, zero soldering; runs the gateway service</t>
+          <t>3m alu mast + wall bracket  -  3 m stozier pre gateway - vyskou sa kupuje dosah</t>
         </is>
       </c>
       <c r="D34" s="51" t="n">
         <v>1</v>
       </c>
       <c r="E34" s="52" t="n">
-        <v>70</v>
+        <v>30</v>
       </c>
       <c r="F34" s="52" t="n">
-        <v>70</v>
+        <v>30</v>
       </c>
     </row>
     <row r="35" ht="15.5" customHeight="1">
@@ -1792,1353 +1792,1357 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" ht="20" customHeight="1">
-      <c r="A44" s="45" t="inlineStr">
+    <row r="43" ht="29" customHeight="1">
+      <c r="A43" s="58" t="inlineStr">
+        <is>
+          <t>I02</t>
+        </is>
+      </c>
+      <c r="B43" s="58" t="inlineStr">
+        <is>
+          <t>Compute</t>
+        </is>
+      </c>
+      <c r="C43" s="17" t="inlineStr">
+        <is>
+          <t>MAM  |  Raspberry Pi 4 4GB + PSU + SD  -  MAM - Raspberry Pi 4, staci mu USB napajanie</t>
+        </is>
+      </c>
+      <c r="D43" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="E43" s="60" t="n">
+        <v>70</v>
+      </c>
+      <c r="F43" s="60" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" ht="20" customHeight="1">
+      <c r="A45" s="45" t="inlineStr">
         <is>
           <t>TECHFUN.SK</t>
         </is>
       </c>
-      <c r="F44" s="46" t="n">
-        <v>49.45</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="47" t="inlineStr">
+      <c r="F45" s="46" t="n">
+        <v>55.45</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="47" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B45" s="47" t="inlineStr">
+      <c r="B46" s="47" t="inlineStr">
         <is>
           <t>Part</t>
         </is>
       </c>
-      <c r="C45" s="47" t="inlineStr">
+      <c r="C46" s="47" t="inlineStr">
         <is>
           <t>Specification / note</t>
         </is>
       </c>
-      <c r="D45" s="48" t="inlineStr">
+      <c r="D46" s="48" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="E45" s="48" t="inlineStr">
+      <c r="E46" s="48" t="inlineStr">
         <is>
           <t>Unit EUR</t>
         </is>
       </c>
-      <c r="F45" s="48" t="inlineStr">
+      <c r="F46" s="48" t="inlineStr">
         <is>
           <t>Total EUR</t>
         </is>
       </c>
     </row>
-    <row r="46" ht="15.5" customHeight="1">
-      <c r="A46" s="49" t="inlineStr">
+    <row r="47" ht="15.5" customHeight="1">
+      <c r="A47" s="49" t="inlineStr">
         <is>
           <t>J03</t>
         </is>
       </c>
-      <c r="B46" s="49" t="inlineStr">
+      <c r="B47" s="49" t="inlineStr">
         <is>
           <t>Epoxy barrier</t>
         </is>
       </c>
-      <c r="C46" s="6" t="inlineStr">
+      <c r="C47" s="6" t="inlineStr">
         <is>
           <t>West System 105 + 206</t>
         </is>
       </c>
-      <c r="D46" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="E46" s="52" t="n">
+      <c r="D47" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="E47" s="52" t="n">
         <v>18</v>
       </c>
-      <c r="F46" s="52" t="n">
+      <c r="F47" s="52" t="n">
         <v>18</v>
       </c>
     </row>
-    <row r="47" ht="29" customHeight="1">
-      <c r="A47" s="53" t="inlineStr">
+    <row r="48" ht="29" customHeight="1">
+      <c r="A48" s="53" t="inlineStr">
         <is>
           <t>B04</t>
         </is>
       </c>
-      <c r="B47" s="57" t="inlineStr">
+      <c r="B48" s="57" t="inlineStr">
         <is>
           <t>Potting compound</t>
         </is>
       </c>
-      <c r="C47" s="54" t="inlineStr">
+      <c r="C48" s="54" t="inlineStr">
         <is>
           <t>3M Scotch-Weld DP270 black 25ml  -  techfun nema DP270; silikonova zalievacia hmota staci na test, epoxid je tuhsi</t>
         </is>
       </c>
-      <c r="D47" s="55" t="n">
-        <v>1</v>
-      </c>
-      <c r="E47" s="56" t="n">
+      <c r="D48" s="55" t="n">
+        <v>1</v>
+      </c>
+      <c r="E48" s="56" t="n">
         <v>14</v>
       </c>
-      <c r="F47" s="56" t="n">
+      <c r="F48" s="56" t="n">
         <v>14</v>
       </c>
     </row>
-    <row r="48" ht="15.5" customHeight="1">
-      <c r="A48" s="49" t="inlineStr">
+    <row r="49" ht="15.5" customHeight="1">
+      <c r="A49" s="49" t="inlineStr">
         <is>
           <t>D07</t>
         </is>
       </c>
-      <c r="B48" s="50" t="inlineStr">
+      <c r="B49" s="50" t="inlineStr">
         <is>
           <t>Turbidity</t>
         </is>
       </c>
-      <c r="C48" s="6" t="inlineStr">
+      <c r="C49" s="6" t="inlineStr">
         <is>
           <t>DFRobot SEN0189 (0-4.5V analog)  -  6 in stock; in model as sensor_turb</t>
         </is>
       </c>
-      <c r="D48" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="E48" s="52" t="n">
+      <c r="D49" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="E49" s="52" t="n">
         <v>12.45</v>
       </c>
-      <c r="F48" s="52" t="n">
+      <c r="F49" s="52" t="n">
         <v>12.45</v>
       </c>
     </row>
-    <row r="49" ht="15.5" customHeight="1">
-      <c r="A49" s="53" t="inlineStr">
+    <row r="50" ht="29" customHeight="1">
+      <c r="A50" s="53" t="inlineStr">
+        <is>
+          <t>G04</t>
+        </is>
+      </c>
+      <c r="B50" s="53" t="inlineStr">
+        <is>
+          <t>Antenna probe</t>
+        </is>
+      </c>
+      <c r="C50" s="54" t="inlineStr">
+        <is>
+          <t>868MHz 5dBi SMA-M omni 195mm  -  jedna 5 dBi na gateway; sonde staci bicik z kitu</t>
+        </is>
+      </c>
+      <c r="D50" s="55" t="n">
+        <v>1</v>
+      </c>
+      <c r="E50" s="56" t="n">
+        <v>6</v>
+      </c>
+      <c r="F50" s="56" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="51" ht="15.5" customHeight="1">
+      <c r="A51" s="49" t="inlineStr">
         <is>
           <t>D04</t>
         </is>
       </c>
-      <c r="B49" s="57" t="inlineStr">
+      <c r="B51" s="50" t="inlineStr">
         <is>
           <t>Temperature</t>
         </is>
       </c>
-      <c r="C49" s="54" t="inlineStr">
+      <c r="C51" s="6" t="inlineStr">
         <is>
           <t>DS18B20 waterproof 1m cable  -  in model as sensor_ntc</t>
         </is>
       </c>
-      <c r="D49" s="55" t="n">
-        <v>1</v>
-      </c>
-      <c r="E49" s="56" t="n">
+      <c r="D51" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="E51" s="52" t="n">
         <v>5</v>
       </c>
-      <c r="F49" s="56" t="n">
+      <c r="F51" s="52" t="n">
         <v>5</v>
       </c>
     </row>
-    <row r="50" ht="29" customHeight="1">
-      <c r="A50" s="49" t="inlineStr">
-        <is>
-          <t>G04</t>
-        </is>
-      </c>
-      <c r="B50" s="49" t="inlineStr">
-        <is>
-          <t>Antenna probe</t>
-        </is>
-      </c>
-      <c r="C50" s="6" t="inlineStr">
-        <is>
-          <t>868MHz 5dBi SMA-M omni 195mm  -  v baleni kazdej Wio-E5 je EU868 antena - samostatne netreba; drzat ako zalohu</t>
-        </is>
-      </c>
-      <c r="D50" s="51" t="n">
+    <row r="53" ht="20" customHeight="1">
+      <c r="A53" s="45" t="inlineStr">
+        <is>
+          <t>RPISHOP.CZ</t>
+        </is>
+      </c>
+      <c r="F53" s="46" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="47" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B54" s="47" t="inlineStr">
+        <is>
+          <t>Part</t>
+        </is>
+      </c>
+      <c r="C54" s="47" t="inlineStr">
+        <is>
+          <t>Specification / note</t>
+        </is>
+      </c>
+      <c r="D54" s="48" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="E54" s="48" t="inlineStr">
+        <is>
+          <t>Unit EUR</t>
+        </is>
+      </c>
+      <c r="F54" s="48" t="inlineStr">
+        <is>
+          <t>Total EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="42.5" customHeight="1">
+      <c r="A55" s="49" t="inlineStr">
+        <is>
+          <t>G03</t>
+        </is>
+      </c>
+      <c r="B55" s="50" t="inlineStr">
+        <is>
+          <t>MCU + radio (single board)</t>
+        </is>
+      </c>
+      <c r="C55" s="6" t="inlineStr">
+        <is>
+          <t>Seeed XIAO nRF52840 + Wio-SX1262 kit (Meshtastic), SEE336 - nRF52840 + SX1262  -  349 Kc, skladom 5+; nahradza Wio-E5, ktory v CZ/SK nie je; antena je v kite</t>
+        </is>
+      </c>
+      <c r="D55" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="E55" s="52" t="n">
+        <v>14</v>
+      </c>
+      <c r="F55" s="52" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="56" ht="42.5" customHeight="1">
+      <c r="A56" s="53" t="inlineStr">
+        <is>
+          <t>I01</t>
+        </is>
+      </c>
+      <c r="B56" s="57" t="inlineStr">
+        <is>
+          <t>Gateway radio (single-channel)</t>
+        </is>
+      </c>
+      <c r="C56" s="54" t="inlineStr">
+        <is>
+          <t>Seeed XIAO nRF52840 + Wio-SX1262 kit (Meshtastic), SEE336 - nRF52840 + SX1262  -  349 Kc, skladom 5+; nahradza Wio-E5, ktory v CZ/SK nie je; antena je v kite</t>
+        </is>
+      </c>
+      <c r="D56" s="55" t="n">
+        <v>1</v>
+      </c>
+      <c r="E56" s="56" t="n">
+        <v>14</v>
+      </c>
+      <c r="F56" s="56" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="58" ht="20" customHeight="1">
+      <c r="A58" s="45" t="inlineStr">
+        <is>
+          <t>X-TEAMRC.COM</t>
+        </is>
+      </c>
+      <c r="F58" s="46" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="47" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B59" s="47" t="inlineStr">
+        <is>
+          <t>Part</t>
+        </is>
+      </c>
+      <c r="C59" s="47" t="inlineStr">
+        <is>
+          <t>Specification / note</t>
+        </is>
+      </c>
+      <c r="D59" s="48" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="E59" s="48" t="inlineStr">
+        <is>
+          <t>Unit EUR</t>
+        </is>
+      </c>
+      <c r="F59" s="48" t="inlineStr">
+        <is>
+          <t>Total EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="42.5" customHeight="1">
+      <c r="A60" s="49" t="inlineStr">
+        <is>
+          <t>C08</t>
+        </is>
+      </c>
+      <c r="B60" s="49" t="inlineStr">
+        <is>
+          <t>Generator</t>
+        </is>
+      </c>
+      <c r="C60" s="6" t="inlineStr">
+        <is>
+          <t>T-Motor GB2208 KV128 or X-TEAM XTG3506 (24N22P 6ohm w/ AS5048A encoder)  -  TEST BEZ GENERATORA: klietka + senzory stacia, generator je dalsi nakup; XTG3506 preferred: encoder = free RPM/flow</t>
+        </is>
+      </c>
+      <c r="D60" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="E60" s="52" t="n">
+        <v>26</v>
+      </c>
+      <c r="F60" s="52" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="62" ht="20" customHeight="1">
+      <c r="A62" s="45" t="inlineStr">
+        <is>
+          <t>LASKAKIT.CZ</t>
+        </is>
+      </c>
+      <c r="F62" s="46" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="47" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B63" s="47" t="inlineStr">
+        <is>
+          <t>Part</t>
+        </is>
+      </c>
+      <c r="C63" s="47" t="inlineStr">
+        <is>
+          <t>Specification / note</t>
+        </is>
+      </c>
+      <c r="D63" s="48" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="E63" s="48" t="inlineStr">
+        <is>
+          <t>Unit EUR</t>
+        </is>
+      </c>
+      <c r="F63" s="48" t="inlineStr">
+        <is>
+          <t>Total EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="15.5" customHeight="1">
+      <c r="A64" s="49" t="inlineStr">
+        <is>
+          <t>G15</t>
+        </is>
+      </c>
+      <c r="B64" s="49" t="inlineStr">
+        <is>
+          <t>Connectors</t>
+        </is>
+      </c>
+      <c r="C64" s="6" t="inlineStr">
+        <is>
+          <t>JST-PH/XH assortment + crimps</t>
+        </is>
+      </c>
+      <c r="D64" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="E64" s="52" t="n">
+        <v>10</v>
+      </c>
+      <c r="F64" s="52" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="66" ht="20" customHeight="1">
+      <c r="A66" s="45" t="inlineStr">
+        <is>
+          <t>SUPERMAGNETICSHOP</t>
+        </is>
+      </c>
+      <c r="F66" s="46" t="n">
+        <v>8.800000000000001</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="47" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B67" s="47" t="inlineStr">
+        <is>
+          <t>Part</t>
+        </is>
+      </c>
+      <c r="C67" s="47" t="inlineStr">
+        <is>
+          <t>Specification / note</t>
+        </is>
+      </c>
+      <c r="D67" s="48" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="E67" s="48" t="inlineStr">
+        <is>
+          <t>Unit EUR</t>
+        </is>
+      </c>
+      <c r="F67" s="48" t="inlineStr">
+        <is>
+          <t>Total EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="29" customHeight="1">
+      <c r="A68" s="49" t="inlineStr">
+        <is>
+          <t>B01</t>
+        </is>
+      </c>
+      <c r="B68" s="50" t="inlineStr">
+        <is>
+          <t>Magnet</t>
+        </is>
+      </c>
+      <c r="C68" s="6" t="inlineStr">
+        <is>
+          <t>N52 D10x5 axially magnetised, canned 316L or epoxy potted  -  16x N52 D10x5 (S-10-05-N52N, 3.3 kg); magsy 10x5 N52 nemá overený</t>
+        </is>
+      </c>
+      <c r="D68" s="51" t="n">
+        <v>16</v>
+      </c>
+      <c r="E68" s="52" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="F68" s="52" t="n">
+        <v>8.800000000000001</v>
+      </c>
+    </row>
+    <row r="70" ht="20" customHeight="1">
+      <c r="A70" s="45" t="inlineStr">
+        <is>
+          <t>PRINTED IN-HOUSE</t>
+        </is>
+      </c>
+      <c r="F70" s="46" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="47" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B71" s="47" t="inlineStr">
+        <is>
+          <t>Part</t>
+        </is>
+      </c>
+      <c r="C71" s="47" t="inlineStr">
+        <is>
+          <t>Specification / note</t>
+        </is>
+      </c>
+      <c r="D71" s="48" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="E71" s="48" t="inlineStr">
+        <is>
+          <t>Unit EUR</t>
+        </is>
+      </c>
+      <c r="F71" s="48" t="inlineStr">
+        <is>
+          <t>Total EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="15.5" customHeight="1">
+      <c r="A72" s="49" t="inlineStr">
+        <is>
+          <t>H06</t>
+        </is>
+      </c>
+      <c r="B72" s="49" t="inlineStr">
+        <is>
+          <t>Hinge collar</t>
+        </is>
+      </c>
+      <c r="C72" s="6" t="inlineStr">
+        <is>
+          <t>printed ASA + M8 A4 bolt</t>
+        </is>
+      </c>
+      <c r="D72" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="E72" s="52" t="n">
+        <v>3</v>
+      </c>
+      <c r="F72" s="52" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="73" ht="15.5" customHeight="1">
+      <c r="A73" s="53" t="inlineStr">
+        <is>
+          <t>C09</t>
+        </is>
+      </c>
+      <c r="B73" s="53" t="inlineStr">
+        <is>
+          <t>Generator mount</t>
+        </is>
+      </c>
+      <c r="C73" s="54" t="inlineStr">
+        <is>
+          <t>printed cradle + 4x M3x8 A4</t>
+        </is>
+      </c>
+      <c r="D73" s="55" t="n">
+        <v>1</v>
+      </c>
+      <c r="E73" s="56" t="n">
+        <v>1</v>
+      </c>
+      <c r="F73" s="56" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="74" ht="29" customHeight="1">
+      <c r="A74" s="49" t="inlineStr">
+        <is>
+          <t>A01</t>
+        </is>
+      </c>
+      <c r="B74" s="49" t="inlineStr">
+        <is>
+          <t>Blade</t>
+        </is>
+      </c>
+      <c r="C74" s="6" t="inlineStr">
+        <is>
+          <t>triple-blade rotor blade NACA4412 D220mm root pitch 28deg tip 2deg  -  ASA or ASA-CF; 6 perimeters; epoxy coat; spare blade = fuse for branch strike</t>
+        </is>
+      </c>
+      <c r="D74" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="E74" s="52" t="n">
         <v>0</v>
       </c>
-      <c r="E50" s="52" t="n">
-        <v>6</v>
-      </c>
-      <c r="F50" s="52" t="n">
+      <c r="F74" s="52" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="52" ht="20" customHeight="1">
-      <c r="A52" s="45" t="inlineStr">
-        <is>
-          <t>RPISHOP.CZ</t>
-        </is>
-      </c>
-      <c r="F52" s="46" t="n">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="47" t="inlineStr">
+    <row r="75" ht="29" customHeight="1">
+      <c r="A75" s="53" t="inlineStr">
+        <is>
+          <t>A02</t>
+        </is>
+      </c>
+      <c r="B75" s="53" t="inlineStr">
+        <is>
+          <t>Hub</t>
+        </is>
+      </c>
+      <c r="C75" s="54" t="inlineStr">
+        <is>
+          <t>Ø64x46mm with 2x M4 heat-set inserts and Ø5 H7 shaft bore  -  brass inserts M4 from TME</t>
+        </is>
+      </c>
+      <c r="D75" s="55" t="n">
+        <v>1</v>
+      </c>
+      <c r="E75" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="F75" s="56" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76" ht="29" customHeight="1">
+      <c r="A76" s="49" t="inlineStr">
+        <is>
+          <t>B02</t>
+        </is>
+      </c>
+      <c r="B76" s="49" t="inlineStr">
+        <is>
+          <t>Magnet cup</t>
+        </is>
+      </c>
+      <c r="C76" s="6" t="inlineStr">
+        <is>
+          <t>D70 rim, 8 pockets D10.2x5.2, printed ASA  -  pockets 10.2 dia (magnet 10 + 0.2 glue), 0.2 mm epoxy recess</t>
+        </is>
+      </c>
+      <c r="D76" s="51" t="n">
+        <v>2</v>
+      </c>
+      <c r="E76" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="F76" s="52" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77" ht="15.5" customHeight="1">
+      <c r="A77" s="53" t="inlineStr">
+        <is>
+          <t>C01</t>
+        </is>
+      </c>
+      <c r="B77" s="53" t="inlineStr">
+        <is>
+          <t>Pod barrel</t>
+        </is>
+      </c>
+      <c r="C77" s="54" t="inlineStr">
+        <is>
+          <t>Ø110x120mm printed ASA wall 2.4mm + epoxy barrier  -  in model as pod</t>
+        </is>
+      </c>
+      <c r="D77" s="55" t="n">
+        <v>1</v>
+      </c>
+      <c r="E77" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="F77" s="56" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78" ht="15.5" customHeight="1">
+      <c r="A78" s="49" t="inlineStr">
+        <is>
+          <t>C02</t>
+        </is>
+      </c>
+      <c r="B78" s="49" t="inlineStr">
+        <is>
+          <t>Tail cone</t>
+        </is>
+      </c>
+      <c r="C78" s="6" t="inlineStr">
+        <is>
+          <t>printed integral</t>
+        </is>
+      </c>
+      <c r="D78" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="E78" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="F78" s="52" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79" ht="15.5" customHeight="1">
+      <c r="A79" s="53" t="inlineStr">
+        <is>
+          <t>E01</t>
+        </is>
+      </c>
+      <c r="B79" s="53" t="inlineStr">
+        <is>
+          <t>Sensor cage</t>
+        </is>
+      </c>
+      <c r="C79" s="54" t="inlineStr">
+        <is>
+          <t>Ø130x150 printed ASA 12 slots  -  in model as cage</t>
+        </is>
+      </c>
+      <c r="D79" s="55" t="n">
+        <v>1</v>
+      </c>
+      <c r="E79" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="F79" s="56" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80" ht="29" customHeight="1">
+      <c r="A80" s="49" t="inlineStr">
+        <is>
+          <t>E03</t>
+        </is>
+      </c>
+      <c r="B80" s="49" t="inlineStr">
+        <is>
+          <t>Sensor holders</t>
+        </is>
+      </c>
+      <c r="C80" s="6" t="inlineStr">
+        <is>
+          <t>printed clips for pH/TDS/turbidity/NTC/MS5837  -  in model as sensor bodies</t>
+        </is>
+      </c>
+      <c r="D80" s="51" t="n">
+        <v>5</v>
+      </c>
+      <c r="E80" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="F80" s="52" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82" ht="20" customHeight="1">
+      <c r="A82" s="45" t="inlineStr">
+        <is>
+          <t>JLCPCB</t>
+        </is>
+      </c>
+      <c r="F82" s="46" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="47" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B53" s="47" t="inlineStr">
+      <c r="B83" s="47" t="inlineStr">
         <is>
           <t>Part</t>
         </is>
       </c>
-      <c r="C53" s="47" t="inlineStr">
+      <c r="C83" s="47" t="inlineStr">
         <is>
           <t>Specification / note</t>
         </is>
       </c>
-      <c r="D53" s="48" t="inlineStr">
+      <c r="D83" s="48" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="E53" s="48" t="inlineStr">
+      <c r="E83" s="48" t="inlineStr">
         <is>
           <t>Unit EUR</t>
         </is>
       </c>
-      <c r="F53" s="48" t="inlineStr">
+      <c r="F83" s="48" t="inlineStr">
         <is>
           <t>Total EUR</t>
         </is>
       </c>
     </row>
-    <row r="54" ht="42.5" customHeight="1">
-      <c r="A54" s="49" t="inlineStr">
-        <is>
-          <t>G03</t>
-        </is>
-      </c>
-      <c r="B54" s="50" t="inlineStr">
-        <is>
-          <t>MCU + radio (single board)</t>
-        </is>
-      </c>
-      <c r="C54" s="6" t="inlineStr">
-        <is>
-          <t>Seeed XIAO nRF52840 + Wio-SX1262 kit (Meshtastic), SEE336 - nRF52840 + SX1262  -  349 Kc, skladom 5+; nahradza Wio-E5, ktory v CZ/SK nie je; antena je v kite</t>
-        </is>
-      </c>
-      <c r="D54" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="E54" s="52" t="n">
-        <v>14</v>
-      </c>
-      <c r="F54" s="52" t="n">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="55" ht="42.5" customHeight="1">
-      <c r="A55" s="53" t="inlineStr">
-        <is>
-          <t>I01</t>
-        </is>
-      </c>
-      <c r="B55" s="57" t="inlineStr">
-        <is>
-          <t>Gateway radio (single-channel)</t>
-        </is>
-      </c>
-      <c r="C55" s="54" t="inlineStr">
-        <is>
-          <t>Seeed XIAO nRF52840 + Wio-SX1262 kit (Meshtastic), SEE336 - nRF52840 + SX1262  -  349 Kc, skladom 5+; nahradza Wio-E5, ktory v CZ/SK nie je; antena je v kite</t>
-        </is>
-      </c>
-      <c r="D55" s="55" t="n">
-        <v>1</v>
-      </c>
-      <c r="E55" s="56" t="n">
-        <v>14</v>
-      </c>
-      <c r="F55" s="56" t="n">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="57" ht="20" customHeight="1">
-      <c r="A57" s="45" t="inlineStr">
-        <is>
-          <t>X-TEAMRC.COM</t>
-        </is>
-      </c>
-      <c r="F57" s="46" t="n">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="47" t="inlineStr">
+    <row r="84" ht="15.5" customHeight="1">
+      <c r="A84" s="49" t="inlineStr">
+        <is>
+          <t>G14</t>
+        </is>
+      </c>
+      <c r="B84" s="49" t="inlineStr">
+        <is>
+          <t>PCB</t>
+        </is>
+      </c>
+      <c r="C84" s="6" t="inlineStr">
+        <is>
+          <t>custom 2-layer 60x80mm  -  panel of 10 amortises</t>
+        </is>
+      </c>
+      <c r="D84" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="E84" s="52" t="n">
+        <v>3</v>
+      </c>
+      <c r="F84" s="52" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="86" ht="20" customHeight="1">
+      <c r="A86" s="45" t="inlineStr">
+        <is>
+          <t>NEREZMATERIAL.CZ</t>
+        </is>
+      </c>
+      <c r="F86" s="46" t="n">
+        <v>2.6</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="47" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B58" s="47" t="inlineStr">
+      <c r="B87" s="47" t="inlineStr">
         <is>
           <t>Part</t>
         </is>
       </c>
-      <c r="C58" s="47" t="inlineStr">
+      <c r="C87" s="47" t="inlineStr">
         <is>
           <t>Specification / note</t>
         </is>
       </c>
-      <c r="D58" s="48" t="inlineStr">
+      <c r="D87" s="48" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="E58" s="48" t="inlineStr">
+      <c r="E87" s="48" t="inlineStr">
         <is>
           <t>Unit EUR</t>
         </is>
       </c>
-      <c r="F58" s="48" t="inlineStr">
+      <c r="F87" s="48" t="inlineStr">
         <is>
           <t>Total EUR</t>
         </is>
       </c>
     </row>
-    <row r="59" ht="42.5" customHeight="1">
-      <c r="A59" s="49" t="inlineStr">
-        <is>
-          <t>C08</t>
-        </is>
-      </c>
-      <c r="B59" s="49" t="inlineStr">
-        <is>
-          <t>Generator</t>
-        </is>
-      </c>
-      <c r="C59" s="6" t="inlineStr">
-        <is>
-          <t>T-Motor GB2208 KV128 or X-TEAM XTG3506 (24N22P 6ohm w/ AS5048A encoder)  -  TEST BEZ GENERATORA: klietka + senzory stacia, generator je dalsi nakup; XTG3506 preferred: encoder = free RPM/flow</t>
-        </is>
-      </c>
-      <c r="D59" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="E59" s="52" t="n">
-        <v>26</v>
-      </c>
-      <c r="F59" s="52" t="n">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="61" ht="20" customHeight="1">
-      <c r="A61" s="45" t="inlineStr">
-        <is>
-          <t>LASKAKIT.CZ</t>
-        </is>
-      </c>
-      <c r="F61" s="46" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="47" t="inlineStr">
+    <row r="88" ht="42.5" customHeight="1">
+      <c r="A88" s="49" t="inlineStr">
+        <is>
+          <t>A03</t>
+        </is>
+      </c>
+      <c r="B88" s="49" t="inlineStr">
+        <is>
+          <t>Wet shaft</t>
+        </is>
+      </c>
+      <c r="C88" s="6" t="inlineStr">
+        <is>
+          <t>316L Ø5 h6 x 115mm ground; 2 flats each end  -  lokalny zeleziar / Hornbach M5 A4 srob - 4. obchod sa nerata, nema postu; 3m bar 63.1 CZK makes ~26 shafts</t>
+        </is>
+      </c>
+      <c r="D88" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="E88" s="52" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="F88" s="52" t="n">
+        <v>2.6</v>
+      </c>
+    </row>
+    <row r="89" ht="29" customHeight="1">
+      <c r="A89" s="53" t="inlineStr">
+        <is>
+          <t>B03</t>
+        </is>
+      </c>
+      <c r="B89" s="53" t="inlineStr">
+        <is>
+          <t>Separation wall</t>
+        </is>
+      </c>
+      <c r="C89" s="54" t="inlineStr">
+        <is>
+          <t>D106 x 4 mm - RECOMMENDED integral with the pod bulkhead (no separate part)  -  4 mm per CAD, not 5; integral removes O-ring C03 and screws C05</t>
+        </is>
+      </c>
+      <c r="D89" s="55" t="n">
+        <v>1</v>
+      </c>
+      <c r="E89" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="F89" s="56" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="91" ht="20" customHeight="1">
+      <c r="A91" s="45" t="inlineStr">
+        <is>
+          <t>PRUSA3D</t>
+        </is>
+      </c>
+      <c r="F91" s="46" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="47" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B62" s="47" t="inlineStr">
+      <c r="B92" s="47" t="inlineStr">
         <is>
           <t>Part</t>
         </is>
       </c>
-      <c r="C62" s="47" t="inlineStr">
+      <c r="C92" s="47" t="inlineStr">
         <is>
           <t>Specification / note</t>
         </is>
       </c>
-      <c r="D62" s="48" t="inlineStr">
+      <c r="D92" s="48" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="E62" s="48" t="inlineStr">
+      <c r="E92" s="48" t="inlineStr">
         <is>
           <t>Unit EUR</t>
         </is>
       </c>
-      <c r="F62" s="48" t="inlineStr">
+      <c r="F92" s="48" t="inlineStr">
         <is>
           <t>Total EUR</t>
         </is>
       </c>
     </row>
-    <row r="63" ht="15.5" customHeight="1">
-      <c r="A63" s="49" t="inlineStr">
-        <is>
-          <t>G15</t>
-        </is>
-      </c>
-      <c r="B63" s="49" t="inlineStr">
-        <is>
-          <t>Connectors</t>
-        </is>
-      </c>
-      <c r="C63" s="6" t="inlineStr">
-        <is>
-          <t>JST-PH/XH assortment + crimps</t>
-        </is>
-      </c>
-      <c r="D63" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="E63" s="52" t="n">
-        <v>10</v>
-      </c>
-      <c r="F63" s="52" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="65" ht="20" customHeight="1">
-      <c r="A65" s="45" t="inlineStr">
-        <is>
-          <t>SUPERMAGNETICSHOP</t>
-        </is>
-      </c>
-      <c r="F65" s="46" t="n">
-        <v>8.800000000000001</v>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="47" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B66" s="47" t="inlineStr">
-        <is>
-          <t>Part</t>
-        </is>
-      </c>
-      <c r="C66" s="47" t="inlineStr">
-        <is>
-          <t>Specification / note</t>
-        </is>
-      </c>
-      <c r="D66" s="48" t="inlineStr">
-        <is>
-          <t>Qty</t>
-        </is>
-      </c>
-      <c r="E66" s="48" t="inlineStr">
-        <is>
-          <t>Unit EUR</t>
-        </is>
-      </c>
-      <c r="F66" s="48" t="inlineStr">
-        <is>
-          <t>Total EUR</t>
-        </is>
-      </c>
-    </row>
-    <row r="67" ht="29" customHeight="1">
-      <c r="A67" s="49" t="inlineStr">
-        <is>
-          <t>B01</t>
-        </is>
-      </c>
-      <c r="B67" s="50" t="inlineStr">
-        <is>
-          <t>Magnet</t>
-        </is>
-      </c>
-      <c r="C67" s="6" t="inlineStr">
-        <is>
-          <t>N52 D10x5 axially magnetised, canned 316L or epoxy potted  -  16x N52 D10x5 (S-10-05-N52N, 3.3 kg); magsy 10x5 N52 nemá overený</t>
-        </is>
-      </c>
-      <c r="D67" s="51" t="n">
-        <v>16</v>
-      </c>
-      <c r="E67" s="52" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="F67" s="52" t="n">
-        <v>8.800000000000001</v>
-      </c>
-    </row>
-    <row r="69" ht="20" customHeight="1">
-      <c r="A69" s="45" t="inlineStr">
-        <is>
-          <t>PRINTED IN-HOUSE</t>
-        </is>
-      </c>
-      <c r="F69" s="46" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="47" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B70" s="47" t="inlineStr">
-        <is>
-          <t>Part</t>
-        </is>
-      </c>
-      <c r="C70" s="47" t="inlineStr">
-        <is>
-          <t>Specification / note</t>
-        </is>
-      </c>
-      <c r="D70" s="48" t="inlineStr">
-        <is>
-          <t>Qty</t>
-        </is>
-      </c>
-      <c r="E70" s="48" t="inlineStr">
-        <is>
-          <t>Unit EUR</t>
-        </is>
-      </c>
-      <c r="F70" s="48" t="inlineStr">
-        <is>
-          <t>Total EUR</t>
-        </is>
-      </c>
-    </row>
-    <row r="71" ht="15.5" customHeight="1">
-      <c r="A71" s="49" t="inlineStr">
-        <is>
-          <t>H06</t>
-        </is>
-      </c>
-      <c r="B71" s="49" t="inlineStr">
-        <is>
-          <t>Hinge collar</t>
-        </is>
-      </c>
-      <c r="C71" s="6" t="inlineStr">
-        <is>
-          <t>printed ASA + M8 A4 bolt</t>
-        </is>
-      </c>
-      <c r="D71" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="E71" s="52" t="n">
-        <v>3</v>
-      </c>
-      <c r="F71" s="52" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="72" ht="15.5" customHeight="1">
-      <c r="A72" s="53" t="inlineStr">
-        <is>
-          <t>C09</t>
-        </is>
-      </c>
-      <c r="B72" s="53" t="inlineStr">
-        <is>
-          <t>Generator mount</t>
-        </is>
-      </c>
-      <c r="C72" s="54" t="inlineStr">
-        <is>
-          <t>printed cradle + 4x M3x8 A4</t>
-        </is>
-      </c>
-      <c r="D72" s="55" t="n">
-        <v>1</v>
-      </c>
-      <c r="E72" s="56" t="n">
-        <v>1</v>
-      </c>
-      <c r="F72" s="56" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="73" ht="29" customHeight="1">
-      <c r="A73" s="49" t="inlineStr">
-        <is>
-          <t>A01</t>
-        </is>
-      </c>
-      <c r="B73" s="49" t="inlineStr">
-        <is>
-          <t>Blade</t>
-        </is>
-      </c>
-      <c r="C73" s="6" t="inlineStr">
-        <is>
-          <t>triple-blade rotor blade NACA4412 D220mm root pitch 28deg tip 2deg  -  ASA or ASA-CF; 6 perimeters; epoxy coat; spare blade = fuse for branch strike</t>
-        </is>
-      </c>
-      <c r="D73" s="51" t="n">
-        <v>3</v>
-      </c>
-      <c r="E73" s="52" t="n">
+    <row r="93" ht="29" customHeight="1">
+      <c r="A93" s="58" t="inlineStr">
+        <is>
+          <t>J01</t>
+        </is>
+      </c>
+      <c r="B93" s="58" t="inlineStr">
+        <is>
+          <t>Filament ASA</t>
+        </is>
+      </c>
+      <c r="C93" s="17" t="inlineStr">
+        <is>
+          <t>MAM  |  Prusament ASA 850g  -  ABS z domaceho spoolu, nie ASA; UV je len na brehu</t>
+        </is>
+      </c>
+      <c r="D93" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="E93" s="60" t="n">
+        <v>32</v>
+      </c>
+      <c r="F93" s="60" t="n">
         <v>0</v>
-      </c>
-      <c r="F73" s="52" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="74" ht="29" customHeight="1">
-      <c r="A74" s="53" t="inlineStr">
-        <is>
-          <t>A02</t>
-        </is>
-      </c>
-      <c r="B74" s="53" t="inlineStr">
-        <is>
-          <t>Hub</t>
-        </is>
-      </c>
-      <c r="C74" s="54" t="inlineStr">
-        <is>
-          <t>Ø64x46mm with 2x M4 heat-set inserts and Ø5 H7 shaft bore  -  brass inserts M4 from TME</t>
-        </is>
-      </c>
-      <c r="D74" s="55" t="n">
-        <v>1</v>
-      </c>
-      <c r="E74" s="56" t="n">
-        <v>0</v>
-      </c>
-      <c r="F74" s="56" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="75" ht="29" customHeight="1">
-      <c r="A75" s="49" t="inlineStr">
-        <is>
-          <t>B02</t>
-        </is>
-      </c>
-      <c r="B75" s="49" t="inlineStr">
-        <is>
-          <t>Magnet cup</t>
-        </is>
-      </c>
-      <c r="C75" s="6" t="inlineStr">
-        <is>
-          <t>D70 rim, 8 pockets D10.2x5.2, printed ASA  -  pockets 10.2 dia (magnet 10 + 0.2 glue), 0.2 mm epoxy recess</t>
-        </is>
-      </c>
-      <c r="D75" s="51" t="n">
-        <v>2</v>
-      </c>
-      <c r="E75" s="52" t="n">
-        <v>0</v>
-      </c>
-      <c r="F75" s="52" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="76" ht="15.5" customHeight="1">
-      <c r="A76" s="53" t="inlineStr">
-        <is>
-          <t>C01</t>
-        </is>
-      </c>
-      <c r="B76" s="53" t="inlineStr">
-        <is>
-          <t>Pod barrel</t>
-        </is>
-      </c>
-      <c r="C76" s="54" t="inlineStr">
-        <is>
-          <t>Ø110x120mm printed ASA wall 2.4mm + epoxy barrier  -  in model as pod</t>
-        </is>
-      </c>
-      <c r="D76" s="55" t="n">
-        <v>1</v>
-      </c>
-      <c r="E76" s="56" t="n">
-        <v>0</v>
-      </c>
-      <c r="F76" s="56" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="77" ht="15.5" customHeight="1">
-      <c r="A77" s="49" t="inlineStr">
-        <is>
-          <t>C02</t>
-        </is>
-      </c>
-      <c r="B77" s="49" t="inlineStr">
-        <is>
-          <t>Tail cone</t>
-        </is>
-      </c>
-      <c r="C77" s="6" t="inlineStr">
-        <is>
-          <t>printed integral</t>
-        </is>
-      </c>
-      <c r="D77" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="E77" s="52" t="n">
-        <v>0</v>
-      </c>
-      <c r="F77" s="52" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="78" ht="15.5" customHeight="1">
-      <c r="A78" s="53" t="inlineStr">
-        <is>
-          <t>E01</t>
-        </is>
-      </c>
-      <c r="B78" s="53" t="inlineStr">
-        <is>
-          <t>Sensor cage</t>
-        </is>
-      </c>
-      <c r="C78" s="54" t="inlineStr">
-        <is>
-          <t>Ø130x150 printed ASA 12 slots  -  in model as cage</t>
-        </is>
-      </c>
-      <c r="D78" s="55" t="n">
-        <v>1</v>
-      </c>
-      <c r="E78" s="56" t="n">
-        <v>0</v>
-      </c>
-      <c r="F78" s="56" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="79" ht="29" customHeight="1">
-      <c r="A79" s="49" t="inlineStr">
-        <is>
-          <t>E03</t>
-        </is>
-      </c>
-      <c r="B79" s="49" t="inlineStr">
-        <is>
-          <t>Sensor holders</t>
-        </is>
-      </c>
-      <c r="C79" s="6" t="inlineStr">
-        <is>
-          <t>printed clips for pH/TDS/turbidity/NTC/MS5837  -  in model as sensor bodies</t>
-        </is>
-      </c>
-      <c r="D79" s="51" t="n">
-        <v>5</v>
-      </c>
-      <c r="E79" s="52" t="n">
-        <v>0</v>
-      </c>
-      <c r="F79" s="52" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="81" ht="20" customHeight="1">
-      <c r="A81" s="45" t="inlineStr">
-        <is>
-          <t>JLCPCB</t>
-        </is>
-      </c>
-      <c r="F81" s="46" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" s="47" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B82" s="47" t="inlineStr">
-        <is>
-          <t>Part</t>
-        </is>
-      </c>
-      <c r="C82" s="47" t="inlineStr">
-        <is>
-          <t>Specification / note</t>
-        </is>
-      </c>
-      <c r="D82" s="48" t="inlineStr">
-        <is>
-          <t>Qty</t>
-        </is>
-      </c>
-      <c r="E82" s="48" t="inlineStr">
-        <is>
-          <t>Unit EUR</t>
-        </is>
-      </c>
-      <c r="F82" s="48" t="inlineStr">
-        <is>
-          <t>Total EUR</t>
-        </is>
-      </c>
-    </row>
-    <row r="83" ht="15.5" customHeight="1">
-      <c r="A83" s="49" t="inlineStr">
-        <is>
-          <t>G14</t>
-        </is>
-      </c>
-      <c r="B83" s="49" t="inlineStr">
-        <is>
-          <t>PCB</t>
-        </is>
-      </c>
-      <c r="C83" s="6" t="inlineStr">
-        <is>
-          <t>custom 2-layer 60x80mm  -  panel of 10 amortises</t>
-        </is>
-      </c>
-      <c r="D83" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="E83" s="52" t="n">
-        <v>3</v>
-      </c>
-      <c r="F83" s="52" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="85" ht="20" customHeight="1">
-      <c r="A85" s="45" t="inlineStr">
-        <is>
-          <t>NEREZMATERIAL.CZ</t>
-        </is>
-      </c>
-      <c r="F85" s="46" t="n">
-        <v>2.6</v>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" s="47" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B86" s="47" t="inlineStr">
-        <is>
-          <t>Part</t>
-        </is>
-      </c>
-      <c r="C86" s="47" t="inlineStr">
-        <is>
-          <t>Specification / note</t>
-        </is>
-      </c>
-      <c r="D86" s="48" t="inlineStr">
-        <is>
-          <t>Qty</t>
-        </is>
-      </c>
-      <c r="E86" s="48" t="inlineStr">
-        <is>
-          <t>Unit EUR</t>
-        </is>
-      </c>
-      <c r="F86" s="48" t="inlineStr">
-        <is>
-          <t>Total EUR</t>
-        </is>
-      </c>
-    </row>
-    <row r="87" ht="42.5" customHeight="1">
-      <c r="A87" s="49" t="inlineStr">
-        <is>
-          <t>A03</t>
-        </is>
-      </c>
-      <c r="B87" s="49" t="inlineStr">
-        <is>
-          <t>Wet shaft</t>
-        </is>
-      </c>
-      <c r="C87" s="6" t="inlineStr">
-        <is>
-          <t>316L Ø5 h6 x 115mm ground; 2 flats each end  -  lokalny zeleziar / Hornbach M5 A4 srob - 4. obchod sa nerata, nema postu; 3m bar 63.1 CZK makes ~26 shafts</t>
-        </is>
-      </c>
-      <c r="D87" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="E87" s="52" t="n">
-        <v>2.6</v>
-      </c>
-      <c r="F87" s="52" t="n">
-        <v>2.6</v>
-      </c>
-    </row>
-    <row r="88" ht="29" customHeight="1">
-      <c r="A88" s="53" t="inlineStr">
-        <is>
-          <t>B03</t>
-        </is>
-      </c>
-      <c r="B88" s="53" t="inlineStr">
-        <is>
-          <t>Separation wall</t>
-        </is>
-      </c>
-      <c r="C88" s="54" t="inlineStr">
-        <is>
-          <t>D106 x 4 mm - RECOMMENDED integral with the pod bulkhead (no separate part)  -  4 mm per CAD, not 5; integral removes O-ring C03 and screws C05</t>
-        </is>
-      </c>
-      <c r="D88" s="55" t="n">
-        <v>1</v>
-      </c>
-      <c r="E88" s="56" t="n">
-        <v>0</v>
-      </c>
-      <c r="F88" s="56" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="90" ht="20" customHeight="1">
-      <c r="A90" s="45" t="inlineStr">
-        <is>
-          <t>PRUSA3D</t>
-        </is>
-      </c>
-      <c r="F90" s="46" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" s="47" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B91" s="47" t="inlineStr">
-        <is>
-          <t>Part</t>
-        </is>
-      </c>
-      <c r="C91" s="47" t="inlineStr">
-        <is>
-          <t>Specification / note</t>
-        </is>
-      </c>
-      <c r="D91" s="48" t="inlineStr">
-        <is>
-          <t>Qty</t>
-        </is>
-      </c>
-      <c r="E91" s="48" t="inlineStr">
-        <is>
-          <t>Unit EUR</t>
-        </is>
-      </c>
-      <c r="F91" s="48" t="inlineStr">
-        <is>
-          <t>Total EUR</t>
-        </is>
-      </c>
-    </row>
-    <row r="92" ht="29" customHeight="1">
-      <c r="A92" s="58" t="inlineStr">
-        <is>
-          <t>J01</t>
-        </is>
-      </c>
-      <c r="B92" s="58" t="inlineStr">
-        <is>
-          <t>Filament ASA</t>
-        </is>
-      </c>
-      <c r="C92" s="17" t="inlineStr">
-        <is>
-          <t>MAM  |  Prusament ASA 850g  -  ABS z domaceho spoolu, nie ASA; UV je len na brehu</t>
-        </is>
-      </c>
-      <c r="D92" s="59" t="n">
-        <v>1</v>
-      </c>
-      <c r="E92" s="60" t="n">
-        <v>32</v>
-      </c>
-      <c r="F92" s="60" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="94" ht="18" customHeight="1">
-      <c r="A94" s="61" t="inlineStr">
-        <is>
-          <t>GOODS</t>
-        </is>
-      </c>
-      <c r="F94" s="62" t="n">
-        <v>436.11</v>
       </c>
     </row>
     <row r="95" ht="18" customHeight="1">
       <c r="A95" s="61" t="inlineStr">
         <is>
+          <t>GOODS</t>
+        </is>
+      </c>
+      <c r="F95" s="62" t="n">
+        <v>402.11</v>
+      </c>
+    </row>
+    <row r="96" ht="18" customHeight="1">
+      <c r="A96" s="61" t="inlineStr">
+        <is>
           <t>shipping, estimated</t>
         </is>
       </c>
-      <c r="F95" s="62" t="n">
+      <c r="F96" s="62" t="n">
         <v>25</v>
       </c>
     </row>
-    <row r="96" ht="22" customHeight="1">
-      <c r="A96" s="63" t="inlineStr">
+    <row r="97" ht="22" customHeight="1">
+      <c r="A97" s="63" t="inlineStr">
         <is>
           <t>LANDED TOTAL</t>
         </is>
       </c>
-      <c r="F96" s="64" t="n">
-        <v>461.11</v>
-      </c>
-    </row>
-    <row r="99" ht="22" customHeight="1">
-      <c r="A99" s="65" t="inlineStr">
+      <c r="F97" s="64" t="n">
+        <v>427.11</v>
+      </c>
+    </row>
+    <row r="100" ht="22" customHeight="1">
+      <c r="A100" s="65" t="inlineStr">
         <is>
           <t>NOT IN THIS ORDER</t>
         </is>
       </c>
     </row>
-    <row r="100">
-      <c r="A100" s="66" t="inlineStr">
+    <row r="101">
+      <c r="A101" s="66" t="inlineStr">
         <is>
           <t>PHASE 2 - BUY LATER</t>
-        </is>
-      </c>
-    </row>
-    <row r="101" ht="15.5" customHeight="1">
-      <c r="A101" s="67" t="inlineStr">
-        <is>
-          <t>D01</t>
-        </is>
-      </c>
-      <c r="B101" s="67" t="inlineStr">
-        <is>
-          <t>pH electrode</t>
-        </is>
-      </c>
-      <c r="C101" s="68" t="inlineStr">
-        <is>
-          <t>pH kit: 39 EUR, 14-30 dni servis | OPTIONAL per site; 14-30 day service; +-0.1 pH after 2-pt cal</t>
-        </is>
-      </c>
-      <c r="E101" s="69" t="inlineStr">
-        <is>
-          <t>39.0</t>
         </is>
       </c>
     </row>
     <row r="102" ht="15.5" customHeight="1">
       <c r="A102" s="67" t="inlineStr">
         <is>
-          <t>D02</t>
+          <t>D01</t>
         </is>
       </c>
       <c r="B102" s="67" t="inlineStr">
         <is>
-          <t>pH spare electrode</t>
+          <t>pH electrode</t>
         </is>
       </c>
       <c r="C102" s="68" t="inlineStr">
         <is>
-          <t>pH spare electrodes: 18 EUR | consumable</t>
+          <t>pH kit: 39 EUR, 14-30 dni servis | OPTIONAL per site; 14-30 day service; +-0.1 pH after 2-pt cal</t>
         </is>
       </c>
       <c r="E102" s="69" t="inlineStr">
         <is>
-          <t>9.0</t>
+          <t>39.0</t>
         </is>
       </c>
     </row>
     <row r="103" ht="15.5" customHeight="1">
       <c r="A103" s="67" t="inlineStr">
         <is>
+          <t>D02</t>
+        </is>
+      </c>
+      <c r="B103" s="67" t="inlineStr">
+        <is>
+          <t>pH spare electrode</t>
+        </is>
+      </c>
+      <c r="C103" s="68" t="inlineStr">
+        <is>
+          <t>pH spare electrodes: 18 EUR | consumable</t>
+        </is>
+      </c>
+      <c r="E103" s="69" t="inlineStr">
+        <is>
+          <t>9.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" ht="15.5" customHeight="1">
+      <c r="A104" s="67" t="inlineStr">
+        <is>
           <t>D03</t>
         </is>
       </c>
-      <c r="B103" s="67" t="inlineStr">
+      <c r="B104" s="67" t="inlineStr">
         <is>
           <t>pH buffer</t>
         </is>
       </c>
-      <c r="C103" s="68" t="inlineStr">
+      <c r="C104" s="68" t="inlineStr">
         <is>
           <t>pH buffers: 12 EUR | consumable</t>
         </is>
       </c>
-      <c r="E103" s="69" t="inlineStr">
+      <c r="E104" s="69" t="inlineStr">
         <is>
           <t>12.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="104" ht="29" customHeight="1">
-      <c r="A104" s="67" t="inlineStr">
-        <is>
-          <t>D09</t>
-        </is>
-      </c>
-      <c r="B104" s="67" t="inlineStr">
-        <is>
-          <t>Dissolved oxygen kit</t>
-        </is>
-      </c>
-      <c r="C104" s="68" t="inlineStr">
-        <is>
-          <t>DO: 175 EUR, membrana 1-2 mesiace - prvy kandidat | HIGHEST-VALUE channel (Budca = hypoxia); membrane 1-2 months in muddy water; 0.5M NaOH filling sol</t>
-        </is>
-      </c>
-      <c r="E104" s="69" t="inlineStr">
-        <is>
-          <t>175.0</t>
         </is>
       </c>
     </row>
     <row r="105" ht="29" customHeight="1">
       <c r="A105" s="67" t="inlineStr">
         <is>
+          <t>D09</t>
+        </is>
+      </c>
+      <c r="B105" s="67" t="inlineStr">
+        <is>
+          <t>Dissolved oxygen kit</t>
+        </is>
+      </c>
+      <c r="C105" s="68" t="inlineStr">
+        <is>
+          <t>DO: 175 EUR, membrana 1-2 mesiace - prvy kandidat | HIGHEST-VALUE channel (Budca = hypoxia); membrane 1-2 months in muddy water; 0.5M NaOH filling sol</t>
+        </is>
+      </c>
+      <c r="E105" s="69" t="inlineStr">
+        <is>
+          <t>175.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" ht="29" customHeight="1">
+      <c r="A106" s="67" t="inlineStr">
+        <is>
           <t>D05</t>
         </is>
       </c>
-      <c r="B105" s="67" t="inlineStr">
+      <c r="B106" s="67" t="inlineStr">
         <is>
           <t>Level / stage probe</t>
         </is>
       </c>
-      <c r="C105" s="68" t="inlineStr">
+      <c r="C106" s="68" t="inlineStr">
         <is>
           <t>level: 110 EUR, quote; bez varovania pred povodnou | MS5837-30BA REJECTED: gel element must be dried daily, 24h max submersion</t>
         </is>
       </c>
-      <c r="E105" s="69" t="inlineStr">
+      <c r="E106" s="69" t="inlineStr">
         <is>
           <t>110.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="106" ht="15.5" customHeight="1">
-      <c r="A106" s="67" t="inlineStr">
-        <is>
-          <t>D08</t>
-        </is>
-      </c>
-      <c r="B106" s="67" t="inlineStr">
-        <is>
-          <t>Sensor cable</t>
-        </is>
-      </c>
-      <c r="C106" s="68" t="inlineStr">
-        <is>
-          <t xml:space="preserve">sensor cable 20 EUR - F01 8-zilovy to unesie | </t>
-        </is>
-      </c>
-      <c r="E106" s="69" t="inlineStr">
-        <is>
-          <t>20.0</t>
         </is>
       </c>
     </row>
     <row r="107" ht="15.5" customHeight="1">
       <c r="A107" s="67" t="inlineStr">
         <is>
-          <t>G01</t>
+          <t>D08</t>
         </is>
       </c>
       <c r="B107" s="67" t="inlineStr">
         <is>
-          <t>Enclosure</t>
+          <t>Sensor cable</t>
         </is>
       </c>
       <c r="C107" s="68" t="inlineStr">
         <is>
-          <t>vynechane: vodotesna krabica na brehu - nie je sucastou stavby | in model as site_box</t>
+          <t xml:space="preserve">sensor cable 20 EUR - F01 8-zilovy to unesie | </t>
         </is>
       </c>
       <c r="E107" s="69" t="inlineStr">
         <is>
-          <t>22.0</t>
+          <t>20.0</t>
         </is>
       </c>
     </row>
     <row r="108" ht="15.5" customHeight="1">
       <c r="A108" s="67" t="inlineStr">
         <is>
-          <t>G13</t>
+          <t>G01</t>
         </is>
       </c>
       <c r="B108" s="67" t="inlineStr">
         <is>
-          <t>Barometer</t>
+          <t>Enclosure</t>
         </is>
       </c>
       <c r="C108" s="68" t="inlineStr">
         <is>
-          <t>barometer 6 EUR - level sonda je gauge, netreba | pressure reference for MS5837</t>
+          <t>vynechane: vodotesna krabica na brehu - nie je sucastou stavby | in model as site_box</t>
         </is>
       </c>
       <c r="E108" s="69" t="inlineStr">
         <is>
-          <t>6.0</t>
+          <t>22.0</t>
         </is>
       </c>
     </row>
     <row r="109" ht="15.5" customHeight="1">
       <c r="A109" s="67" t="inlineStr">
         <is>
-          <t>H03</t>
+          <t>G13</t>
         </is>
       </c>
       <c r="B109" s="67" t="inlineStr">
         <is>
-          <t>Receiver sleeve</t>
+          <t>Barometer</t>
         </is>
       </c>
       <c r="C109" s="68" t="inlineStr">
         <is>
-          <t>receiver sleeve 8 EUR - pole sa da pripinacit priamo | pinned mast interface</t>
+          <t>barometer 6 EUR - level sonda je gauge, netreba | pressure reference for MS5837</t>
         </is>
       </c>
       <c r="E109" s="69" t="inlineStr">
         <is>
-          <t>8.0</t>
+          <t>6.0</t>
         </is>
       </c>
     </row>
     <row r="110" ht="15.5" customHeight="1">
       <c r="A110" s="67" t="inlineStr">
         <is>
-          <t>H08</t>
+          <t>H03</t>
         </is>
       </c>
       <c r="B110" s="67" t="inlineStr">
         <is>
-          <t>Yaw strut</t>
+          <t>Receiver sleeve</t>
         </is>
       </c>
       <c r="C110" s="68" t="inlineStr">
         <is>
-          <t>yaw strut 5 EUR - anti-flutter, vydrzi aj bez na test | anti-flutter</t>
+          <t>receiver sleeve 8 EUR - pole sa da pripinacit priamo | pinned mast interface</t>
         </is>
       </c>
       <c r="E110" s="69" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>8.0</t>
         </is>
       </c>
     </row>
     <row r="111" ht="15.5" customHeight="1">
       <c r="A111" s="67" t="inlineStr">
         <is>
-          <t>H12</t>
+          <t>H08</t>
         </is>
       </c>
       <c r="B111" s="67" t="inlineStr">
         <is>
-          <t>Security fastener</t>
+          <t>Yaw strut</t>
         </is>
       </c>
       <c r="C111" s="68" t="inlineStr">
         <is>
-          <t>security fastener 4 EUR - az pri nasadeni | anti-theft</t>
+          <t>yaw strut 5 EUR - anti-flutter, vydrzi aj bez na test | anti-flutter</t>
         </is>
       </c>
       <c r="E111" s="69" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>5.0</t>
         </is>
       </c>
     </row>
     <row r="112" ht="15.5" customHeight="1">
       <c r="A112" s="67" t="inlineStr">
         <is>
+          <t>H12</t>
+        </is>
+      </c>
+      <c r="B112" s="67" t="inlineStr">
+        <is>
+          <t>Security fastener</t>
+        </is>
+      </c>
+      <c r="C112" s="68" t="inlineStr">
+        <is>
+          <t>security fastener 4 EUR - az pri nasadeni | anti-theft</t>
+        </is>
+      </c>
+      <c r="E112" s="69" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="113" ht="15.5" customHeight="1">
+      <c r="A113" s="67" t="inlineStr">
+        <is>
           <t>H13</t>
         </is>
       </c>
-      <c r="B112" s="67" t="inlineStr">
+      <c r="B113" s="67" t="inlineStr">
         <is>
           <t>Site label</t>
         </is>
       </c>
-      <c r="C112" s="68" t="inlineStr">
+      <c r="C113" s="68" t="inlineStr">
         <is>
           <t>site label 3 EUR - az pri nasadeni | anti-theft by making it unsellable</t>
         </is>
       </c>
-      <c r="E112" s="69" t="inlineStr">
+      <c r="E113" s="69" t="inlineStr">
         <is>
           <t>3.0</t>
         </is>
       </c>
     </row>
-    <row r="113" ht="29" customHeight="1">
-      <c r="A113" s="67" t="inlineStr">
+    <row r="114" ht="29" customHeight="1">
+      <c r="A114" s="67" t="inlineStr">
         <is>
           <t>I03</t>
         </is>
       </c>
-      <c r="B113" s="67" t="inlineStr">
+      <c r="B114" s="67" t="inlineStr">
         <is>
           <t>Antenna</t>
         </is>
       </c>
-      <c r="C113" s="68" t="inlineStr">
+      <c r="C114" s="68" t="inlineStr">
         <is>
           <t>gateway antena 45 EUR - pouzijes svoju 868 + pigtail | range-critical: gateway antenna gain + mast height set the link</t>
         </is>
       </c>
-      <c r="E113" s="69" t="inlineStr">
+      <c r="E114" s="69" t="inlineStr">
         <is>
           <t>45.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="114" ht="15.5" customHeight="1">
-      <c r="A114" s="67" t="inlineStr">
-        <is>
-          <t>I04</t>
-        </is>
-      </c>
-      <c r="B114" s="67" t="inlineStr">
-        <is>
-          <t>Enclosure</t>
-        </is>
-      </c>
-      <c r="C114" s="68" t="inlineStr">
-        <is>
-          <t xml:space="preserve">vynechane: krabica pre gateway na stozieri | </t>
-        </is>
-      </c>
-      <c r="E114" s="69" t="inlineStr">
-        <is>
-          <t>35.0</t>
         </is>
       </c>
     </row>
     <row r="115" ht="15.5" customHeight="1">
       <c r="A115" s="67" t="inlineStr">
         <is>
-          <t>I05</t>
+          <t>I04</t>
         </is>
       </c>
       <c r="B115" s="67" t="inlineStr">
         <is>
-          <t>Mast</t>
+          <t>Enclosure</t>
         </is>
       </c>
       <c r="C115" s="68" t="inlineStr">
         <is>
-          <t>gateway stozier 30 EUR - plot, strom, cokolvek | height sets range</t>
+          <t xml:space="preserve">vynechane: krabica pre gateway na stozieri | </t>
         </is>
       </c>
       <c r="E115" s="69" t="inlineStr">
         <is>
-          <t>30.0</t>
+          <t>35.0</t>
         </is>
       </c>
     </row>
@@ -3394,23 +3398,23 @@
   </sheetData>
   <mergeCells count="18">
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A69:E69"/>
-    <mergeCell ref="A99:F99"/>
-    <mergeCell ref="A61:E61"/>
-    <mergeCell ref="A57:E57"/>
-    <mergeCell ref="A65:E65"/>
-    <mergeCell ref="A81:E81"/>
+    <mergeCell ref="A53:E53"/>
+    <mergeCell ref="A91:E91"/>
+    <mergeCell ref="A62:E62"/>
     <mergeCell ref="A95:E95"/>
-    <mergeCell ref="A52:E52"/>
     <mergeCell ref="A96:E96"/>
+    <mergeCell ref="A86:E86"/>
+    <mergeCell ref="A82:E82"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A90:E90"/>
-    <mergeCell ref="A85:E85"/>
+    <mergeCell ref="A100:F100"/>
     <mergeCell ref="A5:E5"/>
-    <mergeCell ref="A44:E44"/>
+    <mergeCell ref="A45:E45"/>
     <mergeCell ref="A32:E32"/>
-    <mergeCell ref="A94:E94"/>
+    <mergeCell ref="A66:E66"/>
     <mergeCell ref="A3:F3"/>
+    <mergeCell ref="A58:E58"/>
+    <mergeCell ref="A97:E97"/>
+    <mergeCell ref="A70:E70"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId1"/>
@@ -3425,12 +3429,12 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B22" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B24" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B25" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B47" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B48" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B49" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B54" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B55" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B67" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B48" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B49" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B51" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B55" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B56" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B68" r:id="rId18"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
@@ -5831,7 +5835,7 @@
         </is>
       </c>
       <c r="D62" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E62" s="6" t="inlineStr">
         <is>
@@ -5842,7 +5846,7 @@
         <v>6</v>
       </c>
       <c r="G62" s="8" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H62" s="7" t="inlineStr">
         <is>
@@ -5866,7 +5870,7 @@
       </c>
       <c r="L62" s="6" t="inlineStr">
         <is>
-          <t>v baleni kazdej Wio-E5 je EU868 antena - samostatne netreba; drzat ako zalohu</t>
+          <t>jedna 5 dBi na gateway; sonde staci bicik z kitu</t>
         </is>
       </c>
     </row>
@@ -6602,7 +6606,7 @@
       <c r="E76" s="73" t="n"/>
       <c r="F76" s="15" t="n"/>
       <c r="G76" s="15" t="n">
-        <v>102.9</v>
+        <v>108.9</v>
       </c>
       <c r="H76" s="14" t="n"/>
       <c r="I76" s="14" t="n"/>
@@ -7464,7 +7468,7 @@
       </c>
       <c r="L96" s="17" t="inlineStr">
         <is>
-          <t>YOU ALREADY HAVE THIS - reuse, zero soldering | YOU ALREADY HAVE THIS - reuse, zero soldering; runs the gateway service</t>
+          <t>YOU ALREADY HAVE THIS - reuse, zero soldering | MAM - Raspberry Pi 4, staci mu USB napajanie</t>
         </is>
       </c>
     </row>
@@ -7632,7 +7636,7 @@
       </c>
       <c r="L99" s="17" t="inlineStr">
         <is>
-          <t>gateway stozier 30 EUR - plot, strom, cokolvek | height sets range</t>
+          <t>3 m stozier pre gateway - vyskou sa kupuje dosah</t>
         </is>
       </c>
     </row>
@@ -8386,7 +8390,7 @@
       <c r="E120" s="72" t="n"/>
       <c r="F120" s="73" t="n"/>
       <c r="G120" s="25" t="n">
-        <v>716.3100000000001</v>
+        <v>722.3100000000001</v>
       </c>
     </row>
     <row r="121">
@@ -8416,7 +8420,7 @@
       <c r="E122" s="72" t="n"/>
       <c r="F122" s="73" t="n"/>
       <c r="G122" s="29" t="n">
-        <v>1357.31</v>
+        <v>1363.31</v>
       </c>
     </row>
     <row r="123">
@@ -8446,7 +8450,7 @@
       <c r="E124" s="72" t="n"/>
       <c r="F124" s="73" t="n"/>
       <c r="G124" s="33" t="n">
-        <v>1287.31</v>
+        <v>1293.31</v>
       </c>
     </row>
   </sheetData>
@@ -8634,7 +8638,7 @@
         </is>
       </c>
       <c r="B10" s="36" t="n">
-        <v>102.9</v>
+        <v>108.9</v>
       </c>
       <c r="C10" s="36" t="n">
         <v>0</v>
@@ -8714,7 +8718,7 @@
         </is>
       </c>
       <c r="B15" s="38" t="n">
-        <v>716.3100000000001</v>
+        <v>722.3100000000001</v>
       </c>
       <c r="C15" s="38" t="n">
         <v>641</v>

</xml_diff>

<commit_message>
order: links on 41 of 57 lines
Direct product pages where one exists (rpishop kit, x-teamrc 3506, techfun
turbidity/DS18B20/potting, supermagnete N52, TME igus bushings). TME lines carry
a catalogue search link because Cloudflare blocks automated access but a browser
walks straight through. Hardware-store lines point at hornbach.sk, which also
sits behind a bot check, so no per-item URL there.

The 16 unlinked lines are printed parts, in-house CAD items, what he already owns,
and three things with no shop (metal shop, site label, hinge collar pin).
</commit_message>
<xml_diff>
--- a/docs/sub-mission_parts.xlsx
+++ b/docs/sub-mission_parts.xlsx
@@ -405,6 +405,9 @@
     <xf numFmtId="0" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -413,9 +416,6 @@
     </xf>
     <xf numFmtId="4" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top"/>
@@ -924,23 +924,23 @@
           <t>D06</t>
         </is>
       </c>
-      <c r="B8" s="53" t="inlineStr">
+      <c r="B8" s="54" t="inlineStr">
         <is>
           <t>EC/TDS</t>
         </is>
       </c>
-      <c r="C8" s="54" t="inlineStr">
+      <c r="C8" s="55" t="inlineStr">
         <is>
           <t>DFRobot SEN0244 Gravity analog TDS module + probe  -  +-10% FS is the weakest sensor; use as trend indicator, site-calibrate</t>
         </is>
       </c>
-      <c r="D8" s="55" t="n">
-        <v>1</v>
-      </c>
-      <c r="E8" s="56" t="n">
+      <c r="D8" s="56" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="57" t="n">
         <v>14</v>
       </c>
-      <c r="F8" s="56" t="n">
+      <c r="F8" s="57" t="n">
         <v>14</v>
       </c>
     </row>
@@ -976,23 +976,23 @@
           <t>F02</t>
         </is>
       </c>
-      <c r="B10" s="57" t="inlineStr">
+      <c r="B10" s="54" t="inlineStr">
         <is>
           <t>Bulkhead connector</t>
         </is>
       </c>
-      <c r="C10" s="54" t="inlineStr">
+      <c r="C10" s="55" t="inlineStr">
         <is>
           <t>potted gland entry (NOT SubConn)  -  cost cut from 85 EUR wet-mate</t>
         </is>
       </c>
-      <c r="D10" s="55" t="n">
-        <v>1</v>
-      </c>
-      <c r="E10" s="56" t="n">
+      <c r="D10" s="56" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="57" t="n">
         <v>12</v>
       </c>
-      <c r="F10" s="56" t="n">
+      <c r="F10" s="57" t="n">
         <v>12</v>
       </c>
     </row>
@@ -1002,7 +1002,7 @@
           <t>G10</t>
         </is>
       </c>
-      <c r="B11" s="49" t="inlineStr">
+      <c r="B11" s="50" t="inlineStr">
         <is>
           <t>Supercap</t>
         </is>
@@ -1028,23 +1028,23 @@
           <t>G17</t>
         </is>
       </c>
-      <c r="B12" s="57" t="inlineStr">
+      <c r="B12" s="54" t="inlineStr">
         <is>
           <t>Cable glands</t>
         </is>
       </c>
-      <c r="C12" s="54" t="inlineStr">
+      <c r="C12" s="55" t="inlineStr">
         <is>
           <t>M12 IP68 potted x3</t>
         </is>
       </c>
-      <c r="D12" s="55" t="n">
+      <c r="D12" s="56" t="n">
         <v>3</v>
       </c>
-      <c r="E12" s="56" t="n">
+      <c r="E12" s="57" t="n">
         <v>3</v>
       </c>
-      <c r="F12" s="56" t="n">
+      <c r="F12" s="57" t="n">
         <v>9</v>
       </c>
     </row>
@@ -1054,7 +1054,7 @@
           <t>H09</t>
         </is>
       </c>
-      <c r="B13" s="49" t="inlineStr">
+      <c r="B13" s="50" t="inlineStr">
         <is>
           <t>Guy line</t>
         </is>
@@ -1080,23 +1080,23 @@
           <t>E02</t>
         </is>
       </c>
-      <c r="B14" s="57" t="inlineStr">
+      <c r="B14" s="54" t="inlineStr">
         <is>
           <t>Cage fasteners</t>
         </is>
       </c>
-      <c r="C14" s="54" t="inlineStr">
+      <c r="C14" s="55" t="inlineStr">
         <is>
           <t>M3x10 A4 + nylok</t>
         </is>
       </c>
-      <c r="D14" s="55" t="n">
-        <v>1</v>
-      </c>
-      <c r="E14" s="56" t="n">
+      <c r="D14" s="56" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="57" t="n">
         <v>6</v>
       </c>
-      <c r="F14" s="56" t="n">
+      <c r="F14" s="57" t="n">
         <v>6</v>
       </c>
     </row>
@@ -1132,23 +1132,23 @@
           <t>G16</t>
         </is>
       </c>
-      <c r="B16" s="57" t="inlineStr">
+      <c r="B16" s="54" t="inlineStr">
         <is>
           <t>Protection</t>
         </is>
       </c>
-      <c r="C16" s="54" t="inlineStr">
+      <c r="C16" s="55" t="inlineStr">
         <is>
           <t>Fuse 0.5A + TVS + ESD array  -  NEMAM - poistka 0.5A + TVS SMBJ5.0A + ESD array (SOT-23-6)</t>
         </is>
       </c>
-      <c r="D16" s="55" t="n">
-        <v>1</v>
-      </c>
-      <c r="E16" s="56" t="n">
+      <c r="D16" s="56" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" s="57" t="n">
         <v>6</v>
       </c>
-      <c r="F16" s="56" t="n">
+      <c r="F16" s="57" t="n">
         <v>6</v>
       </c>
     </row>
@@ -1184,23 +1184,23 @@
           <t>G06</t>
         </is>
       </c>
-      <c r="B18" s="53" t="inlineStr">
+      <c r="B18" s="54" t="inlineStr">
         <is>
           <t>Boost harvester</t>
         </is>
       </c>
-      <c r="C18" s="54" t="inlineStr">
+      <c r="C18" s="55" t="inlineStr">
         <is>
           <t>LTC3105EFE MPPT boost  -  needed when EMF below bus</t>
         </is>
       </c>
-      <c r="D18" s="55" t="n">
-        <v>1</v>
-      </c>
-      <c r="E18" s="56" t="n">
+      <c r="D18" s="56" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" s="57" t="n">
         <v>5</v>
       </c>
-      <c r="F18" s="56" t="n">
+      <c r="F18" s="57" t="n">
         <v>5</v>
       </c>
     </row>
@@ -1210,7 +1210,7 @@
           <t>G09</t>
         </is>
       </c>
-      <c r="B19" s="49" t="inlineStr">
+      <c r="B19" s="50" t="inlineStr">
         <is>
           <t>Clamp</t>
         </is>
@@ -1236,23 +1236,23 @@
           <t>H11</t>
         </is>
       </c>
-      <c r="B20" s="53" t="inlineStr">
+      <c r="B20" s="54" t="inlineStr">
         <is>
           <t>Safety cable</t>
         </is>
       </c>
-      <c r="C20" s="54" t="inlineStr">
+      <c r="C20" s="55" t="inlineStr">
         <is>
           <t>3mm galv wire + ferrules tethering pod to pole  -  theft/flood retention</t>
         </is>
       </c>
-      <c r="D20" s="55" t="n">
-        <v>1</v>
-      </c>
-      <c r="E20" s="56" t="n">
+      <c r="D20" s="56" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" s="57" t="n">
         <v>4</v>
       </c>
-      <c r="F20" s="56" t="n">
+      <c r="F20" s="57" t="n">
         <v>4</v>
       </c>
     </row>
@@ -1288,23 +1288,23 @@
           <t>C05</t>
         </is>
       </c>
-      <c r="B22" s="57" t="inlineStr">
+      <c r="B22" s="54" t="inlineStr">
         <is>
           <t>Pod clamp screws</t>
         </is>
       </c>
-      <c r="C22" s="54" t="inlineStr">
+      <c r="C22" s="55" t="inlineStr">
         <is>
           <t>M4x30 A4 + washers  -  drzi zadny spoj; integralny bulkhead riesi len prednu stranu</t>
         </is>
       </c>
-      <c r="D22" s="55" t="n">
-        <v>1</v>
-      </c>
-      <c r="E22" s="56" t="n">
+      <c r="D22" s="56" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" s="57" t="n">
         <v>3</v>
       </c>
-      <c r="F22" s="56" t="n">
+      <c r="F22" s="57" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1314,7 +1314,7 @@
           <t>G07</t>
         </is>
       </c>
-      <c r="B23" s="49" t="inlineStr">
+      <c r="B23" s="50" t="inlineStr">
         <is>
           <t>Buck</t>
         </is>
@@ -1340,23 +1340,23 @@
           <t>A04</t>
         </is>
       </c>
-      <c r="B24" s="57" t="inlineStr">
+      <c r="B24" s="54" t="inlineStr">
         <is>
           <t>Wet bearing</t>
         </is>
       </c>
-      <c r="C24" s="54" t="inlineStr">
+      <c r="C24" s="55" t="inlineStr">
         <is>
           <t>igus iglidur J plain bearing JSM-0507-05 5x7x5mm  -  83 pcs in stock; JFM-0507-05 flanged 1.48 USD alt</t>
         </is>
       </c>
-      <c r="D24" s="55" t="n">
+      <c r="D24" s="56" t="n">
         <v>2</v>
       </c>
-      <c r="E24" s="56" t="n">
+      <c r="E24" s="57" t="n">
         <v>1.18</v>
       </c>
-      <c r="F24" s="56" t="n">
+      <c r="F24" s="57" t="n">
         <v>2.36</v>
       </c>
     </row>
@@ -1392,23 +1392,23 @@
           <t>G12</t>
         </is>
       </c>
-      <c r="B26" s="53" t="inlineStr">
+      <c r="B26" s="54" t="inlineStr">
         <is>
           <t>Load switch</t>
         </is>
       </c>
-      <c r="C26" s="54" t="inlineStr">
+      <c r="C26" s="55" t="inlineStr">
         <is>
           <t>TPS22860 x2 for pH/EC sequencing  -  removes ground-loop need</t>
         </is>
       </c>
-      <c r="D26" s="55" t="n">
+      <c r="D26" s="56" t="n">
         <v>2</v>
       </c>
-      <c r="E26" s="56" t="n">
-        <v>1</v>
-      </c>
-      <c r="F26" s="56" t="n">
+      <c r="E26" s="57" t="n">
+        <v>1</v>
+      </c>
+      <c r="F26" s="57" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1418,7 +1418,7 @@
           <t>G11</t>
         </is>
       </c>
-      <c r="B27" s="49" t="inlineStr">
+      <c r="B27" s="50" t="inlineStr">
         <is>
           <t>Voltage supervisor</t>
         </is>
@@ -1449,18 +1449,18 @@
           <t>Shear pin</t>
         </is>
       </c>
-      <c r="C28" s="54" t="inlineStr">
+      <c r="C28" s="55" t="inlineStr">
         <is>
           <t>M4 316SS pin + 2 spares on pole collar  -  releases pod on &gt;150N debris hit</t>
         </is>
       </c>
-      <c r="D28" s="55" t="n">
-        <v>1</v>
-      </c>
-      <c r="E28" s="56" t="n">
-        <v>1</v>
-      </c>
-      <c r="F28" s="56" t="n">
+      <c r="D28" s="56" t="n">
+        <v>1</v>
+      </c>
+      <c r="E28" s="57" t="n">
+        <v>1</v>
+      </c>
+      <c r="F28" s="57" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1470,7 +1470,7 @@
           <t>G08</t>
         </is>
       </c>
-      <c r="B29" s="49" t="inlineStr">
+      <c r="B29" s="50" t="inlineStr">
         <is>
           <t>Rectifier</t>
         </is>
@@ -1564,7 +1564,7 @@
           <t>I05</t>
         </is>
       </c>
-      <c r="B34" s="49" t="inlineStr">
+      <c r="B34" s="50" t="inlineStr">
         <is>
           <t>Mast</t>
         </is>
@@ -1590,23 +1590,23 @@
           <t>H01</t>
         </is>
       </c>
-      <c r="B35" s="53" t="inlineStr">
+      <c r="B35" s="54" t="inlineStr">
         <is>
           <t>Ground screw anchor</t>
         </is>
       </c>
-      <c r="C35" s="54" t="inlineStr">
+      <c r="C35" s="55" t="inlineStr">
         <is>
           <t>M68 x 800mm solar-fence ground screw  -  1-2kN lateral - covers flood case</t>
         </is>
       </c>
-      <c r="D35" s="55" t="n">
-        <v>1</v>
-      </c>
-      <c r="E35" s="56" t="n">
+      <c r="D35" s="56" t="n">
+        <v>1</v>
+      </c>
+      <c r="E35" s="57" t="n">
         <v>25</v>
       </c>
-      <c r="F35" s="56" t="n">
+      <c r="F35" s="57" t="n">
         <v>25</v>
       </c>
     </row>
@@ -1616,7 +1616,7 @@
           <t>H02</t>
         </is>
       </c>
-      <c r="B36" s="49" t="inlineStr">
+      <c r="B36" s="50" t="inlineStr">
         <is>
           <t>Pole</t>
         </is>
@@ -1642,23 +1642,23 @@
           <t>H10</t>
         </is>
       </c>
-      <c r="B37" s="53" t="inlineStr">
+      <c r="B37" s="54" t="inlineStr">
         <is>
           <t>Guy anchor</t>
         </is>
       </c>
-      <c r="C37" s="54" t="inlineStr">
+      <c r="C37" s="55" t="inlineStr">
         <is>
           <t>300mm ground screw x2</t>
         </is>
       </c>
-      <c r="D37" s="55" t="n">
-        <v>1</v>
-      </c>
-      <c r="E37" s="56" t="n">
+      <c r="D37" s="56" t="n">
+        <v>1</v>
+      </c>
+      <c r="E37" s="57" t="n">
         <v>10</v>
       </c>
-      <c r="F37" s="56" t="n">
+      <c r="F37" s="57" t="n">
         <v>10</v>
       </c>
     </row>
@@ -1668,7 +1668,7 @@
           <t>H04</t>
         </is>
       </c>
-      <c r="B38" s="49" t="inlineStr">
+      <c r="B38" s="50" t="inlineStr">
         <is>
           <t>Arm tube</t>
         </is>
@@ -1694,23 +1694,23 @@
           <t>H05</t>
         </is>
       </c>
-      <c r="B39" s="53" t="inlineStr">
+      <c r="B39" s="54" t="inlineStr">
         <is>
           <t>Drop tube</t>
         </is>
       </c>
-      <c r="C39" s="54" t="inlineStr">
+      <c r="C39" s="55" t="inlineStr">
         <is>
           <t>alu Ø22x1.5 x 900mm</t>
         </is>
       </c>
-      <c r="D39" s="55" t="n">
-        <v>1</v>
-      </c>
-      <c r="E39" s="56" t="n">
+      <c r="D39" s="56" t="n">
+        <v>1</v>
+      </c>
+      <c r="E39" s="57" t="n">
         <v>6</v>
       </c>
-      <c r="F39" s="56" t="n">
+      <c r="F39" s="57" t="n">
         <v>6</v>
       </c>
     </row>
@@ -1720,7 +1720,7 @@
           <t>K03</t>
         </is>
       </c>
-      <c r="B40" s="49" t="inlineStr">
+      <c r="B40" s="50" t="inlineStr">
         <is>
           <t>Spring balance</t>
         </is>
@@ -1746,23 +1746,23 @@
           <t>C06</t>
         </is>
       </c>
-      <c r="B41" s="53" t="inlineStr">
+      <c r="B41" s="54" t="inlineStr">
         <is>
           <t>Desiccant</t>
         </is>
       </c>
-      <c r="C41" s="54" t="inlineStr">
+      <c r="C41" s="55" t="inlineStr">
         <is>
           <t>5g silica gel with indicator  -  replace at service</t>
         </is>
       </c>
-      <c r="D41" s="55" t="n">
+      <c r="D41" s="56" t="n">
         <v>2</v>
       </c>
-      <c r="E41" s="56" t="n">
+      <c r="E41" s="57" t="n">
         <v>2</v>
       </c>
-      <c r="F41" s="56" t="n">
+      <c r="F41" s="57" t="n">
         <v>4</v>
       </c>
     </row>
@@ -1866,7 +1866,7 @@
           <t>J03</t>
         </is>
       </c>
-      <c r="B47" s="49" t="inlineStr">
+      <c r="B47" s="50" t="inlineStr">
         <is>
           <t>Epoxy barrier</t>
         </is>
@@ -1892,23 +1892,23 @@
           <t>B04</t>
         </is>
       </c>
-      <c r="B48" s="57" t="inlineStr">
+      <c r="B48" s="54" t="inlineStr">
         <is>
           <t>Potting compound</t>
         </is>
       </c>
-      <c r="C48" s="54" t="inlineStr">
+      <c r="C48" s="55" t="inlineStr">
         <is>
           <t>3M Scotch-Weld DP270 black 25ml  -  techfun nema DP270; silikonova zalievacia hmota staci na test, epoxid je tuhsi</t>
         </is>
       </c>
-      <c r="D48" s="55" t="n">
-        <v>1</v>
-      </c>
-      <c r="E48" s="56" t="n">
+      <c r="D48" s="56" t="n">
+        <v>1</v>
+      </c>
+      <c r="E48" s="57" t="n">
         <v>14</v>
       </c>
-      <c r="F48" s="56" t="n">
+      <c r="F48" s="57" t="n">
         <v>14</v>
       </c>
     </row>
@@ -1944,23 +1944,23 @@
           <t>G04</t>
         </is>
       </c>
-      <c r="B50" s="53" t="inlineStr">
+      <c r="B50" s="54" t="inlineStr">
         <is>
           <t>Antenna probe</t>
         </is>
       </c>
-      <c r="C50" s="54" t="inlineStr">
+      <c r="C50" s="55" t="inlineStr">
         <is>
           <t>868MHz 5dBi SMA-M omni 195mm  -  jedna 5 dBi na gateway; sonde staci bicik z kitu</t>
         </is>
       </c>
-      <c r="D50" s="55" t="n">
-        <v>1</v>
-      </c>
-      <c r="E50" s="56" t="n">
+      <c r="D50" s="56" t="n">
+        <v>1</v>
+      </c>
+      <c r="E50" s="57" t="n">
         <v>6</v>
       </c>
-      <c r="F50" s="56" t="n">
+      <c r="F50" s="57" t="n">
         <v>6</v>
       </c>
     </row>
@@ -2064,23 +2064,23 @@
           <t>I01</t>
         </is>
       </c>
-      <c r="B56" s="57" t="inlineStr">
+      <c r="B56" s="54" t="inlineStr">
         <is>
           <t>Gateway radio (single-channel)</t>
         </is>
       </c>
-      <c r="C56" s="54" t="inlineStr">
+      <c r="C56" s="55" t="inlineStr">
         <is>
           <t>Seeed XIAO nRF52840 + Wio-SX1262 kit (Meshtastic), SEE336 - nRF52840 + SX1262  -  349 Kc, skladom 5+; nahradza Wio-E5, ktory v CZ/SK nie je; antena je v kite</t>
         </is>
       </c>
-      <c r="D56" s="55" t="n">
-        <v>1</v>
-      </c>
-      <c r="E56" s="56" t="n">
+      <c r="D56" s="56" t="n">
+        <v>1</v>
+      </c>
+      <c r="E56" s="57" t="n">
         <v>14</v>
       </c>
-      <c r="F56" s="56" t="n">
+      <c r="F56" s="57" t="n">
         <v>14</v>
       </c>
     </row>
@@ -2132,7 +2132,7 @@
           <t>C08</t>
         </is>
       </c>
-      <c r="B60" s="49" t="inlineStr">
+      <c r="B60" s="50" t="inlineStr">
         <is>
           <t>Generator</t>
         </is>
@@ -2200,7 +2200,7 @@
           <t>G15</t>
         </is>
       </c>
-      <c r="B64" s="49" t="inlineStr">
+      <c r="B64" s="50" t="inlineStr">
         <is>
           <t>Connectors</t>
         </is>
@@ -2367,18 +2367,18 @@
           <t>Generator mount</t>
         </is>
       </c>
-      <c r="C73" s="54" t="inlineStr">
+      <c r="C73" s="55" t="inlineStr">
         <is>
           <t>printed cradle + 4x M3x8 A4</t>
         </is>
       </c>
-      <c r="D73" s="55" t="n">
-        <v>1</v>
-      </c>
-      <c r="E73" s="56" t="n">
-        <v>1</v>
-      </c>
-      <c r="F73" s="56" t="n">
+      <c r="D73" s="56" t="n">
+        <v>1</v>
+      </c>
+      <c r="E73" s="57" t="n">
+        <v>1</v>
+      </c>
+      <c r="F73" s="57" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2419,18 +2419,18 @@
           <t>Hub</t>
         </is>
       </c>
-      <c r="C75" s="54" t="inlineStr">
+      <c r="C75" s="55" t="inlineStr">
         <is>
           <t>Ø64x46mm with 2x M4 heat-set inserts and Ø5 H7 shaft bore  -  brass inserts M4 from TME</t>
         </is>
       </c>
-      <c r="D75" s="55" t="n">
-        <v>1</v>
-      </c>
-      <c r="E75" s="56" t="n">
+      <c r="D75" s="56" t="n">
+        <v>1</v>
+      </c>
+      <c r="E75" s="57" t="n">
         <v>0</v>
       </c>
-      <c r="F75" s="56" t="n">
+      <c r="F75" s="57" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2471,18 +2471,18 @@
           <t>Pod barrel</t>
         </is>
       </c>
-      <c r="C77" s="54" t="inlineStr">
+      <c r="C77" s="55" t="inlineStr">
         <is>
           <t>Ø110x120mm printed ASA wall 2.4mm + epoxy barrier  -  in model as pod</t>
         </is>
       </c>
-      <c r="D77" s="55" t="n">
-        <v>1</v>
-      </c>
-      <c r="E77" s="56" t="n">
+      <c r="D77" s="56" t="n">
+        <v>1</v>
+      </c>
+      <c r="E77" s="57" t="n">
         <v>0</v>
       </c>
-      <c r="F77" s="56" t="n">
+      <c r="F77" s="57" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2523,18 +2523,18 @@
           <t>Sensor cage</t>
         </is>
       </c>
-      <c r="C79" s="54" t="inlineStr">
+      <c r="C79" s="55" t="inlineStr">
         <is>
           <t>Ø130x150 printed ASA 12 slots  -  in model as cage</t>
         </is>
       </c>
-      <c r="D79" s="55" t="n">
-        <v>1</v>
-      </c>
-      <c r="E79" s="56" t="n">
+      <c r="D79" s="56" t="n">
+        <v>1</v>
+      </c>
+      <c r="E79" s="57" t="n">
         <v>0</v>
       </c>
-      <c r="F79" s="56" t="n">
+      <c r="F79" s="57" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2612,7 +2612,7 @@
           <t>G14</t>
         </is>
       </c>
-      <c r="B84" s="49" t="inlineStr">
+      <c r="B84" s="50" t="inlineStr">
         <is>
           <t>PCB</t>
         </is>
@@ -2711,18 +2711,18 @@
           <t>Separation wall</t>
         </is>
       </c>
-      <c r="C89" s="54" t="inlineStr">
+      <c r="C89" s="55" t="inlineStr">
         <is>
           <t>D106 x 4 mm - RECOMMENDED integral with the pod bulkhead (no separate part)  -  4 mm per CAD, not 5; integral removes O-ring C03 and screws C05</t>
         </is>
       </c>
-      <c r="D89" s="55" t="n">
-        <v>1</v>
-      </c>
-      <c r="E89" s="56" t="n">
+      <c r="D89" s="56" t="n">
+        <v>1</v>
+      </c>
+      <c r="E89" s="57" t="n">
         <v>0</v>
       </c>
-      <c r="F89" s="56" t="n">
+      <c r="F89" s="57" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3418,23 +3418,46 @@
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B9" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B10" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B12" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B14" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B15" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B16" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B17" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B21" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B22" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B24" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B25" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B48" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B49" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B51" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B55" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B56" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B68" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B9" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B10" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B12" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B13" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B14" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B15" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B16" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B17" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B18" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B19" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B20" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B21" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B22" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B23" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B24" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B25" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B26" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B27" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B29" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B34" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B35" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B36" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B37" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B38" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B39" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B40" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B41" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B47" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B48" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B49" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B50" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B51" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B55" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B56" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B60" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B64" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B68" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B84" r:id="rId41"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>

</xml_diff>